<commit_message>
Added 5 Test scenarios
Added 5 Test scenarios and Replaced return flag with Asserts
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -149,19 +149,19 @@
     <t>POS</t>
   </si>
   <si>
-    <t>CURRENCYINR</t>
+    <t>CurrencyInr</t>
   </si>
   <si>
     <t>INR</t>
   </si>
   <si>
-    <t>POHTYPE</t>
+    <t>PohType</t>
   </si>
   <si>
     <t>PO - GENERAL</t>
   </si>
   <si>
-    <t>UOMNOS</t>
+    <t>UomNos</t>
   </si>
   <si>
     <t>NOS</t>
@@ -177,6 +177,36 @@
   </si>
   <si>
     <t>PO - SERVICE</t>
+  </si>
+  <si>
+    <t>DissimilarItem</t>
+  </si>
+  <si>
+    <t>GWL_ITEM_DISIMILAR_UOM</t>
+  </si>
+  <si>
+    <t>PR_Service</t>
+  </si>
+  <si>
+    <t>PR - SERVICES</t>
+  </si>
+  <si>
+    <t>Prefix_PRGWL</t>
+  </si>
+  <si>
+    <t>PRGWL</t>
+  </si>
+  <si>
+    <t>GwlItem_Service</t>
+  </si>
+  <si>
+    <t>GWL_SERVICES_02</t>
+  </si>
+  <si>
+    <t>CancelStatus</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
   </si>
 </sst>
 </file>
@@ -1354,24 +1384,44 @@
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
+      <c r="A27" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
+      <c r="A28" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
+      <c r="A29" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
+      <c r="A30" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
+      <c r="A31" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2"/>

</xml_diff>

<commit_message>
Updated and Fixed Test Scenario in Purchase Request.
Added one test scenario and fixed one test case in purchase request.
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -207,6 +207,12 @@
   </si>
   <si>
     <t>Cancelled</t>
+  </si>
+  <si>
+    <t>PRtemplate1Line</t>
+  </si>
+  <si>
+    <t>PRTemplateSingleLine.csv</t>
   </si>
 </sst>
 </file>
@@ -1169,10 +1175,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B33"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="27.1111111111111" customWidth="1"/>
+    <col min="1" max="1" width="30.1090909090909" customWidth="1"/>
+    <col min="2" max="2" width="27.1090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1424,8 +1430,12 @@
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
+      <c r="A32" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2"/>

</xml_diff>

<commit_message>
Added 5 Test Scenarios and Updated Changes
Added 5 Test Scenarios and Updated Changes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="17231" windowHeight="8064"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <oleSize ref="A1:B33"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -213,6 +214,24 @@
   </si>
   <si>
     <t>PRTemplateSingleLine.csv</t>
+  </si>
+  <si>
+    <t>WalmartSupplier</t>
+  </si>
+  <si>
+    <t>WALMART</t>
+  </si>
+  <si>
+    <t>CurrencyUsd</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>DissimilarService</t>
+  </si>
+  <si>
+    <t>GWL_Dissimilar_Services</t>
   </si>
 </sst>
 </file>
@@ -1174,11 +1193,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B33"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B35"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.1090909090909" customWidth="1"/>
-    <col min="2" max="2" width="27.1090909090909" customWidth="1"/>
+    <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
+    <col min="2" max="2" width="27.1111111111111" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1438,8 +1457,28 @@
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
+      <c r="A33" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>66</v>
+      </c>
+      <c r="B35" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added 1 test scenarios
Added 1 test scenarios and Updated Changes in Purchase Order Functions class
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,13 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="17231" windowHeight="8064"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <oleSize ref="A1:B33"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -232,6 +231,60 @@
   </si>
   <si>
     <t>GWL_Dissimilar_Services</t>
+  </si>
+  <si>
+    <t>Location02</t>
+  </si>
+  <si>
+    <t>L0002</t>
+  </si>
+  <si>
+    <t>StockTransferSelect</t>
+  </si>
+  <si>
+    <t>POT</t>
+  </si>
+  <si>
+    <t>U1Supplier</t>
+  </si>
+  <si>
+    <t>SUP00325</t>
+  </si>
+  <si>
+    <t>St_Item_Similar</t>
+  </si>
+  <si>
+    <t>GWL_CHECKING_ST</t>
+  </si>
+  <si>
+    <t>Po_Stock_Transfer</t>
+  </si>
+  <si>
+    <t>PO - STOCK TRANSFER</t>
+  </si>
+  <si>
+    <t>Stock_Item_Dissimilar</t>
+  </si>
+  <si>
+    <t>GWL_Dissimilar_ST_Check</t>
+  </si>
+  <si>
+    <t>DoubleDecimal</t>
+  </si>
+  <si>
+    <t>0.00</t>
+  </si>
+  <si>
+    <t>PackingCharges</t>
+  </si>
+  <si>
+    <t>TVS-CH-00003</t>
+  </si>
+  <si>
+    <t>GlAccDescription</t>
+  </si>
+  <si>
+    <t>ADMINISTRATIVE EXPENES</t>
   </si>
 </sst>
 </file>
@@ -868,12 +921,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1193,7 +1247,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
@@ -1473,11 +1527,83 @@
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" t="s">
+      <c r="A35" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="2" t="s">
         <v>67</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Failure Fixes In Purchase Order And Purchase Request Test Scenarios
Updated Failure Fixes In Purchase Order And Purchase Request Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -182,7 +182,7 @@
     <t>DissimilarItem</t>
   </si>
   <si>
-    <t>GWL_ITEM_DISIMILAR_UOM</t>
+    <t>GWL_ITEM_DISSIMILAR_UOM</t>
   </si>
   <si>
     <t>PR_Service</t>
@@ -243,6 +243,12 @@
   </si>
   <si>
     <t>TEST</t>
+  </si>
+  <si>
+    <t>Kgs</t>
+  </si>
+  <si>
+    <t>KGS</t>
   </si>
 </sst>
 </file>
@@ -1204,11 +1210,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B39"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.1090909090909" customWidth="1"/>
-    <col min="2" max="2" width="27.1090909090909" customWidth="1"/>
+    <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
+    <col min="2" max="2" width="27.1111111111111" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1484,28 +1490,40 @@
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" t="s">
+      <c r="A35" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="2" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" t="s">
+      <c r="A36" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="2" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" t="s">
+      <c r="A37" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="2" t="s">
         <v>71</v>
       </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Data In TestData File
Updated Data In TestData File
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="11471" windowHeight="8520"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -249,6 +249,60 @@
   </si>
   <si>
     <t>KGS</t>
+  </si>
+  <si>
+    <t>Location02</t>
+  </si>
+  <si>
+    <t>L0002</t>
+  </si>
+  <si>
+    <t>StockTransferSelect</t>
+  </si>
+  <si>
+    <t>POT</t>
+  </si>
+  <si>
+    <t>U1Supplier</t>
+  </si>
+  <si>
+    <t>SUP00325</t>
+  </si>
+  <si>
+    <t>St_Item_Similar</t>
+  </si>
+  <si>
+    <t>GWL_CHECKING_ST</t>
+  </si>
+  <si>
+    <t>Po_Stock_Transfer</t>
+  </si>
+  <si>
+    <t>PO - STOCK TRANSFER</t>
+  </si>
+  <si>
+    <t>Stock_Item_Dissimilar</t>
+  </si>
+  <si>
+    <t>GWL_Dissimilar_ST_Check</t>
+  </si>
+  <si>
+    <t>DoubleDecimal</t>
+  </si>
+  <si>
+    <t>0.00</t>
+  </si>
+  <si>
+    <t>PackingCharges</t>
+  </si>
+  <si>
+    <t>TVS-CH-00003</t>
+  </si>
+  <si>
+    <t>GlAccDescription</t>
+  </si>
+  <si>
+    <t>ADMINISTRATIVE EXPENES</t>
   </si>
 </sst>
 </file>
@@ -885,12 +939,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1210,7 +1265,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
@@ -1522,8 +1577,76 @@
       </c>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
+      <c r="A39" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Purchase Request Line Details validation
Updated Purchase Request (Line Details validation)
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11471" windowHeight="8520"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -303,6 +303,12 @@
   </si>
   <si>
     <t>ADMINISTRATIVE EXPENES</t>
+  </si>
+  <si>
+    <t>Unit_100</t>
+  </si>
+  <si>
+    <t>U100</t>
   </si>
 </sst>
 </file>
@@ -939,13 +945,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1265,11 +1272,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <dimension ref="A1:B48"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="27.1111111111111" customWidth="1"/>
+    <col min="1" max="1" width="30.1090909090909" customWidth="1"/>
+    <col min="2" max="2" width="27.1090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1648,6 +1655,14 @@
         <v>91</v>
       </c>
     </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Added Employee Master and Employee Permission Module Test Scenarios
Added Employee Master and Employee Permission Module Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="188">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -327,6 +327,270 @@
   </si>
   <si>
     <t>(2022)</t>
+  </si>
+  <si>
+    <t>Emp_Salution</t>
+  </si>
+  <si>
+    <t>Mr.</t>
+  </si>
+  <si>
+    <t>Emp_FName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GWL Emp - </t>
+  </si>
+  <si>
+    <t>Emp_LName</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>Emp_MaleGender</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Emp_DOB</t>
+  </si>
+  <si>
+    <t>16-02-2000</t>
+  </si>
+  <si>
+    <t>Emp_DOJ</t>
+  </si>
+  <si>
+    <t>16-02-2024</t>
+  </si>
+  <si>
+    <t>Emp_GeneralShift</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>Emp_1to31Calendar</t>
+  </si>
+  <si>
+    <t>1 TO 30/31</t>
+  </si>
+  <si>
+    <t>Emp_GeneralZone</t>
+  </si>
+  <si>
+    <t>GENERAL</t>
+  </si>
+  <si>
+    <t>Emp_SalesCompanyCategory</t>
+  </si>
+  <si>
+    <t>SALES</t>
+  </si>
+  <si>
+    <t>Emp_SalaryAcc-AccountCategory</t>
+  </si>
+  <si>
+    <t>SALARY ACCOUNT</t>
+  </si>
+  <si>
+    <t>Emp_CleanerPayrollGroup</t>
+  </si>
+  <si>
+    <t>CLEANER</t>
+  </si>
+  <si>
+    <t>Emp_NoticePeriod-30</t>
+  </si>
+  <si>
+    <t>Emp_City</t>
+  </si>
+  <si>
+    <t>PLAIN CITY</t>
+  </si>
+  <si>
+    <t>Emp_Qualification</t>
+  </si>
+  <si>
+    <t>B.Tech</t>
+  </si>
+  <si>
+    <t>Emp_BranchofStudy</t>
+  </si>
+  <si>
+    <t>COMPUTER SCIENCE</t>
+  </si>
+  <si>
+    <t>Emp_YearOfPassing</t>
+  </si>
+  <si>
+    <t>Emp_Skill</t>
+  </si>
+  <si>
+    <t>PUNCHUALITY</t>
+  </si>
+  <si>
+    <t>Emp_Level</t>
+  </si>
+  <si>
+    <t>EXCELLENT</t>
+  </si>
+  <si>
+    <t>Emp_SalaryDesignation</t>
+  </si>
+  <si>
+    <t>FINANCE MANAGER</t>
+  </si>
+  <si>
+    <t>Emp_SalaryDepartment</t>
+  </si>
+  <si>
+    <t>PRODUCTION</t>
+  </si>
+  <si>
+    <t>Emp_SalaryGrade</t>
+  </si>
+  <si>
+    <t>GRADE A</t>
+  </si>
+  <si>
+    <t>Emp_AdjmntElement</t>
+  </si>
+  <si>
+    <t>ENCASH</t>
+  </si>
+  <si>
+    <t>Emp_AdjmntStartYear</t>
+  </si>
+  <si>
+    <t>Emp_AdjmntPeriod</t>
+  </si>
+  <si>
+    <t>DEC</t>
+  </si>
+  <si>
+    <t>Emp_AdjmntTotalPeriod</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Emp_AdjmntPeriodAmnt</t>
+  </si>
+  <si>
+    <t>2000</t>
+  </si>
+  <si>
+    <t>LeaveElgblLeave</t>
+  </si>
+  <si>
+    <t>CL</t>
+  </si>
+  <si>
+    <t>LeaveElgblDays</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>EmpLeaveElgblEvery</t>
+  </si>
+  <si>
+    <t>Year(s)</t>
+  </si>
+  <si>
+    <t>EmpLeaveElgblEligibileDays</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>EmpLeaveElgblRoundOff</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>EmpLeaveElgblMaxCarryFreq</t>
+  </si>
+  <si>
+    <t>Yearly</t>
+  </si>
+  <si>
+    <t>EmpLeaveElgblMaxCarryDay</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>EmpLeaveElgblEffYear</t>
+  </si>
+  <si>
+    <t>202324</t>
+  </si>
+  <si>
+    <t>EmpLeaveElgblMaxDay</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>EmpLeaveElgblMinDay</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>EmployeeDurai</t>
+  </si>
+  <si>
+    <t>DURAIRAJ  R</t>
+  </si>
+  <si>
+    <t>PermFromDate</t>
+  </si>
+  <si>
+    <t>24-05-2024</t>
+  </si>
+  <si>
+    <t>PermissionTimeFrom</t>
+  </si>
+  <si>
+    <t>16:30</t>
+  </si>
+  <si>
+    <t>PermissionTimeTo</t>
+  </si>
+  <si>
+    <t>18:30</t>
+  </si>
+  <si>
+    <t>PermissionReference</t>
+  </si>
+  <si>
+    <t>Permission</t>
+  </si>
+  <si>
+    <t>PermissionType</t>
+  </si>
+  <si>
+    <t>On-Duty (Day)</t>
+  </si>
+  <si>
+    <t>OnDutyFindType</t>
+  </si>
+  <si>
+    <t>On - Duty(Day)</t>
+  </si>
+  <si>
+    <t>OnDutyFromDate</t>
+  </si>
+  <si>
+    <t>25-05-2024</t>
+  </si>
+  <si>
+    <t>PermissionFindType</t>
   </si>
 </sst>
 </file>
@@ -339,7 +603,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -354,6 +618,17 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -833,145 +1108,158 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1291,418 +1579,418 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B52"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <dimension ref="A1:B98"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="27.1111111111111" customWidth="1"/>
+    <col min="1" max="1" width="30.1090909090909" customWidth="1"/>
+    <col min="2" max="2" width="27.1090909090909" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="5">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="5">
         <v>150</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="5" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="5" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="5" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="5" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="5" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="5" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="5" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="5" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="5" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="5" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="5" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:2">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="5" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="2" t="s">
+      <c r="A43" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="5" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" s="2" t="s">
+      <c r="A44" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="5" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="2" t="s">
+      <c r="A45" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="5" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="2" t="s">
+      <c r="A46" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="5" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="5" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="2" t="s">
+      <c r="A48" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="5" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="5">
         <v>5</v>
       </c>
     </row>
     <row r="50" spans="1:2">
-      <c r="A50" s="2" t="s">
+      <c r="A50" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="5" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:2">
-      <c r="A51" s="2" t="s">
+      <c r="A51" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="5" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1712,6 +2000,374 @@
       </c>
       <c r="B52" s="5" t="s">
         <v>99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B65" s="7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B69" s="8">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B76" s="8">
+        <v>202425</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B79" s="8" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="B80" s="10" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B81" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B82" s="9" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="B83" s="10" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B84" s="9" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="B85" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B86" s="10" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="B87" s="10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B88" s="10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B89" s="10" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B90" s="10" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="B91" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="B92" s="10" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B93" s="10" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B94" s="10" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="B95" s="10" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="B96" s="10" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B97" s="10" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="B98" s="10" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added and Updated Employee Master Test Scenarios and Added Sales Invoice Test Scenarios
Added and Updated Employee Master Test Scenarios and Added Sales Invoice Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="279">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -687,6 +687,183 @@
   </si>
   <si>
     <t>ZeroValue</t>
+  </si>
+  <si>
+    <t>Sales_Invoice</t>
+  </si>
+  <si>
+    <t>Sales Invoice</t>
+  </si>
+  <si>
+    <t>SI_Type</t>
+  </si>
+  <si>
+    <t>SI - GENERAL</t>
+  </si>
+  <si>
+    <t>CustomerName</t>
+  </si>
+  <si>
+    <t>MURUGAN TRADERS</t>
+  </si>
+  <si>
+    <t>InvoicePrefix</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>Item_ID</t>
+  </si>
+  <si>
+    <t>TVSFG004</t>
+  </si>
+  <si>
+    <t>CPC_Code</t>
+  </si>
+  <si>
+    <t>InvoiceQty</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>UnitPrice</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>SalesGL_Acct</t>
+  </si>
+  <si>
+    <t>4010101001</t>
+  </si>
+  <si>
+    <t>HSNcode_SI</t>
+  </si>
+  <si>
+    <t>88363222</t>
+  </si>
+  <si>
+    <t>SI_HOD</t>
+  </si>
+  <si>
+    <t>Export_Customer_Name</t>
+  </si>
+  <si>
+    <t>FRANCE FOREIGN TRADERS</t>
+  </si>
+  <si>
+    <t>LUT_No</t>
+  </si>
+  <si>
+    <t>2321311</t>
+  </si>
+  <si>
+    <t>Domestic_RC_Customer_Name</t>
+  </si>
+  <si>
+    <t>AJK ENTERPRISES</t>
+  </si>
+  <si>
+    <t>Domestic_RC_Item_ID</t>
+  </si>
+  <si>
+    <t>RC_DOMESTIC_001</t>
+  </si>
+  <si>
+    <t>Export_RC_Customer_Name</t>
+  </si>
+  <si>
+    <t>Export_RC_Item_ID</t>
+  </si>
+  <si>
+    <t>RC_Export_001</t>
+  </si>
+  <si>
+    <t>UD_Disimilar_Domestic_Item_ID</t>
+  </si>
+  <si>
+    <t>UD_Disimilar_Domestic_002</t>
+  </si>
+  <si>
+    <t>Domestic_RC_Item_ID_Disimilar</t>
+  </si>
+  <si>
+    <t>Export_RC_Item_ID_Disimilar</t>
+  </si>
+  <si>
+    <t>Domestic_PL_Item_ID</t>
+  </si>
+  <si>
+    <t>Export_PL_Item_ID</t>
+  </si>
+  <si>
+    <t>Domestic_PL_Item_ID_Disimilar</t>
+  </si>
+  <si>
+    <t>Export_PL_Item_ID_Disimilar</t>
+  </si>
+  <si>
+    <t>Domestic_SP_Item_ID</t>
+  </si>
+  <si>
+    <t>Export_SP_Item_ID</t>
+  </si>
+  <si>
+    <t>Domestic_SP_Item_ID_Disimalar</t>
+  </si>
+  <si>
+    <t>Export_SP_Item_ID_Disimalar</t>
+  </si>
+  <si>
+    <t>Domestic_CG_Item_ID</t>
+  </si>
+  <si>
+    <t>Export_CG_Item_ID</t>
+  </si>
+  <si>
+    <t>Domestic_CG_Item_ID_Disimalar</t>
+  </si>
+  <si>
+    <t>Export_CG_Item_ID_Disimalar</t>
+  </si>
+  <si>
+    <t>EmpAddInfo_HomeType</t>
+  </si>
+  <si>
+    <t>Rent</t>
+  </si>
+  <si>
+    <t>EmpAddInfo_StayType</t>
+  </si>
+  <si>
+    <t>Hosteller</t>
+  </si>
+  <si>
+    <t>EmpAddInfo_VehicleFlag</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>EmpDependentRelation</t>
+  </si>
+  <si>
+    <t>Father</t>
+  </si>
+  <si>
+    <t>EmpDependentRelationDOB</t>
+  </si>
+  <si>
+    <t>20-05-1998</t>
+  </si>
+  <si>
+    <t>Emp_MaritalStatus</t>
+  </si>
+  <si>
+    <t>Single</t>
   </si>
 </sst>
 </file>
@@ -699,7 +876,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -723,6 +900,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -1204,139 +1387,139 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1365,6 +1548,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="51">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1686,11 +1874,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B117"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <dimension ref="A1:B155"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="27.1111111111111" style="1" customWidth="1"/>
+    <col min="1" max="1" width="30.1090909090909" customWidth="1"/>
+    <col min="2" max="2" width="27.1090909090909" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2629,6 +2817,310 @@
         <v>0</v>
       </c>
     </row>
+    <row r="118" spans="1:2">
+      <c r="A118" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="B118" s="19" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="B119" s="19" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="B120" s="19" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="B121" s="19" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B122" s="19" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="B123" s="19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" s="18" t="s">
+        <v>231</v>
+      </c>
+      <c r="B124" s="19" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="B125" s="19" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="B126" s="19" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="B127" s="19" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="B128" s="19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="B129" s="19" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="B130" s="19" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="B131" s="19" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" s="18" t="s">
+        <v>246</v>
+      </c>
+      <c r="B132" s="19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="B133" s="19" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" s="18" t="s">
+        <v>249</v>
+      </c>
+      <c r="B134" s="19" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="18" t="s">
+        <v>251</v>
+      </c>
+      <c r="B135" s="19" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="B136" s="19" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" s="18" t="s">
+        <v>254</v>
+      </c>
+      <c r="B137" s="19" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="B138" s="19" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" s="18" t="s">
+        <v>256</v>
+      </c>
+      <c r="B139" s="19" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="B140" s="19" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" s="18" t="s">
+        <v>258</v>
+      </c>
+      <c r="B141" s="19" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" s="18" t="s">
+        <v>259</v>
+      </c>
+      <c r="B142" s="19" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" s="18" t="s">
+        <v>260</v>
+      </c>
+      <c r="B143" s="19" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" s="18" t="s">
+        <v>261</v>
+      </c>
+      <c r="B144" s="19" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="B145" s="19" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" s="18" t="s">
+        <v>263</v>
+      </c>
+      <c r="B146" s="19" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" s="18" t="s">
+        <v>264</v>
+      </c>
+      <c r="B147" s="19" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" s="18" t="s">
+        <v>265</v>
+      </c>
+      <c r="B148" s="19" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" s="18" t="s">
+        <v>266</v>
+      </c>
+      <c r="B149" s="19" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="B150" s="19" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" s="20" t="s">
+        <v>269</v>
+      </c>
+      <c r="B151" s="19" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="B152" s="19" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" s="20" t="s">
+        <v>273</v>
+      </c>
+      <c r="B153" s="19" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="B154" s="19" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="B155" s="19" t="s">
+        <v>278</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Added Open Sale Order to Payment Receipt ETE Scenario
Added Open Sales Order to Payment Receipt ETE Scenario and updated Open sales order Functions
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="341">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -906,6 +906,150 @@
   </si>
   <si>
     <t>7151922222222265</t>
+  </si>
+  <si>
+    <t>OpenSOItem</t>
+  </si>
+  <si>
+    <t>GWL_OpenSO_Item</t>
+  </si>
+  <si>
+    <t>ERPPrivateLimitedID</t>
+  </si>
+  <si>
+    <t>CUS0000056</t>
+  </si>
+  <si>
+    <t>ERPPrivateLimitedName</t>
+  </si>
+  <si>
+    <t>ERP PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Prefix_OP100</t>
+  </si>
+  <si>
+    <t>OP100</t>
+  </si>
+  <si>
+    <t>Type_Standard</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>HSN2022-5%</t>
+  </si>
+  <si>
+    <t>(2022)5%</t>
+  </si>
+  <si>
+    <t>Sales_Order</t>
+  </si>
+  <si>
+    <t>Sales Order</t>
+  </si>
+  <si>
+    <t>SO_General</t>
+  </si>
+  <si>
+    <t>SO - GENERAL</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>CUS0015</t>
+  </si>
+  <si>
+    <t>SO_Similar_Item</t>
+  </si>
+  <si>
+    <t>HK-FIFO-LOT-BATCH-10001(FG)</t>
+  </si>
+  <si>
+    <t>SO_Qty</t>
+  </si>
+  <si>
+    <t>SO_UnitCost</t>
+  </si>
+  <si>
+    <t>2800</t>
+  </si>
+  <si>
+    <t>SO_HSNCode</t>
+  </si>
+  <si>
+    <t>772213</t>
+  </si>
+  <si>
+    <t>SO_HOD_Value</t>
+  </si>
+  <si>
+    <t>SO_PriceBasis</t>
+  </si>
+  <si>
+    <t>User Defined</t>
+  </si>
+  <si>
+    <t>SO_Export_Customer</t>
+  </si>
+  <si>
+    <t>SO_DisSimilarItem</t>
+  </si>
+  <si>
+    <t>HK-FG-DISSIMILAR-10001</t>
+  </si>
+  <si>
+    <t>SO_Similar_Item_Rate_Contract</t>
+  </si>
+  <si>
+    <t>HK-LOT-MAC-10001(FG)</t>
+  </si>
+  <si>
+    <t>SO_Similar_Item_PriceList</t>
+  </si>
+  <si>
+    <t>HK-LOT-FIFO-LOT-10001(FG)</t>
+  </si>
+  <si>
+    <t>SO_Similar_Item_Catalog</t>
+  </si>
+  <si>
+    <t>HK-FIFO-SER-BATCH-10001(FG)</t>
+  </si>
+  <si>
+    <t>SO_Similar_Item_StandardPrice</t>
+  </si>
+  <si>
+    <t>HK-SER-MAC-10001(FG)</t>
+  </si>
+  <si>
+    <t>SO_DisSimilar_Item_Rate_Contract</t>
+  </si>
+  <si>
+    <t>HK-FG-RC-DISSIMILAR ITEM-10001</t>
+  </si>
+  <si>
+    <t>FinishedGoodWH</t>
+  </si>
+  <si>
+    <t>FINISHED GOODS WH U100</t>
+  </si>
+  <si>
+    <t>SinglePaymentType</t>
+  </si>
+  <si>
+    <t>BankReceipt_BankType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank </t>
+  </si>
+  <si>
+    <t>NEFTText</t>
+  </si>
+  <si>
+    <t>NEFT</t>
   </si>
 </sst>
 </file>
@@ -918,7 +1062,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -954,17 +1098,6 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
@@ -1446,139 +1579,139 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1616,13 +1749,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1946,11 +2080,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B162"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <dimension ref="A1:B188"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="30.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="27.1111111111111" style="1" customWidth="1"/>
+    <col min="1" max="1" width="30.1090909090909" customWidth="1"/>
+    <col min="2" max="2" width="27.1090909090909" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3210,7 +3344,7 @@
       </c>
     </row>
     <row r="158" spans="1:2">
-      <c r="A158" s="4" t="s">
+      <c r="A158" s="9" t="s">
         <v>283</v>
       </c>
       <c r="B158" s="23" t="s">
@@ -3218,35 +3352,243 @@
       </c>
     </row>
     <row r="159" spans="1:2">
-      <c r="A159" s="4" t="s">
+      <c r="A159" s="9" t="s">
         <v>285</v>
       </c>
-      <c r="B159" s="5" t="s">
+      <c r="B159" s="24" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="160" spans="1:2">
-      <c r="A160" s="24" t="s">
+      <c r="A160" s="9" t="s">
         <v>287</v>
       </c>
-      <c r="B160" s="25" t="s">
+      <c r="B160" s="9" t="s">
         <v>288</v>
       </c>
     </row>
     <row r="161" spans="1:2">
-      <c r="A161" s="26" t="s">
+      <c r="A161" s="9" t="s">
         <v>289</v>
       </c>
-      <c r="B161" s="27" t="s">
+      <c r="B161" s="24" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="162" spans="1:2">
-      <c r="A162" s="26" t="s">
+      <c r="A162" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="B162" s="27" t="s">
+      <c r="B162" s="24" t="s">
         <v>292</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="25" t="s">
+        <v>293</v>
+      </c>
+      <c r="B163" s="25" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="25" t="s">
+        <v>295</v>
+      </c>
+      <c r="B164" s="25" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="25" t="s">
+        <v>297</v>
+      </c>
+      <c r="B165" s="26" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="25" t="s">
+        <v>299</v>
+      </c>
+      <c r="B166" s="26" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="B167" s="25" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" s="25" t="s">
+        <v>303</v>
+      </c>
+      <c r="B168" s="25" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" s="25" t="s">
+        <v>305</v>
+      </c>
+      <c r="B169" s="26" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" s="25" t="s">
+        <v>307</v>
+      </c>
+      <c r="B170" s="26" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="B171" s="26" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="B172" s="26" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" s="25" t="s">
+        <v>313</v>
+      </c>
+      <c r="B173" s="26" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" s="25" t="s">
+        <v>314</v>
+      </c>
+      <c r="B174" s="26" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" s="25" t="s">
+        <v>316</v>
+      </c>
+      <c r="B175" s="26" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="B176" s="26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" s="25" t="s">
+        <v>319</v>
+      </c>
+      <c r="B177" s="26" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" s="25" t="s">
+        <v>321</v>
+      </c>
+      <c r="B178" s="26" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" s="25" t="s">
+        <v>322</v>
+      </c>
+      <c r="B179" s="26" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" s="25" t="s">
+        <v>324</v>
+      </c>
+      <c r="B180" s="26" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" s="25" t="s">
+        <v>326</v>
+      </c>
+      <c r="B181" s="26" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" s="25" t="s">
+        <v>328</v>
+      </c>
+      <c r="B182" s="26" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" s="25" t="s">
+        <v>330</v>
+      </c>
+      <c r="B183" s="26" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" s="25" t="s">
+        <v>332</v>
+      </c>
+      <c r="B184" s="26" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" s="25" t="s">
+        <v>334</v>
+      </c>
+      <c r="B185" s="25" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="B186" s="25" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" s="25" t="s">
+        <v>337</v>
+      </c>
+      <c r="B187" s="26" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="B188" s="25" t="s">
+        <v>340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated and Fixed OpenSO to Receipt E2E Test Scenario
Updated and Fixed OpenSO to Receipt E2E Test Scenario
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="343">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -1050,6 +1050,12 @@
   </si>
   <si>
     <t>NEFT</t>
+  </si>
+  <si>
+    <t>InvoicedStatus</t>
+  </si>
+  <si>
+    <t>Invoiced</t>
   </si>
 </sst>
 </file>
@@ -2080,7 +2086,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B188"/>
+  <dimension ref="A1:B189"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="30.1090909090909" customWidth="1"/>
@@ -3384,211 +3390,219 @@
       </c>
     </row>
     <row r="163" spans="1:2">
-      <c r="A163" s="25" t="s">
+      <c r="A163" s="9" t="s">
         <v>293</v>
       </c>
-      <c r="B163" s="25" t="s">
+      <c r="B163" s="9" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="164" spans="1:2">
-      <c r="A164" s="25" t="s">
+      <c r="A164" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="B164" s="25" t="s">
+      <c r="B164" s="9" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="165" spans="1:2">
-      <c r="A165" s="25" t="s">
+      <c r="A165" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="B165" s="26" t="s">
+      <c r="B165" s="24" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="166" spans="1:2">
-      <c r="A166" s="25" t="s">
+      <c r="A166" s="9" t="s">
         <v>299</v>
       </c>
-      <c r="B166" s="26" t="s">
+      <c r="B166" s="24" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="167" spans="1:2">
-      <c r="A167" s="25" t="s">
+      <c r="A167" s="9" t="s">
         <v>301</v>
       </c>
-      <c r="B167" s="25" t="s">
+      <c r="B167" s="9" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="168" spans="1:2">
-      <c r="A168" s="25" t="s">
+      <c r="A168" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="B168" s="25" t="s">
+      <c r="B168" s="9" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="169" spans="1:2">
-      <c r="A169" s="25" t="s">
+      <c r="A169" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="B169" s="26" t="s">
+      <c r="B169" s="24" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="170" spans="1:2">
-      <c r="A170" s="25" t="s">
+      <c r="A170" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="B170" s="26" t="s">
+      <c r="B170" s="24" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="171" spans="1:2">
-      <c r="A171" s="25" t="s">
+      <c r="A171" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="B171" s="26" t="s">
+      <c r="B171" s="24" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="172" spans="1:2">
-      <c r="A172" s="25" t="s">
+      <c r="A172" s="9" t="s">
         <v>311</v>
       </c>
-      <c r="B172" s="26" t="s">
+      <c r="B172" s="24" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="173" spans="1:2">
-      <c r="A173" s="25" t="s">
+      <c r="A173" s="9" t="s">
         <v>313</v>
       </c>
-      <c r="B173" s="26" t="s">
+      <c r="B173" s="24" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="174" spans="1:2">
-      <c r="A174" s="25" t="s">
+      <c r="A174" s="9" t="s">
         <v>314</v>
       </c>
-      <c r="B174" s="26" t="s">
+      <c r="B174" s="24" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="175" spans="1:2">
-      <c r="A175" s="25" t="s">
+      <c r="A175" s="9" t="s">
         <v>316</v>
       </c>
-      <c r="B175" s="26" t="s">
+      <c r="B175" s="24" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="176" spans="1:2">
-      <c r="A176" s="25" t="s">
+      <c r="A176" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="B176" s="26" t="s">
+      <c r="B176" s="24" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="177" spans="1:2">
-      <c r="A177" s="25" t="s">
+      <c r="A177" s="9" t="s">
         <v>319</v>
       </c>
-      <c r="B177" s="26" t="s">
+      <c r="B177" s="24" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="178" spans="1:2">
-      <c r="A178" s="25" t="s">
+      <c r="A178" s="9" t="s">
         <v>321</v>
       </c>
-      <c r="B178" s="26" t="s">
+      <c r="B178" s="24" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="179" spans="1:2">
-      <c r="A179" s="25" t="s">
+      <c r="A179" s="9" t="s">
         <v>322</v>
       </c>
-      <c r="B179" s="26" t="s">
+      <c r="B179" s="24" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="180" spans="1:2">
-      <c r="A180" s="25" t="s">
+      <c r="A180" s="9" t="s">
         <v>324</v>
       </c>
-      <c r="B180" s="26" t="s">
+      <c r="B180" s="24" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="181" spans="1:2">
-      <c r="A181" s="25" t="s">
+      <c r="A181" s="9" t="s">
         <v>326</v>
       </c>
-      <c r="B181" s="26" t="s">
+      <c r="B181" s="24" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="182" spans="1:2">
-      <c r="A182" s="25" t="s">
+      <c r="A182" s="9" t="s">
         <v>328</v>
       </c>
-      <c r="B182" s="26" t="s">
+      <c r="B182" s="24" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="183" spans="1:2">
-      <c r="A183" s="25" t="s">
+      <c r="A183" s="9" t="s">
         <v>330</v>
       </c>
-      <c r="B183" s="26" t="s">
+      <c r="B183" s="24" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="184" spans="1:2">
-      <c r="A184" s="25" t="s">
+      <c r="A184" s="9" t="s">
         <v>332</v>
       </c>
-      <c r="B184" s="26" t="s">
+      <c r="B184" s="24" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="185" spans="1:2">
-      <c r="A185" s="25" t="s">
+      <c r="A185" s="9" t="s">
         <v>334</v>
       </c>
-      <c r="B185" s="25" t="s">
+      <c r="B185" s="9" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="186" spans="1:2">
-      <c r="A186" s="25" t="s">
+      <c r="A186" s="9" t="s">
         <v>336</v>
       </c>
-      <c r="B186" s="25" t="s">
+      <c r="B186" s="9" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="187" spans="1:2">
-      <c r="A187" s="25" t="s">
+      <c r="A187" s="9" t="s">
         <v>337</v>
       </c>
-      <c r="B187" s="26" t="s">
+      <c r="B187" s="24" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="188" spans="1:2">
-      <c r="A188" s="25" t="s">
+      <c r="A188" s="9" t="s">
         <v>339</v>
       </c>
-      <c r="B188" s="25" t="s">
+      <c r="B188" s="9" t="s">
         <v>340</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="25" t="s">
+        <v>341</v>
+      </c>
+      <c r="B189" s="26" t="s">
+        <v>342</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Core Process Test And Added DB Connection Validation For PR Headers
Fixed Core Process Test And Added DB Connection Validation For PR Headers
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15030" windowHeight="6540"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
+    <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="507">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -1441,13 +1441,263 @@
   </si>
   <si>
     <t>Document is cancelled.</t>
+  </si>
+  <si>
+    <t>TDSValue</t>
+  </si>
+  <si>
+    <t>194C</t>
+  </si>
+  <si>
+    <t>PRNO</t>
+  </si>
+  <si>
+    <t>${PRNO}</t>
+  </si>
+  <si>
+    <t>ExptPRNo</t>
+  </si>
+  <si>
+    <t>PR12122-00013</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>ExpectedPcrNo</t>
+  </si>
+  <si>
+    <t>PCRQ-2425-00002</t>
+  </si>
+  <si>
+    <t>UnitValue</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>LocationValue</t>
+  </si>
+  <si>
+    <t>PRH_PLNT_LOC_ID</t>
+  </si>
+  <si>
+    <t>SourceValue</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>PrhValue</t>
+  </si>
+  <si>
+    <t>PRH_RQST_PFX</t>
+  </si>
+  <si>
+    <t>CCCode</t>
+  </si>
+  <si>
+    <t>PRH_CC_CODE</t>
+  </si>
+  <si>
+    <t>DeptValue</t>
+  </si>
+  <si>
+    <t>dept_desc</t>
+  </si>
+  <si>
+    <t>RequestorValue</t>
+  </si>
+  <si>
+    <t>Requestor</t>
+  </si>
+  <si>
+    <t>FG-10001-Item</t>
+  </si>
+  <si>
+    <t>HK-TVS-FG-10001</t>
+  </si>
+  <si>
+    <t>RM-10001-Item</t>
+  </si>
+  <si>
+    <t>HK-TVS-RM-10001</t>
+  </si>
+  <si>
+    <t>ReleasedStatus</t>
+  </si>
+  <si>
+    <t>Released</t>
+  </si>
+  <si>
+    <t>UnreleasedStatus</t>
+  </si>
+  <si>
+    <t>Unreleased</t>
+  </si>
+  <si>
+    <t>PRHeaderQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SELECT prh_plant "Unit",
+       (SELECT bup_name1
+          FROM bus_unit_plants
+         WHERE bup_bu = prh_bu AND bup_plant_id = prh_plant)
+          UNIT,
+       prh_rqst_pfx,
+       PRH_RQST_DEPT_ID,
+       (SELECT NVL (dept_name1, dept_name2)
+          FROM departments
+         WHERE dept_bu = prh_bu AND dept_id = PRH_RQST_DEPT_ID)
+          "dept_desc",
+       prh_rqst_no "Pfx.No.",
+       prh_rqst_date,
+       prh_reqstr_name "Requestor",
+       prh_narration "Narration",
+       prh_status,
+       DECODE (prh_status,
+               'A', 'Approved',
+               'E', 'Draft',
+               'C', 'Cancelled',
+               'R', 'Entry Completed',
+               'L', 'Closeshorted',
+               'R', 'RECEIVED',
+               'P', 'PARTIAL')
+          STATUS,
+       (SELECT DISTINCT apst_sub_type_desc
+          FROM appl_vou_sub_types
+         WHERE     apst_bu = prh_bu
+               AND apst_vou_type = 'PR'
+               AND apst_sub_type = prh_rec_source)
+          "Source",
+       prh_narration "Reference",
+       prh_plnt_loc_id,
+       prh_cc_code,
+       (SELECT pcc_desc
+          FROM profit_cost_centers
+         WHERE     pcc_bu = prh_bu
+               AND pcc_ac_plnt = prh_plant
+               AND pcc_cc_code = prh_cc_code)
+          "CPC Code Desc."
+  FROM pur_req_hd
+  WHERE PRH_RQST_NO ='${PRNO}'
+</t>
+  </si>
+  <si>
+    <t>PRLineQuery</t>
+  </si>
+  <si>
+    <t>SELECT PRH_RQST_NO,
+       prl_prod_id "Item",
+       prl_prod_desc1 "Item Desc.",
+       prl_prod_rev "Rev.",
+       prod_ext_desc1,
+       prl_uom "UOM",
+       prl_class_desc "Item Class",
+       prl_sub_cls_desc "Item SubClass",
+       prl_conv_factor "Conv. Factor",
+       prl_store_name "WH/Dept.",
+       prl_so_schld_desc "SO/Prj. Ref.",
+       prl_required_date prls_required_date,
+       CASE
+          WHEN prl_status = 'E' THEN 'Draft'
+          WHEN prl_status = 'N' THEN 'Entry Completed'
+          WHEN prl_status = 'A' THEN 'Approved'
+          WHEN prl_status = 'C' THEN 'Cancelled'
+          WHEN prl_status = 'L' THEN 'Closeshort'
+       END
+          prl_status,
+       DECODE (prl_status,
+               'A', 'Approved',
+               'E', 'Draft',
+               'C', 'Cancelled',
+               'R', 'Entry Completed',
+               'L', 'Closeshorted',
+               'R', 'RECEIVED',
+               'P', 'PARTIAL')
+          ln_STATUS,
+       prl_pur_acct,
+       prl_cc_code,
+       (SELECT glac_acct_desc1
+          FROM gl_accts
+         WHERE glac_bu = prl_bu AND glac_acct = prl_pur_acct)
+          "GL Acct. Desc.",
+       (SELECT pcc_desc
+          FROM profit_cost_centers
+         WHERE     pcc_bu = prl_bu
+               AND pcc_ac_plnt = prl_plnt
+               AND pcc_cc_code = prl_cc_code)
+          "CPC Code Desc.",
+       (SELECT DISTINCT DECODE (
+                  applctrl_desc_level,
+                  1,    emp_first_name1
+                     || ' '
+                     || emp_middle_name1
+                     || ' '
+                     || emp_last_name1,
+                  NVL (
+                        emp_first_name2
+                     || ' '
+                     || emp_middle_name2
+                     || ' '
+                     || emp_last_name2,
+                        emp_first_name1
+                     || ' '
+                     || emp_middle_name1
+                     || ' '
+                     || emp_last_name1))
+                  AS buyer_desc
+          FROM buyers,
+               employees,
+               appl_control,
+               emp_active_infos
+         WHERE     buyer_bu = emp_bu
+               AND buyer_emp_id = emp_emp_id
+               AND buyer_bu = applctrl_bu
+               AND emp_bu = empai_bu
+               AND emp_emp_id = empai_emp_id
+               AND buyer_bu = prl_bu
+               AND buyer_id = prl_buyer_id)
+          buyer,
+          prh_mrp_no,
+          PRL_SUGG_SUPLR_ID,
+          prl_work_ord_no,
+          PRL_SERV_PROD_ID,
+          PRL_SERV_PROD_DESC "Serv. Item desc",
+          prl_amc_start_date,
+          prl_amc_end_date,
+          PRL_MRP_REL_QTY,
+          (SELECT NVL(suplr_name1,suplr_name2)
+             FROM suppliers
+            WHERE suplr_bu = prl_bu
+            AND suplr_suplr_id = PRL_SUGG_SUPLR_ID) "Supplr. desc",
+       DECODE(prl_qc_required,'Y','Free Pass','N','Always')prl_qc_required
+  FROM pur_req_hd,
+       pur_req_ln,
+       products
+ WHERE  prh_bu ='TVSA'
+   AND PRH_RQST_NO ='${PRNO}'
+       AND prh_bu = prl_bu
+       AND prh_rqst_no = prl_rqst_no
+       AND prl_bu = prod_bu
+       AND prl_prod_id = prod_id
+       AND prl_prod_rev = prod_rev</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1493,14 +1743,156 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Consolas"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1509,12 +1901,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1550,24 +2128,272 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1578,12 +2404,12 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1601,25 +2427,74 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="51">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
-    <cellStyle name="Normal 3" xfId="2"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal 2" xfId="49"/>
+    <cellStyle name="Normal 3" xfId="50"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1881,1997 +2756,1997 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B278"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B294"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="59.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="34.287037037037" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="7" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="7" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="7">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="7">
         <v>150</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="7" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="7" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="7" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="7" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="7" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="7" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="7" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="7" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="7" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="7" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="7" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="7" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="7" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:2">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="7" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="7" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="7" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="7" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="7" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="7" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="7" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="7" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B48" s="7" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B49" s="5">
+      <c r="B49" s="7">
         <v>5</v>
       </c>
     </row>
     <row r="50" spans="1:2">
-      <c r="A50" s="4" t="s">
+      <c r="A50" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:2">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B51" s="7" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="52" spans="1:2">
-      <c r="A52" s="4" t="s">
+      <c r="A52" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="53" spans="1:2">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B53" s="7" t="s">
+      <c r="B53" s="9" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="54" spans="1:2">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="B54" s="9" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="55" spans="1:2">
-      <c r="A55" s="6" t="s">
+      <c r="A55" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="B55" s="9" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="56" spans="1:2">
-      <c r="A56" s="6" t="s">
+      <c r="A56" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B56" s="7" t="s">
+      <c r="B56" s="9" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="57" spans="1:2">
-      <c r="A57" s="6" t="s">
+      <c r="A57" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B57" s="9" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="58" spans="1:2">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B58" s="7" t="s">
+      <c r="B58" s="9" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="59" spans="1:2">
-      <c r="A59" s="6" t="s">
+      <c r="A59" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B59" s="7" t="s">
+      <c r="B59" s="9" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="60" spans="1:2">
-      <c r="A60" s="6" t="s">
+      <c r="A60" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B60" s="7" t="s">
+      <c r="B60" s="9" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="61" spans="1:2">
-      <c r="A61" s="6" t="s">
+      <c r="A61" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="9" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="62" spans="1:2">
-      <c r="A62" s="6" t="s">
+      <c r="A62" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B62" s="7" t="s">
+      <c r="B62" s="9" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="63" spans="1:2">
-      <c r="A63" s="6" t="s">
+      <c r="A63" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B63" s="7" t="s">
+      <c r="B63" s="9" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="64" spans="1:2">
-      <c r="A64" s="6" t="s">
+      <c r="A64" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="B64" s="7" t="s">
+      <c r="B64" s="9" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="65" spans="1:2">
-      <c r="A65" s="6" t="s">
+      <c r="A65" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="B65" s="7">
+      <c r="B65" s="9">
         <v>30</v>
       </c>
     </row>
     <row r="66" spans="1:2">
-      <c r="A66" s="6" t="s">
+      <c r="A66" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B66" s="8" t="s">
+      <c r="B66" s="10" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="67" spans="1:2">
-      <c r="A67" s="6" t="s">
+      <c r="A67" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B67" s="8" t="s">
+      <c r="B67" s="10" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="68" spans="1:2">
-      <c r="A68" s="6" t="s">
+      <c r="A68" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B68" s="8" t="s">
+      <c r="B68" s="10" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="69" spans="1:2">
-      <c r="A69" s="6" t="s">
+      <c r="A69" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B69" s="8">
+      <c r="B69" s="10">
         <v>2012</v>
       </c>
     </row>
     <row r="70" spans="1:2">
-      <c r="A70" s="6" t="s">
+      <c r="A70" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="B70" s="8" t="s">
+      <c r="B70" s="10" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="71" spans="1:2">
-      <c r="A71" s="6" t="s">
+      <c r="A71" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B71" s="8" t="s">
+      <c r="B71" s="10" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="72" spans="1:2">
-      <c r="A72" s="8" t="s">
+      <c r="A72" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B72" s="8" t="s">
+      <c r="B72" s="10" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="73" spans="1:2">
-      <c r="A73" s="8" t="s">
+      <c r="A73" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B73" s="8" t="s">
+      <c r="B73" s="10" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="74" spans="1:2">
-      <c r="A74" s="8" t="s">
+      <c r="A74" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B74" s="8" t="s">
+      <c r="B74" s="10" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="75" spans="1:2">
-      <c r="A75" s="8" t="s">
+      <c r="A75" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B75" s="8" t="s">
+      <c r="B75" s="10" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="76" spans="1:2">
-      <c r="A76" s="8" t="s">
+      <c r="A76" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="B76" s="8">
+      <c r="B76" s="10">
         <v>202425</v>
       </c>
     </row>
     <row r="77" spans="1:2">
-      <c r="A77" s="8" t="s">
+      <c r="A77" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B77" s="8" t="s">
+      <c r="B77" s="10" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="78" spans="1:2">
-      <c r="A78" s="8" t="s">
+      <c r="A78" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="B78" s="8" t="s">
+      <c r="B78" s="10" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="79" spans="1:2">
-      <c r="A79" s="8" t="s">
+      <c r="A79" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="B79" s="8" t="s">
+      <c r="B79" s="10" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="80" spans="1:2">
-      <c r="A80" s="9" t="s">
+      <c r="A80" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="B80" s="10" t="s">
+      <c r="B80" s="12" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="81" spans="1:2">
-      <c r="A81" s="9" t="s">
+      <c r="A81" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="B81" s="10" t="s">
+      <c r="B81" s="12" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="82" spans="1:2">
-      <c r="A82" s="9" t="s">
+      <c r="A82" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="B82" s="9" t="s">
+      <c r="B82" s="11" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="83" spans="1:2">
-      <c r="A83" s="9" t="s">
+      <c r="A83" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="B83" s="10" t="s">
+      <c r="B83" s="12" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="84" spans="1:2">
-      <c r="A84" s="9" t="s">
+      <c r="A84" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="B84" s="9" t="s">
+      <c r="B84" s="11" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="85" spans="1:2">
-      <c r="A85" s="9" t="s">
+      <c r="A85" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="B85" s="9" t="s">
+      <c r="B85" s="11" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="86" spans="1:2">
-      <c r="A86" s="9" t="s">
+      <c r="A86" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="B86" s="10" t="s">
+      <c r="B86" s="12" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="87" spans="1:2">
-      <c r="A87" s="9" t="s">
+      <c r="A87" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="B87" s="10" t="s">
+      <c r="B87" s="12" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="88" spans="1:2">
-      <c r="A88" s="10" t="s">
+      <c r="A88" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="B88" s="10" t="s">
+      <c r="B88" s="12" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="89" spans="1:2">
-      <c r="A89" s="10" t="s">
+      <c r="A89" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="B89" s="10" t="s">
+      <c r="B89" s="12" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="90" spans="1:2">
-      <c r="A90" s="10" t="s">
+      <c r="A90" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="B90" s="10" t="s">
+      <c r="B90" s="12" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="91" spans="1:2">
-      <c r="A91" s="10" t="s">
+      <c r="A91" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="B91" s="10" t="s">
+      <c r="B91" s="12" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="92" spans="1:2">
-      <c r="A92" s="10" t="s">
+      <c r="A92" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="B92" s="10" t="s">
+      <c r="B92" s="12" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="93" spans="1:2">
-      <c r="A93" s="10" t="s">
+      <c r="A93" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="B93" s="10" t="s">
+      <c r="B93" s="12" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="94" spans="1:2">
-      <c r="A94" s="10" t="s">
+      <c r="A94" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="B94" s="10" t="s">
+      <c r="B94" s="12" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="95" spans="1:2">
-      <c r="A95" s="10" t="s">
+      <c r="A95" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="B95" s="10" t="s">
+      <c r="B95" s="12" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="96" spans="1:2">
-      <c r="A96" s="10" t="s">
+      <c r="A96" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B96" s="10" t="s">
+      <c r="B96" s="12" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="97" spans="1:2">
-      <c r="A97" s="10" t="s">
+      <c r="A97" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B97" s="10" t="s">
+      <c r="B97" s="12" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="98" spans="1:2">
-      <c r="A98" s="10" t="s">
+      <c r="A98" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B98" s="10" t="s">
+      <c r="B98" s="12" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="99" spans="1:2">
-      <c r="A99" s="11" t="s">
+      <c r="A99" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="B99" s="11" t="s">
+      <c r="B99" s="13" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="100" spans="1:2">
-      <c r="A100" s="11" t="s">
+      <c r="A100" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="B100" s="12" t="s">
+      <c r="B100" s="14" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="101" spans="1:2">
-      <c r="A101" s="11" t="s">
+      <c r="A101" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="B101" s="11" t="s">
+      <c r="B101" s="13" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="102" spans="1:2">
-      <c r="A102" s="11" t="s">
+      <c r="A102" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="B102" s="11" t="s">
+      <c r="B102" s="13" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="103" spans="1:2">
-      <c r="A103" s="11" t="s">
+      <c r="A103" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="B103" s="12">
+      <c r="B103" s="14">
         <v>1</v>
       </c>
     </row>
     <row r="104" spans="1:2">
-      <c r="A104" s="13" t="s">
+      <c r="A104" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="B104" s="13" t="s">
+      <c r="B104" s="15" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="105" spans="1:2">
-      <c r="A105" s="13" t="s">
+      <c r="A105" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="B105" s="14" t="s">
+      <c r="B105" s="16" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="106" spans="1:2">
-      <c r="A106" s="13" t="s">
+      <c r="A106" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="B106" s="15">
+      <c r="B106" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="107" spans="1:2">
-      <c r="A107" s="13" t="s">
+      <c r="A107" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="B107" s="13" t="s">
+      <c r="B107" s="15" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="108" spans="1:2">
-      <c r="A108" s="13" t="s">
+      <c r="A108" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="B108" s="16" t="s">
+      <c r="B108" s="18" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="109" spans="1:2">
-      <c r="A109" s="13" t="s">
+      <c r="A109" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="B109" s="15">
+      <c r="B109" s="17">
         <v>100</v>
       </c>
     </row>
     <row r="110" spans="1:2">
-      <c r="A110" s="4" t="s">
+      <c r="A110" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="B110" s="4" t="s">
+      <c r="B110" s="2" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="111" spans="1:2">
-      <c r="A111" s="17" t="s">
+      <c r="A111" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="B111" s="17" t="s">
+      <c r="B111" s="19" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="112" spans="1:2">
-      <c r="A112" s="17" t="s">
+      <c r="A112" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="B112" s="17" t="s">
+      <c r="B112" s="19" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="113" spans="1:2">
-      <c r="A113" s="17" t="s">
+      <c r="A113" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="B113" s="4" t="s">
+      <c r="B113" s="2" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="114" spans="1:2">
-      <c r="A114" s="17" t="s">
+      <c r="A114" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="B114" s="4" t="s">
+      <c r="B114" s="2" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="115" spans="1:2">
-      <c r="A115" s="17" t="s">
+      <c r="A115" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="B115" s="4" t="s">
+      <c r="B115" s="2" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="116" spans="1:2">
-      <c r="A116" s="4" t="s">
+      <c r="A116" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B116" s="4" t="s">
+      <c r="B116" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="117" spans="1:2">
-      <c r="A117" s="4" t="s">
+      <c r="A117" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B117" s="4">
+      <c r="B117" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:2">
-      <c r="A118" s="18" t="s">
+      <c r="A118" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="B118" s="19" t="s">
+      <c r="B118" s="21" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="119" spans="1:2">
-      <c r="A119" s="18" t="s">
+      <c r="A119" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="B119" s="19" t="s">
+      <c r="B119" s="21" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="120" spans="1:2">
-      <c r="A120" s="18" t="s">
+      <c r="A120" s="20" t="s">
         <v>224</v>
       </c>
-      <c r="B120" s="19" t="s">
+      <c r="B120" s="21" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="121" spans="1:2">
-      <c r="A121" s="18" t="s">
+      <c r="A121" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="B121" s="19" t="s">
+      <c r="B121" s="21" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="122" spans="1:2">
-      <c r="A122" s="18" t="s">
+      <c r="A122" s="20" t="s">
         <v>228</v>
       </c>
-      <c r="B122" s="19" t="s">
+      <c r="B122" s="21" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="123" spans="1:2">
-      <c r="A123" s="18" t="s">
+      <c r="A123" s="20" t="s">
         <v>230</v>
       </c>
-      <c r="B123" s="19" t="s">
+      <c r="B123" s="21" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="124" spans="1:2">
-      <c r="A124" s="18" t="s">
+      <c r="A124" s="20" t="s">
         <v>231</v>
       </c>
-      <c r="B124" s="19" t="s">
+      <c r="B124" s="21" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="125" spans="1:2">
-      <c r="A125" s="18" t="s">
+      <c r="A125" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="B125" s="19" t="s">
+      <c r="B125" s="21" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="126" spans="1:2">
-      <c r="A126" s="18" t="s">
+      <c r="A126" s="20" t="s">
         <v>235</v>
       </c>
-      <c r="B126" s="19" t="s">
+      <c r="B126" s="21" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="127" spans="1:2">
-      <c r="A127" s="18" t="s">
+      <c r="A127" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="B127" s="19" t="s">
+      <c r="B127" s="21" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="128" spans="1:2">
-      <c r="A128" s="18" t="s">
+      <c r="A128" s="20" t="s">
         <v>239</v>
       </c>
-      <c r="B128" s="19" t="s">
+      <c r="B128" s="21" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="129" spans="1:2">
-      <c r="A129" s="18" t="s">
+      <c r="A129" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="B129" s="19" t="s">
+      <c r="B129" s="21" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="130" spans="1:2">
-      <c r="A130" s="18" t="s">
+      <c r="A130" s="20" t="s">
         <v>242</v>
       </c>
-      <c r="B130" s="19" t="s">
+      <c r="B130" s="21" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="131" spans="1:2">
-      <c r="A131" s="18" t="s">
+      <c r="A131" s="20" t="s">
         <v>244</v>
       </c>
-      <c r="B131" s="19" t="s">
+      <c r="B131" s="21" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="132" spans="1:2">
-      <c r="A132" s="18" t="s">
+      <c r="A132" s="20" t="s">
         <v>246</v>
       </c>
-      <c r="B132" s="19" t="s">
+      <c r="B132" s="21" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="133" spans="1:2">
-      <c r="A133" s="18" t="s">
+      <c r="A133" s="20" t="s">
         <v>248</v>
       </c>
-      <c r="B133" s="19" t="s">
+      <c r="B133" s="21" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="134" spans="1:2">
-      <c r="A134" s="18" t="s">
+      <c r="A134" s="20" t="s">
         <v>249</v>
       </c>
-      <c r="B134" s="19" t="s">
+      <c r="B134" s="21" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="135" spans="1:2">
-      <c r="A135" s="18" t="s">
+      <c r="A135" s="20" t="s">
         <v>251</v>
       </c>
-      <c r="B135" s="19" t="s">
+      <c r="B135" s="21" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="136" spans="1:2">
-      <c r="A136" s="18" t="s">
+      <c r="A136" s="20" t="s">
         <v>253</v>
       </c>
-      <c r="B136" s="19" t="s">
+      <c r="B136" s="21" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="137" spans="1:2">
-      <c r="A137" s="18" t="s">
+      <c r="A137" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="B137" s="19" t="s">
+      <c r="B137" s="21" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="138" spans="1:2">
-      <c r="A138" s="18" t="s">
+      <c r="A138" s="20" t="s">
         <v>255</v>
       </c>
-      <c r="B138" s="19" t="s">
+      <c r="B138" s="21" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="139" spans="1:2">
-      <c r="A139" s="18" t="s">
+      <c r="A139" s="20" t="s">
         <v>256</v>
       </c>
-      <c r="B139" s="19" t="s">
+      <c r="B139" s="21" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="140" spans="1:2">
-      <c r="A140" s="18" t="s">
+      <c r="A140" s="20" t="s">
         <v>257</v>
       </c>
-      <c r="B140" s="19" t="s">
+      <c r="B140" s="21" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="141" spans="1:2">
-      <c r="A141" s="18" t="s">
+      <c r="A141" s="20" t="s">
         <v>258</v>
       </c>
-      <c r="B141" s="19" t="s">
+      <c r="B141" s="21" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="142" spans="1:2">
-      <c r="A142" s="18" t="s">
+      <c r="A142" s="20" t="s">
         <v>259</v>
       </c>
-      <c r="B142" s="19" t="s">
+      <c r="B142" s="21" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="143" spans="1:2">
-      <c r="A143" s="18" t="s">
+      <c r="A143" s="20" t="s">
         <v>260</v>
       </c>
-      <c r="B143" s="19" t="s">
+      <c r="B143" s="21" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="144" spans="1:2">
-      <c r="A144" s="18" t="s">
+      <c r="A144" s="20" t="s">
         <v>261</v>
       </c>
-      <c r="B144" s="19" t="s">
+      <c r="B144" s="21" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="145" spans="1:2">
-      <c r="A145" s="18" t="s">
+      <c r="A145" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="B145" s="19" t="s">
+      <c r="B145" s="21" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="146" spans="1:2">
-      <c r="A146" s="18" t="s">
+      <c r="A146" s="20" t="s">
         <v>263</v>
       </c>
-      <c r="B146" s="19" t="s">
+      <c r="B146" s="21" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="147" spans="1:2">
-      <c r="A147" s="18" t="s">
+      <c r="A147" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="B147" s="19" t="s">
+      <c r="B147" s="21" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="148" spans="1:2">
-      <c r="A148" s="18" t="s">
+      <c r="A148" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="B148" s="19" t="s">
+      <c r="B148" s="21" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="149" spans="1:2">
-      <c r="A149" s="18" t="s">
+      <c r="A149" s="20" t="s">
         <v>266</v>
       </c>
-      <c r="B149" s="19" t="s">
+      <c r="B149" s="21" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="150" spans="1:2">
-      <c r="A150" s="20" t="s">
+      <c r="A150" s="22" t="s">
         <v>267</v>
       </c>
-      <c r="B150" s="19" t="s">
+      <c r="B150" s="21" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="151" spans="1:2">
-      <c r="A151" s="20" t="s">
+      <c r="A151" s="22" t="s">
         <v>269</v>
       </c>
-      <c r="B151" s="19" t="s">
+      <c r="B151" s="21" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="152" spans="1:2">
-      <c r="A152" s="20" t="s">
+      <c r="A152" s="22" t="s">
         <v>271</v>
       </c>
-      <c r="B152" s="19" t="s">
+      <c r="B152" s="21" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="153" spans="1:2">
-      <c r="A153" s="20" t="s">
+      <c r="A153" s="22" t="s">
         <v>273</v>
       </c>
-      <c r="B153" s="19" t="s">
+      <c r="B153" s="21" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="154" spans="1:2">
-      <c r="A154" s="20" t="s">
+      <c r="A154" s="22" t="s">
         <v>275</v>
       </c>
-      <c r="B154" s="19" t="s">
+      <c r="B154" s="21" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="155" spans="1:2">
-      <c r="A155" s="20" t="s">
+      <c r="A155" s="22" t="s">
         <v>277</v>
       </c>
-      <c r="B155" s="19" t="s">
+      <c r="B155" s="21" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="156" spans="1:2">
-      <c r="A156" s="21" t="s">
+      <c r="A156" s="23" t="s">
         <v>279</v>
       </c>
-      <c r="B156" s="22" t="s">
+      <c r="B156" s="24" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="157" spans="1:2">
-      <c r="A157" s="4" t="s">
+      <c r="A157" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="B157" s="4" t="s">
+      <c r="B157" s="2" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="158" spans="1:2">
-      <c r="A158" s="9" t="s">
+      <c r="A158" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="B158" s="23" t="s">
+      <c r="B158" s="25" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="159" spans="1:2">
-      <c r="A159" s="9" t="s">
+      <c r="A159" s="11" t="s">
         <v>285</v>
       </c>
-      <c r="B159" s="24" t="s">
+      <c r="B159" s="26" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="160" spans="1:2">
-      <c r="A160" s="9" t="s">
+      <c r="A160" s="11" t="s">
         <v>287</v>
       </c>
-      <c r="B160" s="9" t="s">
+      <c r="B160" s="11" t="s">
         <v>288</v>
       </c>
     </row>
     <row r="161" spans="1:2">
-      <c r="A161" s="9" t="s">
+      <c r="A161" s="11" t="s">
         <v>289</v>
       </c>
-      <c r="B161" s="24" t="s">
+      <c r="B161" s="26" t="s">
         <v>290</v>
       </c>
     </row>
     <row r="162" spans="1:2">
-      <c r="A162" s="9" t="s">
+      <c r="A162" s="11" t="s">
         <v>291</v>
       </c>
-      <c r="B162" s="24" t="s">
+      <c r="B162" s="26" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="163" spans="1:2">
-      <c r="A163" s="9" t="s">
+      <c r="A163" s="11" t="s">
         <v>293</v>
       </c>
-      <c r="B163" s="9" t="s">
+      <c r="B163" s="11" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="164" spans="1:2">
-      <c r="A164" s="9" t="s">
+      <c r="A164" s="11" t="s">
         <v>295</v>
       </c>
-      <c r="B164" s="9" t="s">
+      <c r="B164" s="11" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="165" spans="1:2">
-      <c r="A165" s="9" t="s">
+      <c r="A165" s="11" t="s">
         <v>297</v>
       </c>
-      <c r="B165" s="24" t="s">
+      <c r="B165" s="26" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="166" spans="1:2">
-      <c r="A166" s="9" t="s">
+      <c r="A166" s="11" t="s">
         <v>299</v>
       </c>
-      <c r="B166" s="24" t="s">
+      <c r="B166" s="26" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="167" spans="1:2">
-      <c r="A167" s="9" t="s">
+      <c r="A167" s="11" t="s">
         <v>301</v>
       </c>
-      <c r="B167" s="9" t="s">
+      <c r="B167" s="11" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="168" spans="1:2">
-      <c r="A168" s="9" t="s">
+      <c r="A168" s="11" t="s">
         <v>303</v>
       </c>
-      <c r="B168" s="9" t="s">
+      <c r="B168" s="11" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="169" spans="1:2">
-      <c r="A169" s="9" t="s">
+      <c r="A169" s="11" t="s">
         <v>305</v>
       </c>
-      <c r="B169" s="24" t="s">
+      <c r="B169" s="26" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="170" spans="1:2">
-      <c r="A170" s="9" t="s">
+      <c r="A170" s="11" t="s">
         <v>307</v>
       </c>
-      <c r="B170" s="24" t="s">
+      <c r="B170" s="26" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="171" spans="1:2">
-      <c r="A171" s="9" t="s">
+      <c r="A171" s="11" t="s">
         <v>309</v>
       </c>
-      <c r="B171" s="24" t="s">
+      <c r="B171" s="26" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="172" spans="1:2">
-      <c r="A172" s="9" t="s">
+      <c r="A172" s="11" t="s">
         <v>311</v>
       </c>
-      <c r="B172" s="24" t="s">
+      <c r="B172" s="26" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="173" spans="1:2">
-      <c r="A173" s="9" t="s">
+      <c r="A173" s="11" t="s">
         <v>313</v>
       </c>
-      <c r="B173" s="24" t="s">
+      <c r="B173" s="26" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="174" spans="1:2">
-      <c r="A174" s="9" t="s">
+      <c r="A174" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="B174" s="24" t="s">
+      <c r="B174" s="26" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="175" spans="1:2">
-      <c r="A175" s="9" t="s">
+      <c r="A175" s="11" t="s">
         <v>316</v>
       </c>
-      <c r="B175" s="24" t="s">
+      <c r="B175" s="26" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="176" spans="1:2">
-      <c r="A176" s="9" t="s">
+      <c r="A176" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="B176" s="24" t="s">
+      <c r="B176" s="26" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="177" spans="1:2">
-      <c r="A177" s="9" t="s">
+      <c r="A177" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="B177" s="24" t="s">
+      <c r="B177" s="26" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="178" spans="1:2">
-      <c r="A178" s="9" t="s">
+      <c r="A178" s="11" t="s">
         <v>321</v>
       </c>
-      <c r="B178" s="24" t="s">
+      <c r="B178" s="26" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="179" spans="1:2">
-      <c r="A179" s="9" t="s">
+      <c r="A179" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="B179" s="24" t="s">
+      <c r="B179" s="26" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="180" spans="1:2">
-      <c r="A180" s="9" t="s">
+      <c r="A180" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="B180" s="24" t="s">
+      <c r="B180" s="26" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="181" spans="1:2">
-      <c r="A181" s="9" t="s">
+      <c r="A181" s="11" t="s">
         <v>326</v>
       </c>
-      <c r="B181" s="24" t="s">
+      <c r="B181" s="26" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="182" spans="1:2">
-      <c r="A182" s="9" t="s">
+      <c r="A182" s="11" t="s">
         <v>328</v>
       </c>
-      <c r="B182" s="24" t="s">
+      <c r="B182" s="26" t="s">
         <v>329</v>
       </c>
     </row>
     <row r="183" spans="1:2">
-      <c r="A183" s="9" t="s">
+      <c r="A183" s="11" t="s">
         <v>330</v>
       </c>
-      <c r="B183" s="24" t="s">
+      <c r="B183" s="26" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="184" spans="1:2">
-      <c r="A184" s="9" t="s">
+      <c r="A184" s="11" t="s">
         <v>332</v>
       </c>
-      <c r="B184" s="24" t="s">
+      <c r="B184" s="26" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="185" spans="1:2">
-      <c r="A185" s="9" t="s">
+      <c r="A185" s="11" t="s">
         <v>334</v>
       </c>
-      <c r="B185" s="9" t="s">
+      <c r="B185" s="11" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="186" spans="1:2">
-      <c r="A186" s="9" t="s">
+      <c r="A186" s="11" t="s">
         <v>336</v>
       </c>
-      <c r="B186" s="9" t="s">
+      <c r="B186" s="11" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="187" spans="1:2">
-      <c r="A187" s="9" t="s">
+      <c r="A187" s="11" t="s">
         <v>337</v>
       </c>
-      <c r="B187" s="24" t="s">
+      <c r="B187" s="26" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="188" spans="1:2">
-      <c r="A188" s="9" t="s">
+      <c r="A188" s="11" t="s">
         <v>339</v>
       </c>
-      <c r="B188" s="9" t="s">
+      <c r="B188" s="11" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="189" spans="1:2">
-      <c r="A189" s="9" t="s">
+      <c r="A189" s="11" t="s">
         <v>341</v>
       </c>
-      <c r="B189" s="24" t="s">
+      <c r="B189" s="26" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="190" spans="1:2">
-      <c r="A190" s="4" t="s">
+      <c r="A190" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="B190" s="25" t="s">
+      <c r="B190" s="27" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="191" spans="1:2">
-      <c r="A191" s="26" t="s">
+      <c r="A191" s="28" t="s">
         <v>196</v>
       </c>
-      <c r="B191" s="26" t="s">
+      <c r="B191" s="28" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="192" spans="1:2">
-      <c r="A192" s="26" t="s">
+      <c r="A192" s="28" t="s">
         <v>198</v>
       </c>
-      <c r="B192" s="27" t="s">
+      <c r="B192" s="29" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="193" spans="1:2">
-      <c r="A193" s="26" t="s">
+      <c r="A193" s="28" t="s">
         <v>200</v>
       </c>
-      <c r="B193" s="12">
+      <c r="B193" s="14">
         <v>2</v>
       </c>
     </row>
     <row r="194" spans="1:2">
-      <c r="A194" s="26" t="s">
+      <c r="A194" s="28" t="s">
         <v>201</v>
       </c>
-      <c r="B194" s="26" t="s">
+      <c r="B194" s="28" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="195" spans="1:2">
-      <c r="A195" s="26" t="s">
+      <c r="A195" s="28" t="s">
         <v>203</v>
       </c>
-      <c r="B195" s="11" t="s">
+      <c r="B195" s="13" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="196" spans="1:2">
-      <c r="A196" s="26" t="s">
+      <c r="A196" s="28" t="s">
         <v>205</v>
       </c>
-      <c r="B196" s="12">
+      <c r="B196" s="14">
         <v>100</v>
       </c>
     </row>
     <row r="197" spans="1:2">
-      <c r="A197" s="26" t="s">
+      <c r="A197" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="B197" s="12" t="s">
+      <c r="B197" s="14" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="198" spans="1:2">
-      <c r="A198" s="26" t="s">
+      <c r="A198" s="28" t="s">
         <v>347</v>
       </c>
-      <c r="B198" s="28" t="s">
+      <c r="B198" s="30" t="s">
         <v>348</v>
       </c>
     </row>
     <row r="199" spans="1:2">
-      <c r="A199" s="26" t="s">
+      <c r="A199" s="28" t="s">
         <v>349</v>
       </c>
-      <c r="B199" s="28" t="s">
+      <c r="B199" s="30" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="200" spans="1:2">
-      <c r="A200" s="26" t="s">
+      <c r="A200" s="28" t="s">
         <v>351</v>
       </c>
-      <c r="B200" s="28" t="s">
+      <c r="B200" s="30" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="201" spans="1:2">
-      <c r="A201" s="26" t="s">
+      <c r="A201" s="28" t="s">
         <v>353</v>
       </c>
-      <c r="B201" s="12">
+      <c r="B201" s="14">
         <v>200</v>
       </c>
     </row>
     <row r="202" spans="1:2">
-      <c r="A202" s="26" t="s">
+      <c r="A202" s="28" t="s">
         <v>354</v>
       </c>
-      <c r="B202" s="12">
+      <c r="B202" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="203" spans="1:2">
-      <c r="A203" s="26" t="s">
+      <c r="A203" s="28" t="s">
         <v>355</v>
       </c>
-      <c r="B203" s="12" t="s">
+      <c r="B203" s="14" t="s">
         <v>356</v>
       </c>
     </row>
     <row r="204" spans="1:2">
-      <c r="A204" s="12" t="s">
+      <c r="A204" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="B204" s="12">
+      <c r="B204" s="14">
         <v>150</v>
       </c>
     </row>
     <row r="205" spans="1:2">
-      <c r="A205" s="12" t="s">
+      <c r="A205" s="14" t="s">
         <v>358</v>
       </c>
-      <c r="B205" s="12">
+      <c r="B205" s="14">
         <v>250</v>
       </c>
     </row>
     <row r="206" spans="1:2">
-      <c r="A206" s="12" t="s">
+      <c r="A206" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="B206" s="12" t="s">
+      <c r="B206" s="14" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="207" spans="1:2">
-      <c r="A207" s="12" t="s">
+      <c r="A207" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="B207" s="12">
+      <c r="B207" s="14">
         <v>123562</v>
       </c>
     </row>
     <row r="208" spans="1:2">
-      <c r="A208" s="12" t="s">
+      <c r="A208" s="14" t="s">
         <v>362</v>
       </c>
-      <c r="B208" s="12">
+      <c r="B208" s="14">
         <v>2</v>
       </c>
     </row>
     <row r="209" spans="1:2">
-      <c r="A209" s="12" t="s">
+      <c r="A209" s="14" t="s">
         <v>363</v>
       </c>
-      <c r="B209" s="12">
+      <c r="B209" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="210" spans="1:2">
-      <c r="A210" s="12" t="s">
+      <c r="A210" s="14" t="s">
         <v>364</v>
       </c>
-      <c r="B210" s="12">
+      <c r="B210" s="14">
         <v>4</v>
       </c>
     </row>
     <row r="211" spans="1:2">
-      <c r="A211" s="12" t="s">
+      <c r="A211" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="B211" s="27" t="s">
+      <c r="B211" s="29" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="212" spans="1:2">
-      <c r="A212" s="12" t="s">
+      <c r="A212" s="14" t="s">
         <v>367</v>
       </c>
-      <c r="B212" s="11" t="s">
+      <c r="B212" s="13" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="213" spans="1:2">
-      <c r="A213" s="12" t="s">
+      <c r="A213" s="14" t="s">
         <v>369</v>
       </c>
-      <c r="B213" s="27" t="s">
+      <c r="B213" s="29" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="214" spans="1:2">
-      <c r="A214" s="12" t="s">
+      <c r="A214" s="14" t="s">
         <v>371</v>
       </c>
-      <c r="B214" s="12">
+      <c r="B214" s="14">
         <v>50</v>
       </c>
     </row>
     <row r="215" spans="1:2">
-      <c r="A215" s="12" t="s">
+      <c r="A215" s="14" t="s">
         <v>372</v>
       </c>
-      <c r="B215" s="12">
+      <c r="B215" s="14">
         <v>50</v>
       </c>
     </row>
     <row r="216" spans="1:2">
-      <c r="A216" s="12" t="s">
+      <c r="A216" s="14" t="s">
         <v>373</v>
       </c>
-      <c r="B216" s="27" t="s">
+      <c r="B216" s="29" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="217" spans="1:2">
-      <c r="A217" s="4" t="s">
+      <c r="A217" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="B217" s="4" t="s">
+      <c r="B217" s="2" t="s">
         <v>282</v>
       </c>
     </row>
     <row r="218" spans="1:2">
-      <c r="A218" s="21" t="s">
+      <c r="A218" s="23" t="s">
         <v>374</v>
       </c>
-      <c r="B218" s="21" t="s">
+      <c r="B218" s="23" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="219" spans="1:2">
-      <c r="A219" s="21" t="s">
+      <c r="A219" s="23" t="s">
         <v>375</v>
       </c>
-      <c r="B219" s="4" t="s">
+      <c r="B219" s="2" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="220" spans="1:2">
-      <c r="A220" s="21" t="s">
+      <c r="A220" s="23" t="s">
         <v>377</v>
       </c>
-      <c r="B220" s="4" t="s">
+      <c r="B220" s="2" t="s">
         <v>378</v>
       </c>
     </row>
     <row r="221" spans="1:2">
-      <c r="A221" s="29" t="s">
+      <c r="A221" s="31" t="s">
         <v>379</v>
       </c>
-      <c r="B221" s="21" t="s">
+      <c r="B221" s="23" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="222" spans="1:2">
-      <c r="A222" s="29" t="s">
+      <c r="A222" s="31" t="s">
         <v>381</v>
       </c>
-      <c r="B222" s="21" t="s">
+      <c r="B222" s="23" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="223" spans="1:2">
-      <c r="A223" s="30" t="s">
+      <c r="A223" s="32" t="s">
         <v>383</v>
       </c>
-      <c r="B223" s="30" t="s">
+      <c r="B223" s="32" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="224" spans="1:2">
-      <c r="A224" s="29" t="s">
+      <c r="A224" s="31" t="s">
         <v>385</v>
       </c>
-      <c r="B224" s="29" t="s">
+      <c r="B224" s="31" t="s">
         <v>386</v>
       </c>
     </row>
     <row r="225" spans="1:2">
-      <c r="A225" s="4" t="s">
+      <c r="A225" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="B225" s="5" t="s">
+      <c r="B225" s="7" t="s">
         <v>388</v>
       </c>
     </row>
     <row r="226" spans="1:2">
-      <c r="A226" s="4" t="s">
+      <c r="A226" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="B226" s="5" t="s">
+      <c r="B226" s="7" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="227" spans="1:2">
-      <c r="A227" s="4" t="s">
+      <c r="A227" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="B227" s="5" t="s">
+      <c r="B227" s="7" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="228" spans="1:2">
-      <c r="A228" s="4" t="s">
+      <c r="A228" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="B228" s="5" t="s">
+      <c r="B228" s="7" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="229" spans="1:2">
-      <c r="A229" s="4" t="s">
+      <c r="A229" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="B229" s="5" t="s">
+      <c r="B229" s="7" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="230" spans="1:2">
-      <c r="A230" s="31" t="s">
+      <c r="A230" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B230" s="32" t="s">
+      <c r="B230" s="7" t="s">
         <v>395</v>
       </c>
     </row>
     <row r="231" spans="1:2">
-      <c r="A231" s="31" t="s">
+      <c r="A231" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B231" s="32" t="s">
+      <c r="B231" s="7" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="232" spans="1:2">
-      <c r="A232" s="31" t="s">
+      <c r="A232" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B232" s="32" t="s">
+      <c r="B232" s="7" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="233" spans="1:2">
-      <c r="A233" s="31" t="s">
+      <c r="A233" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B233" s="32" t="s">
+      <c r="B233" s="7" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="234" spans="1:2">
-      <c r="A234" s="31" t="s">
+      <c r="A234" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B234" s="32" t="s">
+      <c r="B234" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="235" spans="1:2">
-      <c r="A235" s="31" t="s">
+      <c r="A235" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="B235" s="32" t="s">
+      <c r="B235" s="7" t="s">
         <v>397</v>
       </c>
     </row>
     <row r="236" spans="1:2">
-      <c r="A236" s="31" t="s">
+      <c r="A236" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="B236" s="32" t="s">
+      <c r="B236" s="7" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="237" spans="1:2">
-      <c r="A237" s="31" t="s">
+      <c r="A237" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="B237" s="32" t="s">
+      <c r="B237" s="7" t="s">
         <v>401</v>
       </c>
     </row>
     <row r="238" spans="1:2">
-      <c r="A238" s="31" t="s">
+      <c r="A238" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="B238" s="32" t="s">
+      <c r="B238" s="7" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="239" spans="1:2">
-      <c r="A239" s="31" t="s">
+      <c r="A239" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="B239" s="32" t="s">
+      <c r="B239" s="7" t="s">
         <v>405</v>
       </c>
     </row>
     <row r="240" spans="1:2">
-      <c r="A240" s="31" t="s">
+      <c r="A240" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="B240" s="32" t="s">
+      <c r="B240" s="7" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="241" spans="1:2">
-      <c r="A241" s="31" t="s">
+      <c r="A241" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="B241" s="32" t="s">
+      <c r="B241" s="7" t="s">
         <v>409</v>
       </c>
     </row>
     <row r="242" spans="1:2">
-      <c r="A242" s="31" t="s">
+      <c r="A242" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="B242" s="32" t="s">
+      <c r="B242" s="7" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="243" spans="1:2">
-      <c r="A243" s="31" t="s">
+      <c r="A243" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="B243" s="32" t="s">
+      <c r="B243" s="7" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="244" spans="1:2">
-      <c r="A244" s="31" t="s">
+      <c r="A244" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="B244" s="32" t="s">
+      <c r="B244" s="7" t="s">
         <v>414</v>
       </c>
     </row>
     <row r="245" spans="1:2">
-      <c r="A245" s="31" t="s">
+      <c r="A245" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="B245" s="32" t="s">
+      <c r="B245" s="7" t="s">
         <v>416</v>
       </c>
     </row>
     <row r="246" spans="1:2">
-      <c r="A246" s="31" t="s">
+      <c r="A246" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="B246" s="32" t="s">
+      <c r="B246" s="7" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="247" spans="1:2">
-      <c r="A247" s="31" t="s">
+      <c r="A247" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="B247" s="32" t="s">
+      <c r="B247" s="7" t="s">
         <v>419</v>
       </c>
     </row>
     <row r="248" spans="1:2">
-      <c r="A248" s="31" t="s">
+      <c r="A248" s="2" t="s">
         <v>420</v>
       </c>
       <c r="B248" s="33" t="s">
@@ -3879,246 +4754,475 @@
       </c>
     </row>
     <row r="249" spans="1:2">
-      <c r="A249" s="31" t="s">
+      <c r="A249" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="B249" s="32" t="s">
+      <c r="B249" s="7" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="250" spans="1:2">
-      <c r="A250" s="31" t="s">
+      <c r="A250" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="B250" s="32" t="s">
+      <c r="B250" s="7" t="s">
         <v>424</v>
       </c>
     </row>
     <row r="251" spans="1:2">
-      <c r="A251" s="31" t="s">
+      <c r="A251" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="B251" s="32" t="s">
+      <c r="B251" s="7" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="252" spans="1:2">
-      <c r="A252" s="31" t="s">
+      <c r="A252" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="B252" s="32" t="s">
+      <c r="B252" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="253" spans="1:2">
-      <c r="A253" s="31" t="s">
+      <c r="A253" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="B253" s="32" t="s">
+      <c r="B253" s="7" t="s">
         <v>428</v>
       </c>
     </row>
     <row r="254" spans="1:2">
-      <c r="A254" s="31" t="s">
+      <c r="A254" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="B254" s="32" t="s">
+      <c r="B254" s="7" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="255" spans="1:2">
-      <c r="A255" s="31" t="s">
+      <c r="A255" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="B255" s="32" t="s">
+      <c r="B255" s="7" t="s">
         <v>431</v>
       </c>
     </row>
     <row r="256" spans="1:2">
-      <c r="A256" s="31" t="s">
+      <c r="A256" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="B256" s="32" t="s">
+      <c r="B256" s="7" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="257" spans="1:2">
-      <c r="A257" s="31" t="s">
+      <c r="A257" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="B257" s="32" t="s">
+      <c r="B257" s="7" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="258" spans="1:2">
-      <c r="A258" s="31" t="s">
+      <c r="A258" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="B258" s="32" t="s">
+      <c r="B258" s="7" t="s">
         <v>436</v>
       </c>
     </row>
     <row r="259" spans="1:2">
-      <c r="A259" s="31" t="s">
+      <c r="A259" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="B259" s="32" t="s">
+      <c r="B259" s="7" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="260" spans="1:2">
-      <c r="A260" s="31" t="s">
+      <c r="A260" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="B260" s="32" t="s">
+      <c r="B260" s="7" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="261" spans="1:2">
-      <c r="A261" s="31" t="s">
+      <c r="A261" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="B261" s="32" t="s">
+      <c r="B261" s="7" t="s">
         <v>441</v>
       </c>
     </row>
     <row r="262" spans="1:2">
-      <c r="A262" s="31" t="s">
+      <c r="A262" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="B262" s="32" t="s">
+      <c r="B262" s="7" t="s">
         <v>443</v>
       </c>
     </row>
     <row r="263" spans="1:2">
-      <c r="A263" s="31" t="s">
+      <c r="A263" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="B263" s="32" t="s">
+      <c r="B263" s="7" t="s">
         <v>445</v>
       </c>
     </row>
     <row r="264" spans="1:2">
-      <c r="A264" s="31" t="s">
+      <c r="A264" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="B264" s="32" t="s">
+      <c r="B264" s="7" t="s">
         <v>447</v>
       </c>
     </row>
     <row r="265" spans="1:2">
-      <c r="A265" s="31" t="s">
+      <c r="A265" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="B265" s="32" t="s">
+      <c r="B265" s="7" t="s">
         <v>449</v>
       </c>
     </row>
     <row r="266" spans="1:2">
-      <c r="A266" s="31" t="s">
+      <c r="A266" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="B266" s="32" t="s">
+      <c r="B266" s="7" t="s">
         <v>333</v>
       </c>
     </row>
     <row r="267" spans="1:2">
-      <c r="A267" s="31" t="s">
+      <c r="A267" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="B267" s="32" t="s">
+      <c r="B267" s="7" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="268" spans="1:2">
-      <c r="A268" s="31" t="s">
+      <c r="A268" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="B268" s="32" t="s">
+      <c r="B268" s="7" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="269" spans="1:2">
-      <c r="A269" s="31" t="s">
+      <c r="A269" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="B269" s="32" t="s">
+      <c r="B269" s="7" t="s">
         <v>456</v>
       </c>
     </row>
     <row r="270" spans="1:2">
-      <c r="A270" s="31" t="s">
+      <c r="A270" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="B270" s="32" t="s">
+      <c r="B270" s="7" t="s">
         <v>458</v>
       </c>
     </row>
     <row r="271" spans="1:2">
-      <c r="A271" s="31" t="s">
+      <c r="A271" s="2" t="s">
         <v>459</v>
       </c>
-      <c r="B271" s="32" t="s">
+      <c r="B271" s="7" t="s">
         <v>460</v>
       </c>
     </row>
     <row r="272" spans="1:2">
-      <c r="A272" s="31" t="s">
+      <c r="A272" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="B272" s="32" t="s">
+      <c r="B272" s="7" t="s">
         <v>462</v>
       </c>
     </row>
     <row r="273" spans="1:2">
-      <c r="A273" s="31" t="s">
+      <c r="A273" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="B273" s="32" t="s">
+      <c r="B273" s="7" t="s">
         <v>464</v>
       </c>
     </row>
     <row r="274" spans="1:2">
-      <c r="A274" s="31" t="s">
+      <c r="A274" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="B274" s="32" t="s">
+      <c r="B274" s="7" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="275" spans="1:2">
-      <c r="A275" s="31" t="s">
+      <c r="A275" s="2" t="s">
         <v>466</v>
       </c>
-      <c r="B275" s="32" t="s">
+      <c r="B275" s="7" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="276" spans="1:2">
-      <c r="A276" s="31" t="s">
+      <c r="A276" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="B276" s="32" t="s">
+      <c r="B276" s="7" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="277" spans="1:2">
-      <c r="A277" s="17" t="s">
+      <c r="A277" s="19" t="s">
         <v>469</v>
       </c>
-      <c r="B277" s="31" t="s">
+      <c r="B277" s="2" t="s">
         <v>470</v>
       </c>
     </row>
     <row r="278" spans="1:2">
-      <c r="A278" s="31" t="s">
+      <c r="A278" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B278" s="31" t="s">
+      <c r="B278" s="2" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2">
+      <c r="A279" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="B279" s="7" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2">
+      <c r="A280" s="8" t="s">
+        <v>473</v>
+      </c>
+      <c r="B280" s="9" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2">
+      <c r="A281" s="8" t="s">
+        <v>475</v>
+      </c>
+      <c r="B281" s="9" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2">
+      <c r="A282" s="8" t="s">
+        <v>477</v>
+      </c>
+      <c r="B282" s="9" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2">
+      <c r="A283" s="8" t="s">
+        <v>479</v>
+      </c>
+      <c r="B283" s="34" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2">
+      <c r="A284" s="35" t="s">
+        <v>481</v>
+      </c>
+      <c r="B284" s="7" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2">
+      <c r="A285" s="35" t="s">
+        <v>483</v>
+      </c>
+      <c r="B285" s="7" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2">
+      <c r="A286" s="35" t="s">
+        <v>485</v>
+      </c>
+      <c r="B286" s="7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2">
+      <c r="A287" s="35" t="s">
+        <v>487</v>
+      </c>
+      <c r="B287" s="7" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2">
+      <c r="A288" s="35" t="s">
+        <v>489</v>
+      </c>
+      <c r="B288" s="7" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2">
+      <c r="A289" s="35" t="s">
+        <v>491</v>
+      </c>
+      <c r="B289" s="7" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2">
+      <c r="A290" s="35" t="s">
+        <v>493</v>
+      </c>
+      <c r="B290" s="7" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2">
+      <c r="A291" s="36" t="s">
+        <v>495</v>
+      </c>
+      <c r="B291" s="37" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2">
+      <c r="A292" s="36" t="s">
+        <v>497</v>
+      </c>
+      <c r="B292" s="37" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2">
+      <c r="A293" s="36" t="s">
+        <v>499</v>
+      </c>
+      <c r="B293" s="37" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2">
+      <c r="A294" s="36" t="s">
+        <v>501</v>
+      </c>
+      <c r="B294" s="37" t="s">
+        <v>502</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="19.8888888888889" customWidth="1"/>
+    <col min="2" max="2" width="65" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" ht="109" customHeight="1" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="3" ht="114" customHeight="1" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed Failures Po Amendment And PR LIne Detail Validation Using DB Query
Fixed Failures Po Amendment And PR LIne Detail Validation Using DB Query
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="546">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -1600,6 +1600,60 @@
   </si>
   <si>
     <t>OPSO1/00135/24-25</t>
+  </si>
+  <si>
+    <t>ClassValue</t>
+  </si>
+  <si>
+    <t>Item Class</t>
+  </si>
+  <si>
+    <t>SubClassValue</t>
+  </si>
+  <si>
+    <t>Item SubClass</t>
+  </si>
+  <si>
+    <t>WHValue</t>
+  </si>
+  <si>
+    <t>WH/Dept.</t>
+  </si>
+  <si>
+    <t>ConvValue</t>
+  </si>
+  <si>
+    <t>Conv. Factor</t>
+  </si>
+  <si>
+    <t>UOMValue</t>
+  </si>
+  <si>
+    <t>UOM</t>
+  </si>
+  <si>
+    <t>GLValue</t>
+  </si>
+  <si>
+    <t>PRL_PUR_ACCT</t>
+  </si>
+  <si>
+    <t>GLDescValue</t>
+  </si>
+  <si>
+    <t>GL Acct. Desc.</t>
+  </si>
+  <si>
+    <t>CCCodeLineValue</t>
+  </si>
+  <si>
+    <t>PRL_CC_CODE</t>
+  </si>
+  <si>
+    <t>CCDescValue</t>
+  </si>
+  <si>
+    <t>CPC Code Desc.</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -2439,7 +2493,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2500,10 +2554,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="51">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2825,11 +2875,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B307"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B316"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="34.2909090909091" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="4" customWidth="1"/>
+    <col min="1" max="1" width="34.287037037037" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -5185,107 +5235,179 @@
       </c>
     </row>
     <row r="295" spans="1:2">
-      <c r="A295" s="36" t="s">
+      <c r="A295" s="2" t="s">
         <v>503</v>
       </c>
-      <c r="B295" s="37" t="s">
+      <c r="B295" s="7" t="s">
         <v>421</v>
       </c>
     </row>
     <row r="296" spans="1:2">
-      <c r="A296" s="36" t="s">
+      <c r="A296" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="B296" s="37" t="s">
+      <c r="B296" s="7" t="s">
         <v>505</v>
       </c>
     </row>
     <row r="297" spans="1:2">
-      <c r="A297" s="36" t="s">
+      <c r="A297" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="B297" s="37" t="s">
+      <c r="B297" s="7" t="s">
         <v>421</v>
       </c>
     </row>
     <row r="298" spans="1:2">
-      <c r="A298" s="36" t="s">
+      <c r="A298" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="B298" s="37" t="s">
+      <c r="B298" s="7" t="s">
         <v>508</v>
       </c>
     </row>
     <row r="299" spans="1:2">
-      <c r="A299" s="36" t="s">
+      <c r="A299" s="2" t="s">
         <v>509</v>
       </c>
-      <c r="B299" s="37" t="s">
+      <c r="B299" s="7" t="s">
         <v>510</v>
       </c>
     </row>
     <row r="300" spans="1:2">
-      <c r="A300" s="36" t="s">
+      <c r="A300" s="2" t="s">
         <v>511</v>
       </c>
-      <c r="B300" s="37" t="s">
+      <c r="B300" s="7" t="s">
         <v>512</v>
       </c>
     </row>
     <row r="301" spans="1:2">
-      <c r="A301" s="36" t="s">
+      <c r="A301" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="B301" s="37" t="s">
+      <c r="B301" s="7" t="s">
         <v>512</v>
       </c>
     </row>
     <row r="302" spans="1:2">
-      <c r="A302" s="36" t="s">
+      <c r="A302" s="2" t="s">
         <v>514</v>
       </c>
-      <c r="B302" s="37" t="s">
+      <c r="B302" s="7" t="s">
         <v>515</v>
       </c>
     </row>
     <row r="303" spans="1:2">
-      <c r="A303" s="36" t="s">
+      <c r="A303" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="B303" s="37" t="s">
+      <c r="B303" s="7" t="s">
         <v>515</v>
       </c>
     </row>
     <row r="304" spans="1:2">
-      <c r="A304" s="36" t="s">
+      <c r="A304" s="2" t="s">
         <v>517</v>
       </c>
-      <c r="B304" s="37" t="s">
+      <c r="B304" s="7" t="s">
         <v>518</v>
       </c>
     </row>
     <row r="305" spans="1:2">
-      <c r="A305" s="36" t="s">
+      <c r="A305" s="2" t="s">
         <v>519</v>
       </c>
-      <c r="B305" s="37" t="s">
+      <c r="B305" s="7" t="s">
         <v>518</v>
       </c>
     </row>
     <row r="306" spans="1:2">
-      <c r="A306" s="36" t="s">
+      <c r="A306" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="B306" s="37" t="s">
+      <c r="B306" s="7" t="s">
         <v>521</v>
       </c>
     </row>
     <row r="307" spans="1:2">
-      <c r="A307" s="36" t="s">
+      <c r="A307" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="B307" s="37" t="s">
+      <c r="B307" s="7" t="s">
         <v>523</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2">
+      <c r="A308" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="B308" s="7" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2">
+      <c r="A309" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="B309" s="7" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2">
+      <c r="A310" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="B310" s="7" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2">
+      <c r="A311" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="B311" s="7" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2">
+      <c r="A312" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="B312" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2">
+      <c r="A313" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B313" s="7" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2">
+      <c r="A314" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="B314" s="7" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2">
+      <c r="A315" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="B315" s="7" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2">
+      <c r="A316" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="B316" s="7" t="s">
+        <v>541</v>
       </c>
     </row>
   </sheetData>
@@ -5298,9 +5420,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8909090909091" customWidth="1"/>
+    <col min="1" max="1" width="19.8888888888889" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5314,18 +5436,18 @@
     </row>
     <row r="2" ht="109" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>524</v>
+        <v>542</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>525</v>
+        <v>543</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>526</v>
+        <v>544</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>527</v>
+        <v>545</v>
       </c>
     </row>
     <row r="4" spans="1:2">

</xml_diff>

<commit_message>
Updated Sales Invoice, Open SO, Grn Functions Changes
Updated Sales Invoice, Open SO, Grn Functions Changes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="550">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -1539,13 +1539,67 @@
     <t>Unreleased</t>
   </si>
   <si>
+    <t>ClassValue</t>
+  </si>
+  <si>
+    <t>Item Class</t>
+  </si>
+  <si>
+    <t>SubClassValue</t>
+  </si>
+  <si>
+    <t>Item SubClass</t>
+  </si>
+  <si>
+    <t>WHValue</t>
+  </si>
+  <si>
+    <t>WH/Dept.</t>
+  </si>
+  <si>
+    <t>ConvValue</t>
+  </si>
+  <si>
+    <t>Conv. Factor</t>
+  </si>
+  <si>
+    <t>UOMValue</t>
+  </si>
+  <si>
+    <t>UOM</t>
+  </si>
+  <si>
+    <t>GLValue</t>
+  </si>
+  <si>
+    <t>PRL_PUR_ACCT</t>
+  </si>
+  <si>
+    <t>GLDescValue</t>
+  </si>
+  <si>
+    <t>GL Acct. Desc.</t>
+  </si>
+  <si>
+    <t>CCCodeLineValue</t>
+  </si>
+  <si>
+    <t>PRL_CC_CODE</t>
+  </si>
+  <si>
+    <t>CCDescValue</t>
+  </si>
+  <si>
+    <t>CPC Code Desc.</t>
+  </si>
+  <si>
     <t>oso_Docnum_PCC_Local</t>
   </si>
   <si>
     <t>oso_Docnum_Delete</t>
   </si>
   <si>
-    <t>OPSO1/00001/24-25</t>
+    <t>OSOD-2425-00202</t>
   </si>
   <si>
     <t>oso_Docnum_PC_Local</t>
@@ -1575,12 +1629,12 @@
     <t>oso_Docnum_Add_IS</t>
   </si>
   <si>
-    <t>OPSO1/00132/24-25</t>
-  </si>
-  <si>
     <t>oso_Docnum_Delete_IS</t>
   </si>
   <si>
+    <t>OPSO1/00145/24-25</t>
+  </si>
+  <si>
     <t>oso_Docnum_PC_EX</t>
   </si>
   <si>
@@ -1599,61 +1653,19 @@
     <t>oso_Docnum_Delete_EX</t>
   </si>
   <si>
-    <t>OPSO1/00135/24-25</t>
-  </si>
-  <si>
-    <t>ClassValue</t>
-  </si>
-  <si>
-    <t>Item Class</t>
-  </si>
-  <si>
-    <t>SubClassValue</t>
-  </si>
-  <si>
-    <t>Item SubClass</t>
-  </si>
-  <si>
-    <t>WHValue</t>
-  </si>
-  <si>
-    <t>WH/Dept.</t>
-  </si>
-  <si>
-    <t>ConvValue</t>
-  </si>
-  <si>
-    <t>Conv. Factor</t>
-  </si>
-  <si>
-    <t>UOMValue</t>
-  </si>
-  <si>
-    <t>UOM</t>
-  </si>
-  <si>
-    <t>GLValue</t>
-  </si>
-  <si>
-    <t>PRL_PUR_ACCT</t>
-  </si>
-  <si>
-    <t>GLDescValue</t>
-  </si>
-  <si>
-    <t>GL Acct. Desc.</t>
-  </si>
-  <si>
-    <t>CCCodeLineValue</t>
-  </si>
-  <si>
-    <t>PRL_CC_CODE</t>
-  </si>
-  <si>
-    <t>CCDescValue</t>
-  </si>
-  <si>
-    <t>CPC Code Desc.</t>
+    <t>OSOD-2425-00284</t>
+  </si>
+  <si>
+    <t>PI_PaymentTerm</t>
+  </si>
+  <si>
+    <t>T002</t>
+  </si>
+  <si>
+    <t>IntraTransfer</t>
+  </si>
+  <si>
+    <t>Intra Transfer</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -2493,7 +2505,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2554,6 +2566,8 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="51">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2875,7 +2889,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B316"/>
+  <dimension ref="A1:B318"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="34.287037037037" customWidth="1"/>
@@ -5239,159 +5253,159 @@
         <v>503</v>
       </c>
       <c r="B295" s="7" t="s">
-        <v>421</v>
+        <v>504</v>
       </c>
     </row>
     <row r="296" spans="1:2">
       <c r="A296" s="2" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B296" s="7" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="297" spans="1:2">
       <c r="A297" s="2" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B297" s="7" t="s">
-        <v>421</v>
+        <v>508</v>
       </c>
     </row>
     <row r="298" spans="1:2">
       <c r="A298" s="2" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B298" s="7" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="299" spans="1:2">
       <c r="A299" s="2" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B299" s="7" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="300" spans="1:2">
       <c r="A300" s="2" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B300" s="7" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="301" spans="1:2">
       <c r="A301" s="2" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B301" s="7" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
     </row>
     <row r="302" spans="1:2">
       <c r="A302" s="2" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="B302" s="7" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
     </row>
     <row r="303" spans="1:2">
       <c r="A303" s="2" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="B303" s="7" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
     </row>
     <row r="304" spans="1:2">
       <c r="A304" s="2" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="B304" s="7" t="s">
-        <v>518</v>
+        <v>421</v>
       </c>
     </row>
     <row r="305" spans="1:2">
       <c r="A305" s="2" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="B305" s="7" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
     </row>
     <row r="306" spans="1:2">
       <c r="A306" s="2" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="B306" s="7" t="s">
-        <v>521</v>
+        <v>421</v>
       </c>
     </row>
     <row r="307" spans="1:2">
       <c r="A307" s="2" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B307" s="7" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
     </row>
     <row r="308" spans="1:2">
       <c r="A308" s="2" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="B308" s="7" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
     </row>
     <row r="309" spans="1:2">
       <c r="A309" s="2" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B309" s="7" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
     </row>
     <row r="310" spans="1:2">
       <c r="A310" s="2" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="B310" s="7" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="311" spans="1:2">
       <c r="A311" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="B311" s="7" t="s">
         <v>530</v>
-      </c>
-      <c r="B311" s="7" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="312" spans="1:2">
       <c r="A312" s="2" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B312" s="7" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="313" spans="1:2">
       <c r="A313" s="2" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B313" s="7" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="314" spans="1:2">
       <c r="A314" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="B314" s="7" t="s">
         <v>536</v>
-      </c>
-      <c r="B314" s="7" t="s">
-        <v>537</v>
       </c>
     </row>
     <row r="315" spans="1:2">
@@ -5408,6 +5422,22 @@
       </c>
       <c r="B316" s="7" t="s">
         <v>541</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2">
+      <c r="A317" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="B317" s="7" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2">
+      <c r="A318" s="36" t="s">
+        <v>544</v>
+      </c>
+      <c r="B318" s="37" t="s">
+        <v>545</v>
       </c>
     </row>
   </sheetData>
@@ -5436,18 +5466,18 @@
     </row>
     <row r="2" ht="109" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
     </row>
     <row r="4" spans="1:2">

</xml_diff>

<commit_message>
Updated Attendance Leave, Grn Functions, Purchase Request Functions
Updated Attendance Leave, Grn Page, Purchase Request Functions
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="570">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -549,10 +549,10 @@
     <t>DURAIRAJ  R</t>
   </si>
   <si>
-    <t>PermFromDate</t>
-  </si>
-  <si>
-    <t>24-05-2024</t>
+    <t>PermFromDate1</t>
+  </si>
+  <si>
+    <t>07-12-2024</t>
   </si>
   <si>
     <t>PermissionTimeFrom</t>
@@ -1717,6 +1717,15 @@
   </si>
   <si>
     <t>TVS-AMD-DIS-</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>ExpiryDate</t>
+  </si>
+  <si>
+    <t>08-02-2027</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -2556,7 +2565,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2618,9 +2627,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="51">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2942,7 +2948,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B327"/>
+  <dimension ref="A1:B329"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="34.287037037037" customWidth="1"/>
@@ -5534,35 +5540,51 @@
       </c>
     </row>
     <row r="324" spans="1:2">
-      <c r="A324" s="36" t="s">
+      <c r="A324" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="B324" s="37" t="s">
+      <c r="B324" s="7" t="s">
         <v>556</v>
       </c>
     </row>
     <row r="325" spans="1:2">
-      <c r="A325" s="36" t="s">
+      <c r="A325" s="2" t="s">
         <v>557</v>
       </c>
-      <c r="B325" s="37" t="s">
+      <c r="B325" s="7" t="s">
         <v>558</v>
       </c>
     </row>
     <row r="326" spans="1:2">
-      <c r="A326" s="36" t="s">
+      <c r="A326" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="B326" s="37" t="s">
+      <c r="B326" s="7" t="s">
         <v>560</v>
       </c>
     </row>
     <row r="327" spans="1:2">
-      <c r="A327" s="36" t="s">
+      <c r="A327" s="2" t="s">
         <v>561</v>
       </c>
-      <c r="B327" s="37" t="s">
+      <c r="B327" s="7" t="s">
         <v>562</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2">
+      <c r="A328" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B328" s="7" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2">
+      <c r="A329" s="36" t="s">
+        <v>564</v>
+      </c>
+      <c r="B329" s="7" t="s">
+        <v>565</v>
       </c>
     </row>
   </sheetData>
@@ -5591,18 +5613,18 @@
     </row>
     <row r="2" ht="109" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" spans="1:2">

</xml_diff>

<commit_message>
Updated PriceList Page Function And CommonFunctions
Updated PriceList Page Function And CommonFunctions
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="571">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -1726,6 +1726,9 @@
   </si>
   <si>
     <t>08-02-2027</t>
+  </si>
+  <si>
+    <t>Draft</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -2565,7 +2568,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2627,6 +2630,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="51">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2948,7 +2954,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B329"/>
+  <dimension ref="A1:B330"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="34.287037037037" customWidth="1"/>
@@ -5580,11 +5586,19 @@
       </c>
     </row>
     <row r="329" spans="1:2">
-      <c r="A329" s="36" t="s">
+      <c r="A329" s="2" t="s">
         <v>564</v>
       </c>
       <c r="B329" s="7" t="s">
         <v>565</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2">
+      <c r="A330" s="36" t="s">
+        <v>566</v>
+      </c>
+      <c r="B330" s="37" t="s">
+        <v>566</v>
       </c>
     </row>
   </sheetData>
@@ -5613,18 +5627,18 @@
     </row>
     <row r="2" ht="109" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="4" spans="1:2">

</xml_diff>

<commit_message>
Updated Failure Fixes And Added RFQ Functions, E2E Test Scenarios
Updated Failure Fixes And Added RFQ Functions, E2E Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="800">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="832">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -2404,6 +2404,102 @@
   </si>
   <si>
     <t>GRL10/00429/24-25</t>
+  </si>
+  <si>
+    <t>SubcontractorName</t>
+  </si>
+  <si>
+    <t>ACT ON FINISHING (P) LTD</t>
+  </si>
+  <si>
+    <t>GeneralExpense</t>
+  </si>
+  <si>
+    <t>GENERAL EXPENSE</t>
+  </si>
+  <si>
+    <t>ScoItem</t>
+  </si>
+  <si>
+    <t>HK-FIFO-LOT-BATCH-SO-10001(FG)</t>
+  </si>
+  <si>
+    <t>PEELING</t>
+  </si>
+  <si>
+    <t>00</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>RawMaterialSco</t>
+  </si>
+  <si>
+    <t>StandardProd</t>
+  </si>
+  <si>
+    <t>Pro</t>
+  </si>
+  <si>
+    <t>PRC 0</t>
+  </si>
+  <si>
+    <t>SaleOrderNumber</t>
+  </si>
+  <si>
+    <t>SO100/00019/24-25</t>
+  </si>
+  <si>
+    <t>Orderreleases</t>
+  </si>
+  <si>
+    <t>Order Release</t>
+  </si>
+  <si>
+    <t>Inprogress</t>
+  </si>
+  <si>
+    <t>ComQty</t>
+  </si>
+  <si>
+    <t>Completion Quantity</t>
+  </si>
+  <si>
+    <t>NoDataFound</t>
+  </si>
+  <si>
+    <t>No data found</t>
+  </si>
+  <si>
+    <t>AllocatedValue</t>
+  </si>
+  <si>
+    <t>FirstDcNumber</t>
+  </si>
+  <si>
+    <t>DC10-2425-01357</t>
+  </si>
+  <si>
+    <t>FreePass</t>
+  </si>
+  <si>
+    <t>Free Pass</t>
+  </si>
+  <si>
+    <t>DcDetails</t>
+  </si>
+  <si>
+    <t>Select 1 row in the master region</t>
+  </si>
+  <si>
+    <t>FG-WH-KD</t>
+  </si>
+  <si>
+    <t>FG WH KD</t>
+  </si>
+  <si>
+    <t>OrderReleaseOption</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -2714,7 +2810,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2762,18 +2858,6 @@
     <font>
       <sz val="10"/>
       <name val="Consolas"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -3262,7 +3346,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="51">
+  <cellStyleXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
@@ -3279,139 +3363,141 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3433,9 +3519,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3488,9 +3571,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -3529,29 +3609,28 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="51">
+  <cellStyles count="53">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -3603,6 +3682,8 @@
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
     <cellStyle name="Normal 2" xfId="49"/>
     <cellStyle name="Normal 3" xfId="50"/>
+    <cellStyle name="Normal 2 2" xfId="51"/>
+    <cellStyle name="Normal 2 3" xfId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3871,11 +3952,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B461"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B487"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="34.2909090909091" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="4" customWidth="1"/>
+    <col min="1" max="1" width="34.287037037037" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -4402,7 +4483,7 @@
       <c r="A66" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B66" s="10" t="s">
+      <c r="B66" s="9" t="s">
         <v>126</v>
       </c>
     </row>
@@ -4410,7 +4491,7 @@
       <c r="A67" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B67" s="10" t="s">
+      <c r="B67" s="9" t="s">
         <v>128</v>
       </c>
     </row>
@@ -4418,7 +4499,7 @@
       <c r="A68" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B68" s="10" t="s">
+      <c r="B68" s="9" t="s">
         <v>130</v>
       </c>
     </row>
@@ -4426,7 +4507,7 @@
       <c r="A69" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B69" s="10">
+      <c r="B69" s="9">
         <v>2012</v>
       </c>
     </row>
@@ -4434,7 +4515,7 @@
       <c r="A70" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="B70" s="10" t="s">
+      <c r="B70" s="9" t="s">
         <v>133</v>
       </c>
     </row>
@@ -4442,319 +4523,319 @@
       <c r="A71" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B71" s="10" t="s">
+      <c r="B71" s="9" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="72" spans="1:2">
-      <c r="A72" s="11" t="s">
+      <c r="A72" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B72" s="10" t="s">
+      <c r="B72" s="9" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="73" spans="1:2">
-      <c r="A73" s="11" t="s">
+      <c r="A73" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B73" s="10" t="s">
+      <c r="B73" s="9" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="74" spans="1:2">
-      <c r="A74" s="11" t="s">
+      <c r="A74" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B74" s="10" t="s">
+      <c r="B74" s="9" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="75" spans="1:2">
-      <c r="A75" s="11" t="s">
+      <c r="A75" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B75" s="10" t="s">
+      <c r="B75" s="9" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="76" spans="1:2">
-      <c r="A76" s="11" t="s">
+      <c r="A76" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="B76" s="10">
+      <c r="B76" s="9">
         <v>202425</v>
       </c>
     </row>
     <row r="77" spans="1:2">
-      <c r="A77" s="11" t="s">
+      <c r="A77" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B77" s="10" t="s">
+      <c r="B77" s="9" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="78" spans="1:2">
-      <c r="A78" s="11" t="s">
+      <c r="A78" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="B78" s="10" t="s">
+      <c r="B78" s="9" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="79" spans="1:2">
-      <c r="A79" s="11" t="s">
+      <c r="A79" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="B79" s="10" t="s">
+      <c r="B79" s="9" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="80" spans="1:2">
-      <c r="A80" s="12" t="s">
+      <c r="A80" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="B80" s="13" t="s">
+      <c r="B80" s="12" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="81" spans="1:2">
-      <c r="A81" s="12" t="s">
+      <c r="A81" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="B81" s="13" t="s">
+      <c r="B81" s="12" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="82" spans="1:2">
-      <c r="A82" s="12" t="s">
+      <c r="A82" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="B82" s="14" t="s">
+      <c r="B82" s="13" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="83" spans="1:2">
-      <c r="A83" s="12" t="s">
+      <c r="A83" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="B83" s="13" t="s">
+      <c r="B83" s="12" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="84" spans="1:2">
-      <c r="A84" s="12" t="s">
+      <c r="A84" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="B84" s="14" t="s">
+      <c r="B84" s="13" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="85" spans="1:2">
-      <c r="A85" s="12" t="s">
+      <c r="A85" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="B85" s="14" t="s">
+      <c r="B85" s="13" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="86" spans="1:2">
-      <c r="A86" s="12" t="s">
+      <c r="A86" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="B86" s="13" t="s">
+      <c r="B86" s="12" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="87" spans="1:2">
-      <c r="A87" s="12" t="s">
+      <c r="A87" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="B87" s="13" t="s">
+      <c r="B87" s="12" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="88" spans="1:2">
-      <c r="A88" s="15" t="s">
+      <c r="A88" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="B88" s="13" t="s">
+      <c r="B88" s="12" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="89" spans="1:2">
-      <c r="A89" s="15" t="s">
+      <c r="A89" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="B89" s="13" t="s">
+      <c r="B89" s="12" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="90" spans="1:2">
-      <c r="A90" s="16" t="s">
+      <c r="A90" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="B90" s="13" t="s">
+      <c r="B90" s="12" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="91" spans="1:2">
-      <c r="A91" s="15" t="s">
+      <c r="A91" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="B91" s="13" t="s">
+      <c r="B91" s="12" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="92" spans="1:2">
-      <c r="A92" s="15" t="s">
+      <c r="A92" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="B92" s="13" t="s">
+      <c r="B92" s="12" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="93" spans="1:2">
-      <c r="A93" s="15" t="s">
+      <c r="A93" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="B93" s="13" t="s">
+      <c r="B93" s="12" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="94" spans="1:2">
-      <c r="A94" s="15" t="s">
+      <c r="A94" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="B94" s="13" t="s">
+      <c r="B94" s="12" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="95" spans="1:2">
-      <c r="A95" s="15" t="s">
+      <c r="A95" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B95" s="13" t="s">
+      <c r="B95" s="12" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="96" spans="1:2">
-      <c r="A96" s="15" t="s">
+      <c r="A96" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B96" s="13" t="s">
+      <c r="B96" s="12" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="97" spans="1:2">
-      <c r="A97" s="15" t="s">
+      <c r="A97" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="B97" s="13" t="s">
+      <c r="B97" s="12" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="98" spans="1:2">
-      <c r="A98" s="15" t="s">
+      <c r="A98" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="B98" s="13" t="s">
+      <c r="B98" s="12" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="99" spans="1:2">
-      <c r="A99" s="15" t="s">
+      <c r="A99" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B99" s="13" t="s">
+      <c r="B99" s="12" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="100" spans="1:2">
-      <c r="A100" s="17" t="s">
+      <c r="A100" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="B100" s="18" t="s">
+      <c r="B100" s="17" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="101" spans="1:2">
-      <c r="A101" s="17" t="s">
+      <c r="A101" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="B101" s="19" t="s">
+      <c r="B101" s="18" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="102" spans="1:2">
-      <c r="A102" s="17" t="s">
+      <c r="A102" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="B102" s="18" t="s">
+      <c r="B102" s="17" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="103" spans="1:2">
-      <c r="A103" s="17" t="s">
+      <c r="A103" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="B103" s="18" t="s">
+      <c r="B103" s="17" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="104" spans="1:2">
-      <c r="A104" s="17" t="s">
+      <c r="A104" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="B104" s="19">
+      <c r="B104" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="105" spans="1:2">
-      <c r="A105" s="20" t="s">
+      <c r="A105" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="B105" s="21" t="s">
+      <c r="B105" s="20" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="106" spans="1:2">
-      <c r="A106" s="20" t="s">
+      <c r="A106" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="B106" s="22" t="s">
+      <c r="B106" s="21" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="107" spans="1:2">
-      <c r="A107" s="20" t="s">
+      <c r="A107" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="B107" s="23">
+      <c r="B107" s="22">
         <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:2">
-      <c r="A108" s="20" t="s">
+      <c r="A108" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="B108" s="21" t="s">
+      <c r="B108" s="20" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="109" spans="1:2">
-      <c r="A109" s="20" t="s">
+      <c r="A109" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="B109" s="24" t="s">
+      <c r="B109" s="23" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="110" spans="1:2">
-      <c r="A110" s="20" t="s">
+      <c r="A110" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="B110" s="23">
+      <c r="B110" s="22">
         <v>100</v>
       </c>
     </row>
@@ -4762,47 +4843,47 @@
       <c r="A111" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B111" s="25" t="s">
+      <c r="B111" s="24" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="112" spans="1:2">
-      <c r="A112" s="26" t="s">
+      <c r="A112" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="B112" s="27" t="s">
+      <c r="B112" s="26" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="113" spans="1:2">
-      <c r="A113" s="26" t="s">
+      <c r="A113" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="B113" s="27" t="s">
+      <c r="B113" s="26" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="114" spans="1:2">
-      <c r="A114" s="26" t="s">
+      <c r="A114" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="B114" s="25" t="s">
+      <c r="B114" s="24" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="115" spans="1:2">
-      <c r="A115" s="26" t="s">
+      <c r="A115" s="25" t="s">
         <v>211</v>
       </c>
-      <c r="B115" s="25" t="s">
+      <c r="B115" s="24" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="116" spans="1:2">
-      <c r="A116" s="26" t="s">
+      <c r="A116" s="25" t="s">
         <v>213</v>
       </c>
-      <c r="B116" s="25" t="s">
+      <c r="B116" s="24" t="s">
         <v>214</v>
       </c>
     </row>
@@ -4810,7 +4891,7 @@
       <c r="A117" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B117" s="25" t="s">
+      <c r="B117" s="24" t="s">
         <v>17</v>
       </c>
     </row>
@@ -4818,319 +4899,319 @@
       <c r="A118" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B118" s="25">
+      <c r="B118" s="24">
         <v>0</v>
       </c>
     </row>
     <row r="119" spans="1:2">
-      <c r="A119" s="28" t="s">
+      <c r="A119" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="B119" s="29" t="s">
+      <c r="B119" s="28" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="120" spans="1:2">
-      <c r="A120" s="28" t="s">
+      <c r="A120" s="27" t="s">
         <v>219</v>
       </c>
-      <c r="B120" s="29" t="s">
+      <c r="B120" s="28" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="121" spans="1:2">
-      <c r="A121" s="28" t="s">
+      <c r="A121" s="27" t="s">
         <v>221</v>
       </c>
-      <c r="B121" s="29" t="s">
+      <c r="B121" s="28" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="122" spans="1:2">
-      <c r="A122" s="28" t="s">
+      <c r="A122" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="B122" s="29" t="s">
+      <c r="B122" s="28" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="123" spans="1:2">
-      <c r="A123" s="28" t="s">
+      <c r="A123" s="27" t="s">
         <v>225</v>
       </c>
-      <c r="B123" s="29" t="s">
+      <c r="B123" s="28" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="124" spans="1:2">
-      <c r="A124" s="28" t="s">
+      <c r="A124" s="27" t="s">
         <v>227</v>
       </c>
-      <c r="B124" s="29" t="s">
+      <c r="B124" s="28" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="125" spans="1:2">
-      <c r="A125" s="28" t="s">
+      <c r="A125" s="27" t="s">
         <v>228</v>
       </c>
-      <c r="B125" s="29" t="s">
+      <c r="B125" s="28" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="126" spans="1:2">
-      <c r="A126" s="28" t="s">
+      <c r="A126" s="27" t="s">
         <v>230</v>
       </c>
-      <c r="B126" s="29" t="s">
+      <c r="B126" s="28" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="127" spans="1:2">
-      <c r="A127" s="28" t="s">
+      <c r="A127" s="27" t="s">
         <v>232</v>
       </c>
-      <c r="B127" s="29" t="s">
+      <c r="B127" s="28" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="128" spans="1:2">
-      <c r="A128" s="28" t="s">
+      <c r="A128" s="27" t="s">
         <v>234</v>
       </c>
-      <c r="B128" s="29" t="s">
+      <c r="B128" s="28" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="129" spans="1:2">
-      <c r="A129" s="28" t="s">
+      <c r="A129" s="27" t="s">
         <v>236</v>
       </c>
-      <c r="B129" s="29" t="s">
+      <c r="B129" s="28" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="130" spans="1:2">
-      <c r="A130" s="28" t="s">
+      <c r="A130" s="27" t="s">
         <v>237</v>
       </c>
-      <c r="B130" s="29" t="s">
+      <c r="B130" s="28" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="131" spans="1:2">
-      <c r="A131" s="28" t="s">
+      <c r="A131" s="27" t="s">
         <v>239</v>
       </c>
-      <c r="B131" s="29" t="s">
+      <c r="B131" s="28" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="132" spans="1:2">
-      <c r="A132" s="28" t="s">
+      <c r="A132" s="27" t="s">
         <v>241</v>
       </c>
-      <c r="B132" s="29" t="s">
+      <c r="B132" s="28" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="133" spans="1:2">
-      <c r="A133" s="28" t="s">
+      <c r="A133" s="27" t="s">
         <v>243</v>
       </c>
-      <c r="B133" s="29" t="s">
+      <c r="B133" s="28" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="134" spans="1:2">
-      <c r="A134" s="28" t="s">
+      <c r="A134" s="27" t="s">
         <v>245</v>
       </c>
-      <c r="B134" s="29" t="s">
+      <c r="B134" s="28" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="135" spans="1:2">
-      <c r="A135" s="28" t="s">
+      <c r="A135" s="27" t="s">
         <v>246</v>
       </c>
-      <c r="B135" s="29" t="s">
+      <c r="B135" s="28" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="136" spans="1:2">
-      <c r="A136" s="28" t="s">
+      <c r="A136" s="27" t="s">
         <v>248</v>
       </c>
-      <c r="B136" s="29" t="s">
+      <c r="B136" s="28" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="137" spans="1:2">
-      <c r="A137" s="28" t="s">
+      <c r="A137" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="B137" s="29" t="s">
+      <c r="B137" s="28" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="138" spans="1:2">
-      <c r="A138" s="28" t="s">
+      <c r="A138" s="27" t="s">
         <v>251</v>
       </c>
-      <c r="B138" s="29" t="s">
+      <c r="B138" s="28" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="139" spans="1:2">
-      <c r="A139" s="28" t="s">
+      <c r="A139" s="27" t="s">
         <v>252</v>
       </c>
-      <c r="B139" s="29" t="s">
+      <c r="B139" s="28" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="140" spans="1:2">
-      <c r="A140" s="28" t="s">
+      <c r="A140" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="B140" s="29" t="s">
+      <c r="B140" s="28" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="141" spans="1:2">
-      <c r="A141" s="28" t="s">
+      <c r="A141" s="27" t="s">
         <v>254</v>
       </c>
-      <c r="B141" s="29" t="s">
+      <c r="B141" s="28" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="142" spans="1:2">
-      <c r="A142" s="28" t="s">
+      <c r="A142" s="27" t="s">
         <v>255</v>
       </c>
-      <c r="B142" s="29" t="s">
+      <c r="B142" s="28" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="143" spans="1:2">
-      <c r="A143" s="28" t="s">
+      <c r="A143" s="27" t="s">
         <v>256</v>
       </c>
-      <c r="B143" s="29" t="s">
+      <c r="B143" s="28" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="144" spans="1:2">
-      <c r="A144" s="28" t="s">
+      <c r="A144" s="27" t="s">
         <v>257</v>
       </c>
-      <c r="B144" s="29" t="s">
+      <c r="B144" s="28" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="145" spans="1:2">
-      <c r="A145" s="28" t="s">
+      <c r="A145" s="27" t="s">
         <v>258</v>
       </c>
-      <c r="B145" s="29" t="s">
+      <c r="B145" s="28" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="146" spans="1:2">
-      <c r="A146" s="28" t="s">
+      <c r="A146" s="27" t="s">
         <v>259</v>
       </c>
-      <c r="B146" s="29" t="s">
+      <c r="B146" s="28" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="147" spans="1:2">
-      <c r="A147" s="28" t="s">
+      <c r="A147" s="27" t="s">
         <v>260</v>
       </c>
-      <c r="B147" s="29" t="s">
+      <c r="B147" s="28" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="148" spans="1:2">
-      <c r="A148" s="28" t="s">
+      <c r="A148" s="27" t="s">
         <v>261</v>
       </c>
-      <c r="B148" s="29" t="s">
+      <c r="B148" s="28" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="149" spans="1:2">
-      <c r="A149" s="28" t="s">
+      <c r="A149" s="27" t="s">
         <v>262</v>
       </c>
-      <c r="B149" s="29" t="s">
+      <c r="B149" s="28" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="150" spans="1:2">
-      <c r="A150" s="28" t="s">
+      <c r="A150" s="27" t="s">
         <v>263</v>
       </c>
-      <c r="B150" s="29" t="s">
+      <c r="B150" s="28" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="151" spans="1:2">
-      <c r="A151" s="30" t="s">
+      <c r="A151" s="29" t="s">
         <v>264</v>
       </c>
-      <c r="B151" s="29" t="s">
+      <c r="B151" s="28" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="152" spans="1:2">
-      <c r="A152" s="30" t="s">
+      <c r="A152" s="29" t="s">
         <v>266</v>
       </c>
-      <c r="B152" s="29" t="s">
+      <c r="B152" s="28" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="153" spans="1:2">
-      <c r="A153" s="30" t="s">
+      <c r="A153" s="29" t="s">
         <v>268</v>
       </c>
-      <c r="B153" s="29" t="s">
+      <c r="B153" s="28" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="154" spans="1:2">
-      <c r="A154" s="30" t="s">
+      <c r="A154" s="29" t="s">
         <v>270</v>
       </c>
-      <c r="B154" s="29" t="s">
+      <c r="B154" s="28" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="155" spans="1:2">
-      <c r="A155" s="30" t="s">
+      <c r="A155" s="29" t="s">
         <v>272</v>
       </c>
-      <c r="B155" s="29" t="s">
+      <c r="B155" s="28" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="156" spans="1:2">
-      <c r="A156" s="30" t="s">
+      <c r="A156" s="29" t="s">
         <v>274</v>
       </c>
-      <c r="B156" s="29" t="s">
+      <c r="B156" s="28" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="157" spans="1:2">
-      <c r="A157" s="31" t="s">
+      <c r="A157" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="B157" s="32" t="s">
+      <c r="B157" s="31" t="s">
         <v>277</v>
       </c>
     </row>
@@ -5138,263 +5219,263 @@
       <c r="A158" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="B158" s="25" t="s">
+      <c r="B158" s="24" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="159" spans="1:2">
-      <c r="A159" s="12" t="s">
+      <c r="A159" s="11" t="s">
         <v>280</v>
       </c>
-      <c r="B159" s="33" t="s">
+      <c r="B159" s="32" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="160" spans="1:2">
-      <c r="A160" s="12" t="s">
+      <c r="A160" s="11" t="s">
         <v>282</v>
       </c>
-      <c r="B160" s="34" t="s">
+      <c r="B160" s="12" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="161" spans="1:2">
-      <c r="A161" s="12" t="s">
+      <c r="A161" s="11" t="s">
         <v>284</v>
       </c>
-      <c r="B161" s="14" t="s">
+      <c r="B161" s="13" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="162" spans="1:2">
-      <c r="A162" s="12" t="s">
+      <c r="A162" s="11" t="s">
         <v>286</v>
       </c>
-      <c r="B162" s="34" t="s">
+      <c r="B162" s="12" t="s">
         <v>287</v>
       </c>
     </row>
     <row r="163" spans="1:2">
-      <c r="A163" s="12" t="s">
+      <c r="A163" s="11" t="s">
         <v>288</v>
       </c>
-      <c r="B163" s="34" t="s">
+      <c r="B163" s="12" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="164" spans="1:2">
-      <c r="A164" s="12" t="s">
+      <c r="A164" s="11" t="s">
         <v>290</v>
       </c>
-      <c r="B164" s="14" t="s">
+      <c r="B164" s="13" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="165" spans="1:2">
-      <c r="A165" s="12" t="s">
+      <c r="A165" s="11" t="s">
         <v>292</v>
       </c>
-      <c r="B165" s="14" t="s">
+      <c r="B165" s="13" t="s">
         <v>293</v>
       </c>
     </row>
     <row r="166" spans="1:2">
-      <c r="A166" s="12" t="s">
+      <c r="A166" s="11" t="s">
         <v>294</v>
       </c>
-      <c r="B166" s="34" t="s">
+      <c r="B166" s="12" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="167" spans="1:2">
-      <c r="A167" s="12" t="s">
+      <c r="A167" s="11" t="s">
         <v>296</v>
       </c>
-      <c r="B167" s="34" t="s">
+      <c r="B167" s="12" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="168" spans="1:2">
-      <c r="A168" s="12" t="s">
+      <c r="A168" s="11" t="s">
         <v>298</v>
       </c>
-      <c r="B168" s="14" t="s">
+      <c r="B168" s="13" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="169" spans="1:2">
-      <c r="A169" s="12" t="s">
+      <c r="A169" s="11" t="s">
         <v>300</v>
       </c>
-      <c r="B169" s="14" t="s">
+      <c r="B169" s="13" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="170" spans="1:2">
-      <c r="A170" s="12" t="s">
+      <c r="A170" s="11" t="s">
         <v>302</v>
       </c>
-      <c r="B170" s="34" t="s">
+      <c r="B170" s="12" t="s">
         <v>303</v>
       </c>
     </row>
     <row r="171" spans="1:2">
-      <c r="A171" s="12" t="s">
+      <c r="A171" s="11" t="s">
         <v>304</v>
       </c>
-      <c r="B171" s="34" t="s">
+      <c r="B171" s="12" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="172" spans="1:2">
-      <c r="A172" s="12" t="s">
+      <c r="A172" s="11" t="s">
         <v>306</v>
       </c>
-      <c r="B172" s="34" t="s">
+      <c r="B172" s="12" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="173" spans="1:2">
-      <c r="A173" s="12" t="s">
+      <c r="A173" s="11" t="s">
         <v>308</v>
       </c>
-      <c r="B173" s="34" t="s">
+      <c r="B173" s="12" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="174" spans="1:2">
-      <c r="A174" s="12" t="s">
+      <c r="A174" s="11" t="s">
         <v>310</v>
       </c>
-      <c r="B174" s="34" t="s">
+      <c r="B174" s="12" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="175" spans="1:2">
-      <c r="A175" s="12" t="s">
+      <c r="A175" s="11" t="s">
         <v>311</v>
       </c>
-      <c r="B175" s="34" t="s">
+      <c r="B175" s="12" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="176" spans="1:2">
-      <c r="A176" s="12" t="s">
+      <c r="A176" s="11" t="s">
         <v>313</v>
       </c>
-      <c r="B176" s="34" t="s">
+      <c r="B176" s="12" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="177" spans="1:2">
-      <c r="A177" s="12" t="s">
+      <c r="A177" s="11" t="s">
         <v>315</v>
       </c>
-      <c r="B177" s="34" t="s">
+      <c r="B177" s="12" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="178" spans="1:2">
-      <c r="A178" s="12" t="s">
+      <c r="A178" s="11" t="s">
         <v>316</v>
       </c>
-      <c r="B178" s="34" t="s">
+      <c r="B178" s="12" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="179" spans="1:2">
-      <c r="A179" s="12" t="s">
+      <c r="A179" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="B179" s="34" t="s">
+      <c r="B179" s="12" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="180" spans="1:2">
-      <c r="A180" s="12" t="s">
+      <c r="A180" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="B180" s="34" t="s">
+      <c r="B180" s="12" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="181" spans="1:2">
-      <c r="A181" s="12" t="s">
+      <c r="A181" s="11" t="s">
         <v>321</v>
       </c>
-      <c r="B181" s="34" t="s">
+      <c r="B181" s="12" t="s">
         <v>322</v>
       </c>
     </row>
     <row r="182" spans="1:2">
-      <c r="A182" s="12" t="s">
+      <c r="A182" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="B182" s="34" t="s">
+      <c r="B182" s="12" t="s">
         <v>324</v>
       </c>
     </row>
     <row r="183" spans="1:2">
-      <c r="A183" s="12" t="s">
+      <c r="A183" s="11" t="s">
         <v>325</v>
       </c>
-      <c r="B183" s="34" t="s">
+      <c r="B183" s="12" t="s">
         <v>326</v>
       </c>
     </row>
     <row r="184" spans="1:2">
-      <c r="A184" s="12" t="s">
+      <c r="A184" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="B184" s="34" t="s">
+      <c r="B184" s="12" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="185" spans="1:2">
-      <c r="A185" s="12" t="s">
+      <c r="A185" s="11" t="s">
         <v>329</v>
       </c>
-      <c r="B185" s="34" t="s">
+      <c r="B185" s="12" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="186" spans="1:2">
-      <c r="A186" s="12" t="s">
+      <c r="A186" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="B186" s="14" t="s">
+      <c r="B186" s="13" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="187" spans="1:2">
-      <c r="A187" s="12" t="s">
+      <c r="A187" s="11" t="s">
         <v>333</v>
       </c>
-      <c r="B187" s="14" t="s">
+      <c r="B187" s="13" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="188" spans="1:2">
-      <c r="A188" s="12" t="s">
+      <c r="A188" s="11" t="s">
         <v>334</v>
       </c>
-      <c r="B188" s="34" t="s">
+      <c r="B188" s="12" t="s">
         <v>335</v>
       </c>
     </row>
     <row r="189" spans="1:2">
-      <c r="A189" s="12" t="s">
+      <c r="A189" s="11" t="s">
         <v>336</v>
       </c>
-      <c r="B189" s="14" t="s">
+      <c r="B189" s="13" t="s">
         <v>337</v>
       </c>
     </row>
     <row r="190" spans="1:2">
-      <c r="A190" s="12" t="s">
+      <c r="A190" s="11" t="s">
         <v>338</v>
       </c>
-      <c r="B190" s="34" t="s">
+      <c r="B190" s="12" t="s">
         <v>339</v>
       </c>
     </row>
@@ -5402,215 +5483,215 @@
       <c r="A191" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="B191" s="35" t="s">
+      <c r="B191" s="33" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="192" spans="1:2">
-      <c r="A192" s="36" t="s">
+      <c r="A192" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="B192" s="37" t="s">
+      <c r="B192" s="35" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="193" spans="1:2">
-      <c r="A193" s="36" t="s">
+      <c r="A193" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="B193" s="38" t="s">
+      <c r="B193" s="36" t="s">
         <v>342</v>
       </c>
     </row>
     <row r="194" spans="1:2">
-      <c r="A194" s="36" t="s">
+      <c r="A194" s="34" t="s">
         <v>197</v>
       </c>
-      <c r="B194" s="19">
+      <c r="B194" s="18">
         <v>2</v>
       </c>
     </row>
     <row r="195" spans="1:2">
-      <c r="A195" s="36" t="s">
+      <c r="A195" s="34" t="s">
         <v>198</v>
       </c>
-      <c r="B195" s="37" t="s">
+      <c r="B195" s="35" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="196" spans="1:2">
-      <c r="A196" s="36" t="s">
+      <c r="A196" s="34" t="s">
         <v>200</v>
       </c>
-      <c r="B196" s="18" t="s">
+      <c r="B196" s="17" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="197" spans="1:2">
-      <c r="A197" s="36" t="s">
+      <c r="A197" s="34" t="s">
         <v>202</v>
       </c>
-      <c r="B197" s="19">
+      <c r="B197" s="18">
         <v>100</v>
       </c>
     </row>
     <row r="198" spans="1:2">
-      <c r="A198" s="36" t="s">
+      <c r="A198" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="B198" s="19" t="s">
+      <c r="B198" s="18" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="199" spans="1:2">
-      <c r="A199" s="36" t="s">
+      <c r="A199" s="34" t="s">
         <v>344</v>
       </c>
-      <c r="B199" s="39" t="s">
+      <c r="B199" s="37" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="200" spans="1:2">
-      <c r="A200" s="36" t="s">
+      <c r="A200" s="34" t="s">
         <v>346</v>
       </c>
-      <c r="B200" s="39" t="s">
+      <c r="B200" s="37" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="201" spans="1:2">
-      <c r="A201" s="36" t="s">
+      <c r="A201" s="34" t="s">
         <v>348</v>
       </c>
-      <c r="B201" s="39" t="s">
+      <c r="B201" s="37" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="202" spans="1:2">
-      <c r="A202" s="36" t="s">
+      <c r="A202" s="34" t="s">
         <v>350</v>
       </c>
-      <c r="B202" s="19">
+      <c r="B202" s="18">
         <v>200</v>
       </c>
     </row>
     <row r="203" spans="1:2">
-      <c r="A203" s="36" t="s">
+      <c r="A203" s="34" t="s">
         <v>351</v>
       </c>
-      <c r="B203" s="19">
+      <c r="B203" s="18">
         <v>3</v>
       </c>
     </row>
     <row r="204" spans="1:2">
-      <c r="A204" s="36" t="s">
+      <c r="A204" s="34" t="s">
         <v>352</v>
       </c>
-      <c r="B204" s="19" t="s">
+      <c r="B204" s="18" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="205" spans="1:2">
-      <c r="A205" s="40" t="s">
+      <c r="A205" s="38" t="s">
         <v>354</v>
       </c>
-      <c r="B205" s="19">
+      <c r="B205" s="18">
         <v>150</v>
       </c>
     </row>
     <row r="206" spans="1:2">
-      <c r="A206" s="40" t="s">
+      <c r="A206" s="38" t="s">
         <v>355</v>
       </c>
-      <c r="B206" s="19">
+      <c r="B206" s="18">
         <v>250</v>
       </c>
     </row>
     <row r="207" spans="1:2">
-      <c r="A207" s="40" t="s">
+      <c r="A207" s="38" t="s">
         <v>356</v>
       </c>
-      <c r="B207" s="19" t="s">
+      <c r="B207" s="18" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="208" spans="1:2">
-      <c r="A208" s="40" t="s">
+      <c r="A208" s="38" t="s">
         <v>358</v>
       </c>
-      <c r="B208" s="19">
+      <c r="B208" s="18">
         <v>123562</v>
       </c>
     </row>
     <row r="209" spans="1:2">
-      <c r="A209" s="40" t="s">
+      <c r="A209" s="38" t="s">
         <v>359</v>
       </c>
-      <c r="B209" s="19">
+      <c r="B209" s="18">
         <v>2</v>
       </c>
     </row>
     <row r="210" spans="1:2">
-      <c r="A210" s="40" t="s">
+      <c r="A210" s="38" t="s">
         <v>360</v>
       </c>
-      <c r="B210" s="19">
+      <c r="B210" s="18">
         <v>3</v>
       </c>
     </row>
     <row r="211" spans="1:2">
-      <c r="A211" s="40" t="s">
+      <c r="A211" s="38" t="s">
         <v>361</v>
       </c>
-      <c r="B211" s="19">
+      <c r="B211" s="18">
         <v>4</v>
       </c>
     </row>
     <row r="212" spans="1:2">
-      <c r="A212" s="40" t="s">
+      <c r="A212" s="38" t="s">
         <v>362</v>
       </c>
-      <c r="B212" s="38" t="s">
+      <c r="B212" s="36" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="213" spans="1:2">
-      <c r="A213" s="40" t="s">
+      <c r="A213" s="38" t="s">
         <v>364</v>
       </c>
-      <c r="B213" s="18" t="s">
+      <c r="B213" s="17" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="214" spans="1:2">
-      <c r="A214" s="40" t="s">
+      <c r="A214" s="38" t="s">
         <v>366</v>
       </c>
-      <c r="B214" s="38" t="s">
+      <c r="B214" s="36" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="215" spans="1:2">
-      <c r="A215" s="40" t="s">
+      <c r="A215" s="38" t="s">
         <v>368</v>
       </c>
-      <c r="B215" s="19">
+      <c r="B215" s="18">
         <v>50</v>
       </c>
     </row>
     <row r="216" spans="1:2">
-      <c r="A216" s="40" t="s">
+      <c r="A216" s="38" t="s">
         <v>369</v>
       </c>
-      <c r="B216" s="19">
+      <c r="B216" s="18">
         <v>50</v>
       </c>
     </row>
     <row r="217" spans="1:2">
-      <c r="A217" s="40" t="s">
+      <c r="A217" s="38" t="s">
         <v>370</v>
       </c>
-      <c r="B217" s="38" t="s">
+      <c r="B217" s="36" t="s">
         <v>71</v>
       </c>
     </row>
@@ -5618,63 +5699,63 @@
       <c r="A218" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="B218" s="25" t="s">
+      <c r="B218" s="24" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="219" spans="1:2">
-      <c r="A219" s="31" t="s">
+      <c r="A219" s="30" t="s">
         <v>371</v>
       </c>
-      <c r="B219" s="41" t="s">
+      <c r="B219" s="39" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="220" spans="1:2">
-      <c r="A220" s="31" t="s">
+      <c r="A220" s="30" t="s">
         <v>372</v>
       </c>
-      <c r="B220" s="25" t="s">
+      <c r="B220" s="24" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="221" spans="1:2">
-      <c r="A221" s="31" t="s">
+      <c r="A221" s="30" t="s">
         <v>374</v>
       </c>
-      <c r="B221" s="25" t="s">
+      <c r="B221" s="24" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="222" spans="1:2">
-      <c r="A222" s="42" t="s">
+      <c r="A222" s="40" t="s">
         <v>376</v>
       </c>
-      <c r="B222" s="41" t="s">
+      <c r="B222" s="39" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="223" spans="1:2">
-      <c r="A223" s="42" t="s">
+      <c r="A223" s="40" t="s">
         <v>378</v>
       </c>
-      <c r="B223" s="41" t="s">
+      <c r="B223" s="39" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="224" spans="1:2">
-      <c r="A224" s="43" t="s">
+      <c r="A224" s="41" t="s">
         <v>380</v>
       </c>
-      <c r="B224" s="44" t="s">
+      <c r="B224" s="42" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="225" spans="1:2">
-      <c r="A225" s="42" t="s">
+      <c r="A225" s="40" t="s">
         <v>382</v>
       </c>
-      <c r="B225" s="45" t="s">
+      <c r="B225" s="43" t="s">
         <v>383</v>
       </c>
     </row>
@@ -5866,7 +5947,7 @@
       <c r="A249" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="B249" s="46" t="s">
+      <c r="B249" s="44" t="s">
         <v>419</v>
       </c>
     </row>
@@ -6095,10 +6176,10 @@
       </c>
     </row>
     <row r="278" spans="1:2">
-      <c r="A278" s="26" t="s">
+      <c r="A278" s="25" t="s">
         <v>467</v>
       </c>
-      <c r="B278" s="25" t="s">
+      <c r="B278" s="24" t="s">
         <v>468</v>
       </c>
     </row>
@@ -6106,7 +6187,7 @@
       <c r="A279" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B279" s="25" t="s">
+      <c r="B279" s="24" t="s">
         <v>59</v>
       </c>
     </row>
@@ -6146,12 +6227,12 @@
       <c r="A284" s="8" t="s">
         <v>477</v>
       </c>
-      <c r="B284" s="47" t="s">
+      <c r="B284" s="45" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="285" spans="1:2">
-      <c r="A285" s="48" t="s">
+      <c r="A285" s="46" t="s">
         <v>479</v>
       </c>
       <c r="B285" s="7" t="s">
@@ -6159,7 +6240,7 @@
       </c>
     </row>
     <row r="286" spans="1:2">
-      <c r="A286" s="48" t="s">
+      <c r="A286" s="46" t="s">
         <v>481</v>
       </c>
       <c r="B286" s="7" t="s">
@@ -6167,7 +6248,7 @@
       </c>
     </row>
     <row r="287" spans="1:2">
-      <c r="A287" s="48" t="s">
+      <c r="A287" s="46" t="s">
         <v>483</v>
       </c>
       <c r="B287" s="7" t="s">
@@ -6175,7 +6256,7 @@
       </c>
     </row>
     <row r="288" spans="1:2">
-      <c r="A288" s="48" t="s">
+      <c r="A288" s="46" t="s">
         <v>485</v>
       </c>
       <c r="B288" s="7" t="s">
@@ -6183,7 +6264,7 @@
       </c>
     </row>
     <row r="289" spans="1:2">
-      <c r="A289" s="48" t="s">
+      <c r="A289" s="46" t="s">
         <v>487</v>
       </c>
       <c r="B289" s="7" t="s">
@@ -6191,7 +6272,7 @@
       </c>
     </row>
     <row r="290" spans="1:2">
-      <c r="A290" s="48" t="s">
+      <c r="A290" s="46" t="s">
         <v>489</v>
       </c>
       <c r="B290" s="7" t="s">
@@ -6199,7 +6280,7 @@
       </c>
     </row>
     <row r="291" spans="1:2">
-      <c r="A291" s="48" t="s">
+      <c r="A291" s="46" t="s">
         <v>491</v>
       </c>
       <c r="B291" s="7" t="s">
@@ -6426,7 +6507,7 @@
       <c r="A319" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="B319" s="49" t="s">
+      <c r="B319" s="47" t="s">
         <v>543</v>
       </c>
     </row>
@@ -6559,58 +6640,58 @@
       </c>
     </row>
     <row r="336" spans="1:2">
-      <c r="A336" s="30" t="s">
+      <c r="A336" s="29" t="s">
         <v>573</v>
       </c>
-      <c r="B336" s="29" t="s">
+      <c r="B336" s="28" t="s">
         <v>574</v>
       </c>
     </row>
     <row r="337" spans="1:2">
-      <c r="A337" s="30" t="s">
+      <c r="A337" s="29" t="s">
         <v>575</v>
       </c>
-      <c r="B337" s="29" t="s">
+      <c r="B337" s="28" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="338" spans="1:2">
-      <c r="A338" s="30" t="s">
+      <c r="A338" s="29" t="s">
         <v>576</v>
       </c>
-      <c r="B338" s="29" t="s">
+      <c r="B338" s="28" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="339" spans="1:2">
-      <c r="A339" s="30" t="s">
+      <c r="A339" s="29" t="s">
         <v>577</v>
       </c>
-      <c r="B339" s="29" t="s">
+      <c r="B339" s="28" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="340" spans="1:2">
-      <c r="A340" s="30" t="s">
+      <c r="A340" s="29" t="s">
         <v>578</v>
       </c>
-      <c r="B340" s="29" t="s">
+      <c r="B340" s="28" t="s">
         <v>579</v>
       </c>
     </row>
     <row r="341" spans="1:2">
-      <c r="A341" s="30" t="s">
+      <c r="A341" s="29" t="s">
         <v>580</v>
       </c>
-      <c r="B341" s="29" t="s">
+      <c r="B341" s="28" t="s">
         <v>579</v>
       </c>
     </row>
     <row r="342" spans="1:2">
-      <c r="A342" s="30" t="s">
+      <c r="A342" s="29" t="s">
         <v>581</v>
       </c>
-      <c r="B342" s="29" t="s">
+      <c r="B342" s="28" t="s">
         <v>579</v>
       </c>
     </row>
@@ -6722,7 +6803,7 @@
       <c r="A356" s="2" t="s">
         <v>607</v>
       </c>
-      <c r="B356" s="25" t="s">
+      <c r="B356" s="24" t="s">
         <v>608</v>
       </c>
     </row>
@@ -6735,103 +6816,103 @@
       </c>
     </row>
     <row r="358" spans="1:2">
-      <c r="A358" s="26" t="s">
+      <c r="A358" s="25" t="s">
         <v>611</v>
       </c>
-      <c r="B358" s="27" t="s">
+      <c r="B358" s="26" t="s">
         <v>612</v>
       </c>
     </row>
     <row r="359" spans="1:2">
-      <c r="A359" s="26" t="s">
+      <c r="A359" s="25" t="s">
         <v>613</v>
       </c>
-      <c r="B359" s="27" t="s">
+      <c r="B359" s="26" t="s">
         <v>614</v>
       </c>
     </row>
     <row r="360" spans="1:2">
-      <c r="A360" s="26" t="s">
+      <c r="A360" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="B360" s="25">
+      <c r="B360" s="24">
         <v>10</v>
       </c>
     </row>
     <row r="361" spans="1:2">
-      <c r="A361" s="26" t="s">
+      <c r="A361" s="25" t="s">
         <v>616</v>
       </c>
-      <c r="B361" s="25">
+      <c r="B361" s="24">
         <v>1000</v>
       </c>
     </row>
     <row r="362" spans="1:2">
-      <c r="A362" s="26" t="s">
+      <c r="A362" s="25" t="s">
         <v>617</v>
       </c>
-      <c r="B362" s="50">
+      <c r="B362" s="48">
         <v>5</v>
       </c>
     </row>
     <row r="363" spans="1:2">
-      <c r="A363" s="26" t="s">
+      <c r="A363" s="25" t="s">
         <v>618</v>
       </c>
-      <c r="B363" s="25">
+      <c r="B363" s="24">
         <v>1000</v>
       </c>
     </row>
     <row r="364" spans="1:2">
-      <c r="A364" s="26" t="s">
+      <c r="A364" s="25" t="s">
         <v>619</v>
       </c>
-      <c r="B364" s="25" t="s">
+      <c r="B364" s="24" t="s">
         <v>620</v>
       </c>
     </row>
     <row r="365" spans="1:2">
-      <c r="A365" s="26" t="s">
+      <c r="A365" s="25" t="s">
         <v>621</v>
       </c>
-      <c r="B365" s="25" t="s">
+      <c r="B365" s="24" t="s">
         <v>622</v>
       </c>
     </row>
     <row r="366" spans="1:2">
-      <c r="A366" s="26" t="s">
+      <c r="A366" s="25" t="s">
         <v>623</v>
       </c>
-      <c r="B366" s="25" t="s">
+      <c r="B366" s="24" t="s">
         <v>624</v>
       </c>
     </row>
     <row r="367" spans="1:2">
-      <c r="A367" s="26" t="s">
+      <c r="A367" s="25" t="s">
         <v>625</v>
       </c>
-      <c r="B367" s="25">
+      <c r="B367" s="24">
         <v>10000039</v>
       </c>
     </row>
     <row r="368" spans="1:2">
-      <c r="A368" s="26" t="s">
+      <c r="A368" s="25" t="s">
         <v>626</v>
       </c>
-      <c r="B368" s="27" t="s">
+      <c r="B368" s="26" t="s">
         <v>627</v>
       </c>
     </row>
     <row r="369" spans="1:2">
-      <c r="A369" s="26" t="s">
+      <c r="A369" s="25" t="s">
         <v>628</v>
       </c>
-      <c r="B369" s="27" t="s">
+      <c r="B369" s="26" t="s">
         <v>629</v>
       </c>
     </row>
     <row r="370" spans="1:2">
-      <c r="A370" s="26" t="s">
+      <c r="A370" s="25" t="s">
         <v>630</v>
       </c>
       <c r="B370" s="7" t="s">
@@ -6839,7 +6920,7 @@
       </c>
     </row>
     <row r="371" spans="1:2">
-      <c r="A371" s="26" t="s">
+      <c r="A371" s="25" t="s">
         <v>632</v>
       </c>
       <c r="B371" s="7" t="s">
@@ -6847,7 +6928,7 @@
       </c>
     </row>
     <row r="372" spans="1:2">
-      <c r="A372" s="26" t="s">
+      <c r="A372" s="25" t="s">
         <v>634</v>
       </c>
       <c r="B372" s="7" t="s">
@@ -6855,7 +6936,7 @@
       </c>
     </row>
     <row r="373" spans="1:2">
-      <c r="A373" s="26" t="s">
+      <c r="A373" s="25" t="s">
         <v>636</v>
       </c>
       <c r="B373" s="7" t="s">
@@ -6863,7 +6944,7 @@
       </c>
     </row>
     <row r="374" spans="1:2">
-      <c r="A374" s="26" t="s">
+      <c r="A374" s="25" t="s">
         <v>638</v>
       </c>
       <c r="B374" s="7" t="s">
@@ -6871,7 +6952,7 @@
       </c>
     </row>
     <row r="375" spans="1:2">
-      <c r="A375" s="26" t="s">
+      <c r="A375" s="25" t="s">
         <v>640</v>
       </c>
       <c r="B375" s="7" t="s">
@@ -6879,7 +6960,7 @@
       </c>
     </row>
     <row r="376" spans="1:2">
-      <c r="A376" s="26" t="s">
+      <c r="A376" s="25" t="s">
         <v>642</v>
       </c>
       <c r="B376" s="7" t="s">
@@ -6887,7 +6968,7 @@
       </c>
     </row>
     <row r="377" spans="1:2">
-      <c r="A377" s="26" t="s">
+      <c r="A377" s="25" t="s">
         <v>643</v>
       </c>
       <c r="B377" s="7" t="s">
@@ -6895,7 +6976,7 @@
       </c>
     </row>
     <row r="378" spans="1:2">
-      <c r="A378" s="26" t="s">
+      <c r="A378" s="25" t="s">
         <v>645</v>
       </c>
       <c r="B378" s="7" t="s">
@@ -6903,7 +6984,7 @@
       </c>
     </row>
     <row r="379" spans="1:2">
-      <c r="A379" s="26" t="s">
+      <c r="A379" s="25" t="s">
         <v>647</v>
       </c>
       <c r="B379" s="7" t="s">
@@ -6911,7 +6992,7 @@
       </c>
     </row>
     <row r="380" spans="1:2">
-      <c r="A380" s="26" t="s">
+      <c r="A380" s="25" t="s">
         <v>649</v>
       </c>
       <c r="B380" s="7" t="s">
@@ -6919,7 +7000,7 @@
       </c>
     </row>
     <row r="381" spans="1:2">
-      <c r="A381" s="26" t="s">
+      <c r="A381" s="25" t="s">
         <v>650</v>
       </c>
       <c r="B381" s="7" t="s">
@@ -6927,7 +7008,7 @@
       </c>
     </row>
     <row r="382" spans="1:2">
-      <c r="A382" s="26" t="s">
+      <c r="A382" s="25" t="s">
         <v>652</v>
       </c>
       <c r="B382" s="7" t="s">
@@ -6935,7 +7016,7 @@
       </c>
     </row>
     <row r="383" spans="1:2">
-      <c r="A383" s="26" t="s">
+      <c r="A383" s="25" t="s">
         <v>654</v>
       </c>
       <c r="B383" s="7" t="s">
@@ -6943,7 +7024,7 @@
       </c>
     </row>
     <row r="384" spans="1:2">
-      <c r="A384" s="26" t="s">
+      <c r="A384" s="25" t="s">
         <v>656</v>
       </c>
       <c r="B384" s="7" t="s">
@@ -6951,7 +7032,7 @@
       </c>
     </row>
     <row r="385" spans="1:2">
-      <c r="A385" s="26" t="s">
+      <c r="A385" s="25" t="s">
         <v>658</v>
       </c>
       <c r="B385" s="7" t="s">
@@ -6959,7 +7040,7 @@
       </c>
     </row>
     <row r="386" spans="1:2">
-      <c r="A386" s="26" t="s">
+      <c r="A386" s="25" t="s">
         <v>660</v>
       </c>
       <c r="B386" s="7" t="s">
@@ -6967,7 +7048,7 @@
       </c>
     </row>
     <row r="387" spans="1:2">
-      <c r="A387" s="26" t="s">
+      <c r="A387" s="25" t="s">
         <v>662</v>
       </c>
       <c r="B387" s="7" t="s">
@@ -6975,7 +7056,7 @@
       </c>
     </row>
     <row r="388" spans="1:2">
-      <c r="A388" s="26" t="s">
+      <c r="A388" s="25" t="s">
         <v>664</v>
       </c>
       <c r="B388" s="7" t="s">
@@ -6983,7 +7064,7 @@
       </c>
     </row>
     <row r="389" spans="1:2">
-      <c r="A389" s="26" t="s">
+      <c r="A389" s="25" t="s">
         <v>666</v>
       </c>
       <c r="B389" s="7" t="s">
@@ -6991,7 +7072,7 @@
       </c>
     </row>
     <row r="390" spans="1:2">
-      <c r="A390" s="26" t="s">
+      <c r="A390" s="25" t="s">
         <v>668</v>
       </c>
       <c r="B390" s="7" t="s">
@@ -6999,7 +7080,7 @@
       </c>
     </row>
     <row r="391" spans="1:2">
-      <c r="A391" s="26" t="s">
+      <c r="A391" s="25" t="s">
         <v>670</v>
       </c>
       <c r="B391" s="7" t="s">
@@ -7007,7 +7088,7 @@
       </c>
     </row>
     <row r="392" spans="1:2">
-      <c r="A392" s="26" t="s">
+      <c r="A392" s="25" t="s">
         <v>672</v>
       </c>
       <c r="B392" s="7" t="s">
@@ -7015,7 +7096,7 @@
       </c>
     </row>
     <row r="393" spans="1:2">
-      <c r="A393" s="26" t="s">
+      <c r="A393" s="25" t="s">
         <v>674</v>
       </c>
       <c r="B393" s="7" t="s">
@@ -7023,7 +7104,7 @@
       </c>
     </row>
     <row r="394" spans="1:2">
-      <c r="A394" s="26" t="s">
+      <c r="A394" s="25" t="s">
         <v>676</v>
       </c>
       <c r="B394" s="7" t="s">
@@ -7031,7 +7112,7 @@
       </c>
     </row>
     <row r="395" spans="1:2">
-      <c r="A395" s="26" t="s">
+      <c r="A395" s="25" t="s">
         <v>678</v>
       </c>
       <c r="B395" s="7" t="s">
@@ -7039,7 +7120,7 @@
       </c>
     </row>
     <row r="396" spans="1:2">
-      <c r="A396" s="26" t="s">
+      <c r="A396" s="25" t="s">
         <v>680</v>
       </c>
       <c r="B396" s="7" t="s">
@@ -7047,7 +7128,7 @@
       </c>
     </row>
     <row r="397" spans="1:2">
-      <c r="A397" s="26" t="s">
+      <c r="A397" s="25" t="s">
         <v>682</v>
       </c>
       <c r="B397" s="7" t="s">
@@ -7055,7 +7136,7 @@
       </c>
     </row>
     <row r="398" spans="1:2">
-      <c r="A398" s="26" t="s">
+      <c r="A398" s="25" t="s">
         <v>684</v>
       </c>
       <c r="B398" s="7" t="s">
@@ -7063,7 +7144,7 @@
       </c>
     </row>
     <row r="399" spans="1:2">
-      <c r="A399" s="26" t="s">
+      <c r="A399" s="25" t="s">
         <v>686</v>
       </c>
       <c r="B399" s="7" t="s">
@@ -7071,7 +7152,7 @@
       </c>
     </row>
     <row r="400" spans="1:2">
-      <c r="A400" s="26" t="s">
+      <c r="A400" s="25" t="s">
         <v>688</v>
       </c>
       <c r="B400" s="7" t="s">
@@ -7079,7 +7160,7 @@
       </c>
     </row>
     <row r="401" spans="1:2">
-      <c r="A401" s="26" t="s">
+      <c r="A401" s="25" t="s">
         <v>690</v>
       </c>
       <c r="B401" s="7" t="s">
@@ -7087,7 +7168,7 @@
       </c>
     </row>
     <row r="402" spans="1:2">
-      <c r="A402" s="26" t="s">
+      <c r="A402" s="25" t="s">
         <v>692</v>
       </c>
       <c r="B402" s="7" t="s">
@@ -7095,7 +7176,7 @@
       </c>
     </row>
     <row r="403" spans="1:2">
-      <c r="A403" s="26" t="s">
+      <c r="A403" s="25" t="s">
         <v>694</v>
       </c>
       <c r="B403" s="7" t="s">
@@ -7103,7 +7184,7 @@
       </c>
     </row>
     <row r="404" spans="1:2">
-      <c r="A404" s="26" t="s">
+      <c r="A404" s="25" t="s">
         <v>696</v>
       </c>
       <c r="B404" s="7" t="s">
@@ -7111,7 +7192,7 @@
       </c>
     </row>
     <row r="405" spans="1:2">
-      <c r="A405" s="26" t="s">
+      <c r="A405" s="25" t="s">
         <v>698</v>
       </c>
       <c r="B405" s="7" t="s">
@@ -7119,7 +7200,7 @@
       </c>
     </row>
     <row r="406" spans="1:2">
-      <c r="A406" s="26" t="s">
+      <c r="A406" s="25" t="s">
         <v>700</v>
       </c>
       <c r="B406" s="7" t="s">
@@ -7127,7 +7208,7 @@
       </c>
     </row>
     <row r="407" spans="1:2">
-      <c r="A407" s="26" t="s">
+      <c r="A407" s="25" t="s">
         <v>702</v>
       </c>
       <c r="B407" s="7" t="s">
@@ -7135,7 +7216,7 @@
       </c>
     </row>
     <row r="408" spans="1:2">
-      <c r="A408" s="26" t="s">
+      <c r="A408" s="25" t="s">
         <v>704</v>
       </c>
       <c r="B408" s="7" t="s">
@@ -7279,291 +7360,499 @@
       </c>
     </row>
     <row r="426" spans="1:2">
-      <c r="A426" s="12" t="s">
+      <c r="A426" s="11" t="s">
         <v>734</v>
       </c>
-      <c r="B426" s="14" t="s">
+      <c r="B426" s="13" t="s">
         <v>735</v>
       </c>
     </row>
     <row r="427" spans="1:2">
-      <c r="A427" s="12" t="s">
+      <c r="A427" s="11" t="s">
         <v>736</v>
       </c>
-      <c r="B427" s="14" t="s">
+      <c r="B427" s="13" t="s">
         <v>737</v>
       </c>
     </row>
     <row r="428" spans="1:2">
-      <c r="A428" s="12" t="s">
+      <c r="A428" s="11" t="s">
         <v>738</v>
       </c>
-      <c r="B428" s="14" t="s">
+      <c r="B428" s="13" t="s">
         <v>739</v>
       </c>
     </row>
     <row r="429" spans="1:2">
-      <c r="A429" s="12" t="s">
+      <c r="A429" s="11" t="s">
         <v>740</v>
       </c>
-      <c r="B429" s="14" t="s">
+      <c r="B429" s="13" t="s">
         <v>741</v>
       </c>
     </row>
     <row r="430" spans="1:2">
-      <c r="A430" s="12" t="s">
+      <c r="A430" s="11" t="s">
         <v>742</v>
       </c>
-      <c r="B430" s="14" t="s">
+      <c r="B430" s="13" t="s">
         <v>743</v>
       </c>
     </row>
     <row r="431" spans="1:2">
-      <c r="A431" s="12" t="s">
+      <c r="A431" s="11" t="s">
         <v>744</v>
       </c>
-      <c r="B431" s="14" t="s">
+      <c r="B431" s="13" t="s">
         <v>745</v>
       </c>
     </row>
     <row r="432" spans="1:2">
-      <c r="A432" s="12" t="s">
+      <c r="A432" s="11" t="s">
         <v>746</v>
       </c>
-      <c r="B432" s="14" t="s">
+      <c r="B432" s="13" t="s">
         <v>747</v>
       </c>
     </row>
     <row r="433" spans="1:2">
-      <c r="A433" s="12" t="s">
+      <c r="A433" s="11" t="s">
         <v>748</v>
       </c>
-      <c r="B433" s="14" t="s">
+      <c r="B433" s="13" t="s">
         <v>749</v>
       </c>
     </row>
     <row r="434" spans="1:2">
-      <c r="A434" s="12" t="s">
+      <c r="A434" s="11" t="s">
         <v>750</v>
       </c>
-      <c r="B434" s="14" t="s">
+      <c r="B434" s="13" t="s">
         <v>751</v>
       </c>
     </row>
     <row r="435" spans="1:2">
-      <c r="A435" s="12" t="s">
+      <c r="A435" s="11" t="s">
         <v>752</v>
       </c>
-      <c r="B435" s="14" t="s">
+      <c r="B435" s="13" t="s">
         <v>753</v>
       </c>
     </row>
     <row r="436" spans="1:2">
-      <c r="A436" s="12" t="s">
+      <c r="A436" s="11" t="s">
         <v>754</v>
       </c>
-      <c r="B436" s="14" t="s">
+      <c r="B436" s="13" t="s">
         <v>755</v>
       </c>
     </row>
     <row r="437" spans="1:2">
-      <c r="A437" s="12" t="s">
+      <c r="A437" s="11" t="s">
         <v>756</v>
       </c>
-      <c r="B437" s="14" t="s">
+      <c r="B437" s="13" t="s">
         <v>757</v>
       </c>
     </row>
     <row r="438" spans="1:2">
-      <c r="A438" s="12" t="s">
+      <c r="A438" s="11" t="s">
         <v>758</v>
       </c>
-      <c r="B438" s="14" t="s">
+      <c r="B438" s="13" t="s">
         <v>759</v>
       </c>
     </row>
     <row r="439" spans="1:2">
-      <c r="A439" s="12" t="s">
+      <c r="A439" s="11" t="s">
         <v>760</v>
       </c>
-      <c r="B439" s="14" t="s">
+      <c r="B439" s="13" t="s">
         <v>761</v>
       </c>
     </row>
     <row r="440" spans="1:2">
-      <c r="A440" s="30" t="s">
+      <c r="A440" s="29" t="s">
         <v>762</v>
       </c>
-      <c r="B440" s="29" t="s">
+      <c r="B440" s="28" t="s">
         <v>763</v>
       </c>
     </row>
     <row r="441" spans="1:2">
-      <c r="A441" s="51" t="s">
+      <c r="A441" s="49" t="s">
         <v>764</v>
       </c>
-      <c r="B441" s="52" t="s">
+      <c r="B441" s="50" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="442" spans="1:2">
-      <c r="A442" s="51" t="s">
+      <c r="A442" s="49" t="s">
         <v>765</v>
       </c>
-      <c r="B442" s="53" t="s">
+      <c r="B442" s="50" t="s">
         <v>766</v>
       </c>
     </row>
     <row r="443" spans="1:2">
-      <c r="A443" s="51" t="s">
+      <c r="A443" s="49" t="s">
         <v>767</v>
       </c>
-      <c r="B443" s="53" t="s">
+      <c r="B443" s="50" t="s">
         <v>768</v>
       </c>
     </row>
     <row r="444" spans="1:2">
-      <c r="A444" s="51" t="s">
+      <c r="A444" s="49" t="s">
         <v>769</v>
       </c>
-      <c r="B444" s="53" t="s">
+      <c r="B444" s="50" t="s">
         <v>768</v>
       </c>
     </row>
     <row r="445" spans="1:2">
-      <c r="A445" s="51" t="s">
+      <c r="A445" s="49" t="s">
         <v>770</v>
       </c>
-      <c r="B445" s="53" t="s">
+      <c r="B445" s="50" t="s">
         <v>768</v>
       </c>
     </row>
     <row r="446" spans="1:2">
-      <c r="A446" s="51" t="s">
+      <c r="A446" s="49" t="s">
         <v>771</v>
       </c>
-      <c r="B446" s="54" t="s">
+      <c r="B446" s="51" t="s">
         <v>772</v>
       </c>
     </row>
     <row r="447" spans="1:2">
-      <c r="A447" s="51" t="s">
+      <c r="A447" s="49" t="s">
         <v>773</v>
       </c>
-      <c r="B447" s="54" t="s">
+      <c r="B447" s="51" t="s">
         <v>774</v>
       </c>
     </row>
     <row r="448" spans="1:2">
-      <c r="A448" s="51" t="s">
+      <c r="A448" s="49" t="s">
         <v>775</v>
       </c>
-      <c r="B448" s="53" t="s">
+      <c r="B448" s="50" t="s">
         <v>776</v>
       </c>
     </row>
     <row r="449" spans="1:2">
-      <c r="A449" s="51" t="s">
+      <c r="A449" s="49" t="s">
         <v>777</v>
       </c>
-      <c r="B449" s="53" t="s">
+      <c r="B449" s="50" t="s">
         <v>778</v>
       </c>
     </row>
     <row r="450" spans="1:2">
-      <c r="A450" s="51" t="s">
+      <c r="A450" s="49" t="s">
         <v>564</v>
       </c>
-      <c r="B450" s="55" t="s">
+      <c r="B450" s="51" t="s">
         <v>564</v>
       </c>
     </row>
     <row r="451" spans="1:2">
-      <c r="A451" s="51" t="s">
+      <c r="A451" s="49" t="s">
         <v>561</v>
       </c>
-      <c r="B451" s="55" t="s">
+      <c r="B451" s="51" t="s">
         <v>561</v>
       </c>
     </row>
     <row r="452" spans="1:2">
-      <c r="A452" s="56" t="s">
+      <c r="A452" s="52" t="s">
         <v>75</v>
       </c>
-      <c r="B452" s="57" t="s">
+      <c r="B452" s="53" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="453" spans="1:2">
-      <c r="A453" s="56" t="s">
+      <c r="A453" s="52" t="s">
         <v>779</v>
       </c>
-      <c r="B453" s="57" t="s">
+      <c r="B453" s="53" t="s">
         <v>780</v>
       </c>
     </row>
     <row r="454" spans="1:2">
-      <c r="A454" s="51" t="s">
+      <c r="A454" s="49" t="s">
         <v>781</v>
       </c>
-      <c r="B454" s="58" t="s">
+      <c r="B454" s="54" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="455" spans="1:2">
-      <c r="A455" s="51" t="s">
+      <c r="A455" s="49" t="s">
         <v>782</v>
       </c>
-      <c r="B455" s="58" t="s">
+      <c r="B455" s="54" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="456" spans="1:2">
-      <c r="A456" s="59" t="s">
+      <c r="A456" s="49" t="s">
         <v>371</v>
       </c>
-      <c r="B456" s="55" t="s">
+      <c r="B456" s="51" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="457" spans="1:2">
-      <c r="A457" s="59" t="s">
+      <c r="A457" s="49" t="s">
         <v>783</v>
       </c>
-      <c r="B457" s="55" t="s">
+      <c r="B457" s="51" t="s">
         <v>783</v>
       </c>
     </row>
     <row r="458" spans="1:2">
-      <c r="A458" s="59" t="s">
+      <c r="A458" s="49" t="s">
         <v>784</v>
       </c>
-      <c r="B458" s="55" t="s">
+      <c r="B458" s="51" t="s">
         <v>785</v>
       </c>
     </row>
     <row r="459" spans="1:2">
-      <c r="A459" s="59" t="s">
+      <c r="A459" s="49" t="s">
         <v>786</v>
       </c>
-      <c r="B459" s="52" t="s">
+      <c r="B459" s="50" t="s">
         <v>787</v>
       </c>
     </row>
     <row r="460" spans="1:2">
-      <c r="A460" s="51" t="s">
+      <c r="A460" s="49" t="s">
         <v>788</v>
       </c>
-      <c r="B460" s="53" t="s">
+      <c r="B460" s="50" t="s">
         <v>789</v>
       </c>
     </row>
     <row r="461" spans="1:2">
-      <c r="A461" s="51" t="s">
+      <c r="A461" s="49" t="s">
         <v>790</v>
       </c>
-      <c r="B461" s="53" t="s">
+      <c r="B461" s="50" t="s">
         <v>791</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2">
+      <c r="A462" s="55" t="s">
+        <v>359</v>
+      </c>
+      <c r="B462" s="55">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="463" spans="1:2">
+      <c r="A463" s="55" t="s">
+        <v>360</v>
+      </c>
+      <c r="B463" s="55">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="464" spans="1:2">
+      <c r="A464" s="55" t="s">
+        <v>361</v>
+      </c>
+      <c r="B464" s="55">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="465" spans="1:2">
+      <c r="A465" s="56" t="s">
+        <v>354</v>
+      </c>
+      <c r="B465" s="56">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2">
+      <c r="A466" s="56" t="s">
+        <v>355</v>
+      </c>
+      <c r="B466" s="56">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="467" spans="1:2">
+      <c r="A467" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="B467" s="7" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2">
+      <c r="A468" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="B468" s="7" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="469" spans="1:2">
+      <c r="A469" s="2" t="s">
+        <v>796</v>
+      </c>
+      <c r="B469" s="7" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2">
+      <c r="A470" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="B470" s="7" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="471" spans="1:2">
+      <c r="A471" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B471" s="7" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="472" spans="1:2">
+      <c r="A472" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="B472" s="7" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2">
+      <c r="A473" s="2" t="s">
+        <v>801</v>
+      </c>
+      <c r="B473" s="7" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="474" spans="1:2">
+      <c r="A474" s="2" t="s">
+        <v>802</v>
+      </c>
+      <c r="B474" s="7" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="475" spans="1:2">
+      <c r="A475" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="B475" s="7" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2">
+      <c r="A476" s="2" t="s">
+        <v>759</v>
+      </c>
+      <c r="B476" s="7" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="477" spans="1:2">
+      <c r="A477" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="B477" s="7" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="478" spans="1:2">
+      <c r="A478" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="B478" s="7" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="479" spans="1:2">
+      <c r="A479" s="2" t="s">
+        <v>809</v>
+      </c>
+      <c r="B479" s="44" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="480" spans="1:2">
+      <c r="A480" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="B480" s="7" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="481" spans="1:2">
+      <c r="A481" s="2" t="s">
+        <v>812</v>
+      </c>
+      <c r="B481" s="7" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="482" spans="1:2">
+      <c r="A482" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="B482" s="7" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="483" spans="1:2">
+      <c r="A483" s="2" t="s">
+        <v>815</v>
+      </c>
+      <c r="B483" s="7" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="484" spans="1:2">
+      <c r="A484" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="B484" s="7" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="485" spans="1:2">
+      <c r="A485" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="B485" s="7" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="486" spans="1:2">
+      <c r="A486" s="57" t="s">
+        <v>821</v>
+      </c>
+      <c r="B486" s="58" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="487" spans="1:2">
+      <c r="A487" s="57" t="s">
+        <v>823</v>
+      </c>
+      <c r="B487" s="58" t="s">
+        <v>808</v>
       </c>
     </row>
   </sheetData>
@@ -7576,9 +7865,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7592,34 +7881,34 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>792</v>
+        <v>824</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>793</v>
+        <v>825</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>794</v>
+        <v>826</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>795</v>
+        <v>827</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>796</v>
+        <v>828</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>797</v>
+        <v>829</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>798</v>
+        <v>830</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>799</v>
+        <v>831</v>
       </c>
     </row>
     <row r="6" spans="1:2">

</xml_diff>

<commit_message>
Updated Failure Fixes E2E Test Scenarios
Updated Failure Fixes E2E Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="832">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="835">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -2427,10 +2427,13 @@
     <t>PEELING</t>
   </si>
   <si>
+    <t>SourcePEELING</t>
+  </si>
+  <si>
     <t>00</t>
   </si>
   <si>
-    <t>Target</t>
+    <t>TargetPEELING</t>
   </si>
   <si>
     <t>RawMaterialSco</t>
@@ -2500,6 +2503,12 @@
   </si>
   <si>
     <t>OrderReleaseOption</t>
+  </si>
+  <si>
+    <t>SourceSLICING</t>
+  </si>
+  <si>
+    <t>TargetSLICING</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -3497,7 +3506,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3625,10 +3634,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="53">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3952,7 +3957,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B487"/>
+  <dimension ref="A1:B489"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="34.287037037037" customWidth="1"/>
@@ -7721,15 +7726,15 @@
     </row>
     <row r="471" spans="1:2">
       <c r="A471" s="2" t="s">
-        <v>484</v>
+        <v>799</v>
       </c>
       <c r="B471" s="7" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" s="2" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B472" s="7" t="s">
         <v>229</v>
@@ -7737,7 +7742,7 @@
     </row>
     <row r="473" spans="1:2">
       <c r="A473" s="2" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="B473" s="7" t="s">
         <v>281</v>
@@ -7745,7 +7750,7 @@
     </row>
     <row r="474" spans="1:2">
       <c r="A474" s="2" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="B474" s="7" t="s">
         <v>757</v>
@@ -7753,10 +7758,10 @@
     </row>
     <row r="475" spans="1:2">
       <c r="A475" s="2" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="B475" s="7" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
     </row>
     <row r="476" spans="1:2">
@@ -7769,47 +7774,47 @@
     </row>
     <row r="477" spans="1:2">
       <c r="A477" s="2" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="B477" s="7" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" s="2" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="B478" s="7" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" s="2" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="B479" s="44" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" s="2" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="B480" s="7" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" s="2" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B481" s="7" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
     </row>
     <row r="482" spans="1:2">
       <c r="A482" s="2" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="B482" s="7" t="s">
         <v>229</v>
@@ -7817,42 +7822,58 @@
     </row>
     <row r="483" spans="1:2">
       <c r="A483" s="2" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B483" s="7" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" s="2" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="B484" s="7" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" s="2" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="B485" s="7" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
     </row>
     <row r="486" spans="1:2">
-      <c r="A486" s="57" t="s">
-        <v>821</v>
-      </c>
-      <c r="B486" s="58" t="s">
+      <c r="A486" s="2" t="s">
         <v>822</v>
       </c>
+      <c r="B486" s="7" t="s">
+        <v>823</v>
+      </c>
     </row>
     <row r="487" spans="1:2">
-      <c r="A487" s="57" t="s">
-        <v>823</v>
-      </c>
-      <c r="B487" s="58" t="s">
-        <v>808</v>
+      <c r="A487" s="2" t="s">
+        <v>824</v>
+      </c>
+      <c r="B487" s="7" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="488" spans="1:2">
+      <c r="A488" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="B488" s="7" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="489" spans="1:2">
+      <c r="A489" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="B489" s="7" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -7881,34 +7902,34 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>825</v>
+        <v>828</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>826</v>
+        <v>829</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>827</v>
+        <v>830</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>828</v>
+        <v>831</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>829</v>
+        <v>832</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>830</v>
+        <v>833</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
     </row>
     <row r="6" spans="1:2">

</xml_diff>

<commit_message>
Added SubContract To Payment E2E Test SCeanrio And Failure Fixes
Added SubContract To Payment E2E Test SCeanrio And Failure Fixes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="835">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="834">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -2407,9 +2407,6 @@
   </si>
   <si>
     <t>SubcontractorName</t>
-  </si>
-  <si>
-    <t>ACT ON FINISHING (P) LTD</t>
   </si>
   <si>
     <t>GeneralExpense</t>
@@ -7697,44 +7694,44 @@
         <v>792</v>
       </c>
       <c r="B467" s="7" t="s">
-        <v>793</v>
+        <v>357</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="B468" s="7" t="s">
         <v>794</v>
-      </c>
-      <c r="B468" s="7" t="s">
-        <v>795</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="B469" s="7" t="s">
         <v>796</v>
-      </c>
-      <c r="B469" s="7" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" s="2" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B470" s="7" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="B471" s="7" t="s">
         <v>799</v>
-      </c>
-      <c r="B471" s="7" t="s">
-        <v>800</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" s="2" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B472" s="7" t="s">
         <v>229</v>
@@ -7742,7 +7739,7 @@
     </row>
     <row r="473" spans="1:2">
       <c r="A473" s="2" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="B473" s="7" t="s">
         <v>281</v>
@@ -7750,7 +7747,7 @@
     </row>
     <row r="474" spans="1:2">
       <c r="A474" s="2" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B474" s="7" t="s">
         <v>757</v>
@@ -7758,10 +7755,10 @@
     </row>
     <row r="475" spans="1:2">
       <c r="A475" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="B475" s="7" t="s">
         <v>804</v>
-      </c>
-      <c r="B475" s="7" t="s">
-        <v>805</v>
       </c>
     </row>
     <row r="476" spans="1:2">
@@ -7774,47 +7771,47 @@
     </row>
     <row r="477" spans="1:2">
       <c r="A477" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="B477" s="7" t="s">
         <v>806</v>
-      </c>
-      <c r="B477" s="7" t="s">
-        <v>807</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="B478" s="7" t="s">
         <v>808</v>
-      </c>
-      <c r="B478" s="7" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" s="2" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B479" s="44" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="B480" s="7" t="s">
         <v>811</v>
-      </c>
-      <c r="B480" s="7" t="s">
-        <v>812</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" s="2" t="s">
+        <v>812</v>
+      </c>
+      <c r="B481" s="7" t="s">
         <v>813</v>
-      </c>
-      <c r="B481" s="7" t="s">
-        <v>814</v>
       </c>
     </row>
     <row r="482" spans="1:2">
       <c r="A482" s="2" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="B482" s="7" t="s">
         <v>229</v>
@@ -7822,47 +7819,47 @@
     </row>
     <row r="483" spans="1:2">
       <c r="A483" s="2" t="s">
+        <v>815</v>
+      </c>
+      <c r="B483" s="7" t="s">
         <v>816</v>
-      </c>
-      <c r="B483" s="7" t="s">
-        <v>817</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="B484" s="7" t="s">
         <v>818</v>
-      </c>
-      <c r="B484" s="7" t="s">
-        <v>819</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" s="2" t="s">
+        <v>819</v>
+      </c>
+      <c r="B485" s="7" t="s">
         <v>820</v>
-      </c>
-      <c r="B485" s="7" t="s">
-        <v>821</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="B486" s="7" t="s">
         <v>822</v>
-      </c>
-      <c r="B486" s="7" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" s="2" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B487" s="7" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" s="2" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B488" s="7" t="s">
         <v>229</v>
@@ -7870,7 +7867,7 @@
     </row>
     <row r="489" spans="1:2">
       <c r="A489" s="2" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="B489" s="7" t="s">
         <v>148</v>
@@ -7902,34 +7899,34 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>827</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>828</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>829</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>830</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>831</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>832</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
+        <v>832</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>833</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>834</v>
       </c>
     </row>
     <row r="6" spans="1:2">

</xml_diff>

<commit_message>
Updated Grn Page Functions And DB Query
Updated Grn Page Functions And DB Query
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="876">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="878">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -2942,6 +2942,45 @@
    AND stock_prod_id = 'TVS-RM-KDK-10'
    AND stock_prod_rev = '0'
 </t>
+  </si>
+  <si>
+    <t>OsoaQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SELECT srcahd_plnt_loc_id "loc id",
+       srcahd_plnt "unit",
+       srcahd_doc_no "Doc. No.",
+       srcahd_amd_no "Amd. No.",
+       srcahd_cust_id "customer id",
+       (SELECT suplr_name1
+          FROM suppliers
+         WHERE suplr_bu = srcahd_bu AND suplr_suplr_id = srcahd_cust_id)
+          "customer name",
+       srcaln_prod_id "item id",
+       srcaln_prod_rev "item rev",
+       (SELECT prod_desc11
+          FROM products
+         WHERE     prod_bu = srcaln_bu
+               AND prod_id = srcaln_prod_id
+               AND prod_rev = srcaln_prod_rev)
+          "item descripition",
+       srcaln_uom "uom",
+       srcaln_disc_pct "disc_pct",
+       srcaln_old_price "Existing Price",
+       srcaln_new_price "new_price",
+       srcaln_mrp_price "MRP Price",
+       srcaln_hsn_code "HSN code",
+       srcaln_tax_pct "Tax Percent",
+       srcaln_cgst_amt "CGST",
+       srcaln_sgst_amt "SGST",
+       srcaln_igst_amt "IGST",
+       srcaln_utgst_amt "UTGST"
+  FROM sales_rate_contr_ament_hd, sales_rate_contr_ament_ln
+ WHERE     srcahd_bu = srcaln_bu
+       AND srcahd_plnt = srcaln_plnt
+       AND srcahd_doc_no = '${OSOANO}'
+    AND srcahd_doc_no = srcaln_doc_no
+       AND srcahd_bu =  'TVSA' </t>
   </si>
 </sst>
 </file>
@@ -3641,7 +3680,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3772,10 +3811,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="53">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8019,170 +8054,170 @@
       </c>
     </row>
     <row r="490" spans="1:2">
-      <c r="A490" s="58" t="s">
+      <c r="A490" s="2" t="s">
         <v>826</v>
       </c>
-      <c r="B490" s="59" t="s">
+      <c r="B490" s="8" t="s">
         <v>827</v>
       </c>
     </row>
     <row r="491" spans="1:2">
-      <c r="A491" s="58" t="s">
+      <c r="A491" s="2" t="s">
         <v>828</v>
       </c>
-      <c r="B491" s="59" t="s">
+      <c r="B491" s="8" t="s">
         <v>829</v>
       </c>
     </row>
     <row r="492" spans="1:2">
-      <c r="A492" s="58" t="s">
+      <c r="A492" s="2" t="s">
         <v>830</v>
       </c>
-      <c r="B492" s="59" t="s">
+      <c r="B492" s="8" t="s">
         <v>831</v>
       </c>
     </row>
     <row r="493" spans="1:2">
-      <c r="A493" s="58" t="s">
+      <c r="A493" s="2" t="s">
         <v>832</v>
       </c>
-      <c r="B493" s="59" t="s">
+      <c r="B493" s="8" t="s">
         <v>833</v>
       </c>
     </row>
     <row r="494" spans="1:2">
-      <c r="A494" s="58" t="s">
+      <c r="A494" s="2" t="s">
         <v>834</v>
       </c>
-      <c r="B494" s="59" t="s">
+      <c r="B494" s="8" t="s">
         <v>835</v>
       </c>
     </row>
     <row r="495" spans="1:2">
-      <c r="A495" s="58" t="s">
+      <c r="A495" s="2" t="s">
         <v>836</v>
       </c>
-      <c r="B495" s="59" t="s">
+      <c r="B495" s="8" t="s">
         <v>837</v>
       </c>
     </row>
     <row r="496" spans="1:2">
-      <c r="A496" s="58" t="s">
+      <c r="A496" s="2" t="s">
         <v>838</v>
       </c>
-      <c r="B496" s="59" t="s">
+      <c r="B496" s="8" t="s">
         <v>839</v>
       </c>
     </row>
     <row r="497" spans="1:2">
-      <c r="A497" s="58" t="s">
+      <c r="A497" s="2" t="s">
         <v>840</v>
       </c>
-      <c r="B497" s="59" t="s">
+      <c r="B497" s="8" t="s">
         <v>841</v>
       </c>
     </row>
     <row r="498" spans="1:2">
-      <c r="A498" s="58" t="s">
+      <c r="A498" s="2" t="s">
         <v>842</v>
       </c>
-      <c r="B498" s="59" t="s">
+      <c r="B498" s="8" t="s">
         <v>843</v>
       </c>
     </row>
     <row r="499" spans="1:2">
-      <c r="A499" s="58" t="s">
+      <c r="A499" s="2" t="s">
         <v>844</v>
       </c>
-      <c r="B499" s="59" t="s">
+      <c r="B499" s="8" t="s">
         <v>845</v>
       </c>
     </row>
     <row r="500" spans="1:2">
-      <c r="A500" s="58" t="s">
+      <c r="A500" s="2" t="s">
         <v>846</v>
       </c>
-      <c r="B500" s="59" t="s">
+      <c r="B500" s="8" t="s">
         <v>847</v>
       </c>
     </row>
     <row r="501" spans="1:2">
-      <c r="A501" s="58" t="s">
+      <c r="A501" s="2" t="s">
         <v>848</v>
       </c>
-      <c r="B501" s="59" t="s">
+      <c r="B501" s="8" t="s">
         <v>849</v>
       </c>
     </row>
     <row r="502" spans="1:2">
-      <c r="A502" s="58" t="s">
+      <c r="A502" s="2" t="s">
         <v>850</v>
       </c>
-      <c r="B502" s="59" t="s">
+      <c r="B502" s="8" t="s">
         <v>851</v>
       </c>
     </row>
     <row r="503" spans="1:2">
-      <c r="A503" s="58" t="s">
+      <c r="A503" s="2" t="s">
         <v>852</v>
       </c>
-      <c r="B503" s="59" t="s">
+      <c r="B503" s="8" t="s">
         <v>853</v>
       </c>
     </row>
     <row r="504" spans="1:2">
-      <c r="A504" s="58" t="s">
+      <c r="A504" s="2" t="s">
         <v>854</v>
       </c>
-      <c r="B504" s="59" t="s">
+      <c r="B504" s="8" t="s">
         <v>855</v>
       </c>
     </row>
     <row r="505" spans="1:2">
-      <c r="A505" s="58" t="s">
+      <c r="A505" s="2" t="s">
         <v>856</v>
       </c>
-      <c r="B505" s="59" t="s">
+      <c r="B505" s="8" t="s">
         <v>857</v>
       </c>
     </row>
     <row r="506" spans="1:2">
-      <c r="A506" s="58" t="s">
+      <c r="A506" s="2" t="s">
         <v>858</v>
       </c>
-      <c r="B506" s="59" t="s">
+      <c r="B506" s="8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="507" spans="1:2">
-      <c r="A507" s="58" t="s">
+      <c r="A507" s="2" t="s">
         <v>859</v>
       </c>
-      <c r="B507" s="59" t="s">
+      <c r="B507" s="8" t="s">
         <v>860</v>
       </c>
     </row>
     <row r="508" spans="1:2">
-      <c r="A508" s="58" t="s">
+      <c r="A508" s="2" t="s">
         <v>861</v>
       </c>
-      <c r="B508" s="59" t="s">
+      <c r="B508" s="8" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="509" spans="1:2">
-      <c r="A509" s="58" t="s">
+      <c r="A509" s="2" t="s">
         <v>862</v>
       </c>
-      <c r="B509" s="59" t="s">
+      <c r="B509" s="8" t="s">
         <v>863</v>
       </c>
     </row>
     <row r="510" spans="1:2">
-      <c r="A510" s="58" t="s">
+      <c r="A510" s="2" t="s">
         <v>864</v>
       </c>
-      <c r="B510" s="59" t="s">
+      <c r="B510" s="8" t="s">
         <v>865</v>
       </c>
     </row>
@@ -8246,13 +8281,17 @@
       <c r="A6" s="2" t="s">
         <v>874</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>875</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+    <row r="7" ht="409.5" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>876</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>877</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2"/>

</xml_diff>

<commit_message>
Updated For Script For Parallel Testing And Added PO Amendment Test Scenarios
Updated For Script For Parallel Testing And Added PO Amendment Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="1060">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="1061">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -3100,6 +3100,9 @@
   </si>
   <si>
     <t>Nationality</t>
+  </si>
+  <si>
+    <t>Cleared</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -4088,7 +4091,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4224,12 +4227,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4545,40 +4542,40 @@
     <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -5000,11 +4997,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B602"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B603"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7090909090909" style="4" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="5" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="4" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="5" customWidth="1"/>
     <col min="3" max="16384" width="9" style="4"/>
   </cols>
   <sheetData>
@@ -9769,59 +9766,67 @@
       </c>
     </row>
     <row r="596" spans="1:2">
-      <c r="A596" s="40" t="s">
+      <c r="A596" s="8" t="s">
         <v>1011</v>
       </c>
-      <c r="B596" s="41" t="s">
+      <c r="B596" s="9" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="597" spans="1:2">
-      <c r="A597" s="40" t="s">
+      <c r="A597" s="8" t="s">
         <v>1012</v>
       </c>
-      <c r="B597" s="41" t="s">
+      <c r="B597" s="9" t="s">
         <v>1013</v>
       </c>
     </row>
     <row r="598" spans="1:2">
-      <c r="A598" s="40" t="s">
+      <c r="A598" s="8" t="s">
         <v>1014</v>
       </c>
-      <c r="B598" s="41" t="s">
+      <c r="B598" s="9" t="s">
         <v>1015</v>
       </c>
     </row>
     <row r="599" spans="1:2">
-      <c r="A599" s="40" t="s">
+      <c r="A599" s="8" t="s">
         <v>1016</v>
       </c>
-      <c r="B599" s="41" t="s">
+      <c r="B599" s="9" t="s">
         <v>1017</v>
       </c>
     </row>
     <row r="600" spans="1:2">
-      <c r="A600" s="40" t="s">
+      <c r="A600" s="8" t="s">
         <v>1018</v>
       </c>
-      <c r="B600" s="41" t="s">
+      <c r="B600" s="9" t="s">
         <v>1019</v>
       </c>
     </row>
     <row r="601" spans="1:2">
-      <c r="A601" s="40" t="s">
+      <c r="A601" s="8" t="s">
         <v>1020</v>
       </c>
-      <c r="B601" s="41" t="s">
+      <c r="B601" s="9" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="602" spans="1:2">
-      <c r="A602" s="40" t="s">
+      <c r="A602" s="8" t="s">
         <v>1022</v>
       </c>
-      <c r="B602" s="41" t="s">
+      <c r="B602" s="9" t="s">
         <v>1023</v>
+      </c>
+    </row>
+    <row r="603" spans="1:2">
+      <c r="A603" s="40" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B603" s="41" t="s">
+        <v>1024</v>
       </c>
     </row>
   </sheetData>
@@ -9834,9 +9839,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9850,146 +9855,146 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1053</v>
-      </c>
-    </row>
-    <row r="17" ht="377" spans="1:2">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="17" ht="374.4" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="18" ht="409.5" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="19" ht="409.5" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed E2E Scenarios And Added PO Amendment Test Scenarios
Fixed E2E Scenarios And Added PO Amendment Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19320" windowHeight="8867"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="1061">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="1066">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -3103,6 +3103,21 @@
   </si>
   <si>
     <t>Cleared</t>
+  </si>
+  <si>
+    <t>StandardPO</t>
+  </si>
+  <si>
+    <t>Standard(PO)</t>
+  </si>
+  <si>
+    <t>StandardService</t>
+  </si>
+  <si>
+    <t>Standard(Service)</t>
+  </si>
+  <si>
+    <t>StockTransferPO</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -4997,7 +5012,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B603"/>
+  <dimension ref="A1:B606"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="62.712962962963" style="4" customWidth="1"/>
@@ -9822,11 +9837,35 @@
       </c>
     </row>
     <row r="603" spans="1:2">
-      <c r="A603" s="40" t="s">
+      <c r="A603" s="8" t="s">
         <v>1024</v>
       </c>
-      <c r="B603" s="41" t="s">
+      <c r="B603" s="9" t="s">
         <v>1024</v>
+      </c>
+    </row>
+    <row r="604" spans="1:2">
+      <c r="A604" s="40" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B604" s="41" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="605" spans="1:2">
+      <c r="A605" s="40" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B605" s="41" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="606" spans="1:2">
+      <c r="A606" s="40" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B606" s="41" t="s">
+        <v>788</v>
       </c>
     </row>
   </sheetData>
@@ -9855,146 +9894,146 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1025</v>
+        <v>1030</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1026</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1027</v>
+        <v>1032</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1028</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1029</v>
+        <v>1034</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1031</v>
+        <v>1036</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1032</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1034</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1036</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1037</v>
+        <v>1042</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1039</v>
+        <v>1044</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1041</v>
+        <v>1046</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1042</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1044</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1045</v>
+        <v>1050</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1046</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1049</v>
+        <v>1054</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1050</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1051</v>
+        <v>1056</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1052</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1054</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="17" ht="374.4" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1055</v>
+        <v>1060</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1056</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="18" ht="409.5" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1057</v>
+        <v>1062</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1058</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="19" ht="409.5" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1060</v>
+        <v>1065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated and Added Leave and Employee Masters Test Scenarios
Updated Added Leave and Employee Masters Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19320" windowHeight="8867"/>
+    <workbookView windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="1066">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1230" uniqueCount="1078">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -3118,6 +3118,42 @@
   </si>
   <si>
     <t>StockTransferPO</t>
+  </si>
+  <si>
+    <t>Emp_GWP0001</t>
+  </si>
+  <si>
+    <t>GWP0001</t>
+  </si>
+  <si>
+    <t>Year202526</t>
+  </si>
+  <si>
+    <t>202526</t>
+  </si>
+  <si>
+    <t>LOP-Text</t>
+  </si>
+  <si>
+    <t>LOSS OF PAY</t>
+  </si>
+  <si>
+    <t>CasualLeave-Text</t>
+  </si>
+  <si>
+    <t>CASUAL LEAVE</t>
+  </si>
+  <si>
+    <t>CL-Text</t>
+  </si>
+  <si>
+    <t>CL</t>
+  </si>
+  <si>
+    <t>FullSessionText</t>
+  </si>
+  <si>
+    <t>Full</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -5012,11 +5048,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B606"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
+  <dimension ref="A1:B612"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.712962962963" style="4" customWidth="1"/>
-    <col min="2" max="2" width="59.8518518518519" style="5" customWidth="1"/>
+    <col min="1" max="1" width="62.7142857142857" style="4" customWidth="1"/>
+    <col min="2" max="2" width="59.847619047619" style="5" customWidth="1"/>
     <col min="3" max="16384" width="9" style="4"/>
   </cols>
   <sheetData>
@@ -9845,27 +9881,75 @@
       </c>
     </row>
     <row r="604" spans="1:2">
-      <c r="A604" s="40" t="s">
+      <c r="A604" s="8" t="s">
         <v>1025</v>
       </c>
-      <c r="B604" s="41" t="s">
+      <c r="B604" s="9" t="s">
         <v>1026</v>
       </c>
     </row>
     <row r="605" spans="1:2">
-      <c r="A605" s="40" t="s">
+      <c r="A605" s="8" t="s">
         <v>1027</v>
       </c>
-      <c r="B605" s="41" t="s">
+      <c r="B605" s="9" t="s">
         <v>1028</v>
       </c>
     </row>
     <row r="606" spans="1:2">
-      <c r="A606" s="40" t="s">
+      <c r="A606" s="8" t="s">
         <v>1029</v>
       </c>
-      <c r="B606" s="41" t="s">
+      <c r="B606" s="9" t="s">
         <v>788</v>
+      </c>
+    </row>
+    <row r="607" spans="1:2">
+      <c r="A607" s="40" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B607" s="41" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="608" spans="1:2">
+      <c r="A608" s="40" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B608" s="41" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="609" spans="1:2">
+      <c r="A609" s="40" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B609" s="41" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="610" spans="1:2">
+      <c r="A610" s="40" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B610" s="41" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="611" spans="1:2">
+      <c r="A611" s="40" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B611" s="41" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="612" spans="1:2">
+      <c r="A612" s="40" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B612" s="41" t="s">
+        <v>1041</v>
       </c>
     </row>
   </sheetData>
@@ -9878,9 +9962,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
+    <col min="1" max="1" width="19.847619047619" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9894,146 +9978,146 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1030</v>
+        <v>1042</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1031</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1032</v>
+        <v>1044</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1033</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1034</v>
+        <v>1046</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1035</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1036</v>
+        <v>1048</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1037</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1038</v>
+        <v>1050</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1039</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1040</v>
+        <v>1052</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1041</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1042</v>
+        <v>1054</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1043</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1044</v>
+        <v>1056</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1045</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1046</v>
+        <v>1058</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1047</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1048</v>
+        <v>1060</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1049</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1050</v>
+        <v>1062</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1051</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1052</v>
+        <v>1064</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1053</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1054</v>
+        <v>1066</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1055</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1056</v>
+        <v>1068</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1057</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1058</v>
+        <v>1070</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1059</v>
-      </c>
-    </row>
-    <row r="17" ht="374.4" spans="1:2">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="17" ht="405" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1060</v>
+        <v>1072</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1061</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="18" ht="409.5" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1062</v>
+        <v>1074</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1063</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="19" ht="409.5" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1064</v>
+        <v>1076</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1065</v>
+        <v>1077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Approved Supplier, Buyer And Share Of Business Test Scenarios
Added Approved Supplier, Buyer And Share Of Business Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620"/>
+    <workbookView windowWidth="23040" windowHeight="9120" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1843" uniqueCount="1611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2127" uniqueCount="1844">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -4624,6 +4624,663 @@
   </si>
   <si>
     <t>QUALITY</t>
+  </si>
+  <si>
+    <t>AshokSelectValue</t>
+  </si>
+  <si>
+    <t>EMP15</t>
+  </si>
+  <si>
+    <t>AakashValue</t>
+  </si>
+  <si>
+    <t>AAKASH</t>
+  </si>
+  <si>
+    <t>PurchaseManager</t>
+  </si>
+  <si>
+    <t>PURCHASE MANAGER</t>
+  </si>
+  <si>
+    <t>Purchase</t>
+  </si>
+  <si>
+    <t>PURCHASE</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>32549</t>
+  </si>
+  <si>
+    <t>Gmail</t>
+  </si>
+  <si>
+    <t>@gmail.com</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>UserDefinedGeneral</t>
+  </si>
+  <si>
+    <t>User Defined/General</t>
+  </si>
+  <si>
+    <t>Apps</t>
+  </si>
+  <si>
+    <t>APPS</t>
+  </si>
+  <si>
+    <t>RawMaterial10Item</t>
+  </si>
+  <si>
+    <t>TVS-RM00040</t>
+  </si>
+  <si>
+    <t>CostBasis</t>
+  </si>
+  <si>
+    <t>User Defined Price</t>
+  </si>
+  <si>
+    <t>OpenBlanket</t>
+  </si>
+  <si>
+    <t>Open Blanket Order</t>
+  </si>
+  <si>
+    <t>PriceListApprovedSupplier</t>
+  </si>
+  <si>
+    <t>Price List</t>
+  </si>
+  <si>
+    <t>PurchaseType</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>JJAutomobileId</t>
+  </si>
+  <si>
+    <t>ShareOfBusinessItem</t>
+  </si>
+  <si>
+    <t>POSupplierName</t>
+  </si>
+  <si>
+    <t>SobDocNumber</t>
+  </si>
+  <si>
+    <t>SOB1-2425-00001</t>
+  </si>
+  <si>
+    <t>Process10</t>
+  </si>
+  <si>
+    <t>PROCESS-10</t>
+  </si>
+  <si>
+    <t>EffFrom</t>
+  </si>
+  <si>
+    <t>13-05-2025</t>
+  </si>
+  <si>
+    <t>EffTo</t>
+  </si>
+  <si>
+    <t>31-05-2025</t>
+  </si>
+  <si>
+    <t>LovButton</t>
+  </si>
+  <si>
+    <t>SelectType</t>
+  </si>
+  <si>
+    <t>SendTextInput</t>
+  </si>
+  <si>
+    <t>PrNumber</t>
+  </si>
+  <si>
+    <t>PUU1-2526-0010</t>
+  </si>
+  <si>
+    <t>PONumber</t>
+  </si>
+  <si>
+    <t>POS10/25-26/023001</t>
+  </si>
+  <si>
+    <t>FinishedGoods</t>
+  </si>
+  <si>
+    <t>FINISHED GOODS</t>
+  </si>
+  <si>
+    <t>PoMaterial</t>
+  </si>
+  <si>
+    <t>SelvaKumarB</t>
+  </si>
+  <si>
+    <t>SELVA KUMAR B</t>
+  </si>
+  <si>
+    <t>CR_Acpt_Qty</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>WorkCenter</t>
+  </si>
+  <si>
+    <t>L100 CRYOGENIC AREA</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>CRYOGENIC DEFLASHING</t>
+  </si>
+  <si>
+    <t>HARIKRISHNA M (HK)</t>
+  </si>
+  <si>
+    <t>ReworkLocator</t>
+  </si>
+  <si>
+    <t>BF</t>
+  </si>
+  <si>
+    <t>RWNO</t>
+  </si>
+  <si>
+    <t>${RWNO}</t>
+  </si>
+  <si>
+    <t>RWDBLocIDColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_PLNT_LOC_ID</t>
+  </si>
+  <si>
+    <t>RWDBUnitColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_PLNT</t>
+  </si>
+  <si>
+    <t>RWDBPfxColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_ORD_PFX</t>
+  </si>
+  <si>
+    <t>RWDBOrderNoColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_ORD_NO</t>
+  </si>
+  <si>
+    <t>RWDBItemColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_PROD_ID</t>
+  </si>
+  <si>
+    <t>RWDBItemDescColumn</t>
+  </si>
+  <si>
+    <t>PROD_DESC</t>
+  </si>
+  <si>
+    <t>RWDBTypeColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_ORD_TYPE</t>
+  </si>
+  <si>
+    <t>RWDBLotColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_LOT_NO</t>
+  </si>
+  <si>
+    <t>RWDBSourceDocColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_SOU_DOC_NO</t>
+  </si>
+  <si>
+    <t>RWDBSourceDocPfxColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_SOU_DOC_PFX</t>
+  </si>
+  <si>
+    <t>RWDBQtyColumn</t>
+  </si>
+  <si>
+    <t>RWOHD_REWORK_QTY</t>
+  </si>
+  <si>
+    <t>RWCDBLocIDColumn</t>
+  </si>
+  <si>
+    <t>RWOCHD_LOC_ID</t>
+  </si>
+  <si>
+    <t>RWCDBUnitColumn</t>
+  </si>
+  <si>
+    <t>RWOCHD_PLNT</t>
+  </si>
+  <si>
+    <t>RWCDBOrderNoColumn</t>
+  </si>
+  <si>
+    <t>RWOCHD_DOC_NO</t>
+  </si>
+  <si>
+    <t>RWCDBItemColumn</t>
+  </si>
+  <si>
+    <t>RWOCHD_PROD_ID</t>
+  </si>
+  <si>
+    <t>RWCDBSourceWHColumn</t>
+  </si>
+  <si>
+    <t>WHDESC</t>
+  </si>
+  <si>
+    <t>RWCDBStatusColumn</t>
+  </si>
+  <si>
+    <t>RWCDBDraftColumn</t>
+  </si>
+  <si>
+    <t>RWCDBPostedColumn</t>
+  </si>
+  <si>
+    <t>RWCDBApprovedColumn</t>
+  </si>
+  <si>
+    <t>RWCNO</t>
+  </si>
+  <si>
+    <t>${RWCNO}</t>
+  </si>
+  <si>
+    <t>DB_DN_Pfx</t>
+  </si>
+  <si>
+    <t>DBN10</t>
+  </si>
+  <si>
+    <t>DB_Reason</t>
+  </si>
+  <si>
+    <t>EXCESS PROCUREMENT</t>
+  </si>
+  <si>
+    <t>DebitNoteSupplier</t>
+  </si>
+  <si>
+    <t>ACCENTURE INFO TECH</t>
+  </si>
+  <si>
+    <t>DebitNoteTreeNote</t>
+  </si>
+  <si>
+    <t>Debit Note</t>
+  </si>
+  <si>
+    <t>DBNO</t>
+  </si>
+  <si>
+    <t>${DBNO}</t>
+  </si>
+  <si>
+    <t>DBDBLocationColumn</t>
+  </si>
+  <si>
+    <t>DBDBUnitColumn</t>
+  </si>
+  <si>
+    <t>DBDBDocNoColumn</t>
+  </si>
+  <si>
+    <t>DBDBDocPfxColumn</t>
+  </si>
+  <si>
+    <t>DBDBTypeColumn</t>
+  </si>
+  <si>
+    <t>DBDBCustIDColumn</t>
+  </si>
+  <si>
+    <t>DBDBCustNameColumn</t>
+  </si>
+  <si>
+    <t>DBDBGoodsTypeColumn</t>
+  </si>
+  <si>
+    <t>DBDBStatusColumn</t>
+  </si>
+  <si>
+    <t>DBHeaderDraftStatus</t>
+  </si>
+  <si>
+    <t>priceClassName</t>
+  </si>
+  <si>
+    <t>priceBasisValue</t>
+  </si>
+  <si>
+    <t>priceBasisPriceListValue</t>
+  </si>
+  <si>
+    <t>Item_Different_UOM</t>
+  </si>
+  <si>
+    <t>priceClassNameDifferent</t>
+  </si>
+  <si>
+    <t>PriceBasisCatalogue</t>
+  </si>
+  <si>
+    <t>Catalog Price</t>
+  </si>
+  <si>
+    <t>catalogName</t>
+  </si>
+  <si>
+    <t>catalogCustomer</t>
+  </si>
+  <si>
+    <t>CatalogueCurcy</t>
+  </si>
+  <si>
+    <t>WorkFlowType</t>
+  </si>
+  <si>
+    <t>Sales Catalog Price</t>
+  </si>
+  <si>
+    <t>catalogExportCustomer</t>
+  </si>
+  <si>
+    <t>PriceBasisStandard</t>
+  </si>
+  <si>
+    <t>Standard Price</t>
+  </si>
+  <si>
+    <t>L100StdPrice</t>
+  </si>
+  <si>
+    <t>LOCATION 100</t>
+  </si>
+  <si>
+    <t>Dom</t>
+  </si>
+  <si>
+    <t>Inter</t>
+  </si>
+  <si>
+    <t>PlDocNo</t>
+  </si>
+  <si>
+    <t>${PlDocNo}</t>
+  </si>
+  <si>
+    <t>PriceListDbLocId</t>
+  </si>
+  <si>
+    <t>Unit Loc ID</t>
+  </si>
+  <si>
+    <t>PriceListDbPLpfx</t>
+  </si>
+  <si>
+    <t>Doc Pfx</t>
+  </si>
+  <si>
+    <t>PriceListDbCustomerId</t>
+  </si>
+  <si>
+    <t>Customer Id</t>
+  </si>
+  <si>
+    <t>PriceListDbCustomerDesc</t>
+  </si>
+  <si>
+    <t>CUSTOMER_NAME</t>
+  </si>
+  <si>
+    <t>PriceListDbItemId</t>
+  </si>
+  <si>
+    <t>CPL_PROD_ID</t>
+  </si>
+  <si>
+    <t>PriceListDbSalesUOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales UOM </t>
+  </si>
+  <si>
+    <t>PriceListDbSalesPrice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales Price </t>
+  </si>
+  <si>
+    <t>PriceListDbSalesDisc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disc Pct </t>
+  </si>
+  <si>
+    <t>CatDocNo</t>
+  </si>
+  <si>
+    <t>${CatDocNo}</t>
+  </si>
+  <si>
+    <t>PriceListDbAmdNo</t>
+  </si>
+  <si>
+    <t>CPL_AMD_NO</t>
+  </si>
+  <si>
+    <t>CatPriceDbDocno</t>
+  </si>
+  <si>
+    <t>SCTLN_DOC_NO</t>
+  </si>
+  <si>
+    <t>CatPriceDbItemId</t>
+  </si>
+  <si>
+    <t>SCTLN_PROD_ID</t>
+  </si>
+  <si>
+    <t>CatPriceDbItemDesc</t>
+  </si>
+  <si>
+    <t>ITEM_DESC</t>
+  </si>
+  <si>
+    <t>CatPriceDbSalesUom</t>
+  </si>
+  <si>
+    <t>SCTLN_UOM</t>
+  </si>
+  <si>
+    <t>CatPriceDbCatalogId</t>
+  </si>
+  <si>
+    <t>SCTLN_CTLG_ID</t>
+  </si>
+  <si>
+    <t>CatPriceDbCurcyId</t>
+  </si>
+  <si>
+    <t>SCTLN_CURCY_ID</t>
+  </si>
+  <si>
+    <t>CatPriceDbStatus</t>
+  </si>
+  <si>
+    <t>CatPriceEffToDate</t>
+  </si>
+  <si>
+    <t>SCTLN_DATE_TO</t>
+  </si>
+  <si>
+    <t>CatPriceDbEffDate</t>
+  </si>
+  <si>
+    <t>SCTLN_DATE_FROM</t>
+  </si>
+  <si>
+    <t>CatPriceDbMaxiDisc</t>
+  </si>
+  <si>
+    <t>SCTLN_DISC_PCT_MAX</t>
+  </si>
+  <si>
+    <t>CatPriceDbMinDisc</t>
+  </si>
+  <si>
+    <t>SCTLN_DISC_PCT_MIN</t>
+  </si>
+  <si>
+    <t>CatPriceDbSalesPrice</t>
+  </si>
+  <si>
+    <t>SCTLN_PRICE</t>
+  </si>
+  <si>
+    <t>StdItemUniq</t>
+  </si>
+  <si>
+    <t>${StdItemId}</t>
+  </si>
+  <si>
+    <t>StdPriceIocDb</t>
+  </si>
+  <si>
+    <t>Loc.ID</t>
+  </si>
+  <si>
+    <t>StdPriceUnitDb</t>
+  </si>
+  <si>
+    <t>StdPriceItemIdDb</t>
+  </si>
+  <si>
+    <t>Item.Id</t>
+  </si>
+  <si>
+    <t>StdPriceItemDescDb</t>
+  </si>
+  <si>
+    <t>StdPriceCurcyFieldDb</t>
+  </si>
+  <si>
+    <t>Curcy</t>
+  </si>
+  <si>
+    <t>StdPriceUOMFieldDb</t>
+  </si>
+  <si>
+    <t>Price UOM</t>
+  </si>
+  <si>
+    <t>StdPriceEffDateDb</t>
+  </si>
+  <si>
+    <t>Eff.From Date</t>
+  </si>
+  <si>
+    <t>StdPriceEffToDateDb</t>
+  </si>
+  <si>
+    <t>Eff.To Date</t>
+  </si>
+  <si>
+    <t>StdPriceMapFieldDb</t>
+  </si>
+  <si>
+    <t>Map Price</t>
+  </si>
+  <si>
+    <t>StdPriceLandCostDb</t>
+  </si>
+  <si>
+    <t>Landed Cost</t>
+  </si>
+  <si>
+    <t>StdPriceSellingPriceDb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selling Price </t>
+  </si>
+  <si>
+    <t>StdPriceMinDiscPct</t>
+  </si>
+  <si>
+    <t>Disc Min</t>
+  </si>
+  <si>
+    <t>StdPriceMaxDiscPct</t>
+  </si>
+  <si>
+    <t>Disc Max</t>
+  </si>
+  <si>
+    <t>StdPricePriceClassDb</t>
+  </si>
+  <si>
+    <t>Price Class</t>
+  </si>
+  <si>
+    <t>ItemsScreenName</t>
+  </si>
+  <si>
+    <t>Items</t>
+  </si>
+  <si>
+    <t>ItemsAssoScreenName</t>
+  </si>
+  <si>
+    <t>ITEM - UNIT ASSO.</t>
+  </si>
+  <si>
+    <t>CustomerItemsScreenName</t>
+  </si>
+  <si>
+    <t>Customer Item</t>
+  </si>
+  <si>
+    <t>PriceList_Std_CatScreenName</t>
+  </si>
+  <si>
+    <t>Price List/Standard/Catalog</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -6475,6 +7132,246 @@
 AND RFQSUP_RFQ_NO='${RFQNO}'
 AND PQLN_SEQ_NO='${RFQSEQNO}'
 AND RFQSUP_SUPLR_ID='${SUPNO}'</t>
+  </si>
+  <si>
+    <t>ReworkOrderHeaderQuery</t>
+  </si>
+  <si>
+    <t>SELECT rwohd_plnt_loc_id,
+        rwohd_plnt,
+        rwohd_ord_pfx,
+        rwohd_ord_no,
+        rwohd_prod_ord_no,
+        rwohd_prod_id,
+        (SELECT prod_desc11 
+            FROM products
+          WHERE prod_bu = 'TVSA'
+                AND prod_id = rwohd_prod_id
+                AND prod_rev = rwohd_prod_rev) prod_desc,
+        rwohd_ord_type,
+        rwohd_lot_no,
+        rwohd_pp_no,
+        rwohd_sou_doc_no,
+        rwohd_sou_doc_pfx,
+        rwohd_rework_qty,
+        rwohd_so_schld_desc,
+        rwohd_sf_code,
+        DECODE(rwohd_status,'E','Draft','N','Entry Completed','A','Approved','C','Completed','L','Cancelled') Status
+    FROM rework_order_hd
+  WHERE rwohd_bu = 'TVSA'
+        AND rwohd_ord_no = '${RWNO}'
+UNION ALL
+SELECT  rwohdh_plnt_loc_id rwohdh_loc_id,
+        rwohdh_plnt,
+        rwohdh_ord_pfx,
+        rwohdh_ord_no,
+        rwohdh_prod_ord_no,
+        rwohdh_prod_id,
+        (SELECT prod_desc11 
+            FROM products
+          WHERE prod_bu = 'TVSA'
+                AND prod_id = rwohdh_prod_id
+                AND prod_rev = rwohdh_prod_rev) prod_desc,
+        rwohdh_ord_type,
+        rwohdh_lot_no,
+        rwohdh_pp_no,
+        rwohdh_sou_doc_no,
+        rwohdh_sou_doc_pfx,
+        rwohdh_rework_qty,
+        rwohdh_so_schld_desc,
+        rwohdh_sf_code,
+        DECODE(rwohdh_status,'E','Draft','N','Entry Completed','A','Approved','C','Completed','L','Cancelled') Status
+    FROM rework_order_hd_hist
+  WHERE rwohdh_bu = 'TVSA'
+        AND rwohdh_ord_no = '${RWNO}'</t>
+  </si>
+  <si>
+    <t>ReworkCompletionQuery</t>
+  </si>
+  <si>
+    <t>SELECT rwochd_loc_id,
+        rwochd_plnt,
+        rwochd_doc_no,
+        rwochd_source_type,
+        rwochd_prod_id,
+        rwochd_prod_rev,
+        rwochd_sou_store,
+         func_find_store_qry_desc(rwochd_bu,rwochd_sou_store,1) WHDesc,
+        rwochd_so_schld_desc,
+        DECODE(rwochd_status,'N','Draft','E','Entry Completed','F','Forward to QC','Q','QC Completed','C','Cancelled','A','Approved','P','Posted') Status,
+        rwochd_same_lot
+    FROM rework_order_comp_hd
+  WHERE rwochd_bu = 'TVSA'
+        AND rwochd_doc_no = '${RWCNO}'
+UNION ALL
+SELECT rwochdh_loc_id,
+        rwochdh_plnt,
+        rwochdh_doc_no,
+        rwochdh_source_type,
+        rwochdh_prod_id,
+        rwochdh_prod_rev,
+        rwochdh_sou_store,
+        func_find_store_qry_desc(rwochdh_bu,rwochdh_sou_store,1)WHDesc,
+        rwochdh_so_schld_desc,
+        DECODE(rwochdh_status,'N','Draft','E','Entry Completed','F','Forward to QC','Q','QC Completed','C','Cancelled','A','Approved','P','Posted') Status,
+        rwochdh_same_lot
+    FROM rework_order_comp_hd_hist
+  WHERE rwochdh_bu = 'TVSA'
+        AND rwochdh_doc_no = '${RWCNO}'</t>
+  </si>
+  <si>
+    <t>ReworkCompletionDetailQuery</t>
+  </si>
+  <si>
+    <t>SELECT rwocd_doc_no,
+        rwocd_prod_ord_no,
+        rwocd_sou_lot_no,
+        rwocd_rwk_comp_qty,
+        rwocd_rwk_repair_qty,
+        rwocd_rwk_scrap_qty,
+        rwocd_rwk_rej_qty,
+        rwocd_rwk_dis_ass_qty,
+        rwocd_tar_store,
+        rwocd_mat_cost,
+        rwocd_res_cost,
+        rwocd_ot_cost,
+        rwocd_unit_cost
+    FROM rework_order_comp_dtl
+  WHERE rwocd_bu = 'TVSA'
+        AND rwocd_doc_no = '${RWCNO}'
+UNION ALL
+SELECT rwocdh_doc_no,
+        rwocdh_prod_ord_no,
+        rwocdh_sou_lot_no,
+        rwocdh_rwk_comp_qty,
+        rwocdh_rwk_repair_qty,
+        rwocdh_rwk_scrap_qty,
+        rwocdh_rwk_rej_qty,
+        rwocdh_rwk_dis_ass_qty,
+        rwocdh_tar_store,
+        rwocdh_mat_cost,
+        rwocdh_res_cost,
+        rwocdh_ot_cost,
+        rwocdh_unit_cost
+    FROM rework_order_comp_dtl_hist
+  WHERE rwocdh_bu = 'TVSA'
+        AND rwocdh_doc_no = '${RWCNO}'</t>
+  </si>
+  <si>
+    <t>DebitNoteHeaderQuery</t>
+  </si>
+  <si>
+    <t>SELECT sihd_plnt_loc_id,
+       sihd_plant,
+       sihd_doc_no,
+       sihd_doc_pfx,
+       sihd_type,
+       sihd_cust_id,
+       sihd_cust_name,
+       sihd_rtn_goods_dtls,
+       sihd_ref1,
+       DECODE (sihd_status,
+               'N', 'Draft',
+               'I', 'Invoiced',
+               'C', 'Cancelled',
+               'E', 'Entry Completed')
+          sihd_status
+  FROM sales_invoices_hd
+  WHERE SIHD_BU = 'TVSA'
+    AND SIHD_DOC_NO = '${DBNO}'</t>
+  </si>
+  <si>
+    <t>PricelistQuery</t>
+  </si>
+  <si>
+    <t>select cpl_plnt "unit"  ,
+       cpl_plnt_loc_id "Unit Loc ID",
+       cpl_plnt_loc_name "Unit Loc Name",
+         (select bup_name1
+         from bus_unit_plants
+        where bup_bu = cpl_bu
+          and bup_plant_id = cpl_plnt) plant_desc,
+       cpl_doc_pfx "Doc Pfx",     
+       cpl_doc_no "Document No",
+       cpl_doc_date "Doc Date",
+       cpl_cust_id "Customer Id",
+       (select suplr_name1
+          from suppliers
+         where suplr_bu = cpl_bu
+           and suplr_suplr_id = cpl_cust_id 
+           and suplr_status = 'A' ) customer_name,
+       cpl_prod_id,
+       cpl_prod_rev,
+         (select prod_desc11
+            from products
+            where prod_bu = cpl_bu
+              and prod_id = cpl_prod_id
+              and prod_rev = cpl_prod_rev) item_desc,
+       cpl_sales_uom "Sales UOM ",
+       cpl_sales_price  "Sales Price ",
+       cpl_disc_pct "Disc Pct " ,
+       cpl_date_from "Eff From date ",
+       cpl_date_to "Eff To Date ",
+         decode(cpl_status,'N','Draft','A','Approved','C','Cancelled','E','Entry Completed') status,
+       cpl_amd_no
+  from cust_price_list
+  where cpl_bu = 'TVSA'
+    and cpl_plnt = 'U100'
+    and cpl_doc_no = '${PlDocNo}'</t>
+  </si>
+  <si>
+    <t>CatalogueQuery</t>
+  </si>
+  <si>
+    <t>select sctln_doc_no,
+       sctln_prod_id,
+       sctln_prod_rev,
+       (select prod_desc11
+          from products
+         where prod_bu = sctln_bu
+           and prod_id = sctln_prod_id
+           and prod_rev = sctln_prod_rev)item_desc,
+       sctln_uom,
+       to_char(sctln_date_from,'DD-MM-YYYY') sctln_date_from,
+       to_char(sctln_date_to,'DD-MM-YYYY') sctln_date_to,
+       sctln_curcy_id,
+       sctln_seq_no,
+       sctln_ctlg_id,
+       sctln_price,
+       sctln_disc_pct_min,
+       sctln_disc_pct_max,
+       decode (sctln_status,'N','Draft','A','Approved','P','Approved','C','Cancelled','E','Entry Completed')status
+  from sales_catalog_ln
+ where sctln_bu = 'TVSA'
+  and sctln_doc_no = '${CatDocNo}'</t>
+  </si>
+  <si>
+    <t>StdQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     SELECT 
+           SSP_PLNT_LOC_ID "Loc.ID",
+           SSP_PLANT "Unit",
+           SSP_PROD_ID "Item.Id",
+           SSP_PROD_REV "Rev",
+          (SELECT prod_desc11 
+          FROM products
+         WHERE prod_bu = SSP_BU
+           AND prod_id = SSP_PROD_ID
+           AND prod_rev = SSP_PROD_REV) "Item Desc",
+           SSP_CURRENCY "Curcy",
+           SSP_PRICE_UOM "Price UOM",
+           SSP_DATE_FROM "Eff.From Date",
+           SSP_DATE_TO "Eff.To Date",
+           SSP_MAP_PRICE "Map Price" ,
+           SSP_LAND_COST "Landed Cost" ,
+           SSP_STD_PRICE "Selling Price ",
+           SSP_DISC_PCT "Disc Min",
+           SSP_MAX_DISC "Disc Max",
+           SSP_SALES_PRICE_CLASS "Price Class"
+    FROM SALES_STD_PRICES
+    WHERE SSP_BU = 'TVSA'
+    And SSP_PROD_ID = '${StdItemId}'</t>
   </si>
 </sst>
 </file>
@@ -7671,11 +8568,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B894"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75" outlineLevelCol="1"/>
+  <dimension ref="A1:B1029"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7142857142857" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.847619047619" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -14808,27 +15705,1107 @@
       </c>
     </row>
     <row r="892" spans="1:2">
-      <c r="A892" s="71" t="s">
+      <c r="A892" s="34" t="s">
         <v>1526</v>
       </c>
-      <c r="B892" s="72" t="s">
+      <c r="B892" s="35" t="s">
         <v>1527</v>
       </c>
     </row>
     <row r="893" spans="1:2">
-      <c r="A893" s="71" t="s">
+      <c r="A893" s="34" t="s">
         <v>1528</v>
       </c>
-      <c r="B893" s="72" t="s">
+      <c r="B893" s="35" t="s">
         <v>1529</v>
       </c>
     </row>
     <row r="894" spans="1:2">
-      <c r="A894" s="71" t="s">
+      <c r="A894" s="34" t="s">
         <v>1530</v>
       </c>
-      <c r="B894" s="72" t="s">
+      <c r="B894" s="35" t="s">
         <v>1531</v>
+      </c>
+    </row>
+    <row r="895" spans="1:2">
+      <c r="A895" s="71" t="s">
+        <v>1532</v>
+      </c>
+      <c r="B895" s="72" t="s">
+        <v>1533</v>
+      </c>
+    </row>
+    <row r="896" spans="1:2">
+      <c r="A896" s="71" t="s">
+        <v>1534</v>
+      </c>
+      <c r="B896" s="72" t="s">
+        <v>1535</v>
+      </c>
+    </row>
+    <row r="897" spans="1:2">
+      <c r="A897" s="71" t="s">
+        <v>1536</v>
+      </c>
+      <c r="B897" s="72" t="s">
+        <v>1537</v>
+      </c>
+    </row>
+    <row r="898" spans="1:2">
+      <c r="A898" s="71" t="s">
+        <v>1538</v>
+      </c>
+      <c r="B898" s="72" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="899" spans="1:2">
+      <c r="A899" s="71" t="s">
+        <v>1540</v>
+      </c>
+      <c r="B899" s="72" t="s">
+        <v>1541</v>
+      </c>
+    </row>
+    <row r="900" spans="1:2">
+      <c r="A900" s="71" t="s">
+        <v>1542</v>
+      </c>
+      <c r="B900" s="72" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="901" spans="1:2">
+      <c r="A901" s="71" t="s">
+        <v>1544</v>
+      </c>
+      <c r="B901" s="72" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="902" spans="1:2">
+      <c r="A902" s="71" t="s">
+        <v>1545</v>
+      </c>
+      <c r="B902" s="72" t="s">
+        <v>1546</v>
+      </c>
+    </row>
+    <row r="903" spans="1:2">
+      <c r="A903" s="71" t="s">
+        <v>1547</v>
+      </c>
+      <c r="B903" s="72" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="904" spans="1:2">
+      <c r="A904" s="71" t="s">
+        <v>1549</v>
+      </c>
+      <c r="B904" s="72" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="905" spans="1:2">
+      <c r="A905" s="71" t="s">
+        <v>1551</v>
+      </c>
+      <c r="B905" s="72" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="906" spans="1:2">
+      <c r="A906" s="71" t="s">
+        <v>1553</v>
+      </c>
+      <c r="B906" s="72" t="s">
+        <v>1554</v>
+      </c>
+    </row>
+    <row r="907" spans="1:2">
+      <c r="A907" s="71" t="s">
+        <v>1555</v>
+      </c>
+      <c r="B907" s="72" t="s">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="908" spans="1:2">
+      <c r="A908" s="71" t="s">
+        <v>1557</v>
+      </c>
+      <c r="B908" s="72" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="909" spans="1:2">
+      <c r="A909" s="71" t="s">
+        <v>1558</v>
+      </c>
+      <c r="B909" s="72" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="910" spans="1:2">
+      <c r="A910" s="71" t="s">
+        <v>1559</v>
+      </c>
+      <c r="B910" s="72" t="s">
+        <v>1402</v>
+      </c>
+    </row>
+    <row r="911" spans="1:2">
+      <c r="A911" s="71" t="s">
+        <v>1560</v>
+      </c>
+      <c r="B911" s="72" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="912" spans="1:2">
+      <c r="A912" s="34" t="s">
+        <v>1561</v>
+      </c>
+      <c r="B912" s="46" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="913" spans="1:2">
+      <c r="A913" s="71" t="s">
+        <v>1562</v>
+      </c>
+      <c r="B913" s="72" t="s">
+        <v>1563</v>
+      </c>
+    </row>
+    <row r="914" spans="1:2">
+      <c r="A914" s="71" t="s">
+        <v>1564</v>
+      </c>
+      <c r="B914" s="72" t="s">
+        <v>1565</v>
+      </c>
+    </row>
+    <row r="915" spans="1:2">
+      <c r="A915" s="71" t="s">
+        <v>1566</v>
+      </c>
+      <c r="B915" s="72" t="s">
+        <v>1567</v>
+      </c>
+    </row>
+    <row r="916" spans="1:2">
+      <c r="A916" s="71" t="s">
+        <v>1568</v>
+      </c>
+      <c r="B916" s="72" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="917" spans="1:2">
+      <c r="A917" s="71" t="s">
+        <v>1570</v>
+      </c>
+      <c r="B917" s="71" t="s">
+        <v>1570</v>
+      </c>
+    </row>
+    <row r="918" spans="1:2">
+      <c r="A918" s="71" t="s">
+        <v>1571</v>
+      </c>
+      <c r="B918" s="71" t="s">
+        <v>1571</v>
+      </c>
+    </row>
+    <row r="919" spans="1:2">
+      <c r="A919" s="71" t="s">
+        <v>1572</v>
+      </c>
+      <c r="B919" s="71" t="s">
+        <v>1572</v>
+      </c>
+    </row>
+    <row r="920" spans="1:2">
+      <c r="A920" s="71" t="s">
+        <v>1573</v>
+      </c>
+      <c r="B920" s="72" t="s">
+        <v>1574</v>
+      </c>
+    </row>
+    <row r="921" spans="1:2">
+      <c r="A921" s="71" t="s">
+        <v>1575</v>
+      </c>
+      <c r="B921" s="72" t="s">
+        <v>1576</v>
+      </c>
+    </row>
+    <row r="922" spans="1:2">
+      <c r="A922" s="71" t="s">
+        <v>1577</v>
+      </c>
+      <c r="B922" s="72" t="s">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="923" spans="1:2">
+      <c r="A923" s="71" t="s">
+        <v>1579</v>
+      </c>
+      <c r="B923" s="72" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="924" spans="1:2">
+      <c r="A924" s="71" t="s">
+        <v>1580</v>
+      </c>
+      <c r="B924" s="72" t="s">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="925" spans="1:2">
+      <c r="A925" s="71" t="s">
+        <v>1582</v>
+      </c>
+      <c r="B925" s="72" t="s">
+        <v>1583</v>
+      </c>
+    </row>
+    <row r="926" spans="1:2">
+      <c r="A926" s="71" t="s">
+        <v>1584</v>
+      </c>
+      <c r="B926" s="72" t="s">
+        <v>1585</v>
+      </c>
+    </row>
+    <row r="927" spans="1:2">
+      <c r="A927" s="71" t="s">
+        <v>1586</v>
+      </c>
+      <c r="B927" s="72" t="s">
+        <v>1587</v>
+      </c>
+    </row>
+    <row r="928" spans="1:2">
+      <c r="A928" s="71" t="s">
+        <v>761</v>
+      </c>
+      <c r="B928" s="72" t="s">
+        <v>1588</v>
+      </c>
+    </row>
+    <row r="929" spans="1:2">
+      <c r="A929" s="71" t="s">
+        <v>1589</v>
+      </c>
+      <c r="B929" s="72" t="s">
+        <v>1590</v>
+      </c>
+    </row>
+    <row r="930" spans="1:2">
+      <c r="A930" s="71" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B930" s="72" t="s">
+        <v>1592</v>
+      </c>
+    </row>
+    <row r="931" spans="1:2">
+      <c r="A931" s="71" t="s">
+        <v>1593</v>
+      </c>
+      <c r="B931" s="72" t="s">
+        <v>1594</v>
+      </c>
+    </row>
+    <row r="932" spans="1:2">
+      <c r="A932" s="71" t="s">
+        <v>1595</v>
+      </c>
+      <c r="B932" s="72" t="s">
+        <v>1596</v>
+      </c>
+    </row>
+    <row r="933" spans="1:2">
+      <c r="A933" s="71" t="s">
+        <v>1597</v>
+      </c>
+      <c r="B933" s="72" t="s">
+        <v>1598</v>
+      </c>
+    </row>
+    <row r="934" spans="1:2">
+      <c r="A934" s="71" t="s">
+        <v>1599</v>
+      </c>
+      <c r="B934" s="72" t="s">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="935" spans="1:2">
+      <c r="A935" s="71" t="s">
+        <v>1601</v>
+      </c>
+      <c r="B935" s="72" t="s">
+        <v>1602</v>
+      </c>
+    </row>
+    <row r="936" spans="1:2">
+      <c r="A936" s="71" t="s">
+        <v>1603</v>
+      </c>
+      <c r="B936" s="72" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="937" spans="1:2">
+      <c r="A937" s="71" t="s">
+        <v>1605</v>
+      </c>
+      <c r="B937" s="72" t="s">
+        <v>1606</v>
+      </c>
+    </row>
+    <row r="938" spans="1:2">
+      <c r="A938" s="71" t="s">
+        <v>1607</v>
+      </c>
+      <c r="B938" s="72" t="s">
+        <v>1608</v>
+      </c>
+    </row>
+    <row r="939" spans="1:2">
+      <c r="A939" s="71" t="s">
+        <v>1609</v>
+      </c>
+      <c r="B939" s="72" t="s">
+        <v>1610</v>
+      </c>
+    </row>
+    <row r="940" spans="1:2">
+      <c r="A940" s="71" t="s">
+        <v>1611</v>
+      </c>
+      <c r="B940" s="72" t="s">
+        <v>1612</v>
+      </c>
+    </row>
+    <row r="941" spans="1:2">
+      <c r="A941" s="71" t="s">
+        <v>1613</v>
+      </c>
+      <c r="B941" s="72" t="s">
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="942" spans="1:2">
+      <c r="A942" s="71" t="s">
+        <v>1615</v>
+      </c>
+      <c r="B942" s="72" t="s">
+        <v>1616</v>
+      </c>
+    </row>
+    <row r="943" spans="1:2">
+      <c r="A943" s="71" t="s">
+        <v>1617</v>
+      </c>
+      <c r="B943" s="72" t="s">
+        <v>1618</v>
+      </c>
+    </row>
+    <row r="944" spans="1:2">
+      <c r="A944" s="71" t="s">
+        <v>1619</v>
+      </c>
+      <c r="B944" s="72" t="s">
+        <v>1620</v>
+      </c>
+    </row>
+    <row r="945" spans="1:2">
+      <c r="A945" s="71" t="s">
+        <v>1621</v>
+      </c>
+      <c r="B945" s="72" t="s">
+        <v>1622</v>
+      </c>
+    </row>
+    <row r="946" spans="1:2">
+      <c r="A946" s="71" t="s">
+        <v>1623</v>
+      </c>
+      <c r="B946" s="72" t="s">
+        <v>1624</v>
+      </c>
+    </row>
+    <row r="947" spans="1:2">
+      <c r="A947" s="71" t="s">
+        <v>1625</v>
+      </c>
+      <c r="B947" s="72" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="948" spans="1:2">
+      <c r="A948" s="71" t="s">
+        <v>1626</v>
+      </c>
+      <c r="B948" s="72" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="949" spans="1:2">
+      <c r="A949" s="71" t="s">
+        <v>1627</v>
+      </c>
+      <c r="B949" s="72" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="950" spans="1:2">
+      <c r="A950" s="71" t="s">
+        <v>1628</v>
+      </c>
+      <c r="B950" s="72" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="951" spans="1:2">
+      <c r="A951" s="71" t="s">
+        <v>1629</v>
+      </c>
+      <c r="B951" s="72" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="952" spans="1:2">
+      <c r="A952" s="71" t="s">
+        <v>1631</v>
+      </c>
+      <c r="B952" s="72" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="953" spans="1:2">
+      <c r="A953" s="71" t="s">
+        <v>1633</v>
+      </c>
+      <c r="B953" s="72" t="s">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="954" spans="1:2">
+      <c r="A954" s="71" t="s">
+        <v>1635</v>
+      </c>
+      <c r="B954" s="72" t="s">
+        <v>1636</v>
+      </c>
+    </row>
+    <row r="955" spans="1:2">
+      <c r="A955" s="71" t="s">
+        <v>1637</v>
+      </c>
+      <c r="B955" s="72" t="s">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="956" spans="1:2">
+      <c r="A956" s="71" t="s">
+        <v>1639</v>
+      </c>
+      <c r="B956" s="72" t="s">
+        <v>1640</v>
+      </c>
+    </row>
+    <row r="957" spans="1:2">
+      <c r="A957" s="71" t="s">
+        <v>1641</v>
+      </c>
+      <c r="B957" s="72" t="s">
+        <v>1254</v>
+      </c>
+    </row>
+    <row r="958" spans="1:2">
+      <c r="A958" s="71" t="s">
+        <v>1642</v>
+      </c>
+      <c r="B958" s="72" t="s">
+        <v>1256</v>
+      </c>
+    </row>
+    <row r="959" spans="1:2">
+      <c r="A959" s="71" t="s">
+        <v>1643</v>
+      </c>
+      <c r="B959" s="72" t="s">
+        <v>1258</v>
+      </c>
+    </row>
+    <row r="960" spans="1:2">
+      <c r="A960" s="71" t="s">
+        <v>1644</v>
+      </c>
+      <c r="B960" s="72" t="s">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="961" spans="1:2">
+      <c r="A961" s="71" t="s">
+        <v>1645</v>
+      </c>
+      <c r="B961" s="72" t="s">
+        <v>1262</v>
+      </c>
+    </row>
+    <row r="962" spans="1:2">
+      <c r="A962" s="71" t="s">
+        <v>1646</v>
+      </c>
+      <c r="B962" s="72" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="963" spans="1:2">
+      <c r="A963" s="71" t="s">
+        <v>1647</v>
+      </c>
+      <c r="B963" s="72" t="s">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="964" spans="1:2">
+      <c r="A964" s="71" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B964" s="72" t="s">
+        <v>1268</v>
+      </c>
+    </row>
+    <row r="965" spans="1:2">
+      <c r="A965" s="71" t="s">
+        <v>1649</v>
+      </c>
+      <c r="B965" s="72" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="966" spans="1:2">
+      <c r="A966" s="71" t="s">
+        <v>1650</v>
+      </c>
+      <c r="B966" s="72" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="967" spans="1:2">
+      <c r="A967" s="71" t="s">
+        <v>858</v>
+      </c>
+      <c r="B967" s="72" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="968" spans="1:2">
+      <c r="A968" s="71" t="s">
+        <v>859</v>
+      </c>
+      <c r="B968" s="72" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="969" spans="1:2">
+      <c r="A969" s="71" t="s">
+        <v>861</v>
+      </c>
+      <c r="B969" s="72" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="970" spans="1:2">
+      <c r="A970" s="71" t="s">
+        <v>862</v>
+      </c>
+      <c r="B970" s="72" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="971" spans="1:2">
+      <c r="A971" s="71" t="s">
+        <v>864</v>
+      </c>
+      <c r="B971" s="72" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="972" spans="1:2">
+      <c r="A972" s="71" t="s">
+        <v>1651</v>
+      </c>
+      <c r="B972" s="72" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="973" spans="1:2">
+      <c r="A973" s="71" t="s">
+        <v>1652</v>
+      </c>
+      <c r="B973" s="72" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="974" spans="1:2">
+      <c r="A974" s="71" t="s">
+        <v>610</v>
+      </c>
+      <c r="B974" s="72" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="975" spans="1:2">
+      <c r="A975" s="71" t="s">
+        <v>1653</v>
+      </c>
+      <c r="B975" s="72" t="s">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="976" spans="1:2">
+      <c r="A976" s="71" t="s">
+        <v>1654</v>
+      </c>
+      <c r="B976" s="72" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="977" spans="1:2">
+      <c r="A977" s="71" t="s">
+        <v>1655</v>
+      </c>
+      <c r="B977" s="72" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="978" spans="1:2">
+      <c r="A978" s="71" t="s">
+        <v>1656</v>
+      </c>
+      <c r="B978" s="72" t="s">
+        <v>1657</v>
+      </c>
+    </row>
+    <row r="979" spans="1:2">
+      <c r="A979" s="71" t="s">
+        <v>1658</v>
+      </c>
+      <c r="B979" s="72" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="980" spans="1:2">
+      <c r="A980" s="71" t="s">
+        <v>1659</v>
+      </c>
+      <c r="B980" s="72" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="981" spans="1:2">
+      <c r="A981" s="71" t="s">
+        <v>1660</v>
+      </c>
+      <c r="B981" s="72" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="982" spans="1:2">
+      <c r="A982" s="71" t="s">
+        <v>1661</v>
+      </c>
+      <c r="B982" s="72" t="s">
+        <v>1662</v>
+      </c>
+    </row>
+    <row r="983" spans="1:2">
+      <c r="A983" s="71" t="s">
+        <v>1663</v>
+      </c>
+      <c r="B983" s="72" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="984" spans="1:2">
+      <c r="A984" s="71" t="s">
+        <v>1664</v>
+      </c>
+      <c r="B984" s="72" t="s">
+        <v>1665</v>
+      </c>
+    </row>
+    <row r="985" spans="1:2">
+      <c r="A985" s="71" t="s">
+        <v>1666</v>
+      </c>
+      <c r="B985" s="72" t="s">
+        <v>1667</v>
+      </c>
+    </row>
+    <row r="986" spans="1:2">
+      <c r="A986" s="71" t="s">
+        <v>1668</v>
+      </c>
+      <c r="B986" s="72" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="987" spans="1:2">
+      <c r="A987" s="71" t="s">
+        <v>1669</v>
+      </c>
+      <c r="B987" s="72" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="988" spans="1:2">
+      <c r="A988" s="71" t="s">
+        <v>1670</v>
+      </c>
+      <c r="B988" s="72" t="s">
+        <v>1671</v>
+      </c>
+    </row>
+    <row r="989" spans="1:2">
+      <c r="A989" s="71" t="s">
+        <v>1672</v>
+      </c>
+      <c r="B989" s="72" t="s">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="990" spans="1:2">
+      <c r="A990" s="71" t="s">
+        <v>1674</v>
+      </c>
+      <c r="B990" s="72" t="s">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="991" spans="1:2">
+      <c r="A991" s="71" t="s">
+        <v>1676</v>
+      </c>
+      <c r="B991" s="72" t="s">
+        <v>1677</v>
+      </c>
+    </row>
+    <row r="992" spans="1:2">
+      <c r="A992" s="71" t="s">
+        <v>1678</v>
+      </c>
+      <c r="B992" s="72" t="s">
+        <v>1679</v>
+      </c>
+    </row>
+    <row r="993" spans="1:2">
+      <c r="A993" s="71" t="s">
+        <v>1680</v>
+      </c>
+      <c r="B993" s="72" t="s">
+        <v>1681</v>
+      </c>
+    </row>
+    <row r="994" spans="1:2">
+      <c r="A994" s="71" t="s">
+        <v>1682</v>
+      </c>
+      <c r="B994" s="72" t="s">
+        <v>1683</v>
+      </c>
+    </row>
+    <row r="995" spans="1:2">
+      <c r="A995" s="71" t="s">
+        <v>1684</v>
+      </c>
+      <c r="B995" s="72" t="s">
+        <v>1685</v>
+      </c>
+    </row>
+    <row r="996" spans="1:2">
+      <c r="A996" s="71" t="s">
+        <v>1686</v>
+      </c>
+      <c r="B996" s="72" t="s">
+        <v>1687</v>
+      </c>
+    </row>
+    <row r="997" spans="1:2">
+      <c r="A997" s="71" t="s">
+        <v>1688</v>
+      </c>
+      <c r="B997" s="72" t="s">
+        <v>1689</v>
+      </c>
+    </row>
+    <row r="998" spans="1:2">
+      <c r="A998" s="71" t="s">
+        <v>1690</v>
+      </c>
+      <c r="B998" s="72" t="s">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="999" spans="1:2">
+      <c r="A999" s="71" t="s">
+        <v>1692</v>
+      </c>
+      <c r="B999" s="72" t="s">
+        <v>1693</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:2">
+      <c r="A1000" s="71" t="s">
+        <v>1694</v>
+      </c>
+      <c r="B1000" s="72" t="s">
+        <v>1695</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:2">
+      <c r="A1001" s="71" t="s">
+        <v>1696</v>
+      </c>
+      <c r="B1001" s="72" t="s">
+        <v>1697</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:2">
+      <c r="A1002" s="71" t="s">
+        <v>1698</v>
+      </c>
+      <c r="B1002" s="72" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:2">
+      <c r="A1003" s="71" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B1003" s="72" t="s">
+        <v>1701</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:2">
+      <c r="A1004" s="71" t="s">
+        <v>1702</v>
+      </c>
+      <c r="B1004" s="72" t="s">
+        <v>1703</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:2">
+      <c r="A1005" s="71" t="s">
+        <v>1704</v>
+      </c>
+      <c r="B1005" s="72" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:2">
+      <c r="A1006" s="71" t="s">
+        <v>1705</v>
+      </c>
+      <c r="B1006" s="72" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:2">
+      <c r="A1007" s="71" t="s">
+        <v>1707</v>
+      </c>
+      <c r="B1007" s="72" t="s">
+        <v>1708</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:2">
+      <c r="A1008" s="71" t="s">
+        <v>1709</v>
+      </c>
+      <c r="B1008" s="72" t="s">
+        <v>1710</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:2">
+      <c r="A1009" s="71" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B1009" s="72" t="s">
+        <v>1712</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:2">
+      <c r="A1010" s="71" t="s">
+        <v>1713</v>
+      </c>
+      <c r="B1010" s="72" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:2">
+      <c r="A1011" s="71" t="s">
+        <v>1715</v>
+      </c>
+      <c r="B1011" s="72" t="s">
+        <v>1716</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:2">
+      <c r="A1012" s="71" t="s">
+        <v>1717</v>
+      </c>
+      <c r="B1012" s="72" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:2">
+      <c r="A1013" s="71" t="s">
+        <v>1719</v>
+      </c>
+      <c r="B1013" s="72" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:2">
+      <c r="A1014" s="71" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B1014" s="72" t="s">
+        <v>1721</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:2">
+      <c r="A1015" s="71" t="s">
+        <v>1722</v>
+      </c>
+      <c r="B1015" s="72" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:2">
+      <c r="A1016" s="71" t="s">
+        <v>1723</v>
+      </c>
+      <c r="B1016" s="72" t="s">
+        <v>1724</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:2">
+      <c r="A1017" s="71" t="s">
+        <v>1725</v>
+      </c>
+      <c r="B1017" s="72" t="s">
+        <v>1726</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:2">
+      <c r="A1018" s="71" t="s">
+        <v>1727</v>
+      </c>
+      <c r="B1018" s="72" t="s">
+        <v>1728</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:2">
+      <c r="A1019" s="71" t="s">
+        <v>1729</v>
+      </c>
+      <c r="B1019" s="72" t="s">
+        <v>1730</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:2">
+      <c r="A1020" s="71" t="s">
+        <v>1731</v>
+      </c>
+      <c r="B1020" s="72" t="s">
+        <v>1732</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:2">
+      <c r="A1021" s="71" t="s">
+        <v>1733</v>
+      </c>
+      <c r="B1021" s="72" t="s">
+        <v>1734</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:2">
+      <c r="A1022" s="71" t="s">
+        <v>1735</v>
+      </c>
+      <c r="B1022" s="72" t="s">
+        <v>1736</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:2">
+      <c r="A1023" s="71" t="s">
+        <v>1737</v>
+      </c>
+      <c r="B1023" s="72" t="s">
+        <v>1738</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:2">
+      <c r="A1024" s="71" t="s">
+        <v>1739</v>
+      </c>
+      <c r="B1024" s="72" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:2">
+      <c r="A1025" s="71" t="s">
+        <v>1741</v>
+      </c>
+      <c r="B1025" s="72" t="s">
+        <v>1742</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:2">
+      <c r="A1026" s="71" t="s">
+        <v>1743</v>
+      </c>
+      <c r="B1026" s="72" t="s">
+        <v>1744</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:2">
+      <c r="A1027" s="71" t="s">
+        <v>1745</v>
+      </c>
+      <c r="B1027" s="72" t="s">
+        <v>1746</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:2">
+      <c r="A1028" s="71" t="s">
+        <v>1747</v>
+      </c>
+      <c r="B1028" s="72" t="s">
+        <v>1748</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:2">
+      <c r="A1029" s="71" t="s">
+        <v>1749</v>
+      </c>
+      <c r="B1029" s="72" t="s">
+        <v>1750</v>
       </c>
     </row>
   </sheetData>
@@ -14840,10 +16817,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B44"/>
-  <sheetFormatPr defaultColWidth="8.84761904761905" defaultRowHeight="15" outlineLevelCol="1"/>
+  <dimension ref="A1:B51"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.847619047619" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -14857,346 +16834,402 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1532</v>
+        <v>1751</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1533</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1534</v>
+        <v>1753</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1535</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1536</v>
+        <v>1755</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1537</v>
+        <v>1756</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1538</v>
+        <v>1757</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1539</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1540</v>
+        <v>1759</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1541</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1542</v>
+        <v>1761</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1543</v>
+        <v>1762</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1544</v>
+        <v>1763</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1545</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1546</v>
+        <v>1765</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1547</v>
+        <v>1766</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1548</v>
+        <v>1767</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1549</v>
+        <v>1768</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1550</v>
+        <v>1769</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1551</v>
+        <v>1770</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1552</v>
+        <v>1771</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1553</v>
+        <v>1772</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1554</v>
+        <v>1773</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1555</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1556</v>
+        <v>1775</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1557</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1558</v>
+        <v>1777</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1559</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1560</v>
+        <v>1779</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1561</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1562</v>
+        <v>1781</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1563</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1564</v>
+        <v>1783</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1565</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1566</v>
+        <v>1785</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1567</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>1568</v>
+        <v>1787</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1569</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>1570</v>
+        <v>1789</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1571</v>
-      </c>
-    </row>
-    <row r="22" customHeight="1" spans="1:2">
+        <v>1790</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>1572</v>
+        <v>1791</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1573</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>1574</v>
+        <v>1793</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>1575</v>
-      </c>
-    </row>
-    <row r="24" ht="255" spans="1:2">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="24" ht="244.8" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>1576</v>
+        <v>1795</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1577</v>
-      </c>
-    </row>
-    <row r="25" ht="240" spans="1:2">
+        <v>1796</v>
+      </c>
+    </row>
+    <row r="25" ht="230.4" spans="1:2">
       <c r="A25" t="s">
-        <v>1578</v>
+        <v>1797</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1579</v>
-      </c>
-    </row>
-    <row r="26" ht="270" spans="1:2">
+        <v>1798</v>
+      </c>
+    </row>
+    <row r="26" ht="259.2" spans="1:2">
       <c r="A26" t="s">
-        <v>1580</v>
+        <v>1799</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1581</v>
-      </c>
-    </row>
-    <row r="27" ht="210" spans="1:2">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="27" ht="201.6" spans="1:2">
       <c r="A27" t="s">
-        <v>1582</v>
+        <v>1801</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1583</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>1584</v>
+        <v>1803</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1585</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1532</v>
+        <v>1751</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1533</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1534</v>
+        <v>1753</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1535</v>
-      </c>
-    </row>
-    <row r="31" ht="180" spans="1:2">
+        <v>1754</v>
+      </c>
+    </row>
+    <row r="31" ht="172.8" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1540</v>
+        <v>1759</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1541</v>
-      </c>
-    </row>
-    <row r="32" ht="135" spans="1:2">
+        <v>1760</v>
+      </c>
+    </row>
+    <row r="32" ht="129.6" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>1586</v>
+        <v>1805</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>1587</v>
-      </c>
-    </row>
-    <row r="33" ht="180" spans="1:2">
+        <v>1806</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>1588</v>
+        <v>1807</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>1589</v>
-      </c>
-    </row>
-    <row r="34" ht="180" spans="1:2">
+        <v>1808</v>
+      </c>
+    </row>
+    <row r="34" ht="172.8" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>1590</v>
+        <v>1809</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>1591</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>1562</v>
+        <v>1781</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>1592</v>
-      </c>
-    </row>
-    <row r="36" ht="409.5" spans="1:2">
+        <v>1811</v>
+      </c>
+    </row>
+    <row r="36" ht="403.2" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>1593</v>
+        <v>1812</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>1594</v>
+        <v>1813</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>1595</v>
+        <v>1814</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>1596</v>
+        <v>1815</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>1597</v>
+        <v>1816</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1598</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>1599</v>
+        <v>1818</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>1600</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>1601</v>
+        <v>1820</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>1602</v>
-      </c>
-    </row>
-    <row r="41" ht="120" spans="1:2">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="41" ht="115.2" spans="1:2">
       <c r="A41" t="s">
-        <v>1603</v>
+        <v>1822</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>1604</v>
-      </c>
-    </row>
-    <row r="42" ht="180" spans="1:2">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="42" ht="172.8" spans="1:2">
       <c r="A42" t="s">
-        <v>1605</v>
+        <v>1824</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>1606</v>
-      </c>
-    </row>
-    <row r="43" ht="195" spans="1:2">
+        <v>1825</v>
+      </c>
+    </row>
+    <row r="43" ht="187.2" spans="1:2">
       <c r="A43" t="s">
-        <v>1607</v>
+        <v>1826</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>1608</v>
-      </c>
-    </row>
-    <row r="44" ht="120" spans="1:2">
+        <v>1827</v>
+      </c>
+    </row>
+    <row r="44" ht="115.2" spans="1:2">
       <c r="A44" t="s">
-        <v>1609</v>
+        <v>1828</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>1610</v>
+        <v>1829</v>
+      </c>
+    </row>
+    <row r="45" ht="409.5" spans="1:2">
+      <c r="A45" t="s">
+        <v>1830</v>
+      </c>
+      <c r="B45" s="29" t="s">
+        <v>1831</v>
+      </c>
+    </row>
+    <row r="46" ht="409.5" spans="1:2">
+      <c r="A46" t="s">
+        <v>1832</v>
+      </c>
+      <c r="B46" s="29" t="s">
+        <v>1833</v>
+      </c>
+    </row>
+    <row r="47" ht="409.5" spans="1:2">
+      <c r="A47" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B47" s="29" t="s">
+        <v>1835</v>
+      </c>
+    </row>
+    <row r="48" ht="259.2" spans="1:2">
+      <c r="A48" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B48" s="29" t="s">
+        <v>1837</v>
+      </c>
+    </row>
+    <row r="49" ht="409.5" spans="1:2">
+      <c r="A49" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B49" s="29" t="s">
+        <v>1839</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
+      <c r="A50" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B50" s="29" t="s">
+        <v>1841</v>
+      </c>
+    </row>
+    <row r="51" ht="331.2" spans="1:2">
+      <c r="A51" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B51" s="29" t="s">
+        <v>1843</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Employee Adjustment Test Scenarios and Fixed Navigation Screen Scripts
Added Employee Adjustment Test Scenarios and Fixed Navigation Screen Scripts
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" activeTab="1"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2127" uniqueCount="1844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2137" uniqueCount="1853">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5281,6 +5281,33 @@
   </si>
   <si>
     <t>Price List/Standard/Catalog</t>
+  </si>
+  <si>
+    <t>BonusText</t>
+  </si>
+  <si>
+    <t>BONUS</t>
+  </si>
+  <si>
+    <t>HoldStatus</t>
+  </si>
+  <si>
+    <t>Hold</t>
+  </si>
+  <si>
+    <t>ProcessStatus</t>
+  </si>
+  <si>
+    <t>EndedStatus</t>
+  </si>
+  <si>
+    <t>Ended</t>
+  </si>
+  <si>
+    <t>Year202425</t>
+  </si>
+  <si>
+    <t>202425</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -8568,11 +8595,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1029"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
+  <dimension ref="A1:B1034"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -15729,138 +15756,138 @@
       </c>
     </row>
     <row r="895" spans="1:2">
-      <c r="A895" s="71" t="s">
+      <c r="A895" s="34" t="s">
         <v>1532</v>
       </c>
-      <c r="B895" s="72" t="s">
+      <c r="B895" s="35" t="s">
         <v>1533</v>
       </c>
     </row>
     <row r="896" spans="1:2">
-      <c r="A896" s="71" t="s">
+      <c r="A896" s="34" t="s">
         <v>1534</v>
       </c>
-      <c r="B896" s="72" t="s">
+      <c r="B896" s="35" t="s">
         <v>1535</v>
       </c>
     </row>
     <row r="897" spans="1:2">
-      <c r="A897" s="71" t="s">
+      <c r="A897" s="34" t="s">
         <v>1536</v>
       </c>
-      <c r="B897" s="72" t="s">
+      <c r="B897" s="35" t="s">
         <v>1537</v>
       </c>
     </row>
     <row r="898" spans="1:2">
-      <c r="A898" s="71" t="s">
+      <c r="A898" s="34" t="s">
         <v>1538</v>
       </c>
-      <c r="B898" s="72" t="s">
+      <c r="B898" s="35" t="s">
         <v>1539</v>
       </c>
     </row>
     <row r="899" spans="1:2">
-      <c r="A899" s="71" t="s">
+      <c r="A899" s="34" t="s">
         <v>1540</v>
       </c>
-      <c r="B899" s="72" t="s">
+      <c r="B899" s="35" t="s">
         <v>1541</v>
       </c>
     </row>
     <row r="900" spans="1:2">
-      <c r="A900" s="71" t="s">
+      <c r="A900" s="34" t="s">
         <v>1542</v>
       </c>
-      <c r="B900" s="72" t="s">
+      <c r="B900" s="35" t="s">
         <v>1543</v>
       </c>
     </row>
     <row r="901" spans="1:2">
-      <c r="A901" s="71" t="s">
+      <c r="A901" s="34" t="s">
         <v>1544</v>
       </c>
-      <c r="B901" s="72" t="s">
+      <c r="B901" s="35" t="s">
         <v>1544</v>
       </c>
     </row>
     <row r="902" spans="1:2">
-      <c r="A902" s="71" t="s">
+      <c r="A902" s="34" t="s">
         <v>1545</v>
       </c>
-      <c r="B902" s="72" t="s">
+      <c r="B902" s="35" t="s">
         <v>1546</v>
       </c>
     </row>
     <row r="903" spans="1:2">
-      <c r="A903" s="71" t="s">
+      <c r="A903" s="34" t="s">
         <v>1547</v>
       </c>
-      <c r="B903" s="72" t="s">
+      <c r="B903" s="35" t="s">
         <v>1548</v>
       </c>
     </row>
     <row r="904" spans="1:2">
-      <c r="A904" s="71" t="s">
+      <c r="A904" s="34" t="s">
         <v>1549</v>
       </c>
-      <c r="B904" s="72" t="s">
+      <c r="B904" s="35" t="s">
         <v>1550</v>
       </c>
     </row>
     <row r="905" spans="1:2">
-      <c r="A905" s="71" t="s">
+      <c r="A905" s="34" t="s">
         <v>1551</v>
       </c>
-      <c r="B905" s="72" t="s">
+      <c r="B905" s="35" t="s">
         <v>1552</v>
       </c>
     </row>
     <row r="906" spans="1:2">
-      <c r="A906" s="71" t="s">
+      <c r="A906" s="34" t="s">
         <v>1553</v>
       </c>
-      <c r="B906" s="72" t="s">
+      <c r="B906" s="35" t="s">
         <v>1554</v>
       </c>
     </row>
     <row r="907" spans="1:2">
-      <c r="A907" s="71" t="s">
+      <c r="A907" s="34" t="s">
         <v>1555</v>
       </c>
-      <c r="B907" s="72" t="s">
+      <c r="B907" s="35" t="s">
         <v>1556</v>
       </c>
     </row>
     <row r="908" spans="1:2">
-      <c r="A908" s="71" t="s">
+      <c r="A908" s="34" t="s">
         <v>1557</v>
       </c>
-      <c r="B908" s="72" t="s">
+      <c r="B908" s="35" t="s">
         <v>1538</v>
       </c>
     </row>
     <row r="909" spans="1:2">
-      <c r="A909" s="71" t="s">
+      <c r="A909" s="34" t="s">
         <v>1558</v>
       </c>
-      <c r="B909" s="72" t="s">
+      <c r="B909" s="35" t="s">
         <v>1558</v>
       </c>
     </row>
     <row r="910" spans="1:2">
-      <c r="A910" s="71" t="s">
+      <c r="A910" s="34" t="s">
         <v>1559</v>
       </c>
-      <c r="B910" s="72" t="s">
+      <c r="B910" s="35" t="s">
         <v>1402</v>
       </c>
     </row>
     <row r="911" spans="1:2">
-      <c r="A911" s="71" t="s">
+      <c r="A911" s="34" t="s">
         <v>1560</v>
       </c>
-      <c r="B911" s="72" t="s">
+      <c r="B911" s="35" t="s">
         <v>496</v>
       </c>
     </row>
@@ -15873,939 +15900,979 @@
       </c>
     </row>
     <row r="913" spans="1:2">
-      <c r="A913" s="71" t="s">
+      <c r="A913" s="34" t="s">
         <v>1562</v>
       </c>
-      <c r="B913" s="72" t="s">
+      <c r="B913" s="35" t="s">
         <v>1563</v>
       </c>
     </row>
     <row r="914" spans="1:2">
-      <c r="A914" s="71" t="s">
+      <c r="A914" s="34" t="s">
         <v>1564</v>
       </c>
-      <c r="B914" s="72" t="s">
+      <c r="B914" s="35" t="s">
         <v>1565</v>
       </c>
     </row>
     <row r="915" spans="1:2">
-      <c r="A915" s="71" t="s">
+      <c r="A915" s="34" t="s">
         <v>1566</v>
       </c>
-      <c r="B915" s="72" t="s">
+      <c r="B915" s="35" t="s">
         <v>1567</v>
       </c>
     </row>
     <row r="916" spans="1:2">
-      <c r="A916" s="71" t="s">
+      <c r="A916" s="34" t="s">
         <v>1568</v>
       </c>
-      <c r="B916" s="72" t="s">
+      <c r="B916" s="35" t="s">
         <v>1569</v>
       </c>
     </row>
     <row r="917" spans="1:2">
-      <c r="A917" s="71" t="s">
+      <c r="A917" s="34" t="s">
         <v>1570</v>
       </c>
-      <c r="B917" s="71" t="s">
+      <c r="B917" s="34" t="s">
         <v>1570</v>
       </c>
     </row>
     <row r="918" spans="1:2">
-      <c r="A918" s="71" t="s">
+      <c r="A918" s="34" t="s">
         <v>1571</v>
       </c>
-      <c r="B918" s="71" t="s">
+      <c r="B918" s="34" t="s">
         <v>1571</v>
       </c>
     </row>
     <row r="919" spans="1:2">
-      <c r="A919" s="71" t="s">
+      <c r="A919" s="34" t="s">
         <v>1572</v>
       </c>
-      <c r="B919" s="71" t="s">
+      <c r="B919" s="34" t="s">
         <v>1572</v>
       </c>
     </row>
     <row r="920" spans="1:2">
-      <c r="A920" s="71" t="s">
+      <c r="A920" s="34" t="s">
         <v>1573</v>
       </c>
-      <c r="B920" s="72" t="s">
+      <c r="B920" s="35" t="s">
         <v>1574</v>
       </c>
     </row>
     <row r="921" spans="1:2">
-      <c r="A921" s="71" t="s">
+      <c r="A921" s="34" t="s">
         <v>1575</v>
       </c>
-      <c r="B921" s="72" t="s">
+      <c r="B921" s="35" t="s">
         <v>1576</v>
       </c>
     </row>
     <row r="922" spans="1:2">
-      <c r="A922" s="71" t="s">
+      <c r="A922" s="34" t="s">
         <v>1577</v>
       </c>
-      <c r="B922" s="72" t="s">
+      <c r="B922" s="35" t="s">
         <v>1578</v>
       </c>
     </row>
     <row r="923" spans="1:2">
-      <c r="A923" s="71" t="s">
+      <c r="A923" s="34" t="s">
         <v>1579</v>
       </c>
-      <c r="B923" s="72" t="s">
+      <c r="B923" s="35" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="924" spans="1:2">
-      <c r="A924" s="71" t="s">
+      <c r="A924" s="34" t="s">
         <v>1580</v>
       </c>
-      <c r="B924" s="72" t="s">
+      <c r="B924" s="35" t="s">
         <v>1581</v>
       </c>
     </row>
     <row r="925" spans="1:2">
-      <c r="A925" s="71" t="s">
+      <c r="A925" s="34" t="s">
         <v>1582</v>
       </c>
-      <c r="B925" s="72" t="s">
+      <c r="B925" s="35" t="s">
         <v>1583</v>
       </c>
     </row>
     <row r="926" spans="1:2">
-      <c r="A926" s="71" t="s">
+      <c r="A926" s="34" t="s">
         <v>1584</v>
       </c>
-      <c r="B926" s="72" t="s">
+      <c r="B926" s="35" t="s">
         <v>1585</v>
       </c>
     </row>
     <row r="927" spans="1:2">
-      <c r="A927" s="71" t="s">
+      <c r="A927" s="34" t="s">
         <v>1586</v>
       </c>
-      <c r="B927" s="72" t="s">
+      <c r="B927" s="35" t="s">
         <v>1587</v>
       </c>
     </row>
     <row r="928" spans="1:2">
-      <c r="A928" s="71" t="s">
+      <c r="A928" s="34" t="s">
         <v>761</v>
       </c>
-      <c r="B928" s="72" t="s">
+      <c r="B928" s="35" t="s">
         <v>1588</v>
       </c>
     </row>
     <row r="929" spans="1:2">
-      <c r="A929" s="71" t="s">
+      <c r="A929" s="34" t="s">
         <v>1589</v>
       </c>
-      <c r="B929" s="72" t="s">
+      <c r="B929" s="35" t="s">
         <v>1590</v>
       </c>
     </row>
     <row r="930" spans="1:2">
-      <c r="A930" s="71" t="s">
+      <c r="A930" s="34" t="s">
         <v>1591</v>
       </c>
-      <c r="B930" s="72" t="s">
+      <c r="B930" s="35" t="s">
         <v>1592</v>
       </c>
     </row>
     <row r="931" spans="1:2">
-      <c r="A931" s="71" t="s">
+      <c r="A931" s="34" t="s">
         <v>1593</v>
       </c>
-      <c r="B931" s="72" t="s">
+      <c r="B931" s="35" t="s">
         <v>1594</v>
       </c>
     </row>
     <row r="932" spans="1:2">
-      <c r="A932" s="71" t="s">
+      <c r="A932" s="34" t="s">
         <v>1595</v>
       </c>
-      <c r="B932" s="72" t="s">
+      <c r="B932" s="35" t="s">
         <v>1596</v>
       </c>
     </row>
     <row r="933" spans="1:2">
-      <c r="A933" s="71" t="s">
+      <c r="A933" s="34" t="s">
         <v>1597</v>
       </c>
-      <c r="B933" s="72" t="s">
+      <c r="B933" s="35" t="s">
         <v>1598</v>
       </c>
     </row>
     <row r="934" spans="1:2">
-      <c r="A934" s="71" t="s">
+      <c r="A934" s="34" t="s">
         <v>1599</v>
       </c>
-      <c r="B934" s="72" t="s">
+      <c r="B934" s="35" t="s">
         <v>1600</v>
       </c>
     </row>
     <row r="935" spans="1:2">
-      <c r="A935" s="71" t="s">
+      <c r="A935" s="34" t="s">
         <v>1601</v>
       </c>
-      <c r="B935" s="72" t="s">
+      <c r="B935" s="35" t="s">
         <v>1602</v>
       </c>
     </row>
     <row r="936" spans="1:2">
-      <c r="A936" s="71" t="s">
+      <c r="A936" s="34" t="s">
         <v>1603</v>
       </c>
-      <c r="B936" s="72" t="s">
+      <c r="B936" s="35" t="s">
         <v>1604</v>
       </c>
     </row>
     <row r="937" spans="1:2">
-      <c r="A937" s="71" t="s">
+      <c r="A937" s="34" t="s">
         <v>1605</v>
       </c>
-      <c r="B937" s="72" t="s">
+      <c r="B937" s="35" t="s">
         <v>1606</v>
       </c>
     </row>
     <row r="938" spans="1:2">
-      <c r="A938" s="71" t="s">
+      <c r="A938" s="34" t="s">
         <v>1607</v>
       </c>
-      <c r="B938" s="72" t="s">
+      <c r="B938" s="35" t="s">
         <v>1608</v>
       </c>
     </row>
     <row r="939" spans="1:2">
-      <c r="A939" s="71" t="s">
+      <c r="A939" s="34" t="s">
         <v>1609</v>
       </c>
-      <c r="B939" s="72" t="s">
+      <c r="B939" s="35" t="s">
         <v>1610</v>
       </c>
     </row>
     <row r="940" spans="1:2">
-      <c r="A940" s="71" t="s">
+      <c r="A940" s="34" t="s">
         <v>1611</v>
       </c>
-      <c r="B940" s="72" t="s">
+      <c r="B940" s="35" t="s">
         <v>1612</v>
       </c>
     </row>
     <row r="941" spans="1:2">
-      <c r="A941" s="71" t="s">
+      <c r="A941" s="34" t="s">
         <v>1613</v>
       </c>
-      <c r="B941" s="72" t="s">
+      <c r="B941" s="35" t="s">
         <v>1614</v>
       </c>
     </row>
     <row r="942" spans="1:2">
-      <c r="A942" s="71" t="s">
+      <c r="A942" s="34" t="s">
         <v>1615</v>
       </c>
-      <c r="B942" s="72" t="s">
+      <c r="B942" s="35" t="s">
         <v>1616</v>
       </c>
     </row>
     <row r="943" spans="1:2">
-      <c r="A943" s="71" t="s">
+      <c r="A943" s="34" t="s">
         <v>1617</v>
       </c>
-      <c r="B943" s="72" t="s">
+      <c r="B943" s="35" t="s">
         <v>1618</v>
       </c>
     </row>
     <row r="944" spans="1:2">
-      <c r="A944" s="71" t="s">
+      <c r="A944" s="34" t="s">
         <v>1619</v>
       </c>
-      <c r="B944" s="72" t="s">
+      <c r="B944" s="35" t="s">
         <v>1620</v>
       </c>
     </row>
     <row r="945" spans="1:2">
-      <c r="A945" s="71" t="s">
+      <c r="A945" s="34" t="s">
         <v>1621</v>
       </c>
-      <c r="B945" s="72" t="s">
+      <c r="B945" s="35" t="s">
         <v>1622</v>
       </c>
     </row>
     <row r="946" spans="1:2">
-      <c r="A946" s="71" t="s">
+      <c r="A946" s="34" t="s">
         <v>1623</v>
       </c>
-      <c r="B946" s="72" t="s">
+      <c r="B946" s="35" t="s">
         <v>1624</v>
       </c>
     </row>
     <row r="947" spans="1:2">
-      <c r="A947" s="71" t="s">
+      <c r="A947" s="34" t="s">
         <v>1625</v>
       </c>
-      <c r="B947" s="72" t="s">
+      <c r="B947" s="35" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="948" spans="1:2">
-      <c r="A948" s="71" t="s">
+      <c r="A948" s="34" t="s">
         <v>1626</v>
       </c>
-      <c r="B948" s="72" t="s">
+      <c r="B948" s="35" t="s">
         <v>564</v>
       </c>
     </row>
     <row r="949" spans="1:2">
-      <c r="A949" s="71" t="s">
+      <c r="A949" s="34" t="s">
         <v>1627</v>
       </c>
-      <c r="B949" s="72" t="s">
+      <c r="B949" s="35" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="950" spans="1:2">
-      <c r="A950" s="71" t="s">
+      <c r="A950" s="34" t="s">
         <v>1628</v>
       </c>
-      <c r="B950" s="72" t="s">
+      <c r="B950" s="35" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="951" spans="1:2">
-      <c r="A951" s="71" t="s">
+      <c r="A951" s="34" t="s">
         <v>1629</v>
       </c>
-      <c r="B951" s="72" t="s">
+      <c r="B951" s="35" t="s">
         <v>1630</v>
       </c>
     </row>
     <row r="952" spans="1:2">
-      <c r="A952" s="71" t="s">
+      <c r="A952" s="34" t="s">
         <v>1631</v>
       </c>
-      <c r="B952" s="72" t="s">
+      <c r="B952" s="35" t="s">
         <v>1632</v>
       </c>
     </row>
     <row r="953" spans="1:2">
-      <c r="A953" s="71" t="s">
+      <c r="A953" s="34" t="s">
         <v>1633</v>
       </c>
-      <c r="B953" s="72" t="s">
+      <c r="B953" s="35" t="s">
         <v>1634</v>
       </c>
     </row>
     <row r="954" spans="1:2">
-      <c r="A954" s="71" t="s">
+      <c r="A954" s="34" t="s">
         <v>1635</v>
       </c>
-      <c r="B954" s="72" t="s">
+      <c r="B954" s="35" t="s">
         <v>1636</v>
       </c>
     </row>
     <row r="955" spans="1:2">
-      <c r="A955" s="71" t="s">
+      <c r="A955" s="34" t="s">
         <v>1637</v>
       </c>
-      <c r="B955" s="72" t="s">
+      <c r="B955" s="35" t="s">
         <v>1638</v>
       </c>
     </row>
     <row r="956" spans="1:2">
-      <c r="A956" s="71" t="s">
+      <c r="A956" s="34" t="s">
         <v>1639</v>
       </c>
-      <c r="B956" s="72" t="s">
+      <c r="B956" s="35" t="s">
         <v>1640</v>
       </c>
     </row>
     <row r="957" spans="1:2">
-      <c r="A957" s="71" t="s">
+      <c r="A957" s="34" t="s">
         <v>1641</v>
       </c>
-      <c r="B957" s="72" t="s">
+      <c r="B957" s="35" t="s">
         <v>1254</v>
       </c>
     </row>
     <row r="958" spans="1:2">
-      <c r="A958" s="71" t="s">
+      <c r="A958" s="34" t="s">
         <v>1642</v>
       </c>
-      <c r="B958" s="72" t="s">
+      <c r="B958" s="35" t="s">
         <v>1256</v>
       </c>
     </row>
     <row r="959" spans="1:2">
-      <c r="A959" s="71" t="s">
+      <c r="A959" s="34" t="s">
         <v>1643</v>
       </c>
-      <c r="B959" s="72" t="s">
+      <c r="B959" s="35" t="s">
         <v>1258</v>
       </c>
     </row>
     <row r="960" spans="1:2">
-      <c r="A960" s="71" t="s">
+      <c r="A960" s="34" t="s">
         <v>1644</v>
       </c>
-      <c r="B960" s="72" t="s">
+      <c r="B960" s="35" t="s">
         <v>1260</v>
       </c>
     </row>
     <row r="961" spans="1:2">
-      <c r="A961" s="71" t="s">
+      <c r="A961" s="34" t="s">
         <v>1645</v>
       </c>
-      <c r="B961" s="72" t="s">
+      <c r="B961" s="35" t="s">
         <v>1262</v>
       </c>
     </row>
     <row r="962" spans="1:2">
-      <c r="A962" s="71" t="s">
+      <c r="A962" s="34" t="s">
         <v>1646</v>
       </c>
-      <c r="B962" s="72" t="s">
+      <c r="B962" s="35" t="s">
         <v>1264</v>
       </c>
     </row>
     <row r="963" spans="1:2">
-      <c r="A963" s="71" t="s">
+      <c r="A963" s="34" t="s">
         <v>1647</v>
       </c>
-      <c r="B963" s="72" t="s">
+      <c r="B963" s="35" t="s">
         <v>1266</v>
       </c>
     </row>
     <row r="964" spans="1:2">
-      <c r="A964" s="71" t="s">
+      <c r="A964" s="34" t="s">
         <v>1648</v>
       </c>
-      <c r="B964" s="72" t="s">
+      <c r="B964" s="35" t="s">
         <v>1268</v>
       </c>
     </row>
     <row r="965" spans="1:2">
-      <c r="A965" s="71" t="s">
+      <c r="A965" s="34" t="s">
         <v>1649</v>
       </c>
-      <c r="B965" s="72" t="s">
+      <c r="B965" s="35" t="s">
         <v>1270</v>
       </c>
     </row>
     <row r="966" spans="1:2">
-      <c r="A966" s="71" t="s">
+      <c r="A966" s="34" t="s">
         <v>1650</v>
       </c>
-      <c r="B966" s="72" t="s">
+      <c r="B966" s="35" t="s">
         <v>564</v>
       </c>
     </row>
     <row r="967" spans="1:2">
-      <c r="A967" s="71" t="s">
+      <c r="A967" s="34" t="s">
         <v>858</v>
       </c>
-      <c r="B967" s="72" t="s">
+      <c r="B967" s="35" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="968" spans="1:2">
-      <c r="A968" s="71" t="s">
+      <c r="A968" s="34" t="s">
         <v>859</v>
       </c>
-      <c r="B968" s="72" t="s">
+      <c r="B968" s="35" t="s">
         <v>860</v>
       </c>
     </row>
     <row r="969" spans="1:2">
-      <c r="A969" s="71" t="s">
+      <c r="A969" s="34" t="s">
         <v>861</v>
       </c>
-      <c r="B969" s="72" t="s">
+      <c r="B969" s="35" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="970" spans="1:2">
-      <c r="A970" s="71" t="s">
+      <c r="A970" s="34" t="s">
         <v>862</v>
       </c>
-      <c r="B970" s="72" t="s">
+      <c r="B970" s="35" t="s">
         <v>863</v>
       </c>
     </row>
     <row r="971" spans="1:2">
-      <c r="A971" s="71" t="s">
+      <c r="A971" s="34" t="s">
         <v>864</v>
       </c>
-      <c r="B971" s="72" t="s">
+      <c r="B971" s="35" t="s">
         <v>865</v>
       </c>
     </row>
     <row r="972" spans="1:2">
-      <c r="A972" s="71" t="s">
+      <c r="A972" s="34" t="s">
         <v>1651</v>
       </c>
-      <c r="B972" s="72" t="s">
+      <c r="B972" s="35" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="973" spans="1:2">
-      <c r="A973" s="71" t="s">
+      <c r="A973" s="34" t="s">
         <v>1652</v>
       </c>
-      <c r="B973" s="72" t="s">
+      <c r="B973" s="35" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="974" spans="1:2">
-      <c r="A974" s="71" t="s">
+      <c r="A974" s="34" t="s">
         <v>610</v>
       </c>
-      <c r="B974" s="72" t="s">
+      <c r="B974" s="35" t="s">
         <v>610</v>
       </c>
     </row>
     <row r="975" spans="1:2">
-      <c r="A975" s="71" t="s">
+      <c r="A975" s="34" t="s">
         <v>1653</v>
       </c>
-      <c r="B975" s="72" t="s">
+      <c r="B975" s="35" t="s">
         <v>1556</v>
       </c>
     </row>
     <row r="976" spans="1:2">
-      <c r="A976" s="71" t="s">
+      <c r="A976" s="34" t="s">
         <v>1654</v>
       </c>
-      <c r="B976" s="72" t="s">
+      <c r="B976" s="35" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="977" spans="1:2">
-      <c r="A977" s="71" t="s">
+      <c r="A977" s="34" t="s">
         <v>1655</v>
       </c>
-      <c r="B977" s="72" t="s">
+      <c r="B977" s="35" t="s">
         <v>410</v>
       </c>
     </row>
     <row r="978" spans="1:2">
-      <c r="A978" s="71" t="s">
+      <c r="A978" s="34" t="s">
         <v>1656</v>
       </c>
-      <c r="B978" s="72" t="s">
+      <c r="B978" s="35" t="s">
         <v>1657</v>
       </c>
     </row>
     <row r="979" spans="1:2">
-      <c r="A979" s="71" t="s">
+      <c r="A979" s="34" t="s">
         <v>1658</v>
       </c>
-      <c r="B979" s="72" t="s">
+      <c r="B979" s="35" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="980" spans="1:2">
-      <c r="A980" s="71" t="s">
+      <c r="A980" s="34" t="s">
         <v>1659</v>
       </c>
-      <c r="B980" s="72" t="s">
+      <c r="B980" s="35" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="981" spans="1:2">
-      <c r="A981" s="71" t="s">
+      <c r="A981" s="34" t="s">
         <v>1660</v>
       </c>
-      <c r="B981" s="72" t="s">
+      <c r="B981" s="35" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="982" spans="1:2">
-      <c r="A982" s="71" t="s">
+      <c r="A982" s="34" t="s">
         <v>1661</v>
       </c>
-      <c r="B982" s="72" t="s">
+      <c r="B982" s="35" t="s">
         <v>1662</v>
       </c>
     </row>
     <row r="983" spans="1:2">
-      <c r="A983" s="71" t="s">
+      <c r="A983" s="34" t="s">
         <v>1663</v>
       </c>
-      <c r="B983" s="72" t="s">
+      <c r="B983" s="35" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="984" spans="1:2">
-      <c r="A984" s="71" t="s">
+      <c r="A984" s="34" t="s">
         <v>1664</v>
       </c>
-      <c r="B984" s="72" t="s">
+      <c r="B984" s="35" t="s">
         <v>1665</v>
       </c>
     </row>
     <row r="985" spans="1:2">
-      <c r="A985" s="71" t="s">
+      <c r="A985" s="34" t="s">
         <v>1666</v>
       </c>
-      <c r="B985" s="72" t="s">
+      <c r="B985" s="35" t="s">
         <v>1667</v>
       </c>
     </row>
     <row r="986" spans="1:2">
-      <c r="A986" s="71" t="s">
+      <c r="A986" s="34" t="s">
         <v>1668</v>
       </c>
-      <c r="B986" s="72" t="s">
+      <c r="B986" s="35" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="987" spans="1:2">
-      <c r="A987" s="71" t="s">
+      <c r="A987" s="34" t="s">
         <v>1669</v>
       </c>
-      <c r="B987" s="72" t="s">
+      <c r="B987" s="35" t="s">
         <v>410</v>
       </c>
     </row>
     <row r="988" spans="1:2">
-      <c r="A988" s="71" t="s">
+      <c r="A988" s="34" t="s">
         <v>1670</v>
       </c>
-      <c r="B988" s="72" t="s">
+      <c r="B988" s="35" t="s">
         <v>1671</v>
       </c>
     </row>
     <row r="989" spans="1:2">
-      <c r="A989" s="71" t="s">
+      <c r="A989" s="34" t="s">
         <v>1672</v>
       </c>
-      <c r="B989" s="72" t="s">
+      <c r="B989" s="35" t="s">
         <v>1673</v>
       </c>
     </row>
     <row r="990" spans="1:2">
-      <c r="A990" s="71" t="s">
+      <c r="A990" s="34" t="s">
         <v>1674</v>
       </c>
-      <c r="B990" s="72" t="s">
+      <c r="B990" s="35" t="s">
         <v>1675</v>
       </c>
     </row>
     <row r="991" spans="1:2">
-      <c r="A991" s="71" t="s">
+      <c r="A991" s="34" t="s">
         <v>1676</v>
       </c>
-      <c r="B991" s="72" t="s">
+      <c r="B991" s="35" t="s">
         <v>1677</v>
       </c>
     </row>
     <row r="992" spans="1:2">
-      <c r="A992" s="71" t="s">
+      <c r="A992" s="34" t="s">
         <v>1678</v>
       </c>
-      <c r="B992" s="72" t="s">
+      <c r="B992" s="35" t="s">
         <v>1679</v>
       </c>
     </row>
     <row r="993" spans="1:2">
-      <c r="A993" s="71" t="s">
+      <c r="A993" s="34" t="s">
         <v>1680</v>
       </c>
-      <c r="B993" s="72" t="s">
+      <c r="B993" s="35" t="s">
         <v>1681</v>
       </c>
     </row>
     <row r="994" spans="1:2">
-      <c r="A994" s="71" t="s">
+      <c r="A994" s="34" t="s">
         <v>1682</v>
       </c>
-      <c r="B994" s="72" t="s">
+      <c r="B994" s="35" t="s">
         <v>1683</v>
       </c>
     </row>
     <row r="995" spans="1:2">
-      <c r="A995" s="71" t="s">
+      <c r="A995" s="34" t="s">
         <v>1684</v>
       </c>
-      <c r="B995" s="72" t="s">
+      <c r="B995" s="35" t="s">
         <v>1685</v>
       </c>
     </row>
     <row r="996" spans="1:2">
-      <c r="A996" s="71" t="s">
+      <c r="A996" s="34" t="s">
         <v>1686</v>
       </c>
-      <c r="B996" s="72" t="s">
+      <c r="B996" s="35" t="s">
         <v>1687</v>
       </c>
     </row>
     <row r="997" spans="1:2">
-      <c r="A997" s="71" t="s">
+      <c r="A997" s="34" t="s">
         <v>1688</v>
       </c>
-      <c r="B997" s="72" t="s">
+      <c r="B997" s="35" t="s">
         <v>1689</v>
       </c>
     </row>
     <row r="998" spans="1:2">
-      <c r="A998" s="71" t="s">
+      <c r="A998" s="34" t="s">
         <v>1690</v>
       </c>
-      <c r="B998" s="72" t="s">
+      <c r="B998" s="35" t="s">
         <v>1691</v>
       </c>
     </row>
     <row r="999" spans="1:2">
-      <c r="A999" s="71" t="s">
+      <c r="A999" s="34" t="s">
         <v>1692</v>
       </c>
-      <c r="B999" s="72" t="s">
+      <c r="B999" s="35" t="s">
         <v>1693</v>
       </c>
     </row>
     <row r="1000" spans="1:2">
-      <c r="A1000" s="71" t="s">
+      <c r="A1000" s="34" t="s">
         <v>1694</v>
       </c>
-      <c r="B1000" s="72" t="s">
+      <c r="B1000" s="35" t="s">
         <v>1695</v>
       </c>
     </row>
     <row r="1001" spans="1:2">
-      <c r="A1001" s="71" t="s">
+      <c r="A1001" s="34" t="s">
         <v>1696</v>
       </c>
-      <c r="B1001" s="72" t="s">
+      <c r="B1001" s="35" t="s">
         <v>1697</v>
       </c>
     </row>
     <row r="1002" spans="1:2">
-      <c r="A1002" s="71" t="s">
+      <c r="A1002" s="34" t="s">
         <v>1698</v>
       </c>
-      <c r="B1002" s="72" t="s">
+      <c r="B1002" s="35" t="s">
         <v>1699</v>
       </c>
     </row>
     <row r="1003" spans="1:2">
-      <c r="A1003" s="71" t="s">
+      <c r="A1003" s="34" t="s">
         <v>1700</v>
       </c>
-      <c r="B1003" s="72" t="s">
+      <c r="B1003" s="35" t="s">
         <v>1701</v>
       </c>
     </row>
     <row r="1004" spans="1:2">
-      <c r="A1004" s="71" t="s">
+      <c r="A1004" s="34" t="s">
         <v>1702</v>
       </c>
-      <c r="B1004" s="72" t="s">
+      <c r="B1004" s="35" t="s">
         <v>1703</v>
       </c>
     </row>
     <row r="1005" spans="1:2">
-      <c r="A1005" s="71" t="s">
+      <c r="A1005" s="34" t="s">
         <v>1704</v>
       </c>
-      <c r="B1005" s="72" t="s">
+      <c r="B1005" s="35" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="1006" spans="1:2">
-      <c r="A1006" s="71" t="s">
+      <c r="A1006" s="34" t="s">
         <v>1705</v>
       </c>
-      <c r="B1006" s="72" t="s">
+      <c r="B1006" s="35" t="s">
         <v>1706</v>
       </c>
     </row>
     <row r="1007" spans="1:2">
-      <c r="A1007" s="71" t="s">
+      <c r="A1007" s="34" t="s">
         <v>1707</v>
       </c>
-      <c r="B1007" s="72" t="s">
+      <c r="B1007" s="35" t="s">
         <v>1708</v>
       </c>
     </row>
     <row r="1008" spans="1:2">
-      <c r="A1008" s="71" t="s">
+      <c r="A1008" s="34" t="s">
         <v>1709</v>
       </c>
-      <c r="B1008" s="72" t="s">
+      <c r="B1008" s="35" t="s">
         <v>1710</v>
       </c>
     </row>
     <row r="1009" spans="1:2">
-      <c r="A1009" s="71" t="s">
+      <c r="A1009" s="34" t="s">
         <v>1711</v>
       </c>
-      <c r="B1009" s="72" t="s">
+      <c r="B1009" s="35" t="s">
         <v>1712</v>
       </c>
     </row>
     <row r="1010" spans="1:2">
-      <c r="A1010" s="71" t="s">
+      <c r="A1010" s="34" t="s">
         <v>1713</v>
       </c>
-      <c r="B1010" s="72" t="s">
+      <c r="B1010" s="35" t="s">
         <v>1714</v>
       </c>
     </row>
     <row r="1011" spans="1:2">
-      <c r="A1011" s="71" t="s">
+      <c r="A1011" s="34" t="s">
         <v>1715</v>
       </c>
-      <c r="B1011" s="72" t="s">
+      <c r="B1011" s="35" t="s">
         <v>1716</v>
       </c>
     </row>
     <row r="1012" spans="1:2">
-      <c r="A1012" s="71" t="s">
+      <c r="A1012" s="34" t="s">
         <v>1717</v>
       </c>
-      <c r="B1012" s="72" t="s">
+      <c r="B1012" s="35" t="s">
         <v>1718</v>
       </c>
     </row>
     <row r="1013" spans="1:2">
-      <c r="A1013" s="71" t="s">
+      <c r="A1013" s="34" t="s">
         <v>1719</v>
       </c>
-      <c r="B1013" s="72" t="s">
+      <c r="B1013" s="35" t="s">
         <v>480</v>
       </c>
     </row>
     <row r="1014" spans="1:2">
-      <c r="A1014" s="71" t="s">
+      <c r="A1014" s="34" t="s">
         <v>1720</v>
       </c>
-      <c r="B1014" s="72" t="s">
+      <c r="B1014" s="35" t="s">
         <v>1721</v>
       </c>
     </row>
     <row r="1015" spans="1:2">
-      <c r="A1015" s="71" t="s">
+      <c r="A1015" s="34" t="s">
         <v>1722</v>
       </c>
-      <c r="B1015" s="72" t="s">
+      <c r="B1015" s="35" t="s">
         <v>661</v>
       </c>
     </row>
     <row r="1016" spans="1:2">
-      <c r="A1016" s="71" t="s">
+      <c r="A1016" s="34" t="s">
         <v>1723</v>
       </c>
-      <c r="B1016" s="72" t="s">
+      <c r="B1016" s="35" t="s">
         <v>1724</v>
       </c>
     </row>
     <row r="1017" spans="1:2">
-      <c r="A1017" s="71" t="s">
+      <c r="A1017" s="34" t="s">
         <v>1725</v>
       </c>
-      <c r="B1017" s="72" t="s">
+      <c r="B1017" s="35" t="s">
         <v>1726</v>
       </c>
     </row>
     <row r="1018" spans="1:2">
-      <c r="A1018" s="71" t="s">
+      <c r="A1018" s="34" t="s">
         <v>1727</v>
       </c>
-      <c r="B1018" s="72" t="s">
+      <c r="B1018" s="35" t="s">
         <v>1728</v>
       </c>
     </row>
     <row r="1019" spans="1:2">
-      <c r="A1019" s="71" t="s">
+      <c r="A1019" s="34" t="s">
         <v>1729</v>
       </c>
-      <c r="B1019" s="72" t="s">
+      <c r="B1019" s="35" t="s">
         <v>1730</v>
       </c>
     </row>
     <row r="1020" spans="1:2">
-      <c r="A1020" s="71" t="s">
+      <c r="A1020" s="34" t="s">
         <v>1731</v>
       </c>
-      <c r="B1020" s="72" t="s">
+      <c r="B1020" s="35" t="s">
         <v>1732</v>
       </c>
     </row>
     <row r="1021" spans="1:2">
-      <c r="A1021" s="71" t="s">
+      <c r="A1021" s="34" t="s">
         <v>1733</v>
       </c>
-      <c r="B1021" s="72" t="s">
+      <c r="B1021" s="35" t="s">
         <v>1734</v>
       </c>
     </row>
     <row r="1022" spans="1:2">
-      <c r="A1022" s="71" t="s">
+      <c r="A1022" s="34" t="s">
         <v>1735</v>
       </c>
-      <c r="B1022" s="72" t="s">
+      <c r="B1022" s="35" t="s">
         <v>1736</v>
       </c>
     </row>
     <row r="1023" spans="1:2">
-      <c r="A1023" s="71" t="s">
+      <c r="A1023" s="34" t="s">
         <v>1737</v>
       </c>
-      <c r="B1023" s="72" t="s">
+      <c r="B1023" s="35" t="s">
         <v>1738</v>
       </c>
     </row>
     <row r="1024" spans="1:2">
-      <c r="A1024" s="71" t="s">
+      <c r="A1024" s="34" t="s">
         <v>1739</v>
       </c>
-      <c r="B1024" s="72" t="s">
+      <c r="B1024" s="35" t="s">
         <v>1740</v>
       </c>
     </row>
     <row r="1025" spans="1:2">
-      <c r="A1025" s="71" t="s">
+      <c r="A1025" s="34" t="s">
         <v>1741</v>
       </c>
-      <c r="B1025" s="72" t="s">
+      <c r="B1025" s="35" t="s">
         <v>1742</v>
       </c>
     </row>
     <row r="1026" spans="1:2">
-      <c r="A1026" s="71" t="s">
+      <c r="A1026" s="34" t="s">
         <v>1743</v>
       </c>
-      <c r="B1026" s="72" t="s">
+      <c r="B1026" s="35" t="s">
         <v>1744</v>
       </c>
     </row>
     <row r="1027" spans="1:2">
-      <c r="A1027" s="71" t="s">
+      <c r="A1027" s="34" t="s">
         <v>1745</v>
       </c>
-      <c r="B1027" s="72" t="s">
+      <c r="B1027" s="35" t="s">
         <v>1746</v>
       </c>
     </row>
     <row r="1028" spans="1:2">
-      <c r="A1028" s="71" t="s">
+      <c r="A1028" s="34" t="s">
         <v>1747</v>
       </c>
-      <c r="B1028" s="72" t="s">
+      <c r="B1028" s="35" t="s">
         <v>1748</v>
       </c>
     </row>
     <row r="1029" spans="1:2">
-      <c r="A1029" s="71" t="s">
+      <c r="A1029" s="34" t="s">
         <v>1749</v>
       </c>
-      <c r="B1029" s="72" t="s">
+      <c r="B1029" s="35" t="s">
         <v>1750</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:2">
+      <c r="A1030" s="71" t="s">
+        <v>1751</v>
+      </c>
+      <c r="B1030" s="72" t="s">
+        <v>1752</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:2">
+      <c r="A1031" s="71" t="s">
+        <v>1753</v>
+      </c>
+      <c r="B1031" s="72" t="s">
+        <v>1754</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:2">
+      <c r="A1032" s="71" t="s">
+        <v>1755</v>
+      </c>
+      <c r="B1032" s="72" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:2">
+      <c r="A1033" s="71" t="s">
+        <v>1756</v>
+      </c>
+      <c r="B1033" s="72" t="s">
+        <v>1757</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:2">
+      <c r="A1034" s="71" t="s">
+        <v>1758</v>
+      </c>
+      <c r="B1034" s="72" t="s">
+        <v>1759</v>
       </c>
     </row>
   </sheetData>
@@ -16818,9 +16885,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B51"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
+    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16834,402 +16901,402 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1751</v>
+        <v>1760</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1752</v>
+        <v>1761</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1753</v>
+        <v>1762</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1754</v>
+        <v>1763</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1755</v>
+        <v>1764</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1756</v>
+        <v>1765</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1757</v>
+        <v>1766</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1758</v>
+        <v>1767</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1759</v>
+        <v>1768</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1760</v>
+        <v>1769</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1761</v>
+        <v>1770</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1762</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1763</v>
+        <v>1772</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1764</v>
+        <v>1773</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1765</v>
+        <v>1774</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1766</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1767</v>
+        <v>1776</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1768</v>
+        <v>1777</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1769</v>
+        <v>1778</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1770</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1771</v>
+        <v>1780</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1772</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1773</v>
+        <v>1782</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1774</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1775</v>
+        <v>1784</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1776</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1777</v>
+        <v>1786</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1778</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1779</v>
+        <v>1788</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1780</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1781</v>
+        <v>1790</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1782</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1783</v>
+        <v>1792</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1784</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1785</v>
+        <v>1794</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1786</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>1787</v>
+        <v>1796</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1788</v>
+        <v>1797</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>1789</v>
+        <v>1798</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1790</v>
+        <v>1799</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>1791</v>
+        <v>1800</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1792</v>
+        <v>1801</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>1793</v>
+        <v>1802</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>1794</v>
-      </c>
-    </row>
-    <row r="24" ht="244.8" spans="1:2">
+        <v>1803</v>
+      </c>
+    </row>
+    <row r="24" ht="246.5" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>1795</v>
+        <v>1804</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1796</v>
-      </c>
-    </row>
-    <row r="25" ht="230.4" spans="1:2">
+        <v>1805</v>
+      </c>
+    </row>
+    <row r="25" ht="232" spans="1:2">
       <c r="A25" t="s">
-        <v>1797</v>
+        <v>1806</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1798</v>
-      </c>
-    </row>
-    <row r="26" ht="259.2" spans="1:2">
+        <v>1807</v>
+      </c>
+    </row>
+    <row r="26" ht="261" spans="1:2">
       <c r="A26" t="s">
-        <v>1799</v>
+        <v>1808</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="27" ht="201.6" spans="1:2">
+        <v>1809</v>
+      </c>
+    </row>
+    <row r="27" ht="203" spans="1:2">
       <c r="A27" t="s">
-        <v>1801</v>
+        <v>1810</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1802</v>
+        <v>1811</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>1803</v>
+        <v>1812</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1804</v>
+        <v>1813</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1751</v>
+        <v>1760</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1752</v>
+        <v>1761</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1753</v>
+        <v>1762</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1754</v>
-      </c>
-    </row>
-    <row r="31" ht="172.8" spans="1:2">
+        <v>1763</v>
+      </c>
+    </row>
+    <row r="31" ht="174" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1759</v>
+        <v>1768</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1760</v>
-      </c>
-    </row>
-    <row r="32" ht="129.6" spans="1:2">
+        <v>1769</v>
+      </c>
+    </row>
+    <row r="32" ht="130.5" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>1805</v>
+        <v>1814</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>1806</v>
-      </c>
-    </row>
-    <row r="33" ht="172.8" spans="1:2">
+        <v>1815</v>
+      </c>
+    </row>
+    <row r="33" ht="174" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>1807</v>
+        <v>1816</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>1808</v>
-      </c>
-    </row>
-    <row r="34" ht="172.8" spans="1:2">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="34" ht="174" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>1809</v>
+        <v>1818</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>1810</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>1781</v>
+        <v>1790</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>1811</v>
-      </c>
-    </row>
-    <row r="36" ht="403.2" spans="1:2">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="36" ht="406" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>1812</v>
+        <v>1821</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>1813</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>1814</v>
+        <v>1823</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>1815</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>1816</v>
+        <v>1825</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1817</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>1818</v>
+        <v>1827</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>1819</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>1820</v>
+        <v>1829</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="41" ht="115.2" spans="1:2">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="41" ht="116" spans="1:2">
       <c r="A41" t="s">
-        <v>1822</v>
+        <v>1831</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>1823</v>
-      </c>
-    </row>
-    <row r="42" ht="172.8" spans="1:2">
+        <v>1832</v>
+      </c>
+    </row>
+    <row r="42" ht="174" spans="1:2">
       <c r="A42" t="s">
-        <v>1824</v>
+        <v>1833</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>1825</v>
-      </c>
-    </row>
-    <row r="43" ht="187.2" spans="1:2">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="43" ht="188.5" spans="1:2">
       <c r="A43" t="s">
-        <v>1826</v>
+        <v>1835</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>1827</v>
-      </c>
-    </row>
-    <row r="44" ht="115.2" spans="1:2">
+        <v>1836</v>
+      </c>
+    </row>
+    <row r="44" ht="116" spans="1:2">
       <c r="A44" t="s">
-        <v>1828</v>
+        <v>1837</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>1829</v>
+        <v>1838</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>1830</v>
+        <v>1839</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>1831</v>
+        <v>1840</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>1832</v>
+        <v>1841</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>1833</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
-        <v>1834</v>
+        <v>1843</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>1835</v>
-      </c>
-    </row>
-    <row r="48" ht="259.2" spans="1:2">
+        <v>1844</v>
+      </c>
+    </row>
+    <row r="48" ht="261" spans="1:2">
       <c r="A48" t="s">
-        <v>1836</v>
+        <v>1845</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>1837</v>
+        <v>1846</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
-        <v>1838</v>
+        <v>1847</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>1839</v>
-      </c>
-    </row>
-    <row r="50" ht="331.2" spans="1:2">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="50" ht="333.5" spans="1:2">
       <c r="A50" t="s">
-        <v>1840</v>
+        <v>1849</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>1841</v>
-      </c>
-    </row>
-    <row r="51" ht="331.2" spans="1:2">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="51" ht="333.5" spans="1:2">
       <c r="A51" t="s">
-        <v>1842</v>
+        <v>1851</v>
       </c>
       <c r="B51" s="29" t="s">
-        <v>1843</v>
+        <v>1852</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Grn Test Scenarios And Core Process Fixes
Added Grn Test Scenarios And Core Process Fixes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2137" uniqueCount="1853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2151" uniqueCount="1866">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5308,6 +5308,45 @@
   </si>
   <si>
     <t>202425</t>
+  </si>
+  <si>
+    <t>BomNumberOutsideAndInside</t>
+  </si>
+  <si>
+    <t>BOM00/00168/25-26</t>
+  </si>
+  <si>
+    <t>Outside</t>
+  </si>
+  <si>
+    <t>MultipleType</t>
+  </si>
+  <si>
+    <t>Multiple</t>
+  </si>
+  <si>
+    <t>ItemType</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>BothType</t>
+  </si>
+  <si>
+    <t>Both</t>
+  </si>
+  <si>
+    <t>BOMNumberOutsideAndBoth</t>
+  </si>
+  <si>
+    <t>BOM00/00171/25-26</t>
+  </si>
+  <si>
+    <t>Machines100</t>
+  </si>
+  <si>
+    <t>MACHINES100</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -8595,11 +8634,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1034"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B1041"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -16836,43 +16875,99 @@
       </c>
     </row>
     <row r="1030" spans="1:2">
-      <c r="A1030" s="71" t="s">
+      <c r="A1030" s="34" t="s">
         <v>1751</v>
       </c>
-      <c r="B1030" s="72" t="s">
+      <c r="B1030" s="35" t="s">
         <v>1752</v>
       </c>
     </row>
     <row r="1031" spans="1:2">
-      <c r="A1031" s="71" t="s">
+      <c r="A1031" s="34" t="s">
         <v>1753</v>
       </c>
-      <c r="B1031" s="72" t="s">
+      <c r="B1031" s="35" t="s">
         <v>1754</v>
       </c>
     </row>
     <row r="1032" spans="1:2">
-      <c r="A1032" s="71" t="s">
+      <c r="A1032" s="34" t="s">
         <v>1755</v>
       </c>
-      <c r="B1032" s="72" t="s">
+      <c r="B1032" s="35" t="s">
         <v>1586</v>
       </c>
     </row>
     <row r="1033" spans="1:2">
-      <c r="A1033" s="71" t="s">
+      <c r="A1033" s="34" t="s">
         <v>1756</v>
       </c>
-      <c r="B1033" s="72" t="s">
+      <c r="B1033" s="35" t="s">
         <v>1757</v>
       </c>
     </row>
     <row r="1034" spans="1:2">
-      <c r="A1034" s="71" t="s">
+      <c r="A1034" s="34" t="s">
         <v>1758</v>
       </c>
-      <c r="B1034" s="72" t="s">
+      <c r="B1034" s="35" t="s">
         <v>1759</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:2">
+      <c r="A1035" s="71" t="s">
+        <v>1760</v>
+      </c>
+      <c r="B1035" s="72" t="s">
+        <v>1761</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:2">
+      <c r="A1036" s="71" t="s">
+        <v>1762</v>
+      </c>
+      <c r="B1036" s="72" t="s">
+        <v>1762</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:2">
+      <c r="A1037" s="71" t="s">
+        <v>1763</v>
+      </c>
+      <c r="B1037" s="72" t="s">
+        <v>1764</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:2">
+      <c r="A1038" s="71" t="s">
+        <v>1765</v>
+      </c>
+      <c r="B1038" s="72" t="s">
+        <v>1766</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:2">
+      <c r="A1039" s="71" t="s">
+        <v>1767</v>
+      </c>
+      <c r="B1039" s="72" t="s">
+        <v>1768</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:2">
+      <c r="A1040" s="71" t="s">
+        <v>1769</v>
+      </c>
+      <c r="B1040" s="72" t="s">
+        <v>1770</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:2">
+      <c r="A1041" s="71" t="s">
+        <v>1771</v>
+      </c>
+      <c r="B1041" s="72" t="s">
+        <v>1772</v>
       </c>
     </row>
   </sheetData>
@@ -16885,9 +16980,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B51"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16901,402 +16996,402 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1760</v>
+        <v>1773</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1761</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1762</v>
+        <v>1775</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1763</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1764</v>
+        <v>1777</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1765</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1766</v>
+        <v>1779</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1767</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1768</v>
+        <v>1781</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1769</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1770</v>
+        <v>1783</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1771</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1772</v>
+        <v>1785</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1773</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1774</v>
+        <v>1787</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1775</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1776</v>
+        <v>1789</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1777</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1778</v>
+        <v>1791</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1779</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1780</v>
+        <v>1793</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1781</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1782</v>
+        <v>1795</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1783</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1784</v>
+        <v>1797</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1785</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1786</v>
+        <v>1799</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1787</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1788</v>
+        <v>1801</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1789</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1790</v>
+        <v>1803</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1791</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1792</v>
+        <v>1805</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1793</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1794</v>
+        <v>1807</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1795</v>
+        <v>1808</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>1796</v>
+        <v>1809</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1797</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>1798</v>
+        <v>1811</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1799</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>1800</v>
+        <v>1813</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1801</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>1802</v>
+        <v>1815</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>1803</v>
-      </c>
-    </row>
-    <row r="24" ht="246.5" spans="1:2">
+        <v>1816</v>
+      </c>
+    </row>
+    <row r="24" ht="244.8" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>1804</v>
+        <v>1817</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1805</v>
-      </c>
-    </row>
-    <row r="25" ht="232" spans="1:2">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="25" ht="230.4" spans="1:2">
       <c r="A25" t="s">
-        <v>1806</v>
+        <v>1819</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1807</v>
-      </c>
-    </row>
-    <row r="26" ht="261" spans="1:2">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="26" ht="259.2" spans="1:2">
       <c r="A26" t="s">
-        <v>1808</v>
+        <v>1821</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1809</v>
-      </c>
-    </row>
-    <row r="27" ht="203" spans="1:2">
+        <v>1822</v>
+      </c>
+    </row>
+    <row r="27" ht="201.6" spans="1:2">
       <c r="A27" t="s">
-        <v>1810</v>
+        <v>1823</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1811</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>1812</v>
+        <v>1825</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1813</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1760</v>
+        <v>1773</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1761</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1762</v>
+        <v>1775</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1763</v>
-      </c>
-    </row>
-    <row r="31" ht="174" spans="1:2">
+        <v>1776</v>
+      </c>
+    </row>
+    <row r="31" ht="172.8" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1768</v>
+        <v>1781</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1769</v>
-      </c>
-    </row>
-    <row r="32" ht="130.5" spans="1:2">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="32" ht="129.6" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>1814</v>
+        <v>1827</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>1815</v>
-      </c>
-    </row>
-    <row r="33" ht="174" spans="1:2">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>1816</v>
+        <v>1829</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>1817</v>
-      </c>
-    </row>
-    <row r="34" ht="174" spans="1:2">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="34" ht="172.8" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>1818</v>
+        <v>1831</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>1819</v>
+        <v>1832</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>1790</v>
+        <v>1803</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>1820</v>
-      </c>
-    </row>
-    <row r="36" ht="406" spans="1:2">
+        <v>1833</v>
+      </c>
+    </row>
+    <row r="36" ht="403.2" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>1821</v>
+        <v>1834</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>1822</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>1823</v>
+        <v>1836</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>1824</v>
+        <v>1837</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>1825</v>
+        <v>1838</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1826</v>
+        <v>1839</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>1827</v>
+        <v>1840</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>1828</v>
+        <v>1841</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>1829</v>
+        <v>1842</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>1830</v>
-      </c>
-    </row>
-    <row r="41" ht="116" spans="1:2">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="41" ht="115.2" spans="1:2">
       <c r="A41" t="s">
-        <v>1831</v>
+        <v>1844</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>1832</v>
-      </c>
-    </row>
-    <row r="42" ht="174" spans="1:2">
+        <v>1845</v>
+      </c>
+    </row>
+    <row r="42" ht="172.8" spans="1:2">
       <c r="A42" t="s">
-        <v>1833</v>
+        <v>1846</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>1834</v>
-      </c>
-    </row>
-    <row r="43" ht="188.5" spans="1:2">
+        <v>1847</v>
+      </c>
+    </row>
+    <row r="43" ht="187.2" spans="1:2">
       <c r="A43" t="s">
-        <v>1835</v>
+        <v>1848</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>1836</v>
-      </c>
-    </row>
-    <row r="44" ht="116" spans="1:2">
+        <v>1849</v>
+      </c>
+    </row>
+    <row r="44" ht="115.2" spans="1:2">
       <c r="A44" t="s">
-        <v>1837</v>
+        <v>1850</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>1838</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>1839</v>
+        <v>1852</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>1840</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>1841</v>
+        <v>1854</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>1842</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
-        <v>1843</v>
+        <v>1856</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>1844</v>
-      </c>
-    </row>
-    <row r="48" ht="261" spans="1:2">
+        <v>1857</v>
+      </c>
+    </row>
+    <row r="48" ht="259.2" spans="1:2">
       <c r="A48" t="s">
-        <v>1845</v>
+        <v>1858</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>1846</v>
+        <v>1859</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
-        <v>1847</v>
+        <v>1860</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>1848</v>
-      </c>
-    </row>
-    <row r="50" ht="333.5" spans="1:2">
+        <v>1861</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
       <c r="A50" t="s">
-        <v>1849</v>
+        <v>1862</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>1850</v>
-      </c>
-    </row>
-    <row r="51" ht="333.5" spans="1:2">
+        <v>1863</v>
+      </c>
+    </row>
+    <row r="51" ht="331.2" spans="1:2">
       <c r="A51" t="s">
-        <v>1851</v>
+        <v>1864</v>
       </c>
       <c r="B51" s="29" t="s">
-        <v>1852</v>
+        <v>1865</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated E2E Fixes and Added Production Module BOM and MRP Test Scenarios
Updated E2E Fixes and Added Production Module BOM and MRP Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2151" uniqueCount="1866">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2161" uniqueCount="1876">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5347,6 +5347,36 @@
   </si>
   <si>
     <t>MACHINES100</t>
+  </si>
+  <si>
+    <t>InactiveStatus</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>FG-10002-Item</t>
+  </si>
+  <si>
+    <t>HK-TVS-FG-10002</t>
+  </si>
+  <si>
+    <t>SetupSalesScreen</t>
+  </si>
+  <si>
+    <t>Setup - Sales</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>South_Region_</t>
+  </si>
+  <si>
+    <t>SalesRegionManager</t>
+  </si>
+  <si>
+    <t>EMP26</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -8634,11 +8664,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1041"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
+  <dimension ref="A1:B1046"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -16915,59 +16945,99 @@
       </c>
     </row>
     <row r="1035" spans="1:2">
-      <c r="A1035" s="71" t="s">
+      <c r="A1035" s="34" t="s">
         <v>1760</v>
       </c>
-      <c r="B1035" s="72" t="s">
+      <c r="B1035" s="35" t="s">
         <v>1761</v>
       </c>
     </row>
     <row r="1036" spans="1:2">
-      <c r="A1036" s="71" t="s">
+      <c r="A1036" s="34" t="s">
         <v>1762</v>
       </c>
-      <c r="B1036" s="72" t="s">
+      <c r="B1036" s="35" t="s">
         <v>1762</v>
       </c>
     </row>
     <row r="1037" spans="1:2">
-      <c r="A1037" s="71" t="s">
+      <c r="A1037" s="34" t="s">
         <v>1763</v>
       </c>
-      <c r="B1037" s="72" t="s">
+      <c r="B1037" s="35" t="s">
         <v>1764</v>
       </c>
     </row>
     <row r="1038" spans="1:2">
-      <c r="A1038" s="71" t="s">
+      <c r="A1038" s="34" t="s">
         <v>1765</v>
       </c>
-      <c r="B1038" s="72" t="s">
+      <c r="B1038" s="35" t="s">
         <v>1766</v>
       </c>
     </row>
     <row r="1039" spans="1:2">
-      <c r="A1039" s="71" t="s">
+      <c r="A1039" s="34" t="s">
         <v>1767</v>
       </c>
-      <c r="B1039" s="72" t="s">
+      <c r="B1039" s="35" t="s">
         <v>1768</v>
       </c>
     </row>
     <row r="1040" spans="1:2">
-      <c r="A1040" s="71" t="s">
+      <c r="A1040" s="34" t="s">
         <v>1769</v>
       </c>
-      <c r="B1040" s="72" t="s">
+      <c r="B1040" s="35" t="s">
         <v>1770</v>
       </c>
     </row>
     <row r="1041" spans="1:2">
-      <c r="A1041" s="71" t="s">
+      <c r="A1041" s="34" t="s">
         <v>1771</v>
       </c>
-      <c r="B1041" s="72" t="s">
+      <c r="B1041" s="35" t="s">
         <v>1772</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:2">
+      <c r="A1042" s="71" t="s">
+        <v>1773</v>
+      </c>
+      <c r="B1042" s="72" t="s">
+        <v>1774</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:2">
+      <c r="A1043" s="71" t="s">
+        <v>1775</v>
+      </c>
+      <c r="B1043" s="72" t="s">
+        <v>1776</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:2">
+      <c r="A1044" s="71" t="s">
+        <v>1777</v>
+      </c>
+      <c r="B1044" s="72" t="s">
+        <v>1778</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:2">
+      <c r="A1045" s="71" t="s">
+        <v>1779</v>
+      </c>
+      <c r="B1045" s="72" t="s">
+        <v>1780</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:2">
+      <c r="A1046" s="71" t="s">
+        <v>1781</v>
+      </c>
+      <c r="B1046" s="72" t="s">
+        <v>1782</v>
       </c>
     </row>
   </sheetData>
@@ -16980,9 +17050,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B51"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
+    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16996,402 +17066,402 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1773</v>
+        <v>1783</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1774</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1775</v>
+        <v>1785</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1776</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1777</v>
+        <v>1787</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1778</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1779</v>
+        <v>1789</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1780</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1781</v>
+        <v>1791</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1782</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1783</v>
+        <v>1793</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1784</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1785</v>
+        <v>1795</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1786</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1787</v>
+        <v>1797</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1788</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1789</v>
+        <v>1799</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1790</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1791</v>
+        <v>1801</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1792</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1793</v>
+        <v>1803</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1794</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1795</v>
+        <v>1805</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1796</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1797</v>
+        <v>1807</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1798</v>
+        <v>1808</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1799</v>
+        <v>1809</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1800</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1801</v>
+        <v>1811</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1802</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1803</v>
+        <v>1813</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1804</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1805</v>
+        <v>1815</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1806</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1807</v>
+        <v>1817</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1808</v>
+        <v>1818</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>1809</v>
+        <v>1819</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1810</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>1811</v>
+        <v>1821</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1812</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>1813</v>
+        <v>1823</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1814</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>1815</v>
+        <v>1825</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="24" ht="244.8" spans="1:2">
+        <v>1826</v>
+      </c>
+    </row>
+    <row r="24" ht="246.5" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>1817</v>
+        <v>1827</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="25" ht="230.4" spans="1:2">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="25" ht="232" spans="1:2">
       <c r="A25" t="s">
-        <v>1819</v>
+        <v>1829</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1820</v>
-      </c>
-    </row>
-    <row r="26" ht="259.2" spans="1:2">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="26" ht="261" spans="1:2">
       <c r="A26" t="s">
-        <v>1821</v>
+        <v>1831</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1822</v>
-      </c>
-    </row>
-    <row r="27" ht="201.6" spans="1:2">
+        <v>1832</v>
+      </c>
+    </row>
+    <row r="27" ht="203" spans="1:2">
       <c r="A27" t="s">
-        <v>1823</v>
+        <v>1833</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1824</v>
+        <v>1834</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>1825</v>
+        <v>1835</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1826</v>
+        <v>1836</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1773</v>
+        <v>1783</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1774</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1775</v>
+        <v>1785</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1776</v>
-      </c>
-    </row>
-    <row r="31" ht="172.8" spans="1:2">
+        <v>1786</v>
+      </c>
+    </row>
+    <row r="31" ht="174" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1781</v>
+        <v>1791</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1782</v>
-      </c>
-    </row>
-    <row r="32" ht="129.6" spans="1:2">
+        <v>1792</v>
+      </c>
+    </row>
+    <row r="32" ht="130.5" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>1827</v>
+        <v>1837</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>1828</v>
-      </c>
-    </row>
-    <row r="33" ht="172.8" spans="1:2">
+        <v>1838</v>
+      </c>
+    </row>
+    <row r="33" ht="174" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>1829</v>
+        <v>1839</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>1830</v>
-      </c>
-    </row>
-    <row r="34" ht="172.8" spans="1:2">
+        <v>1840</v>
+      </c>
+    </row>
+    <row r="34" ht="174" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>1831</v>
+        <v>1841</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>1832</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>1803</v>
+        <v>1813</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>1833</v>
-      </c>
-    </row>
-    <row r="36" ht="403.2" spans="1:2">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="36" ht="406" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>1834</v>
+        <v>1844</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>1835</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>1836</v>
+        <v>1846</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>1837</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>1838</v>
+        <v>1848</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1839</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>1840</v>
+        <v>1850</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>1841</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>1842</v>
+        <v>1852</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>1843</v>
-      </c>
-    </row>
-    <row r="41" ht="115.2" spans="1:2">
+        <v>1853</v>
+      </c>
+    </row>
+    <row r="41" ht="116" spans="1:2">
       <c r="A41" t="s">
-        <v>1844</v>
+        <v>1854</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>1845</v>
-      </c>
-    </row>
-    <row r="42" ht="172.8" spans="1:2">
+        <v>1855</v>
+      </c>
+    </row>
+    <row r="42" ht="174" spans="1:2">
       <c r="A42" t="s">
-        <v>1846</v>
+        <v>1856</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>1847</v>
-      </c>
-    </row>
-    <row r="43" ht="187.2" spans="1:2">
+        <v>1857</v>
+      </c>
+    </row>
+    <row r="43" ht="188.5" spans="1:2">
       <c r="A43" t="s">
-        <v>1848</v>
+        <v>1858</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>1849</v>
-      </c>
-    </row>
-    <row r="44" ht="115.2" spans="1:2">
+        <v>1859</v>
+      </c>
+    </row>
+    <row r="44" ht="116" spans="1:2">
       <c r="A44" t="s">
-        <v>1850</v>
+        <v>1860</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>1851</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>1852</v>
+        <v>1862</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>1853</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>1854</v>
+        <v>1864</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>1855</v>
+        <v>1865</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
-        <v>1856</v>
+        <v>1866</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>1857</v>
-      </c>
-    </row>
-    <row r="48" ht="259.2" spans="1:2">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="48" ht="261" spans="1:2">
       <c r="A48" t="s">
-        <v>1858</v>
+        <v>1868</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>1859</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
-        <v>1860</v>
+        <v>1870</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>1861</v>
-      </c>
-    </row>
-    <row r="50" ht="331.2" spans="1:2">
+        <v>1871</v>
+      </c>
+    </row>
+    <row r="50" ht="333.5" spans="1:2">
       <c r="A50" t="s">
-        <v>1862</v>
+        <v>1872</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>1863</v>
-      </c>
-    </row>
-    <row r="51" ht="331.2" spans="1:2">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="51" ht="333.5" spans="1:2">
       <c r="A51" t="s">
-        <v>1864</v>
+        <v>1874</v>
       </c>
       <c r="B51" s="29" t="s">
-        <v>1865</v>
+        <v>1875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Production Order Test Scenarios Changes
Added Production Order Test Scenarios Changes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2161" uniqueCount="1876">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2163" uniqueCount="1878">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5313,7 +5313,7 @@
     <t>BomNumberOutsideAndInside</t>
   </si>
   <si>
-    <t>BOM00/00168/25-26</t>
+    <t>BOM00/00223/25-26</t>
   </si>
   <si>
     <t>Outside</t>
@@ -5377,6 +5377,12 @@
   </si>
   <si>
     <t>EMP26</t>
+  </si>
+  <si>
+    <t>BomOutsideAndInsideWithMaterial</t>
+  </si>
+  <si>
+    <t>BOM00/00226/25-26</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -8664,11 +8670,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1046"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B1047"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -17001,43 +17007,51 @@
       </c>
     </row>
     <row r="1042" spans="1:2">
-      <c r="A1042" s="71" t="s">
+      <c r="A1042" s="34" t="s">
         <v>1773</v>
       </c>
-      <c r="B1042" s="72" t="s">
+      <c r="B1042" s="35" t="s">
         <v>1774</v>
       </c>
     </row>
     <row r="1043" spans="1:2">
-      <c r="A1043" s="71" t="s">
+      <c r="A1043" s="34" t="s">
         <v>1775</v>
       </c>
-      <c r="B1043" s="72" t="s">
+      <c r="B1043" s="35" t="s">
         <v>1776</v>
       </c>
     </row>
     <row r="1044" spans="1:2">
-      <c r="A1044" s="71" t="s">
+      <c r="A1044" s="34" t="s">
         <v>1777</v>
       </c>
-      <c r="B1044" s="72" t="s">
+      <c r="B1044" s="35" t="s">
         <v>1778</v>
       </c>
     </row>
     <row r="1045" spans="1:2">
-      <c r="A1045" s="71" t="s">
+      <c r="A1045" s="34" t="s">
         <v>1779</v>
       </c>
-      <c r="B1045" s="72" t="s">
+      <c r="B1045" s="35" t="s">
         <v>1780</v>
       </c>
     </row>
     <row r="1046" spans="1:2">
-      <c r="A1046" s="71" t="s">
+      <c r="A1046" s="34" t="s">
         <v>1781</v>
       </c>
-      <c r="B1046" s="72" t="s">
+      <c r="B1046" s="35" t="s">
         <v>1782</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:2">
+      <c r="A1047" s="71" t="s">
+        <v>1783</v>
+      </c>
+      <c r="B1047" s="72" t="s">
+        <v>1784</v>
       </c>
     </row>
   </sheetData>
@@ -17050,9 +17064,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B51"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -17066,402 +17080,402 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1785</v>
+        <v>1787</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1786</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1787</v>
+        <v>1789</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1788</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1789</v>
+        <v>1791</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1790</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1791</v>
+        <v>1793</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1792</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1793</v>
+        <v>1795</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1794</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1795</v>
+        <v>1797</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1796</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1797</v>
+        <v>1799</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1798</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1799</v>
+        <v>1801</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1800</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1801</v>
+        <v>1803</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1802</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1803</v>
+        <v>1805</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1804</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1805</v>
+        <v>1807</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1806</v>
+        <v>1808</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1807</v>
+        <v>1809</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1808</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1809</v>
+        <v>1811</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1810</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1811</v>
+        <v>1813</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1812</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1813</v>
+        <v>1815</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1814</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1815</v>
+        <v>1817</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1816</v>
+        <v>1818</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1817</v>
+        <v>1819</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>1819</v>
+        <v>1821</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1820</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>1821</v>
+        <v>1823</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1822</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>1823</v>
+        <v>1825</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1824</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>1825</v>
+        <v>1827</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>1826</v>
-      </c>
-    </row>
-    <row r="24" ht="246.5" spans="1:2">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="24" ht="244.8" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>1827</v>
+        <v>1829</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1828</v>
-      </c>
-    </row>
-    <row r="25" ht="232" spans="1:2">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="25" ht="230.4" spans="1:2">
       <c r="A25" t="s">
-        <v>1829</v>
+        <v>1831</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1830</v>
-      </c>
-    </row>
-    <row r="26" ht="261" spans="1:2">
+        <v>1832</v>
+      </c>
+    </row>
+    <row r="26" ht="259.2" spans="1:2">
       <c r="A26" t="s">
-        <v>1831</v>
+        <v>1833</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1832</v>
-      </c>
-    </row>
-    <row r="27" ht="203" spans="1:2">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="27" ht="201.6" spans="1:2">
       <c r="A27" t="s">
-        <v>1833</v>
+        <v>1835</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1834</v>
+        <v>1836</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>1835</v>
+        <v>1837</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1836</v>
+        <v>1838</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1783</v>
+        <v>1785</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1784</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1785</v>
+        <v>1787</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1786</v>
-      </c>
-    </row>
-    <row r="31" ht="174" spans="1:2">
+        <v>1788</v>
+      </c>
+    </row>
+    <row r="31" ht="172.8" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1791</v>
+        <v>1793</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1792</v>
-      </c>
-    </row>
-    <row r="32" ht="130.5" spans="1:2">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="32" ht="129.6" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>1837</v>
+        <v>1839</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>1838</v>
-      </c>
-    </row>
-    <row r="33" ht="174" spans="1:2">
+        <v>1840</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>1839</v>
+        <v>1841</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>1840</v>
-      </c>
-    </row>
-    <row r="34" ht="174" spans="1:2">
+        <v>1842</v>
+      </c>
+    </row>
+    <row r="34" ht="172.8" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>1841</v>
+        <v>1843</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>1842</v>
+        <v>1844</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>1813</v>
+        <v>1815</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>1843</v>
-      </c>
-    </row>
-    <row r="36" ht="406" spans="1:2">
+        <v>1845</v>
+      </c>
+    </row>
+    <row r="36" ht="403.2" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>1844</v>
+        <v>1846</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>1845</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>1846</v>
+        <v>1848</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>1847</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>1848</v>
+        <v>1850</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1849</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>1850</v>
+        <v>1852</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>1851</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>1852</v>
+        <v>1854</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>1853</v>
-      </c>
-    </row>
-    <row r="41" ht="116" spans="1:2">
+        <v>1855</v>
+      </c>
+    </row>
+    <row r="41" ht="115.2" spans="1:2">
       <c r="A41" t="s">
-        <v>1854</v>
+        <v>1856</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>1855</v>
-      </c>
-    </row>
-    <row r="42" ht="174" spans="1:2">
+        <v>1857</v>
+      </c>
+    </row>
+    <row r="42" ht="172.8" spans="1:2">
       <c r="A42" t="s">
-        <v>1856</v>
+        <v>1858</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>1857</v>
-      </c>
-    </row>
-    <row r="43" ht="188.5" spans="1:2">
+        <v>1859</v>
+      </c>
+    </row>
+    <row r="43" ht="187.2" spans="1:2">
       <c r="A43" t="s">
-        <v>1858</v>
+        <v>1860</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>1859</v>
-      </c>
-    </row>
-    <row r="44" ht="116" spans="1:2">
+        <v>1861</v>
+      </c>
+    </row>
+    <row r="44" ht="115.2" spans="1:2">
       <c r="A44" t="s">
-        <v>1860</v>
+        <v>1862</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>1861</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>1862</v>
+        <v>1864</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>1863</v>
+        <v>1865</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>1864</v>
+        <v>1866</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>1865</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
-        <v>1866</v>
+        <v>1868</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>1867</v>
-      </c>
-    </row>
-    <row r="48" ht="261" spans="1:2">
+        <v>1869</v>
+      </c>
+    </row>
+    <row r="48" ht="259.2" spans="1:2">
       <c r="A48" t="s">
-        <v>1868</v>
+        <v>1870</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>1869</v>
+        <v>1871</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
-        <v>1870</v>
+        <v>1872</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>1871</v>
-      </c>
-    </row>
-    <row r="50" ht="333.5" spans="1:2">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
       <c r="A50" t="s">
-        <v>1872</v>
+        <v>1874</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>1873</v>
-      </c>
-    </row>
-    <row r="51" ht="333.5" spans="1:2">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="51" ht="331.2" spans="1:2">
       <c r="A51" t="s">
-        <v>1874</v>
+        <v>1876</v>
       </c>
       <c r="B51" s="29" t="s">
-        <v>1875</v>
+        <v>1877</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Production Order Test Scenarios and Updated Locators
Added Production Order Test Scenarios and Updated Locators
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2163" uniqueCount="1878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2169" uniqueCount="1884">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5383,6 +5383,24 @@
   </si>
   <si>
     <t>BOM00/00226/25-26</t>
+  </si>
+  <si>
+    <t>ProdOrderNonStandard</t>
+  </si>
+  <si>
+    <t>Production Order - Non Standard</t>
+  </si>
+  <si>
+    <t>GWL_Item(SOStandard)</t>
+  </si>
+  <si>
+    <t>GWL_SO(Standard)_Item</t>
+  </si>
+  <si>
+    <t>BomAllInside</t>
+  </si>
+  <si>
+    <t>BOM00/00327/25-26</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -8176,7 +8194,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -8334,6 +8352,7 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="66">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8410,6 +8429,13 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
+<customStorage xmlns="https://web.wps.cn/et/2018/main">
+  <book/>
+  <sheets/>
+</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8670,11 +8696,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1047"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
+  <dimension ref="A1:B1050"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -17047,11 +17073,35 @@
       </c>
     </row>
     <row r="1047" spans="1:2">
-      <c r="A1047" s="71" t="s">
+      <c r="A1047" s="34" t="s">
         <v>1783</v>
       </c>
-      <c r="B1047" s="72" t="s">
+      <c r="B1047" s="35" t="s">
         <v>1784</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:2">
+      <c r="A1048" s="71" t="s">
+        <v>1785</v>
+      </c>
+      <c r="B1048" s="72" t="s">
+        <v>1786</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:2">
+      <c r="A1049" s="71" t="s">
+        <v>1787</v>
+      </c>
+      <c r="B1049" s="73" t="s">
+        <v>1788</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:2">
+      <c r="A1050" s="71" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B1050" s="72" t="s">
+        <v>1790</v>
       </c>
     </row>
   </sheetData>
@@ -17064,9 +17114,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B51"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
+    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -17080,402 +17130,402 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1785</v>
+        <v>1791</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1786</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1787</v>
+        <v>1793</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1788</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1789</v>
+        <v>1795</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1791</v>
+        <v>1797</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1792</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1793</v>
+        <v>1799</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1794</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1795</v>
+        <v>1801</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1796</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1797</v>
+        <v>1803</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1798</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1799</v>
+        <v>1805</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1800</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1801</v>
+        <v>1807</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1802</v>
+        <v>1808</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1803</v>
+        <v>1809</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1804</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1805</v>
+        <v>1811</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1806</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1807</v>
+        <v>1813</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1808</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1809</v>
+        <v>1815</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1810</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1811</v>
+        <v>1817</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1812</v>
+        <v>1818</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1813</v>
+        <v>1819</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1814</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1815</v>
+        <v>1821</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1816</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1817</v>
+        <v>1823</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1818</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1819</v>
+        <v>1825</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1820</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>1821</v>
+        <v>1827</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1822</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>1823</v>
+        <v>1829</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1824</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>1825</v>
+        <v>1831</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1826</v>
+        <v>1832</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>1827</v>
+        <v>1833</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>1828</v>
-      </c>
-    </row>
-    <row r="24" ht="244.8" spans="1:2">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="24" ht="246.5" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>1829</v>
+        <v>1835</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1830</v>
-      </c>
-    </row>
-    <row r="25" ht="230.4" spans="1:2">
+        <v>1836</v>
+      </c>
+    </row>
+    <row r="25" ht="232" spans="1:2">
       <c r="A25" t="s">
-        <v>1831</v>
+        <v>1837</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1832</v>
-      </c>
-    </row>
-    <row r="26" ht="259.2" spans="1:2">
+        <v>1838</v>
+      </c>
+    </row>
+    <row r="26" ht="261" spans="1:2">
       <c r="A26" t="s">
-        <v>1833</v>
+        <v>1839</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1834</v>
-      </c>
-    </row>
-    <row r="27" ht="201.6" spans="1:2">
+        <v>1840</v>
+      </c>
+    </row>
+    <row r="27" ht="203" spans="1:2">
       <c r="A27" t="s">
-        <v>1835</v>
+        <v>1841</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1836</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>1837</v>
+        <v>1843</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1838</v>
+        <v>1844</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1785</v>
+        <v>1791</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1786</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1787</v>
+        <v>1793</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1788</v>
-      </c>
-    </row>
-    <row r="31" ht="172.8" spans="1:2">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="31" ht="174" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1793</v>
+        <v>1799</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1794</v>
-      </c>
-    </row>
-    <row r="32" ht="129.6" spans="1:2">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="32" ht="130.5" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>1839</v>
+        <v>1845</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>1840</v>
-      </c>
-    </row>
-    <row r="33" ht="172.8" spans="1:2">
+        <v>1846</v>
+      </c>
+    </row>
+    <row r="33" ht="174" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>1841</v>
+        <v>1847</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>1842</v>
-      </c>
-    </row>
-    <row r="34" ht="172.8" spans="1:2">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="34" ht="174" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>1843</v>
+        <v>1849</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>1844</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>1815</v>
+        <v>1821</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>1845</v>
-      </c>
-    </row>
-    <row r="36" ht="403.2" spans="1:2">
+        <v>1851</v>
+      </c>
+    </row>
+    <row r="36" ht="406" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>1846</v>
+        <v>1852</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>1847</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>1848</v>
+        <v>1854</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>1849</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>1850</v>
+        <v>1856</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1851</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>1852</v>
+        <v>1858</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>1853</v>
+        <v>1859</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>1854</v>
+        <v>1860</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>1855</v>
-      </c>
-    </row>
-    <row r="41" ht="115.2" spans="1:2">
+        <v>1861</v>
+      </c>
+    </row>
+    <row r="41" ht="116" spans="1:2">
       <c r="A41" t="s">
-        <v>1856</v>
+        <v>1862</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>1857</v>
-      </c>
-    </row>
-    <row r="42" ht="172.8" spans="1:2">
+        <v>1863</v>
+      </c>
+    </row>
+    <row r="42" ht="174" spans="1:2">
       <c r="A42" t="s">
-        <v>1858</v>
+        <v>1864</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>1859</v>
-      </c>
-    </row>
-    <row r="43" ht="187.2" spans="1:2">
+        <v>1865</v>
+      </c>
+    </row>
+    <row r="43" ht="188.5" spans="1:2">
       <c r="A43" t="s">
-        <v>1860</v>
+        <v>1866</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>1861</v>
-      </c>
-    </row>
-    <row r="44" ht="115.2" spans="1:2">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="44" ht="116" spans="1:2">
       <c r="A44" t="s">
-        <v>1862</v>
+        <v>1868</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>1863</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>1864</v>
+        <v>1870</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>1865</v>
+        <v>1871</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>1866</v>
+        <v>1872</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>1867</v>
+        <v>1873</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
-        <v>1868</v>
+        <v>1874</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>1869</v>
-      </c>
-    </row>
-    <row r="48" ht="259.2" spans="1:2">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="48" ht="261" spans="1:2">
       <c r="A48" t="s">
-        <v>1870</v>
+        <v>1876</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>1871</v>
+        <v>1877</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
-        <v>1872</v>
+        <v>1878</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>1873</v>
-      </c>
-    </row>
-    <row r="50" ht="331.2" spans="1:2">
+        <v>1879</v>
+      </c>
+    </row>
+    <row r="50" ht="333.5" spans="1:2">
       <c r="A50" t="s">
-        <v>1874</v>
+        <v>1880</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>1875</v>
-      </c>
-    </row>
-    <row r="51" ht="331.2" spans="1:2">
+        <v>1881</v>
+      </c>
+    </row>
+    <row r="51" ht="333.5" spans="1:2">
       <c r="A51" t="s">
-        <v>1876</v>
+        <v>1882</v>
       </c>
       <c r="B51" s="29" t="s">
-        <v>1877</v>
+        <v>1883</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Production Order, Po Amendement, purchase Order, Purchase Request With Material Type Test Scenarios
Added Production Order, Po Amendement, purchase Order, Purchase Request With Material Type Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2169" uniqueCount="1884">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2203" uniqueCount="1916">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5382,7 +5382,7 @@
     <t>BomOutsideAndInsideWithMaterial</t>
   </si>
   <si>
-    <t>BOM00/00226/25-26</t>
+    <t>BOM00/00292/25-26</t>
   </si>
   <si>
     <t>ProdOrderNonStandard</t>
@@ -5401,6 +5401,102 @@
   </si>
   <si>
     <t>BOM00/00327/25-26</t>
+  </si>
+  <si>
+    <t>BomOutsideAndInsideForMultiple</t>
+  </si>
+  <si>
+    <t>BOM00/00345/25-26</t>
+  </si>
+  <si>
+    <t>BomAllProcessBoth</t>
+  </si>
+  <si>
+    <t>BOM00/00299/25-26</t>
+  </si>
+  <si>
+    <t>T1001</t>
+  </si>
+  <si>
+    <t>ErpAdmin</t>
+  </si>
+  <si>
+    <t>ERPADMIN</t>
+  </si>
+  <si>
+    <t>PRMaterialType</t>
+  </si>
+  <si>
+    <t>PR - MATERIAL</t>
+  </si>
+  <si>
+    <t>IrpPrefix</t>
+  </si>
+  <si>
+    <t>PRM01</t>
+  </si>
+  <si>
+    <t>AsianLeathers</t>
+  </si>
+  <si>
+    <t>ASIAN LEATHERS</t>
+  </si>
+  <si>
+    <t>Tvsa</t>
+  </si>
+  <si>
+    <t>TVSA</t>
+  </si>
+  <si>
+    <t>ErpUserId</t>
+  </si>
+  <si>
+    <t>ERP10012</t>
+  </si>
+  <si>
+    <t>DevaValue</t>
+  </si>
+  <si>
+    <t>DEVA</t>
+  </si>
+  <si>
+    <t>Kare</t>
+  </si>
+  <si>
+    <t>KARE</t>
+  </si>
+  <si>
+    <t>(10059030)-15%</t>
+  </si>
+  <si>
+    <t>HatsunSupplier</t>
+  </si>
+  <si>
+    <t>PRODUCT SUPPLIERS AND  GOODS</t>
+  </si>
+  <si>
+    <t>BomProdWithResourcesSingle</t>
+  </si>
+  <si>
+    <t>BOM00/00344/25-26</t>
+  </si>
+  <si>
+    <t>GwlMachine1</t>
+  </si>
+  <si>
+    <t>GWL MACHINE 1</t>
+  </si>
+  <si>
+    <t>GwlMan1</t>
+  </si>
+  <si>
+    <t>GWL MAN 1</t>
+  </si>
+  <si>
+    <t>LabourCost</t>
+  </si>
+  <si>
+    <t>Labour Cost</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -8194,7 +8290,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -8347,10 +8443,6 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -8696,11 +8788,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1050"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B1067"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -17081,27 +17173,163 @@
       </c>
     </row>
     <row r="1048" spans="1:2">
-      <c r="A1048" s="71" t="s">
+      <c r="A1048" s="34" t="s">
         <v>1785</v>
       </c>
-      <c r="B1048" s="72" t="s">
+      <c r="B1048" s="35" t="s">
         <v>1786</v>
       </c>
     </row>
     <row r="1049" spans="1:2">
-      <c r="A1049" s="71" t="s">
+      <c r="A1049" s="34" t="s">
         <v>1787</v>
       </c>
-      <c r="B1049" s="73" t="s">
+      <c r="B1049" s="71" t="s">
         <v>1788</v>
       </c>
     </row>
     <row r="1050" spans="1:2">
-      <c r="A1050" s="71" t="s">
+      <c r="A1050" s="34" t="s">
         <v>1789</v>
       </c>
-      <c r="B1050" s="72" t="s">
+      <c r="B1050" s="35" t="s">
         <v>1790</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:2">
+      <c r="A1051" s="34" t="s">
+        <v>1791</v>
+      </c>
+      <c r="B1051" s="35" t="s">
+        <v>1792</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:2">
+      <c r="A1052" s="34" t="s">
+        <v>1793</v>
+      </c>
+      <c r="B1052" s="35" t="s">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:2">
+      <c r="A1053" s="34" t="s">
+        <v>1795</v>
+      </c>
+      <c r="B1053" s="35" t="s">
+        <v>1795</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:2">
+      <c r="A1054" s="34" t="s">
+        <v>1796</v>
+      </c>
+      <c r="B1054" s="35" t="s">
+        <v>1797</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:2">
+      <c r="A1055" s="34" t="s">
+        <v>1798</v>
+      </c>
+      <c r="B1055" s="35" t="s">
+        <v>1799</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:2">
+      <c r="A1056" s="34" t="s">
+        <v>1800</v>
+      </c>
+      <c r="B1056" s="35" t="s">
+        <v>1801</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:2">
+      <c r="A1057" s="34" t="s">
+        <v>1802</v>
+      </c>
+      <c r="B1057" s="35" t="s">
+        <v>1803</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:2">
+      <c r="A1058" s="34" t="s">
+        <v>1804</v>
+      </c>
+      <c r="B1058" s="35" t="s">
+        <v>1805</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:2">
+      <c r="A1059" s="34" t="s">
+        <v>1806</v>
+      </c>
+      <c r="B1059" s="35" t="s">
+        <v>1807</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:2">
+      <c r="A1060" s="34" t="s">
+        <v>1808</v>
+      </c>
+      <c r="B1060" s="35" t="s">
+        <v>1809</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:2">
+      <c r="A1061" s="34" t="s">
+        <v>1810</v>
+      </c>
+      <c r="B1061" s="35" t="s">
+        <v>1811</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:2">
+      <c r="A1062" s="34" t="s">
+        <v>1812</v>
+      </c>
+      <c r="B1062" s="35" t="s">
+        <v>1812</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:2">
+      <c r="A1063" s="34" t="s">
+        <v>1813</v>
+      </c>
+      <c r="B1063" s="35" t="s">
+        <v>1814</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:2">
+      <c r="A1064" s="34" t="s">
+        <v>1815</v>
+      </c>
+      <c r="B1064" s="35" t="s">
+        <v>1816</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:2">
+      <c r="A1065" s="34" t="s">
+        <v>1817</v>
+      </c>
+      <c r="B1065" s="35" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:2">
+      <c r="A1066" s="34" t="s">
+        <v>1819</v>
+      </c>
+      <c r="B1066" s="35" t="s">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:2">
+      <c r="A1067" s="34" t="s">
+        <v>1821</v>
+      </c>
+      <c r="B1067" s="35" t="s">
+        <v>1822</v>
       </c>
     </row>
   </sheetData>
@@ -17114,9 +17342,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B51"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -17130,402 +17358,402 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1791</v>
+        <v>1823</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1792</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1793</v>
+        <v>1825</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1794</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1795</v>
+        <v>1827</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1796</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1797</v>
+        <v>1829</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1798</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1799</v>
+        <v>1831</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1800</v>
+        <v>1832</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1801</v>
+        <v>1833</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1802</v>
+        <v>1834</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1803</v>
+        <v>1835</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1804</v>
+        <v>1836</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1805</v>
+        <v>1837</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1806</v>
+        <v>1838</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1807</v>
+        <v>1839</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1808</v>
+        <v>1840</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1809</v>
+        <v>1841</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1810</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1811</v>
+        <v>1843</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1812</v>
+        <v>1844</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1813</v>
+        <v>1845</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1814</v>
+        <v>1846</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1815</v>
+        <v>1847</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1816</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1817</v>
+        <v>1849</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1818</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1819</v>
+        <v>1851</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1820</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1821</v>
+        <v>1853</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1822</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1823</v>
+        <v>1855</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1824</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1825</v>
+        <v>1857</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1826</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>1827</v>
+        <v>1859</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1828</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>1829</v>
+        <v>1861</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1830</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>1831</v>
+        <v>1863</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1832</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>1833</v>
+        <v>1865</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>1834</v>
-      </c>
-    </row>
-    <row r="24" ht="246.5" spans="1:2">
+        <v>1866</v>
+      </c>
+    </row>
+    <row r="24" ht="244.8" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>1835</v>
+        <v>1867</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1836</v>
-      </c>
-    </row>
-    <row r="25" ht="232" spans="1:2">
+        <v>1868</v>
+      </c>
+    </row>
+    <row r="25" ht="230.4" spans="1:2">
       <c r="A25" t="s">
-        <v>1837</v>
+        <v>1869</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1838</v>
-      </c>
-    </row>
-    <row r="26" ht="261" spans="1:2">
+        <v>1870</v>
+      </c>
+    </row>
+    <row r="26" ht="259.2" spans="1:2">
       <c r="A26" t="s">
-        <v>1839</v>
+        <v>1871</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1840</v>
-      </c>
-    </row>
-    <row r="27" ht="203" spans="1:2">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="27" ht="201.6" spans="1:2">
       <c r="A27" t="s">
-        <v>1841</v>
+        <v>1873</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1842</v>
+        <v>1874</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>1843</v>
+        <v>1875</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1844</v>
+        <v>1876</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1791</v>
+        <v>1823</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1792</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1793</v>
+        <v>1825</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1794</v>
-      </c>
-    </row>
-    <row r="31" ht="174" spans="1:2">
+        <v>1826</v>
+      </c>
+    </row>
+    <row r="31" ht="172.8" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1799</v>
+        <v>1831</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="32" ht="130.5" spans="1:2">
+        <v>1832</v>
+      </c>
+    </row>
+    <row r="32" ht="129.6" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>1845</v>
+        <v>1877</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>1846</v>
-      </c>
-    </row>
-    <row r="33" ht="174" spans="1:2">
+        <v>1878</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>1847</v>
+        <v>1879</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>1848</v>
-      </c>
-    </row>
-    <row r="34" ht="174" spans="1:2">
+        <v>1880</v>
+      </c>
+    </row>
+    <row r="34" ht="172.8" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>1849</v>
+        <v>1881</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>1850</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>1821</v>
+        <v>1853</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>1851</v>
-      </c>
-    </row>
-    <row r="36" ht="406" spans="1:2">
+        <v>1883</v>
+      </c>
+    </row>
+    <row r="36" ht="403.2" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>1852</v>
+        <v>1884</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>1853</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>1854</v>
+        <v>1886</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>1855</v>
+        <v>1887</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>1856</v>
+        <v>1888</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1857</v>
+        <v>1889</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>1858</v>
+        <v>1890</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>1859</v>
+        <v>1891</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>1860</v>
+        <v>1892</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>1861</v>
-      </c>
-    </row>
-    <row r="41" ht="116" spans="1:2">
+        <v>1893</v>
+      </c>
+    </row>
+    <row r="41" ht="115.2" spans="1:2">
       <c r="A41" t="s">
-        <v>1862</v>
+        <v>1894</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>1863</v>
-      </c>
-    </row>
-    <row r="42" ht="174" spans="1:2">
+        <v>1895</v>
+      </c>
+    </row>
+    <row r="42" ht="172.8" spans="1:2">
       <c r="A42" t="s">
-        <v>1864</v>
+        <v>1896</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>1865</v>
-      </c>
-    </row>
-    <row r="43" ht="188.5" spans="1:2">
+        <v>1897</v>
+      </c>
+    </row>
+    <row r="43" ht="187.2" spans="1:2">
       <c r="A43" t="s">
-        <v>1866</v>
+        <v>1898</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>1867</v>
-      </c>
-    </row>
-    <row r="44" ht="116" spans="1:2">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="44" ht="115.2" spans="1:2">
       <c r="A44" t="s">
-        <v>1868</v>
+        <v>1900</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>1869</v>
+        <v>1901</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>1870</v>
+        <v>1902</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>1871</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>1872</v>
+        <v>1904</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>1873</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
-        <v>1874</v>
+        <v>1906</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>1875</v>
-      </c>
-    </row>
-    <row r="48" ht="261" spans="1:2">
+        <v>1907</v>
+      </c>
+    </row>
+    <row r="48" ht="259.2" spans="1:2">
       <c r="A48" t="s">
-        <v>1876</v>
+        <v>1908</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>1877</v>
+        <v>1909</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
-        <v>1878</v>
+        <v>1910</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>1879</v>
-      </c>
-    </row>
-    <row r="50" ht="333.5" spans="1:2">
+        <v>1911</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
       <c r="A50" t="s">
-        <v>1880</v>
+        <v>1912</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>1881</v>
-      </c>
-    </row>
-    <row r="51" ht="333.5" spans="1:2">
+        <v>1913</v>
+      </c>
+    </row>
+    <row r="51" ht="331.2" spans="1:2">
       <c r="A51" t="s">
-        <v>1882</v>
+        <v>1914</v>
       </c>
       <c r="B51" s="29" t="s">
-        <v>1883</v>
+        <v>1915</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated GRN, PO, Loan Request and Inspection Documents (Locators & Functions)... Added Eight Manual Production Order Test Scenarios
Updated GRN, PO, Loan Request and Inspection Documents (Locators & Functions)... Added Eight Manual Production Order Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19200" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2293" uniqueCount="1987">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2561" uniqueCount="2082">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5692,6 +5692,291 @@
   </si>
   <si>
     <t>DURAI</t>
+  </si>
+  <si>
+    <t>POS10/003935/25</t>
+  </si>
+  <si>
+    <t>ChargeItemForGrn</t>
+  </si>
+  <si>
+    <t>FRIEGHT CHARGES</t>
+  </si>
+  <si>
+    <t>ChargeGlAccount</t>
+  </si>
+  <si>
+    <t>1011134888</t>
+  </si>
+  <si>
+    <t>Percentage</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>GrnUtgstAmount</t>
+  </si>
+  <si>
+    <t>porl_utgst_amt</t>
+  </si>
+  <si>
+    <t>QcGRNNumber</t>
+  </si>
+  <si>
+    <t>GRM10/00292/25-26</t>
+  </si>
+  <si>
+    <t>GRNPONumber</t>
+  </si>
+  <si>
+    <t>POS10/00403/25-26</t>
+  </si>
+  <si>
+    <t>Avail</t>
+  </si>
+  <si>
+    <t>NotAvail</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Differed</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>LandedCostItem</t>
+  </si>
+  <si>
+    <t>TVS-CH-00011</t>
+  </si>
+  <si>
+    <t>ItemTol</t>
+  </si>
+  <si>
+    <t>PK-NA-MAC-10001</t>
+  </si>
+  <si>
+    <t>LineWiseStatus</t>
+  </si>
+  <si>
+    <t>DocumentWiseStatus</t>
+  </si>
+  <si>
+    <t>Cancel</t>
+  </si>
+  <si>
+    <t>GRNcancellReason</t>
+  </si>
+  <si>
+    <t>NOT REQUIRED</t>
+  </si>
+  <si>
+    <t>Location14</t>
+  </si>
+  <si>
+    <t>UtgstSupllier</t>
+  </si>
+  <si>
+    <t>OpenPoIgstSup</t>
+  </si>
+  <si>
+    <t>SUP20222</t>
+  </si>
+  <si>
+    <t>GrnLineAmount</t>
+  </si>
+  <si>
+    <t>GRN_LINE_AMT</t>
+  </si>
+  <si>
+    <t>GRNIgstAmount</t>
+  </si>
+  <si>
+    <t>GRNSgstAmount</t>
+  </si>
+  <si>
+    <t>GRNCgstAmount</t>
+  </si>
+  <si>
+    <t>CGST AMT</t>
+  </si>
+  <si>
+    <t>GRNUnitCost</t>
+  </si>
+  <si>
+    <t>UNIT COST</t>
+  </si>
+  <si>
+    <t>GRNDiscPct</t>
+  </si>
+  <si>
+    <t>GRN DISC PCT</t>
+  </si>
+  <si>
+    <t>Defect</t>
+  </si>
+  <si>
+    <t>CUTTING</t>
+  </si>
+  <si>
+    <t>GRNPG</t>
+  </si>
+  <si>
+    <t>GRNPM</t>
+  </si>
+  <si>
+    <t>GRNPS</t>
+  </si>
+  <si>
+    <t>GRNSourceNumber</t>
+  </si>
+  <si>
+    <t>${GRNVNO}</t>
+  </si>
+  <si>
+    <t>MRVNo</t>
+  </si>
+  <si>
+    <t>ISTLN_DOC_NO</t>
+  </si>
+  <si>
+    <t>MRVDBDocStatus</t>
+  </si>
+  <si>
+    <t>ISTLN_STATUS</t>
+  </si>
+  <si>
+    <t>MRVNumber</t>
+  </si>
+  <si>
+    <t>MRAD-2425-00086</t>
+  </si>
+  <si>
+    <t>ProdNumber</t>
+  </si>
+  <si>
+    <t>PD30-2425-00006</t>
+  </si>
+  <si>
+    <t>ReceiverWH</t>
+  </si>
+  <si>
+    <t>ReceiverWHDesc</t>
+  </si>
+  <si>
+    <t>MrvItem</t>
+  </si>
+  <si>
+    <t>TVS-RM-KDK-25</t>
+  </si>
+  <si>
+    <t>MrvItemDesc</t>
+  </si>
+  <si>
+    <t>03-07-2025</t>
+  </si>
+  <si>
+    <t>ProcessFlowStatus</t>
+  </si>
+  <si>
+    <t>QualityEnabled</t>
+  </si>
+  <si>
+    <t>AutoCreationMRV</t>
+  </si>
+  <si>
+    <t>AUTO_CREATION_MRV</t>
+  </si>
+  <si>
+    <t>AutoPostMRV</t>
+  </si>
+  <si>
+    <t>AUTO_POST_MRV</t>
+  </si>
+  <si>
+    <t>APLCTRLBU</t>
+  </si>
+  <si>
+    <t>${APLBU}</t>
+  </si>
+  <si>
+    <t>ControlBU</t>
+  </si>
+  <si>
+    <t>NotCheck</t>
+  </si>
+  <si>
+    <t>ImportSupplier</t>
+  </si>
+  <si>
+    <t>SUP00375</t>
+  </si>
+  <si>
+    <t>UnregisterSupplier</t>
+  </si>
+  <si>
+    <t>SUP00465</t>
+  </si>
+  <si>
+    <t>InterstateUnregisterSupplier</t>
+  </si>
+  <si>
+    <t>SUP10387</t>
+  </si>
+  <si>
+    <t>PoCessAmount</t>
+  </si>
+  <si>
+    <t>pol_cess_amt</t>
+  </si>
+  <si>
+    <t>PoCessPct</t>
+  </si>
+  <si>
+    <t>pol_cess_pct</t>
+  </si>
+  <si>
+    <t>GrnCessAmount</t>
+  </si>
+  <si>
+    <t>porl_cess_amt</t>
+  </si>
+  <si>
+    <t>LoanTypes</t>
+  </si>
+  <si>
+    <t>SALARY ADVANCE</t>
+  </si>
+  <si>
+    <t>LoanReference</t>
+  </si>
+  <si>
+    <t>LoanAmount</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>LoanInstallmentAmount</t>
+  </si>
+  <si>
+    <t>LoanSuretyEmployee1</t>
+  </si>
+  <si>
+    <t>DEEPAN  R</t>
+  </si>
+  <si>
+    <t>LoanSuretyEmployee2</t>
+  </si>
+  <si>
+    <t>DIPAK SWAIN</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -7952,7 +8237,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7989,6 +8274,30 @@
     <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF262626"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -8495,133 +8804,133 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -8642,7 +8951,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -8797,9 +9106,22 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="66">
@@ -9137,11 +9459,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1109"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
+  <dimension ref="A1:B1243"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -18002,22 +18324,1097 @@
       </c>
     </row>
     <row r="1108" spans="1:2">
-      <c r="A1108" s="72" t="s">
+      <c r="A1108" s="34" t="s">
         <v>1884</v>
       </c>
-      <c r="B1108" s="73" t="s">
+      <c r="B1108" s="35" t="s">
         <v>1885</v>
       </c>
     </row>
     <row r="1109" spans="1:2">
-      <c r="A1109" s="72" t="s">
+      <c r="A1109" s="34" t="s">
         <v>1886</v>
       </c>
-      <c r="B1109" s="73" t="s">
+      <c r="B1109" s="35" t="s">
         <v>1887</v>
       </c>
     </row>
+    <row r="1110" spans="1:2">
+      <c r="A1110" s="47" t="s">
+        <v>553</v>
+      </c>
+      <c r="B1110" s="72" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:2">
+      <c r="A1111" s="73" t="s">
+        <v>1574</v>
+      </c>
+      <c r="B1111" s="73" t="s">
+        <v>1888</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:2">
+      <c r="A1112" s="47" t="s">
+        <v>1889</v>
+      </c>
+      <c r="B1112" s="72" t="s">
+        <v>1890</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:2">
+      <c r="A1113" s="47" t="s">
+        <v>1891</v>
+      </c>
+      <c r="B1113" s="72" t="s">
+        <v>1892</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:2">
+      <c r="A1114" s="47" t="s">
+        <v>1893</v>
+      </c>
+      <c r="B1114" s="72" t="s">
+        <v>1894</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:2">
+      <c r="A1115" s="47" t="s">
+        <v>616</v>
+      </c>
+      <c r="B1115" s="72" t="s">
+        <v>1895</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:2">
+      <c r="A1116" s="73" t="s">
+        <v>1329</v>
+      </c>
+      <c r="B1116" s="73" t="s">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:2">
+      <c r="A1117" s="74" t="s">
+        <v>915</v>
+      </c>
+      <c r="B1117" s="72" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:2">
+      <c r="A1118" s="74" t="s">
+        <v>917</v>
+      </c>
+      <c r="B1118" s="72" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:2">
+      <c r="A1119" s="74" t="s">
+        <v>919</v>
+      </c>
+      <c r="B1119" s="72" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:2">
+      <c r="A1120" s="74" t="s">
+        <v>630</v>
+      </c>
+      <c r="B1120" s="72" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:2">
+      <c r="A1121" s="74" t="s">
+        <v>921</v>
+      </c>
+      <c r="B1121" s="72" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:2">
+      <c r="A1122" s="74" t="s">
+        <v>923</v>
+      </c>
+      <c r="B1122" s="72" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:2">
+      <c r="A1123" s="74" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B1123" s="75" t="s">
+        <v>1332</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:2">
+      <c r="A1124" s="74" t="s">
+        <v>471</v>
+      </c>
+      <c r="B1124" s="72" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:2">
+      <c r="A1125" s="74" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B1125" s="72" t="s">
+        <v>1334</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:2">
+      <c r="A1126" s="74" t="s">
+        <v>931</v>
+      </c>
+      <c r="B1126" s="72" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:2">
+      <c r="A1127" s="74" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B1127" s="75" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:2">
+      <c r="A1128" s="74" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B1128" s="75" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:2">
+      <c r="A1129" s="74" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B1129" s="75" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:2">
+      <c r="A1130" s="74" t="s">
+        <v>975</v>
+      </c>
+      <c r="B1130" s="75" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:2">
+      <c r="A1131" s="74" t="s">
+        <v>1338</v>
+      </c>
+      <c r="B1131" s="72" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:2">
+      <c r="A1132" s="74" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B1132" s="72" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:2">
+      <c r="A1133" s="74" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B1133" s="72" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:2">
+      <c r="A1134" s="74" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B1134" s="72" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:2">
+      <c r="A1135" s="74" t="s">
+        <v>1342</v>
+      </c>
+      <c r="B1135" s="76" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:2">
+      <c r="A1136" s="74" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B1136" s="72" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:2">
+      <c r="A1137" s="74" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B1137" s="72" t="s">
+        <v>1346</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:2">
+      <c r="A1138" s="74" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B1138" s="72" t="s">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:2">
+      <c r="A1139" s="74" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B1139" s="72" t="s">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:2">
+      <c r="A1140" s="74" t="s">
+        <v>1351</v>
+      </c>
+      <c r="B1140" s="72" t="s">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:2">
+      <c r="A1141" s="74" t="s">
+        <v>1353</v>
+      </c>
+      <c r="B1141" s="72" t="s">
+        <v>1354</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:2">
+      <c r="A1142" s="74" t="s">
+        <v>1355</v>
+      </c>
+      <c r="B1142" s="72" t="s">
+        <v>1356</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:2">
+      <c r="A1143" s="74" t="s">
+        <v>1357</v>
+      </c>
+      <c r="B1143" s="72" t="s">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:2">
+      <c r="A1144" s="73" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B1144" s="72" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:2">
+      <c r="A1145" s="73" t="s">
+        <v>1359</v>
+      </c>
+      <c r="B1145" s="72" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:2">
+      <c r="A1146" s="73" t="s">
+        <v>1360</v>
+      </c>
+      <c r="B1146" s="72" t="s">
+        <v>1361</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:2">
+      <c r="A1147" s="73" t="s">
+        <v>1362</v>
+      </c>
+      <c r="B1147" s="72" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:2">
+      <c r="A1148" s="73" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B1148" s="72" t="s">
+        <v>1364</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:2">
+      <c r="A1149" s="73" t="s">
+        <v>1365</v>
+      </c>
+      <c r="B1149" s="72" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:2">
+      <c r="A1150" s="73" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B1150" s="72" t="s">
+        <v>1368</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:2">
+      <c r="A1151" s="73" t="s">
+        <v>1369</v>
+      </c>
+      <c r="B1151" s="72" t="s">
+        <v>1370</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:2">
+      <c r="A1152" s="73" t="s">
+        <v>1896</v>
+      </c>
+      <c r="B1152" s="75" t="s">
+        <v>1897</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:2">
+      <c r="A1153" s="73" t="s">
+        <v>1371</v>
+      </c>
+      <c r="B1153" s="72" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:2">
+      <c r="A1154" s="73" t="s">
+        <v>1373</v>
+      </c>
+      <c r="B1154" s="72" t="s">
+        <v>1374</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:2">
+      <c r="A1155" s="73" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B1155" s="72" t="s">
+        <v>1376</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:2">
+      <c r="A1156" s="73" t="s">
+        <v>1377</v>
+      </c>
+      <c r="B1156" s="72" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:2">
+      <c r="A1157" s="73" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B1157" s="72" t="s">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:2">
+      <c r="A1158" s="73" t="s">
+        <v>1381</v>
+      </c>
+      <c r="B1158" s="72" t="s">
+        <v>1382</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:2">
+      <c r="A1159" s="73" t="s">
+        <v>1383</v>
+      </c>
+      <c r="B1159" s="72" t="s">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:2">
+      <c r="A1160" s="73" t="s">
+        <v>1385</v>
+      </c>
+      <c r="B1160" s="72" t="s">
+        <v>1386</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:2">
+      <c r="A1161" s="73" t="s">
+        <v>1387</v>
+      </c>
+      <c r="B1161" s="72" t="s">
+        <v>1388</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:2">
+      <c r="A1162" s="73" t="s">
+        <v>1389</v>
+      </c>
+      <c r="B1162" s="72" t="s">
+        <v>1390</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:2">
+      <c r="A1163" s="73" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B1163" s="72" t="s">
+        <v>1392</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:2">
+      <c r="A1164" s="73" t="s">
+        <v>1393</v>
+      </c>
+      <c r="B1164" s="72" t="s">
+        <v>1394</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:2">
+      <c r="A1165" s="73" t="s">
+        <v>1395</v>
+      </c>
+      <c r="B1165" s="72" t="s">
+        <v>1396</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:2">
+      <c r="A1166" s="73" t="s">
+        <v>1397</v>
+      </c>
+      <c r="B1166" s="72" t="s">
+        <v>1398</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:2">
+      <c r="A1167" s="73" t="s">
+        <v>1399</v>
+      </c>
+      <c r="B1167" s="72" t="s">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:2">
+      <c r="A1168" s="73" t="s">
+        <v>1898</v>
+      </c>
+      <c r="B1168" s="72" t="s">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:2">
+      <c r="A1169" s="73" t="s">
+        <v>1900</v>
+      </c>
+      <c r="B1169" s="72" t="s">
+        <v>1901</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:2">
+      <c r="A1170" s="73" t="s">
+        <v>1902</v>
+      </c>
+      <c r="B1170" s="72" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:2">
+      <c r="A1171" s="73" t="s">
+        <v>1903</v>
+      </c>
+      <c r="B1171" s="72" t="s">
+        <v>1904</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:2">
+      <c r="A1172" s="73" t="s">
+        <v>1905</v>
+      </c>
+      <c r="B1172" s="72" t="s">
+        <v>1906</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:2">
+      <c r="A1173" s="73" t="s">
+        <v>1907</v>
+      </c>
+      <c r="B1173" s="72" t="s">
+        <v>1908</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:2">
+      <c r="A1174" s="73" t="s">
+        <v>1909</v>
+      </c>
+      <c r="B1174" s="77" t="s">
+        <v>1910</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:2">
+      <c r="A1175" s="73" t="s">
+        <v>1911</v>
+      </c>
+      <c r="B1175" s="73" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:2">
+      <c r="A1176" s="73" t="s">
+        <v>1912</v>
+      </c>
+      <c r="B1176" s="73" t="s">
+        <v>1913</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:2">
+      <c r="A1177" s="73" t="s">
+        <v>1914</v>
+      </c>
+      <c r="B1177" s="72" t="s">
+        <v>1915</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:2">
+      <c r="A1178" s="73" t="s">
+        <v>1916</v>
+      </c>
+      <c r="B1178" s="78" t="s">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:2">
+      <c r="A1179" s="73" t="s">
+        <v>1917</v>
+      </c>
+      <c r="B1179" s="78" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:2">
+      <c r="A1180" s="73" t="s">
+        <v>1918</v>
+      </c>
+      <c r="B1180" s="79" t="s">
+        <v>1919</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:2">
+      <c r="A1181" s="74" t="s">
+        <v>1920</v>
+      </c>
+      <c r="B1181" s="72" t="s">
+        <v>1921</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:2">
+      <c r="A1182" s="74" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B1182" s="72" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:2">
+      <c r="A1183" s="74" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B1183" s="72" t="s">
+        <v>1346</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:2">
+      <c r="A1184" s="74" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B1184" s="72" t="s">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:2">
+      <c r="A1185" s="74" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B1185" s="72" t="s">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:2">
+      <c r="A1186" s="74" t="s">
+        <v>1351</v>
+      </c>
+      <c r="B1186" s="72" t="s">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:2">
+      <c r="A1187" s="74" t="s">
+        <v>1353</v>
+      </c>
+      <c r="B1187" s="72" t="s">
+        <v>1354</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:2">
+      <c r="A1188" s="74" t="s">
+        <v>1355</v>
+      </c>
+      <c r="B1188" s="72" t="s">
+        <v>1356</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:2">
+      <c r="A1189" s="74" t="s">
+        <v>1357</v>
+      </c>
+      <c r="B1189" s="72" t="s">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:2">
+      <c r="A1190" s="74" t="s">
+        <v>1922</v>
+      </c>
+      <c r="B1190" s="72" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:2">
+      <c r="A1191" s="74" t="s">
+        <v>1923</v>
+      </c>
+      <c r="B1191" s="72" t="s">
+        <v>1368</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:2">
+      <c r="A1192" s="74" t="s">
+        <v>1924</v>
+      </c>
+      <c r="B1192" s="72" t="s">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:2">
+      <c r="A1193" s="74" t="s">
+        <v>1926</v>
+      </c>
+      <c r="B1193" s="72" t="s">
+        <v>1927</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:2">
+      <c r="A1194" s="74" t="s">
+        <v>1928</v>
+      </c>
+      <c r="B1194" s="72" t="s">
+        <v>1929</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:2">
+      <c r="A1195" s="74" t="s">
+        <v>1930</v>
+      </c>
+      <c r="B1195" s="72" t="s">
+        <v>1931</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:2">
+      <c r="A1196" s="74" t="s">
+        <v>1932</v>
+      </c>
+      <c r="B1196" s="72" t="s">
+        <v>1932</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:2">
+      <c r="A1197" s="74" t="s">
+        <v>1933</v>
+      </c>
+      <c r="B1197" s="72" t="s">
+        <v>1933</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:2">
+      <c r="A1198" s="74" t="s">
+        <v>1934</v>
+      </c>
+      <c r="B1198" s="72" t="s">
+        <v>1934</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:2">
+      <c r="A1199" s="74" t="s">
+        <v>1441</v>
+      </c>
+      <c r="B1199" s="72" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:2">
+      <c r="A1200" s="74" t="s">
+        <v>1443</v>
+      </c>
+      <c r="B1200" s="72" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:2">
+      <c r="A1201" s="74" t="s">
+        <v>1445</v>
+      </c>
+      <c r="B1201" s="72" t="s">
+        <v>1446</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:2">
+      <c r="A1202" s="74" t="s">
+        <v>1447</v>
+      </c>
+      <c r="B1202" s="72" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:2">
+      <c r="A1203" s="74" t="s">
+        <v>1449</v>
+      </c>
+      <c r="B1203" s="72" t="s">
+        <v>1376</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:2">
+      <c r="A1204" s="74" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B1204" s="72" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:2">
+      <c r="A1205" s="74" t="s">
+        <v>1451</v>
+      </c>
+      <c r="B1205" s="72" t="s">
+        <v>1452</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:2">
+      <c r="A1206" s="73" t="s">
+        <v>1935</v>
+      </c>
+      <c r="B1206" s="72" t="s">
+        <v>1936</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:2">
+      <c r="A1207" s="74" t="s">
+        <v>1937</v>
+      </c>
+      <c r="B1207" s="72" t="s">
+        <v>1938</v>
+      </c>
+    </row>
+    <row r="1208" spans="1:2">
+      <c r="A1208" s="74" t="s">
+        <v>1939</v>
+      </c>
+      <c r="B1208" s="72" t="s">
+        <v>1940</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:2">
+      <c r="A1209" s="74" t="s">
+        <v>1519</v>
+      </c>
+      <c r="B1209" s="72" t="s">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:2">
+      <c r="A1210" s="74" t="s">
+        <v>1521</v>
+      </c>
+      <c r="B1210" s="72" t="s">
+        <v>1522</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:2">
+      <c r="A1211" s="73" t="s">
+        <v>1941</v>
+      </c>
+      <c r="B1211" s="74" t="s">
+        <v>1942</v>
+      </c>
+    </row>
+    <row r="1212" spans="1:2">
+      <c r="A1212" s="73" t="s">
+        <v>1943</v>
+      </c>
+      <c r="B1212" s="79" t="s">
+        <v>1944</v>
+      </c>
+    </row>
+    <row r="1213" spans="1:2">
+      <c r="A1213" s="73" t="s">
+        <v>1945</v>
+      </c>
+      <c r="B1213" s="80" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="1214" spans="1:2">
+      <c r="A1214" s="73" t="s">
+        <v>1946</v>
+      </c>
+      <c r="B1214" s="80" t="s">
+        <v>1414</v>
+      </c>
+    </row>
+    <row r="1215" spans="1:2">
+      <c r="A1215" s="73" t="s">
+        <v>1947</v>
+      </c>
+      <c r="B1215" s="72" t="s">
+        <v>1948</v>
+      </c>
+    </row>
+    <row r="1216" spans="1:2">
+      <c r="A1216" s="73" t="s">
+        <v>1949</v>
+      </c>
+      <c r="B1216" s="72" t="s">
+        <v>1948</v>
+      </c>
+    </row>
+    <row r="1217" spans="1:2">
+      <c r="A1217" s="73" t="s">
+        <v>283</v>
+      </c>
+      <c r="B1217" s="72" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="1218" spans="1:2">
+      <c r="A1218" s="74" t="s">
+        <v>1565</v>
+      </c>
+      <c r="B1218" s="72" t="s">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="1219" spans="1:2">
+      <c r="A1219" s="74" t="s">
+        <v>1567</v>
+      </c>
+      <c r="B1219" s="72" t="s">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="1220" spans="1:2">
+      <c r="A1220" s="74" t="s">
+        <v>1569</v>
+      </c>
+      <c r="B1220" s="72" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="1221" spans="1:2">
+      <c r="A1221" s="74" t="s">
+        <v>1570</v>
+      </c>
+      <c r="B1221" s="72" t="s">
+        <v>1570</v>
+      </c>
+    </row>
+    <row r="1222" spans="1:2">
+      <c r="A1222" s="74" t="s">
+        <v>1571</v>
+      </c>
+      <c r="B1222" s="72" t="s">
+        <v>1571</v>
+      </c>
+    </row>
+    <row r="1223" spans="1:2">
+      <c r="A1223" s="73" t="s">
+        <v>542</v>
+      </c>
+      <c r="B1223" s="72" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="1224" spans="1:2">
+      <c r="A1224" s="74" t="s">
+        <v>1951</v>
+      </c>
+      <c r="B1224" s="74" t="s">
+        <v>1859</v>
+      </c>
+    </row>
+    <row r="1225" spans="1:2">
+      <c r="A1225" s="73" t="s">
+        <v>1952</v>
+      </c>
+      <c r="B1225" s="75" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="1226" spans="1:2">
+      <c r="A1226" s="74" t="s">
+        <v>1953</v>
+      </c>
+      <c r="B1226" s="72" t="s">
+        <v>1954</v>
+      </c>
+    </row>
+    <row r="1227" spans="1:2">
+      <c r="A1227" s="73" t="s">
+        <v>1955</v>
+      </c>
+      <c r="B1227" s="72" t="s">
+        <v>1956</v>
+      </c>
+    </row>
+    <row r="1228" spans="1:2">
+      <c r="A1228" s="74" t="s">
+        <v>1957</v>
+      </c>
+      <c r="B1228" s="72" t="s">
+        <v>1958</v>
+      </c>
+    </row>
+    <row r="1229" spans="1:2">
+      <c r="A1229" s="73" t="s">
+        <v>1959</v>
+      </c>
+      <c r="B1229" s="72" t="s">
+        <v>1803</v>
+      </c>
+    </row>
+    <row r="1230" spans="1:2">
+      <c r="A1230" s="74" t="s">
+        <v>1960</v>
+      </c>
+      <c r="B1230" s="72" t="s">
+        <v>1904</v>
+      </c>
+    </row>
+    <row r="1231" spans="1:2">
+      <c r="A1231" s="73" t="s">
+        <v>1961</v>
+      </c>
+      <c r="B1231" s="72" t="s">
+        <v>1962</v>
+      </c>
+    </row>
+    <row r="1232" spans="1:2">
+      <c r="A1232" s="73" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1232" s="77" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1233" spans="1:2">
+      <c r="A1233" s="73" t="s">
+        <v>1963</v>
+      </c>
+      <c r="B1233" s="77" t="s">
+        <v>1964</v>
+      </c>
+    </row>
+    <row r="1234" spans="1:2">
+      <c r="A1234" s="73" t="s">
+        <v>1965</v>
+      </c>
+      <c r="B1234" s="77" t="s">
+        <v>1966</v>
+      </c>
+    </row>
+    <row r="1235" spans="1:2">
+      <c r="A1235" s="73" t="s">
+        <v>1967</v>
+      </c>
+      <c r="B1235" s="72" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="1236" spans="1:2">
+      <c r="A1236" s="73" t="s">
+        <v>1969</v>
+      </c>
+      <c r="B1236" s="72" t="s">
+        <v>1970</v>
+      </c>
+    </row>
+    <row r="1237" spans="1:2">
+      <c r="A1237" s="73" t="s">
+        <v>1971</v>
+      </c>
+      <c r="B1237" s="72" t="s">
+        <v>1972</v>
+      </c>
+    </row>
+    <row r="1238" spans="1:2">
+      <c r="A1238" s="74" t="s">
+        <v>1973</v>
+      </c>
+      <c r="B1238" s="72" t="s">
+        <v>1974</v>
+      </c>
+    </row>
+    <row r="1239" spans="1:2">
+      <c r="A1239" s="74" t="s">
+        <v>1975</v>
+      </c>
+      <c r="B1239" s="72" t="s">
+        <v>1974</v>
+      </c>
+    </row>
+    <row r="1240" spans="1:2">
+      <c r="A1240" s="74" t="s">
+        <v>1976</v>
+      </c>
+      <c r="B1240" s="72" t="s">
+        <v>1977</v>
+      </c>
+    </row>
+    <row r="1241" spans="1:2">
+      <c r="A1241" s="74" t="s">
+        <v>1978</v>
+      </c>
+      <c r="B1241" s="72" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="1242" spans="1:2">
+      <c r="A1242" s="74" t="s">
+        <v>1979</v>
+      </c>
+      <c r="B1242" s="72" t="s">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="1243" spans="1:2">
+      <c r="A1243" s="74" t="s">
+        <v>1981</v>
+      </c>
+      <c r="B1243" s="72" t="s">
+        <v>1982</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1211" r:id="rId1" display="MRAD-2425-00086"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
@@ -18027,9 +19424,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B54"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
+    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -18043,426 +19440,426 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1888</v>
+        <v>1983</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1889</v>
+        <v>1984</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1890</v>
+        <v>1985</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1891</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1892</v>
+        <v>1987</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1893</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1894</v>
+        <v>1989</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1895</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1896</v>
+        <v>1991</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1897</v>
+        <v>1992</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1898</v>
+        <v>1993</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1899</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1900</v>
+        <v>1995</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1901</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1902</v>
+        <v>1997</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1903</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1904</v>
+        <v>1999</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1905</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>1906</v>
+        <v>2001</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1907</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>1908</v>
+        <v>2003</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1909</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>1910</v>
+        <v>2005</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1911</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>1912</v>
+        <v>2007</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1913</v>
+        <v>2008</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>1914</v>
+        <v>2009</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1915</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>1916</v>
+        <v>2011</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1917</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>1918</v>
+        <v>2013</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1919</v>
+        <v>2014</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>1920</v>
+        <v>2015</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1921</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>1922</v>
+        <v>2017</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1923</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>1924</v>
+        <v>2019</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>1925</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>1926</v>
+        <v>2021</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1927</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>1928</v>
+        <v>2023</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>1929</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>1930</v>
+        <v>2025</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>1931</v>
-      </c>
-    </row>
-    <row r="24" ht="244.8" spans="1:2">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="24" ht="246.5" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>1932</v>
+        <v>2027</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1933</v>
-      </c>
-    </row>
-    <row r="25" ht="230.4" spans="1:2">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="25" ht="232" spans="1:2">
       <c r="A25" t="s">
-        <v>1934</v>
+        <v>2029</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1935</v>
-      </c>
-    </row>
-    <row r="26" ht="259.2" spans="1:2">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="26" ht="261" spans="1:2">
       <c r="A26" t="s">
-        <v>1936</v>
+        <v>2031</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1937</v>
-      </c>
-    </row>
-    <row r="27" ht="201.6" spans="1:2">
+        <v>2032</v>
+      </c>
+    </row>
+    <row r="27" ht="203" spans="1:2">
       <c r="A27" t="s">
-        <v>1938</v>
+        <v>2033</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1939</v>
+        <v>2034</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>1940</v>
+        <v>2035</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1941</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1888</v>
+        <v>1983</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1889</v>
+        <v>1984</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1890</v>
+        <v>1985</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1891</v>
-      </c>
-    </row>
-    <row r="31" ht="172.8" spans="1:2">
+        <v>1986</v>
+      </c>
+    </row>
+    <row r="31" ht="174" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1896</v>
+        <v>1991</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1897</v>
-      </c>
-    </row>
-    <row r="32" ht="129.6" spans="1:2">
+        <v>1992</v>
+      </c>
+    </row>
+    <row r="32" ht="130.5" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>1942</v>
+        <v>2037</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>1943</v>
-      </c>
-    </row>
-    <row r="33" ht="172.8" spans="1:2">
+        <v>2038</v>
+      </c>
+    </row>
+    <row r="33" ht="174" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>1944</v>
+        <v>2039</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>1945</v>
-      </c>
-    </row>
-    <row r="34" ht="172.8" spans="1:2">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="34" ht="174" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>1946</v>
+        <v>2041</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>1947</v>
+        <v>2042</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>1918</v>
+        <v>2013</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>1948</v>
-      </c>
-    </row>
-    <row r="36" ht="403.2" spans="1:2">
+        <v>2043</v>
+      </c>
+    </row>
+    <row r="36" ht="406" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>1949</v>
+        <v>2044</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>1950</v>
+        <v>2045</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>1951</v>
+        <v>2046</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>1952</v>
+        <v>2047</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>1953</v>
+        <v>2048</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>1954</v>
+        <v>2049</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>1955</v>
+        <v>2050</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>1956</v>
+        <v>2051</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>1957</v>
+        <v>2052</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>1958</v>
-      </c>
-    </row>
-    <row r="41" ht="115.2" spans="1:2">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="41" ht="116" spans="1:2">
       <c r="A41" t="s">
-        <v>1959</v>
+        <v>2054</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>1960</v>
-      </c>
-    </row>
-    <row r="42" ht="172.8" spans="1:2">
+        <v>2055</v>
+      </c>
+    </row>
+    <row r="42" ht="174" spans="1:2">
       <c r="A42" t="s">
-        <v>1961</v>
+        <v>2056</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>1962</v>
-      </c>
-    </row>
-    <row r="43" ht="187.2" spans="1:2">
+        <v>2057</v>
+      </c>
+    </row>
+    <row r="43" ht="188.5" spans="1:2">
       <c r="A43" t="s">
-        <v>1963</v>
+        <v>2058</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>1964</v>
-      </c>
-    </row>
-    <row r="44" ht="115.2" spans="1:2">
+        <v>2059</v>
+      </c>
+    </row>
+    <row r="44" ht="116" spans="1:2">
       <c r="A44" t="s">
-        <v>1965</v>
+        <v>2060</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>1966</v>
+        <v>2061</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>1967</v>
+        <v>2062</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>1968</v>
+        <v>2063</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>1969</v>
+        <v>2064</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>1970</v>
+        <v>2065</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
-        <v>1971</v>
+        <v>2066</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>1972</v>
-      </c>
-    </row>
-    <row r="48" ht="259.2" spans="1:2">
+        <v>2067</v>
+      </c>
+    </row>
+    <row r="48" ht="261" spans="1:2">
       <c r="A48" t="s">
-        <v>1973</v>
+        <v>2068</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>1974</v>
+        <v>2069</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
-        <v>1975</v>
+        <v>2070</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>1976</v>
-      </c>
-    </row>
-    <row r="50" ht="331.2" spans="1:2">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="50" ht="333.5" spans="1:2">
       <c r="A50" t="s">
-        <v>1977</v>
+        <v>2072</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>1978</v>
-      </c>
-    </row>
-    <row r="51" ht="331.2" spans="1:2">
+        <v>2073</v>
+      </c>
+    </row>
+    <row r="51" ht="333.5" spans="1:2">
       <c r="A51" t="s">
-        <v>1979</v>
+        <v>2074</v>
       </c>
       <c r="B51" s="29" t="s">
-        <v>1980</v>
+        <v>2075</v>
       </c>
     </row>
     <row r="52" ht="36" customHeight="1" spans="1:2">
       <c r="A52" t="s">
-        <v>1981</v>
+        <v>2076</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>1982</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="53" ht="23.25" customHeight="1" spans="1:2">
       <c r="A53" t="s">
-        <v>1983</v>
+        <v>2078</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>1984</v>
+        <v>2079</v>
       </c>
     </row>
     <row r="54" ht="27.75" customHeight="1" spans="1:2">
       <c r="A54" t="s">
-        <v>1985</v>
+        <v>2080</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>1986</v>
+        <v>2081</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Core Process Fixes And Added Purchase Order And Po Amendment Test Scenarios
Added Core Process Fixes And Added Purchase Order And Po Amendment Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2561" uniqueCount="2082">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2575" uniqueCount="2091">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5977,6 +5977,33 @@
   </si>
   <si>
     <t>DIPAK SWAIN</t>
+  </si>
+  <si>
+    <t>Pol_Cess_pct</t>
+  </si>
+  <si>
+    <t>POL_CESS_PCT</t>
+  </si>
+  <si>
+    <t>Pol_Cess_Amt</t>
+  </si>
+  <si>
+    <t>POL_CESS_AMT</t>
+  </si>
+  <si>
+    <t>TrdSupplier</t>
+  </si>
+  <si>
+    <t>Equip1000</t>
+  </si>
+  <si>
+    <t>EQUIP-1000</t>
+  </si>
+  <si>
+    <t>AgrCeramics</t>
+  </si>
+  <si>
+    <t>TAX-FJD</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -8237,7 +8264,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8268,24 +8295,6 @@
     </font>
     <font>
       <sz val="14"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -8804,133 +8813,133 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -8951,7 +8960,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9106,21 +9115,8 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9459,11 +9455,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B1243"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B1250"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -18343,15 +18339,15 @@
       <c r="A1110" s="47" t="s">
         <v>553</v>
       </c>
-      <c r="B1110" s="72" t="s">
+      <c r="B1110" s="35" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="1111" spans="1:2">
-      <c r="A1111" s="73" t="s">
+      <c r="A1111" s="34" t="s">
         <v>1574</v>
       </c>
-      <c r="B1111" s="73" t="s">
+      <c r="B1111" s="34" t="s">
         <v>1888</v>
       </c>
     </row>
@@ -18359,7 +18355,7 @@
       <c r="A1112" s="47" t="s">
         <v>1889</v>
       </c>
-      <c r="B1112" s="72" t="s">
+      <c r="B1112" s="35" t="s">
         <v>1890</v>
       </c>
     </row>
@@ -18367,7 +18363,7 @@
       <c r="A1113" s="47" t="s">
         <v>1891</v>
       </c>
-      <c r="B1113" s="72" t="s">
+      <c r="B1113" s="35" t="s">
         <v>1892</v>
       </c>
     </row>
@@ -18375,7 +18371,7 @@
       <c r="A1114" s="47" t="s">
         <v>1893</v>
       </c>
-      <c r="B1114" s="72" t="s">
+      <c r="B1114" s="35" t="s">
         <v>1894</v>
       </c>
     </row>
@@ -18383,1032 +18379,1088 @@
       <c r="A1115" s="47" t="s">
         <v>616</v>
       </c>
-      <c r="B1115" s="72" t="s">
+      <c r="B1115" s="35" t="s">
         <v>1895</v>
       </c>
     </row>
     <row r="1116" spans="1:2">
-      <c r="A1116" s="73" t="s">
+      <c r="A1116" s="34" t="s">
         <v>1329</v>
       </c>
-      <c r="B1116" s="73" t="s">
+      <c r="B1116" s="34" t="s">
         <v>1330</v>
       </c>
     </row>
     <row r="1117" spans="1:2">
-      <c r="A1117" s="74" t="s">
+      <c r="A1117" s="34" t="s">
         <v>915</v>
       </c>
-      <c r="B1117" s="72" t="s">
+      <c r="B1117" s="35" t="s">
         <v>916</v>
       </c>
     </row>
     <row r="1118" spans="1:2">
-      <c r="A1118" s="74" t="s">
+      <c r="A1118" s="34" t="s">
         <v>917</v>
       </c>
-      <c r="B1118" s="72" t="s">
+      <c r="B1118" s="35" t="s">
         <v>918</v>
       </c>
     </row>
     <row r="1119" spans="1:2">
-      <c r="A1119" s="74" t="s">
+      <c r="A1119" s="34" t="s">
         <v>919</v>
       </c>
-      <c r="B1119" s="72" t="s">
+      <c r="B1119" s="35" t="s">
         <v>920</v>
       </c>
     </row>
     <row r="1120" spans="1:2">
-      <c r="A1120" s="74" t="s">
+      <c r="A1120" s="34" t="s">
         <v>630</v>
       </c>
-      <c r="B1120" s="72" t="s">
+      <c r="B1120" s="35" t="s">
         <v>631</v>
       </c>
     </row>
     <row r="1121" spans="1:2">
-      <c r="A1121" s="74" t="s">
+      <c r="A1121" s="34" t="s">
         <v>921</v>
       </c>
-      <c r="B1121" s="72" t="s">
+      <c r="B1121" s="35" t="s">
         <v>922</v>
       </c>
     </row>
     <row r="1122" spans="1:2">
-      <c r="A1122" s="74" t="s">
+      <c r="A1122" s="34" t="s">
         <v>923</v>
       </c>
-      <c r="B1122" s="72" t="s">
+      <c r="B1122" s="35" t="s">
         <v>924</v>
       </c>
     </row>
     <row r="1123" spans="1:2">
-      <c r="A1123" s="74" t="s">
+      <c r="A1123" s="34" t="s">
         <v>1331</v>
       </c>
-      <c r="B1123" s="75" t="s">
+      <c r="B1123" s="35" t="s">
         <v>1332</v>
       </c>
     </row>
     <row r="1124" spans="1:2">
-      <c r="A1124" s="74" t="s">
+      <c r="A1124" s="34" t="s">
         <v>471</v>
       </c>
-      <c r="B1124" s="72" t="s">
+      <c r="B1124" s="35" t="s">
         <v>472</v>
       </c>
     </row>
     <row r="1125" spans="1:2">
-      <c r="A1125" s="74" t="s">
+      <c r="A1125" s="34" t="s">
         <v>1333</v>
       </c>
-      <c r="B1125" s="72" t="s">
+      <c r="B1125" s="35" t="s">
         <v>1334</v>
       </c>
     </row>
     <row r="1126" spans="1:2">
-      <c r="A1126" s="74" t="s">
+      <c r="A1126" s="34" t="s">
         <v>931</v>
       </c>
-      <c r="B1126" s="72" t="s">
+      <c r="B1126" s="35" t="s">
         <v>932</v>
       </c>
     </row>
     <row r="1127" spans="1:2">
-      <c r="A1127" s="74" t="s">
+      <c r="A1127" s="34" t="s">
         <v>1335</v>
       </c>
-      <c r="B1127" s="75" t="s">
+      <c r="B1127" s="35" t="s">
         <v>978</v>
       </c>
     </row>
     <row r="1128" spans="1:2">
-      <c r="A1128" s="74" t="s">
+      <c r="A1128" s="34" t="s">
         <v>1336</v>
       </c>
-      <c r="B1128" s="75" t="s">
+      <c r="B1128" s="35" t="s">
         <v>979</v>
       </c>
     </row>
     <row r="1129" spans="1:2">
-      <c r="A1129" s="74" t="s">
+      <c r="A1129" s="34" t="s">
         <v>1337</v>
       </c>
-      <c r="B1129" s="75" t="s">
+      <c r="B1129" s="35" t="s">
         <v>980</v>
       </c>
     </row>
     <row r="1130" spans="1:2">
-      <c r="A1130" s="74" t="s">
+      <c r="A1130" s="34" t="s">
         <v>975</v>
       </c>
-      <c r="B1130" s="75" t="s">
+      <c r="B1130" s="35" t="s">
         <v>976</v>
       </c>
     </row>
     <row r="1131" spans="1:2">
-      <c r="A1131" s="74" t="s">
+      <c r="A1131" s="34" t="s">
         <v>1338</v>
       </c>
-      <c r="B1131" s="72" t="s">
+      <c r="B1131" s="35" t="s">
         <v>981</v>
       </c>
     </row>
     <row r="1132" spans="1:2">
-      <c r="A1132" s="74" t="s">
+      <c r="A1132" s="34" t="s">
         <v>1339</v>
       </c>
-      <c r="B1132" s="72" t="s">
+      <c r="B1132" s="35" t="s">
         <v>982</v>
       </c>
     </row>
     <row r="1133" spans="1:2">
-      <c r="A1133" s="74" t="s">
+      <c r="A1133" s="34" t="s">
         <v>1340</v>
       </c>
-      <c r="B1133" s="72" t="s">
+      <c r="B1133" s="35" t="s">
         <v>983</v>
       </c>
     </row>
     <row r="1134" spans="1:2">
-      <c r="A1134" s="74" t="s">
+      <c r="A1134" s="34" t="s">
         <v>1341</v>
       </c>
-      <c r="B1134" s="72" t="s">
+      <c r="B1134" s="35" t="s">
         <v>988</v>
       </c>
     </row>
     <row r="1135" spans="1:2">
-      <c r="A1135" s="74" t="s">
+      <c r="A1135" s="34" t="s">
         <v>1342</v>
       </c>
-      <c r="B1135" s="76" t="s">
+      <c r="B1135" s="58" t="s">
         <v>987</v>
       </c>
     </row>
     <row r="1136" spans="1:2">
-      <c r="A1136" s="74" t="s">
+      <c r="A1136" s="34" t="s">
         <v>1343</v>
       </c>
-      <c r="B1136" s="72" t="s">
+      <c r="B1136" s="35" t="s">
         <v>1344</v>
       </c>
     </row>
     <row r="1137" spans="1:2">
-      <c r="A1137" s="74" t="s">
+      <c r="A1137" s="34" t="s">
         <v>1345</v>
       </c>
-      <c r="B1137" s="72" t="s">
+      <c r="B1137" s="35" t="s">
         <v>1346</v>
       </c>
     </row>
     <row r="1138" spans="1:2">
-      <c r="A1138" s="74" t="s">
+      <c r="A1138" s="34" t="s">
         <v>1347</v>
       </c>
-      <c r="B1138" s="72" t="s">
+      <c r="B1138" s="35" t="s">
         <v>1348</v>
       </c>
     </row>
     <row r="1139" spans="1:2">
-      <c r="A1139" s="74" t="s">
+      <c r="A1139" s="34" t="s">
         <v>1349</v>
       </c>
-      <c r="B1139" s="72" t="s">
+      <c r="B1139" s="35" t="s">
         <v>1350</v>
       </c>
     </row>
     <row r="1140" spans="1:2">
-      <c r="A1140" s="74" t="s">
+      <c r="A1140" s="34" t="s">
         <v>1351</v>
       </c>
-      <c r="B1140" s="72" t="s">
+      <c r="B1140" s="35" t="s">
         <v>1352</v>
       </c>
     </row>
     <row r="1141" spans="1:2">
-      <c r="A1141" s="74" t="s">
+      <c r="A1141" s="34" t="s">
         <v>1353</v>
       </c>
-      <c r="B1141" s="72" t="s">
+      <c r="B1141" s="35" t="s">
         <v>1354</v>
       </c>
     </row>
     <row r="1142" spans="1:2">
-      <c r="A1142" s="74" t="s">
+      <c r="A1142" s="34" t="s">
         <v>1355</v>
       </c>
-      <c r="B1142" s="72" t="s">
+      <c r="B1142" s="35" t="s">
         <v>1356</v>
       </c>
     </row>
     <row r="1143" spans="1:2">
-      <c r="A1143" s="74" t="s">
+      <c r="A1143" s="34" t="s">
         <v>1357</v>
       </c>
-      <c r="B1143" s="72" t="s">
+      <c r="B1143" s="35" t="s">
         <v>1358</v>
       </c>
     </row>
     <row r="1144" spans="1:2">
-      <c r="A1144" s="73" t="s">
+      <c r="A1144" s="34" t="s">
         <v>1341</v>
       </c>
-      <c r="B1144" s="72" t="s">
+      <c r="B1144" s="35" t="s">
         <v>988</v>
       </c>
     </row>
     <row r="1145" spans="1:2">
-      <c r="A1145" s="73" t="s">
+      <c r="A1145" s="34" t="s">
         <v>1359</v>
       </c>
-      <c r="B1145" s="72" t="s">
+      <c r="B1145" s="35" t="s">
         <v>985</v>
       </c>
     </row>
     <row r="1146" spans="1:2">
-      <c r="A1146" s="73" t="s">
+      <c r="A1146" s="34" t="s">
         <v>1360</v>
       </c>
-      <c r="B1146" s="72" t="s">
+      <c r="B1146" s="35" t="s">
         <v>1361</v>
       </c>
     </row>
     <row r="1147" spans="1:2">
-      <c r="A1147" s="73" t="s">
+      <c r="A1147" s="34" t="s">
         <v>1362</v>
       </c>
-      <c r="B1147" s="72" t="s">
+      <c r="B1147" s="35" t="s">
         <v>986</v>
       </c>
     </row>
     <row r="1148" spans="1:2">
-      <c r="A1148" s="73" t="s">
+      <c r="A1148" s="34" t="s">
         <v>1363</v>
       </c>
-      <c r="B1148" s="72" t="s">
+      <c r="B1148" s="35" t="s">
         <v>1364</v>
       </c>
     </row>
     <row r="1149" spans="1:2">
-      <c r="A1149" s="73" t="s">
+      <c r="A1149" s="34" t="s">
         <v>1365</v>
       </c>
-      <c r="B1149" s="72" t="s">
+      <c r="B1149" s="35" t="s">
         <v>1366</v>
       </c>
     </row>
     <row r="1150" spans="1:2">
-      <c r="A1150" s="73" t="s">
+      <c r="A1150" s="34" t="s">
         <v>1367</v>
       </c>
-      <c r="B1150" s="72" t="s">
+      <c r="B1150" s="35" t="s">
         <v>1368</v>
       </c>
     </row>
     <row r="1151" spans="1:2">
-      <c r="A1151" s="73" t="s">
+      <c r="A1151" s="34" t="s">
         <v>1369</v>
       </c>
-      <c r="B1151" s="72" t="s">
+      <c r="B1151" s="35" t="s">
         <v>1370</v>
       </c>
     </row>
     <row r="1152" spans="1:2">
-      <c r="A1152" s="73" t="s">
+      <c r="A1152" s="34" t="s">
         <v>1896</v>
       </c>
-      <c r="B1152" s="75" t="s">
+      <c r="B1152" s="35" t="s">
         <v>1897</v>
       </c>
     </row>
     <row r="1153" spans="1:2">
-      <c r="A1153" s="73" t="s">
+      <c r="A1153" s="34" t="s">
         <v>1371</v>
       </c>
-      <c r="B1153" s="72" t="s">
+      <c r="B1153" s="35" t="s">
         <v>1372</v>
       </c>
     </row>
     <row r="1154" spans="1:2">
-      <c r="A1154" s="73" t="s">
+      <c r="A1154" s="34" t="s">
         <v>1373</v>
       </c>
-      <c r="B1154" s="72" t="s">
+      <c r="B1154" s="35" t="s">
         <v>1374</v>
       </c>
     </row>
     <row r="1155" spans="1:2">
-      <c r="A1155" s="73" t="s">
+      <c r="A1155" s="34" t="s">
         <v>1375</v>
       </c>
-      <c r="B1155" s="72" t="s">
+      <c r="B1155" s="35" t="s">
         <v>1376</v>
       </c>
     </row>
     <row r="1156" spans="1:2">
-      <c r="A1156" s="73" t="s">
+      <c r="A1156" s="34" t="s">
         <v>1377</v>
       </c>
-      <c r="B1156" s="72" t="s">
+      <c r="B1156" s="35" t="s">
         <v>1378</v>
       </c>
     </row>
     <row r="1157" spans="1:2">
-      <c r="A1157" s="73" t="s">
+      <c r="A1157" s="34" t="s">
         <v>1379</v>
       </c>
-      <c r="B1157" s="72" t="s">
+      <c r="B1157" s="35" t="s">
         <v>1380</v>
       </c>
     </row>
     <row r="1158" spans="1:2">
-      <c r="A1158" s="73" t="s">
+      <c r="A1158" s="34" t="s">
         <v>1381</v>
       </c>
-      <c r="B1158" s="72" t="s">
+      <c r="B1158" s="35" t="s">
         <v>1382</v>
       </c>
     </row>
     <row r="1159" spans="1:2">
-      <c r="A1159" s="73" t="s">
+      <c r="A1159" s="34" t="s">
         <v>1383</v>
       </c>
-      <c r="B1159" s="72" t="s">
+      <c r="B1159" s="35" t="s">
         <v>1384</v>
       </c>
     </row>
     <row r="1160" spans="1:2">
-      <c r="A1160" s="73" t="s">
+      <c r="A1160" s="34" t="s">
         <v>1385</v>
       </c>
-      <c r="B1160" s="72" t="s">
+      <c r="B1160" s="35" t="s">
         <v>1386</v>
       </c>
     </row>
     <row r="1161" spans="1:2">
-      <c r="A1161" s="73" t="s">
+      <c r="A1161" s="34" t="s">
         <v>1387</v>
       </c>
-      <c r="B1161" s="72" t="s">
+      <c r="B1161" s="35" t="s">
         <v>1388</v>
       </c>
     </row>
     <row r="1162" spans="1:2">
-      <c r="A1162" s="73" t="s">
+      <c r="A1162" s="34" t="s">
         <v>1389</v>
       </c>
-      <c r="B1162" s="72" t="s">
+      <c r="B1162" s="35" t="s">
         <v>1390</v>
       </c>
     </row>
     <row r="1163" spans="1:2">
-      <c r="A1163" s="73" t="s">
+      <c r="A1163" s="34" t="s">
         <v>1391</v>
       </c>
-      <c r="B1163" s="72" t="s">
+      <c r="B1163" s="35" t="s">
         <v>1392</v>
       </c>
     </row>
     <row r="1164" spans="1:2">
-      <c r="A1164" s="73" t="s">
+      <c r="A1164" s="34" t="s">
         <v>1393</v>
       </c>
-      <c r="B1164" s="72" t="s">
+      <c r="B1164" s="35" t="s">
         <v>1394</v>
       </c>
     </row>
     <row r="1165" spans="1:2">
-      <c r="A1165" s="73" t="s">
+      <c r="A1165" s="34" t="s">
         <v>1395</v>
       </c>
-      <c r="B1165" s="72" t="s">
+      <c r="B1165" s="35" t="s">
         <v>1396</v>
       </c>
     </row>
     <row r="1166" spans="1:2">
-      <c r="A1166" s="73" t="s">
+      <c r="A1166" s="34" t="s">
         <v>1397</v>
       </c>
-      <c r="B1166" s="72" t="s">
+      <c r="B1166" s="35" t="s">
         <v>1398</v>
       </c>
     </row>
     <row r="1167" spans="1:2">
-      <c r="A1167" s="73" t="s">
+      <c r="A1167" s="34" t="s">
         <v>1399</v>
       </c>
-      <c r="B1167" s="72" t="s">
+      <c r="B1167" s="35" t="s">
         <v>1400</v>
       </c>
     </row>
     <row r="1168" spans="1:2">
-      <c r="A1168" s="73" t="s">
+      <c r="A1168" s="34" t="s">
         <v>1898</v>
       </c>
-      <c r="B1168" s="72" t="s">
+      <c r="B1168" s="35" t="s">
         <v>1899</v>
       </c>
     </row>
     <row r="1169" spans="1:2">
-      <c r="A1169" s="73" t="s">
+      <c r="A1169" s="34" t="s">
         <v>1900</v>
       </c>
-      <c r="B1169" s="72" t="s">
+      <c r="B1169" s="35" t="s">
         <v>1901</v>
       </c>
     </row>
     <row r="1170" spans="1:2">
-      <c r="A1170" s="73" t="s">
+      <c r="A1170" s="34" t="s">
         <v>1902</v>
       </c>
-      <c r="B1170" s="72" t="s">
+      <c r="B1170" s="35" t="s">
         <v>561</v>
       </c>
     </row>
     <row r="1171" spans="1:2">
-      <c r="A1171" s="73" t="s">
+      <c r="A1171" s="34" t="s">
         <v>1903</v>
       </c>
-      <c r="B1171" s="72" t="s">
+      <c r="B1171" s="35" t="s">
         <v>1904</v>
       </c>
     </row>
     <row r="1172" spans="1:2">
-      <c r="A1172" s="73" t="s">
+      <c r="A1172" s="34" t="s">
         <v>1905</v>
       </c>
-      <c r="B1172" s="72" t="s">
+      <c r="B1172" s="35" t="s">
         <v>1906</v>
       </c>
     </row>
     <row r="1173" spans="1:2">
-      <c r="A1173" s="73" t="s">
+      <c r="A1173" s="34" t="s">
         <v>1907</v>
       </c>
-      <c r="B1173" s="72" t="s">
+      <c r="B1173" s="35" t="s">
         <v>1908</v>
       </c>
     </row>
     <row r="1174" spans="1:2">
-      <c r="A1174" s="73" t="s">
+      <c r="A1174" s="34" t="s">
         <v>1909</v>
       </c>
-      <c r="B1174" s="77" t="s">
+      <c r="B1174" s="71" t="s">
         <v>1910</v>
       </c>
     </row>
     <row r="1175" spans="1:2">
-      <c r="A1175" s="73" t="s">
+      <c r="A1175" s="34" t="s">
         <v>1911</v>
       </c>
-      <c r="B1175" s="73" t="s">
+      <c r="B1175" s="34" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="1176" spans="1:2">
-      <c r="A1176" s="73" t="s">
+      <c r="A1176" s="34" t="s">
         <v>1912</v>
       </c>
-      <c r="B1176" s="73" t="s">
+      <c r="B1176" s="34" t="s">
         <v>1913</v>
       </c>
     </row>
     <row r="1177" spans="1:2">
-      <c r="A1177" s="73" t="s">
+      <c r="A1177" s="34" t="s">
         <v>1914</v>
       </c>
-      <c r="B1177" s="72" t="s">
+      <c r="B1177" s="35" t="s">
         <v>1915</v>
       </c>
     </row>
     <row r="1178" spans="1:2">
-      <c r="A1178" s="73" t="s">
+      <c r="A1178" s="34" t="s">
         <v>1916</v>
       </c>
-      <c r="B1178" s="78" t="s">
+      <c r="B1178" s="71" t="s">
         <v>1496</v>
       </c>
     </row>
     <row r="1179" spans="1:2">
-      <c r="A1179" s="73" t="s">
+      <c r="A1179" s="34" t="s">
         <v>1917</v>
       </c>
-      <c r="B1179" s="78" t="s">
+      <c r="B1179" s="71" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="1180" spans="1:2">
-      <c r="A1180" s="73" t="s">
+      <c r="A1180" s="34" t="s">
         <v>1918</v>
       </c>
-      <c r="B1180" s="79" t="s">
+      <c r="B1180" s="72" t="s">
         <v>1919</v>
       </c>
     </row>
     <row r="1181" spans="1:2">
-      <c r="A1181" s="74" t="s">
+      <c r="A1181" s="34" t="s">
         <v>1920</v>
       </c>
-      <c r="B1181" s="72" t="s">
+      <c r="B1181" s="35" t="s">
         <v>1921</v>
       </c>
     </row>
     <row r="1182" spans="1:2">
-      <c r="A1182" s="74" t="s">
+      <c r="A1182" s="34" t="s">
         <v>1343</v>
       </c>
-      <c r="B1182" s="72" t="s">
+      <c r="B1182" s="35" t="s">
         <v>1344</v>
       </c>
     </row>
     <row r="1183" spans="1:2">
-      <c r="A1183" s="74" t="s">
+      <c r="A1183" s="34" t="s">
         <v>1345</v>
       </c>
-      <c r="B1183" s="72" t="s">
+      <c r="B1183" s="35" t="s">
         <v>1346</v>
       </c>
     </row>
     <row r="1184" spans="1:2">
-      <c r="A1184" s="74" t="s">
+      <c r="A1184" s="34" t="s">
         <v>1347</v>
       </c>
-      <c r="B1184" s="72" t="s">
+      <c r="B1184" s="35" t="s">
         <v>1348</v>
       </c>
     </row>
     <row r="1185" spans="1:2">
-      <c r="A1185" s="74" t="s">
+      <c r="A1185" s="34" t="s">
         <v>1349</v>
       </c>
-      <c r="B1185" s="72" t="s">
+      <c r="B1185" s="35" t="s">
         <v>1350</v>
       </c>
     </row>
     <row r="1186" spans="1:2">
-      <c r="A1186" s="74" t="s">
+      <c r="A1186" s="34" t="s">
         <v>1351</v>
       </c>
-      <c r="B1186" s="72" t="s">
+      <c r="B1186" s="35" t="s">
         <v>1352</v>
       </c>
     </row>
     <row r="1187" spans="1:2">
-      <c r="A1187" s="74" t="s">
+      <c r="A1187" s="34" t="s">
         <v>1353</v>
       </c>
-      <c r="B1187" s="72" t="s">
+      <c r="B1187" s="35" t="s">
         <v>1354</v>
       </c>
     </row>
     <row r="1188" spans="1:2">
-      <c r="A1188" s="74" t="s">
+      <c r="A1188" s="34" t="s">
         <v>1355</v>
       </c>
-      <c r="B1188" s="72" t="s">
+      <c r="B1188" s="35" t="s">
         <v>1356</v>
       </c>
     </row>
     <row r="1189" spans="1:2">
-      <c r="A1189" s="74" t="s">
+      <c r="A1189" s="34" t="s">
         <v>1357</v>
       </c>
-      <c r="B1189" s="72" t="s">
+      <c r="B1189" s="35" t="s">
         <v>1358</v>
       </c>
     </row>
     <row r="1190" spans="1:2">
-      <c r="A1190" s="74" t="s">
+      <c r="A1190" s="34" t="s">
         <v>1922</v>
       </c>
-      <c r="B1190" s="72" t="s">
+      <c r="B1190" s="35" t="s">
         <v>1366</v>
       </c>
     </row>
     <row r="1191" spans="1:2">
-      <c r="A1191" s="74" t="s">
+      <c r="A1191" s="34" t="s">
         <v>1923</v>
       </c>
-      <c r="B1191" s="72" t="s">
+      <c r="B1191" s="35" t="s">
         <v>1368</v>
       </c>
     </row>
     <row r="1192" spans="1:2">
-      <c r="A1192" s="74" t="s">
+      <c r="A1192" s="34" t="s">
         <v>1924</v>
       </c>
-      <c r="B1192" s="72" t="s">
+      <c r="B1192" s="35" t="s">
         <v>1925</v>
       </c>
     </row>
     <row r="1193" spans="1:2">
-      <c r="A1193" s="74" t="s">
+      <c r="A1193" s="34" t="s">
         <v>1926</v>
       </c>
-      <c r="B1193" s="72" t="s">
+      <c r="B1193" s="35" t="s">
         <v>1927</v>
       </c>
     </row>
     <row r="1194" spans="1:2">
-      <c r="A1194" s="74" t="s">
+      <c r="A1194" s="34" t="s">
         <v>1928</v>
       </c>
-      <c r="B1194" s="72" t="s">
+      <c r="B1194" s="35" t="s">
         <v>1929</v>
       </c>
     </row>
     <row r="1195" spans="1:2">
-      <c r="A1195" s="74" t="s">
+      <c r="A1195" s="34" t="s">
         <v>1930</v>
       </c>
-      <c r="B1195" s="72" t="s">
+      <c r="B1195" s="35" t="s">
         <v>1931</v>
       </c>
     </row>
     <row r="1196" spans="1:2">
-      <c r="A1196" s="74" t="s">
+      <c r="A1196" s="34" t="s">
         <v>1932</v>
       </c>
-      <c r="B1196" s="72" t="s">
+      <c r="B1196" s="35" t="s">
         <v>1932</v>
       </c>
     </row>
     <row r="1197" spans="1:2">
-      <c r="A1197" s="74" t="s">
+      <c r="A1197" s="34" t="s">
         <v>1933</v>
       </c>
-      <c r="B1197" s="72" t="s">
+      <c r="B1197" s="35" t="s">
         <v>1933</v>
       </c>
     </row>
     <row r="1198" spans="1:2">
-      <c r="A1198" s="74" t="s">
+      <c r="A1198" s="34" t="s">
         <v>1934</v>
       </c>
-      <c r="B1198" s="72" t="s">
+      <c r="B1198" s="35" t="s">
         <v>1934</v>
       </c>
     </row>
     <row r="1199" spans="1:2">
-      <c r="A1199" s="74" t="s">
+      <c r="A1199" s="34" t="s">
         <v>1441</v>
       </c>
-      <c r="B1199" s="72" t="s">
+      <c r="B1199" s="35" t="s">
         <v>1442</v>
       </c>
     </row>
     <row r="1200" spans="1:2">
-      <c r="A1200" s="74" t="s">
+      <c r="A1200" s="34" t="s">
         <v>1443</v>
       </c>
-      <c r="B1200" s="72" t="s">
+      <c r="B1200" s="35" t="s">
         <v>1444</v>
       </c>
     </row>
     <row r="1201" spans="1:2">
-      <c r="A1201" s="74" t="s">
+      <c r="A1201" s="34" t="s">
         <v>1445</v>
       </c>
-      <c r="B1201" s="72" t="s">
+      <c r="B1201" s="35" t="s">
         <v>1446</v>
       </c>
     </row>
     <row r="1202" spans="1:2">
-      <c r="A1202" s="74" t="s">
+      <c r="A1202" s="34" t="s">
         <v>1447</v>
       </c>
-      <c r="B1202" s="72" t="s">
+      <c r="B1202" s="35" t="s">
         <v>1448</v>
       </c>
     </row>
     <row r="1203" spans="1:2">
-      <c r="A1203" s="74" t="s">
+      <c r="A1203" s="34" t="s">
         <v>1449</v>
       </c>
-      <c r="B1203" s="72" t="s">
+      <c r="B1203" s="35" t="s">
         <v>1376</v>
       </c>
     </row>
     <row r="1204" spans="1:2">
-      <c r="A1204" s="74" t="s">
+      <c r="A1204" s="34" t="s">
         <v>1450</v>
       </c>
-      <c r="B1204" s="72" t="s">
+      <c r="B1204" s="35" t="s">
         <v>1378</v>
       </c>
     </row>
     <row r="1205" spans="1:2">
-      <c r="A1205" s="74" t="s">
+      <c r="A1205" s="34" t="s">
         <v>1451</v>
       </c>
-      <c r="B1205" s="72" t="s">
+      <c r="B1205" s="35" t="s">
         <v>1452</v>
       </c>
     </row>
     <row r="1206" spans="1:2">
-      <c r="A1206" s="73" t="s">
+      <c r="A1206" s="34" t="s">
         <v>1935</v>
       </c>
-      <c r="B1206" s="72" t="s">
+      <c r="B1206" s="35" t="s">
         <v>1936</v>
       </c>
     </row>
     <row r="1207" spans="1:2">
-      <c r="A1207" s="74" t="s">
+      <c r="A1207" s="34" t="s">
         <v>1937</v>
       </c>
-      <c r="B1207" s="72" t="s">
+      <c r="B1207" s="35" t="s">
         <v>1938</v>
       </c>
     </row>
     <row r="1208" spans="1:2">
-      <c r="A1208" s="74" t="s">
+      <c r="A1208" s="34" t="s">
         <v>1939</v>
       </c>
-      <c r="B1208" s="72" t="s">
+      <c r="B1208" s="35" t="s">
         <v>1940</v>
       </c>
     </row>
     <row r="1209" spans="1:2">
-      <c r="A1209" s="74" t="s">
+      <c r="A1209" s="34" t="s">
         <v>1519</v>
       </c>
-      <c r="B1209" s="72" t="s">
+      <c r="B1209" s="35" t="s">
         <v>1520</v>
       </c>
     </row>
     <row r="1210" spans="1:2">
-      <c r="A1210" s="74" t="s">
+      <c r="A1210" s="34" t="s">
         <v>1521</v>
       </c>
-      <c r="B1210" s="72" t="s">
+      <c r="B1210" s="35" t="s">
         <v>1522</v>
       </c>
     </row>
     <row r="1211" spans="1:2">
-      <c r="A1211" s="73" t="s">
+      <c r="A1211" s="34" t="s">
         <v>1941</v>
       </c>
-      <c r="B1211" s="74" t="s">
+      <c r="B1211" s="34" t="s">
         <v>1942</v>
       </c>
     </row>
     <row r="1212" spans="1:2">
-      <c r="A1212" s="73" t="s">
+      <c r="A1212" s="34" t="s">
         <v>1943</v>
       </c>
-      <c r="B1212" s="79" t="s">
+      <c r="B1212" s="72" t="s">
         <v>1944</v>
       </c>
     </row>
     <row r="1213" spans="1:2">
-      <c r="A1213" s="73" t="s">
+      <c r="A1213" s="34" t="s">
         <v>1945</v>
       </c>
-      <c r="B1213" s="80" t="s">
+      <c r="B1213" s="73" t="s">
         <v>918</v>
       </c>
     </row>
     <row r="1214" spans="1:2">
-      <c r="A1214" s="73" t="s">
+      <c r="A1214" s="34" t="s">
         <v>1946</v>
       </c>
-      <c r="B1214" s="80" t="s">
+      <c r="B1214" s="73" t="s">
         <v>1414</v>
       </c>
     </row>
     <row r="1215" spans="1:2">
-      <c r="A1215" s="73" t="s">
+      <c r="A1215" s="34" t="s">
         <v>1947</v>
       </c>
-      <c r="B1215" s="72" t="s">
+      <c r="B1215" s="35" t="s">
         <v>1948</v>
       </c>
     </row>
     <row r="1216" spans="1:2">
-      <c r="A1216" s="73" t="s">
+      <c r="A1216" s="34" t="s">
         <v>1949</v>
       </c>
-      <c r="B1216" s="72" t="s">
+      <c r="B1216" s="35" t="s">
         <v>1948</v>
       </c>
     </row>
     <row r="1217" spans="1:2">
-      <c r="A1217" s="73" t="s">
+      <c r="A1217" s="34" t="s">
         <v>283</v>
       </c>
-      <c r="B1217" s="72" t="s">
+      <c r="B1217" s="35" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="1218" spans="1:2">
-      <c r="A1218" s="74" t="s">
+      <c r="A1218" s="34" t="s">
         <v>1565</v>
       </c>
-      <c r="B1218" s="72" t="s">
+      <c r="B1218" s="35" t="s">
         <v>1950</v>
       </c>
     </row>
     <row r="1219" spans="1:2">
-      <c r="A1219" s="74" t="s">
+      <c r="A1219" s="34" t="s">
         <v>1567</v>
       </c>
-      <c r="B1219" s="72" t="s">
+      <c r="B1219" s="35" t="s">
         <v>1950</v>
       </c>
     </row>
     <row r="1220" spans="1:2">
-      <c r="A1220" s="74" t="s">
+      <c r="A1220" s="34" t="s">
         <v>1569</v>
       </c>
-      <c r="B1220" s="72" t="s">
+      <c r="B1220" s="35" t="s">
         <v>1569</v>
       </c>
     </row>
     <row r="1221" spans="1:2">
-      <c r="A1221" s="74" t="s">
+      <c r="A1221" s="34" t="s">
         <v>1570</v>
       </c>
-      <c r="B1221" s="72" t="s">
+      <c r="B1221" s="35" t="s">
         <v>1570</v>
       </c>
     </row>
     <row r="1222" spans="1:2">
-      <c r="A1222" s="74" t="s">
+      <c r="A1222" s="34" t="s">
         <v>1571</v>
       </c>
-      <c r="B1222" s="72" t="s">
+      <c r="B1222" s="35" t="s">
         <v>1571</v>
       </c>
     </row>
     <row r="1223" spans="1:2">
-      <c r="A1223" s="73" t="s">
+      <c r="A1223" s="34" t="s">
         <v>542</v>
       </c>
-      <c r="B1223" s="72" t="s">
+      <c r="B1223" s="35" t="s">
         <v>543</v>
       </c>
     </row>
     <row r="1224" spans="1:2">
-      <c r="A1224" s="74" t="s">
+      <c r="A1224" s="34" t="s">
         <v>1951</v>
       </c>
-      <c r="B1224" s="74" t="s">
+      <c r="B1224" s="34" t="s">
         <v>1859</v>
       </c>
     </row>
     <row r="1225" spans="1:2">
-      <c r="A1225" s="73" t="s">
+      <c r="A1225" s="34" t="s">
         <v>1952</v>
       </c>
-      <c r="B1225" s="75" t="s">
+      <c r="B1225" s="35" t="s">
         <v>564</v>
       </c>
     </row>
     <row r="1226" spans="1:2">
-      <c r="A1226" s="74" t="s">
+      <c r="A1226" s="34" t="s">
         <v>1953</v>
       </c>
-      <c r="B1226" s="72" t="s">
+      <c r="B1226" s="35" t="s">
         <v>1954</v>
       </c>
     </row>
     <row r="1227" spans="1:2">
-      <c r="A1227" s="73" t="s">
+      <c r="A1227" s="34" t="s">
         <v>1955</v>
       </c>
-      <c r="B1227" s="72" t="s">
+      <c r="B1227" s="35" t="s">
         <v>1956</v>
       </c>
     </row>
     <row r="1228" spans="1:2">
-      <c r="A1228" s="74" t="s">
+      <c r="A1228" s="34" t="s">
         <v>1957</v>
       </c>
-      <c r="B1228" s="72" t="s">
+      <c r="B1228" s="35" t="s">
         <v>1958</v>
       </c>
     </row>
     <row r="1229" spans="1:2">
-      <c r="A1229" s="73" t="s">
+      <c r="A1229" s="34" t="s">
         <v>1959</v>
       </c>
-      <c r="B1229" s="72" t="s">
+      <c r="B1229" s="35" t="s">
         <v>1803</v>
       </c>
     </row>
     <row r="1230" spans="1:2">
-      <c r="A1230" s="74" t="s">
+      <c r="A1230" s="34" t="s">
         <v>1960</v>
       </c>
-      <c r="B1230" s="72" t="s">
+      <c r="B1230" s="35" t="s">
         <v>1904</v>
       </c>
     </row>
     <row r="1231" spans="1:2">
-      <c r="A1231" s="73" t="s">
+      <c r="A1231" s="34" t="s">
         <v>1961</v>
       </c>
-      <c r="B1231" s="72" t="s">
+      <c r="B1231" s="35" t="s">
         <v>1962</v>
       </c>
     </row>
     <row r="1232" spans="1:2">
-      <c r="A1232" s="73" t="s">
+      <c r="A1232" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B1232" s="77" t="s">
+      <c r="B1232" s="71" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="1233" spans="1:2">
-      <c r="A1233" s="73" t="s">
+      <c r="A1233" s="34" t="s">
         <v>1963</v>
       </c>
-      <c r="B1233" s="77" t="s">
+      <c r="B1233" s="71" t="s">
         <v>1964</v>
       </c>
     </row>
     <row r="1234" spans="1:2">
-      <c r="A1234" s="73" t="s">
+      <c r="A1234" s="34" t="s">
         <v>1965</v>
       </c>
-      <c r="B1234" s="77" t="s">
+      <c r="B1234" s="71" t="s">
         <v>1966</v>
       </c>
     </row>
     <row r="1235" spans="1:2">
-      <c r="A1235" s="73" t="s">
+      <c r="A1235" s="34" t="s">
         <v>1967</v>
       </c>
-      <c r="B1235" s="72" t="s">
+      <c r="B1235" s="35" t="s">
         <v>1968</v>
       </c>
     </row>
     <row r="1236" spans="1:2">
-      <c r="A1236" s="73" t="s">
+      <c r="A1236" s="34" t="s">
         <v>1969</v>
       </c>
-      <c r="B1236" s="72" t="s">
+      <c r="B1236" s="35" t="s">
         <v>1970</v>
       </c>
     </row>
     <row r="1237" spans="1:2">
-      <c r="A1237" s="73" t="s">
+      <c r="A1237" s="34" t="s">
         <v>1971</v>
       </c>
-      <c r="B1237" s="72" t="s">
+      <c r="B1237" s="35" t="s">
         <v>1972</v>
       </c>
     </row>
     <row r="1238" spans="1:2">
-      <c r="A1238" s="74" t="s">
+      <c r="A1238" s="34" t="s">
         <v>1973</v>
       </c>
-      <c r="B1238" s="72" t="s">
+      <c r="B1238" s="35" t="s">
         <v>1974</v>
       </c>
     </row>
     <row r="1239" spans="1:2">
-      <c r="A1239" s="74" t="s">
+      <c r="A1239" s="34" t="s">
         <v>1975</v>
       </c>
-      <c r="B1239" s="72" t="s">
+      <c r="B1239" s="35" t="s">
         <v>1974</v>
       </c>
     </row>
     <row r="1240" spans="1:2">
-      <c r="A1240" s="74" t="s">
+      <c r="A1240" s="34" t="s">
         <v>1976</v>
       </c>
-      <c r="B1240" s="72" t="s">
+      <c r="B1240" s="35" t="s">
         <v>1977</v>
       </c>
     </row>
     <row r="1241" spans="1:2">
-      <c r="A1241" s="74" t="s">
+      <c r="A1241" s="34" t="s">
         <v>1978</v>
       </c>
-      <c r="B1241" s="72" t="s">
+      <c r="B1241" s="35" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="1242" spans="1:2">
-      <c r="A1242" s="74" t="s">
+      <c r="A1242" s="34" t="s">
         <v>1979</v>
       </c>
-      <c r="B1242" s="72" t="s">
+      <c r="B1242" s="35" t="s">
         <v>1980</v>
       </c>
     </row>
     <row r="1243" spans="1:2">
-      <c r="A1243" s="74" t="s">
+      <c r="A1243" s="34" t="s">
         <v>1981</v>
       </c>
-      <c r="B1243" s="72" t="s">
+      <c r="B1243" s="35" t="s">
         <v>1982</v>
+      </c>
+    </row>
+    <row r="1244" spans="1:2">
+      <c r="A1244" s="34" t="s">
+        <v>1983</v>
+      </c>
+      <c r="B1244" s="35" t="s">
+        <v>1984</v>
+      </c>
+    </row>
+    <row r="1245" spans="1:2">
+      <c r="A1245" s="34" t="s">
+        <v>1985</v>
+      </c>
+      <c r="B1245" s="35" t="s">
+        <v>1986</v>
+      </c>
+    </row>
+    <row r="1246" spans="1:2">
+      <c r="A1246" s="34" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1246" s="35" t="s">
+        <v>1919</v>
+      </c>
+    </row>
+    <row r="1247" spans="1:2">
+      <c r="A1247" s="34" t="s">
+        <v>1963</v>
+      </c>
+      <c r="B1247" s="35" t="s">
+        <v>1964</v>
+      </c>
+    </row>
+    <row r="1248" spans="1:2">
+      <c r="A1248" s="34" t="s">
+        <v>1965</v>
+      </c>
+      <c r="B1248" s="35" t="s">
+        <v>1966</v>
+      </c>
+    </row>
+    <row r="1249" spans="1:2">
+      <c r="A1249" s="34" t="s">
+        <v>1988</v>
+      </c>
+      <c r="B1249" s="35" t="s">
+        <v>1989</v>
+      </c>
+    </row>
+    <row r="1250" spans="1:2">
+      <c r="A1250" s="34" t="s">
+        <v>1990</v>
+      </c>
+      <c r="B1250" s="35" t="s">
+        <v>1991</v>
       </c>
     </row>
   </sheetData>
@@ -19424,9 +19476,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B54"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -19440,426 +19492,426 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>1983</v>
+        <v>1992</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1984</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>1985</v>
+        <v>1994</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1986</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>1987</v>
+        <v>1996</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1988</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>1989</v>
+        <v>1998</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1990</v>
+        <v>1999</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>1991</v>
+        <v>2000</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1992</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>1993</v>
+        <v>2002</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1994</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>1995</v>
+        <v>2004</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1996</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>1997</v>
+        <v>2006</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1998</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>1999</v>
+        <v>2008</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>2000</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>2001</v>
+        <v>2010</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>2002</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>2003</v>
+        <v>2012</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>2004</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>2005</v>
+        <v>2014</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>2006</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>2007</v>
+        <v>2016</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>2008</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>2009</v>
+        <v>2018</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>2010</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>2011</v>
+        <v>2020</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>2012</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>2013</v>
+        <v>2022</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>2014</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>2015</v>
+        <v>2024</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>2016</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>2017</v>
+        <v>2026</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>2018</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>2019</v>
+        <v>2028</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>2020</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>2021</v>
+        <v>2030</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>2022</v>
+        <v>2031</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>2023</v>
+        <v>2032</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>2024</v>
+        <v>2033</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>2025</v>
+        <v>2034</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="24" ht="246.5" spans="1:2">
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="24" ht="244.8" spans="1:2">
       <c r="A24" s="2" t="s">
-        <v>2027</v>
+        <v>2036</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="25" ht="232" spans="1:2">
+        <v>2037</v>
+      </c>
+    </row>
+    <row r="25" ht="230.4" spans="1:2">
       <c r="A25" t="s">
-        <v>2029</v>
+        <v>2038</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>2030</v>
-      </c>
-    </row>
-    <row r="26" ht="261" spans="1:2">
+        <v>2039</v>
+      </c>
+    </row>
+    <row r="26" ht="259.2" spans="1:2">
       <c r="A26" t="s">
-        <v>2031</v>
+        <v>2040</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>2032</v>
-      </c>
-    </row>
-    <row r="27" ht="203" spans="1:2">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="27" ht="201.6" spans="1:2">
       <c r="A27" t="s">
-        <v>2033</v>
+        <v>2042</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>2034</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>2035</v>
+        <v>2044</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>2036</v>
+        <v>2045</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>1983</v>
+        <v>1992</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1984</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>1985</v>
+        <v>1994</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1986</v>
-      </c>
-    </row>
-    <row r="31" ht="174" spans="1:2">
+        <v>1995</v>
+      </c>
+    </row>
+    <row r="31" ht="172.8" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>1991</v>
+        <v>2000</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>1992</v>
-      </c>
-    </row>
-    <row r="32" ht="130.5" spans="1:2">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="32" ht="129.6" spans="1:2">
       <c r="A32" s="13" t="s">
-        <v>2037</v>
+        <v>2046</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>2038</v>
-      </c>
-    </row>
-    <row r="33" ht="174" spans="1:2">
+        <v>2047</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
       <c r="A33" s="15" t="s">
-        <v>2039</v>
+        <v>2048</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>2040</v>
-      </c>
-    </row>
-    <row r="34" ht="174" spans="1:2">
+        <v>2049</v>
+      </c>
+    </row>
+    <row r="34" ht="172.8" spans="1:2">
       <c r="A34" s="17" t="s">
-        <v>2041</v>
+        <v>2050</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>2042</v>
+        <v>2051</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>2013</v>
+        <v>2022</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>2043</v>
-      </c>
-    </row>
-    <row r="36" ht="406" spans="1:2">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="36" ht="403.2" spans="1:2">
       <c r="A36" s="21" t="s">
-        <v>2044</v>
+        <v>2053</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>2045</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>2046</v>
+        <v>2055</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>2047</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>2048</v>
+        <v>2057</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>2049</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>2050</v>
+        <v>2059</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>2051</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
-        <v>2052</v>
+        <v>2061</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>2053</v>
-      </c>
-    </row>
-    <row r="41" ht="116" spans="1:2">
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="41" ht="115.2" spans="1:2">
       <c r="A41" t="s">
-        <v>2054</v>
+        <v>2063</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>2055</v>
-      </c>
-    </row>
-    <row r="42" ht="174" spans="1:2">
+        <v>2064</v>
+      </c>
+    </row>
+    <row r="42" ht="172.8" spans="1:2">
       <c r="A42" t="s">
-        <v>2056</v>
+        <v>2065</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>2057</v>
-      </c>
-    </row>
-    <row r="43" ht="188.5" spans="1:2">
+        <v>2066</v>
+      </c>
+    </row>
+    <row r="43" ht="187.2" spans="1:2">
       <c r="A43" t="s">
-        <v>2058</v>
+        <v>2067</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>2059</v>
-      </c>
-    </row>
-    <row r="44" ht="116" spans="1:2">
+        <v>2068</v>
+      </c>
+    </row>
+    <row r="44" ht="115.2" spans="1:2">
       <c r="A44" t="s">
-        <v>2060</v>
+        <v>2069</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>2061</v>
+        <v>2070</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>2062</v>
+        <v>2071</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>2063</v>
+        <v>2072</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>2064</v>
+        <v>2073</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>2065</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
-        <v>2066</v>
+        <v>2075</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>2067</v>
-      </c>
-    </row>
-    <row r="48" ht="261" spans="1:2">
+        <v>2076</v>
+      </c>
+    </row>
+    <row r="48" ht="259.2" spans="1:2">
       <c r="A48" t="s">
-        <v>2068</v>
+        <v>2077</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>2069</v>
+        <v>2078</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
-        <v>2070</v>
+        <v>2079</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>2071</v>
-      </c>
-    </row>
-    <row r="50" ht="333.5" spans="1:2">
+        <v>2080</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
       <c r="A50" t="s">
-        <v>2072</v>
+        <v>2081</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>2073</v>
-      </c>
-    </row>
-    <row r="51" ht="333.5" spans="1:2">
+        <v>2082</v>
+      </c>
+    </row>
+    <row r="51" ht="331.2" spans="1:2">
       <c r="A51" t="s">
-        <v>2074</v>
+        <v>2083</v>
       </c>
       <c r="B51" s="29" t="s">
-        <v>2075</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="52" ht="36" customHeight="1" spans="1:2">
       <c r="A52" t="s">
-        <v>2076</v>
+        <v>2085</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>2077</v>
+        <v>2086</v>
       </c>
     </row>
     <row r="53" ht="23.25" customHeight="1" spans="1:2">
       <c r="A53" t="s">
-        <v>2078</v>
+        <v>2087</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>2079</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="54" ht="27.75" customHeight="1" spans="1:2">
       <c r="A54" t="s">
-        <v>2080</v>
+        <v>2089</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>2081</v>
+        <v>2090</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated locators and Open So , Open so Amd , Items , Item Unit Asso , Customer Item , Catalogue Price , Price List ,Std Price Script Stabled
Updated locators and Open So , Open so Amd , Items , Item Unit Asso , Customer Item , Catalogue Price , Price List ,Std Price Script Stabled
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="8400" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="125725"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2647" uniqueCount="2151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2651" uniqueCount="2154">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -8444,6 +8444,15 @@
 AND LSS_VOU_NO = '${SONO}'
 AND LSS_PROD_ID = '${PONO}'
 AND LSS_SER_NO = '${SRNO}'</t>
+  </si>
+  <si>
+    <t>QcFlag</t>
+  </si>
+  <si>
+    <t>PriceBasisOpenSo</t>
+  </si>
+  <si>
+    <t>Open SO</t>
   </si>
 </sst>
 </file>
@@ -9053,7 +9062,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1282"/>
+  <dimension ref="A1:B1284"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
@@ -19315,6 +19324,22 @@
       </c>
       <c r="B1282" s="77" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="1283" spans="1:2">
+      <c r="A1283" s="76" t="s">
+        <v>2151</v>
+      </c>
+      <c r="B1283" s="77" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="1284" spans="1:2">
+      <c r="A1284" s="76" t="s">
+        <v>2152</v>
+      </c>
+      <c r="B1284" s="77" t="s">
+        <v>2153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stabilized OpenPo, SOB, Setup Purchase Screens
Stabilized OpenPo, SOB, Setup Purchase Screens
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="8400" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2761" uniqueCount="2244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2763" uniqueCount="2244">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -4662,9 +4662,6 @@
     <t>UserDefinedGeneral</t>
   </si>
   <si>
-    <t>User Defined/General</t>
-  </si>
-  <si>
     <t>Apps</t>
   </si>
   <si>
@@ -4678,9 +4675,6 @@
   </si>
   <si>
     <t>CostBasis</t>
-  </si>
-  <si>
-    <t>User Defined Price</t>
   </si>
   <si>
     <t>OpenBlanket</t>
@@ -8781,6 +8775,139 @@
 ICMCTRL_AUTO_MTR_COMPL_FLAG  Auto_Post_MRV from ICM_CONTROL
 where ICMCTRL_BU ='${APLBU}'</t>
   </si>
+  <si>
+    <t>PRLineDetailsQueryKARE</t>
+  </si>
+  <si>
+    <t>SELECT prl_bu,
+       prl_rqst_no,
+       prl_seq_no,
+       prl_prod_id,
+       prl_prod_rev,
+       prl_prod_desc1,
+       prl_class_id,
+       prl_class_desc,
+       prl_sub_cls_id,
+       prl_sub_cls_desc,
+       prl_uom,
+       prl_prod_uom,
+       prl_conv_factor,
+       prl_requested_qty,
+       (prl_requested_qty * prl_bc_unit_cost) line_amount,
+       prl_ordered_qty,
+       prl_receipt_qty,
+       prl_bc_unit_cost,
+       prl_disc_pct,
+       prl_stocked,
+       prl_qc_required,
+       prl_quote_pfx,
+       prl_quote_no,
+       prl_order_pfx,
+       prl_order_no,
+       prl_net_disc_flag,
+       prl_status,
+      case when prl_status = 'R' then 'Entry Completed'
+            when prl_status = 'A' then 'Approved'
+            when prl_status = 'C' then 'Cancelled'
+            when prl_status = 'L' then 'Close Shorted'
+            when prl_status = 'E' then 'Draft' END  STATUS, 
+       prl_prod_temp_id,
+       prl_prod_temp_rev,
+       prl_work_ord_no,
+       prl_select_flag,
+       prl_ins_plan_no,
+       prl_ins_plan_rev,
+       prl_prod_ord_no,
+       prl_sf_code,
+       prl_test_req_flag,
+       prl_cert_id,
+       prl_print_seq_no,
+       prl_prod_temp_desc1,
+       prl_ref,
+       prl_prod_ext_desc,
+       prl_cs_narr,
+       prl_drawing_no,
+       prl_drawing_rev,
+       prl_spr_type,
+       prl_rcpt_rcvd_qty,
+       prl_dim_req_flag,
+       prl_thickness,
+       prl_length,
+       prl_width,
+       prl_qty_in_nos,
+       prl_serv_prod_id,
+       prl_serv_io_type,
+       prl_amc_start_date,
+       prl_amc_end_date,
+       prl_serv_prod_desc,
+       prl_tool_wo_no,
+       prl_sugg_suplr_id,
+       prl_cls_sel_user,
+       prl_cls_qty,
+       prl_cls_proc_qty,
+       prl_cap_asset_id,
+       prl_cust_drw_no,
+       prl_cust_drw_rev,
+       prl_catalog_no,
+       prl_mchn_id,
+       prl_sub_dept_id,
+       prl_priority,
+       prl_buyer_id,
+       prl_mrp_rel_qty,
+       prl_mftr_id,
+       prl_mftr_part_no,
+       prl_eqpmt_id,
+       prl_eqpmt_desc,
+       prl_buyer_emp_id,
+       prl_lpp_rcpt_pfx,
+       prl_lpp_rcpt_no,
+       prl_mchn_grp_id,
+       prl_pr_plan_no,
+       prl_prod_outer_dia,
+       prl_cre_by,
+       prl_cre_ip_addr,
+       prl_cre_os_user,
+       prl_cre_date,
+       prl_upd_by,
+       prl_upd_ip_addr,
+       prl_upd_os_user,
+       prl_upd_date,
+       prl_cre_emp_id,
+       prl_upd_emp_id,
+       prl_last_po_price,
+       prl_prod_chng_flag,
+       prl_batch_no,
+       prl_expiry_date,
+       prl_mfg_date,
+       prl_sterilize_date,
+       prl_iss_code,
+       prl_height,
+       prl_inner_dia,
+       prl_density,
+       prl_pur_acct,
+       prl_cc_code,
+       prl_fab_item_type,
+       prl_gla_fxd_flag,
+       prl_cpc_fxd_flag,
+      prl_store_id,
+      prl_store_name,
+      prl_required_date,
+      prl_so_type,
+      prl_so_pfx,
+      prl_so_no,
+      prl_so_seq_no,
+      prl_so_sub_seq_no,
+      prl_proj_id,
+      prl_task_id,
+      prl_so_schld_desc,  
+      prl_shipto_loc_id,
+      prl_shipto_loc_name,
+      prl_rfq
+   FROM pur_req_ln
+  WHERE prl_bu       ='KARE'                    
+    AND PRL_RQST_NO  ='${PRNO}'
+    AND PRL_PROD_ID  ='${ItemId}'</t>
+  </si>
 </sst>
 </file>
 
@@ -8792,7 +8919,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8835,12 +8962,6 @@
     <font>
       <sz val="14"/>
       <color rgb="FF262626"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -8989,7 +9110,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -9125,12 +9246,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -9353,13 +9468,16 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -9368,118 +9486,115 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -9500,7 +9615,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9644,9 +9759,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -9655,11 +9767,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -10000,10 +10107,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B1335"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -14955,7 +15062,7 @@
       <c r="A619" s="47" t="s">
         <v>1050</v>
       </c>
-      <c r="B619" s="67">
+      <c r="B619" s="66">
         <v>3</v>
       </c>
     </row>
@@ -16331,7 +16438,7 @@
       <c r="A791" s="41" t="s">
         <v>1341</v>
       </c>
-      <c r="B791" s="68" t="s">
+      <c r="B791" s="67" t="s">
         <v>986</v>
       </c>
     </row>
@@ -17220,52 +17327,52 @@
         <v>1543</v>
       </c>
       <c r="B902" s="35" t="s">
-        <v>1544</v>
+        <v>316</v>
       </c>
     </row>
     <row r="903" spans="1:2">
       <c r="A903" s="34" t="s">
+        <v>1544</v>
+      </c>
+      <c r="B903" s="35" t="s">
         <v>1545</v>
-      </c>
-      <c r="B903" s="35" t="s">
-        <v>1546</v>
       </c>
     </row>
     <row r="904" spans="1:2">
       <c r="A904" s="34" t="s">
+        <v>1546</v>
+      </c>
+      <c r="B904" s="35" t="s">
         <v>1547</v>
-      </c>
-      <c r="B904" s="35" t="s">
-        <v>1548</v>
       </c>
     </row>
     <row r="905" spans="1:2">
       <c r="A905" s="34" t="s">
-        <v>1549</v>
+        <v>1548</v>
       </c>
       <c r="B905" s="35" t="s">
-        <v>1550</v>
+        <v>316</v>
       </c>
     </row>
     <row r="906" spans="1:2">
       <c r="A906" s="34" t="s">
-        <v>1551</v>
+        <v>1549</v>
       </c>
       <c r="B906" s="35" t="s">
-        <v>1552</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="907" spans="1:2">
       <c r="A907" s="34" t="s">
-        <v>1553</v>
+        <v>1551</v>
       </c>
       <c r="B907" s="35" t="s">
-        <v>1554</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="908" spans="1:2">
       <c r="A908" s="34" t="s">
-        <v>1555</v>
+        <v>1553</v>
       </c>
       <c r="B908" s="35" t="s">
         <v>1536</v>
@@ -17273,15 +17380,15 @@
     </row>
     <row r="909" spans="1:2">
       <c r="A909" s="34" t="s">
-        <v>1556</v>
+        <v>1554</v>
       </c>
       <c r="B909" s="35" t="s">
-        <v>1556</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="910" spans="1:2">
       <c r="A910" s="34" t="s">
-        <v>1557</v>
+        <v>1555</v>
       </c>
       <c r="B910" s="35" t="s">
         <v>1400</v>
@@ -17289,7 +17396,7 @@
     </row>
     <row r="911" spans="1:2">
       <c r="A911" s="34" t="s">
-        <v>1558</v>
+        <v>1556</v>
       </c>
       <c r="B911" s="35" t="s">
         <v>495</v>
@@ -17297,7 +17404,7 @@
     </row>
     <row r="912" spans="1:2">
       <c r="A912" s="34" t="s">
-        <v>1559</v>
+        <v>1557</v>
       </c>
       <c r="B912" s="46" t="s">
         <v>278</v>
@@ -17305,87 +17412,87 @@
     </row>
     <row r="913" spans="1:2">
       <c r="A913" s="34" t="s">
-        <v>1560</v>
+        <v>1558</v>
       </c>
       <c r="B913" s="35" t="s">
-        <v>1561</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="914" spans="1:2">
       <c r="A914" s="34" t="s">
-        <v>1562</v>
+        <v>1560</v>
       </c>
       <c r="B914" s="35" t="s">
-        <v>1563</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="915" spans="1:2">
       <c r="A915" s="34" t="s">
-        <v>1564</v>
+        <v>1562</v>
       </c>
       <c r="B915" s="35" t="s">
-        <v>1565</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="916" spans="1:2">
       <c r="A916" s="34" t="s">
-        <v>1566</v>
+        <v>1564</v>
       </c>
       <c r="B916" s="35" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="917" spans="1:2">
       <c r="A917" s="34" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="B917" s="34" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="918" spans="1:2">
       <c r="A918" s="34" t="s">
-        <v>1569</v>
+        <v>1567</v>
       </c>
       <c r="B918" s="34" t="s">
-        <v>1569</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="919" spans="1:2">
       <c r="A919" s="34" t="s">
-        <v>1570</v>
+        <v>1568</v>
       </c>
       <c r="B919" s="34" t="s">
-        <v>1570</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="920" spans="1:2">
       <c r="A920" s="34" t="s">
-        <v>1571</v>
+        <v>1569</v>
       </c>
       <c r="B920" s="35" t="s">
-        <v>1572</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="921" spans="1:2">
       <c r="A921" s="34" t="s">
-        <v>1573</v>
+        <v>1571</v>
       </c>
       <c r="B921" s="35" t="s">
-        <v>1574</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="922" spans="1:2">
       <c r="A922" s="34" t="s">
-        <v>1575</v>
+        <v>1573</v>
       </c>
       <c r="B922" s="35" t="s">
-        <v>1576</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="923" spans="1:2">
       <c r="A923" s="34" t="s">
-        <v>1577</v>
+        <v>1575</v>
       </c>
       <c r="B923" s="35" t="s">
         <v>47</v>
@@ -17393,15 +17500,15 @@
     </row>
     <row r="924" spans="1:2">
       <c r="A924" s="34" t="s">
-        <v>1578</v>
+        <v>1576</v>
       </c>
       <c r="B924" s="35" t="s">
-        <v>1579</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="925" spans="1:2">
       <c r="A925" s="34" t="s">
-        <v>1580</v>
+        <v>1578</v>
       </c>
       <c r="B925" s="35" t="s">
         <v>166</v>
@@ -17409,18 +17516,18 @@
     </row>
     <row r="926" spans="1:2">
       <c r="A926" s="34" t="s">
-        <v>1581</v>
+        <v>1579</v>
       </c>
       <c r="B926" s="35" t="s">
-        <v>1582</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="927" spans="1:2">
       <c r="A927" s="34" t="s">
-        <v>1583</v>
+        <v>1581</v>
       </c>
       <c r="B927" s="35" t="s">
-        <v>1584</v>
+        <v>1582</v>
       </c>
     </row>
     <row r="928" spans="1:2">
@@ -17428,156 +17535,156 @@
         <v>760</v>
       </c>
       <c r="B928" s="35" t="s">
-        <v>1585</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="929" spans="1:2">
       <c r="A929" s="34" t="s">
-        <v>1586</v>
+        <v>1584</v>
       </c>
       <c r="B929" s="35" t="s">
-        <v>1587</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="930" spans="1:2">
       <c r="A930" s="34" t="s">
-        <v>1588</v>
+        <v>1586</v>
       </c>
       <c r="B930" s="35" t="s">
-        <v>1589</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="931" spans="1:2">
       <c r="A931" s="34" t="s">
-        <v>1590</v>
+        <v>1588</v>
       </c>
       <c r="B931" s="35" t="s">
-        <v>1591</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="932" spans="1:2">
       <c r="A932" s="34" t="s">
-        <v>1592</v>
+        <v>1590</v>
       </c>
       <c r="B932" s="35" t="s">
-        <v>1593</v>
+        <v>1591</v>
       </c>
     </row>
     <row r="933" spans="1:2">
       <c r="A933" s="34" t="s">
-        <v>1594</v>
+        <v>1592</v>
       </c>
       <c r="B933" s="35" t="s">
-        <v>1595</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="934" spans="1:2">
       <c r="A934" s="34" t="s">
-        <v>1596</v>
+        <v>1594</v>
       </c>
       <c r="B934" s="35" t="s">
-        <v>1597</v>
+        <v>1595</v>
       </c>
     </row>
     <row r="935" spans="1:2">
       <c r="A935" s="34" t="s">
-        <v>1598</v>
+        <v>1596</v>
       </c>
       <c r="B935" s="35" t="s">
-        <v>1599</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="936" spans="1:2">
       <c r="A936" s="34" t="s">
-        <v>1600</v>
+        <v>1598</v>
       </c>
       <c r="B936" s="35" t="s">
-        <v>1601</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="937" spans="1:2">
       <c r="A937" s="34" t="s">
-        <v>1602</v>
+        <v>1600</v>
       </c>
       <c r="B937" s="35" t="s">
-        <v>1603</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="938" spans="1:2">
       <c r="A938" s="34" t="s">
-        <v>1604</v>
+        <v>1602</v>
       </c>
       <c r="B938" s="35" t="s">
-        <v>1605</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="939" spans="1:2">
       <c r="A939" s="34" t="s">
-        <v>1606</v>
+        <v>1604</v>
       </c>
       <c r="B939" s="35" t="s">
-        <v>1607</v>
+        <v>1605</v>
       </c>
     </row>
     <row r="940" spans="1:2">
       <c r="A940" s="34" t="s">
-        <v>1608</v>
+        <v>1606</v>
       </c>
       <c r="B940" s="35" t="s">
-        <v>1609</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="941" spans="1:2">
       <c r="A941" s="34" t="s">
-        <v>1610</v>
+        <v>1608</v>
       </c>
       <c r="B941" s="35" t="s">
-        <v>1611</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="942" spans="1:2">
       <c r="A942" s="34" t="s">
-        <v>1612</v>
+        <v>1610</v>
       </c>
       <c r="B942" s="35" t="s">
-        <v>1613</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="943" spans="1:2">
       <c r="A943" s="34" t="s">
-        <v>1614</v>
+        <v>1612</v>
       </c>
       <c r="B943" s="35" t="s">
-        <v>1615</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="944" spans="1:2">
       <c r="A944" s="34" t="s">
-        <v>1616</v>
+        <v>1614</v>
       </c>
       <c r="B944" s="35" t="s">
-        <v>1617</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="945" spans="1:2">
       <c r="A945" s="34" t="s">
-        <v>1618</v>
+        <v>1616</v>
       </c>
       <c r="B945" s="35" t="s">
-        <v>1619</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="946" spans="1:2">
       <c r="A946" s="34" t="s">
-        <v>1620</v>
+        <v>1618</v>
       </c>
       <c r="B946" s="35" t="s">
-        <v>1621</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="947" spans="1:2">
       <c r="A947" s="34" t="s">
-        <v>1622</v>
+        <v>1620</v>
       </c>
       <c r="B947" s="35" t="s">
         <v>475</v>
@@ -17585,7 +17692,7 @@
     </row>
     <row r="948" spans="1:2">
       <c r="A948" s="34" t="s">
-        <v>1623</v>
+        <v>1621</v>
       </c>
       <c r="B948" s="35" t="s">
         <v>563</v>
@@ -17593,7 +17700,7 @@
     </row>
     <row r="949" spans="1:2">
       <c r="A949" s="34" t="s">
-        <v>1624</v>
+        <v>1622</v>
       </c>
       <c r="B949" s="35" t="s">
         <v>69</v>
@@ -17601,7 +17708,7 @@
     </row>
     <row r="950" spans="1:2">
       <c r="A950" s="34" t="s">
-        <v>1625</v>
+        <v>1623</v>
       </c>
       <c r="B950" s="35" t="s">
         <v>35</v>
@@ -17609,55 +17716,55 @@
     </row>
     <row r="951" spans="1:2">
       <c r="A951" s="34" t="s">
-        <v>1626</v>
+        <v>1624</v>
       </c>
       <c r="B951" s="35" t="s">
-        <v>1627</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="952" spans="1:2">
       <c r="A952" s="34" t="s">
-        <v>1628</v>
+        <v>1626</v>
       </c>
       <c r="B952" s="35" t="s">
-        <v>1629</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="953" spans="1:2">
       <c r="A953" s="34" t="s">
-        <v>1630</v>
+        <v>1628</v>
       </c>
       <c r="B953" s="35" t="s">
-        <v>1631</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="954" spans="1:2">
       <c r="A954" s="34" t="s">
-        <v>1632</v>
+        <v>1630</v>
       </c>
       <c r="B954" s="35" t="s">
-        <v>1633</v>
+        <v>1631</v>
       </c>
     </row>
     <row r="955" spans="1:2">
       <c r="A955" s="34" t="s">
-        <v>1634</v>
+        <v>1632</v>
       </c>
       <c r="B955" s="35" t="s">
-        <v>1635</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="956" spans="1:2">
       <c r="A956" s="34" t="s">
-        <v>1636</v>
+        <v>1634</v>
       </c>
       <c r="B956" s="35" t="s">
-        <v>1637</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="957" spans="1:2">
       <c r="A957" s="34" t="s">
-        <v>1638</v>
+        <v>1636</v>
       </c>
       <c r="B957" s="35" t="s">
         <v>1252</v>
@@ -17665,7 +17772,7 @@
     </row>
     <row r="958" spans="1:2">
       <c r="A958" s="34" t="s">
-        <v>1639</v>
+        <v>1637</v>
       </c>
       <c r="B958" s="35" t="s">
         <v>1254</v>
@@ -17673,7 +17780,7 @@
     </row>
     <row r="959" spans="1:2">
       <c r="A959" s="34" t="s">
-        <v>1640</v>
+        <v>1638</v>
       </c>
       <c r="B959" s="35" t="s">
         <v>1256</v>
@@ -17681,7 +17788,7 @@
     </row>
     <row r="960" spans="1:2">
       <c r="A960" s="34" t="s">
-        <v>1641</v>
+        <v>1639</v>
       </c>
       <c r="B960" s="35" t="s">
         <v>1258</v>
@@ -17689,7 +17796,7 @@
     </row>
     <row r="961" spans="1:2">
       <c r="A961" s="34" t="s">
-        <v>1642</v>
+        <v>1640</v>
       </c>
       <c r="B961" s="35" t="s">
         <v>1260</v>
@@ -17697,7 +17804,7 @@
     </row>
     <row r="962" spans="1:2">
       <c r="A962" s="34" t="s">
-        <v>1643</v>
+        <v>1641</v>
       </c>
       <c r="B962" s="35" t="s">
         <v>1262</v>
@@ -17705,7 +17812,7 @@
     </row>
     <row r="963" spans="1:2">
       <c r="A963" s="34" t="s">
-        <v>1644</v>
+        <v>1642</v>
       </c>
       <c r="B963" s="35" t="s">
         <v>1264</v>
@@ -17713,7 +17820,7 @@
     </row>
     <row r="964" spans="1:2">
       <c r="A964" s="34" t="s">
-        <v>1645</v>
+        <v>1643</v>
       </c>
       <c r="B964" s="35" t="s">
         <v>1266</v>
@@ -17721,7 +17828,7 @@
     </row>
     <row r="965" spans="1:2">
       <c r="A965" s="34" t="s">
-        <v>1646</v>
+        <v>1644</v>
       </c>
       <c r="B965" s="35" t="s">
         <v>1268</v>
@@ -17729,7 +17836,7 @@
     </row>
     <row r="966" spans="1:2">
       <c r="A966" s="34" t="s">
-        <v>1647</v>
+        <v>1645</v>
       </c>
       <c r="B966" s="35" t="s">
         <v>563</v>
@@ -17777,7 +17884,7 @@
     </row>
     <row r="972" spans="1:2">
       <c r="A972" s="34" t="s">
-        <v>1648</v>
+        <v>1646</v>
       </c>
       <c r="B972" s="35" t="s">
         <v>406</v>
@@ -17785,7 +17892,7 @@
     </row>
     <row r="973" spans="1:2">
       <c r="A973" s="34" t="s">
-        <v>1649</v>
+        <v>1647</v>
       </c>
       <c r="B973" s="35" t="s">
         <v>316</v>
@@ -17801,15 +17908,15 @@
     </row>
     <row r="975" spans="1:2">
       <c r="A975" s="34" t="s">
-        <v>1650</v>
+        <v>1648</v>
       </c>
       <c r="B975" s="35" t="s">
-        <v>1554</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="976" spans="1:2">
       <c r="A976" s="34" t="s">
-        <v>1651</v>
+        <v>1649</v>
       </c>
       <c r="B976" s="35" t="s">
         <v>319</v>
@@ -17817,7 +17924,7 @@
     </row>
     <row r="977" spans="1:2">
       <c r="A977" s="34" t="s">
-        <v>1652</v>
+        <v>1650</v>
       </c>
       <c r="B977" s="35" t="s">
         <v>409</v>
@@ -17825,15 +17932,15 @@
     </row>
     <row r="978" spans="1:2">
       <c r="A978" s="34" t="s">
-        <v>1653</v>
+        <v>1651</v>
       </c>
       <c r="B978" s="35" t="s">
-        <v>1654</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="979" spans="1:2">
       <c r="A979" s="34" t="s">
-        <v>1655</v>
+        <v>1653</v>
       </c>
       <c r="B979" s="35" t="s">
         <v>117</v>
@@ -17841,7 +17948,7 @@
     </row>
     <row r="980" spans="1:2">
       <c r="A980" s="34" t="s">
-        <v>1656</v>
+        <v>1654</v>
       </c>
       <c r="B980" s="35" t="s">
         <v>453</v>
@@ -17849,7 +17956,7 @@
     </row>
     <row r="981" spans="1:2">
       <c r="A981" s="34" t="s">
-        <v>1657</v>
+        <v>1655</v>
       </c>
       <c r="B981" s="35" t="s">
         <v>41</v>
@@ -17857,15 +17964,15 @@
     </row>
     <row r="982" spans="1:2">
       <c r="A982" s="34" t="s">
-        <v>1658</v>
+        <v>1656</v>
       </c>
       <c r="B982" s="35" t="s">
-        <v>1659</v>
+        <v>1657</v>
       </c>
     </row>
     <row r="983" spans="1:2">
       <c r="A983" s="34" t="s">
-        <v>1660</v>
+        <v>1658</v>
       </c>
       <c r="B983" s="35" t="s">
         <v>237</v>
@@ -17873,23 +17980,23 @@
     </row>
     <row r="984" spans="1:2">
       <c r="A984" s="34" t="s">
-        <v>1661</v>
+        <v>1659</v>
       </c>
       <c r="B984" s="35" t="s">
-        <v>1662</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="985" spans="1:2">
       <c r="A985" s="34" t="s">
-        <v>1663</v>
+        <v>1661</v>
       </c>
       <c r="B985" s="35" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="986" spans="1:2">
       <c r="A986" s="34" t="s">
-        <v>1665</v>
+        <v>1663</v>
       </c>
       <c r="B986" s="35" t="s">
         <v>406</v>
@@ -17897,7 +18004,7 @@
     </row>
     <row r="987" spans="1:2">
       <c r="A987" s="34" t="s">
-        <v>1666</v>
+        <v>1664</v>
       </c>
       <c r="B987" s="35" t="s">
         <v>409</v>
@@ -17905,143 +18012,143 @@
     </row>
     <row r="988" spans="1:2">
       <c r="A988" s="34" t="s">
-        <v>1667</v>
+        <v>1665</v>
       </c>
       <c r="B988" s="35" t="s">
-        <v>1668</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="989" spans="1:2">
       <c r="A989" s="34" t="s">
-        <v>1669</v>
+        <v>1667</v>
       </c>
       <c r="B989" s="35" t="s">
-        <v>1670</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="990" spans="1:2">
       <c r="A990" s="34" t="s">
-        <v>1671</v>
+        <v>1669</v>
       </c>
       <c r="B990" s="35" t="s">
-        <v>1672</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="991" spans="1:2">
       <c r="A991" s="34" t="s">
-        <v>1673</v>
+        <v>1671</v>
       </c>
       <c r="B991" s="35" t="s">
-        <v>1674</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="992" spans="1:2">
       <c r="A992" s="34" t="s">
-        <v>1675</v>
+        <v>1673</v>
       </c>
       <c r="B992" s="35" t="s">
-        <v>1676</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="993" spans="1:2">
       <c r="A993" s="34" t="s">
-        <v>1677</v>
+        <v>1675</v>
       </c>
       <c r="B993" s="35" t="s">
-        <v>1678</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="994" spans="1:2">
       <c r="A994" s="34" t="s">
-        <v>1679</v>
+        <v>1677</v>
       </c>
       <c r="B994" s="35" t="s">
-        <v>1680</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="995" spans="1:2">
       <c r="A995" s="34" t="s">
-        <v>1681</v>
+        <v>1679</v>
       </c>
       <c r="B995" s="35" t="s">
-        <v>1682</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="996" spans="1:2">
       <c r="A996" s="34" t="s">
-        <v>1683</v>
+        <v>1681</v>
       </c>
       <c r="B996" s="35" t="s">
-        <v>1684</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="997" spans="1:2">
       <c r="A997" s="34" t="s">
-        <v>1685</v>
+        <v>1683</v>
       </c>
       <c r="B997" s="35" t="s">
-        <v>1686</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="998" spans="1:2">
       <c r="A998" s="34" t="s">
-        <v>1687</v>
+        <v>1685</v>
       </c>
       <c r="B998" s="35" t="s">
-        <v>1688</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="999" spans="1:2">
       <c r="A999" s="34" t="s">
-        <v>1689</v>
+        <v>1687</v>
       </c>
       <c r="B999" s="35" t="s">
-        <v>1690</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="1000" spans="1:2">
       <c r="A1000" s="34" t="s">
-        <v>1691</v>
+        <v>1689</v>
       </c>
       <c r="B1000" s="35" t="s">
-        <v>1692</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="1001" spans="1:2">
       <c r="A1001" s="34" t="s">
-        <v>1693</v>
+        <v>1691</v>
       </c>
       <c r="B1001" s="35" t="s">
-        <v>1694</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="1002" spans="1:2">
       <c r="A1002" s="34" t="s">
-        <v>1695</v>
+        <v>1693</v>
       </c>
       <c r="B1002" s="35" t="s">
-        <v>1696</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="1003" spans="1:2">
       <c r="A1003" s="34" t="s">
-        <v>1697</v>
+        <v>1695</v>
       </c>
       <c r="B1003" s="35" t="s">
-        <v>1698</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="1004" spans="1:2">
       <c r="A1004" s="34" t="s">
-        <v>1699</v>
+        <v>1697</v>
       </c>
       <c r="B1004" s="35" t="s">
-        <v>1700</v>
+        <v>1698</v>
       </c>
     </row>
     <row r="1005" spans="1:2">
       <c r="A1005" s="34" t="s">
-        <v>1701</v>
+        <v>1699</v>
       </c>
       <c r="B1005" s="35" t="s">
         <v>475</v>
@@ -18049,63 +18156,63 @@
     </row>
     <row r="1006" spans="1:2">
       <c r="A1006" s="34" t="s">
-        <v>1702</v>
+        <v>1700</v>
       </c>
       <c r="B1006" s="35" t="s">
-        <v>1703</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="1007" spans="1:2">
       <c r="A1007" s="34" t="s">
-        <v>1704</v>
+        <v>1702</v>
       </c>
       <c r="B1007" s="35" t="s">
-        <v>1705</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="1008" spans="1:2">
       <c r="A1008" s="34" t="s">
-        <v>1706</v>
+        <v>1704</v>
       </c>
       <c r="B1008" s="35" t="s">
-        <v>1707</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="1009" spans="1:2">
       <c r="A1009" s="34" t="s">
-        <v>1708</v>
+        <v>1706</v>
       </c>
       <c r="B1009" s="35" t="s">
-        <v>1709</v>
+        <v>1707</v>
       </c>
     </row>
     <row r="1010" spans="1:2">
       <c r="A1010" s="34" t="s">
-        <v>1710</v>
+        <v>1708</v>
       </c>
       <c r="B1010" s="35" t="s">
-        <v>1711</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="1011" spans="1:2">
       <c r="A1011" s="34" t="s">
-        <v>1712</v>
+        <v>1710</v>
       </c>
       <c r="B1011" s="35" t="s">
-        <v>1713</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="1012" spans="1:2">
       <c r="A1012" s="34" t="s">
-        <v>1714</v>
+        <v>1712</v>
       </c>
       <c r="B1012" s="35" t="s">
-        <v>1715</v>
+        <v>1713</v>
       </c>
     </row>
     <row r="1013" spans="1:2">
       <c r="A1013" s="34" t="s">
-        <v>1716</v>
+        <v>1714</v>
       </c>
       <c r="B1013" s="35" t="s">
         <v>479</v>
@@ -18113,15 +18220,15 @@
     </row>
     <row r="1014" spans="1:2">
       <c r="A1014" s="34" t="s">
-        <v>1717</v>
+        <v>1715</v>
       </c>
       <c r="B1014" s="35" t="s">
-        <v>1718</v>
+        <v>1716</v>
       </c>
     </row>
     <row r="1015" spans="1:2">
       <c r="A1015" s="34" t="s">
-        <v>1719</v>
+        <v>1717</v>
       </c>
       <c r="B1015" s="35" t="s">
         <v>660</v>
@@ -18129,418 +18236,418 @@
     </row>
     <row r="1016" spans="1:2">
       <c r="A1016" s="34" t="s">
-        <v>1720</v>
+        <v>1718</v>
       </c>
       <c r="B1016" s="35" t="s">
-        <v>1721</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="1017" spans="1:2">
       <c r="A1017" s="34" t="s">
-        <v>1722</v>
+        <v>1720</v>
       </c>
       <c r="B1017" s="35" t="s">
-        <v>1723</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="1018" spans="1:2">
       <c r="A1018" s="34" t="s">
-        <v>1724</v>
+        <v>1722</v>
       </c>
       <c r="B1018" s="35" t="s">
-        <v>1725</v>
+        <v>1723</v>
       </c>
     </row>
     <row r="1019" spans="1:2">
       <c r="A1019" s="34" t="s">
-        <v>1726</v>
+        <v>1724</v>
       </c>
       <c r="B1019" s="35" t="s">
-        <v>1727</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="1020" spans="1:2">
       <c r="A1020" s="34" t="s">
-        <v>1728</v>
+        <v>1726</v>
       </c>
       <c r="B1020" s="35" t="s">
-        <v>1729</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="1021" spans="1:2">
       <c r="A1021" s="34" t="s">
-        <v>1730</v>
+        <v>1728</v>
       </c>
       <c r="B1021" s="35" t="s">
-        <v>1731</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="1022" spans="1:2">
       <c r="A1022" s="34" t="s">
-        <v>1732</v>
+        <v>1730</v>
       </c>
       <c r="B1022" s="35" t="s">
-        <v>1733</v>
+        <v>1731</v>
       </c>
     </row>
     <row r="1023" spans="1:2">
       <c r="A1023" s="34" t="s">
-        <v>1734</v>
+        <v>1732</v>
       </c>
       <c r="B1023" s="35" t="s">
-        <v>1735</v>
+        <v>1733</v>
       </c>
     </row>
     <row r="1024" spans="1:2">
       <c r="A1024" s="34" t="s">
-        <v>1736</v>
+        <v>1734</v>
       </c>
       <c r="B1024" s="35" t="s">
-        <v>1737</v>
+        <v>1735</v>
       </c>
     </row>
     <row r="1025" spans="1:2">
       <c r="A1025" s="34" t="s">
-        <v>1738</v>
+        <v>1736</v>
       </c>
       <c r="B1025" s="35" t="s">
-        <v>1739</v>
+        <v>1737</v>
       </c>
     </row>
     <row r="1026" spans="1:2">
       <c r="A1026" s="34" t="s">
-        <v>1740</v>
+        <v>1738</v>
       </c>
       <c r="B1026" s="35" t="s">
-        <v>1741</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="1027" spans="1:2">
       <c r="A1027" s="34" t="s">
-        <v>1742</v>
+        <v>1740</v>
       </c>
       <c r="B1027" s="35" t="s">
-        <v>1743</v>
+        <v>1741</v>
       </c>
     </row>
     <row r="1028" spans="1:2">
       <c r="A1028" s="34" t="s">
-        <v>1744</v>
+        <v>1742</v>
       </c>
       <c r="B1028" s="35" t="s">
-        <v>1745</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="1029" spans="1:2">
       <c r="A1029" s="34" t="s">
-        <v>1746</v>
+        <v>1744</v>
       </c>
       <c r="B1029" s="35" t="s">
-        <v>1747</v>
+        <v>1745</v>
       </c>
     </row>
     <row r="1030" spans="1:2">
       <c r="A1030" s="34" t="s">
-        <v>1748</v>
+        <v>1746</v>
       </c>
       <c r="B1030" s="35" t="s">
-        <v>1749</v>
+        <v>1747</v>
       </c>
     </row>
     <row r="1031" spans="1:2">
       <c r="A1031" s="34" t="s">
-        <v>1750</v>
+        <v>1748</v>
       </c>
       <c r="B1031" s="35" t="s">
-        <v>1751</v>
+        <v>1749</v>
       </c>
     </row>
     <row r="1032" spans="1:2">
       <c r="A1032" s="34" t="s">
-        <v>1752</v>
+        <v>1750</v>
       </c>
       <c r="B1032" s="35" t="s">
-        <v>1583</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="1033" spans="1:2">
       <c r="A1033" s="34" t="s">
-        <v>1753</v>
+        <v>1751</v>
       </c>
       <c r="B1033" s="35" t="s">
-        <v>1754</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="1034" spans="1:2">
       <c r="A1034" s="34" t="s">
-        <v>1755</v>
+        <v>1753</v>
       </c>
       <c r="B1034" s="35" t="s">
-        <v>1756</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="1035" spans="1:2">
       <c r="A1035" s="34" t="s">
-        <v>1757</v>
+        <v>1755</v>
       </c>
       <c r="B1035" s="35" t="s">
-        <v>1758</v>
+        <v>1756</v>
       </c>
     </row>
     <row r="1036" spans="1:2">
       <c r="A1036" s="34" t="s">
-        <v>1759</v>
+        <v>1757</v>
       </c>
       <c r="B1036" s="35" t="s">
-        <v>1759</v>
+        <v>1757</v>
       </c>
     </row>
     <row r="1037" spans="1:2">
       <c r="A1037" s="34" t="s">
-        <v>1760</v>
+        <v>1758</v>
       </c>
       <c r="B1037" s="35" t="s">
-        <v>1761</v>
+        <v>1759</v>
       </c>
     </row>
     <row r="1038" spans="1:2">
       <c r="A1038" s="34" t="s">
-        <v>1762</v>
+        <v>1760</v>
       </c>
       <c r="B1038" s="35" t="s">
-        <v>1763</v>
+        <v>1761</v>
       </c>
     </row>
     <row r="1039" spans="1:2">
       <c r="A1039" s="34" t="s">
-        <v>1764</v>
+        <v>1762</v>
       </c>
       <c r="B1039" s="35" t="s">
-        <v>1765</v>
+        <v>1763</v>
       </c>
     </row>
     <row r="1040" spans="1:2">
       <c r="A1040" s="34" t="s">
-        <v>1766</v>
+        <v>1764</v>
       </c>
       <c r="B1040" s="35" t="s">
-        <v>1767</v>
+        <v>1765</v>
       </c>
     </row>
     <row r="1041" spans="1:2">
       <c r="A1041" s="34" t="s">
-        <v>1768</v>
+        <v>1766</v>
       </c>
       <c r="B1041" s="35" t="s">
-        <v>1769</v>
+        <v>1767</v>
       </c>
     </row>
     <row r="1042" spans="1:2">
       <c r="A1042" s="34" t="s">
-        <v>1770</v>
+        <v>1768</v>
       </c>
       <c r="B1042" s="35" t="s">
-        <v>1771</v>
+        <v>1769</v>
       </c>
     </row>
     <row r="1043" spans="1:2">
       <c r="A1043" s="34" t="s">
-        <v>1772</v>
+        <v>1770</v>
       </c>
       <c r="B1043" s="35" t="s">
-        <v>1773</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="1044" spans="1:2">
       <c r="A1044" s="34" t="s">
-        <v>1774</v>
+        <v>1772</v>
       </c>
       <c r="B1044" s="35" t="s">
-        <v>1775</v>
+        <v>1773</v>
       </c>
     </row>
     <row r="1045" spans="1:2">
       <c r="A1045" s="34" t="s">
-        <v>1776</v>
+        <v>1774</v>
       </c>
       <c r="B1045" s="35" t="s">
-        <v>1777</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="1046" spans="1:2">
       <c r="A1046" s="34" t="s">
-        <v>1778</v>
+        <v>1776</v>
       </c>
       <c r="B1046" s="35" t="s">
-        <v>1779</v>
+        <v>1777</v>
       </c>
     </row>
     <row r="1047" spans="1:2">
       <c r="A1047" s="34" t="s">
-        <v>1780</v>
+        <v>1778</v>
       </c>
       <c r="B1047" s="35" t="s">
-        <v>1781</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="1048" spans="1:2">
       <c r="A1048" s="34" t="s">
-        <v>1782</v>
+        <v>1780</v>
       </c>
       <c r="B1048" s="35" t="s">
-        <v>1783</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="1049" spans="1:2">
       <c r="A1049" s="34" t="s">
-        <v>1784</v>
-      </c>
-      <c r="B1049" s="69" t="s">
-        <v>1785</v>
+        <v>1782</v>
+      </c>
+      <c r="B1049" s="68" t="s">
+        <v>1783</v>
       </c>
     </row>
     <row r="1050" spans="1:2">
       <c r="A1050" s="34" t="s">
-        <v>1786</v>
+        <v>1784</v>
       </c>
       <c r="B1050" s="35" t="s">
-        <v>1787</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="1051" spans="1:2">
       <c r="A1051" s="34" t="s">
-        <v>1788</v>
+        <v>1786</v>
       </c>
       <c r="B1051" s="35" t="s">
-        <v>1758</v>
+        <v>1756</v>
       </c>
     </row>
     <row r="1052" spans="1:2">
       <c r="A1052" s="34" t="s">
-        <v>1789</v>
+        <v>1787</v>
       </c>
       <c r="B1052" s="35" t="s">
-        <v>1790</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="1053" spans="1:2">
       <c r="A1053" s="34" t="s">
-        <v>1791</v>
+        <v>1789</v>
       </c>
       <c r="B1053" s="35" t="s">
-        <v>1791</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="1054" spans="1:2">
       <c r="A1054" s="34" t="s">
-        <v>1792</v>
+        <v>1790</v>
       </c>
       <c r="B1054" s="35" t="s">
-        <v>1793</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="1055" spans="1:2">
       <c r="A1055" s="34" t="s">
-        <v>1794</v>
+        <v>1792</v>
       </c>
       <c r="B1055" s="35" t="s">
-        <v>1795</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="1056" spans="1:2">
       <c r="A1056" s="34" t="s">
-        <v>1796</v>
+        <v>1794</v>
       </c>
       <c r="B1056" s="35" t="s">
-        <v>1797</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="1057" spans="1:2">
       <c r="A1057" s="34" t="s">
-        <v>1798</v>
+        <v>1796</v>
       </c>
       <c r="B1057" s="35" t="s">
-        <v>1799</v>
+        <v>1797</v>
       </c>
     </row>
     <row r="1058" spans="1:2">
       <c r="A1058" s="34" t="s">
-        <v>1800</v>
+        <v>1798</v>
       </c>
       <c r="B1058" s="35" t="s">
-        <v>1801</v>
+        <v>1799</v>
       </c>
     </row>
     <row r="1059" spans="1:2">
       <c r="A1059" s="34" t="s">
-        <v>1802</v>
+        <v>1800</v>
       </c>
       <c r="B1059" s="35" t="s">
-        <v>1803</v>
+        <v>1801</v>
       </c>
     </row>
     <row r="1060" spans="1:2">
       <c r="A1060" s="34" t="s">
-        <v>1804</v>
+        <v>1802</v>
       </c>
       <c r="B1060" s="35" t="s">
-        <v>1805</v>
+        <v>1803</v>
       </c>
     </row>
     <row r="1061" spans="1:2">
       <c r="A1061" s="34" t="s">
-        <v>1806</v>
+        <v>1804</v>
       </c>
       <c r="B1061" s="35" t="s">
-        <v>1807</v>
+        <v>1805</v>
       </c>
     </row>
     <row r="1062" spans="1:2">
       <c r="A1062" s="34" t="s">
-        <v>1808</v>
+        <v>1806</v>
       </c>
       <c r="B1062" s="35" t="s">
-        <v>1808</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="1063" spans="1:2">
       <c r="A1063" s="34" t="s">
-        <v>1809</v>
+        <v>1807</v>
       </c>
       <c r="B1063" s="35" t="s">
-        <v>1810</v>
+        <v>1808</v>
       </c>
     </row>
     <row r="1064" spans="1:2">
       <c r="A1064" s="34" t="s">
-        <v>1811</v>
+        <v>1809</v>
       </c>
       <c r="B1064" s="35" t="s">
-        <v>1812</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="1065" spans="1:2">
       <c r="A1065" s="34" t="s">
-        <v>1813</v>
+        <v>1811</v>
       </c>
       <c r="B1065" s="35" t="s">
-        <v>1814</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="1066" spans="1:2">
       <c r="A1066" s="34" t="s">
-        <v>1815</v>
+        <v>1813</v>
       </c>
       <c r="B1066" s="35" t="s">
-        <v>1816</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="1067" spans="1:2">
       <c r="A1067" s="34" t="s">
-        <v>1817</v>
+        <v>1815</v>
       </c>
       <c r="B1067" s="35" t="s">
-        <v>1818</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="1068" spans="1:2">
@@ -18572,12 +18679,12 @@
         <v>1506</v>
       </c>
       <c r="B1071" s="34" t="s">
-        <v>1819</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="1072" spans="1:2">
       <c r="A1072" s="34" t="s">
-        <v>1820</v>
+        <v>1818</v>
       </c>
       <c r="B1072" s="35" t="s">
         <v>59</v>
@@ -18585,63 +18692,63 @@
     </row>
     <row r="1073" spans="1:2">
       <c r="A1073" s="34" t="s">
-        <v>1821</v>
+        <v>1819</v>
       </c>
       <c r="B1073" s="35" t="s">
-        <v>1822</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="1074" spans="1:2">
       <c r="A1074" s="34" t="s">
-        <v>1823</v>
+        <v>1821</v>
       </c>
       <c r="B1074" s="35" t="s">
-        <v>1824</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="1075" spans="1:2">
       <c r="A1075" s="34" t="s">
-        <v>1825</v>
+        <v>1823</v>
       </c>
       <c r="B1075" s="35" t="s">
-        <v>1826</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="1076" spans="1:2">
       <c r="A1076" s="34" t="s">
-        <v>1827</v>
+        <v>1825</v>
       </c>
       <c r="B1076" s="35" t="s">
-        <v>1828</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="1077" spans="1:2">
       <c r="A1077" s="34" t="s">
-        <v>1829</v>
+        <v>1827</v>
       </c>
       <c r="B1077" s="35" t="s">
-        <v>1830</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="1078" spans="1:2">
       <c r="A1078" s="34" t="s">
-        <v>1831</v>
+        <v>1829</v>
       </c>
       <c r="B1078" s="35" t="s">
-        <v>1832</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="1079" spans="1:2">
       <c r="A1079" s="34" t="s">
-        <v>1833</v>
+        <v>1831</v>
       </c>
       <c r="B1079" s="35" t="s">
-        <v>1834</v>
+        <v>1832</v>
       </c>
     </row>
     <row r="1080" spans="1:2">
       <c r="A1080" s="34" t="s">
-        <v>1835</v>
+        <v>1833</v>
       </c>
       <c r="B1080" s="35" t="s">
         <v>858</v>
@@ -18649,71 +18756,71 @@
     </row>
     <row r="1081" spans="1:2">
       <c r="A1081" s="34" t="s">
-        <v>1836</v>
+        <v>1834</v>
       </c>
       <c r="B1081" s="35" t="s">
-        <v>1664</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="1082" spans="1:2">
       <c r="A1082" s="34" t="s">
-        <v>1837</v>
+        <v>1835</v>
       </c>
       <c r="B1082" s="35" t="s">
-        <v>1838</v>
+        <v>1836</v>
       </c>
     </row>
     <row r="1083" spans="1:2">
       <c r="A1083" s="34" t="s">
-        <v>1839</v>
+        <v>1837</v>
       </c>
       <c r="B1083" s="35" t="s">
-        <v>1840</v>
+        <v>1838</v>
       </c>
     </row>
     <row r="1084" spans="1:2">
       <c r="A1084" s="34" t="s">
-        <v>1841</v>
+        <v>1839</v>
       </c>
       <c r="B1084" s="35" t="s">
-        <v>1842</v>
+        <v>1840</v>
       </c>
     </row>
     <row r="1085" spans="1:2">
       <c r="A1085" s="34" t="s">
-        <v>1843</v>
+        <v>1841</v>
       </c>
       <c r="B1085" s="35" t="s">
-        <v>1844</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="1086" spans="1:2">
       <c r="A1086" s="34" t="s">
-        <v>1845</v>
+        <v>1843</v>
       </c>
       <c r="B1086" s="35" t="s">
-        <v>1846</v>
+        <v>1844</v>
       </c>
     </row>
     <row r="1087" spans="1:2">
       <c r="A1087" s="34" t="s">
-        <v>1847</v>
+        <v>1845</v>
       </c>
       <c r="B1087" s="35" t="s">
-        <v>1848</v>
+        <v>1846</v>
       </c>
     </row>
     <row r="1088" spans="1:2">
       <c r="A1088" s="34" t="s">
-        <v>1849</v>
+        <v>1847</v>
       </c>
       <c r="B1088" s="35" t="s">
-        <v>1850</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="1089" spans="1:2">
       <c r="A1089" s="34" t="s">
-        <v>1851</v>
+        <v>1849</v>
       </c>
       <c r="B1089" s="35" t="s">
         <v>479</v>
@@ -18721,39 +18828,39 @@
     </row>
     <row r="1090" spans="1:2">
       <c r="A1090" s="34" t="s">
-        <v>1852</v>
+        <v>1850</v>
       </c>
       <c r="B1090" s="35" t="s">
-        <v>1853</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="1091" spans="1:2">
       <c r="A1091" s="34" t="s">
-        <v>1854</v>
+        <v>1852</v>
       </c>
       <c r="B1091" s="35" t="s">
-        <v>1855</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="1092" spans="1:2">
       <c r="A1092" s="34" t="s">
-        <v>1856</v>
+        <v>1854</v>
       </c>
       <c r="B1092" s="35" t="s">
-        <v>1857</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="1093" spans="1:2">
       <c r="A1093" s="34" t="s">
-        <v>1858</v>
+        <v>1856</v>
       </c>
       <c r="B1093" s="35" t="s">
-        <v>1859</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="1094" spans="1:2">
       <c r="A1094" s="34" t="s">
-        <v>1860</v>
+        <v>1858</v>
       </c>
       <c r="B1094" s="35" t="s">
         <v>636</v>
@@ -18761,55 +18868,55 @@
     </row>
     <row r="1095" spans="1:2">
       <c r="A1095" s="34" t="s">
-        <v>1861</v>
+        <v>1859</v>
       </c>
       <c r="B1095" s="35" t="s">
-        <v>1862</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="1096" spans="1:2">
       <c r="A1096" s="34" t="s">
-        <v>1863</v>
+        <v>1861</v>
       </c>
       <c r="B1096" s="35" t="s">
-        <v>1763</v>
+        <v>1761</v>
       </c>
     </row>
     <row r="1097" spans="1:2">
       <c r="A1097" s="34" t="s">
-        <v>1864</v>
+        <v>1862</v>
       </c>
       <c r="B1097" s="35" t="s">
-        <v>1865</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="1098" spans="1:2">
       <c r="A1098" s="34" t="s">
-        <v>1866</v>
+        <v>1864</v>
       </c>
       <c r="B1098" s="35" t="s">
-        <v>1867</v>
+        <v>1865</v>
       </c>
     </row>
     <row r="1099" spans="1:2">
       <c r="A1099" s="34" t="s">
-        <v>1868</v>
+        <v>1866</v>
       </c>
       <c r="B1099" s="35" t="s">
-        <v>1869</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="1100" spans="1:2">
       <c r="A1100" s="34" t="s">
-        <v>1870</v>
+        <v>1868</v>
       </c>
       <c r="B1100" s="35" t="s">
-        <v>1871</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="1101" spans="1:2">
       <c r="A1101" s="34" t="s">
-        <v>1872</v>
+        <v>1870</v>
       </c>
       <c r="B1101" s="35" t="s">
         <v>688</v>
@@ -18817,15 +18924,15 @@
     </row>
     <row r="1102" spans="1:2">
       <c r="A1102" s="34" t="s">
-        <v>1873</v>
+        <v>1871</v>
       </c>
       <c r="B1102" s="35" t="s">
-        <v>1874</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="1103" spans="1:2">
       <c r="A1103" s="34" t="s">
-        <v>1875</v>
+        <v>1873</v>
       </c>
       <c r="B1103" s="35" t="s">
         <v>929</v>
@@ -18833,7 +18940,7 @@
     </row>
     <row r="1104" spans="1:2">
       <c r="A1104" s="34" t="s">
-        <v>1876</v>
+        <v>1874</v>
       </c>
       <c r="B1104" s="35" t="s">
         <v>925</v>
@@ -18841,7 +18948,7 @@
     </row>
     <row r="1105" spans="1:2">
       <c r="A1105" s="34" t="s">
-        <v>1877</v>
+        <v>1875</v>
       </c>
       <c r="B1105" s="35" t="s">
         <v>927</v>
@@ -18849,34 +18956,34 @@
     </row>
     <row r="1106" spans="1:2">
       <c r="A1106" s="34" t="s">
-        <v>1878</v>
+        <v>1876</v>
       </c>
       <c r="B1106" s="35" t="s">
-        <v>1879</v>
+        <v>1877</v>
       </c>
     </row>
     <row r="1107" spans="1:2">
       <c r="A1107" s="34" t="s">
-        <v>1880</v>
+        <v>1878</v>
       </c>
       <c r="B1107" s="35" t="s">
-        <v>1881</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="1108" spans="1:2">
       <c r="A1108" s="34" t="s">
-        <v>1882</v>
+        <v>1880</v>
       </c>
       <c r="B1108" s="35" t="s">
-        <v>1883</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="1109" spans="1:2">
       <c r="A1109" s="34" t="s">
-        <v>1884</v>
+        <v>1882</v>
       </c>
       <c r="B1109" s="35" t="s">
-        <v>1885</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="1110" spans="1:2">
@@ -18889,34 +18996,34 @@
     </row>
     <row r="1111" spans="1:2">
       <c r="A1111" s="34" t="s">
-        <v>1573</v>
+        <v>1571</v>
       </c>
       <c r="B1111" s="34" t="s">
-        <v>1886</v>
+        <v>1884</v>
       </c>
     </row>
     <row r="1112" spans="1:2">
       <c r="A1112" s="47" t="s">
-        <v>1887</v>
+        <v>1885</v>
       </c>
       <c r="B1112" s="35" t="s">
-        <v>1888</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="1113" spans="1:2">
       <c r="A1113" s="47" t="s">
-        <v>1889</v>
+        <v>1887</v>
       </c>
       <c r="B1113" s="35" t="s">
-        <v>1890</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="1114" spans="1:2">
       <c r="A1114" s="47" t="s">
-        <v>1891</v>
+        <v>1889</v>
       </c>
       <c r="B1114" s="35" t="s">
-        <v>1892</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="1115" spans="1:2">
@@ -18924,7 +19031,7 @@
         <v>615</v>
       </c>
       <c r="B1115" s="35" t="s">
-        <v>1893</v>
+        <v>1891</v>
       </c>
     </row>
     <row r="1116" spans="1:2">
@@ -19217,10 +19324,10 @@
     </row>
     <row r="1152" spans="1:2">
       <c r="A1152" s="34" t="s">
-        <v>1894</v>
+        <v>1892</v>
       </c>
       <c r="B1152" s="35" t="s">
-        <v>1895</v>
+        <v>1893</v>
       </c>
     </row>
     <row r="1153" spans="1:2">
@@ -19345,23 +19452,23 @@
     </row>
     <row r="1168" spans="1:2">
       <c r="A1168" s="34" t="s">
-        <v>1896</v>
+        <v>1894</v>
       </c>
       <c r="B1168" s="35" t="s">
-        <v>1897</v>
+        <v>1895</v>
       </c>
     </row>
     <row r="1169" spans="1:2">
       <c r="A1169" s="34" t="s">
-        <v>1898</v>
+        <v>1896</v>
       </c>
       <c r="B1169" s="35" t="s">
-        <v>1899</v>
+        <v>1897</v>
       </c>
     </row>
     <row r="1170" spans="1:2">
       <c r="A1170" s="34" t="s">
-        <v>1900</v>
+        <v>1898</v>
       </c>
       <c r="B1170" s="35" t="s">
         <v>560</v>
@@ -19369,39 +19476,39 @@
     </row>
     <row r="1171" spans="1:2">
       <c r="A1171" s="34" t="s">
-        <v>1901</v>
+        <v>1899</v>
       </c>
       <c r="B1171" s="35" t="s">
-        <v>1902</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="1172" spans="1:2">
       <c r="A1172" s="34" t="s">
-        <v>1903</v>
+        <v>1901</v>
       </c>
       <c r="B1172" s="35" t="s">
-        <v>1904</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="1173" spans="1:2">
       <c r="A1173" s="34" t="s">
-        <v>1905</v>
+        <v>1903</v>
       </c>
       <c r="B1173" s="35" t="s">
-        <v>1906</v>
+        <v>1904</v>
       </c>
     </row>
     <row r="1174" spans="1:2">
       <c r="A1174" s="34" t="s">
-        <v>1907</v>
-      </c>
-      <c r="B1174" s="69" t="s">
-        <v>1908</v>
+        <v>1905</v>
+      </c>
+      <c r="B1174" s="68" t="s">
+        <v>1906</v>
       </c>
     </row>
     <row r="1175" spans="1:2">
       <c r="A1175" s="34" t="s">
-        <v>1909</v>
+        <v>1907</v>
       </c>
       <c r="B1175" s="34" t="s">
         <v>59</v>
@@ -19409,50 +19516,50 @@
     </row>
     <row r="1176" spans="1:2">
       <c r="A1176" s="34" t="s">
-        <v>1910</v>
+        <v>1908</v>
       </c>
       <c r="B1176" s="34" t="s">
-        <v>1911</v>
+        <v>1909</v>
       </c>
     </row>
     <row r="1177" spans="1:2">
       <c r="A1177" s="34" t="s">
-        <v>1912</v>
+        <v>1910</v>
       </c>
       <c r="B1177" s="35" t="s">
-        <v>1913</v>
+        <v>1911</v>
       </c>
     </row>
     <row r="1178" spans="1:2">
       <c r="A1178" s="34" t="s">
-        <v>1914</v>
-      </c>
-      <c r="B1178" s="69" t="s">
+        <v>1912</v>
+      </c>
+      <c r="B1178" s="68" t="s">
         <v>1495</v>
       </c>
     </row>
     <row r="1179" spans="1:2">
       <c r="A1179" s="34" t="s">
-        <v>1915</v>
-      </c>
-      <c r="B1179" s="69" t="s">
+        <v>1913</v>
+      </c>
+      <c r="B1179" s="68" t="s">
         <v>306</v>
       </c>
     </row>
     <row r="1180" spans="1:2">
       <c r="A1180" s="34" t="s">
-        <v>1916</v>
-      </c>
-      <c r="B1180" s="70" t="s">
-        <v>1917</v>
+        <v>1914</v>
+      </c>
+      <c r="B1180" s="69" t="s">
+        <v>1915</v>
       </c>
     </row>
     <row r="1181" spans="1:2">
       <c r="A1181" s="34" t="s">
-        <v>1918</v>
+        <v>1916</v>
       </c>
       <c r="B1181" s="35" t="s">
-        <v>1919</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="1182" spans="1:2">
@@ -19521,7 +19628,7 @@
     </row>
     <row r="1190" spans="1:2">
       <c r="A1190" s="34" t="s">
-        <v>1920</v>
+        <v>1918</v>
       </c>
       <c r="B1190" s="35" t="s">
         <v>1365</v>
@@ -19529,7 +19636,7 @@
     </row>
     <row r="1191" spans="1:2">
       <c r="A1191" s="34" t="s">
-        <v>1921</v>
+        <v>1919</v>
       </c>
       <c r="B1191" s="35" t="s">
         <v>1367</v>
@@ -19537,58 +19644,58 @@
     </row>
     <row r="1192" spans="1:2">
       <c r="A1192" s="34" t="s">
-        <v>1922</v>
+        <v>1920</v>
       </c>
       <c r="B1192" s="35" t="s">
-        <v>1923</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="1193" spans="1:2">
       <c r="A1193" s="34" t="s">
-        <v>1924</v>
+        <v>1922</v>
       </c>
       <c r="B1193" s="35" t="s">
-        <v>1925</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="1194" spans="1:2">
       <c r="A1194" s="34" t="s">
-        <v>1926</v>
+        <v>1924</v>
       </c>
       <c r="B1194" s="35" t="s">
-        <v>1927</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="1195" spans="1:2">
       <c r="A1195" s="34" t="s">
-        <v>1928</v>
+        <v>1926</v>
       </c>
       <c r="B1195" s="35" t="s">
-        <v>1929</v>
+        <v>1927</v>
       </c>
     </row>
     <row r="1196" spans="1:2">
       <c r="A1196" s="34" t="s">
-        <v>1930</v>
+        <v>1928</v>
       </c>
       <c r="B1196" s="35" t="s">
-        <v>1930</v>
+        <v>1928</v>
       </c>
     </row>
     <row r="1197" spans="1:2">
       <c r="A1197" s="34" t="s">
-        <v>1931</v>
+        <v>1929</v>
       </c>
       <c r="B1197" s="35" t="s">
-        <v>1931</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="1198" spans="1:2">
       <c r="A1198" s="34" t="s">
-        <v>1932</v>
+        <v>1930</v>
       </c>
       <c r="B1198" s="35" t="s">
-        <v>1932</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="1199" spans="1:2">
@@ -19649,26 +19756,26 @@
     </row>
     <row r="1206" spans="1:2">
       <c r="A1206" s="34" t="s">
-        <v>1933</v>
+        <v>1931</v>
       </c>
       <c r="B1206" s="35" t="s">
-        <v>1934</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="1207" spans="1:2">
       <c r="A1207" s="34" t="s">
-        <v>1935</v>
+        <v>1933</v>
       </c>
       <c r="B1207" s="35" t="s">
-        <v>1936</v>
+        <v>1934</v>
       </c>
     </row>
     <row r="1208" spans="1:2">
       <c r="A1208" s="34" t="s">
-        <v>1937</v>
+        <v>1935</v>
       </c>
       <c r="B1208" s="35" t="s">
-        <v>1938</v>
+        <v>1936</v>
       </c>
     </row>
     <row r="1209" spans="1:2">
@@ -19689,50 +19796,50 @@
     </row>
     <row r="1211" spans="1:2">
       <c r="A1211" s="34" t="s">
-        <v>1939</v>
+        <v>1937</v>
       </c>
       <c r="B1211" s="34" t="s">
-        <v>1940</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="1212" spans="1:2">
       <c r="A1212" s="34" t="s">
-        <v>1941</v>
-      </c>
-      <c r="B1212" s="70" t="s">
-        <v>1942</v>
+        <v>1939</v>
+      </c>
+      <c r="B1212" s="69" t="s">
+        <v>1940</v>
       </c>
     </row>
     <row r="1213" spans="1:2">
       <c r="A1213" s="34" t="s">
-        <v>1943</v>
-      </c>
-      <c r="B1213" s="71" t="s">
+        <v>1941</v>
+      </c>
+      <c r="B1213" s="70" t="s">
         <v>917</v>
       </c>
     </row>
     <row r="1214" spans="1:2">
       <c r="A1214" s="34" t="s">
-        <v>1944</v>
-      </c>
-      <c r="B1214" s="71" t="s">
+        <v>1942</v>
+      </c>
+      <c r="B1214" s="70" t="s">
         <v>1413</v>
       </c>
     </row>
     <row r="1215" spans="1:2">
       <c r="A1215" s="34" t="s">
-        <v>1945</v>
+        <v>1943</v>
       </c>
       <c r="B1215" s="35" t="s">
-        <v>1946</v>
+        <v>1944</v>
       </c>
     </row>
     <row r="1216" spans="1:2">
       <c r="A1216" s="34" t="s">
-        <v>1947</v>
+        <v>1945</v>
       </c>
       <c r="B1216" s="35" t="s">
-        <v>1946</v>
+        <v>1944</v>
       </c>
     </row>
     <row r="1217" spans="1:2">
@@ -19745,42 +19852,42 @@
     </row>
     <row r="1218" spans="1:2">
       <c r="A1218" s="34" t="s">
-        <v>1564</v>
+        <v>1562</v>
       </c>
       <c r="B1218" s="35" t="s">
-        <v>1948</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="1219" spans="1:2">
       <c r="A1219" s="34" t="s">
-        <v>1566</v>
+        <v>1564</v>
       </c>
       <c r="B1219" s="35" t="s">
-        <v>1948</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="1220" spans="1:2">
       <c r="A1220" s="34" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="B1220" s="35" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="1221" spans="1:2">
       <c r="A1221" s="34" t="s">
-        <v>1569</v>
+        <v>1567</v>
       </c>
       <c r="B1221" s="35" t="s">
-        <v>1569</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="1222" spans="1:2">
       <c r="A1222" s="34" t="s">
-        <v>1570</v>
+        <v>1568</v>
       </c>
       <c r="B1222" s="35" t="s">
-        <v>1570</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="1223" spans="1:2">
@@ -19793,15 +19900,15 @@
     </row>
     <row r="1224" spans="1:2">
       <c r="A1224" s="34" t="s">
-        <v>1949</v>
+        <v>1947</v>
       </c>
       <c r="B1224" s="34" t="s">
-        <v>1857</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="1225" spans="1:2">
       <c r="A1225" s="34" t="s">
-        <v>1950</v>
+        <v>1948</v>
       </c>
       <c r="B1225" s="35" t="s">
         <v>563</v>
@@ -19809,127 +19916,127 @@
     </row>
     <row r="1226" spans="1:2">
       <c r="A1226" s="34" t="s">
-        <v>1951</v>
+        <v>1949</v>
       </c>
       <c r="B1226" s="35" t="s">
-        <v>1952</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="1227" spans="1:2">
       <c r="A1227" s="34" t="s">
-        <v>1953</v>
+        <v>1951</v>
       </c>
       <c r="B1227" s="35" t="s">
-        <v>1954</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="1228" spans="1:2">
       <c r="A1228" s="34" t="s">
-        <v>1955</v>
+        <v>1953</v>
       </c>
       <c r="B1228" s="35" t="s">
-        <v>1956</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="1229" spans="1:2">
       <c r="A1229" s="34" t="s">
-        <v>1957</v>
+        <v>1955</v>
       </c>
       <c r="B1229" s="35" t="s">
-        <v>1801</v>
+        <v>1799</v>
       </c>
     </row>
     <row r="1230" spans="1:2">
       <c r="A1230" s="34" t="s">
-        <v>1958</v>
+        <v>1956</v>
       </c>
       <c r="B1230" s="35" t="s">
-        <v>1902</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="1231" spans="1:2">
       <c r="A1231" s="34" t="s">
-        <v>1959</v>
+        <v>1957</v>
       </c>
       <c r="B1231" s="35" t="s">
-        <v>1960</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="1232" spans="1:2">
       <c r="A1232" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B1232" s="69" t="s">
+      <c r="B1232" s="68" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="1233" spans="1:2">
       <c r="A1233" s="34" t="s">
-        <v>1961</v>
-      </c>
-      <c r="B1233" s="69" t="s">
-        <v>1962</v>
+        <v>1959</v>
+      </c>
+      <c r="B1233" s="68" t="s">
+        <v>1960</v>
       </c>
     </row>
     <row r="1234" spans="1:2">
       <c r="A1234" s="34" t="s">
-        <v>1963</v>
-      </c>
-      <c r="B1234" s="69" t="s">
-        <v>1964</v>
+        <v>1961</v>
+      </c>
+      <c r="B1234" s="68" t="s">
+        <v>1962</v>
       </c>
     </row>
     <row r="1235" spans="1:2">
       <c r="A1235" s="34" t="s">
-        <v>1965</v>
+        <v>1963</v>
       </c>
       <c r="B1235" s="35" t="s">
-        <v>1966</v>
+        <v>1964</v>
       </c>
     </row>
     <row r="1236" spans="1:2">
       <c r="A1236" s="34" t="s">
-        <v>1967</v>
+        <v>1965</v>
       </c>
       <c r="B1236" s="35" t="s">
-        <v>1968</v>
+        <v>1966</v>
       </c>
     </row>
     <row r="1237" spans="1:2">
       <c r="A1237" s="34" t="s">
-        <v>1969</v>
+        <v>1967</v>
       </c>
       <c r="B1237" s="35" t="s">
-        <v>1970</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="1238" spans="1:2">
       <c r="A1238" s="34" t="s">
-        <v>1971</v>
+        <v>1969</v>
       </c>
       <c r="B1238" s="35" t="s">
-        <v>1972</v>
+        <v>1970</v>
       </c>
     </row>
     <row r="1239" spans="1:2">
       <c r="A1239" s="34" t="s">
-        <v>1973</v>
+        <v>1971</v>
       </c>
       <c r="B1239" s="35" t="s">
-        <v>1972</v>
+        <v>1970</v>
       </c>
     </row>
     <row r="1240" spans="1:2">
       <c r="A1240" s="34" t="s">
-        <v>1974</v>
+        <v>1972</v>
       </c>
       <c r="B1240" s="35" t="s">
-        <v>1975</v>
+        <v>1973</v>
       </c>
     </row>
     <row r="1241" spans="1:2">
       <c r="A1241" s="34" t="s">
-        <v>1976</v>
+        <v>1974</v>
       </c>
       <c r="B1241" s="35" t="s">
         <v>388</v>
@@ -19937,119 +20044,119 @@
     </row>
     <row r="1242" spans="1:2">
       <c r="A1242" s="34" t="s">
-        <v>1977</v>
+        <v>1975</v>
       </c>
       <c r="B1242" s="35" t="s">
-        <v>1978</v>
+        <v>1976</v>
       </c>
     </row>
     <row r="1243" spans="1:2">
       <c r="A1243" s="34" t="s">
-        <v>1979</v>
+        <v>1977</v>
       </c>
       <c r="B1243" s="35" t="s">
-        <v>1980</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="1244" spans="1:2">
       <c r="A1244" s="34" t="s">
-        <v>1981</v>
+        <v>1979</v>
       </c>
       <c r="B1244" s="35" t="s">
-        <v>1982</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="1245" spans="1:2">
       <c r="A1245" s="34" t="s">
-        <v>1983</v>
+        <v>1981</v>
       </c>
       <c r="B1245" s="35" t="s">
-        <v>1984</v>
+        <v>1982</v>
       </c>
     </row>
     <row r="1246" spans="1:2">
       <c r="A1246" s="34" t="s">
-        <v>1985</v>
+        <v>1983</v>
       </c>
       <c r="B1246" s="35" t="s">
-        <v>1917</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="1247" spans="1:2">
       <c r="A1247" s="34" t="s">
-        <v>1961</v>
+        <v>1959</v>
       </c>
       <c r="B1247" s="35" t="s">
-        <v>1962</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="1248" spans="1:2">
       <c r="A1248" s="34" t="s">
-        <v>1963</v>
+        <v>1961</v>
       </c>
       <c r="B1248" s="35" t="s">
-        <v>1964</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="1249" spans="1:2">
       <c r="A1249" s="34" t="s">
-        <v>1986</v>
+        <v>1984</v>
       </c>
       <c r="B1249" s="35" t="s">
-        <v>1987</v>
+        <v>1985</v>
       </c>
     </row>
     <row r="1250" spans="1:2">
       <c r="A1250" s="34" t="s">
-        <v>1988</v>
+        <v>1986</v>
       </c>
       <c r="B1250" s="35" t="s">
-        <v>1989</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="1251" spans="1:2">
       <c r="A1251" s="36" t="s">
-        <v>1990</v>
+        <v>1988</v>
       </c>
       <c r="B1251" s="37" t="s">
-        <v>1991</v>
+        <v>1989</v>
       </c>
     </row>
     <row r="1252" spans="1:2">
       <c r="A1252" s="34" t="s">
-        <v>1992</v>
+        <v>1990</v>
       </c>
       <c r="B1252" s="35" t="s">
-        <v>1993</v>
+        <v>1991</v>
       </c>
     </row>
     <row r="1253" spans="1:2">
       <c r="A1253" s="34" t="s">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="B1253" s="35" t="s">
-        <v>1801</v>
+        <v>1799</v>
       </c>
     </row>
     <row r="1254" spans="1:2">
       <c r="A1254" s="34" t="s">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="B1254" s="35" t="s">
-        <v>1996</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="1255" spans="1:2">
       <c r="A1255" s="34" t="s">
-        <v>1997</v>
+        <v>1995</v>
       </c>
       <c r="B1255" s="35" t="s">
-        <v>1998</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="1256" spans="1:2">
       <c r="A1256" s="34" t="s">
-        <v>1999</v>
+        <v>1997</v>
       </c>
       <c r="B1256" s="35" t="s">
         <v>571</v>
@@ -20057,7 +20164,7 @@
     </row>
     <row r="1257" spans="1:2">
       <c r="A1257" s="34" t="s">
-        <v>2000</v>
+        <v>1998</v>
       </c>
       <c r="B1257" s="35" t="s">
         <v>305</v>
@@ -20065,7 +20172,7 @@
     </row>
     <row r="1258" spans="1:2">
       <c r="A1258" s="34" t="s">
-        <v>2001</v>
+        <v>1999</v>
       </c>
       <c r="B1258" s="35" t="s">
         <v>917</v>
@@ -20073,7 +20180,7 @@
     </row>
     <row r="1259" spans="1:2">
       <c r="A1259" s="34" t="s">
-        <v>2002</v>
+        <v>2000</v>
       </c>
       <c r="B1259" s="35" t="s">
         <v>1413</v>
@@ -20081,55 +20188,55 @@
     </row>
     <row r="1260" spans="1:2">
       <c r="A1260" s="34" t="s">
-        <v>2003</v>
+        <v>2001</v>
       </c>
       <c r="B1260" s="35" t="s">
-        <v>2004</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="1261" spans="1:2">
       <c r="A1261" s="34" t="s">
-        <v>2005</v>
+        <v>2003</v>
       </c>
       <c r="B1261" s="35" t="s">
-        <v>2006</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="1262" spans="1:2">
       <c r="A1262" s="34" t="s">
-        <v>2007</v>
+        <v>2005</v>
       </c>
       <c r="B1262" s="35" t="s">
-        <v>2008</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="1263" spans="1:2">
       <c r="A1263" s="34" t="s">
-        <v>2009</v>
+        <v>2007</v>
       </c>
       <c r="B1263" s="35" t="s">
-        <v>2010</v>
+        <v>2008</v>
       </c>
     </row>
     <row r="1264" spans="1:2">
       <c r="A1264" s="34" t="s">
-        <v>2011</v>
+        <v>2009</v>
       </c>
       <c r="B1264" s="35" t="s">
-        <v>2012</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="1265" spans="1:2">
       <c r="A1265" s="34" t="s">
-        <v>2013</v>
+        <v>2011</v>
       </c>
       <c r="B1265" s="35" t="s">
-        <v>2014</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="1266" spans="1:2">
       <c r="A1266" s="34" t="s">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="B1266" s="35" t="s">
         <v>915</v>
@@ -20137,119 +20244,119 @@
     </row>
     <row r="1267" spans="1:2">
       <c r="A1267" s="34" t="s">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="B1267" s="35" t="s">
-        <v>2017</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="1268" spans="1:2">
       <c r="A1268" s="34" t="s">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="B1268" s="35" t="s">
-        <v>2019</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="1269" spans="1:2">
       <c r="A1269" s="34" t="s">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="B1269" s="35" t="s">
-        <v>2021</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="1270" spans="1:2">
       <c r="A1270" s="34" t="s">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="B1270" s="35" t="s">
-        <v>2023</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="1271" spans="1:2">
       <c r="A1271" s="34" t="s">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="B1271" s="35" t="s">
-        <v>2025</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="1272" spans="1:2">
       <c r="A1272" s="34" t="s">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="B1272" s="35" t="s">
-        <v>2027</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="1273" spans="1:2">
       <c r="A1273" s="34" t="s">
-        <v>2028</v>
+        <v>2026</v>
       </c>
       <c r="B1273" s="35" t="s">
-        <v>2029</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="1274" spans="1:2">
       <c r="A1274" s="34" t="s">
-        <v>2030</v>
+        <v>2028</v>
       </c>
       <c r="B1274" s="35" t="s">
-        <v>2031</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="1275" spans="1:2">
       <c r="A1275" s="34" t="s">
-        <v>2032</v>
+        <v>2030</v>
       </c>
       <c r="B1275" s="35" t="s">
-        <v>2033</v>
+        <v>2031</v>
       </c>
     </row>
     <row r="1276" spans="1:2">
       <c r="A1276" s="34" t="s">
-        <v>2034</v>
+        <v>2032</v>
       </c>
       <c r="B1276" s="35" t="s">
-        <v>2035</v>
+        <v>2033</v>
       </c>
     </row>
     <row r="1277" spans="1:2">
       <c r="A1277" s="34" t="s">
-        <v>2036</v>
+        <v>2034</v>
       </c>
       <c r="B1277" s="35" t="s">
-        <v>2037</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="1278" spans="1:2">
       <c r="A1278" s="34" t="s">
-        <v>2038</v>
+        <v>2036</v>
       </c>
       <c r="B1278" s="35" t="s">
-        <v>2039</v>
+        <v>2037</v>
       </c>
     </row>
     <row r="1279" spans="1:2">
-      <c r="A1279" s="72" t="s">
-        <v>1880</v>
-      </c>
-      <c r="B1279" s="73" t="s">
-        <v>1881</v>
+      <c r="A1279" s="34" t="s">
+        <v>1878</v>
+      </c>
+      <c r="B1279" s="35" t="s">
+        <v>1879</v>
       </c>
     </row>
     <row r="1280" spans="1:2">
       <c r="A1280" s="34" t="s">
-        <v>2040</v>
+        <v>2038</v>
       </c>
       <c r="B1280" s="35" t="s">
-        <v>2041</v>
+        <v>2039</v>
       </c>
     </row>
     <row r="1281" spans="1:2">
       <c r="A1281" s="34" t="s">
-        <v>2042</v>
+        <v>2040</v>
       </c>
       <c r="B1281" s="35" t="s">
         <v>563</v>
@@ -20257,7 +20364,7 @@
     </row>
     <row r="1282" spans="1:2">
       <c r="A1282" s="34" t="s">
-        <v>2043</v>
+        <v>2041</v>
       </c>
       <c r="B1282" s="35" t="s">
         <v>59</v>
@@ -20265,7 +20372,7 @@
     </row>
     <row r="1283" spans="1:2">
       <c r="A1283" s="34" t="s">
-        <v>2044</v>
+        <v>2042</v>
       </c>
       <c r="B1283" s="35" t="s">
         <v>378</v>
@@ -20273,23 +20380,23 @@
     </row>
     <row r="1284" spans="1:2">
       <c r="A1284" s="34" t="s">
-        <v>2045</v>
+        <v>2043</v>
       </c>
       <c r="B1284" s="35" t="s">
-        <v>2046</v>
+        <v>2044</v>
       </c>
     </row>
     <row r="1285" spans="1:2">
       <c r="A1285" s="34" t="s">
-        <v>2047</v>
+        <v>2045</v>
       </c>
       <c r="B1285" s="35" t="s">
-        <v>2048</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="1286" spans="1:2">
       <c r="A1286" s="34" t="s">
-        <v>2049</v>
+        <v>2047</v>
       </c>
       <c r="B1286" s="35" t="s">
         <v>716</v>
@@ -20297,71 +20404,71 @@
     </row>
     <row r="1287" spans="1:2">
       <c r="A1287" s="34" t="s">
-        <v>2050</v>
+        <v>2048</v>
       </c>
       <c r="B1287" s="35" t="s">
-        <v>2051</v>
+        <v>2049</v>
       </c>
     </row>
     <row r="1288" spans="1:2">
       <c r="A1288" s="34" t="s">
-        <v>2052</v>
+        <v>2050</v>
       </c>
       <c r="B1288" s="35" t="s">
-        <v>2053</v>
+        <v>2051</v>
       </c>
     </row>
     <row r="1289" spans="1:2">
       <c r="A1289" s="34" t="s">
-        <v>2054</v>
+        <v>2052</v>
       </c>
       <c r="B1289" s="35" t="s">
-        <v>2055</v>
+        <v>2053</v>
       </c>
     </row>
     <row r="1290" spans="1:2">
       <c r="A1290" s="34" t="s">
-        <v>2056</v>
+        <v>2054</v>
       </c>
       <c r="B1290" s="35" t="s">
-        <v>2057</v>
+        <v>2055</v>
       </c>
     </row>
     <row r="1291" spans="1:2">
       <c r="A1291" s="34" t="s">
-        <v>2058</v>
+        <v>2056</v>
       </c>
       <c r="B1291" s="35" t="s">
-        <v>1583</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="1292" spans="1:2">
       <c r="A1292" s="34" t="s">
-        <v>2059</v>
+        <v>2057</v>
       </c>
       <c r="B1292" s="35" t="s">
-        <v>2060</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="1293" spans="1:2">
       <c r="A1293" s="34" t="s">
-        <v>2061</v>
+        <v>2059</v>
       </c>
       <c r="B1293" s="35" t="s">
-        <v>2062</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="1294" spans="1:2">
       <c r="A1294" s="34" t="s">
-        <v>2063</v>
+        <v>2061</v>
       </c>
       <c r="B1294" s="35" t="s">
-        <v>2064</v>
+        <v>2062</v>
       </c>
     </row>
     <row r="1295" spans="1:2">
       <c r="A1295" s="34" t="s">
-        <v>2065</v>
+        <v>2063</v>
       </c>
       <c r="B1295" s="35" t="s">
         <v>93</v>
@@ -20369,15 +20476,15 @@
     </row>
     <row r="1296" spans="1:2">
       <c r="A1296" s="34" t="s">
-        <v>2066</v>
+        <v>2064</v>
       </c>
       <c r="B1296" s="35" t="s">
-        <v>2067</v>
+        <v>2065</v>
       </c>
     </row>
     <row r="1297" spans="1:2">
       <c r="A1297" s="34" t="s">
-        <v>2068</v>
+        <v>2066</v>
       </c>
       <c r="B1297" s="35" t="s">
         <v>567</v>
@@ -20385,7 +20492,7 @@
     </row>
     <row r="1298" spans="1:2">
       <c r="A1298" s="34" t="s">
-        <v>2069</v>
+        <v>2067</v>
       </c>
       <c r="B1298" s="35" t="s">
         <v>331</v>
@@ -20393,7 +20500,7 @@
     </row>
     <row r="1299" spans="1:2">
       <c r="A1299" s="34" t="s">
-        <v>2070</v>
+        <v>2068</v>
       </c>
       <c r="B1299" s="35" t="s">
         <v>7</v>
@@ -20401,15 +20508,15 @@
     </row>
     <row r="1300" spans="1:2">
       <c r="A1300" s="34" t="s">
-        <v>2071</v>
+        <v>2069</v>
       </c>
       <c r="B1300" s="35" t="s">
-        <v>2072</v>
+        <v>2070</v>
       </c>
     </row>
     <row r="1301" spans="1:2">
       <c r="A1301" s="34" t="s">
-        <v>2073</v>
+        <v>2071</v>
       </c>
       <c r="B1301" s="35" t="s">
         <v>223</v>
@@ -20417,15 +20524,15 @@
     </row>
     <row r="1302" spans="1:2">
       <c r="A1302" s="34" t="s">
-        <v>2074</v>
+        <v>2072</v>
       </c>
       <c r="B1302" s="35" t="s">
-        <v>2075</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="1303" spans="1:2">
       <c r="A1303" s="34" t="s">
-        <v>2076</v>
+        <v>2074</v>
       </c>
       <c r="B1303" s="35" t="s">
         <v>152</v>
@@ -20433,7 +20540,7 @@
     </row>
     <row r="1304" spans="1:2">
       <c r="A1304" s="34" t="s">
-        <v>2077</v>
+        <v>2075</v>
       </c>
       <c r="B1304" s="35" t="s">
         <v>223</v>
@@ -20441,7 +20548,7 @@
     </row>
     <row r="1305" spans="1:2">
       <c r="A1305" s="34" t="s">
-        <v>2078</v>
+        <v>2076</v>
       </c>
       <c r="B1305" s="35" t="s">
         <v>223</v>
@@ -20449,183 +20556,183 @@
     </row>
     <row r="1306" spans="1:2">
       <c r="A1306" s="34" t="s">
-        <v>2079</v>
+        <v>2077</v>
       </c>
       <c r="B1306" s="35" t="s">
-        <v>2080</v>
+        <v>2078</v>
       </c>
     </row>
     <row r="1307" spans="1:2">
       <c r="A1307" s="34" t="s">
-        <v>2081</v>
+        <v>2079</v>
       </c>
       <c r="B1307" s="35" t="s">
-        <v>1993</v>
+        <v>1991</v>
       </c>
     </row>
     <row r="1308" spans="1:2">
       <c r="A1308" s="34" t="s">
-        <v>2082</v>
+        <v>2080</v>
       </c>
       <c r="B1308" s="35" t="s">
-        <v>2083</v>
+        <v>2081</v>
       </c>
     </row>
     <row r="1309" spans="1:2">
       <c r="A1309" s="34" t="s">
-        <v>2084</v>
+        <v>2082</v>
       </c>
       <c r="B1309" s="35" t="s">
-        <v>2085</v>
+        <v>2083</v>
       </c>
     </row>
     <row r="1310" spans="1:2">
       <c r="A1310" s="34" t="s">
-        <v>2086</v>
+        <v>2084</v>
       </c>
       <c r="B1310" s="35" t="s">
-        <v>2087</v>
+        <v>2085</v>
       </c>
     </row>
     <row r="1311" spans="1:2">
       <c r="A1311" s="34" t="s">
-        <v>2088</v>
+        <v>2086</v>
       </c>
       <c r="B1311" s="35" t="s">
-        <v>2089</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="1312" spans="1:2">
       <c r="A1312" s="34" t="s">
-        <v>2090</v>
+        <v>2088</v>
       </c>
       <c r="B1312" s="35" t="s">
-        <v>2091</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="1313" spans="1:2">
       <c r="A1313" s="34" t="s">
-        <v>2092</v>
+        <v>2090</v>
       </c>
       <c r="B1313" s="35" t="s">
-        <v>2093</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="1314" spans="1:2">
       <c r="A1314" s="34" t="s">
-        <v>2094</v>
+        <v>2092</v>
       </c>
       <c r="B1314" s="35" t="s">
-        <v>2095</v>
+        <v>2093</v>
       </c>
     </row>
     <row r="1315" spans="1:2">
       <c r="A1315" s="34" t="s">
-        <v>2096</v>
+        <v>2094</v>
       </c>
       <c r="B1315" s="35" t="s">
-        <v>2097</v>
+        <v>2095</v>
       </c>
     </row>
     <row r="1316" spans="1:2">
       <c r="A1316" s="34" t="s">
-        <v>2098</v>
+        <v>2096</v>
       </c>
       <c r="B1316" s="35" t="s">
-        <v>2099</v>
+        <v>2097</v>
       </c>
     </row>
     <row r="1317" spans="1:2">
       <c r="A1317" s="34" t="s">
-        <v>2100</v>
+        <v>2098</v>
       </c>
       <c r="B1317" s="35" t="s">
-        <v>2101</v>
+        <v>2099</v>
       </c>
     </row>
     <row r="1318" spans="1:2">
       <c r="A1318" s="34" t="s">
-        <v>2102</v>
+        <v>2100</v>
       </c>
       <c r="B1318" s="35" t="s">
-        <v>2097</v>
+        <v>2095</v>
       </c>
     </row>
     <row r="1319" spans="1:2">
       <c r="A1319" s="34" t="s">
-        <v>2103</v>
+        <v>2101</v>
       </c>
       <c r="B1319" s="35" t="s">
-        <v>2104</v>
+        <v>2102</v>
       </c>
     </row>
     <row r="1320" spans="1:2">
       <c r="A1320" s="34" t="s">
-        <v>2105</v>
+        <v>2103</v>
       </c>
       <c r="B1320" s="35" t="s">
-        <v>2106</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="1321" spans="1:2">
       <c r="A1321" s="34" t="s">
-        <v>2107</v>
+        <v>2105</v>
       </c>
       <c r="B1321" s="35" t="s">
-        <v>1633</v>
+        <v>1631</v>
       </c>
     </row>
     <row r="1322" spans="1:2">
       <c r="A1322" s="34" t="s">
-        <v>2108</v>
+        <v>2106</v>
       </c>
       <c r="B1322" s="35" t="s">
-        <v>2109</v>
+        <v>2107</v>
       </c>
     </row>
     <row r="1323" spans="1:2">
       <c r="A1323" s="34" t="s">
-        <v>2110</v>
+        <v>2108</v>
       </c>
       <c r="B1323" s="35" t="s">
-        <v>2111</v>
+        <v>2109</v>
       </c>
     </row>
     <row r="1324" spans="1:2">
       <c r="A1324" s="34" t="s">
-        <v>2112</v>
+        <v>2110</v>
       </c>
       <c r="B1324" s="35" t="s">
-        <v>2113</v>
+        <v>2111</v>
       </c>
     </row>
     <row r="1325" spans="1:2">
       <c r="A1325" s="34" t="s">
-        <v>2114</v>
+        <v>2112</v>
       </c>
       <c r="B1325" s="35" t="s">
-        <v>1583</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="1326" spans="1:2">
       <c r="A1326" s="34" t="s">
-        <v>2115</v>
+        <v>2113</v>
       </c>
       <c r="B1326" s="35" t="s">
-        <v>2116</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="1327" spans="1:2">
       <c r="A1327" s="34" t="s">
-        <v>2117</v>
+        <v>2115</v>
       </c>
       <c r="B1327" s="35" t="s">
-        <v>2106</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="1328" spans="1:2">
       <c r="A1328" s="34" t="s">
-        <v>2118</v>
+        <v>2116</v>
       </c>
       <c r="B1328" s="35" t="s">
         <v>228</v>
@@ -20633,58 +20740,58 @@
     </row>
     <row r="1329" spans="1:2">
       <c r="A1329" s="34" t="s">
-        <v>2119</v>
+        <v>2117</v>
       </c>
       <c r="B1329" s="35" t="s">
-        <v>2120</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="1330" spans="1:2">
       <c r="A1330" s="34" t="s">
-        <v>2121</v>
+        <v>2119</v>
       </c>
       <c r="B1330" s="35" t="s">
-        <v>2106</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="1331" spans="1:2">
       <c r="A1331" s="34" t="s">
-        <v>2122</v>
+        <v>2120</v>
       </c>
       <c r="B1331" s="35" t="s">
-        <v>2116</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="1332" spans="1:2">
       <c r="A1332" s="34" t="s">
-        <v>2123</v>
+        <v>2121</v>
       </c>
       <c r="B1332" s="35" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="1333" spans="1:2">
-      <c r="A1333" s="74" t="s">
+      <c r="A1333" s="68" t="s">
+        <v>2122</v>
+      </c>
+      <c r="B1333" s="71" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="1334" spans="1:2">
+      <c r="A1334" s="68" t="s">
+        <v>2123</v>
+      </c>
+      <c r="B1334" s="71" t="s">
         <v>2124</v>
       </c>
-      <c r="B1333" s="75" t="s">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="1334" spans="1:2">
-      <c r="A1334" s="74" t="s">
+    </row>
+    <row r="1335" spans="1:2">
+      <c r="A1335" s="68" t="s">
         <v>2125</v>
       </c>
-      <c r="B1334" s="75" t="s">
+      <c r="B1335" s="71" t="s">
         <v>2126</v>
-      </c>
-    </row>
-    <row r="1335" spans="1:2">
-      <c r="A1335" s="74" t="s">
-        <v>2127</v>
-      </c>
-      <c r="B1335" s="75" t="s">
-        <v>2128</v>
       </c>
     </row>
   </sheetData>
@@ -20699,10 +20806,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B62"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <dimension ref="A1:B63"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -20716,489 +20823,497 @@
     </row>
     <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>2129</v>
+        <v>2127</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>2130</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>2131</v>
+        <v>2129</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2132</v>
+        <v>2130</v>
       </c>
     </row>
     <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>2133</v>
+        <v>2131</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2134</v>
+        <v>2132</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>2135</v>
+        <v>2133</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2136</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>2137</v>
+        <v>2135</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2138</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>2139</v>
+        <v>2137</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>2140</v>
+        <v>2138</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>2141</v>
+        <v>2139</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>2142</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>2143</v>
+        <v>2141</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>2144</v>
+        <v>2142</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>2145</v>
+        <v>2143</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>2146</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>2147</v>
+        <v>2145</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>2148</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>2149</v>
+        <v>2147</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>2150</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>2151</v>
+        <v>2149</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>2152</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>2153</v>
+        <v>2151</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>2154</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>2155</v>
+        <v>2153</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>2156</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>2157</v>
+        <v>2155</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>2158</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>2159</v>
+        <v>2157</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>2160</v>
+        <v>2158</v>
       </c>
     </row>
     <row r="18" ht="43.5" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>2161</v>
+        <v>2159</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>2162</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>2163</v>
+        <v>2161</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>2164</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="20" ht="52.5" customHeight="1" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>2165</v>
+        <v>2163</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>2166</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>2167</v>
+        <v>2165</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>2168</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:2">
       <c r="A22" s="4" t="s">
-        <v>2169</v>
+        <v>2167</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>2170</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="23" ht="409.5" spans="1:2">
       <c r="A23" s="2" t="s">
+        <v>2169</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>2170</v>
+      </c>
+    </row>
+    <row r="24" ht="244.8" spans="1:2">
+      <c r="A24" s="2" t="s">
         <v>2171</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B24" s="5" t="s">
         <v>2172</v>
       </c>
     </row>
-    <row r="24" ht="246.5" spans="1:2">
-      <c r="A24" s="2" t="s">
+    <row r="25" ht="230.4" spans="1:2">
+      <c r="A25" t="s">
         <v>2173</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>2174</v>
       </c>
     </row>
-    <row r="25" ht="232" spans="1:2">
-      <c r="A25" t="s">
+    <row r="26" ht="259.2" spans="1:2">
+      <c r="A26" t="s">
         <v>2175</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B26" s="6" t="s">
         <v>2176</v>
       </c>
     </row>
-    <row r="26" ht="261" spans="1:2">
-      <c r="A26" t="s">
+    <row r="27" ht="201.6" spans="1:2">
+      <c r="A27" t="s">
         <v>2177</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B27" s="6" t="s">
         <v>2178</v>
-      </c>
-    </row>
-    <row r="27" ht="203" spans="1:2">
-      <c r="A27" t="s">
-        <v>2179</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>2180</v>
       </c>
     </row>
     <row r="28" ht="61.5" customHeight="1" spans="1:2">
       <c r="A28" t="s">
-        <v>2181</v>
+        <v>2179</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>2182</v>
+        <v>2180</v>
       </c>
     </row>
     <row r="29" ht="105.75" customHeight="1" spans="1:2">
       <c r="A29" s="7" t="s">
-        <v>2129</v>
+        <v>2127</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>2130</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="30" ht="83.25" customHeight="1" spans="1:2">
       <c r="A30" s="9" t="s">
-        <v>2131</v>
+        <v>2129</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>2132</v>
-      </c>
-    </row>
-    <row r="31" ht="174" spans="1:2">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="31" ht="172.8" spans="1:2">
       <c r="A31" s="11" t="s">
-        <v>2137</v>
+        <v>2135</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>2138</v>
-      </c>
-    </row>
-    <row r="32" ht="130.5" spans="1:2">
+        <v>2136</v>
+      </c>
+    </row>
+    <row r="32" ht="129.6" spans="1:2">
       <c r="A32" s="13" t="s">
+        <v>2181</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
+      <c r="A33" s="15" t="s">
         <v>2183</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B33" s="16" t="s">
         <v>2184</v>
       </c>
     </row>
-    <row r="33" ht="174" spans="1:2">
-      <c r="A33" s="15" t="s">
+    <row r="34" ht="172.8" spans="1:2">
+      <c r="A34" s="17" t="s">
         <v>2185</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B34" s="18" t="s">
         <v>2186</v>
-      </c>
-    </row>
-    <row r="34" ht="174" spans="1:2">
-      <c r="A34" s="17" t="s">
-        <v>2187</v>
-      </c>
-      <c r="B34" s="18" t="s">
-        <v>2188</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:2">
       <c r="A35" s="19" t="s">
-        <v>2159</v>
+        <v>2157</v>
       </c>
       <c r="B35" s="20" t="s">
+        <v>2187</v>
+      </c>
+    </row>
+    <row r="36" ht="403.2" spans="1:2">
+      <c r="A36" s="21" t="s">
+        <v>2188</v>
+      </c>
+      <c r="B36" s="22" t="s">
         <v>2189</v>
-      </c>
-    </row>
-    <row r="36" ht="406" spans="1:2">
-      <c r="A36" s="21" t="s">
-        <v>2190</v>
-      </c>
-      <c r="B36" s="22" t="s">
-        <v>2191</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="23" t="s">
-        <v>2192</v>
+        <v>2190</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>2193</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="25" t="s">
-        <v>2194</v>
+        <v>2192</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>2195</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:2">
       <c r="A39" s="27" t="s">
-        <v>2196</v>
+        <v>2194</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>2197</v>
+        <v>2195</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:2">
       <c r="A40" t="s">
+        <v>2196</v>
+      </c>
+      <c r="B40" s="29" t="s">
+        <v>2197</v>
+      </c>
+    </row>
+    <row r="41" ht="115.2" spans="1:2">
+      <c r="A41" t="s">
         <v>2198</v>
       </c>
-      <c r="B40" s="29" t="s">
+      <c r="B41" s="29" t="s">
         <v>2199</v>
       </c>
     </row>
-    <row r="41" ht="116" spans="1:2">
-      <c r="A41" t="s">
+    <row r="42" ht="172.8" spans="1:2">
+      <c r="A42" t="s">
         <v>2200</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B42" s="29" t="s">
         <v>2201</v>
       </c>
     </row>
-    <row r="42" ht="174" spans="1:2">
-      <c r="A42" t="s">
+    <row r="43" ht="187.2" spans="1:2">
+      <c r="A43" t="s">
         <v>2202</v>
       </c>
-      <c r="B42" s="29" t="s">
+      <c r="B43" s="29" t="s">
         <v>2203</v>
       </c>
     </row>
-    <row r="43" ht="188.5" spans="1:2">
-      <c r="A43" t="s">
+    <row r="44" ht="115.2" spans="1:2">
+      <c r="A44" t="s">
         <v>2204</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B44" s="29" t="s">
         <v>2205</v>
-      </c>
-    </row>
-    <row r="44" ht="116" spans="1:2">
-      <c r="A44" t="s">
-        <v>2206</v>
-      </c>
-      <c r="B44" s="29" t="s">
-        <v>2207</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>2208</v>
+        <v>2206</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>2209</v>
+        <v>2207</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>2210</v>
+        <v>2208</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>2211</v>
+        <v>2209</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:2">
       <c r="A47" t="s">
+        <v>2210</v>
+      </c>
+      <c r="B47" s="29" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="48" ht="259.2" spans="1:2">
+      <c r="A48" t="s">
         <v>2212</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B48" s="29" t="s">
         <v>2213</v>
-      </c>
-    </row>
-    <row r="48" ht="261" spans="1:2">
-      <c r="A48" t="s">
-        <v>2214</v>
-      </c>
-      <c r="B48" s="29" t="s">
-        <v>2215</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:2">
       <c r="A49" t="s">
+        <v>2214</v>
+      </c>
+      <c r="B49" s="29" t="s">
+        <v>2215</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
+      <c r="A50" t="s">
         <v>2216</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B50" s="29" t="s">
         <v>2217</v>
       </c>
     </row>
-    <row r="50" ht="333.5" spans="1:2">
-      <c r="A50" t="s">
+    <row r="51" ht="331.2" spans="1:2">
+      <c r="A51" t="s">
         <v>2218</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B51" s="29" t="s">
         <v>2219</v>
-      </c>
-    </row>
-    <row r="51" ht="333.5" spans="1:2">
-      <c r="A51" t="s">
-        <v>2220</v>
-      </c>
-      <c r="B51" s="29" t="s">
-        <v>2221</v>
       </c>
     </row>
     <row r="52" ht="36" customHeight="1" spans="1:2">
       <c r="A52" t="s">
-        <v>2222</v>
+        <v>2220</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>2223</v>
+        <v>2221</v>
       </c>
     </row>
     <row r="53" ht="23.25" customHeight="1" spans="1:2">
       <c r="A53" t="s">
-        <v>2224</v>
+        <v>2222</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>2225</v>
+        <v>2223</v>
       </c>
     </row>
     <row r="54" ht="27.75" customHeight="1" spans="1:2">
       <c r="A54" t="s">
+        <v>2224</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>2225</v>
+      </c>
+    </row>
+    <row r="55" ht="57.6" spans="1:2">
+      <c r="A55" t="s">
         <v>2226</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B55" s="6" t="s">
         <v>2227</v>
       </c>
     </row>
-    <row r="55" ht="58" spans="1:2">
-      <c r="A55" t="s">
+    <row r="56" ht="43.2" spans="1:2">
+      <c r="A56" t="s">
         <v>2228</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B56" s="29" t="s">
         <v>2229</v>
       </c>
     </row>
-    <row r="56" ht="43.5" spans="1:2">
-      <c r="A56" t="s">
+    <row r="57" ht="57.6" spans="1:2">
+      <c r="A57" t="s">
         <v>2230</v>
       </c>
-      <c r="B56" s="29" t="s">
+      <c r="B57" s="29" t="s">
         <v>2231</v>
       </c>
     </row>
-    <row r="57" ht="58" spans="1:2">
-      <c r="A57" t="s">
+    <row r="58" ht="72" spans="1:2">
+      <c r="A58" t="s">
         <v>2232</v>
       </c>
-      <c r="B57" s="29" t="s">
+      <c r="B58" s="29" t="s">
         <v>2233</v>
-      </c>
-    </row>
-    <row r="58" ht="72.5" spans="1:2">
-      <c r="A58" t="s">
-        <v>2234</v>
-      </c>
-      <c r="B58" s="29" t="s">
-        <v>2235</v>
       </c>
     </row>
     <row r="59" ht="409.5" spans="1:2">
       <c r="A59" t="s">
+        <v>2234</v>
+      </c>
+      <c r="B59" s="29" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="60" ht="86.4" spans="1:2">
+      <c r="A60" t="s">
         <v>2236</v>
       </c>
-      <c r="B59" s="29" t="s">
+      <c r="B60" s="29" t="s">
         <v>2237</v>
       </c>
     </row>
-    <row r="60" ht="87" spans="1:2">
-      <c r="A60" t="s">
+    <row r="61" ht="345.6" spans="1:2">
+      <c r="A61" t="s">
         <v>2238</v>
       </c>
-      <c r="B60" s="29" t="s">
+      <c r="B61" s="29" t="s">
         <v>2239</v>
       </c>
     </row>
-    <row r="61" ht="348" spans="1:2">
-      <c r="A61" t="s">
+    <row r="62" ht="57.6" spans="1:2">
+      <c r="A62" t="s">
         <v>2240</v>
       </c>
-      <c r="B61" s="29" t="s">
+      <c r="B62" s="29" t="s">
         <v>2241</v>
       </c>
     </row>
-    <row r="62" ht="58" spans="1:2">
-      <c r="A62" t="s">
+    <row r="63" ht="409.5" spans="1:2">
+      <c r="A63" t="s">
         <v>2242</v>
       </c>
-      <c r="B62" s="29" t="s">
+      <c r="B63" s="29" t="s">
         <v>2243</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated Fixes In OpenPO, SOB Test Scenarios
Updated Fixes In OpenPO, SOB Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="8400" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2763" uniqueCount="2243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2763" uniqueCount="2244">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -5523,6 +5523,9 @@
     <t>CSDisSimilarItem</t>
   </si>
   <si>
+    <t>SH-FG-100003</t>
+  </si>
+  <si>
     <t>PriceListPrefix</t>
   </si>
   <si>
@@ -6403,6 +6406,12 @@
   </si>
   <si>
     <t>Day(s)</t>
+  </si>
+  <si>
+    <t>HsnCode80200</t>
+  </si>
+  <si>
+    <t>85080200</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -6556,7 +6565,155 @@
     <t>SOHeaderQuery</t>
   </si>
   <si>
+    <t>SELECT soh_cust_id "Customer ID",
+       soh_cust_name "Customer Description",
+       soh_currency "Currency",
+       soh_exchange_rate "Exchange Rate",
+       soh_term_id "Payment Term",
+       soh_fob_id "INCO Term",
+       soh_shipvia_id "Ship VIA",
+       (  SELECT DECODE (applctrl_desc_level, 1, sv_desc1, sv_desc2)Shipvis_Description
+    FROM ship_vias, appl_control
+   WHERE sv_bu = soh_bu AND applctrl_bu = soh_bu AND sv_shipvia_id  = soh_shipvia_id)"Ship VIA Desc.",
+   ( SELECT TERM_EXT_DESC Term_Description
+    FROM terms_hd
+   WHERE term_bu = soh_bu
+     AND term_term_id =soh_term_id )"Payment Term Desc1.",
+     ( SELECT TERM_DESC1 Term_Description1
+    FROM terms_hd
+   WHERE term_bu = soh_bu
+     AND term_term_id =soh_term_id )"Payment Term Desc2.",
+     ( SELECT DECODE (applctrl_desc_level, 1, fob_desc1, fob_desc2) Fob_Description
+    FROM fobs, appl_control
+   WHERE fob_bu = soh_bu AND applctrl_bu = soh_bu AND fob_fob_id =soh_fob_id )"INCO Term Desc.",
+       soh_cc_id "CPC Code",
+       (SELECT pcc_desc
+          FROM profit_cost_centers
+         WHERE pcc_bu = soh_bu AND pcc_cc_code = soh_cc_id)
+          "CPC Code Desc",
+       NVL (suplr_prnt_capn, soh_cust_name) "Customer Print Name",
+       soh_sales_person "Sales Person",
+       soh_sub_terr_id "Sub Territory",
+       soh_terr_id "Sales Zone",
+       soh_sales_area "Sales Region",
+       soh_te_mgr_id "Sales Zone Manager",
+       suplr_group_id "Customer Group",
+       suplr_subgroup "Customer Sub Group",
+       soh_plnt_loc_id "Location ID",
+       soh_plant "Unit ID",
+       soh_order_type "Sub Voucher Type",
+       soh_order_pfx "SO prefix",
+       soh_order_no "SO Number",
+       SOH_TOT_AMT "SO Total Amount",
+         (SELECT DISTINCT apst_sub_type_desc
+             FROM appl_vou_sub_types
+            WHERE     apst_bu = soh_bu
+                  AND apst_vou_type = soh_vou_type
+                  AND apst_sub_type = soh_order_type)"Sub Voucher Desc",
+                    (SELECT sa_area_desc1
+             FROM sales_areas
+            WHERE sa_bu = soh_bu AND sa_area = soh_sales_area)"Area",
+                (SELECT sat_terr_desc1
+             FROM sales_area_terr
+            WHERE sat_bu = soh_bu AND sat_terr_id = soh_terr_id) "Territory",
+                     (SELECT sst_desc1
+             FROM sales_sub_terr
+            WHERE sst_bu = soh_bu AND sst_sub_terr_id = soh_sub_terr_id) "Sub Territory",
+              (SELECT sp_person_name1
+             FROM sales_persons
+            WHERE sp_bu = soh_bu AND sp_person = soh_sales_person) "Sales Person",
+              (SELECT DISTINCT supgrp_desc1
+             FROM supplier_groups, suppliers
+            WHERE     supgrp_bu = soh_bu
+                  AND supgrp_group_id = suplr_group_id
+                  AND supgrp_bu = suplr_bu
+                  AND suplr_bu = soh_bu
+                  AND suplr_suplr_id = soh_cust_id) "Group",
+                   (SELECT DISTINCT supsubgroup_desc1
+             FROM supplier_subgroup, suppliers
+            WHERE     supsubgroup_bu = soh_bu
+                  AND supsubgroup_type_id = suplr_subgroup
+                  AND supsubgroup_bu = suplr_bu
+                  AND suplr_bu = soh_bu
+                  AND suplr_suplr_id = soh_cust_id) "SubGroup",
+                  func_find_employee_desc(soh_bu ,SOH_TE_MGR_ID,1) "Sales Zone Mgr"   ,
+                  DECODE(soh_status,'N','Draft','A','Approved','O','Entry Completed','L','Cancelled','C','CloseShort')soh_status
+  FROM sales_order_hd, suppliers
+ WHERE     soh_bu = suplr_bu
+       AND soh_cust_id = suplr_suplr_id
+       AND suplr_status = 'A'
+       AND soh_bu = 'TVSA'
+       AND soh_order_no ='${SONO}'</t>
+  </si>
+  <si>
     <t>SOLineQuery</t>
+  </si>
+  <si>
+    <t>SELECT soq_prod_id "Item ID",soq_prod_rev "Item Rev",
+       soq_prod_desc1 "Item Desc",
+       soq_uom "Sale UOM",
+       soq_hsn_code "HSN Code",
+       soq_tax_pct "Tax Percentage",
+       soq_price_basis "Price Basis Type",
+       DECODE (soq_price_basis,
+               'C', 'Open Order',
+               'L', 'Catalog Price',
+               'P', 'Price List',
+               'S', 'Standard Price',
+               'U', 'User Defined')
+          "Price Basis Desc",
+       soq_cont_cat_no "Contract Number",
+       soq_catalog_no "Catalog / Price List Number",
+       soq_prod_uom "Stock UOM",
+       soq_conv_factor "Conversion Factor",
+       soq_tolr_type "Tolerance Type",
+       soq_cust_prod_id "Customer Item ID",
+       soq_cust_prod_desc "Customer Item Desc",
+       (SELECT store_desc1
+          FROM stores
+         WHERE store_bu = soq_bu AND store_id = soq_store_id
+        UNION ALL
+        SELECT dept_name1
+          FROM departments
+         WHERE dept_bu = soq_bu AND dept_id = soq_store_id)
+          "Warehouse Description",
+       soq_prod_subcls_desc "SubClass Desc",
+       soq_prod_cls_desc "Class Desc",
+       (SELECT spc_class_desc
+          FROM sales_price_classes
+         WHERE spc_bu = soq_bu AND spc_class_id = soq_sales_price_class)
+          "Price Class",
+       soq_promotion_flag "Promotional",
+       soq_trd_assbl_val "Trade Ass. Val.",
+       soq_disc_pct "Trade Disc. %",
+       soq_disc_amt "Trade Disc. Amt.",
+       soq_spl_assbl_val "Spl. Ass. Val.",
+       soq_spl_disc_pct "Spl. Disc. %",
+       soq_spl_disc_amt "Spl. Disc. Amt.",
+       soq_cash_assbl_val "Cash Ass. Val.",
+       soq_cash_disc_pct "Cash Disc. %",
+       soq_cash_disc_amt "Cash Disc. Amt.",
+       soq_gross_amt "Gross Amt.",
+       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
+       soq_tax_amt "Tax Amt.",
+       soq_net_amt "Net Amt.",
+       soq_gross_amt "Gross Amt.",
+       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
+       soq_tax_amt "Tax Amt.",
+       soq_net_amt "Net Amt.",
+       soq_qty_ordered "Ord. Qty.",
+       soq_price "Unit Price",
+       soq_tot_disc_amt "Disc. Amt.",
+       soq_igst_amt "IGST Amt.",
+       soq_sgst_amt "SGST Amt.",
+       soq_cgst_amt "CGST Amt.",
+       soq_utgst_amt,
+       DECODE(soq_status,'N','Draft','A','Approved','O','Entry Completed','L','Cancelled')Line_Status
+  FROM sales_order_hd, sales_order_qtys
+ WHERE     soh_bu = soq_bu
+       AND soh_order_no = soq_order_no
+       AND soh_bu = 'TVSA'
+       AND soh_order_no = '${SONO}'</t>
   </si>
   <si>
     <t>Stock Query</t>
@@ -6790,37 +6947,6 @@
 SELECT PS_SS_PROD_ID, PS_SS_PROD_REV, seq_no, PSI_SS_PROD_DESC, PS_SS_QTY, UOM
 FROM numbered_rows
 WHERE seq_no = '${PONO}'</t>
-  </si>
-  <si>
-    <t>POQuery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  SELECT pol_order_no,
-                       pol_trd_disc_amt,
-                      pol_spl_disc_amt,
-                      pol_cash_disc_amt,
-                      pol_trd_assbl_val,
-                      pol_spl_assbl_val,
-                      pol_cash_assbl_val,
-                      pol_tax_pct,
-                      pol_cgst_amt,
-                      pol_utgst_amt,
-                      pol_cess_amt,
-                      pol_cess_pct,
-                      pol_gst_exempt_flag,
-                      pol_gst_input_type,
-                      pol_pur_acct,
-                      pol_cc_code,
-                      pol_cost_basis,
-                      pol_ordered_qty,
-                      pol_proc_qty,
-                      pol_received_qty,
-                      pol_cls_qty,
-                     ((pol_ordered_qty * pol_sc_unit_cost) - pol_disc_amt) Line_amt
-              FROM pur_order_ln
-           WHERE pol_bu ='TVSA'
-               AND pol_order_no ='${PONO}'
-               and pol_prod_id ='${POID}'</t>
   </si>
   <si>
     <t>PRLineDetailsQuery</t>
@@ -7411,6 +7537,9 @@
    AND stock_store_id = '${SONO}'
    AND stock_prod_id ='${PRNO}'
    AND stock_prod_rev = '0'</t>
+  </si>
+  <si>
+    <t>POQuery</t>
   </si>
   <si>
     <t xml:space="preserve">        SELECT pol_order_no,
@@ -8352,6 +8481,74 @@
     <t>SOAfterSOALineQuery</t>
   </si>
   <si>
+    <t>SELECT soq_seq_no "SEQ NO",soq_prod_id "Item ID",soq_prod_rev "Item Rev",
+       soq_prod_desc1 "Item Desc",
+       soq_uom "Sale UOM",
+       soq_hsn_code "HSN Code",
+       soq_tax_pct "Tax Percentage",
+       soq_price_basis "Price Basis Type",
+       DECODE (soq_price_basis,
+               'C', 'Open Order',
+               'L', 'Catalog Price',
+               'P', 'Price List',
+               'S', 'Standard Price',
+               'U', 'User Defined')
+          "Price Basis Desc",
+       soq_cont_cat_no "Contract Number",
+       soq_catalog_no "Catalog / Price List Number",
+       soq_prod_uom "Stock UOM",
+       soq_conv_factor "Conversion Factor",
+       soq_tolr_type "Tolerance Type",
+       soq_cust_prod_id "Customer Item ID",
+       soq_cust_prod_desc "Customer Item Desc",
+       (SELECT store_desc1
+          FROM stores
+         WHERE store_bu = soq_bu AND store_id = soq_store_id
+        UNION ALL
+        SELECT dept_name1
+          FROM departments
+         WHERE dept_bu = soq_bu AND dept_id = soq_store_id)
+          "Warehouse Description",
+       soq_prod_subcls_desc "SubClass Desc",
+       soq_prod_cls_desc "Class Desc",
+       (SELECT spc_class_desc
+          FROM sales_price_classes
+         WHERE spc_bu = soq_bu AND spc_class_id = soq_sales_price_class)
+          "Price Class",
+       soq_promotion_flag "Promotional",
+       soq_trd_assbl_val "Trade Ass. Val.",
+       soq_disc_pct "Trade Disc. %",
+       soq_disc_amt "Trade Disc. Amt.",
+       soq_spl_assbl_val "Spl. Ass. Val.",
+       soq_spl_disc_pct "Spl. Disc. %",
+       soq_spl_disc_amt "Spl. Disc. Amt.",
+       soq_cash_assbl_val "Cash Ass. Val.",
+       soq_cash_disc_pct "Cash Disc. %",
+       soq_cash_disc_amt "Cash Disc. Amt.",
+       soq_gross_amt "Gross Amt.",
+       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
+       soq_tax_amt "Tax Amt.",
+       soq_net_amt "Net Amt.",
+       soq_gross_amt "Gross Amt.",
+       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
+       soq_tax_amt "Tax Amt.",
+       soq_net_amt "Net Amt.",
+       soq_qty_ordered "Ord. Qty.",
+       soq_price "Unit Price",
+       soq_tot_disc_amt "Disc. Amt.",
+       soq_igst_amt "IGST Amt.",
+       soq_sgst_amt "SGST Amt.",
+       soq_cgst_amt "CGST Amt.",
+       soq_utgst_amt,
+        DECODE(soq_status,'N','Draft','A','Approved','O','Entry Completed','L','Cancelled','C','CloseShort')Line_Status
+  FROM sales_order_hd, sales_order_qtys
+ WHERE     soh_bu = soq_bu
+       AND soh_order_no = soq_order_no
+       AND soh_bu = 'TVSA'
+       AND soh_order_no = '${SONO}'
+       AND soq_seq_no = '${PONO}'</t>
+  </si>
+  <si>
     <t>CSHeaderQuery</t>
   </si>
   <si>
@@ -8688,231 +8885,18 @@
     AND PRL_RQST_NO  ='${PRNO}'
     AND PRL_PROD_ID  ='${ItemId}'</t>
   </si>
-  <si>
-    <t>SELECT soh_cust_id "Customer ID",
-       soh_cust_name "Customer Description",
-       soh_currency "Currency",
-       soh_exchange_rate "Exchange Rate",
-       soh_term_id "Payment Term",
-       soh_fob_id "INCO Term",
-       soh_shipvia_id "Ship VIA",
-       (  SELECT DECODE (applctrl_desc_level, 1, sv_desc1, sv_desc2)Shipvis_Description
-    FROM ship_vias, appl_control
-   WHERE sv_bu = soh_bu AND applctrl_bu = soh_bu AND sv_shipvia_id  = soh_shipvia_id)"Ship VIA Desc.",
-   ( SELECT TERM_EXT_DESC Term_Description
-    FROM terms_hd
-   WHERE term_bu = soh_bu
-     AND term_term_id =soh_term_id )"Payment Term Desc1.",
-     ( SELECT TERM_DESC1 Term_Description1
-    FROM terms_hd
-   WHERE term_bu = soh_bu
-     AND term_term_id =soh_term_id )"Payment Term Desc2.",
-     ( SELECT DECODE (applctrl_desc_level, 1, fob_desc1, fob_desc2) Fob_Description
-    FROM fobs, appl_control
-   WHERE fob_bu = soh_bu AND applctrl_bu = soh_bu AND fob_fob_id =soh_fob_id )"INCO Term Desc.",
-       soh_cc_id "CPC Code",
-       (SELECT pcc_desc
-          FROM profit_cost_centers
-         WHERE pcc_bu = soh_bu AND pcc_cc_code = soh_cc_id)
-          "CPC Code Desc",
-       NVL (suplr_prnt_capn, soh_cust_name) "Customer Print Name",
-       soh_sales_person "Sales Person",
-       soh_sub_terr_id "Sub Territory",
-       soh_terr_id "Sales Zone",
-       soh_sales_area "Sales Region",
-       soh_te_mgr_id "Sales Zone Manager",
-       suplr_group_id "Customer Group",
-       suplr_subgroup "Customer Sub Group",
-       soh_plnt_loc_id "Location ID",
-       soh_plant "Unit ID",
-       soh_order_type "Sub Voucher Type",
-       soh_order_pfx "SO prefix",
-       soh_order_no "SO Number",
-       SOH_TOT_AMT "SO Total Amount",
-         (SELECT DISTINCT apst_sub_type_desc
-             FROM appl_vou_sub_types
-            WHERE     apst_bu = soh_bu
-                  AND apst_vou_type = soh_vou_type
-                  AND apst_sub_type = soh_order_type)"Sub Voucher Desc",
-                    (SELECT sa_area_desc1
-             FROM sales_areas
-            WHERE sa_bu = soh_bu AND sa_area = soh_sales_area)"Area",
-                (SELECT sat_terr_desc1
-             FROM sales_area_terr
-            WHERE sat_bu = soh_bu AND sat_terr_id = soh_terr_id) "Territory",
-                     (SELECT sst_desc1
-             FROM sales_sub_terr
-            WHERE sst_bu = soh_bu AND sst_sub_terr_id = soh_sub_terr_id) "Sub Territory",
-              (SELECT sp_person_name1
-             FROM sales_persons
-            WHERE sp_bu = soh_bu AND sp_person = soh_sales_person) "Sales Person",
-              (SELECT DISTINCT supgrp_desc1
-             FROM supplier_groups, suppliers
-            WHERE     supgrp_bu = soh_bu
-                  AND supgrp_group_id = suplr_group_id
-                  AND supgrp_bu = suplr_bu
-                  AND suplr_bu = soh_bu
-                  AND suplr_suplr_id = soh_cust_id) "Group",
-                   (SELECT DISTINCT supsubgroup_desc1
-             FROM supplier_subgroup, suppliers
-            WHERE     supsubgroup_bu = soh_bu
-                  AND supsubgroup_type_id = suplr_subgroup
-                  AND supsubgroup_bu = suplr_bu
-                  AND suplr_bu = soh_bu
-                  AND suplr_suplr_id = soh_cust_id) "SubGroup",
-                  func_find_employee_desc(soh_bu ,SOH_TE_MGR_ID,1) "Sales Zone Mgr"   ,
-                  DECODE(soh_status,'N','Draft','A','Approved','O','Entry Completed','L','Cancelled','C','CloseShort')soh_status
-  FROM sales_order_hd, suppliers
- WHERE     soh_bu = suplr_bu
-       AND soh_cust_id = suplr_suplr_id
-       AND suplr_status = 'A'
-       AND soh_bu = 'TVSA'
-       AND soh_order_no ='${SONO}'</t>
-  </si>
-  <si>
-    <t>SELECT soq_prod_id "Item ID",soq_prod_rev "Item Rev",
-       soq_prod_desc1 "Item Desc",
-       soq_uom "Sale UOM",
-       soq_hsn_code "HSN Code",
-       soq_tax_pct "Tax Percentage",
-       soq_price_basis "Price Basis Type",
-       DECODE (soq_price_basis,
-               'C', 'Open Order',
-               'L', 'Catalog Price',
-               'P', 'Price List',
-               'S', 'Standard Price',
-               'U', 'User Defined')
-          "Price Basis Desc",
-       soq_cont_cat_no "Contract Number",
-       soq_catalog_no "Catalog / Price List Number",
-       soq_prod_uom "Stock UOM",
-       soq_conv_factor "Conversion Factor",
-       soq_tolr_type "Tolerance Type",
-       soq_cust_prod_id "Customer Item ID",
-       soq_cust_prod_desc "Customer Item Desc",
-       (SELECT store_desc1
-          FROM stores
-         WHERE store_bu = soq_bu AND store_id = soq_store_id
-        UNION ALL
-        SELECT dept_name1
-          FROM departments
-         WHERE dept_bu = soq_bu AND dept_id = soq_store_id)
-          "Warehouse Description",
-       soq_prod_subcls_desc "SubClass Desc",
-       soq_prod_cls_desc "Class Desc",
-       (SELECT spc_class_desc
-          FROM sales_price_classes
-         WHERE spc_bu = soq_bu AND spc_class_id = soq_sales_price_class)
-          "Price Class",
-       soq_promotion_flag "Promotional",
-       soq_trd_assbl_val "Trade Ass. Val.",
-       soq_disc_pct "Trade Disc. %",
-       soq_disc_amt "Trade Disc. Amt.",
-       soq_spl_assbl_val "Spl. Ass. Val.",
-       soq_spl_disc_pct "Spl. Disc. %",
-       soq_spl_disc_amt "Spl. Disc. Amt.",
-       soq_cash_assbl_val "Cash Ass. Val.",
-       soq_cash_disc_pct "Cash Disc. %",
-       soq_cash_disc_amt "Cash Disc. Amt.",
-       soq_gross_amt "Gross Amt.",
-       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
-       soq_tax_amt "Tax Amt.",
-       soq_net_amt "Net Amt.",
-       soq_gross_amt "Gross Amt.",
-       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
-       soq_tax_amt "Tax Amt.",
-       soq_net_amt "Net Amt.",
-       soq_qty_ordered "Ord. Qty.",
-       soq_price "Unit Price",
-       soq_tot_disc_amt "Disc. Amt.",
-       soq_igst_amt "IGST Amt.",
-       soq_sgst_amt "SGST Amt.",
-       soq_cgst_amt "CGST Amt.",
-       soq_utgst_amt,
-       DECODE(soq_status,'N','Draft','A','Approved','O','Entry Completed','L','Cancelled')Line_Status
-  FROM sales_order_hd, sales_order_qtys
- WHERE     soh_bu = soq_bu
-       AND soh_order_no = soq_order_no
-       AND soh_bu = 'TVSA'
-       AND soh_order_no = '${SONO}'</t>
-  </si>
-  <si>
-    <t>SELECT soq_seq_no "SEQ NO",soq_prod_id "Item ID",soq_prod_rev "Item Rev",
-       soq_prod_desc1 "Item Desc",
-       soq_uom "Sale UOM",
-       soq_hsn_code "HSN Code",
-       soq_tax_pct "Tax Percentage",
-       soq_price_basis "Price Basis Type",
-       DECODE (soq_price_basis,
-               'C', 'Open Order',
-               'L', 'Catalog Price',
-               'P', 'Price List',
-               'S', 'Standard Price',
-               'U', 'User Defined')
-          "Price Basis Desc",
-       soq_cont_cat_no "Contract Number",
-       soq_catalog_no "Catalog / Price List Number",
-       soq_prod_uom "Stock UOM",
-       soq_conv_factor "Conversion Factor",
-       soq_tolr_type "Tolerance Type",
-       soq_cust_prod_id "Customer Item ID",
-       soq_cust_prod_desc "Customer Item Desc",
-       (SELECT store_desc1
-          FROM stores
-         WHERE store_bu = soq_bu AND store_id = soq_store_id
-        UNION ALL
-        SELECT dept_name1
-          FROM departments
-         WHERE dept_bu = soq_bu AND dept_id = soq_store_id)
-          "Warehouse Description",
-       soq_prod_subcls_desc "SubClass Desc",
-       soq_prod_cls_desc "Class Desc",
-       (SELECT spc_class_desc
-          FROM sales_price_classes
-         WHERE spc_bu = soq_bu AND spc_class_id = soq_sales_price_class)
-          "Price Class",
-       soq_promotion_flag "Promotional",
-       soq_trd_assbl_val "Trade Ass. Val.",
-       soq_disc_pct "Trade Disc. %",
-       soq_disc_amt "Trade Disc. Amt.",
-       soq_spl_assbl_val "Spl. Ass. Val.",
-       soq_spl_disc_pct "Spl. Disc. %",
-       soq_spl_disc_amt "Spl. Disc. Amt.",
-       soq_cash_assbl_val "Cash Ass. Val.",
-       soq_cash_disc_pct "Cash Disc. %",
-       soq_cash_disc_amt "Cash Disc. Amt.",
-       soq_gross_amt "Gross Amt.",
-       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
-       soq_tax_amt "Tax Amt.",
-       soq_net_amt "Net Amt.",
-       soq_gross_amt "Gross Amt.",
-       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
-       soq_tax_amt "Tax Amt.",
-       soq_net_amt "Net Amt.",
-       soq_qty_ordered "Ord. Qty.",
-       soq_price "Unit Price",
-       soq_tot_disc_amt "Disc. Amt.",
-       soq_igst_amt "IGST Amt.",
-       soq_sgst_amt "SGST Amt.",
-       soq_cgst_amt "CGST Amt.",
-       soq_utgst_amt,
-        DECODE(soq_status,'N','Draft','A','Approved','O','Entry Completed','L','Cancelled','C','CloseShort')Line_Status
-  FROM sales_order_hd, sales_order_qtys
- WHERE     soh_bu = soq_bu
-       AND soh_order_no = soq_order_no
-       AND soh_bu = 'TVSA'
-       AND soh_order_no = '${SONO}'
-       AND soq_seq_no = '${PONO}'</t>
-  </si>
-  <si>
-    <t>SH-FG-100003</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8959,14 +8943,151 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -8991,8 +9112,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -9028,26 +9335,268 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="18">
+  <cellStyleXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -9065,48 +9614,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="15" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="16" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="16" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="64" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="64" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="53"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -9135,15 +9684,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -9163,11 +9712,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -9181,19 +9730,19 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="59" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="60" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -9205,27 +9754,74 @@
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="18">
+  <cellStyles count="66">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1"/>
-    <cellStyle name="Normal 11" xfId="2"/>
-    <cellStyle name="Normal 13" xfId="3"/>
-    <cellStyle name="Normal 14" xfId="4"/>
-    <cellStyle name="Normal 15" xfId="5"/>
-    <cellStyle name="Normal 16" xfId="6"/>
-    <cellStyle name="Normal 17" xfId="7"/>
-    <cellStyle name="Normal 18" xfId="8"/>
-    <cellStyle name="Normal 19" xfId="9"/>
-    <cellStyle name="Normal 2" xfId="10"/>
-    <cellStyle name="Normal 2 2" xfId="11"/>
-    <cellStyle name="Normal 2 3" xfId="12"/>
-    <cellStyle name="Normal 20" xfId="13"/>
-    <cellStyle name="Normal 3" xfId="14"/>
-    <cellStyle name="Normal 7" xfId="15"/>
-    <cellStyle name="Normal 8" xfId="16"/>
-    <cellStyle name="Normal 9" xfId="17"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal 10" xfId="49"/>
+    <cellStyle name="Normal 11" xfId="50"/>
+    <cellStyle name="Normal 13" xfId="51"/>
+    <cellStyle name="Normal 14" xfId="52"/>
+    <cellStyle name="Normal 15" xfId="53"/>
+    <cellStyle name="Normal 16" xfId="54"/>
+    <cellStyle name="Normal 17" xfId="55"/>
+    <cellStyle name="Normal 18" xfId="56"/>
+    <cellStyle name="Normal 19" xfId="57"/>
+    <cellStyle name="Normal 2" xfId="58"/>
+    <cellStyle name="Normal 2 2" xfId="59"/>
+    <cellStyle name="Normal 2 3" xfId="60"/>
+    <cellStyle name="Normal 20" xfId="61"/>
+    <cellStyle name="Normal 3" xfId="62"/>
+    <cellStyle name="Normal 7" xfId="63"/>
+    <cellStyle name="Normal 8" xfId="64"/>
+    <cellStyle name="Normal 9" xfId="65"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -9487,17 +10083,17 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1335"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B1336"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.85546875" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -18130,12 +18726,12 @@
         <v>1830</v>
       </c>
       <c r="B1079" s="35" t="s">
-        <v>2242</v>
+        <v>1831</v>
       </c>
     </row>
     <row r="1080" spans="1:2">
       <c r="A1080" s="34" t="s">
-        <v>1831</v>
+        <v>1832</v>
       </c>
       <c r="B1080" s="35" t="s">
         <v>857</v>
@@ -18143,7 +18739,7 @@
     </row>
     <row r="1081" spans="1:2">
       <c r="A1081" s="34" t="s">
-        <v>1832</v>
+        <v>1833</v>
       </c>
       <c r="B1081" s="35" t="s">
         <v>1661</v>
@@ -18151,63 +18747,63 @@
     </row>
     <row r="1082" spans="1:2">
       <c r="A1082" s="34" t="s">
-        <v>1833</v>
+        <v>1834</v>
       </c>
       <c r="B1082" s="35" t="s">
-        <v>1834</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="1083" spans="1:2">
       <c r="A1083" s="34" t="s">
-        <v>1835</v>
+        <v>1836</v>
       </c>
       <c r="B1083" s="35" t="s">
-        <v>1836</v>
+        <v>1837</v>
       </c>
     </row>
     <row r="1084" spans="1:2">
       <c r="A1084" s="34" t="s">
-        <v>1837</v>
+        <v>1838</v>
       </c>
       <c r="B1084" s="35" t="s">
-        <v>1838</v>
+        <v>1839</v>
       </c>
     </row>
     <row r="1085" spans="1:2">
       <c r="A1085" s="34" t="s">
-        <v>1839</v>
+        <v>1840</v>
       </c>
       <c r="B1085" s="35" t="s">
-        <v>1840</v>
+        <v>1841</v>
       </c>
     </row>
     <row r="1086" spans="1:2">
       <c r="A1086" s="34" t="s">
-        <v>1841</v>
+        <v>1842</v>
       </c>
       <c r="B1086" s="35" t="s">
-        <v>1842</v>
+        <v>1843</v>
       </c>
     </row>
     <row r="1087" spans="1:2">
       <c r="A1087" s="34" t="s">
-        <v>1843</v>
+        <v>1844</v>
       </c>
       <c r="B1087" s="35" t="s">
-        <v>1844</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="1088" spans="1:2">
       <c r="A1088" s="34" t="s">
-        <v>1845</v>
+        <v>1846</v>
       </c>
       <c r="B1088" s="35" t="s">
-        <v>1846</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="1089" spans="1:2">
       <c r="A1089" s="34" t="s">
-        <v>1847</v>
+        <v>1848</v>
       </c>
       <c r="B1089" s="35" t="s">
         <v>478</v>
@@ -18215,39 +18811,39 @@
     </row>
     <row r="1090" spans="1:2">
       <c r="A1090" s="34" t="s">
-        <v>1848</v>
+        <v>1849</v>
       </c>
       <c r="B1090" s="35" t="s">
-        <v>1849</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="1091" spans="1:2">
       <c r="A1091" s="34" t="s">
-        <v>1850</v>
+        <v>1851</v>
       </c>
       <c r="B1091" s="35" t="s">
-        <v>1851</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="1092" spans="1:2">
       <c r="A1092" s="34" t="s">
-        <v>1852</v>
+        <v>1853</v>
       </c>
       <c r="B1092" s="35" t="s">
-        <v>1853</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="1093" spans="1:2">
       <c r="A1093" s="34" t="s">
-        <v>1854</v>
+        <v>1855</v>
       </c>
       <c r="B1093" s="35" t="s">
-        <v>1855</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="1094" spans="1:2">
       <c r="A1094" s="34" t="s">
-        <v>1856</v>
+        <v>1857</v>
       </c>
       <c r="B1094" s="35" t="s">
         <v>635</v>
@@ -18255,15 +18851,15 @@
     </row>
     <row r="1095" spans="1:2">
       <c r="A1095" s="34" t="s">
-        <v>1857</v>
+        <v>1858</v>
       </c>
       <c r="B1095" s="35" t="s">
-        <v>1858</v>
+        <v>1859</v>
       </c>
     </row>
     <row r="1096" spans="1:2">
       <c r="A1096" s="34" t="s">
-        <v>1859</v>
+        <v>1860</v>
       </c>
       <c r="B1096" s="35" t="s">
         <v>1760</v>
@@ -18271,39 +18867,39 @@
     </row>
     <row r="1097" spans="1:2">
       <c r="A1097" s="34" t="s">
-        <v>1860</v>
+        <v>1861</v>
       </c>
       <c r="B1097" s="35" t="s">
-        <v>1861</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="1098" spans="1:2">
       <c r="A1098" s="34" t="s">
-        <v>1862</v>
+        <v>1863</v>
       </c>
       <c r="B1098" s="35" t="s">
-        <v>1863</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="1099" spans="1:2">
       <c r="A1099" s="34" t="s">
-        <v>1864</v>
+        <v>1865</v>
       </c>
       <c r="B1099" s="35" t="s">
-        <v>1865</v>
+        <v>1866</v>
       </c>
     </row>
     <row r="1100" spans="1:2">
       <c r="A1100" s="34" t="s">
-        <v>1866</v>
+        <v>1867</v>
       </c>
       <c r="B1100" s="35" t="s">
-        <v>1867</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="1101" spans="1:2">
       <c r="A1101" s="34" t="s">
-        <v>1868</v>
+        <v>1869</v>
       </c>
       <c r="B1101" s="35" t="s">
         <v>687</v>
@@ -18311,15 +18907,15 @@
     </row>
     <row r="1102" spans="1:2">
       <c r="A1102" s="34" t="s">
-        <v>1869</v>
+        <v>1870</v>
       </c>
       <c r="B1102" s="35" t="s">
-        <v>1870</v>
+        <v>1871</v>
       </c>
     </row>
     <row r="1103" spans="1:2">
       <c r="A1103" s="34" t="s">
-        <v>1871</v>
+        <v>1872</v>
       </c>
       <c r="B1103" s="35" t="s">
         <v>928</v>
@@ -18327,7 +18923,7 @@
     </row>
     <row r="1104" spans="1:2">
       <c r="A1104" s="34" t="s">
-        <v>1872</v>
+        <v>1873</v>
       </c>
       <c r="B1104" s="35" t="s">
         <v>924</v>
@@ -18335,7 +18931,7 @@
     </row>
     <row r="1105" spans="1:2">
       <c r="A1105" s="34" t="s">
-        <v>1873</v>
+        <v>1874</v>
       </c>
       <c r="B1105" s="35" t="s">
         <v>926</v>
@@ -18343,34 +18939,34 @@
     </row>
     <row r="1106" spans="1:2">
       <c r="A1106" s="34" t="s">
-        <v>1874</v>
+        <v>1875</v>
       </c>
       <c r="B1106" s="35" t="s">
-        <v>1875</v>
+        <v>1876</v>
       </c>
     </row>
     <row r="1107" spans="1:2">
       <c r="A1107" s="34" t="s">
-        <v>1876</v>
+        <v>1877</v>
       </c>
       <c r="B1107" s="35" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="1108" spans="1:2">
       <c r="A1108" s="34" t="s">
-        <v>1878</v>
+        <v>1879</v>
       </c>
       <c r="B1108" s="35" t="s">
-        <v>1879</v>
+        <v>1880</v>
       </c>
     </row>
     <row r="1109" spans="1:2">
       <c r="A1109" s="34" t="s">
-        <v>1880</v>
+        <v>1881</v>
       </c>
       <c r="B1109" s="35" t="s">
-        <v>1881</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="1110" spans="1:2">
@@ -18386,31 +18982,31 @@
         <v>1570</v>
       </c>
       <c r="B1111" s="34" t="s">
-        <v>1882</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="1112" spans="1:2">
       <c r="A1112" s="47" t="s">
-        <v>1883</v>
+        <v>1884</v>
       </c>
       <c r="B1112" s="35" t="s">
-        <v>1884</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="1113" spans="1:2">
       <c r="A1113" s="47" t="s">
-        <v>1885</v>
+        <v>1886</v>
       </c>
       <c r="B1113" s="35" t="s">
-        <v>1886</v>
+        <v>1887</v>
       </c>
     </row>
     <row r="1114" spans="1:2">
       <c r="A1114" s="47" t="s">
-        <v>1887</v>
+        <v>1888</v>
       </c>
       <c r="B1114" s="35" t="s">
-        <v>1888</v>
+        <v>1889</v>
       </c>
     </row>
     <row r="1115" spans="1:2">
@@ -18418,7 +19014,7 @@
         <v>614</v>
       </c>
       <c r="B1115" s="35" t="s">
-        <v>1889</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="1116" spans="1:2">
@@ -18711,10 +19307,10 @@
     </row>
     <row r="1152" spans="1:2">
       <c r="A1152" s="34" t="s">
-        <v>1890</v>
+        <v>1891</v>
       </c>
       <c r="B1152" s="35" t="s">
-        <v>1891</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="1153" spans="1:2">
@@ -18839,23 +19435,23 @@
     </row>
     <row r="1168" spans="1:2">
       <c r="A1168" s="34" t="s">
-        <v>1892</v>
+        <v>1893</v>
       </c>
       <c r="B1168" s="35" t="s">
-        <v>1893</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="1169" spans="1:2">
       <c r="A1169" s="34" t="s">
-        <v>1894</v>
+        <v>1895</v>
       </c>
       <c r="B1169" s="35" t="s">
-        <v>1895</v>
+        <v>1896</v>
       </c>
     </row>
     <row r="1170" spans="1:2">
       <c r="A1170" s="34" t="s">
-        <v>1896</v>
+        <v>1897</v>
       </c>
       <c r="B1170" s="35" t="s">
         <v>559</v>
@@ -18863,39 +19459,39 @@
     </row>
     <row r="1171" spans="1:2">
       <c r="A1171" s="34" t="s">
-        <v>1897</v>
+        <v>1898</v>
       </c>
       <c r="B1171" s="35" t="s">
-        <v>1898</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="1172" spans="1:2">
       <c r="A1172" s="34" t="s">
-        <v>1899</v>
+        <v>1900</v>
       </c>
       <c r="B1172" s="35" t="s">
-        <v>1900</v>
+        <v>1901</v>
       </c>
     </row>
     <row r="1173" spans="1:2">
       <c r="A1173" s="34" t="s">
-        <v>1901</v>
+        <v>1902</v>
       </c>
       <c r="B1173" s="35" t="s">
-        <v>1902</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="1174" spans="1:2">
       <c r="A1174" s="34" t="s">
-        <v>1903</v>
+        <v>1904</v>
       </c>
       <c r="B1174" s="68" t="s">
-        <v>1904</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="1175" spans="1:2">
       <c r="A1175" s="34" t="s">
-        <v>1905</v>
+        <v>1906</v>
       </c>
       <c r="B1175" s="34" t="s">
         <v>59</v>
@@ -18903,23 +19499,23 @@
     </row>
     <row r="1176" spans="1:2">
       <c r="A1176" s="34" t="s">
-        <v>1906</v>
+        <v>1907</v>
       </c>
       <c r="B1176" s="34" t="s">
-        <v>1907</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="1177" spans="1:2">
       <c r="A1177" s="34" t="s">
-        <v>1908</v>
+        <v>1909</v>
       </c>
       <c r="B1177" s="35" t="s">
-        <v>1909</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="1178" spans="1:2">
       <c r="A1178" s="34" t="s">
-        <v>1910</v>
+        <v>1911</v>
       </c>
       <c r="B1178" s="68" t="s">
         <v>1494</v>
@@ -18927,7 +19523,7 @@
     </row>
     <row r="1179" spans="1:2">
       <c r="A1179" s="34" t="s">
-        <v>1911</v>
+        <v>1912</v>
       </c>
       <c r="B1179" s="68" t="s">
         <v>306</v>
@@ -18935,18 +19531,18 @@
     </row>
     <row r="1180" spans="1:2">
       <c r="A1180" s="34" t="s">
-        <v>1912</v>
+        <v>1913</v>
       </c>
       <c r="B1180" s="69" t="s">
-        <v>1913</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="1181" spans="1:2">
       <c r="A1181" s="34" t="s">
-        <v>1914</v>
+        <v>1915</v>
       </c>
       <c r="B1181" s="35" t="s">
-        <v>1915</v>
+        <v>1916</v>
       </c>
     </row>
     <row r="1182" spans="1:2">
@@ -19015,7 +19611,7 @@
     </row>
     <row r="1190" spans="1:2">
       <c r="A1190" s="34" t="s">
-        <v>1916</v>
+        <v>1917</v>
       </c>
       <c r="B1190" s="35" t="s">
         <v>1364</v>
@@ -19023,7 +19619,7 @@
     </row>
     <row r="1191" spans="1:2">
       <c r="A1191" s="34" t="s">
-        <v>1917</v>
+        <v>1918</v>
       </c>
       <c r="B1191" s="35" t="s">
         <v>1366</v>
@@ -19031,58 +19627,58 @@
     </row>
     <row r="1192" spans="1:2">
       <c r="A1192" s="34" t="s">
-        <v>1918</v>
+        <v>1919</v>
       </c>
       <c r="B1192" s="35" t="s">
-        <v>1919</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="1193" spans="1:2">
       <c r="A1193" s="34" t="s">
-        <v>1920</v>
+        <v>1921</v>
       </c>
       <c r="B1193" s="35" t="s">
-        <v>1921</v>
+        <v>1922</v>
       </c>
     </row>
     <row r="1194" spans="1:2">
       <c r="A1194" s="34" t="s">
-        <v>1922</v>
+        <v>1923</v>
       </c>
       <c r="B1194" s="35" t="s">
-        <v>1923</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="1195" spans="1:2">
       <c r="A1195" s="34" t="s">
-        <v>1924</v>
+        <v>1925</v>
       </c>
       <c r="B1195" s="35" t="s">
-        <v>1925</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="1196" spans="1:2">
       <c r="A1196" s="34" t="s">
-        <v>1926</v>
+        <v>1927</v>
       </c>
       <c r="B1196" s="35" t="s">
-        <v>1926</v>
+        <v>1927</v>
       </c>
     </row>
     <row r="1197" spans="1:2">
       <c r="A1197" s="34" t="s">
-        <v>1927</v>
+        <v>1928</v>
       </c>
       <c r="B1197" s="35" t="s">
-        <v>1927</v>
+        <v>1928</v>
       </c>
     </row>
     <row r="1198" spans="1:2">
       <c r="A1198" s="34" t="s">
-        <v>1928</v>
+        <v>1929</v>
       </c>
       <c r="B1198" s="35" t="s">
-        <v>1928</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="1199" spans="1:2">
@@ -19143,26 +19739,26 @@
     </row>
     <row r="1206" spans="1:2">
       <c r="A1206" s="34" t="s">
-        <v>1929</v>
+        <v>1930</v>
       </c>
       <c r="B1206" s="35" t="s">
-        <v>1930</v>
+        <v>1931</v>
       </c>
     </row>
     <row r="1207" spans="1:2">
       <c r="A1207" s="34" t="s">
-        <v>1931</v>
+        <v>1932</v>
       </c>
       <c r="B1207" s="35" t="s">
-        <v>1932</v>
+        <v>1933</v>
       </c>
     </row>
     <row r="1208" spans="1:2">
       <c r="A1208" s="34" t="s">
-        <v>1933</v>
+        <v>1934</v>
       </c>
       <c r="B1208" s="35" t="s">
-        <v>1934</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="1209" spans="1:2">
@@ -19183,23 +19779,23 @@
     </row>
     <row r="1211" spans="1:2">
       <c r="A1211" s="34" t="s">
-        <v>1935</v>
+        <v>1936</v>
       </c>
       <c r="B1211" s="34" t="s">
-        <v>1936</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="1212" spans="1:2">
       <c r="A1212" s="34" t="s">
-        <v>1937</v>
+        <v>1938</v>
       </c>
       <c r="B1212" s="69" t="s">
-        <v>1938</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="1213" spans="1:2">
       <c r="A1213" s="34" t="s">
-        <v>1939</v>
+        <v>1940</v>
       </c>
       <c r="B1213" s="70" t="s">
         <v>916</v>
@@ -19207,7 +19803,7 @@
     </row>
     <row r="1214" spans="1:2">
       <c r="A1214" s="34" t="s">
-        <v>1940</v>
+        <v>1941</v>
       </c>
       <c r="B1214" s="70" t="s">
         <v>1412</v>
@@ -19215,18 +19811,18 @@
     </row>
     <row r="1215" spans="1:2">
       <c r="A1215" s="34" t="s">
-        <v>1941</v>
+        <v>1942</v>
       </c>
       <c r="B1215" s="35" t="s">
-        <v>1942</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="1216" spans="1:2">
       <c r="A1216" s="34" t="s">
+        <v>1944</v>
+      </c>
+      <c r="B1216" s="35" t="s">
         <v>1943</v>
-      </c>
-      <c r="B1216" s="35" t="s">
-        <v>1942</v>
       </c>
     </row>
     <row r="1217" spans="1:2">
@@ -19242,7 +19838,7 @@
         <v>1561</v>
       </c>
       <c r="B1218" s="35" t="s">
-        <v>1944</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="1219" spans="1:2">
@@ -19250,7 +19846,7 @@
         <v>1563</v>
       </c>
       <c r="B1219" s="35" t="s">
-        <v>1944</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="1220" spans="1:2">
@@ -19287,15 +19883,15 @@
     </row>
     <row r="1224" spans="1:2">
       <c r="A1224" s="34" t="s">
-        <v>1945</v>
+        <v>1946</v>
       </c>
       <c r="B1224" s="34" t="s">
-        <v>1853</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="1225" spans="1:2">
       <c r="A1225" s="34" t="s">
-        <v>1946</v>
+        <v>1947</v>
       </c>
       <c r="B1225" s="35" t="s">
         <v>562</v>
@@ -19303,31 +19899,31 @@
     </row>
     <row r="1226" spans="1:2">
       <c r="A1226" s="34" t="s">
-        <v>1947</v>
+        <v>1948</v>
       </c>
       <c r="B1226" s="35" t="s">
-        <v>1948</v>
+        <v>1949</v>
       </c>
     </row>
     <row r="1227" spans="1:2">
       <c r="A1227" s="34" t="s">
-        <v>1949</v>
+        <v>1950</v>
       </c>
       <c r="B1227" s="35" t="s">
-        <v>1950</v>
+        <v>1951</v>
       </c>
     </row>
     <row r="1228" spans="1:2">
       <c r="A1228" s="34" t="s">
-        <v>1951</v>
+        <v>1952</v>
       </c>
       <c r="B1228" s="35" t="s">
-        <v>1952</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="1229" spans="1:2">
       <c r="A1229" s="34" t="s">
-        <v>1953</v>
+        <v>1954</v>
       </c>
       <c r="B1229" s="35" t="s">
         <v>1798</v>
@@ -19335,18 +19931,18 @@
     </row>
     <row r="1230" spans="1:2">
       <c r="A1230" s="34" t="s">
-        <v>1954</v>
+        <v>1955</v>
       </c>
       <c r="B1230" s="35" t="s">
-        <v>1898</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="1231" spans="1:2">
       <c r="A1231" s="34" t="s">
-        <v>1955</v>
+        <v>1956</v>
       </c>
       <c r="B1231" s="35" t="s">
-        <v>1956</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="1232" spans="1:2">
@@ -19359,71 +19955,71 @@
     </row>
     <row r="1233" spans="1:2">
       <c r="A1233" s="34" t="s">
-        <v>1957</v>
+        <v>1958</v>
       </c>
       <c r="B1233" s="68" t="s">
-        <v>1958</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="1234" spans="1:2">
       <c r="A1234" s="34" t="s">
-        <v>1959</v>
+        <v>1960</v>
       </c>
       <c r="B1234" s="68" t="s">
-        <v>1960</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="1235" spans="1:2">
       <c r="A1235" s="34" t="s">
-        <v>1961</v>
+        <v>1962</v>
       </c>
       <c r="B1235" s="35" t="s">
-        <v>1962</v>
+        <v>1963</v>
       </c>
     </row>
     <row r="1236" spans="1:2">
       <c r="A1236" s="34" t="s">
-        <v>1963</v>
+        <v>1964</v>
       </c>
       <c r="B1236" s="35" t="s">
-        <v>1964</v>
+        <v>1965</v>
       </c>
     </row>
     <row r="1237" spans="1:2">
       <c r="A1237" s="34" t="s">
-        <v>1965</v>
+        <v>1966</v>
       </c>
       <c r="B1237" s="35" t="s">
-        <v>1966</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="1238" spans="1:2">
       <c r="A1238" s="34" t="s">
-        <v>1967</v>
+        <v>1968</v>
       </c>
       <c r="B1238" s="35" t="s">
-        <v>1968</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="1239" spans="1:2">
       <c r="A1239" s="34" t="s">
+        <v>1970</v>
+      </c>
+      <c r="B1239" s="35" t="s">
         <v>1969</v>
-      </c>
-      <c r="B1239" s="35" t="s">
-        <v>1968</v>
       </c>
     </row>
     <row r="1240" spans="1:2">
       <c r="A1240" s="34" t="s">
-        <v>1970</v>
+        <v>1971</v>
       </c>
       <c r="B1240" s="35" t="s">
-        <v>1971</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="1241" spans="1:2">
       <c r="A1241" s="34" t="s">
-        <v>1972</v>
+        <v>1973</v>
       </c>
       <c r="B1241" s="35" t="s">
         <v>387</v>
@@ -19431,95 +20027,95 @@
     </row>
     <row r="1242" spans="1:2">
       <c r="A1242" s="34" t="s">
-        <v>1973</v>
+        <v>1974</v>
       </c>
       <c r="B1242" s="35" t="s">
-        <v>1974</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="1243" spans="1:2">
       <c r="A1243" s="34" t="s">
-        <v>1975</v>
+        <v>1976</v>
       </c>
       <c r="B1243" s="35" t="s">
-        <v>1976</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="1244" spans="1:2">
       <c r="A1244" s="34" t="s">
-        <v>1977</v>
+        <v>1978</v>
       </c>
       <c r="B1244" s="35" t="s">
-        <v>1978</v>
+        <v>1979</v>
       </c>
     </row>
     <row r="1245" spans="1:2">
       <c r="A1245" s="34" t="s">
-        <v>1979</v>
+        <v>1980</v>
       </c>
       <c r="B1245" s="35" t="s">
-        <v>1980</v>
+        <v>1981</v>
       </c>
     </row>
     <row r="1246" spans="1:2">
       <c r="A1246" s="34" t="s">
-        <v>1981</v>
+        <v>1982</v>
       </c>
       <c r="B1246" s="35" t="s">
-        <v>1913</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="1247" spans="1:2">
       <c r="A1247" s="34" t="s">
-        <v>1957</v>
+        <v>1958</v>
       </c>
       <c r="B1247" s="35" t="s">
-        <v>1958</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="1248" spans="1:2">
       <c r="A1248" s="34" t="s">
-        <v>1959</v>
+        <v>1960</v>
       </c>
       <c r="B1248" s="35" t="s">
-        <v>1960</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="1249" spans="1:2">
       <c r="A1249" s="34" t="s">
-        <v>1982</v>
+        <v>1983</v>
       </c>
       <c r="B1249" s="35" t="s">
-        <v>1983</v>
+        <v>1984</v>
       </c>
     </row>
     <row r="1250" spans="1:2">
       <c r="A1250" s="34" t="s">
-        <v>1984</v>
+        <v>1985</v>
       </c>
       <c r="B1250" s="35" t="s">
-        <v>1985</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="1251" spans="1:2">
       <c r="A1251" s="36" t="s">
-        <v>1986</v>
+        <v>1987</v>
       </c>
       <c r="B1251" s="37" t="s">
-        <v>1987</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="1252" spans="1:2">
       <c r="A1252" s="34" t="s">
-        <v>1988</v>
+        <v>1989</v>
       </c>
       <c r="B1252" s="35" t="s">
-        <v>1989</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="1253" spans="1:2">
       <c r="A1253" s="34" t="s">
-        <v>1990</v>
+        <v>1991</v>
       </c>
       <c r="B1253" s="35" t="s">
         <v>1798</v>
@@ -19527,23 +20123,23 @@
     </row>
     <row r="1254" spans="1:2">
       <c r="A1254" s="34" t="s">
-        <v>1991</v>
+        <v>1992</v>
       </c>
       <c r="B1254" s="35" t="s">
-        <v>1992</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="1255" spans="1:2">
       <c r="A1255" s="34" t="s">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="B1255" s="35" t="s">
-        <v>1994</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="1256" spans="1:2">
       <c r="A1256" s="34" t="s">
-        <v>1995</v>
+        <v>1996</v>
       </c>
       <c r="B1256" s="35" t="s">
         <v>570</v>
@@ -19551,7 +20147,7 @@
     </row>
     <row r="1257" spans="1:2">
       <c r="A1257" s="34" t="s">
-        <v>1996</v>
+        <v>1997</v>
       </c>
       <c r="B1257" s="35" t="s">
         <v>305</v>
@@ -19559,7 +20155,7 @@
     </row>
     <row r="1258" spans="1:2">
       <c r="A1258" s="34" t="s">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="B1258" s="35" t="s">
         <v>916</v>
@@ -19567,7 +20163,7 @@
     </row>
     <row r="1259" spans="1:2">
       <c r="A1259" s="34" t="s">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="B1259" s="35" t="s">
         <v>1412</v>
@@ -19575,55 +20171,55 @@
     </row>
     <row r="1260" spans="1:2">
       <c r="A1260" s="34" t="s">
-        <v>1999</v>
+        <v>2000</v>
       </c>
       <c r="B1260" s="35" t="s">
-        <v>2000</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="1261" spans="1:2">
       <c r="A1261" s="34" t="s">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="B1261" s="35" t="s">
-        <v>2002</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="1262" spans="1:2">
       <c r="A1262" s="34" t="s">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="B1262" s="35" t="s">
-        <v>2004</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="1263" spans="1:2">
       <c r="A1263" s="34" t="s">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="B1263" s="35" t="s">
-        <v>2006</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="1264" spans="1:2">
       <c r="A1264" s="34" t="s">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="B1264" s="35" t="s">
-        <v>2008</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="1265" spans="1:2">
       <c r="A1265" s="34" t="s">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="B1265" s="35" t="s">
-        <v>2010</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="1266" spans="1:2">
       <c r="A1266" s="34" t="s">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="B1266" s="35" t="s">
         <v>914</v>
@@ -19631,119 +20227,119 @@
     </row>
     <row r="1267" spans="1:2">
       <c r="A1267" s="34" t="s">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="B1267" s="35" t="s">
-        <v>2013</v>
+        <v>2014</v>
       </c>
     </row>
     <row r="1268" spans="1:2">
       <c r="A1268" s="34" t="s">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="B1268" s="35" t="s">
-        <v>2015</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="1269" spans="1:2">
       <c r="A1269" s="34" t="s">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="B1269" s="35" t="s">
-        <v>2017</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="1270" spans="1:2">
       <c r="A1270" s="34" t="s">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B1270" s="35" t="s">
-        <v>2019</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="1271" spans="1:2">
       <c r="A1271" s="34" t="s">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B1271" s="35" t="s">
-        <v>2021</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="1272" spans="1:2">
       <c r="A1272" s="34" t="s">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B1272" s="35" t="s">
-        <v>2023</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1273" spans="1:2">
       <c r="A1273" s="34" t="s">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B1273" s="35" t="s">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="1274" spans="1:2">
       <c r="A1274" s="34" t="s">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="B1274" s="35" t="s">
-        <v>2027</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="1275" spans="1:2">
       <c r="A1275" s="34" t="s">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="B1275" s="35" t="s">
-        <v>2029</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="1276" spans="1:2">
       <c r="A1276" s="34" t="s">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="B1276" s="35" t="s">
-        <v>2031</v>
+        <v>2032</v>
       </c>
     </row>
     <row r="1277" spans="1:2">
       <c r="A1277" s="34" t="s">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="B1277" s="35" t="s">
-        <v>2033</v>
+        <v>2034</v>
       </c>
     </row>
     <row r="1278" spans="1:2">
       <c r="A1278" s="34" t="s">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="B1278" s="35" t="s">
-        <v>2035</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="1279" spans="1:2">
       <c r="A1279" s="34" t="s">
-        <v>1876</v>
+        <v>1877</v>
       </c>
       <c r="B1279" s="35" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="1280" spans="1:2">
       <c r="A1280" s="34" t="s">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="B1280" s="35" t="s">
-        <v>2037</v>
+        <v>2038</v>
       </c>
     </row>
     <row r="1281" spans="1:2">
       <c r="A1281" s="34" t="s">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="B1281" s="35" t="s">
         <v>562</v>
@@ -19751,7 +20347,7 @@
     </row>
     <row r="1282" spans="1:2">
       <c r="A1282" s="34" t="s">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="B1282" s="35" t="s">
         <v>59</v>
@@ -19759,7 +20355,7 @@
     </row>
     <row r="1283" spans="1:2">
       <c r="A1283" s="34" t="s">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="B1283" s="35" t="s">
         <v>377</v>
@@ -19767,23 +20363,23 @@
     </row>
     <row r="1284" spans="1:2">
       <c r="A1284" s="34" t="s">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="B1284" s="35" t="s">
-        <v>2042</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="1285" spans="1:2">
       <c r="A1285" s="34" t="s">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="B1285" s="35" t="s">
-        <v>2044</v>
+        <v>2045</v>
       </c>
     </row>
     <row r="1286" spans="1:2">
       <c r="A1286" s="34" t="s">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="B1286" s="35" t="s">
         <v>715</v>
@@ -19791,39 +20387,39 @@
     </row>
     <row r="1287" spans="1:2">
       <c r="A1287" s="34" t="s">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="B1287" s="35" t="s">
-        <v>2047</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="1288" spans="1:2">
       <c r="A1288" s="34" t="s">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="B1288" s="35" t="s">
-        <v>2049</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="1289" spans="1:2">
       <c r="A1289" s="34" t="s">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="B1289" s="35" t="s">
-        <v>2051</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="1290" spans="1:2">
       <c r="A1290" s="34" t="s">
-        <v>2052</v>
+        <v>2053</v>
       </c>
       <c r="B1290" s="35" t="s">
-        <v>2053</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="1291" spans="1:2">
       <c r="A1291" s="34" t="s">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="B1291" s="35" t="s">
         <v>1580</v>
@@ -19831,31 +20427,31 @@
     </row>
     <row r="1292" spans="1:2">
       <c r="A1292" s="34" t="s">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="B1292" s="35" t="s">
-        <v>2056</v>
+        <v>2057</v>
       </c>
     </row>
     <row r="1293" spans="1:2">
       <c r="A1293" s="34" t="s">
-        <v>2057</v>
+        <v>2058</v>
       </c>
       <c r="B1293" s="35" t="s">
-        <v>2058</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="1294" spans="1:2">
       <c r="A1294" s="34" t="s">
-        <v>2059</v>
+        <v>2060</v>
       </c>
       <c r="B1294" s="35" t="s">
-        <v>2060</v>
+        <v>2061</v>
       </c>
     </row>
     <row r="1295" spans="1:2">
       <c r="A1295" s="34" t="s">
-        <v>2061</v>
+        <v>2062</v>
       </c>
       <c r="B1295" s="35" t="s">
         <v>93</v>
@@ -19863,15 +20459,15 @@
     </row>
     <row r="1296" spans="1:2">
       <c r="A1296" s="34" t="s">
-        <v>2062</v>
+        <v>2063</v>
       </c>
       <c r="B1296" s="35" t="s">
-        <v>2063</v>
+        <v>2064</v>
       </c>
     </row>
     <row r="1297" spans="1:2">
       <c r="A1297" s="34" t="s">
-        <v>2064</v>
+        <v>2065</v>
       </c>
       <c r="B1297" s="35" t="s">
         <v>566</v>
@@ -19879,7 +20475,7 @@
     </row>
     <row r="1298" spans="1:2">
       <c r="A1298" s="34" t="s">
-        <v>2065</v>
+        <v>2066</v>
       </c>
       <c r="B1298" s="35" t="s">
         <v>330</v>
@@ -19887,7 +20483,7 @@
     </row>
     <row r="1299" spans="1:2">
       <c r="A1299" s="34" t="s">
-        <v>2066</v>
+        <v>2067</v>
       </c>
       <c r="B1299" s="35" t="s">
         <v>7</v>
@@ -19895,15 +20491,15 @@
     </row>
     <row r="1300" spans="1:2">
       <c r="A1300" s="34" t="s">
-        <v>2067</v>
+        <v>2068</v>
       </c>
       <c r="B1300" s="35" t="s">
-        <v>2068</v>
+        <v>2069</v>
       </c>
     </row>
     <row r="1301" spans="1:2">
       <c r="A1301" s="34" t="s">
-        <v>2069</v>
+        <v>2070</v>
       </c>
       <c r="B1301" s="35" t="s">
         <v>223</v>
@@ -19911,15 +20507,15 @@
     </row>
     <row r="1302" spans="1:2">
       <c r="A1302" s="34" t="s">
-        <v>2070</v>
+        <v>2071</v>
       </c>
       <c r="B1302" s="35" t="s">
-        <v>2071</v>
+        <v>2072</v>
       </c>
     </row>
     <row r="1303" spans="1:2">
       <c r="A1303" s="34" t="s">
-        <v>2072</v>
+        <v>2073</v>
       </c>
       <c r="B1303" s="35" t="s">
         <v>152</v>
@@ -19927,7 +20523,7 @@
     </row>
     <row r="1304" spans="1:2">
       <c r="A1304" s="34" t="s">
-        <v>2073</v>
+        <v>2074</v>
       </c>
       <c r="B1304" s="35" t="s">
         <v>223</v>
@@ -19935,7 +20531,7 @@
     </row>
     <row r="1305" spans="1:2">
       <c r="A1305" s="34" t="s">
-        <v>2074</v>
+        <v>2075</v>
       </c>
       <c r="B1305" s="35" t="s">
         <v>223</v>
@@ -19943,127 +20539,127 @@
     </row>
     <row r="1306" spans="1:2">
       <c r="A1306" s="34" t="s">
-        <v>2075</v>
+        <v>2076</v>
       </c>
       <c r="B1306" s="35" t="s">
-        <v>2076</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="1307" spans="1:2">
       <c r="A1307" s="34" t="s">
-        <v>2077</v>
+        <v>2078</v>
       </c>
       <c r="B1307" s="35" t="s">
-        <v>1989</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="1308" spans="1:2">
       <c r="A1308" s="34" t="s">
-        <v>2078</v>
+        <v>2079</v>
       </c>
       <c r="B1308" s="35" t="s">
-        <v>2079</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="1309" spans="1:2">
       <c r="A1309" s="34" t="s">
-        <v>2080</v>
+        <v>2081</v>
       </c>
       <c r="B1309" s="35" t="s">
-        <v>2081</v>
+        <v>2082</v>
       </c>
     </row>
     <row r="1310" spans="1:2">
       <c r="A1310" s="34" t="s">
-        <v>2082</v>
+        <v>2083</v>
       </c>
       <c r="B1310" s="35" t="s">
-        <v>2083</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="1311" spans="1:2">
       <c r="A1311" s="34" t="s">
-        <v>2084</v>
+        <v>2085</v>
       </c>
       <c r="B1311" s="35" t="s">
-        <v>2085</v>
+        <v>2086</v>
       </c>
     </row>
     <row r="1312" spans="1:2">
       <c r="A1312" s="34" t="s">
-        <v>2086</v>
+        <v>2087</v>
       </c>
       <c r="B1312" s="35" t="s">
-        <v>2087</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="1313" spans="1:2">
       <c r="A1313" s="34" t="s">
-        <v>2088</v>
+        <v>2089</v>
       </c>
       <c r="B1313" s="35" t="s">
-        <v>2089</v>
+        <v>2090</v>
       </c>
     </row>
     <row r="1314" spans="1:2">
       <c r="A1314" s="34" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="B1314" s="35" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="1315" spans="1:2">
       <c r="A1315" s="34" t="s">
-        <v>2092</v>
+        <v>2093</v>
       </c>
       <c r="B1315" s="35" t="s">
-        <v>2093</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="1316" spans="1:2">
       <c r="A1316" s="34" t="s">
-        <v>2094</v>
+        <v>2095</v>
       </c>
       <c r="B1316" s="35" t="s">
-        <v>2095</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="1317" spans="1:2">
       <c r="A1317" s="34" t="s">
-        <v>2096</v>
+        <v>2097</v>
       </c>
       <c r="B1317" s="35" t="s">
-        <v>2097</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="1318" spans="1:2">
       <c r="A1318" s="34" t="s">
-        <v>2098</v>
+        <v>2099</v>
       </c>
       <c r="B1318" s="35" t="s">
-        <v>2093</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="1319" spans="1:2">
       <c r="A1319" s="34" t="s">
-        <v>2099</v>
+        <v>2100</v>
       </c>
       <c r="B1319" s="35" t="s">
-        <v>2100</v>
+        <v>2101</v>
       </c>
     </row>
     <row r="1320" spans="1:2">
       <c r="A1320" s="34" t="s">
-        <v>2101</v>
+        <v>2102</v>
       </c>
       <c r="B1320" s="35" t="s">
-        <v>2102</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="1321" spans="1:2">
       <c r="A1321" s="34" t="s">
-        <v>2103</v>
+        <v>2104</v>
       </c>
       <c r="B1321" s="35" t="s">
         <v>1630</v>
@@ -20071,31 +20667,31 @@
     </row>
     <row r="1322" spans="1:2">
       <c r="A1322" s="34" t="s">
-        <v>2104</v>
+        <v>2105</v>
       </c>
       <c r="B1322" s="35" t="s">
-        <v>2105</v>
+        <v>2106</v>
       </c>
     </row>
     <row r="1323" spans="1:2">
       <c r="A1323" s="34" t="s">
-        <v>2106</v>
+        <v>2107</v>
       </c>
       <c r="B1323" s="35" t="s">
-        <v>2107</v>
+        <v>2108</v>
       </c>
     </row>
     <row r="1324" spans="1:2">
       <c r="A1324" s="34" t="s">
-        <v>2108</v>
+        <v>2109</v>
       </c>
       <c r="B1324" s="35" t="s">
-        <v>2109</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="1325" spans="1:2">
       <c r="A1325" s="34" t="s">
-        <v>2110</v>
+        <v>2111</v>
       </c>
       <c r="B1325" s="35" t="s">
         <v>1580</v>
@@ -20103,23 +20699,23 @@
     </row>
     <row r="1326" spans="1:2">
       <c r="A1326" s="34" t="s">
-        <v>2111</v>
+        <v>2112</v>
       </c>
       <c r="B1326" s="35" t="s">
-        <v>2112</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="1327" spans="1:2">
       <c r="A1327" s="34" t="s">
-        <v>2113</v>
+        <v>2114</v>
       </c>
       <c r="B1327" s="35" t="s">
-        <v>2102</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="1328" spans="1:2">
       <c r="A1328" s="34" t="s">
-        <v>2114</v>
+        <v>2115</v>
       </c>
       <c r="B1328" s="35" t="s">
         <v>228</v>
@@ -20127,31 +20723,31 @@
     </row>
     <row r="1329" spans="1:2">
       <c r="A1329" s="34" t="s">
-        <v>2115</v>
+        <v>2116</v>
       </c>
       <c r="B1329" s="35" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
     </row>
     <row r="1330" spans="1:2">
       <c r="A1330" s="34" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
       <c r="B1330" s="35" t="s">
-        <v>2102</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="1331" spans="1:2">
       <c r="A1331" s="34" t="s">
-        <v>2118</v>
+        <v>2119</v>
       </c>
       <c r="B1331" s="35" t="s">
-        <v>2112</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="1332" spans="1:2">
       <c r="A1332" s="34" t="s">
-        <v>2119</v>
+        <v>2120</v>
       </c>
       <c r="B1332" s="35" t="s">
         <v>166</v>
@@ -20159,7 +20755,7 @@
     </row>
     <row r="1333" spans="1:2">
       <c r="A1333" s="68" t="s">
-        <v>2120</v>
+        <v>2121</v>
       </c>
       <c r="B1333" s="71" t="s">
         <v>1308</v>
@@ -20167,34 +20763,44 @@
     </row>
     <row r="1334" spans="1:2">
       <c r="A1334" s="68" t="s">
-        <v>2121</v>
+        <v>2122</v>
       </c>
       <c r="B1334" s="71" t="s">
-        <v>2122</v>
+        <v>2123</v>
       </c>
     </row>
     <row r="1335" spans="1:2">
       <c r="A1335" s="68" t="s">
-        <v>2123</v>
+        <v>2124</v>
       </c>
       <c r="B1335" s="71" t="s">
-        <v>2124</v>
+        <v>2125</v>
+      </c>
+    </row>
+    <row r="1336" spans="1:2">
+      <c r="A1336" s="34" t="s">
+        <v>2126</v>
+      </c>
+      <c r="B1336" s="35" t="s">
+        <v>2127</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1211" r:id="rId1"/>
+    <hyperlink ref="B1211" r:id="rId1" display="MRAD-2425-00086"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B63"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B62"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -20206,503 +20812,496 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="108.95" customHeight="1">
+    <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>2125</v>
+        <v>2128</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>2126</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="114" customHeight="1">
+        <v>2129</v>
+      </c>
+    </row>
+    <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>2127</v>
+        <v>2130</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="4" ht="80.25" customHeight="1" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>2132</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>2133</v>
+      </c>
+    </row>
+    <row r="5" ht="69.75" customHeight="1" spans="1:2">
+      <c r="A5" s="2" t="s">
+        <v>2134</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>2135</v>
+      </c>
+    </row>
+    <row r="6" ht="51.75" customHeight="1" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>2136</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>2137</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>2138</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>2139</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>2140</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>2141</v>
+      </c>
+    </row>
+    <row r="9" ht="39" customHeight="1" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>2142</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>2143</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1" spans="1:2">
+      <c r="A10" s="2" t="s">
+        <v>2144</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>2145</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" spans="1:2">
+      <c r="A11" s="2" t="s">
+        <v>2146</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>2147</v>
+      </c>
+    </row>
+    <row r="12" ht="26.25" customHeight="1" spans="1:2">
+      <c r="A12" s="2" t="s">
+        <v>2148</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>2149</v>
+      </c>
+    </row>
+    <row r="13" ht="28.5" customHeight="1" spans="1:2">
+      <c r="A13" s="2" t="s">
+        <v>2150</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>2151</v>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1" spans="1:2">
+      <c r="A14" s="2" t="s">
+        <v>2152</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1" spans="1:2">
+      <c r="A15" s="2" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>2155</v>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1" spans="1:2">
+      <c r="A16" s="2" t="s">
+        <v>2156</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>2157</v>
+      </c>
+    </row>
+    <row r="17" ht="43.5" customHeight="1" spans="1:2">
+      <c r="A17" s="2" t="s">
+        <v>2158</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1" spans="1:2">
+      <c r="A18" s="2" t="s">
+        <v>2160</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>2161</v>
+      </c>
+    </row>
+    <row r="19" ht="52.5" customHeight="1" spans="1:2">
+      <c r="A19" s="2" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>2163</v>
+      </c>
+    </row>
+    <row r="20" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A20" s="4" t="s">
+        <v>2164</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" spans="1:2">
+      <c r="A21" s="4" t="s">
+        <v>2166</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>2167</v>
+      </c>
+    </row>
+    <row r="22" ht="409.5" spans="1:2">
+      <c r="A22" s="2" t="s">
+        <v>2168</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="23" ht="244.8" spans="1:2">
+      <c r="A23" s="2" t="s">
+        <v>2170</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>2171</v>
+      </c>
+    </row>
+    <row r="24" ht="230.4" spans="1:2">
+      <c r="A24" t="s">
+        <v>2172</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>2173</v>
+      </c>
+    </row>
+    <row r="25" ht="259.2" spans="1:2">
+      <c r="A25" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>2175</v>
+      </c>
+    </row>
+    <row r="26" ht="201.6" spans="1:2">
+      <c r="A26" t="s">
+        <v>2176</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="27" ht="61.5" customHeight="1" spans="1:2">
+      <c r="A27" t="s">
+        <v>2178</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>2179</v>
+      </c>
+    </row>
+    <row r="28" ht="105.75" customHeight="1" spans="1:2">
+      <c r="A28" s="7" t="s">
         <v>2128</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="80.25" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="B28" s="8" t="s">
         <v>2129</v>
       </c>
-      <c r="B4" s="3" t="s">
+    </row>
+    <row r="29" ht="83.25" customHeight="1" spans="1:2">
+      <c r="A29" s="9" t="s">
+        <v>2130</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>2131</v>
+      </c>
+    </row>
+    <row r="30" ht="172.8" spans="1:2">
+      <c r="A30" s="11" t="s">
+        <v>2136</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>2137</v>
+      </c>
+    </row>
+    <row r="31" ht="129.6" spans="1:2">
+      <c r="A31" s="13" t="s">
+        <v>2180</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>2181</v>
+      </c>
+    </row>
+    <row r="32" ht="172.8" spans="1:2">
+      <c r="A32" s="15" t="s">
+        <v>2182</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>2183</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
+      <c r="A33" s="17" t="s">
+        <v>2184</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>2185</v>
+      </c>
+    </row>
+    <row r="34" ht="409.5" spans="1:2">
+      <c r="A34" s="19" t="s">
+        <v>2186</v>
+      </c>
+      <c r="B34" s="20" t="s">
+        <v>2187</v>
+      </c>
+    </row>
+    <row r="35" ht="403.2" spans="1:2">
+      <c r="A35" s="21" t="s">
+        <v>2188</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>2189</v>
+      </c>
+    </row>
+    <row r="36" ht="409.5" spans="1:2">
+      <c r="A36" s="23" t="s">
+        <v>2190</v>
+      </c>
+      <c r="B36" s="24" t="s">
+        <v>2191</v>
+      </c>
+    </row>
+    <row r="37" ht="409.5" spans="1:2">
+      <c r="A37" s="25" t="s">
+        <v>2192</v>
+      </c>
+      <c r="B37" s="26" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="38" ht="409.5" spans="1:2">
+      <c r="A38" s="27" t="s">
+        <v>2194</v>
+      </c>
+      <c r="B38" s="28" t="s">
+        <v>2195</v>
+      </c>
+    </row>
+    <row r="39" ht="409.5" spans="1:2">
+      <c r="A39" t="s">
+        <v>2196</v>
+      </c>
+      <c r="B39" s="29" t="s">
+        <v>2197</v>
+      </c>
+    </row>
+    <row r="40" ht="115.2" spans="1:2">
+      <c r="A40" t="s">
+        <v>2198</v>
+      </c>
+      <c r="B40" s="29" t="s">
+        <v>2199</v>
+      </c>
+    </row>
+    <row r="41" ht="172.8" spans="1:2">
+      <c r="A41" t="s">
+        <v>2200</v>
+      </c>
+      <c r="B41" s="29" t="s">
+        <v>2201</v>
+      </c>
+    </row>
+    <row r="42" ht="187.2" spans="1:2">
+      <c r="A42" t="s">
+        <v>2202</v>
+      </c>
+      <c r="B42" s="29" t="s">
+        <v>2203</v>
+      </c>
+    </row>
+    <row r="43" ht="115.2" spans="1:2">
+      <c r="A43" t="s">
+        <v>2204</v>
+      </c>
+      <c r="B43" s="29" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="44" ht="409.5" spans="1:2">
+      <c r="A44" t="s">
+        <v>2206</v>
+      </c>
+      <c r="B44" s="29" t="s">
+        <v>2207</v>
+      </c>
+    </row>
+    <row r="45" ht="409.5" spans="1:2">
+      <c r="A45" t="s">
+        <v>2208</v>
+      </c>
+      <c r="B45" s="29" t="s">
+        <v>2209</v>
+      </c>
+    </row>
+    <row r="46" ht="409.5" spans="1:2">
+      <c r="A46" t="s">
+        <v>2210</v>
+      </c>
+      <c r="B46" s="29" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="47" ht="259.2" spans="1:2">
+      <c r="A47" t="s">
+        <v>2212</v>
+      </c>
+      <c r="B47" s="29" t="s">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="48" ht="409.5" spans="1:2">
+      <c r="A48" t="s">
+        <v>2214</v>
+      </c>
+      <c r="B48" s="29" t="s">
+        <v>2215</v>
+      </c>
+    </row>
+    <row r="49" ht="331.2" spans="1:2">
+      <c r="A49" t="s">
+        <v>2216</v>
+      </c>
+      <c r="B49" s="29" t="s">
+        <v>2217</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
+      <c r="A50" t="s">
+        <v>2218</v>
+      </c>
+      <c r="B50" s="29" t="s">
+        <v>2219</v>
+      </c>
+    </row>
+    <row r="51" ht="36" customHeight="1" spans="1:2">
+      <c r="A51" t="s">
+        <v>2220</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>2221</v>
+      </c>
+    </row>
+    <row r="52" ht="23.25" customHeight="1" spans="1:2">
+      <c r="A52" t="s">
+        <v>2222</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>2223</v>
+      </c>
+    </row>
+    <row r="53" ht="27.75" customHeight="1" spans="1:2">
+      <c r="A53" t="s">
+        <v>2224</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>2225</v>
+      </c>
+    </row>
+    <row r="54" ht="57.6" spans="1:2">
+      <c r="A54" t="s">
+        <v>2226</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>2227</v>
+      </c>
+    </row>
+    <row r="55" ht="43.2" spans="1:2">
+      <c r="A55" t="s">
+        <v>2228</v>
+      </c>
+      <c r="B55" s="29" t="s">
+        <v>2229</v>
+      </c>
+    </row>
+    <row r="56" ht="57.6" spans="1:2">
+      <c r="A56" t="s">
+        <v>2230</v>
+      </c>
+      <c r="B56" s="29" t="s">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="57" ht="72" spans="1:2">
+      <c r="A57" t="s">
+        <v>2232</v>
+      </c>
+      <c r="B57" s="29" t="s">
+        <v>2233</v>
+      </c>
+    </row>
+    <row r="58" ht="409.5" spans="1:2">
+      <c r="A58" t="s">
+        <v>2234</v>
+      </c>
+      <c r="B58" s="29" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="59" ht="86.4" spans="1:2">
+      <c r="A59" t="s">
+        <v>2236</v>
+      </c>
+      <c r="B59" s="29" t="s">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="60" ht="345.6" spans="1:2">
+      <c r="A60" t="s">
+        <v>2238</v>
+      </c>
+      <c r="B60" s="29" t="s">
         <v>2239</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="69.75" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>2130</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="61" ht="57.6" spans="1:2">
+      <c r="A61" t="s">
         <v>2240</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="51.75" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>2131</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>2132</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="30" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>2133</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>2134</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="18" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>2135</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>2136</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="39" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>2137</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>2138</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="22.5" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>2139</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>2140</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="18" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>2141</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>2142</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="26.25" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>2143</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>2144</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="28.5" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>2145</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>2146</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="24" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>2147</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>2148</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="36" customHeight="1">
-      <c r="A15" s="2" t="s">
-        <v>2149</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>2150</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1">
-      <c r="A16" s="2" t="s">
-        <v>2151</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>2152</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="27.75" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>2153</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>2154</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="43.5" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>2155</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>2156</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="42" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>2157</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>2158</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="52.5" customHeight="1">
-      <c r="A20" s="2" t="s">
-        <v>2159</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>2160</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A21" s="4" t="s">
-        <v>2161</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>2162</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15" customHeight="1">
-      <c r="A22" s="4" t="s">
-        <v>2163</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>2164</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="409.5">
-      <c r="A23" s="2" t="s">
-        <v>2165</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>2166</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="255">
-      <c r="A24" s="2" t="s">
-        <v>2167</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>2168</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="240">
-      <c r="A25" t="s">
-        <v>2169</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>2170</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="270">
-      <c r="A26" t="s">
-        <v>2171</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>2172</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="210">
-      <c r="A27" t="s">
-        <v>2173</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>2174</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="61.5" customHeight="1">
-      <c r="A28" t="s">
-        <v>2175</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>2176</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="105.75" customHeight="1">
-      <c r="A29" s="7" t="s">
-        <v>2125</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>2126</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="83.25" customHeight="1">
-      <c r="A30" s="9" t="s">
-        <v>2127</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>2128</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="180">
-      <c r="A31" s="11" t="s">
-        <v>2131</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>2132</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="135">
-      <c r="A32" s="13" t="s">
-        <v>2177</v>
-      </c>
-      <c r="B32" s="14" t="s">
-        <v>2178</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="180">
-      <c r="A33" s="15" t="s">
-        <v>2179</v>
-      </c>
-      <c r="B33" s="16" t="s">
-        <v>2180</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="180">
-      <c r="A34" s="17" t="s">
-        <v>2181</v>
-      </c>
-      <c r="B34" s="18" t="s">
-        <v>2182</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="409.5">
-      <c r="A35" s="19" t="s">
-        <v>2153</v>
-      </c>
-      <c r="B35" s="20" t="s">
-        <v>2183</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="409.5">
-      <c r="A36" s="21" t="s">
-        <v>2184</v>
-      </c>
-      <c r="B36" s="22" t="s">
-        <v>2185</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="409.5">
-      <c r="A37" s="23" t="s">
-        <v>2186</v>
-      </c>
-      <c r="B37" s="24" t="s">
-        <v>2187</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="409.5">
-      <c r="A38" s="25" t="s">
-        <v>2188</v>
-      </c>
-      <c r="B38" s="26" t="s">
-        <v>2189</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="409.5">
-      <c r="A39" s="27" t="s">
-        <v>2190</v>
-      </c>
-      <c r="B39" s="28" t="s">
-        <v>2191</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="409.5">
-      <c r="A40" t="s">
-        <v>2192</v>
-      </c>
-      <c r="B40" s="29" t="s">
-        <v>2193</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="120">
-      <c r="A41" t="s">
-        <v>2194</v>
-      </c>
-      <c r="B41" s="29" t="s">
-        <v>2195</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="180">
-      <c r="A42" t="s">
-        <v>2196</v>
-      </c>
-      <c r="B42" s="29" t="s">
-        <v>2197</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="195">
-      <c r="A43" t="s">
-        <v>2198</v>
-      </c>
-      <c r="B43" s="29" t="s">
-        <v>2199</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="120">
-      <c r="A44" t="s">
-        <v>2200</v>
-      </c>
-      <c r="B44" s="29" t="s">
-        <v>2201</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="409.5">
-      <c r="A45" t="s">
-        <v>2202</v>
-      </c>
-      <c r="B45" s="29" t="s">
-        <v>2203</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="409.5">
-      <c r="A46" t="s">
-        <v>2204</v>
-      </c>
-      <c r="B46" s="29" t="s">
-        <v>2205</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="409.5">
-      <c r="A47" t="s">
-        <v>2206</v>
-      </c>
-      <c r="B47" s="29" t="s">
-        <v>2207</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="270">
-      <c r="A48" t="s">
-        <v>2208</v>
-      </c>
-      <c r="B48" s="29" t="s">
-        <v>2209</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="409.5">
-      <c r="A49" t="s">
-        <v>2210</v>
-      </c>
-      <c r="B49" s="29" t="s">
-        <v>2211</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="345">
-      <c r="A50" t="s">
-        <v>2212</v>
-      </c>
-      <c r="B50" s="29" t="s">
-        <v>2213</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="345">
-      <c r="A51" t="s">
-        <v>2214</v>
-      </c>
-      <c r="B51" s="29" t="s">
-        <v>2215</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="36" customHeight="1">
-      <c r="A52" t="s">
-        <v>2216</v>
-      </c>
-      <c r="B52" s="6" t="s">
+      <c r="B61" s="29" t="s">
         <v>2241</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="23.25" customHeight="1">
-      <c r="A53" t="s">
-        <v>2217</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>2218</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="27.75" customHeight="1">
-      <c r="A54" t="s">
-        <v>2219</v>
-      </c>
-      <c r="B54" s="6" t="s">
-        <v>2220</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="60">
-      <c r="A55" t="s">
-        <v>2221</v>
-      </c>
-      <c r="B55" s="6" t="s">
-        <v>2222</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="45">
-      <c r="A56" t="s">
-        <v>2223</v>
-      </c>
-      <c r="B56" s="29" t="s">
-        <v>2224</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="60">
-      <c r="A57" t="s">
-        <v>2225</v>
-      </c>
-      <c r="B57" s="29" t="s">
-        <v>2226</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="75">
-      <c r="A58" t="s">
-        <v>2227</v>
-      </c>
-      <c r="B58" s="29" t="s">
-        <v>2228</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="409.5">
-      <c r="A59" t="s">
-        <v>2229</v>
-      </c>
-      <c r="B59" s="29" t="s">
-        <v>2230</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="90">
-      <c r="A60" t="s">
-        <v>2231</v>
-      </c>
-      <c r="B60" s="29" t="s">
-        <v>2232</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="360">
-      <c r="A61" t="s">
-        <v>2233</v>
-      </c>
-      <c r="B61" s="29" t="s">
-        <v>2234</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="75">
+    <row r="62" ht="409.5" spans="1:2">
       <c r="A62" t="s">
-        <v>2235</v>
+        <v>2242</v>
       </c>
       <c r="B62" s="29" t="s">
-        <v>2236</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" ht="409.5">
-      <c r="A63" t="s">
-        <v>2237</v>
-      </c>
-      <c r="B63" s="29" t="s">
-        <v>2238</v>
+        <v>2243</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Subcontract Order Setup And Subcontract Order Function Newly Added
Subcontract Order Setup With DB Validation And Subcontract Order Function Newly Added.
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="8400" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2763" uniqueCount="2244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2819" uniqueCount="2298">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -8885,18 +8885,205 @@
     AND PRL_RQST_NO  ='${PRNO}'
     AND PRL_PROD_ID  ='${ItemId}'</t>
   </si>
+  <si>
+    <t>SCOVoutype</t>
+  </si>
+  <si>
+    <t>SCO - VAL. ADD.</t>
+  </si>
+  <si>
+    <t>ValueAdditionPFX</t>
+  </si>
+  <si>
+    <t>SV100</t>
+  </si>
+  <si>
+    <t>ProcessGLacct</t>
+  </si>
+  <si>
+    <t>CHARGES ACCOUNT</t>
+  </si>
+  <si>
+    <t>BOMITEMWITHCONVFACTOR</t>
+  </si>
+  <si>
+    <t>FG0004</t>
+  </si>
+  <si>
+    <t>BOMITEMWITHSOREF</t>
+  </si>
+  <si>
+    <t>FG20001</t>
+  </si>
+  <si>
+    <t>BOMITEMWITHSOREFANDCONV</t>
+  </si>
+  <si>
+    <t>FG30001</t>
+  </si>
+  <si>
+    <t>BOMSOREFWITHCONV</t>
+  </si>
+  <si>
+    <t>SO100/05697/25-26</t>
+  </si>
+  <si>
+    <t>BOMSOREF</t>
+  </si>
+  <si>
+    <t>SO100/05696/25-26</t>
+  </si>
+  <si>
+    <t>BOMProject</t>
+  </si>
+  <si>
+    <t>VJ-PROJECT</t>
+  </si>
+  <si>
+    <t>OSPNO</t>
+  </si>
+  <si>
+    <t>${OSPNO}</t>
+  </si>
+  <si>
+    <t>OSPDBLOCATIONCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PLNT_LOC_ID</t>
+  </si>
+  <si>
+    <t>OSPDBITEMCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PROD_ID</t>
+  </si>
+  <si>
+    <t>OSPDBTYPECOLUMN</t>
+  </si>
+  <si>
+    <t>LVL_TYPE</t>
+  </si>
+  <si>
+    <t>OSPDBPFXCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PO_PFX</t>
+  </si>
+  <si>
+    <t>OSPDBDOCNOCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PO_NO</t>
+  </si>
+  <si>
+    <t>OSPDBDATECOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PO_DATE</t>
+  </si>
+  <si>
+    <t>OSPDBSTATUSCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_STATUS</t>
+  </si>
+  <si>
+    <t>OSPDBUNITCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCLN_PLNT</t>
+  </si>
+  <si>
+    <t>OSPDBUOMCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCLN_UOM</t>
+  </si>
+  <si>
+    <t>OSPDBBATCHQTYCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCLN_BATCH_QTY</t>
+  </si>
+  <si>
+    <t>OSPDBBATCHCOSTCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCLN_UNIT_COST</t>
+  </si>
+  <si>
+    <t>OSPDBPROCESSCOLUMN</t>
+  </si>
+  <si>
+    <t>PROCESS_DESC</t>
+  </si>
+  <si>
+    <t>OSPDBSUPPLIERIDCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_SUPLR_ID</t>
+  </si>
+  <si>
+    <t>OpenSCOApprovedstatus</t>
+  </si>
+  <si>
+    <t>OpenSCOCancelledstatus</t>
+  </si>
+  <si>
+    <t>OpenSCORevisedstatus</t>
+  </si>
+  <si>
+    <t>Revised</t>
+  </si>
+  <si>
+    <t>OSPHeaderQuery</t>
+  </si>
+  <si>
+    <t>SELECT SPRCHD_PLNT_LOC_ID,
+SPRCHD_PROD_ID,
+SPRCHD_LVL_TYPE,
+SPRCHD_PO_PFX,
+SPRCHD_PO_DATE,
+SPRCHD_SUPLR_ID,
+       CASE WHEN SPRCHD_STATUS = 'N' THEN 'Draft'
+            WHEN SPRCHD_STATUS = 'R' THEN 'Revised'
+            WHEN SPRCHD_STATUS = 'E' THEN 'Entry Completed'
+            WHEN SPRCHD_STATUS = 'A' THEN 'Approved'
+            WHEN SPRCHD_STATUS = 'C' THEN 'Cancelled'
+       END SPRCHD_STATUS,
+              CASE WHEN SPRCHD_LVL_TYPE = 'SIP' THEN 'Supplier + Item + Process'
+            WHEN SPRCHD_LVL_TYPE = 'SP'  THEN 'Supplier + Process'
+            WHEN SPRCHD_LVL_TYPE = 'IP'  THEN 'Item + Process'
+            WHEN SPRCHD_LVL_TYPE = 'P'   THEN 'Process'
+       END LVL_TYPE
+  FROM subctr_proc_rate_contr_hd
+ WHERE sprchd_bu = 'TVSA'
+   AND sprchd_po_no = '${OSPNO}'</t>
+  </si>
+  <si>
+    <t>OSPLineQuery</t>
+  </si>
+  <si>
+    <t>SELECT 
+SPRCLN_UOM,
+SPRCLN_BATCH_QTY,
+SPRCLN_UNIT_COST,
+           func_find_mfg_oper_desc(sprchd_bu,sprchd_plnt,sprcln_proc_id,1) process_desc
+  FROM subctr_proc_rate_contr_hd,
+       subctr_proc_rate_contr_ln  
+ WHERE sprchd_bu = sprcln_bu
+   AND sprchd_plnt = sprcln_plnt 
+   AND sprchd_po_pfx = sprcln_po_pfx
+   AND sprchd_po_no = sprcln_po_no 
+   AND sprchd_bu = 'TVSA'
+AND sprchd_po_no = '${OSPNO}'</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="26">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8943,151 +9130,14 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -9112,194 +9162,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -9335,268 +9199,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="66">
+  <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -9614,48 +9236,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="15" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="64" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="64" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="16" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="16" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="53"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -9684,15 +9306,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -9712,11 +9334,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -9730,19 +9352,19 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="59" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="60" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -9754,74 +9376,27 @@
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="66">
+  <cellStyles count="18">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 10" xfId="49"/>
-    <cellStyle name="Normal 11" xfId="50"/>
-    <cellStyle name="Normal 13" xfId="51"/>
-    <cellStyle name="Normal 14" xfId="52"/>
-    <cellStyle name="Normal 15" xfId="53"/>
-    <cellStyle name="Normal 16" xfId="54"/>
-    <cellStyle name="Normal 17" xfId="55"/>
-    <cellStyle name="Normal 18" xfId="56"/>
-    <cellStyle name="Normal 19" xfId="57"/>
-    <cellStyle name="Normal 2" xfId="58"/>
-    <cellStyle name="Normal 2 2" xfId="59"/>
-    <cellStyle name="Normal 2 3" xfId="60"/>
-    <cellStyle name="Normal 20" xfId="61"/>
-    <cellStyle name="Normal 3" xfId="62"/>
-    <cellStyle name="Normal 7" xfId="63"/>
-    <cellStyle name="Normal 8" xfId="64"/>
-    <cellStyle name="Normal 9" xfId="65"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Normal 11" xfId="2"/>
+    <cellStyle name="Normal 13" xfId="3"/>
+    <cellStyle name="Normal 14" xfId="4"/>
+    <cellStyle name="Normal 15" xfId="5"/>
+    <cellStyle name="Normal 16" xfId="6"/>
+    <cellStyle name="Normal 17" xfId="7"/>
+    <cellStyle name="Normal 18" xfId="8"/>
+    <cellStyle name="Normal 19" xfId="9"/>
+    <cellStyle name="Normal 2" xfId="10"/>
+    <cellStyle name="Normal 2 2" xfId="11"/>
+    <cellStyle name="Normal 2 3" xfId="12"/>
+    <cellStyle name="Normal 20" xfId="13"/>
+    <cellStyle name="Normal 3" xfId="14"/>
+    <cellStyle name="Normal 7" xfId="15"/>
+    <cellStyle name="Normal 8" xfId="16"/>
+    <cellStyle name="Normal 9" xfId="17"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -10083,17 +9658,17 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B1336"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B1362"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.85546875" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -20785,22 +20360,228 @@
         <v>2127</v>
       </c>
     </row>
+    <row r="1337" spans="1:2">
+      <c r="A1337" s="30" t="s">
+        <v>2244</v>
+      </c>
+      <c r="B1337" s="31" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="1338" spans="1:2">
+      <c r="A1338" s="30" t="s">
+        <v>2246</v>
+      </c>
+      <c r="B1338" s="31" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="1339" spans="1:2">
+      <c r="A1339" s="30" t="s">
+        <v>2248</v>
+      </c>
+      <c r="B1339" s="31" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="1340" spans="1:2">
+      <c r="A1340" s="30" t="s">
+        <v>2250</v>
+      </c>
+      <c r="B1340" s="31" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="1341" spans="1:2">
+      <c r="A1341" s="30" t="s">
+        <v>2252</v>
+      </c>
+      <c r="B1341" s="31" t="s">
+        <v>2253</v>
+      </c>
+    </row>
+    <row r="1342" spans="1:2">
+      <c r="A1342" s="30" t="s">
+        <v>2254</v>
+      </c>
+      <c r="B1342" s="31" t="s">
+        <v>2255</v>
+      </c>
+    </row>
+    <row r="1343" spans="1:2">
+      <c r="A1343" s="30" t="s">
+        <v>2256</v>
+      </c>
+      <c r="B1343" s="31" t="s">
+        <v>2257</v>
+      </c>
+    </row>
+    <row r="1344" spans="1:2">
+      <c r="A1344" s="30" t="s">
+        <v>2258</v>
+      </c>
+      <c r="B1344" s="31" t="s">
+        <v>2259</v>
+      </c>
+    </row>
+    <row r="1345" spans="1:2">
+      <c r="A1345" s="30" t="s">
+        <v>2260</v>
+      </c>
+      <c r="B1345" s="31" t="s">
+        <v>2261</v>
+      </c>
+    </row>
+    <row r="1346" spans="1:2">
+      <c r="A1346" s="30" t="s">
+        <v>2262</v>
+      </c>
+      <c r="B1346" s="31" t="s">
+        <v>2263</v>
+      </c>
+    </row>
+    <row r="1347" spans="1:2">
+      <c r="A1347" s="30" t="s">
+        <v>2264</v>
+      </c>
+      <c r="B1347" s="31" t="s">
+        <v>2265</v>
+      </c>
+    </row>
+    <row r="1348" spans="1:2">
+      <c r="A1348" s="30" t="s">
+        <v>2266</v>
+      </c>
+      <c r="B1348" s="31" t="s">
+        <v>2267</v>
+      </c>
+    </row>
+    <row r="1349" spans="1:2">
+      <c r="A1349" s="30" t="s">
+        <v>2268</v>
+      </c>
+      <c r="B1349" s="31" t="s">
+        <v>2269</v>
+      </c>
+    </row>
+    <row r="1350" spans="1:2">
+      <c r="A1350" s="30" t="s">
+        <v>2270</v>
+      </c>
+      <c r="B1350" s="31" t="s">
+        <v>2271</v>
+      </c>
+    </row>
+    <row r="1351" spans="1:2">
+      <c r="A1351" s="30" t="s">
+        <v>2272</v>
+      </c>
+      <c r="B1351" s="31" t="s">
+        <v>2273</v>
+      </c>
+    </row>
+    <row r="1352" spans="1:2">
+      <c r="A1352" s="30" t="s">
+        <v>2274</v>
+      </c>
+      <c r="B1352" s="31" t="s">
+        <v>2275</v>
+      </c>
+    </row>
+    <row r="1353" spans="1:2">
+      <c r="A1353" s="30" t="s">
+        <v>2276</v>
+      </c>
+      <c r="B1353" s="31" t="s">
+        <v>2277</v>
+      </c>
+    </row>
+    <row r="1354" spans="1:2">
+      <c r="A1354" s="30" t="s">
+        <v>2278</v>
+      </c>
+      <c r="B1354" s="31" t="s">
+        <v>2279</v>
+      </c>
+    </row>
+    <row r="1355" spans="1:2">
+      <c r="A1355" s="30" t="s">
+        <v>2280</v>
+      </c>
+      <c r="B1355" s="31" t="s">
+        <v>2281</v>
+      </c>
+    </row>
+    <row r="1356" spans="1:2">
+      <c r="A1356" s="30" t="s">
+        <v>2282</v>
+      </c>
+      <c r="B1356" s="31" t="s">
+        <v>2283</v>
+      </c>
+    </row>
+    <row r="1357" spans="1:2">
+      <c r="A1357" s="30" t="s">
+        <v>2284</v>
+      </c>
+      <c r="B1357" s="31" t="s">
+        <v>2285</v>
+      </c>
+    </row>
+    <row r="1358" spans="1:2">
+      <c r="A1358" s="30" t="s">
+        <v>2286</v>
+      </c>
+      <c r="B1358" s="31" t="s">
+        <v>2287</v>
+      </c>
+    </row>
+    <row r="1359" spans="1:2">
+      <c r="A1359" s="30" t="s">
+        <v>2288</v>
+      </c>
+      <c r="B1359" s="31" t="s">
+        <v>2289</v>
+      </c>
+    </row>
+    <row r="1360" spans="1:2">
+      <c r="A1360" s="30" t="s">
+        <v>2290</v>
+      </c>
+      <c r="B1360" s="31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1361" spans="1:2">
+      <c r="A1361" s="30" t="s">
+        <v>2291</v>
+      </c>
+      <c r="B1361" s="31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1362" spans="1:2">
+      <c r="A1362" s="30" t="s">
+        <v>2292</v>
+      </c>
+      <c r="B1362" s="31" t="s">
+        <v>2293</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1211" r:id="rId1" display="MRAD-2425-00086"/>
+    <hyperlink ref="B1211" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B62"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B65"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -20812,7 +20593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="108.95" customHeight="1" spans="1:2">
+    <row r="2" spans="1:2" ht="108.95" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2128</v>
       </c>
@@ -20820,7 +20601,7 @@
         <v>2129</v>
       </c>
     </row>
-    <row r="3" ht="114" customHeight="1" spans="1:2">
+    <row r="3" spans="1:2" ht="114" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>2130</v>
       </c>
@@ -20828,7 +20609,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="4" ht="80.25" customHeight="1" spans="1:2">
+    <row r="4" spans="1:2" ht="80.25" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>2132</v>
       </c>
@@ -20836,7 +20617,7 @@
         <v>2133</v>
       </c>
     </row>
-    <row r="5" ht="69.75" customHeight="1" spans="1:2">
+    <row r="5" spans="1:2" ht="69.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2134</v>
       </c>
@@ -20844,7 +20625,7 @@
         <v>2135</v>
       </c>
     </row>
-    <row r="6" ht="51.75" customHeight="1" spans="1:2">
+    <row r="6" spans="1:2" ht="51.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>2136</v>
       </c>
@@ -20852,7 +20633,7 @@
         <v>2137</v>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" spans="1:2">
+    <row r="7" spans="1:2" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>2138</v>
       </c>
@@ -20860,7 +20641,7 @@
         <v>2139</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:2">
+    <row r="8" spans="1:2" ht="18" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>2140</v>
       </c>
@@ -20868,7 +20649,7 @@
         <v>2141</v>
       </c>
     </row>
-    <row r="9" ht="39" customHeight="1" spans="1:2">
+    <row r="9" spans="1:2" ht="39" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>2142</v>
       </c>
@@ -20876,7 +20657,7 @@
         <v>2143</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1" spans="1:2">
+    <row r="10" spans="1:2" ht="22.5" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>2144</v>
       </c>
@@ -20884,7 +20665,7 @@
         <v>2145</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" spans="1:2">
+    <row r="11" spans="1:2" ht="18" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>2146</v>
       </c>
@@ -20892,7 +20673,7 @@
         <v>2147</v>
       </c>
     </row>
-    <row r="12" ht="26.25" customHeight="1" spans="1:2">
+    <row r="12" spans="1:2" ht="26.25" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>2148</v>
       </c>
@@ -20900,7 +20681,7 @@
         <v>2149</v>
       </c>
     </row>
-    <row r="13" ht="28.5" customHeight="1" spans="1:2">
+    <row r="13" spans="1:2" ht="28.5" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>2150</v>
       </c>
@@ -20908,7 +20689,7 @@
         <v>2151</v>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" spans="1:2">
+    <row r="14" spans="1:2" ht="24" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>2152</v>
       </c>
@@ -20916,7 +20697,7 @@
         <v>2153</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:2">
+    <row r="15" spans="1:2" ht="36" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>2154</v>
       </c>
@@ -20924,7 +20705,7 @@
         <v>2155</v>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1" spans="1:2">
+    <row r="16" spans="1:2" ht="45" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>2156</v>
       </c>
@@ -20932,7 +20713,7 @@
         <v>2157</v>
       </c>
     </row>
-    <row r="17" ht="43.5" customHeight="1" spans="1:2">
+    <row r="17" spans="1:2" ht="43.5" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>2158</v>
       </c>
@@ -20940,7 +20721,7 @@
         <v>2159</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1" spans="1:2">
+    <row r="18" spans="1:2" ht="42" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>2160</v>
       </c>
@@ -20948,7 +20729,7 @@
         <v>2161</v>
       </c>
     </row>
-    <row r="19" ht="52.5" customHeight="1" spans="1:2">
+    <row r="19" spans="1:2" ht="52.5" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>2162</v>
       </c>
@@ -20956,7 +20737,7 @@
         <v>2163</v>
       </c>
     </row>
-    <row r="20" ht="17.25" customHeight="1" spans="1:2">
+    <row r="20" spans="1:2" ht="17.25" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>2164</v>
       </c>
@@ -20964,7 +20745,7 @@
         <v>2165</v>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:2">
+    <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>2166</v>
       </c>
@@ -20972,7 +20753,7 @@
         <v>2167</v>
       </c>
     </row>
-    <row r="22" ht="409.5" spans="1:2">
+    <row r="22" spans="1:2" ht="409.5">
       <c r="A22" s="2" t="s">
         <v>2168</v>
       </c>
@@ -20980,7 +20761,7 @@
         <v>2169</v>
       </c>
     </row>
-    <row r="23" ht="244.8" spans="1:2">
+    <row r="23" spans="1:2" ht="255">
       <c r="A23" s="2" t="s">
         <v>2170</v>
       </c>
@@ -20988,7 +20769,7 @@
         <v>2171</v>
       </c>
     </row>
-    <row r="24" ht="230.4" spans="1:2">
+    <row r="24" spans="1:2" ht="240">
       <c r="A24" t="s">
         <v>2172</v>
       </c>
@@ -20996,7 +20777,7 @@
         <v>2173</v>
       </c>
     </row>
-    <row r="25" ht="259.2" spans="1:2">
+    <row r="25" spans="1:2" ht="270">
       <c r="A25" t="s">
         <v>2174</v>
       </c>
@@ -21004,7 +20785,7 @@
         <v>2175</v>
       </c>
     </row>
-    <row r="26" ht="201.6" spans="1:2">
+    <row r="26" spans="1:2" ht="210">
       <c r="A26" t="s">
         <v>2176</v>
       </c>
@@ -21012,7 +20793,7 @@
         <v>2177</v>
       </c>
     </row>
-    <row r="27" ht="61.5" customHeight="1" spans="1:2">
+    <row r="27" spans="1:2" ht="61.5" customHeight="1">
       <c r="A27" t="s">
         <v>2178</v>
       </c>
@@ -21020,7 +20801,7 @@
         <v>2179</v>
       </c>
     </row>
-    <row r="28" ht="105.75" customHeight="1" spans="1:2">
+    <row r="28" spans="1:2" ht="105.75" customHeight="1">
       <c r="A28" s="7" t="s">
         <v>2128</v>
       </c>
@@ -21028,7 +20809,7 @@
         <v>2129</v>
       </c>
     </row>
-    <row r="29" ht="83.25" customHeight="1" spans="1:2">
+    <row r="29" spans="1:2" ht="83.25" customHeight="1">
       <c r="A29" s="9" t="s">
         <v>2130</v>
       </c>
@@ -21036,7 +20817,7 @@
         <v>2131</v>
       </c>
     </row>
-    <row r="30" ht="172.8" spans="1:2">
+    <row r="30" spans="1:2" ht="180">
       <c r="A30" s="11" t="s">
         <v>2136</v>
       </c>
@@ -21044,7 +20825,7 @@
         <v>2137</v>
       </c>
     </row>
-    <row r="31" ht="129.6" spans="1:2">
+    <row r="31" spans="1:2" ht="135">
       <c r="A31" s="13" t="s">
         <v>2180</v>
       </c>
@@ -21052,7 +20833,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="32" ht="172.8" spans="1:2">
+    <row r="32" spans="1:2" ht="180">
       <c r="A32" s="15" t="s">
         <v>2182</v>
       </c>
@@ -21060,7 +20841,7 @@
         <v>2183</v>
       </c>
     </row>
-    <row r="33" ht="172.8" spans="1:2">
+    <row r="33" spans="1:2" ht="180">
       <c r="A33" s="17" t="s">
         <v>2184</v>
       </c>
@@ -21068,7 +20849,7 @@
         <v>2185</v>
       </c>
     </row>
-    <row r="34" ht="409.5" spans="1:2">
+    <row r="34" spans="1:2" ht="409.5">
       <c r="A34" s="19" t="s">
         <v>2186</v>
       </c>
@@ -21076,7 +20857,7 @@
         <v>2187</v>
       </c>
     </row>
-    <row r="35" ht="403.2" spans="1:2">
+    <row r="35" spans="1:2" ht="409.5">
       <c r="A35" s="21" t="s">
         <v>2188</v>
       </c>
@@ -21084,7 +20865,7 @@
         <v>2189</v>
       </c>
     </row>
-    <row r="36" ht="409.5" spans="1:2">
+    <row r="36" spans="1:2" ht="409.5">
       <c r="A36" s="23" t="s">
         <v>2190</v>
       </c>
@@ -21092,7 +20873,7 @@
         <v>2191</v>
       </c>
     </row>
-    <row r="37" ht="409.5" spans="1:2">
+    <row r="37" spans="1:2" ht="409.5">
       <c r="A37" s="25" t="s">
         <v>2192</v>
       </c>
@@ -21100,7 +20881,7 @@
         <v>2193</v>
       </c>
     </row>
-    <row r="38" ht="409.5" spans="1:2">
+    <row r="38" spans="1:2" ht="409.5">
       <c r="A38" s="27" t="s">
         <v>2194</v>
       </c>
@@ -21108,7 +20889,7 @@
         <v>2195</v>
       </c>
     </row>
-    <row r="39" ht="409.5" spans="1:2">
+    <row r="39" spans="1:2" ht="409.5">
       <c r="A39" t="s">
         <v>2196</v>
       </c>
@@ -21116,7 +20897,7 @@
         <v>2197</v>
       </c>
     </row>
-    <row r="40" ht="115.2" spans="1:2">
+    <row r="40" spans="1:2" ht="120">
       <c r="A40" t="s">
         <v>2198</v>
       </c>
@@ -21124,7 +20905,7 @@
         <v>2199</v>
       </c>
     </row>
-    <row r="41" ht="172.8" spans="1:2">
+    <row r="41" spans="1:2" ht="180">
       <c r="A41" t="s">
         <v>2200</v>
       </c>
@@ -21132,7 +20913,7 @@
         <v>2201</v>
       </c>
     </row>
-    <row r="42" ht="187.2" spans="1:2">
+    <row r="42" spans="1:2" ht="195">
       <c r="A42" t="s">
         <v>2202</v>
       </c>
@@ -21140,7 +20921,7 @@
         <v>2203</v>
       </c>
     </row>
-    <row r="43" ht="115.2" spans="1:2">
+    <row r="43" spans="1:2" ht="120">
       <c r="A43" t="s">
         <v>2204</v>
       </c>
@@ -21148,7 +20929,7 @@
         <v>2205</v>
       </c>
     </row>
-    <row r="44" ht="409.5" spans="1:2">
+    <row r="44" spans="1:2" ht="409.5">
       <c r="A44" t="s">
         <v>2206</v>
       </c>
@@ -21156,7 +20937,7 @@
         <v>2207</v>
       </c>
     </row>
-    <row r="45" ht="409.5" spans="1:2">
+    <row r="45" spans="1:2" ht="409.5">
       <c r="A45" t="s">
         <v>2208</v>
       </c>
@@ -21164,7 +20945,7 @@
         <v>2209</v>
       </c>
     </row>
-    <row r="46" ht="409.5" spans="1:2">
+    <row r="46" spans="1:2" ht="409.5">
       <c r="A46" t="s">
         <v>2210</v>
       </c>
@@ -21172,7 +20953,7 @@
         <v>2211</v>
       </c>
     </row>
-    <row r="47" ht="259.2" spans="1:2">
+    <row r="47" spans="1:2" ht="270">
       <c r="A47" t="s">
         <v>2212</v>
       </c>
@@ -21180,7 +20961,7 @@
         <v>2213</v>
       </c>
     </row>
-    <row r="48" ht="409.5" spans="1:2">
+    <row r="48" spans="1:2" ht="409.5">
       <c r="A48" t="s">
         <v>2214</v>
       </c>
@@ -21188,7 +20969,7 @@
         <v>2215</v>
       </c>
     </row>
-    <row r="49" ht="331.2" spans="1:2">
+    <row r="49" spans="1:2" ht="345">
       <c r="A49" t="s">
         <v>2216</v>
       </c>
@@ -21196,7 +20977,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="50" ht="331.2" spans="1:2">
+    <row r="50" spans="1:2" ht="345">
       <c r="A50" t="s">
         <v>2218</v>
       </c>
@@ -21204,7 +20985,7 @@
         <v>2219</v>
       </c>
     </row>
-    <row r="51" ht="36" customHeight="1" spans="1:2">
+    <row r="51" spans="1:2" ht="36" customHeight="1">
       <c r="A51" t="s">
         <v>2220</v>
       </c>
@@ -21212,7 +20993,7 @@
         <v>2221</v>
       </c>
     </row>
-    <row r="52" ht="23.25" customHeight="1" spans="1:2">
+    <row r="52" spans="1:2" ht="23.25" customHeight="1">
       <c r="A52" t="s">
         <v>2222</v>
       </c>
@@ -21220,7 +21001,7 @@
         <v>2223</v>
       </c>
     </row>
-    <row r="53" ht="27.75" customHeight="1" spans="1:2">
+    <row r="53" spans="1:2" ht="27.75" customHeight="1">
       <c r="A53" t="s">
         <v>2224</v>
       </c>
@@ -21228,7 +21009,7 @@
         <v>2225</v>
       </c>
     </row>
-    <row r="54" ht="57.6" spans="1:2">
+    <row r="54" spans="1:2" ht="60">
       <c r="A54" t="s">
         <v>2226</v>
       </c>
@@ -21236,7 +21017,7 @@
         <v>2227</v>
       </c>
     </row>
-    <row r="55" ht="43.2" spans="1:2">
+    <row r="55" spans="1:2" ht="45">
       <c r="A55" t="s">
         <v>2228</v>
       </c>
@@ -21244,7 +21025,7 @@
         <v>2229</v>
       </c>
     </row>
-    <row r="56" ht="57.6" spans="1:2">
+    <row r="56" spans="1:2" ht="60">
       <c r="A56" t="s">
         <v>2230</v>
       </c>
@@ -21252,7 +21033,7 @@
         <v>2231</v>
       </c>
     </row>
-    <row r="57" ht="72" spans="1:2">
+    <row r="57" spans="1:2" ht="75">
       <c r="A57" t="s">
         <v>2232</v>
       </c>
@@ -21260,7 +21041,7 @@
         <v>2233</v>
       </c>
     </row>
-    <row r="58" ht="409.5" spans="1:2">
+    <row r="58" spans="1:2" ht="409.5">
       <c r="A58" t="s">
         <v>2234</v>
       </c>
@@ -21268,7 +21049,7 @@
         <v>2235</v>
       </c>
     </row>
-    <row r="59" ht="86.4" spans="1:2">
+    <row r="59" spans="1:2" ht="90">
       <c r="A59" t="s">
         <v>2236</v>
       </c>
@@ -21276,7 +21057,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="60" ht="345.6" spans="1:2">
+    <row r="60" spans="1:2" ht="360">
       <c r="A60" t="s">
         <v>2238</v>
       </c>
@@ -21284,7 +21065,7 @@
         <v>2239</v>
       </c>
     </row>
-    <row r="61" ht="57.6" spans="1:2">
+    <row r="61" spans="1:2" ht="75">
       <c r="A61" t="s">
         <v>2240</v>
       </c>
@@ -21292,7 +21073,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="62" ht="409.5" spans="1:2">
+    <row r="62" spans="1:2" ht="409.5">
       <c r="A62" t="s">
         <v>2242</v>
       </c>
@@ -21300,8 +21081,24 @@
         <v>2243</v>
       </c>
     </row>
+    <row r="63" spans="1:2" ht="87.75" customHeight="1">
+      <c r="A63" t="s">
+        <v>2294</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>2295</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="71.25" customHeight="1">
+      <c r="A64" t="s">
+        <v>2296</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>2297</v>
+      </c>
+    </row>
+    <row r="65" ht="15.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Locators Updated For Direct GRN RFQ Pricelist
Locators Updated For Direct GRN RFQ Pricelist
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2819" uniqueCount="2298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2833" uniqueCount="2306">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -9078,6 +9078,30 @@
    AND sprchd_bu = 'TVSA'
 AND sprchd_po_no = '${OSPNO}'</t>
   </si>
+  <si>
+    <t>PRLNumber</t>
+  </si>
+  <si>
+    <t>PRL10/00665/25-26</t>
+  </si>
+  <si>
+    <t>PRLItem</t>
+  </si>
+  <si>
+    <t>TVS-AMD-SIM-651631</t>
+  </si>
+  <si>
+    <t>AmendedStatus</t>
+  </si>
+  <si>
+    <t>RFQNumber</t>
+  </si>
+  <si>
+    <t>RFQ10/00725/25-26</t>
+  </si>
+  <si>
+    <t>Rfqitem</t>
+  </si>
 </sst>
 </file>
 
@@ -9096,44 +9120,44 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="14"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="14"/>
       <color rgb="FF262626"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -9664,7 +9688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1362"/>
+  <dimension ref="A1:B1368"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
@@ -20568,9 +20592,58 @@
         <v>2293</v>
       </c>
     </row>
+    <row r="1363" spans="1:2">
+      <c r="A1363" s="30" t="s">
+        <v>2298</v>
+      </c>
+      <c r="B1363" s="31" t="s">
+        <v>2299</v>
+      </c>
+    </row>
+    <row r="1364" spans="1:2">
+      <c r="A1364" s="30" t="s">
+        <v>2300</v>
+      </c>
+      <c r="B1364" s="31" t="s">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="1365" spans="1:2">
+      <c r="A1365" s="30" t="s">
+        <v>2302</v>
+      </c>
+      <c r="B1365" s="31" t="s">
+        <v>2036</v>
+      </c>
+    </row>
+    <row r="1366" spans="1:2">
+      <c r="A1366" s="30" t="s">
+        <v>2303</v>
+      </c>
+      <c r="B1366" s="30" t="s">
+        <v>2304</v>
+      </c>
+    </row>
+    <row r="1367" spans="1:2">
+      <c r="A1367" s="30" t="s">
+        <v>2305</v>
+      </c>
+      <c r="B1367" s="30" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:2">
+      <c r="A1368" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1368" s="30" t="s">
+        <v>193</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B1211" r:id="rId1"/>
+    <hyperlink ref="B1366" r:id="rId2" display="javascript:$s('P1615131058_RFQHD_RFQ_PFX','RFQ10');$s('P1615131058_RFQHD_RFQ_NO','RFQ10/00725/25-26');$s('P1615131058_RFQHD_STATUS','A');apex.submit('RFQ');"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21097,7 +21170,14 @@
         <v>2297</v>
       </c>
     </row>
-    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="65" spans="1:2" ht="54" customHeight="1">
+      <c r="A65" t="s">
+        <v>2202</v>
+      </c>
+      <c r="B65" s="29" t="s">
+        <v>2203</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
navigation screen , config properties ,  locators changes and modification in scrpit
navigation screen , config properties ,
locators changes and modification in script , common UL locators ,catalogue , price list , std customer items changes and locators fixes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="8400" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="125725"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2833" uniqueCount="2306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2845" uniqueCount="2317">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -9102,12 +9102,45 @@
   <si>
     <t>Rfqitem</t>
   </si>
+  <si>
+    <t>UTGST_cus</t>
+  </si>
+  <si>
+    <t>A2B HOTEL MANAGEMENT</t>
+  </si>
+  <si>
+    <t>Open_So_Amd_Ex_Doc</t>
+  </si>
+  <si>
+    <t>OPSO1/00639/25-26</t>
+  </si>
+  <si>
+    <t>Open_So_Amd_Utgst_Doc</t>
+  </si>
+  <si>
+    <t>OSO7-2526-00003</t>
+  </si>
+  <si>
+    <t>Open_So_Amd_Interstate_Doc</t>
+  </si>
+  <si>
+    <t>OPSO1/00665/25-26</t>
+  </si>
+  <si>
+    <t>Open_So_Amd_Dom_Cus</t>
+  </si>
+  <si>
+    <t>OPSO1/00696/25-26</t>
+  </si>
+  <si>
+    <t>Openso_Price</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9159,6 +9192,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="5">
@@ -9244,7 +9283,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9397,6 +9436,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -9688,7 +9731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1368"/>
+  <dimension ref="A1:B1374"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
@@ -20385,259 +20428,307 @@
       </c>
     </row>
     <row r="1337" spans="1:2">
-      <c r="A1337" s="30" t="s">
+      <c r="A1337" s="34" t="s">
         <v>2244</v>
       </c>
-      <c r="B1337" s="31" t="s">
+      <c r="B1337" s="35" t="s">
         <v>2245</v>
       </c>
     </row>
     <row r="1338" spans="1:2">
-      <c r="A1338" s="30" t="s">
+      <c r="A1338" s="34" t="s">
         <v>2246</v>
       </c>
-      <c r="B1338" s="31" t="s">
+      <c r="B1338" s="35" t="s">
         <v>2247</v>
       </c>
     </row>
     <row r="1339" spans="1:2">
-      <c r="A1339" s="30" t="s">
+      <c r="A1339" s="34" t="s">
         <v>2248</v>
       </c>
-      <c r="B1339" s="31" t="s">
+      <c r="B1339" s="35" t="s">
         <v>2249</v>
       </c>
     </row>
     <row r="1340" spans="1:2">
-      <c r="A1340" s="30" t="s">
+      <c r="A1340" s="34" t="s">
         <v>2250</v>
       </c>
-      <c r="B1340" s="31" t="s">
+      <c r="B1340" s="35" t="s">
         <v>2251</v>
       </c>
     </row>
     <row r="1341" spans="1:2">
-      <c r="A1341" s="30" t="s">
+      <c r="A1341" s="34" t="s">
         <v>2252</v>
       </c>
-      <c r="B1341" s="31" t="s">
+      <c r="B1341" s="35" t="s">
         <v>2253</v>
       </c>
     </row>
     <row r="1342" spans="1:2">
-      <c r="A1342" s="30" t="s">
+      <c r="A1342" s="34" t="s">
         <v>2254</v>
       </c>
-      <c r="B1342" s="31" t="s">
+      <c r="B1342" s="35" t="s">
         <v>2255</v>
       </c>
     </row>
     <row r="1343" spans="1:2">
-      <c r="A1343" s="30" t="s">
+      <c r="A1343" s="34" t="s">
         <v>2256</v>
       </c>
-      <c r="B1343" s="31" t="s">
+      <c r="B1343" s="35" t="s">
         <v>2257</v>
       </c>
     </row>
     <row r="1344" spans="1:2">
-      <c r="A1344" s="30" t="s">
+      <c r="A1344" s="34" t="s">
         <v>2258</v>
       </c>
-      <c r="B1344" s="31" t="s">
+      <c r="B1344" s="35" t="s">
         <v>2259</v>
       </c>
     </row>
     <row r="1345" spans="1:2">
-      <c r="A1345" s="30" t="s">
+      <c r="A1345" s="34" t="s">
         <v>2260</v>
       </c>
-      <c r="B1345" s="31" t="s">
+      <c r="B1345" s="35" t="s">
         <v>2261</v>
       </c>
     </row>
     <row r="1346" spans="1:2">
-      <c r="A1346" s="30" t="s">
+      <c r="A1346" s="34" t="s">
         <v>2262</v>
       </c>
-      <c r="B1346" s="31" t="s">
+      <c r="B1346" s="35" t="s">
         <v>2263</v>
       </c>
     </row>
     <row r="1347" spans="1:2">
-      <c r="A1347" s="30" t="s">
+      <c r="A1347" s="34" t="s">
         <v>2264</v>
       </c>
-      <c r="B1347" s="31" t="s">
+      <c r="B1347" s="35" t="s">
         <v>2265</v>
       </c>
     </row>
     <row r="1348" spans="1:2">
-      <c r="A1348" s="30" t="s">
+      <c r="A1348" s="34" t="s">
         <v>2266</v>
       </c>
-      <c r="B1348" s="31" t="s">
+      <c r="B1348" s="35" t="s">
         <v>2267</v>
       </c>
     </row>
     <row r="1349" spans="1:2">
-      <c r="A1349" s="30" t="s">
+      <c r="A1349" s="34" t="s">
         <v>2268</v>
       </c>
-      <c r="B1349" s="31" t="s">
+      <c r="B1349" s="35" t="s">
         <v>2269</v>
       </c>
     </row>
     <row r="1350" spans="1:2">
-      <c r="A1350" s="30" t="s">
+      <c r="A1350" s="34" t="s">
         <v>2270</v>
       </c>
-      <c r="B1350" s="31" t="s">
+      <c r="B1350" s="35" t="s">
         <v>2271</v>
       </c>
     </row>
     <row r="1351" spans="1:2">
-      <c r="A1351" s="30" t="s">
+      <c r="A1351" s="34" t="s">
         <v>2272</v>
       </c>
-      <c r="B1351" s="31" t="s">
+      <c r="B1351" s="35" t="s">
         <v>2273</v>
       </c>
     </row>
     <row r="1352" spans="1:2">
-      <c r="A1352" s="30" t="s">
+      <c r="A1352" s="34" t="s">
         <v>2274</v>
       </c>
-      <c r="B1352" s="31" t="s">
+      <c r="B1352" s="35" t="s">
         <v>2275</v>
       </c>
     </row>
     <row r="1353" spans="1:2">
-      <c r="A1353" s="30" t="s">
+      <c r="A1353" s="34" t="s">
         <v>2276</v>
       </c>
-      <c r="B1353" s="31" t="s">
+      <c r="B1353" s="35" t="s">
         <v>2277</v>
       </c>
     </row>
     <row r="1354" spans="1:2">
-      <c r="A1354" s="30" t="s">
+      <c r="A1354" s="34" t="s">
         <v>2278</v>
       </c>
-      <c r="B1354" s="31" t="s">
+      <c r="B1354" s="35" t="s">
         <v>2279</v>
       </c>
     </row>
     <row r="1355" spans="1:2">
-      <c r="A1355" s="30" t="s">
+      <c r="A1355" s="34" t="s">
         <v>2280</v>
       </c>
-      <c r="B1355" s="31" t="s">
+      <c r="B1355" s="35" t="s">
         <v>2281</v>
       </c>
     </row>
     <row r="1356" spans="1:2">
-      <c r="A1356" s="30" t="s">
+      <c r="A1356" s="34" t="s">
         <v>2282</v>
       </c>
-      <c r="B1356" s="31" t="s">
+      <c r="B1356" s="35" t="s">
         <v>2283</v>
       </c>
     </row>
     <row r="1357" spans="1:2">
-      <c r="A1357" s="30" t="s">
+      <c r="A1357" s="34" t="s">
         <v>2284</v>
       </c>
-      <c r="B1357" s="31" t="s">
+      <c r="B1357" s="35" t="s">
         <v>2285</v>
       </c>
     </row>
     <row r="1358" spans="1:2">
-      <c r="A1358" s="30" t="s">
+      <c r="A1358" s="34" t="s">
         <v>2286</v>
       </c>
-      <c r="B1358" s="31" t="s">
+      <c r="B1358" s="35" t="s">
         <v>2287</v>
       </c>
     </row>
     <row r="1359" spans="1:2">
-      <c r="A1359" s="30" t="s">
+      <c r="A1359" s="34" t="s">
         <v>2288</v>
       </c>
-      <c r="B1359" s="31" t="s">
+      <c r="B1359" s="35" t="s">
         <v>2289</v>
       </c>
     </row>
     <row r="1360" spans="1:2">
-      <c r="A1360" s="30" t="s">
+      <c r="A1360" s="34" t="s">
         <v>2290</v>
       </c>
-      <c r="B1360" s="31" t="s">
+      <c r="B1360" s="35" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="1361" spans="1:2">
-      <c r="A1361" s="30" t="s">
+      <c r="A1361" s="34" t="s">
         <v>2291</v>
       </c>
-      <c r="B1361" s="31" t="s">
+      <c r="B1361" s="35" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="1362" spans="1:2">
-      <c r="A1362" s="30" t="s">
+      <c r="A1362" s="34" t="s">
         <v>2292</v>
       </c>
-      <c r="B1362" s="31" t="s">
+      <c r="B1362" s="35" t="s">
         <v>2293</v>
       </c>
     </row>
     <row r="1363" spans="1:2">
-      <c r="A1363" s="30" t="s">
+      <c r="A1363" s="34" t="s">
         <v>2298</v>
       </c>
-      <c r="B1363" s="31" t="s">
+      <c r="B1363" s="35" t="s">
         <v>2299</v>
       </c>
     </row>
     <row r="1364" spans="1:2">
-      <c r="A1364" s="30" t="s">
+      <c r="A1364" s="34" t="s">
         <v>2300</v>
       </c>
-      <c r="B1364" s="31" t="s">
+      <c r="B1364" s="35" t="s">
         <v>2301</v>
       </c>
     </row>
     <row r="1365" spans="1:2">
-      <c r="A1365" s="30" t="s">
+      <c r="A1365" s="34" t="s">
         <v>2302</v>
       </c>
-      <c r="B1365" s="31" t="s">
+      <c r="B1365" s="35" t="s">
         <v>2036</v>
       </c>
     </row>
     <row r="1366" spans="1:2">
-      <c r="A1366" s="30" t="s">
+      <c r="A1366" s="34" t="s">
         <v>2303</v>
       </c>
-      <c r="B1366" s="30" t="s">
+      <c r="B1366" s="34" t="s">
         <v>2304</v>
       </c>
     </row>
     <row r="1367" spans="1:2">
-      <c r="A1367" s="30" t="s">
+      <c r="A1367" s="34" t="s">
         <v>2305</v>
       </c>
-      <c r="B1367" s="30" t="s">
+      <c r="B1367" s="34" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="1368" spans="1:2">
-      <c r="A1368" s="30" t="s">
+      <c r="A1368" s="34" t="s">
         <v>193</v>
       </c>
-      <c r="B1368" s="30" t="s">
+      <c r="B1368" s="34" t="s">
         <v>193</v>
+      </c>
+    </row>
+    <row r="1369" spans="1:2">
+      <c r="A1369" s="72" t="s">
+        <v>2306</v>
+      </c>
+      <c r="B1369" s="73" t="s">
+        <v>2307</v>
+      </c>
+    </row>
+    <row r="1370" spans="1:2">
+      <c r="A1370" s="72" t="s">
+        <v>2308</v>
+      </c>
+      <c r="B1370" s="73" t="s">
+        <v>2309</v>
+      </c>
+    </row>
+    <row r="1371" spans="1:2">
+      <c r="A1371" s="72" t="s">
+        <v>2310</v>
+      </c>
+      <c r="B1371" s="73" t="s">
+        <v>2311</v>
+      </c>
+    </row>
+    <row r="1372" spans="1:2">
+      <c r="A1372" s="72" t="s">
+        <v>2312</v>
+      </c>
+      <c r="B1372" s="73" t="s">
+        <v>2313</v>
+      </c>
+    </row>
+    <row r="1373" spans="1:2">
+      <c r="A1373" s="72" t="s">
+        <v>2314</v>
+      </c>
+      <c r="B1373" s="73" t="s">
+        <v>2315</v>
+      </c>
+    </row>
+    <row r="1374" spans="1:2">
+      <c r="A1374" s="72" t="s">
+        <v>2316</v>
+      </c>
+      <c r="B1374" s="73" t="s">
+        <v>405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed PO, PR And POA Test Scenarios Changes
Fixed PO, PR And POA Test Scenarios Changes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2845" uniqueCount="2317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2849" uniqueCount="2319">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -6412,6 +6412,219 @@
   </si>
   <si>
     <t>85080200</t>
+  </si>
+  <si>
+    <t>SCOVoutype</t>
+  </si>
+  <si>
+    <t>SCO - VAL. ADD.</t>
+  </si>
+  <si>
+    <t>ValueAdditionPFX</t>
+  </si>
+  <si>
+    <t>SV100</t>
+  </si>
+  <si>
+    <t>ProcessGLacct</t>
+  </si>
+  <si>
+    <t>CHARGES ACCOUNT</t>
+  </si>
+  <si>
+    <t>BOMITEMWITHCONVFACTOR</t>
+  </si>
+  <si>
+    <t>FG0004</t>
+  </si>
+  <si>
+    <t>BOMITEMWITHSOREF</t>
+  </si>
+  <si>
+    <t>FG20001</t>
+  </si>
+  <si>
+    <t>BOMITEMWITHSOREFANDCONV</t>
+  </si>
+  <si>
+    <t>FG30001</t>
+  </si>
+  <si>
+    <t>BOMSOREFWITHCONV</t>
+  </si>
+  <si>
+    <t>SO100/05697/25-26</t>
+  </si>
+  <si>
+    <t>BOMSOREF</t>
+  </si>
+  <si>
+    <t>SO100/05696/25-26</t>
+  </si>
+  <si>
+    <t>BOMProject</t>
+  </si>
+  <si>
+    <t>VJ-PROJECT</t>
+  </si>
+  <si>
+    <t>OSPNO</t>
+  </si>
+  <si>
+    <t>${OSPNO}</t>
+  </si>
+  <si>
+    <t>OSPDBLOCATIONCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PLNT_LOC_ID</t>
+  </si>
+  <si>
+    <t>OSPDBITEMCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PROD_ID</t>
+  </si>
+  <si>
+    <t>OSPDBTYPECOLUMN</t>
+  </si>
+  <si>
+    <t>LVL_TYPE</t>
+  </si>
+  <si>
+    <t>OSPDBPFXCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PO_PFX</t>
+  </si>
+  <si>
+    <t>OSPDBDOCNOCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PO_NO</t>
+  </si>
+  <si>
+    <t>OSPDBDATECOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_PO_DATE</t>
+  </si>
+  <si>
+    <t>OSPDBSTATUSCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_STATUS</t>
+  </si>
+  <si>
+    <t>OSPDBUNITCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCLN_PLNT</t>
+  </si>
+  <si>
+    <t>OSPDBUOMCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCLN_UOM</t>
+  </si>
+  <si>
+    <t>OSPDBBATCHQTYCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCLN_BATCH_QTY</t>
+  </si>
+  <si>
+    <t>OSPDBBATCHCOSTCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCLN_UNIT_COST</t>
+  </si>
+  <si>
+    <t>OSPDBPROCESSCOLUMN</t>
+  </si>
+  <si>
+    <t>PROCESS_DESC</t>
+  </si>
+  <si>
+    <t>OSPDBSUPPLIERIDCOLUMN</t>
+  </si>
+  <si>
+    <t>SPRCHD_SUPLR_ID</t>
+  </si>
+  <si>
+    <t>OpenSCOApprovedstatus</t>
+  </si>
+  <si>
+    <t>OpenSCOCancelledstatus</t>
+  </si>
+  <si>
+    <t>OpenSCORevisedstatus</t>
+  </si>
+  <si>
+    <t>Revised</t>
+  </si>
+  <si>
+    <t>PRLNumber</t>
+  </si>
+  <si>
+    <t>PRL10/00665/25-26</t>
+  </si>
+  <si>
+    <t>PRLItem</t>
+  </si>
+  <si>
+    <t>TVS-AMD-SIM-651631</t>
+  </si>
+  <si>
+    <t>AmendedStatus</t>
+  </si>
+  <si>
+    <t>RFQNumber</t>
+  </si>
+  <si>
+    <t>RFQ10/00725/25-26</t>
+  </si>
+  <si>
+    <t>Rfqitem</t>
+  </si>
+  <si>
+    <t>UTGST_cus</t>
+  </si>
+  <si>
+    <t>A2B HOTEL MANAGEMENT</t>
+  </si>
+  <si>
+    <t>Open_So_Amd_Ex_Doc</t>
+  </si>
+  <si>
+    <t>OPSO1/00639/25-26</t>
+  </si>
+  <si>
+    <t>Open_So_Amd_Utgst_Doc</t>
+  </si>
+  <si>
+    <t>OSO7-2526-00003</t>
+  </si>
+  <si>
+    <t>Open_So_Amd_Interstate_Doc</t>
+  </si>
+  <si>
+    <t>OPSO1/00665/25-26</t>
+  </si>
+  <si>
+    <t>Open_So_Amd_Dom_Cus</t>
+  </si>
+  <si>
+    <t>OPSO1/00696/25-26</t>
+  </si>
+  <si>
+    <t>Openso_Price</t>
+  </si>
+  <si>
+    <t>HsnCode75052200</t>
+  </si>
+  <si>
+    <t>75052200</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -8886,156 +9099,6 @@
     AND PRL_PROD_ID  ='${ItemId}'</t>
   </si>
   <si>
-    <t>SCOVoutype</t>
-  </si>
-  <si>
-    <t>SCO - VAL. ADD.</t>
-  </si>
-  <si>
-    <t>ValueAdditionPFX</t>
-  </si>
-  <si>
-    <t>SV100</t>
-  </si>
-  <si>
-    <t>ProcessGLacct</t>
-  </si>
-  <si>
-    <t>CHARGES ACCOUNT</t>
-  </si>
-  <si>
-    <t>BOMITEMWITHCONVFACTOR</t>
-  </si>
-  <si>
-    <t>FG0004</t>
-  </si>
-  <si>
-    <t>BOMITEMWITHSOREF</t>
-  </si>
-  <si>
-    <t>FG20001</t>
-  </si>
-  <si>
-    <t>BOMITEMWITHSOREFANDCONV</t>
-  </si>
-  <si>
-    <t>FG30001</t>
-  </si>
-  <si>
-    <t>BOMSOREFWITHCONV</t>
-  </si>
-  <si>
-    <t>SO100/05697/25-26</t>
-  </si>
-  <si>
-    <t>BOMSOREF</t>
-  </si>
-  <si>
-    <t>SO100/05696/25-26</t>
-  </si>
-  <si>
-    <t>BOMProject</t>
-  </si>
-  <si>
-    <t>VJ-PROJECT</t>
-  </si>
-  <si>
-    <t>OSPNO</t>
-  </si>
-  <si>
-    <t>${OSPNO}</t>
-  </si>
-  <si>
-    <t>OSPDBLOCATIONCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCHD_PLNT_LOC_ID</t>
-  </si>
-  <si>
-    <t>OSPDBITEMCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCHD_PROD_ID</t>
-  </si>
-  <si>
-    <t>OSPDBTYPECOLUMN</t>
-  </si>
-  <si>
-    <t>LVL_TYPE</t>
-  </si>
-  <si>
-    <t>OSPDBPFXCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCHD_PO_PFX</t>
-  </si>
-  <si>
-    <t>OSPDBDOCNOCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCHD_PO_NO</t>
-  </si>
-  <si>
-    <t>OSPDBDATECOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCHD_PO_DATE</t>
-  </si>
-  <si>
-    <t>OSPDBSTATUSCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCHD_STATUS</t>
-  </si>
-  <si>
-    <t>OSPDBUNITCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCLN_PLNT</t>
-  </si>
-  <si>
-    <t>OSPDBUOMCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCLN_UOM</t>
-  </si>
-  <si>
-    <t>OSPDBBATCHQTYCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCLN_BATCH_QTY</t>
-  </si>
-  <si>
-    <t>OSPDBBATCHCOSTCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCLN_UNIT_COST</t>
-  </si>
-  <si>
-    <t>OSPDBPROCESSCOLUMN</t>
-  </si>
-  <si>
-    <t>PROCESS_DESC</t>
-  </si>
-  <si>
-    <t>OSPDBSUPPLIERIDCOLUMN</t>
-  </si>
-  <si>
-    <t>SPRCHD_SUPLR_ID</t>
-  </si>
-  <si>
-    <t>OpenSCOApprovedstatus</t>
-  </si>
-  <si>
-    <t>OpenSCOCancelledstatus</t>
-  </si>
-  <si>
-    <t>OpenSCORevisedstatus</t>
-  </si>
-  <si>
-    <t>Revised</t>
-  </si>
-  <si>
     <t>OSPHeaderQuery</t>
   </si>
   <si>
@@ -9078,69 +9141,18 @@
    AND sprchd_bu = 'TVSA'
 AND sprchd_po_no = '${OSPNO}'</t>
   </si>
-  <si>
-    <t>PRLNumber</t>
-  </si>
-  <si>
-    <t>PRL10/00665/25-26</t>
-  </si>
-  <si>
-    <t>PRLItem</t>
-  </si>
-  <si>
-    <t>TVS-AMD-SIM-651631</t>
-  </si>
-  <si>
-    <t>AmendedStatus</t>
-  </si>
-  <si>
-    <t>RFQNumber</t>
-  </si>
-  <si>
-    <t>RFQ10/00725/25-26</t>
-  </si>
-  <si>
-    <t>Rfqitem</t>
-  </si>
-  <si>
-    <t>UTGST_cus</t>
-  </si>
-  <si>
-    <t>A2B HOTEL MANAGEMENT</t>
-  </si>
-  <si>
-    <t>Open_So_Amd_Ex_Doc</t>
-  </si>
-  <si>
-    <t>OPSO1/00639/25-26</t>
-  </si>
-  <si>
-    <t>Open_So_Amd_Utgst_Doc</t>
-  </si>
-  <si>
-    <t>OSO7-2526-00003</t>
-  </si>
-  <si>
-    <t>Open_So_Amd_Interstate_Doc</t>
-  </si>
-  <si>
-    <t>OPSO1/00665/25-26</t>
-  </si>
-  <si>
-    <t>Open_So_Amd_Dom_Cus</t>
-  </si>
-  <si>
-    <t>OPSO1/00696/25-26</t>
-  </si>
-  <si>
-    <t>Openso_Price</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9153,44 +9165,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF262626"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -9199,8 +9181,182 @@
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF262626"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -9225,8 +9381,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -9262,28 +9604,270 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="18">
+  <cellStyleXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9299,143 +9883,147 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="15" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="63" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="16" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="16" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="64" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="64" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="52" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="53"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="56" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="61" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="61" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="62" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="59" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="60" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -9443,27 +10031,74 @@
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="18">
+  <cellStyles count="66">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1"/>
-    <cellStyle name="Normal 11" xfId="2"/>
-    <cellStyle name="Normal 13" xfId="3"/>
-    <cellStyle name="Normal 14" xfId="4"/>
-    <cellStyle name="Normal 15" xfId="5"/>
-    <cellStyle name="Normal 16" xfId="6"/>
-    <cellStyle name="Normal 17" xfId="7"/>
-    <cellStyle name="Normal 18" xfId="8"/>
-    <cellStyle name="Normal 19" xfId="9"/>
-    <cellStyle name="Normal 2" xfId="10"/>
-    <cellStyle name="Normal 2 2" xfId="11"/>
-    <cellStyle name="Normal 2 3" xfId="12"/>
-    <cellStyle name="Normal 20" xfId="13"/>
-    <cellStyle name="Normal 3" xfId="14"/>
-    <cellStyle name="Normal 7" xfId="15"/>
-    <cellStyle name="Normal 8" xfId="16"/>
-    <cellStyle name="Normal 9" xfId="17"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal 10" xfId="49"/>
+    <cellStyle name="Normal 11" xfId="50"/>
+    <cellStyle name="Normal 13" xfId="51"/>
+    <cellStyle name="Normal 14" xfId="52"/>
+    <cellStyle name="Normal 15" xfId="53"/>
+    <cellStyle name="Normal 16" xfId="54"/>
+    <cellStyle name="Normal 17" xfId="55"/>
+    <cellStyle name="Normal 18" xfId="56"/>
+    <cellStyle name="Normal 19" xfId="57"/>
+    <cellStyle name="Normal 2" xfId="58"/>
+    <cellStyle name="Normal 2 2" xfId="59"/>
+    <cellStyle name="Normal 2 3" xfId="60"/>
+    <cellStyle name="Normal 20" xfId="61"/>
+    <cellStyle name="Normal 3" xfId="62"/>
+    <cellStyle name="Normal 7" xfId="63"/>
+    <cellStyle name="Normal 8" xfId="64"/>
+    <cellStyle name="Normal 9" xfId="65"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -9725,17 +10360,17 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1374"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B1376"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.85546875" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -20429,191 +21064,191 @@
     </row>
     <row r="1337" spans="1:2">
       <c r="A1337" s="34" t="s">
-        <v>2244</v>
+        <v>2128</v>
       </c>
       <c r="B1337" s="35" t="s">
-        <v>2245</v>
+        <v>2129</v>
       </c>
     </row>
     <row r="1338" spans="1:2">
       <c r="A1338" s="34" t="s">
-        <v>2246</v>
+        <v>2130</v>
       </c>
       <c r="B1338" s="35" t="s">
-        <v>2247</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="1339" spans="1:2">
       <c r="A1339" s="34" t="s">
-        <v>2248</v>
+        <v>2132</v>
       </c>
       <c r="B1339" s="35" t="s">
-        <v>2249</v>
+        <v>2133</v>
       </c>
     </row>
     <row r="1340" spans="1:2">
       <c r="A1340" s="34" t="s">
-        <v>2250</v>
+        <v>2134</v>
       </c>
       <c r="B1340" s="35" t="s">
-        <v>2251</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="1341" spans="1:2">
       <c r="A1341" s="34" t="s">
-        <v>2252</v>
+        <v>2136</v>
       </c>
       <c r="B1341" s="35" t="s">
-        <v>2253</v>
+        <v>2137</v>
       </c>
     </row>
     <row r="1342" spans="1:2">
       <c r="A1342" s="34" t="s">
-        <v>2254</v>
+        <v>2138</v>
       </c>
       <c r="B1342" s="35" t="s">
-        <v>2255</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="1343" spans="1:2">
       <c r="A1343" s="34" t="s">
-        <v>2256</v>
+        <v>2140</v>
       </c>
       <c r="B1343" s="35" t="s">
-        <v>2257</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="1344" spans="1:2">
       <c r="A1344" s="34" t="s">
-        <v>2258</v>
+        <v>2142</v>
       </c>
       <c r="B1344" s="35" t="s">
-        <v>2259</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="1345" spans="1:2">
       <c r="A1345" s="34" t="s">
-        <v>2260</v>
+        <v>2144</v>
       </c>
       <c r="B1345" s="35" t="s">
-        <v>2261</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="1346" spans="1:2">
       <c r="A1346" s="34" t="s">
-        <v>2262</v>
+        <v>2146</v>
       </c>
       <c r="B1346" s="35" t="s">
-        <v>2263</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="1347" spans="1:2">
       <c r="A1347" s="34" t="s">
-        <v>2264</v>
+        <v>2148</v>
       </c>
       <c r="B1347" s="35" t="s">
-        <v>2265</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="1348" spans="1:2">
       <c r="A1348" s="34" t="s">
-        <v>2266</v>
+        <v>2150</v>
       </c>
       <c r="B1348" s="35" t="s">
-        <v>2267</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="1349" spans="1:2">
       <c r="A1349" s="34" t="s">
-        <v>2268</v>
+        <v>2152</v>
       </c>
       <c r="B1349" s="35" t="s">
-        <v>2269</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="1350" spans="1:2">
       <c r="A1350" s="34" t="s">
-        <v>2270</v>
+        <v>2154</v>
       </c>
       <c r="B1350" s="35" t="s">
-        <v>2271</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="1351" spans="1:2">
       <c r="A1351" s="34" t="s">
-        <v>2272</v>
+        <v>2156</v>
       </c>
       <c r="B1351" s="35" t="s">
-        <v>2273</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="1352" spans="1:2">
       <c r="A1352" s="34" t="s">
-        <v>2274</v>
+        <v>2158</v>
       </c>
       <c r="B1352" s="35" t="s">
-        <v>2275</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="1353" spans="1:2">
       <c r="A1353" s="34" t="s">
-        <v>2276</v>
+        <v>2160</v>
       </c>
       <c r="B1353" s="35" t="s">
-        <v>2277</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="1354" spans="1:2">
       <c r="A1354" s="34" t="s">
-        <v>2278</v>
+        <v>2162</v>
       </c>
       <c r="B1354" s="35" t="s">
-        <v>2279</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="1355" spans="1:2">
       <c r="A1355" s="34" t="s">
-        <v>2280</v>
+        <v>2164</v>
       </c>
       <c r="B1355" s="35" t="s">
-        <v>2281</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="1356" spans="1:2">
       <c r="A1356" s="34" t="s">
-        <v>2282</v>
+        <v>2166</v>
       </c>
       <c r="B1356" s="35" t="s">
-        <v>2283</v>
+        <v>2167</v>
       </c>
     </row>
     <row r="1357" spans="1:2">
       <c r="A1357" s="34" t="s">
-        <v>2284</v>
+        <v>2168</v>
       </c>
       <c r="B1357" s="35" t="s">
-        <v>2285</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="1358" spans="1:2">
       <c r="A1358" s="34" t="s">
-        <v>2286</v>
+        <v>2170</v>
       </c>
       <c r="B1358" s="35" t="s">
-        <v>2287</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="1359" spans="1:2">
       <c r="A1359" s="34" t="s">
-        <v>2288</v>
+        <v>2172</v>
       </c>
       <c r="B1359" s="35" t="s">
-        <v>2289</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="1360" spans="1:2">
       <c r="A1360" s="34" t="s">
-        <v>2290</v>
+        <v>2174</v>
       </c>
       <c r="B1360" s="35" t="s">
         <v>35</v>
@@ -20621,7 +21256,7 @@
     </row>
     <row r="1361" spans="1:2">
       <c r="A1361" s="34" t="s">
-        <v>2291</v>
+        <v>2175</v>
       </c>
       <c r="B1361" s="35" t="s">
         <v>59</v>
@@ -20629,31 +21264,31 @@
     </row>
     <row r="1362" spans="1:2">
       <c r="A1362" s="34" t="s">
-        <v>2292</v>
+        <v>2176</v>
       </c>
       <c r="B1362" s="35" t="s">
-        <v>2293</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="1363" spans="1:2">
       <c r="A1363" s="34" t="s">
-        <v>2298</v>
+        <v>2178</v>
       </c>
       <c r="B1363" s="35" t="s">
-        <v>2299</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="1364" spans="1:2">
       <c r="A1364" s="34" t="s">
-        <v>2300</v>
+        <v>2180</v>
       </c>
       <c r="B1364" s="35" t="s">
-        <v>2301</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="1365" spans="1:2">
       <c r="A1365" s="34" t="s">
-        <v>2302</v>
+        <v>2182</v>
       </c>
       <c r="B1365" s="35" t="s">
         <v>2036</v>
@@ -20661,15 +21296,15 @@
     </row>
     <row r="1366" spans="1:2">
       <c r="A1366" s="34" t="s">
-        <v>2303</v>
+        <v>2183</v>
       </c>
       <c r="B1366" s="34" t="s">
-        <v>2304</v>
+        <v>2184</v>
       </c>
     </row>
     <row r="1367" spans="1:2">
       <c r="A1367" s="34" t="s">
-        <v>2305</v>
+        <v>2185</v>
       </c>
       <c r="B1367" s="34" t="s">
         <v>351</v>
@@ -20685,67 +21320,85 @@
     </row>
     <row r="1369" spans="1:2">
       <c r="A1369" s="72" t="s">
-        <v>2306</v>
+        <v>2186</v>
       </c>
       <c r="B1369" s="73" t="s">
-        <v>2307</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="1370" spans="1:2">
       <c r="A1370" s="72" t="s">
-        <v>2308</v>
+        <v>2188</v>
       </c>
       <c r="B1370" s="73" t="s">
-        <v>2309</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="1371" spans="1:2">
       <c r="A1371" s="72" t="s">
-        <v>2310</v>
+        <v>2190</v>
       </c>
       <c r="B1371" s="73" t="s">
-        <v>2311</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="1372" spans="1:2">
       <c r="A1372" s="72" t="s">
-        <v>2312</v>
+        <v>2192</v>
       </c>
       <c r="B1372" s="73" t="s">
-        <v>2313</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="1373" spans="1:2">
       <c r="A1373" s="72" t="s">
-        <v>2314</v>
+        <v>2194</v>
       </c>
       <c r="B1373" s="73" t="s">
-        <v>2315</v>
+        <v>2195</v>
       </c>
     </row>
     <row r="1374" spans="1:2">
       <c r="A1374" s="72" t="s">
-        <v>2316</v>
+        <v>2196</v>
       </c>
       <c r="B1374" s="73" t="s">
         <v>405</v>
       </c>
     </row>
+    <row r="1375" spans="1:2">
+      <c r="A1375" s="72" t="s">
+        <v>2126</v>
+      </c>
+      <c r="B1375" s="73" t="s">
+        <v>2127</v>
+      </c>
+    </row>
+    <row r="1376" spans="1:2">
+      <c r="A1376" s="74" t="s">
+        <v>2197</v>
+      </c>
+      <c r="B1376" s="75" t="s">
+        <v>2198</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1211" r:id="rId1"/>
-    <hyperlink ref="B1366" r:id="rId2" display="javascript:$s('P1615131058_RFQHD_RFQ_PFX','RFQ10');$s('P1615131058_RFQHD_RFQ_NO','RFQ10/00725/25-26');$s('P1615131058_RFQHD_STATUS','A');apex.submit('RFQ');"/>
+    <hyperlink ref="B1211" r:id="rId1" display="MRAD-2425-00086"/>
+    <hyperlink ref="B1366" r:id="rId2" display="RFQ10/00725/25-26"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B65"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -20757,519 +21410,520 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="108.95" customHeight="1">
+    <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>2128</v>
+        <v>2199</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>2129</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="114" customHeight="1">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>2130</v>
+        <v>2201</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2131</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="80.25" customHeight="1">
+        <v>2202</v>
+      </c>
+    </row>
+    <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>2132</v>
+        <v>2203</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2133</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="69.75" customHeight="1">
+        <v>2204</v>
+      </c>
+    </row>
+    <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>2134</v>
+        <v>2205</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="51.75" customHeight="1">
+        <v>2206</v>
+      </c>
+    </row>
+    <row r="6" ht="51.75" customHeight="1" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>2136</v>
+        <v>2207</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2137</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="30" customHeight="1">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>2138</v>
+        <v>2209</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>2139</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="18" customHeight="1">
+        <v>2210</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>2140</v>
+        <v>2211</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>2141</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="39" customHeight="1">
+        <v>2212</v>
+      </c>
+    </row>
+    <row r="9" ht="39" customHeight="1" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>2142</v>
+        <v>2213</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>2143</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="22.5" customHeight="1">
+        <v>2214</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>2144</v>
+        <v>2215</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>2145</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="18" customHeight="1">
+        <v>2216</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>2146</v>
+        <v>2217</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>2147</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="26.25" customHeight="1">
+        <v>2218</v>
+      </c>
+    </row>
+    <row r="12" ht="26.25" customHeight="1" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>2148</v>
+        <v>2219</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>2149</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="28.5" customHeight="1">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="13" ht="28.5" customHeight="1" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>2150</v>
+        <v>2221</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>2151</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="24" customHeight="1">
+        <v>2222</v>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>2152</v>
+        <v>2223</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>2153</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="36" customHeight="1">
+        <v>2224</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>2154</v>
+        <v>2225</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>2155</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1">
+        <v>2226</v>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>2156</v>
+        <v>2227</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>2157</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="43.5" customHeight="1">
+        <v>2228</v>
+      </c>
+    </row>
+    <row r="17" ht="43.5" customHeight="1" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>2158</v>
+        <v>2229</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>2159</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="42" customHeight="1">
+        <v>2230</v>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>2160</v>
+        <v>2231</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>2161</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="52.5" customHeight="1">
+        <v>2232</v>
+      </c>
+    </row>
+    <row r="19" ht="52.5" customHeight="1" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>2162</v>
+        <v>2233</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>2163</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="17.25" customHeight="1">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="20" ht="17.25" customHeight="1" spans="1:2">
       <c r="A20" s="4" t="s">
-        <v>2164</v>
+        <v>2235</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>2165</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15" customHeight="1">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" spans="1:2">
       <c r="A21" s="4" t="s">
-        <v>2166</v>
+        <v>2237</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>2167</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="409.5">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="22" ht="409.5" spans="1:2">
       <c r="A22" s="2" t="s">
-        <v>2168</v>
+        <v>2239</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>2169</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="255">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="23" ht="244.8" spans="1:2">
       <c r="A23" s="2" t="s">
-        <v>2170</v>
+        <v>2241</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>2171</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="240">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="24" ht="230.4" spans="1:2">
       <c r="A24" t="s">
-        <v>2172</v>
+        <v>2243</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>2173</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="270">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="25" ht="259.2" spans="1:2">
       <c r="A25" t="s">
-        <v>2174</v>
+        <v>2245</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>2175</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="210">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="26" ht="201.6" spans="1:2">
       <c r="A26" t="s">
-        <v>2176</v>
+        <v>2247</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>2177</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="61.5" customHeight="1">
+        <v>2248</v>
+      </c>
+    </row>
+    <row r="27" ht="61.5" customHeight="1" spans="1:2">
       <c r="A27" t="s">
-        <v>2178</v>
+        <v>2249</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>2179</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="105.75" customHeight="1">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="28" ht="105.75" customHeight="1" spans="1:2">
       <c r="A28" s="7" t="s">
-        <v>2128</v>
+        <v>2199</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>2129</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="83.25" customHeight="1">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="29" ht="83.25" customHeight="1" spans="1:2">
       <c r="A29" s="9" t="s">
-        <v>2130</v>
+        <v>2201</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>2131</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="180">
+        <v>2202</v>
+      </c>
+    </row>
+    <row r="30" ht="172.8" spans="1:2">
       <c r="A30" s="11" t="s">
-        <v>2136</v>
+        <v>2207</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>2137</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="135">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="31" ht="129.6" spans="1:2">
       <c r="A31" s="13" t="s">
-        <v>2180</v>
+        <v>2251</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>2181</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="180">
+        <v>2252</v>
+      </c>
+    </row>
+    <row r="32" ht="172.8" spans="1:2">
       <c r="A32" s="15" t="s">
-        <v>2182</v>
+        <v>2253</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>2183</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="180">
+        <v>2254</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
       <c r="A33" s="17" t="s">
-        <v>2184</v>
+        <v>2255</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>2185</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="409.5">
+        <v>2256</v>
+      </c>
+    </row>
+    <row r="34" ht="409.5" spans="1:2">
       <c r="A34" s="19" t="s">
-        <v>2186</v>
+        <v>2257</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>2187</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="409.5">
+        <v>2258</v>
+      </c>
+    </row>
+    <row r="35" ht="403.2" spans="1:2">
       <c r="A35" s="21" t="s">
-        <v>2188</v>
+        <v>2259</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>2189</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="409.5">
+        <v>2260</v>
+      </c>
+    </row>
+    <row r="36" ht="409.5" spans="1:2">
       <c r="A36" s="23" t="s">
-        <v>2190</v>
+        <v>2261</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>2191</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="409.5">
+        <v>2262</v>
+      </c>
+    </row>
+    <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="25" t="s">
-        <v>2192</v>
+        <v>2263</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>2193</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="409.5">
+        <v>2264</v>
+      </c>
+    </row>
+    <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="27" t="s">
-        <v>2194</v>
+        <v>2265</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>2195</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="409.5">
+        <v>2266</v>
+      </c>
+    </row>
+    <row r="39" ht="409.5" spans="1:2">
       <c r="A39" t="s">
-        <v>2196</v>
+        <v>2267</v>
       </c>
       <c r="B39" s="29" t="s">
-        <v>2197</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="120">
+        <v>2268</v>
+      </c>
+    </row>
+    <row r="40" ht="115.2" spans="1:2">
       <c r="A40" t="s">
-        <v>2198</v>
+        <v>2269</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>2199</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="180">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="41" ht="172.8" spans="1:2">
       <c r="A41" t="s">
-        <v>2200</v>
+        <v>2271</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>2201</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="195">
+        <v>2272</v>
+      </c>
+    </row>
+    <row r="42" ht="187.2" spans="1:2">
       <c r="A42" t="s">
-        <v>2202</v>
+        <v>2273</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>2203</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="120">
+        <v>2274</v>
+      </c>
+    </row>
+    <row r="43" ht="115.2" spans="1:2">
       <c r="A43" t="s">
-        <v>2204</v>
+        <v>2275</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>2205</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="409.5">
+        <v>2276</v>
+      </c>
+    </row>
+    <row r="44" ht="409.5" spans="1:2">
       <c r="A44" t="s">
-        <v>2206</v>
+        <v>2277</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>2207</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="409.5">
+        <v>2278</v>
+      </c>
+    </row>
+    <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>2208</v>
+        <v>2279</v>
       </c>
       <c r="B45" s="29" t="s">
-        <v>2209</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="409.5">
+        <v>2280</v>
+      </c>
+    </row>
+    <row r="46" ht="409.5" spans="1:2">
       <c r="A46" t="s">
-        <v>2210</v>
+        <v>2281</v>
       </c>
       <c r="B46" s="29" t="s">
-        <v>2211</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="270">
+        <v>2282</v>
+      </c>
+    </row>
+    <row r="47" ht="259.2" spans="1:2">
       <c r="A47" t="s">
-        <v>2212</v>
+        <v>2283</v>
       </c>
       <c r="B47" s="29" t="s">
-        <v>2213</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="409.5">
+        <v>2284</v>
+      </c>
+    </row>
+    <row r="48" ht="409.5" spans="1:2">
       <c r="A48" t="s">
-        <v>2214</v>
+        <v>2285</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>2215</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="345">
+        <v>2286</v>
+      </c>
+    </row>
+    <row r="49" ht="331.2" spans="1:2">
       <c r="A49" t="s">
-        <v>2216</v>
+        <v>2287</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>2217</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="345">
+        <v>2288</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
       <c r="A50" t="s">
-        <v>2218</v>
+        <v>2289</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>2219</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="36" customHeight="1">
+        <v>2290</v>
+      </c>
+    </row>
+    <row r="51" ht="36" customHeight="1" spans="1:2">
       <c r="A51" t="s">
-        <v>2220</v>
+        <v>2291</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>2221</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="23.25" customHeight="1">
+        <v>2292</v>
+      </c>
+    </row>
+    <row r="52" ht="23.25" customHeight="1" spans="1:2">
       <c r="A52" t="s">
-        <v>2222</v>
+        <v>2293</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>2223</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="27.75" customHeight="1">
+        <v>2294</v>
+      </c>
+    </row>
+    <row r="53" ht="27.75" customHeight="1" spans="1:2">
       <c r="A53" t="s">
-        <v>2224</v>
+        <v>2295</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>2225</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="60">
+        <v>2296</v>
+      </c>
+    </row>
+    <row r="54" ht="57.6" spans="1:2">
       <c r="A54" t="s">
-        <v>2226</v>
+        <v>2297</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>2227</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="45">
+        <v>2298</v>
+      </c>
+    </row>
+    <row r="55" ht="43.2" spans="1:2">
       <c r="A55" t="s">
-        <v>2228</v>
+        <v>2299</v>
       </c>
       <c r="B55" s="29" t="s">
-        <v>2229</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="60">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="56" ht="57.6" spans="1:2">
       <c r="A56" t="s">
-        <v>2230</v>
+        <v>2301</v>
       </c>
       <c r="B56" s="29" t="s">
-        <v>2231</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="75">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="57" ht="72" spans="1:2">
       <c r="A57" t="s">
-        <v>2232</v>
+        <v>2303</v>
       </c>
       <c r="B57" s="29" t="s">
-        <v>2233</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="409.5">
+        <v>2304</v>
+      </c>
+    </row>
+    <row r="58" ht="409.5" spans="1:2">
       <c r="A58" t="s">
-        <v>2234</v>
+        <v>2305</v>
       </c>
       <c r="B58" s="29" t="s">
-        <v>2235</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="90">
+        <v>2306</v>
+      </c>
+    </row>
+    <row r="59" ht="86.4" spans="1:2">
       <c r="A59" t="s">
-        <v>2236</v>
+        <v>2307</v>
       </c>
       <c r="B59" s="29" t="s">
-        <v>2237</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="360">
+        <v>2308</v>
+      </c>
+    </row>
+    <row r="60" ht="345.6" spans="1:2">
       <c r="A60" t="s">
-        <v>2238</v>
+        <v>2309</v>
       </c>
       <c r="B60" s="29" t="s">
-        <v>2239</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="75">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="61" ht="57.6" spans="1:2">
       <c r="A61" t="s">
-        <v>2240</v>
+        <v>2311</v>
       </c>
       <c r="B61" s="29" t="s">
-        <v>2241</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="409.5">
+        <v>2312</v>
+      </c>
+    </row>
+    <row r="62" ht="409.5" spans="1:2">
       <c r="A62" t="s">
-        <v>2242</v>
+        <v>2313</v>
       </c>
       <c r="B62" s="29" t="s">
-        <v>2243</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" ht="87.75" customHeight="1">
+        <v>2314</v>
+      </c>
+    </row>
+    <row r="63" ht="87.75" customHeight="1" spans="1:2">
       <c r="A63" t="s">
-        <v>2294</v>
+        <v>2315</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>2295</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="71.25" customHeight="1">
+        <v>2316</v>
+      </c>
+    </row>
+    <row r="64" ht="71.25" customHeight="1" spans="1:2">
       <c r="A64" t="s">
-        <v>2296</v>
+        <v>2317</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>2297</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="54" customHeight="1">
+        <v>2318</v>
+      </c>
+    </row>
+    <row r="65" ht="54" customHeight="1" spans="1:2">
       <c r="A65" t="s">
-        <v>2202</v>
+        <v>2273</v>
       </c>
       <c r="B65" s="29" t="s">
-        <v>2203</v>
+        <v>2274</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixes For Direct Grn and Po To Grn
Fixes For Direct Grn and Po To Grn
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -11,7 +11,6 @@
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2853" uniqueCount="2322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2849" uniqueCount="2322">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -9740,7 +9739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1378"/>
+  <dimension ref="A1:B1376"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
@@ -18966,1816 +18965,1800 @@
     </row>
     <row r="1153" spans="1:2">
       <c r="A1153" s="34" t="s">
-        <v>1369</v>
+        <v>1373</v>
       </c>
       <c r="B1153" s="35" t="s">
-        <v>1370</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="1154" spans="1:2">
       <c r="A1154" s="34" t="s">
-        <v>1369</v>
+        <v>1375</v>
       </c>
       <c r="B1154" s="35" t="s">
-        <v>1372</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="1155" spans="1:2">
       <c r="A1155" s="34" t="s">
-        <v>1373</v>
+        <v>1377</v>
       </c>
       <c r="B1155" s="35" t="s">
-        <v>1374</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="1156" spans="1:2">
       <c r="A1156" s="34" t="s">
-        <v>1375</v>
+        <v>1379</v>
       </c>
       <c r="B1156" s="35" t="s">
-        <v>1376</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="1157" spans="1:2">
       <c r="A1157" s="34" t="s">
-        <v>1377</v>
+        <v>1381</v>
       </c>
       <c r="B1157" s="35" t="s">
-        <v>1378</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="1158" spans="1:2">
       <c r="A1158" s="34" t="s">
-        <v>1379</v>
+        <v>1383</v>
       </c>
       <c r="B1158" s="35" t="s">
-        <v>1380</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="1159" spans="1:2">
       <c r="A1159" s="34" t="s">
-        <v>1381</v>
+        <v>1385</v>
       </c>
       <c r="B1159" s="35" t="s">
-        <v>1382</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="1160" spans="1:2">
       <c r="A1160" s="34" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
       <c r="B1160" s="35" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="1161" spans="1:2">
       <c r="A1161" s="34" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
       <c r="B1161" s="35" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="1162" spans="1:2">
       <c r="A1162" s="34" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
       <c r="B1162" s="35" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="1163" spans="1:2">
       <c r="A1163" s="34" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
       <c r="B1163" s="35" t="s">
-        <v>1390</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="1164" spans="1:2">
       <c r="A1164" s="34" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
       <c r="B1164" s="35" t="s">
-        <v>1392</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="1165" spans="1:2">
       <c r="A1165" s="34" t="s">
-        <v>1393</v>
+        <v>1397</v>
       </c>
       <c r="B1165" s="35" t="s">
-        <v>1394</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="1166" spans="1:2">
       <c r="A1166" s="34" t="s">
-        <v>1395</v>
+        <v>1893</v>
       </c>
       <c r="B1166" s="35" t="s">
-        <v>1396</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="1167" spans="1:2">
       <c r="A1167" s="34" t="s">
-        <v>1397</v>
+        <v>1895</v>
       </c>
       <c r="B1167" s="35" t="s">
-        <v>1398</v>
+        <v>1896</v>
       </c>
     </row>
     <row r="1168" spans="1:2">
       <c r="A1168" s="34" t="s">
-        <v>1893</v>
+        <v>1897</v>
       </c>
       <c r="B1168" s="35" t="s">
-        <v>1894</v>
+        <v>559</v>
       </c>
     </row>
     <row r="1169" spans="1:2">
       <c r="A1169" s="34" t="s">
-        <v>1895</v>
+        <v>1898</v>
       </c>
       <c r="B1169" s="35" t="s">
-        <v>1896</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="1170" spans="1:2">
       <c r="A1170" s="34" t="s">
-        <v>1897</v>
+        <v>1900</v>
       </c>
       <c r="B1170" s="35" t="s">
-        <v>559</v>
+        <v>1901</v>
       </c>
     </row>
     <row r="1171" spans="1:2">
       <c r="A1171" s="34" t="s">
-        <v>1898</v>
+        <v>1902</v>
       </c>
       <c r="B1171" s="35" t="s">
-        <v>1899</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="1172" spans="1:2">
       <c r="A1172" s="34" t="s">
-        <v>1900</v>
-      </c>
-      <c r="B1172" s="35" t="s">
-        <v>1901</v>
+        <v>1904</v>
+      </c>
+      <c r="B1172" s="68" t="s">
+        <v>1905</v>
       </c>
     </row>
     <row r="1173" spans="1:2">
       <c r="A1173" s="34" t="s">
-        <v>1902</v>
-      </c>
-      <c r="B1173" s="35" t="s">
-        <v>1903</v>
+        <v>1906</v>
+      </c>
+      <c r="B1173" s="34" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="1174" spans="1:2">
       <c r="A1174" s="34" t="s">
-        <v>1904</v>
-      </c>
-      <c r="B1174" s="68" t="s">
-        <v>1905</v>
+        <v>1907</v>
+      </c>
+      <c r="B1174" s="34" t="s">
+        <v>1908</v>
       </c>
     </row>
     <row r="1175" spans="1:2">
       <c r="A1175" s="34" t="s">
-        <v>1906</v>
-      </c>
-      <c r="B1175" s="34" t="s">
-        <v>59</v>
+        <v>1909</v>
+      </c>
+      <c r="B1175" s="35" t="s">
+        <v>1910</v>
       </c>
     </row>
     <row r="1176" spans="1:2">
       <c r="A1176" s="34" t="s">
-        <v>1907</v>
-      </c>
-      <c r="B1176" s="34" t="s">
-        <v>1908</v>
+        <v>1911</v>
+      </c>
+      <c r="B1176" s="68" t="s">
+        <v>1494</v>
       </c>
     </row>
     <row r="1177" spans="1:2">
       <c r="A1177" s="34" t="s">
-        <v>1909</v>
-      </c>
-      <c r="B1177" s="35" t="s">
-        <v>1910</v>
+        <v>1912</v>
+      </c>
+      <c r="B1177" s="68" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="1178" spans="1:2">
       <c r="A1178" s="34" t="s">
-        <v>1911</v>
-      </c>
-      <c r="B1178" s="68" t="s">
-        <v>1494</v>
+        <v>1913</v>
+      </c>
+      <c r="B1178" s="69" t="s">
+        <v>1914</v>
       </c>
     </row>
     <row r="1179" spans="1:2">
       <c r="A1179" s="34" t="s">
-        <v>1912</v>
-      </c>
-      <c r="B1179" s="68" t="s">
-        <v>306</v>
+        <v>1915</v>
+      </c>
+      <c r="B1179" s="35" t="s">
+        <v>1916</v>
       </c>
     </row>
     <row r="1180" spans="1:2">
       <c r="A1180" s="34" t="s">
-        <v>1913</v>
-      </c>
-      <c r="B1180" s="69" t="s">
-        <v>1914</v>
+        <v>1341</v>
+      </c>
+      <c r="B1180" s="35" t="s">
+        <v>1342</v>
       </c>
     </row>
     <row r="1181" spans="1:2">
       <c r="A1181" s="34" t="s">
-        <v>1915</v>
+        <v>1343</v>
       </c>
       <c r="B1181" s="35" t="s">
-        <v>1916</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="1182" spans="1:2">
       <c r="A1182" s="34" t="s">
-        <v>1341</v>
+        <v>1345</v>
       </c>
       <c r="B1182" s="35" t="s">
-        <v>1342</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="1183" spans="1:2">
       <c r="A1183" s="34" t="s">
-        <v>1343</v>
+        <v>1347</v>
       </c>
       <c r="B1183" s="35" t="s">
-        <v>1344</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="1184" spans="1:2">
       <c r="A1184" s="34" t="s">
-        <v>1345</v>
+        <v>1349</v>
       </c>
       <c r="B1184" s="35" t="s">
-        <v>1346</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="1185" spans="1:2">
       <c r="A1185" s="34" t="s">
-        <v>1347</v>
+        <v>1351</v>
       </c>
       <c r="B1185" s="35" t="s">
-        <v>1348</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="1186" spans="1:2">
       <c r="A1186" s="34" t="s">
-        <v>1349</v>
+        <v>1353</v>
       </c>
       <c r="B1186" s="35" t="s">
-        <v>1350</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="1187" spans="1:2">
       <c r="A1187" s="34" t="s">
-        <v>1351</v>
+        <v>1355</v>
       </c>
       <c r="B1187" s="35" t="s">
-        <v>1352</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="1188" spans="1:2">
       <c r="A1188" s="34" t="s">
-        <v>1353</v>
+        <v>1917</v>
       </c>
       <c r="B1188" s="35" t="s">
-        <v>1354</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="1189" spans="1:2">
       <c r="A1189" s="34" t="s">
-        <v>1355</v>
+        <v>1918</v>
       </c>
       <c r="B1189" s="35" t="s">
-        <v>1356</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="1190" spans="1:2">
       <c r="A1190" s="34" t="s">
-        <v>1917</v>
+        <v>1919</v>
       </c>
       <c r="B1190" s="35" t="s">
-        <v>1364</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="1191" spans="1:2">
       <c r="A1191" s="34" t="s">
-        <v>1918</v>
+        <v>1921</v>
       </c>
       <c r="B1191" s="35" t="s">
-        <v>1366</v>
+        <v>1922</v>
       </c>
     </row>
     <row r="1192" spans="1:2">
       <c r="A1192" s="34" t="s">
-        <v>1919</v>
+        <v>1923</v>
       </c>
       <c r="B1192" s="35" t="s">
-        <v>1920</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="1193" spans="1:2">
       <c r="A1193" s="34" t="s">
-        <v>1921</v>
+        <v>1925</v>
       </c>
       <c r="B1193" s="35" t="s">
-        <v>1922</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="1194" spans="1:2">
       <c r="A1194" s="34" t="s">
-        <v>1923</v>
+        <v>1927</v>
       </c>
       <c r="B1194" s="35" t="s">
-        <v>1924</v>
+        <v>1927</v>
       </c>
     </row>
     <row r="1195" spans="1:2">
       <c r="A1195" s="34" t="s">
-        <v>1925</v>
+        <v>1928</v>
       </c>
       <c r="B1195" s="35" t="s">
-        <v>1926</v>
+        <v>1928</v>
       </c>
     </row>
     <row r="1196" spans="1:2">
       <c r="A1196" s="34" t="s">
-        <v>1927</v>
+        <v>1929</v>
       </c>
       <c r="B1196" s="35" t="s">
-        <v>1927</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="1197" spans="1:2">
       <c r="A1197" s="34" t="s">
-        <v>1928</v>
+        <v>1439</v>
       </c>
       <c r="B1197" s="35" t="s">
-        <v>1928</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="1198" spans="1:2">
       <c r="A1198" s="34" t="s">
-        <v>1929</v>
+        <v>1441</v>
       </c>
       <c r="B1198" s="35" t="s">
-        <v>1929</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="1199" spans="1:2">
       <c r="A1199" s="34" t="s">
-        <v>1439</v>
+        <v>1443</v>
       </c>
       <c r="B1199" s="35" t="s">
-        <v>1440</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="1200" spans="1:2">
       <c r="A1200" s="34" t="s">
-        <v>1441</v>
+        <v>1445</v>
       </c>
       <c r="B1200" s="35" t="s">
-        <v>1442</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="1201" spans="1:2">
       <c r="A1201" s="34" t="s">
-        <v>1443</v>
+        <v>1447</v>
       </c>
       <c r="B1201" s="35" t="s">
-        <v>1444</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="1202" spans="1:2">
       <c r="A1202" s="34" t="s">
-        <v>1445</v>
+        <v>1448</v>
       </c>
       <c r="B1202" s="35" t="s">
-        <v>1446</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="1203" spans="1:2">
       <c r="A1203" s="34" t="s">
-        <v>1447</v>
+        <v>1449</v>
       </c>
       <c r="B1203" s="35" t="s">
-        <v>1374</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="1204" spans="1:2">
       <c r="A1204" s="34" t="s">
-        <v>1448</v>
+        <v>1930</v>
       </c>
       <c r="B1204" s="35" t="s">
-        <v>1376</v>
+        <v>1931</v>
       </c>
     </row>
     <row r="1205" spans="1:2">
       <c r="A1205" s="34" t="s">
-        <v>1449</v>
+        <v>1932</v>
       </c>
       <c r="B1205" s="35" t="s">
-        <v>1450</v>
+        <v>1933</v>
       </c>
     </row>
     <row r="1206" spans="1:2">
       <c r="A1206" s="34" t="s">
-        <v>1930</v>
+        <v>1934</v>
       </c>
       <c r="B1206" s="35" t="s">
-        <v>1931</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="1207" spans="1:2">
       <c r="A1207" s="34" t="s">
-        <v>1932</v>
+        <v>1517</v>
       </c>
       <c r="B1207" s="35" t="s">
-        <v>1933</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="1208" spans="1:2">
       <c r="A1208" s="34" t="s">
-        <v>1934</v>
+        <v>1519</v>
       </c>
       <c r="B1208" s="35" t="s">
-        <v>1935</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="1209" spans="1:2">
       <c r="A1209" s="34" t="s">
-        <v>1517</v>
-      </c>
-      <c r="B1209" s="35" t="s">
-        <v>1518</v>
+        <v>1936</v>
+      </c>
+      <c r="B1209" s="34" t="s">
+        <v>1937</v>
       </c>
     </row>
     <row r="1210" spans="1:2">
       <c r="A1210" s="34" t="s">
-        <v>1519</v>
-      </c>
-      <c r="B1210" s="35" t="s">
-        <v>1520</v>
+        <v>1938</v>
+      </c>
+      <c r="B1210" s="69" t="s">
+        <v>1939</v>
       </c>
     </row>
     <row r="1211" spans="1:2">
       <c r="A1211" s="34" t="s">
-        <v>1936</v>
-      </c>
-      <c r="B1211" s="34" t="s">
-        <v>1937</v>
+        <v>1940</v>
+      </c>
+      <c r="B1211" s="70" t="s">
+        <v>916</v>
       </c>
     </row>
     <row r="1212" spans="1:2">
       <c r="A1212" s="34" t="s">
-        <v>1938</v>
-      </c>
-      <c r="B1212" s="69" t="s">
-        <v>1939</v>
+        <v>1941</v>
+      </c>
+      <c r="B1212" s="70" t="s">
+        <v>1412</v>
       </c>
     </row>
     <row r="1213" spans="1:2">
       <c r="A1213" s="34" t="s">
-        <v>1940</v>
-      </c>
-      <c r="B1213" s="70" t="s">
-        <v>916</v>
+        <v>1942</v>
+      </c>
+      <c r="B1213" s="35" t="s">
+        <v>1943</v>
       </c>
     </row>
     <row r="1214" spans="1:2">
       <c r="A1214" s="34" t="s">
-        <v>1941</v>
-      </c>
-      <c r="B1214" s="70" t="s">
-        <v>1412</v>
+        <v>1944</v>
+      </c>
+      <c r="B1214" s="35" t="s">
+        <v>1943</v>
       </c>
     </row>
     <row r="1215" spans="1:2">
       <c r="A1215" s="34" t="s">
-        <v>1942</v>
+        <v>282</v>
       </c>
       <c r="B1215" s="35" t="s">
-        <v>1943</v>
+        <v>282</v>
       </c>
     </row>
     <row r="1216" spans="1:2">
       <c r="A1216" s="34" t="s">
-        <v>1944</v>
+        <v>1561</v>
       </c>
       <c r="B1216" s="35" t="s">
-        <v>1943</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="1217" spans="1:2">
       <c r="A1217" s="34" t="s">
-        <v>282</v>
+        <v>1563</v>
       </c>
       <c r="B1217" s="35" t="s">
-        <v>282</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="1218" spans="1:2">
       <c r="A1218" s="34" t="s">
-        <v>1561</v>
+        <v>1565</v>
       </c>
       <c r="B1218" s="35" t="s">
-        <v>1945</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="1219" spans="1:2">
       <c r="A1219" s="34" t="s">
-        <v>1563</v>
+        <v>1566</v>
       </c>
       <c r="B1219" s="35" t="s">
-        <v>1945</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="1220" spans="1:2">
       <c r="A1220" s="34" t="s">
-        <v>1565</v>
+        <v>1567</v>
       </c>
       <c r="B1220" s="35" t="s">
-        <v>1565</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="1221" spans="1:2">
       <c r="A1221" s="34" t="s">
-        <v>1566</v>
+        <v>540</v>
       </c>
       <c r="B1221" s="35" t="s">
-        <v>1566</v>
+        <v>541</v>
       </c>
     </row>
     <row r="1222" spans="1:2">
       <c r="A1222" s="34" t="s">
-        <v>1567</v>
-      </c>
-      <c r="B1222" s="35" t="s">
-        <v>1567</v>
+        <v>1946</v>
+      </c>
+      <c r="B1222" s="34" t="s">
+        <v>1854</v>
       </c>
     </row>
     <row r="1223" spans="1:2">
       <c r="A1223" s="34" t="s">
-        <v>540</v>
+        <v>1947</v>
       </c>
       <c r="B1223" s="35" t="s">
-        <v>541</v>
+        <v>562</v>
       </c>
     </row>
     <row r="1224" spans="1:2">
       <c r="A1224" s="34" t="s">
-        <v>1946</v>
-      </c>
-      <c r="B1224" s="34" t="s">
-        <v>1854</v>
+        <v>1948</v>
+      </c>
+      <c r="B1224" s="35" t="s">
+        <v>1949</v>
       </c>
     </row>
     <row r="1225" spans="1:2">
       <c r="A1225" s="34" t="s">
-        <v>1947</v>
+        <v>1950</v>
       </c>
       <c r="B1225" s="35" t="s">
-        <v>562</v>
+        <v>1951</v>
       </c>
     </row>
     <row r="1226" spans="1:2">
       <c r="A1226" s="34" t="s">
-        <v>1948</v>
+        <v>1952</v>
       </c>
       <c r="B1226" s="35" t="s">
-        <v>1949</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="1227" spans="1:2">
       <c r="A1227" s="34" t="s">
-        <v>1950</v>
+        <v>1954</v>
       </c>
       <c r="B1227" s="35" t="s">
-        <v>1951</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="1228" spans="1:2">
       <c r="A1228" s="34" t="s">
-        <v>1952</v>
+        <v>1955</v>
       </c>
       <c r="B1228" s="35" t="s">
-        <v>1953</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="1229" spans="1:2">
       <c r="A1229" s="34" t="s">
-        <v>1954</v>
+        <v>1956</v>
       </c>
       <c r="B1229" s="35" t="s">
-        <v>1798</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="1230" spans="1:2">
       <c r="A1230" s="34" t="s">
-        <v>1955</v>
-      </c>
-      <c r="B1230" s="35" t="s">
-        <v>1899</v>
+        <v>64</v>
+      </c>
+      <c r="B1230" s="68" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="1231" spans="1:2">
       <c r="A1231" s="34" t="s">
-        <v>1956</v>
-      </c>
-      <c r="B1231" s="35" t="s">
-        <v>1957</v>
+        <v>1958</v>
+      </c>
+      <c r="B1231" s="68" t="s">
+        <v>1959</v>
       </c>
     </row>
     <row r="1232" spans="1:2">
       <c r="A1232" s="34" t="s">
-        <v>64</v>
+        <v>1960</v>
       </c>
       <c r="B1232" s="68" t="s">
-        <v>65</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="1233" spans="1:2">
       <c r="A1233" s="34" t="s">
-        <v>1958</v>
-      </c>
-      <c r="B1233" s="68" t="s">
-        <v>1959</v>
+        <v>1962</v>
+      </c>
+      <c r="B1233" s="35" t="s">
+        <v>1963</v>
       </c>
     </row>
     <row r="1234" spans="1:2">
       <c r="A1234" s="34" t="s">
-        <v>1960</v>
-      </c>
-      <c r="B1234" s="68" t="s">
-        <v>1961</v>
+        <v>1964</v>
+      </c>
+      <c r="B1234" s="35" t="s">
+        <v>1965</v>
       </c>
     </row>
     <row r="1235" spans="1:2">
       <c r="A1235" s="34" t="s">
-        <v>1962</v>
+        <v>1966</v>
       </c>
       <c r="B1235" s="35" t="s">
-        <v>1963</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="1236" spans="1:2">
       <c r="A1236" s="34" t="s">
-        <v>1964</v>
+        <v>1968</v>
       </c>
       <c r="B1236" s="35" t="s">
-        <v>1965</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="1237" spans="1:2">
       <c r="A1237" s="34" t="s">
-        <v>1966</v>
+        <v>1970</v>
       </c>
       <c r="B1237" s="35" t="s">
-        <v>1967</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="1238" spans="1:2">
       <c r="A1238" s="34" t="s">
-        <v>1968</v>
+        <v>1971</v>
       </c>
       <c r="B1238" s="35" t="s">
-        <v>1969</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="1239" spans="1:2">
       <c r="A1239" s="34" t="s">
-        <v>1970</v>
+        <v>1973</v>
       </c>
       <c r="B1239" s="35" t="s">
-        <v>1969</v>
+        <v>387</v>
       </c>
     </row>
     <row r="1240" spans="1:2">
       <c r="A1240" s="34" t="s">
-        <v>1971</v>
+        <v>1974</v>
       </c>
       <c r="B1240" s="35" t="s">
-        <v>1972</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="1241" spans="1:2">
       <c r="A1241" s="34" t="s">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="B1241" s="35" t="s">
-        <v>387</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="1242" spans="1:2">
       <c r="A1242" s="34" t="s">
-        <v>1974</v>
+        <v>1978</v>
       </c>
       <c r="B1242" s="35" t="s">
-        <v>1975</v>
+        <v>1979</v>
       </c>
     </row>
     <row r="1243" spans="1:2">
       <c r="A1243" s="34" t="s">
-        <v>1976</v>
+        <v>1980</v>
       </c>
       <c r="B1243" s="35" t="s">
-        <v>1977</v>
+        <v>1981</v>
       </c>
     </row>
     <row r="1244" spans="1:2">
       <c r="A1244" s="34" t="s">
-        <v>1978</v>
+        <v>1982</v>
       </c>
       <c r="B1244" s="35" t="s">
-        <v>1979</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="1245" spans="1:2">
       <c r="A1245" s="34" t="s">
-        <v>1980</v>
+        <v>1958</v>
       </c>
       <c r="B1245" s="35" t="s">
-        <v>1981</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="1246" spans="1:2">
       <c r="A1246" s="34" t="s">
-        <v>1982</v>
+        <v>1960</v>
       </c>
       <c r="B1246" s="35" t="s">
-        <v>1914</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="1247" spans="1:2">
       <c r="A1247" s="34" t="s">
-        <v>1958</v>
+        <v>1983</v>
       </c>
       <c r="B1247" s="35" t="s">
-        <v>1959</v>
+        <v>1984</v>
       </c>
     </row>
     <row r="1248" spans="1:2">
       <c r="A1248" s="34" t="s">
-        <v>1960</v>
+        <v>1985</v>
       </c>
       <c r="B1248" s="35" t="s">
-        <v>1961</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="1249" spans="1:2">
-      <c r="A1249" s="34" t="s">
-        <v>1983</v>
-      </c>
-      <c r="B1249" s="35" t="s">
-        <v>1984</v>
+      <c r="A1249" s="36" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B1249" s="37" t="s">
+        <v>1988</v>
       </c>
     </row>
     <row r="1250" spans="1:2">
       <c r="A1250" s="34" t="s">
-        <v>1985</v>
+        <v>1989</v>
       </c>
       <c r="B1250" s="35" t="s">
-        <v>1986</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="1251" spans="1:2">
-      <c r="A1251" s="36" t="s">
-        <v>1987</v>
-      </c>
-      <c r="B1251" s="37" t="s">
-        <v>1988</v>
+      <c r="A1251" s="34" t="s">
+        <v>1991</v>
+      </c>
+      <c r="B1251" s="35" t="s">
+        <v>1798</v>
       </c>
     </row>
     <row r="1252" spans="1:2">
       <c r="A1252" s="34" t="s">
-        <v>1989</v>
+        <v>1992</v>
       </c>
       <c r="B1252" s="35" t="s">
-        <v>1990</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="1253" spans="1:2">
       <c r="A1253" s="34" t="s">
-        <v>1991</v>
+        <v>1994</v>
       </c>
       <c r="B1253" s="35" t="s">
-        <v>1798</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="1254" spans="1:2">
       <c r="A1254" s="34" t="s">
-        <v>1992</v>
+        <v>1996</v>
       </c>
       <c r="B1254" s="35" t="s">
-        <v>1993</v>
+        <v>570</v>
       </c>
     </row>
     <row r="1255" spans="1:2">
       <c r="A1255" s="34" t="s">
-        <v>1994</v>
+        <v>1997</v>
       </c>
       <c r="B1255" s="35" t="s">
-        <v>1995</v>
+        <v>305</v>
       </c>
     </row>
     <row r="1256" spans="1:2">
       <c r="A1256" s="34" t="s">
-        <v>1996</v>
+        <v>1998</v>
       </c>
       <c r="B1256" s="35" t="s">
-        <v>570</v>
+        <v>916</v>
       </c>
     </row>
     <row r="1257" spans="1:2">
       <c r="A1257" s="34" t="s">
-        <v>1997</v>
+        <v>1999</v>
       </c>
       <c r="B1257" s="35" t="s">
-        <v>305</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="1258" spans="1:2">
       <c r="A1258" s="34" t="s">
-        <v>1998</v>
+        <v>2000</v>
       </c>
       <c r="B1258" s="35" t="s">
-        <v>916</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="1259" spans="1:2">
       <c r="A1259" s="34" t="s">
-        <v>1999</v>
+        <v>2002</v>
       </c>
       <c r="B1259" s="35" t="s">
-        <v>1412</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="1260" spans="1:2">
       <c r="A1260" s="34" t="s">
-        <v>2000</v>
+        <v>2004</v>
       </c>
       <c r="B1260" s="35" t="s">
-        <v>2001</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="1261" spans="1:2">
       <c r="A1261" s="34" t="s">
-        <v>2002</v>
+        <v>2006</v>
       </c>
       <c r="B1261" s="35" t="s">
-        <v>2003</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="1262" spans="1:2">
       <c r="A1262" s="34" t="s">
-        <v>2004</v>
+        <v>2008</v>
       </c>
       <c r="B1262" s="35" t="s">
-        <v>2005</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="1263" spans="1:2">
       <c r="A1263" s="34" t="s">
-        <v>2006</v>
+        <v>2010</v>
       </c>
       <c r="B1263" s="35" t="s">
-        <v>2007</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="1264" spans="1:2">
       <c r="A1264" s="34" t="s">
-        <v>2008</v>
+        <v>2012</v>
       </c>
       <c r="B1264" s="35" t="s">
-        <v>2009</v>
+        <v>914</v>
       </c>
     </row>
     <row r="1265" spans="1:2">
       <c r="A1265" s="34" t="s">
-        <v>2010</v>
+        <v>2013</v>
       </c>
       <c r="B1265" s="35" t="s">
-        <v>2011</v>
+        <v>2014</v>
       </c>
     </row>
     <row r="1266" spans="1:2">
       <c r="A1266" s="34" t="s">
-        <v>2012</v>
+        <v>2015</v>
       </c>
       <c r="B1266" s="35" t="s">
-        <v>914</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="1267" spans="1:2">
       <c r="A1267" s="34" t="s">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="B1267" s="35" t="s">
-        <v>2014</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="1268" spans="1:2">
       <c r="A1268" s="34" t="s">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="B1268" s="35" t="s">
-        <v>2016</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="1269" spans="1:2">
       <c r="A1269" s="34" t="s">
-        <v>2017</v>
+        <v>2021</v>
       </c>
       <c r="B1269" s="35" t="s">
-        <v>2018</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="1270" spans="1:2">
       <c r="A1270" s="34" t="s">
-        <v>2019</v>
+        <v>2023</v>
       </c>
       <c r="B1270" s="35" t="s">
-        <v>2020</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="1271" spans="1:2">
       <c r="A1271" s="34" t="s">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="B1271" s="35" t="s">
-        <v>2022</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="1272" spans="1:2">
       <c r="A1272" s="34" t="s">
-        <v>2023</v>
+        <v>2027</v>
       </c>
       <c r="B1272" s="35" t="s">
-        <v>2024</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="1273" spans="1:2">
       <c r="A1273" s="34" t="s">
-        <v>2025</v>
+        <v>2029</v>
       </c>
       <c r="B1273" s="35" t="s">
-        <v>2026</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="1274" spans="1:2">
       <c r="A1274" s="34" t="s">
-        <v>2027</v>
+        <v>2031</v>
       </c>
       <c r="B1274" s="35" t="s">
-        <v>2028</v>
+        <v>2032</v>
       </c>
     </row>
     <row r="1275" spans="1:2">
       <c r="A1275" s="34" t="s">
-        <v>2029</v>
+        <v>2033</v>
       </c>
       <c r="B1275" s="35" t="s">
-        <v>2030</v>
+        <v>2034</v>
       </c>
     </row>
     <row r="1276" spans="1:2">
       <c r="A1276" s="34" t="s">
-        <v>2031</v>
+        <v>2035</v>
       </c>
       <c r="B1276" s="35" t="s">
-        <v>2032</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="1277" spans="1:2">
       <c r="A1277" s="34" t="s">
-        <v>2033</v>
+        <v>1877</v>
       </c>
       <c r="B1277" s="35" t="s">
-        <v>2034</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="1278" spans="1:2">
       <c r="A1278" s="34" t="s">
-        <v>2035</v>
+        <v>2037</v>
       </c>
       <c r="B1278" s="35" t="s">
-        <v>2036</v>
+        <v>2038</v>
       </c>
     </row>
     <row r="1279" spans="1:2">
       <c r="A1279" s="34" t="s">
-        <v>1877</v>
+        <v>2039</v>
       </c>
       <c r="B1279" s="35" t="s">
-        <v>1878</v>
+        <v>562</v>
       </c>
     </row>
     <row r="1280" spans="1:2">
       <c r="A1280" s="34" t="s">
-        <v>2037</v>
+        <v>2040</v>
       </c>
       <c r="B1280" s="35" t="s">
-        <v>2038</v>
+        <v>59</v>
       </c>
     </row>
     <row r="1281" spans="1:2">
       <c r="A1281" s="34" t="s">
-        <v>2039</v>
+        <v>2041</v>
       </c>
       <c r="B1281" s="35" t="s">
-        <v>562</v>
+        <v>377</v>
       </c>
     </row>
     <row r="1282" spans="1:2">
       <c r="A1282" s="34" t="s">
-        <v>2040</v>
+        <v>2042</v>
       </c>
       <c r="B1282" s="35" t="s">
-        <v>59</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="1283" spans="1:2">
       <c r="A1283" s="34" t="s">
-        <v>2041</v>
+        <v>2044</v>
       </c>
       <c r="B1283" s="35" t="s">
-        <v>377</v>
+        <v>2045</v>
       </c>
     </row>
     <row r="1284" spans="1:2">
       <c r="A1284" s="34" t="s">
-        <v>2042</v>
+        <v>2046</v>
       </c>
       <c r="B1284" s="35" t="s">
-        <v>2043</v>
+        <v>715</v>
       </c>
     </row>
     <row r="1285" spans="1:2">
       <c r="A1285" s="34" t="s">
-        <v>2044</v>
+        <v>2047</v>
       </c>
       <c r="B1285" s="35" t="s">
-        <v>2045</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="1286" spans="1:2">
       <c r="A1286" s="34" t="s">
-        <v>2046</v>
+        <v>2049</v>
       </c>
       <c r="B1286" s="35" t="s">
-        <v>715</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="1287" spans="1:2">
       <c r="A1287" s="34" t="s">
-        <v>2047</v>
+        <v>2051</v>
       </c>
       <c r="B1287" s="35" t="s">
-        <v>2048</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="1288" spans="1:2">
       <c r="A1288" s="34" t="s">
-        <v>2049</v>
+        <v>2053</v>
       </c>
       <c r="B1288" s="35" t="s">
-        <v>2050</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="1289" spans="1:2">
       <c r="A1289" s="34" t="s">
-        <v>2051</v>
+        <v>2055</v>
       </c>
       <c r="B1289" s="35" t="s">
-        <v>2052</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="1290" spans="1:2">
       <c r="A1290" s="34" t="s">
-        <v>2053</v>
+        <v>2056</v>
       </c>
       <c r="B1290" s="35" t="s">
-        <v>2054</v>
+        <v>2057</v>
       </c>
     </row>
     <row r="1291" spans="1:2">
       <c r="A1291" s="34" t="s">
-        <v>2055</v>
+        <v>2058</v>
       </c>
       <c r="B1291" s="35" t="s">
-        <v>1580</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="1292" spans="1:2">
       <c r="A1292" s="34" t="s">
-        <v>2056</v>
+        <v>2060</v>
       </c>
       <c r="B1292" s="35" t="s">
-        <v>2057</v>
+        <v>2061</v>
       </c>
     </row>
     <row r="1293" spans="1:2">
       <c r="A1293" s="34" t="s">
-        <v>2058</v>
+        <v>2062</v>
       </c>
       <c r="B1293" s="35" t="s">
-        <v>2059</v>
+        <v>93</v>
       </c>
     </row>
     <row r="1294" spans="1:2">
       <c r="A1294" s="34" t="s">
-        <v>2060</v>
+        <v>2063</v>
       </c>
       <c r="B1294" s="35" t="s">
-        <v>2061</v>
+        <v>2064</v>
       </c>
     </row>
     <row r="1295" spans="1:2">
       <c r="A1295" s="34" t="s">
-        <v>2062</v>
+        <v>2065</v>
       </c>
       <c r="B1295" s="35" t="s">
-        <v>93</v>
+        <v>566</v>
       </c>
     </row>
     <row r="1296" spans="1:2">
       <c r="A1296" s="34" t="s">
-        <v>2063</v>
+        <v>2066</v>
       </c>
       <c r="B1296" s="35" t="s">
-        <v>2064</v>
+        <v>330</v>
       </c>
     </row>
     <row r="1297" spans="1:2">
       <c r="A1297" s="34" t="s">
-        <v>2065</v>
+        <v>2067</v>
       </c>
       <c r="B1297" s="35" t="s">
-        <v>566</v>
+        <v>7</v>
       </c>
     </row>
     <row r="1298" spans="1:2">
       <c r="A1298" s="34" t="s">
-        <v>2066</v>
+        <v>2068</v>
       </c>
       <c r="B1298" s="35" t="s">
-        <v>330</v>
+        <v>2069</v>
       </c>
     </row>
     <row r="1299" spans="1:2">
       <c r="A1299" s="34" t="s">
-        <v>2067</v>
+        <v>2070</v>
       </c>
       <c r="B1299" s="35" t="s">
-        <v>7</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1300" spans="1:2">
       <c r="A1300" s="34" t="s">
-        <v>2068</v>
+        <v>2071</v>
       </c>
       <c r="B1300" s="35" t="s">
-        <v>2069</v>
+        <v>2072</v>
       </c>
     </row>
     <row r="1301" spans="1:2">
       <c r="A1301" s="34" t="s">
-        <v>2070</v>
+        <v>2073</v>
       </c>
       <c r="B1301" s="35" t="s">
-        <v>223</v>
+        <v>152</v>
       </c>
     </row>
     <row r="1302" spans="1:2">
       <c r="A1302" s="34" t="s">
-        <v>2071</v>
+        <v>2074</v>
       </c>
       <c r="B1302" s="35" t="s">
-        <v>2072</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1303" spans="1:2">
       <c r="A1303" s="34" t="s">
-        <v>2073</v>
+        <v>2075</v>
       </c>
       <c r="B1303" s="35" t="s">
-        <v>152</v>
+        <v>223</v>
       </c>
     </row>
     <row r="1304" spans="1:2">
       <c r="A1304" s="34" t="s">
-        <v>2074</v>
+        <v>2076</v>
       </c>
       <c r="B1304" s="35" t="s">
-        <v>223</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="1305" spans="1:2">
       <c r="A1305" s="34" t="s">
-        <v>2075</v>
+        <v>2078</v>
       </c>
       <c r="B1305" s="35" t="s">
-        <v>223</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="1306" spans="1:2">
       <c r="A1306" s="34" t="s">
-        <v>2076</v>
+        <v>2079</v>
       </c>
       <c r="B1306" s="35" t="s">
-        <v>2077</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="1307" spans="1:2">
       <c r="A1307" s="34" t="s">
-        <v>2078</v>
+        <v>2081</v>
       </c>
       <c r="B1307" s="35" t="s">
-        <v>1990</v>
+        <v>2082</v>
       </c>
     </row>
     <row r="1308" spans="1:2">
       <c r="A1308" s="34" t="s">
-        <v>2079</v>
+        <v>2083</v>
       </c>
       <c r="B1308" s="35" t="s">
-        <v>2080</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="1309" spans="1:2">
       <c r="A1309" s="34" t="s">
-        <v>2081</v>
+        <v>2085</v>
       </c>
       <c r="B1309" s="35" t="s">
-        <v>2082</v>
+        <v>2086</v>
       </c>
     </row>
     <row r="1310" spans="1:2">
       <c r="A1310" s="34" t="s">
-        <v>2083</v>
+        <v>2087</v>
       </c>
       <c r="B1310" s="35" t="s">
-        <v>2084</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="1311" spans="1:2">
       <c r="A1311" s="34" t="s">
-        <v>2085</v>
+        <v>2089</v>
       </c>
       <c r="B1311" s="35" t="s">
-        <v>2086</v>
+        <v>2090</v>
       </c>
     </row>
     <row r="1312" spans="1:2">
       <c r="A1312" s="34" t="s">
-        <v>2087</v>
+        <v>2091</v>
       </c>
       <c r="B1312" s="35" t="s">
-        <v>2088</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="1313" spans="1:2">
       <c r="A1313" s="34" t="s">
-        <v>2089</v>
+        <v>2093</v>
       </c>
       <c r="B1313" s="35" t="s">
-        <v>2090</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="1314" spans="1:2">
       <c r="A1314" s="34" t="s">
-        <v>2091</v>
+        <v>2095</v>
       </c>
       <c r="B1314" s="35" t="s">
-        <v>2092</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="1315" spans="1:2">
       <c r="A1315" s="34" t="s">
-        <v>2093</v>
+        <v>2097</v>
       </c>
       <c r="B1315" s="35" t="s">
-        <v>2094</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="1316" spans="1:2">
       <c r="A1316" s="34" t="s">
-        <v>2095</v>
+        <v>2099</v>
       </c>
       <c r="B1316" s="35" t="s">
-        <v>2096</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="1317" spans="1:2">
       <c r="A1317" s="34" t="s">
-        <v>2097</v>
+        <v>2100</v>
       </c>
       <c r="B1317" s="35" t="s">
-        <v>2098</v>
+        <v>2101</v>
       </c>
     </row>
     <row r="1318" spans="1:2">
       <c r="A1318" s="34" t="s">
-        <v>2099</v>
+        <v>2102</v>
       </c>
       <c r="B1318" s="35" t="s">
-        <v>2094</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="1319" spans="1:2">
       <c r="A1319" s="34" t="s">
-        <v>2100</v>
+        <v>2104</v>
       </c>
       <c r="B1319" s="35" t="s">
-        <v>2101</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="1320" spans="1:2">
       <c r="A1320" s="34" t="s">
-        <v>2102</v>
+        <v>2105</v>
       </c>
       <c r="B1320" s="35" t="s">
-        <v>2103</v>
+        <v>2106</v>
       </c>
     </row>
     <row r="1321" spans="1:2">
       <c r="A1321" s="34" t="s">
-        <v>2104</v>
+        <v>2107</v>
       </c>
       <c r="B1321" s="35" t="s">
-        <v>1630</v>
+        <v>2108</v>
       </c>
     </row>
     <row r="1322" spans="1:2">
       <c r="A1322" s="34" t="s">
-        <v>2105</v>
+        <v>2109</v>
       </c>
       <c r="B1322" s="35" t="s">
-        <v>2106</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="1323" spans="1:2">
       <c r="A1323" s="34" t="s">
-        <v>2107</v>
+        <v>2111</v>
       </c>
       <c r="B1323" s="35" t="s">
-        <v>2108</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="1324" spans="1:2">
       <c r="A1324" s="34" t="s">
-        <v>2109</v>
+        <v>2112</v>
       </c>
       <c r="B1324" s="35" t="s">
-        <v>2110</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="1325" spans="1:2">
       <c r="A1325" s="34" t="s">
-        <v>2111</v>
+        <v>2114</v>
       </c>
       <c r="B1325" s="35" t="s">
-        <v>1580</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="1326" spans="1:2">
       <c r="A1326" s="34" t="s">
-        <v>2112</v>
+        <v>2115</v>
       </c>
       <c r="B1326" s="35" t="s">
-        <v>2113</v>
+        <v>228</v>
       </c>
     </row>
     <row r="1327" spans="1:2">
       <c r="A1327" s="34" t="s">
-        <v>2114</v>
+        <v>2116</v>
       </c>
       <c r="B1327" s="35" t="s">
-        <v>2103</v>
+        <v>2117</v>
       </c>
     </row>
     <row r="1328" spans="1:2">
       <c r="A1328" s="34" t="s">
-        <v>2115</v>
+        <v>2118</v>
       </c>
       <c r="B1328" s="35" t="s">
-        <v>228</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="1329" spans="1:2">
       <c r="A1329" s="34" t="s">
-        <v>2116</v>
+        <v>2119</v>
       </c>
       <c r="B1329" s="35" t="s">
-        <v>2117</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="1330" spans="1:2">
       <c r="A1330" s="34" t="s">
-        <v>2118</v>
+        <v>2120</v>
       </c>
       <c r="B1330" s="35" t="s">
-        <v>2103</v>
+        <v>166</v>
       </c>
     </row>
     <row r="1331" spans="1:2">
-      <c r="A1331" s="34" t="s">
-        <v>2119</v>
-      </c>
-      <c r="B1331" s="35" t="s">
-        <v>2113</v>
+      <c r="A1331" s="68" t="s">
+        <v>2121</v>
+      </c>
+      <c r="B1331" s="71" t="s">
+        <v>1308</v>
       </c>
     </row>
     <row r="1332" spans="1:2">
-      <c r="A1332" s="34" t="s">
-        <v>2120</v>
-      </c>
-      <c r="B1332" s="35" t="s">
-        <v>166</v>
+      <c r="A1332" s="68" t="s">
+        <v>2122</v>
+      </c>
+      <c r="B1332" s="71" t="s">
+        <v>2123</v>
       </c>
     </row>
     <row r="1333" spans="1:2">
       <c r="A1333" s="68" t="s">
-        <v>2121</v>
+        <v>2124</v>
       </c>
       <c r="B1333" s="71" t="s">
-        <v>1308</v>
+        <v>2125</v>
       </c>
     </row>
     <row r="1334" spans="1:2">
-      <c r="A1334" s="68" t="s">
-        <v>2122</v>
-      </c>
-      <c r="B1334" s="71" t="s">
-        <v>2123</v>
+      <c r="A1334" s="34" t="s">
+        <v>2126</v>
+      </c>
+      <c r="B1334" s="35" t="s">
+        <v>2127</v>
       </c>
     </row>
     <row r="1335" spans="1:2">
-      <c r="A1335" s="68" t="s">
-        <v>2124</v>
-      </c>
-      <c r="B1335" s="71" t="s">
-        <v>2125</v>
+      <c r="A1335" s="34" t="s">
+        <v>2128</v>
+      </c>
+      <c r="B1335" s="35" t="s">
+        <v>2129</v>
       </c>
     </row>
     <row r="1336" spans="1:2">
       <c r="A1336" s="34" t="s">
-        <v>2126</v>
+        <v>2130</v>
       </c>
       <c r="B1336" s="35" t="s">
-        <v>2127</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="1337" spans="1:2">
       <c r="A1337" s="34" t="s">
-        <v>2128</v>
+        <v>2132</v>
       </c>
       <c r="B1337" s="35" t="s">
-        <v>2129</v>
+        <v>2133</v>
       </c>
     </row>
     <row r="1338" spans="1:2">
       <c r="A1338" s="34" t="s">
-        <v>2130</v>
+        <v>2134</v>
       </c>
       <c r="B1338" s="35" t="s">
-        <v>2131</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="1339" spans="1:2">
       <c r="A1339" s="34" t="s">
-        <v>2132</v>
+        <v>2136</v>
       </c>
       <c r="B1339" s="35" t="s">
-        <v>2133</v>
+        <v>2137</v>
       </c>
     </row>
     <row r="1340" spans="1:2">
       <c r="A1340" s="34" t="s">
-        <v>2134</v>
+        <v>2138</v>
       </c>
       <c r="B1340" s="35" t="s">
-        <v>2135</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="1341" spans="1:2">
       <c r="A1341" s="34" t="s">
-        <v>2136</v>
+        <v>2140</v>
       </c>
       <c r="B1341" s="35" t="s">
-        <v>2137</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="1342" spans="1:2">
       <c r="A1342" s="34" t="s">
-        <v>2138</v>
+        <v>2142</v>
       </c>
       <c r="B1342" s="35" t="s">
-        <v>2139</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="1343" spans="1:2">
       <c r="A1343" s="34" t="s">
-        <v>2140</v>
+        <v>2144</v>
       </c>
       <c r="B1343" s="35" t="s">
-        <v>2141</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="1344" spans="1:2">
       <c r="A1344" s="34" t="s">
-        <v>2142</v>
+        <v>2146</v>
       </c>
       <c r="B1344" s="35" t="s">
-        <v>2143</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="1345" spans="1:2">
       <c r="A1345" s="34" t="s">
-        <v>2144</v>
+        <v>2148</v>
       </c>
       <c r="B1345" s="35" t="s">
-        <v>2145</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="1346" spans="1:2">
       <c r="A1346" s="34" t="s">
-        <v>2146</v>
+        <v>2150</v>
       </c>
       <c r="B1346" s="35" t="s">
-        <v>2147</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="1347" spans="1:2">
       <c r="A1347" s="34" t="s">
-        <v>2148</v>
+        <v>2152</v>
       </c>
       <c r="B1347" s="35" t="s">
-        <v>2149</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="1348" spans="1:2">
       <c r="A1348" s="34" t="s">
-        <v>2150</v>
+        <v>2154</v>
       </c>
       <c r="B1348" s="35" t="s">
-        <v>2151</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="1349" spans="1:2">
       <c r="A1349" s="34" t="s">
-        <v>2152</v>
+        <v>2156</v>
       </c>
       <c r="B1349" s="35" t="s">
-        <v>2153</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="1350" spans="1:2">
       <c r="A1350" s="34" t="s">
-        <v>2154</v>
+        <v>2158</v>
       </c>
       <c r="B1350" s="35" t="s">
-        <v>2155</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="1351" spans="1:2">
       <c r="A1351" s="34" t="s">
-        <v>2156</v>
+        <v>2160</v>
       </c>
       <c r="B1351" s="35" t="s">
-        <v>2157</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="1352" spans="1:2">
       <c r="A1352" s="34" t="s">
-        <v>2158</v>
+        <v>2162</v>
       </c>
       <c r="B1352" s="35" t="s">
-        <v>2159</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="1353" spans="1:2">
       <c r="A1353" s="34" t="s">
-        <v>2160</v>
+        <v>2164</v>
       </c>
       <c r="B1353" s="35" t="s">
-        <v>2161</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="1354" spans="1:2">
       <c r="A1354" s="34" t="s">
-        <v>2162</v>
+        <v>2166</v>
       </c>
       <c r="B1354" s="35" t="s">
-        <v>2163</v>
+        <v>2167</v>
       </c>
     </row>
     <row r="1355" spans="1:2">
       <c r="A1355" s="34" t="s">
-        <v>2164</v>
+        <v>2168</v>
       </c>
       <c r="B1355" s="35" t="s">
-        <v>2165</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="1356" spans="1:2">
       <c r="A1356" s="34" t="s">
-        <v>2166</v>
+        <v>2170</v>
       </c>
       <c r="B1356" s="35" t="s">
-        <v>2167</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="1357" spans="1:2">
       <c r="A1357" s="34" t="s">
-        <v>2168</v>
+        <v>2172</v>
       </c>
       <c r="B1357" s="35" t="s">
-        <v>2169</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="1358" spans="1:2">
       <c r="A1358" s="34" t="s">
-        <v>2170</v>
+        <v>2174</v>
       </c>
       <c r="B1358" s="35" t="s">
-        <v>2171</v>
+        <v>35</v>
       </c>
     </row>
     <row r="1359" spans="1:2">
       <c r="A1359" s="34" t="s">
-        <v>2172</v>
+        <v>2175</v>
       </c>
       <c r="B1359" s="35" t="s">
-        <v>2173</v>
+        <v>59</v>
       </c>
     </row>
     <row r="1360" spans="1:2">
       <c r="A1360" s="34" t="s">
-        <v>2174</v>
+        <v>2176</v>
       </c>
       <c r="B1360" s="35" t="s">
-        <v>35</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="1361" spans="1:2">
       <c r="A1361" s="34" t="s">
-        <v>2175</v>
+        <v>2178</v>
       </c>
       <c r="B1361" s="35" t="s">
-        <v>59</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="1362" spans="1:2">
       <c r="A1362" s="34" t="s">
-        <v>2176</v>
+        <v>2180</v>
       </c>
       <c r="B1362" s="35" t="s">
-        <v>2177</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="1363" spans="1:2">
       <c r="A1363" s="34" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
       <c r="B1363" s="35" t="s">
-        <v>2179</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="1364" spans="1:2">
       <c r="A1364" s="34" t="s">
-        <v>2180</v>
-      </c>
-      <c r="B1364" s="35" t="s">
-        <v>2181</v>
+        <v>2183</v>
+      </c>
+      <c r="B1364" s="34" t="s">
+        <v>2184</v>
       </c>
     </row>
     <row r="1365" spans="1:2">
       <c r="A1365" s="34" t="s">
-        <v>2182</v>
-      </c>
-      <c r="B1365" s="35" t="s">
-        <v>2036</v>
+        <v>2185</v>
+      </c>
+      <c r="B1365" s="34" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="1366" spans="1:2">
       <c r="A1366" s="34" t="s">
-        <v>2183</v>
+        <v>193</v>
       </c>
       <c r="B1366" s="34" t="s">
-        <v>2184</v>
+        <v>193</v>
       </c>
     </row>
     <row r="1367" spans="1:2">
       <c r="A1367" s="34" t="s">
-        <v>2185</v>
-      </c>
-      <c r="B1367" s="34" t="s">
-        <v>351</v>
+        <v>2186</v>
+      </c>
+      <c r="B1367" s="35" t="s">
+        <v>2187</v>
       </c>
     </row>
     <row r="1368" spans="1:2">
       <c r="A1368" s="34" t="s">
-        <v>193</v>
-      </c>
-      <c r="B1368" s="34" t="s">
-        <v>193</v>
+        <v>2188</v>
+      </c>
+      <c r="B1368" s="35" t="s">
+        <v>2189</v>
       </c>
     </row>
     <row r="1369" spans="1:2">
       <c r="A1369" s="34" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="B1369" s="35" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="1370" spans="1:2">
       <c r="A1370" s="34" t="s">
-        <v>2188</v>
+        <v>2192</v>
       </c>
       <c r="B1370" s="35" t="s">
-        <v>2189</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="1371" spans="1:2">
       <c r="A1371" s="34" t="s">
-        <v>2190</v>
+        <v>2194</v>
       </c>
       <c r="B1371" s="35" t="s">
-        <v>2191</v>
+        <v>2195</v>
       </c>
     </row>
     <row r="1372" spans="1:2">
       <c r="A1372" s="34" t="s">
-        <v>2192</v>
+        <v>2196</v>
       </c>
       <c r="B1372" s="35" t="s">
-        <v>2193</v>
+        <v>405</v>
       </c>
     </row>
     <row r="1373" spans="1:2">
       <c r="A1373" s="34" t="s">
-        <v>2194</v>
+        <v>2126</v>
       </c>
       <c r="B1373" s="35" t="s">
-        <v>2195</v>
+        <v>2127</v>
       </c>
     </row>
     <row r="1374" spans="1:2">
       <c r="A1374" s="34" t="s">
-        <v>2196</v>
+        <v>2197</v>
       </c>
       <c r="B1374" s="35" t="s">
-        <v>405</v>
+        <v>2198</v>
       </c>
     </row>
     <row r="1375" spans="1:2">
-      <c r="A1375" s="34" t="s">
-        <v>2126</v>
-      </c>
-      <c r="B1375" s="35" t="s">
-        <v>2127</v>
+      <c r="A1375" s="72" t="s">
+        <v>2199</v>
+      </c>
+      <c r="B1375" s="72" t="s">
+        <v>2200</v>
       </c>
     </row>
     <row r="1376" spans="1:2">
       <c r="A1376" s="34" t="s">
-        <v>2197</v>
+        <v>2321</v>
       </c>
       <c r="B1376" s="35" t="s">
-        <v>2198</v>
-      </c>
-    </row>
-    <row r="1377" spans="1:2">
-      <c r="A1377" s="72" t="s">
-        <v>2199</v>
-      </c>
-      <c r="B1377" s="72" t="s">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="1378" spans="1:2">
-      <c r="A1378" s="34" t="s">
-        <v>2321</v>
-      </c>
-      <c r="B1378" s="35" t="s">
         <v>1819</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1211" r:id="rId1"/>
-    <hyperlink ref="B1366" r:id="rId2"/>
+    <hyperlink ref="B1209" r:id="rId1"/>
+    <hyperlink ref="B1364" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Subcontract Functions And New Scenarios Added
Updated Subcontract Functions And New Scenarios Added
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2849" uniqueCount="2322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2967" uniqueCount="2436">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -9149,6 +9149,348 @@
   </si>
   <si>
     <t>CloseShortStatus</t>
+  </si>
+  <si>
+    <t>SCODBLOCATIONCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_PLNT_LOC_ID</t>
+  </si>
+  <si>
+    <t>SCODBPREFIXCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_ORDER_PFX</t>
+  </si>
+  <si>
+    <t>SCODBDOCNOCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_ORDER_NO</t>
+  </si>
+  <si>
+    <t>SCODBTYPECOLUMN</t>
+  </si>
+  <si>
+    <t>TYPE1</t>
+  </si>
+  <si>
+    <t>SCODBSUPPLIERIDCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_SUPLR_ID</t>
+  </si>
+  <si>
+    <t>SCODBSUPPLIERNAMECOLUMN</t>
+  </si>
+  <si>
+    <t>POH_SUPLR_NAME</t>
+  </si>
+  <si>
+    <t>SCODBCURCYCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_CURRENCY</t>
+  </si>
+  <si>
+    <t>SCODBEXRATECOLUMN</t>
+  </si>
+  <si>
+    <t>POH_EXCHANGE_RATE</t>
+  </si>
+  <si>
+    <t>SCODBMATAMTCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_MAT_AMT</t>
+  </si>
+  <si>
+    <t>SCODBTAXAMTCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_TAX_AMT</t>
+  </si>
+  <si>
+    <t>SCODBTOTALAMTCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_TOTAL_AMT</t>
+  </si>
+  <si>
+    <t>SCODBSTATUSCOLUMN</t>
+  </si>
+  <si>
+    <t>POH_STATUS1</t>
+  </si>
+  <si>
+    <t>SCONO</t>
+  </si>
+  <si>
+    <t>${SCONO}</t>
+  </si>
+  <si>
+    <t>SCODBITEMCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_PROD_ID</t>
+  </si>
+  <si>
+    <t>SCODBQTYCOLUMN</t>
+  </si>
+  <si>
+    <t>SCODBUNITCOLUMN</t>
+  </si>
+  <si>
+    <t>SCODBHSNCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_HSN_CODE</t>
+  </si>
+  <si>
+    <t>SCODBPROCESSUOMCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_UOM</t>
+  </si>
+  <si>
+    <t>SCODBBATCHQTYCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_BATCH_QTY</t>
+  </si>
+  <si>
+    <t>SCODBBATCHCOSTCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_BATCH_COST</t>
+  </si>
+  <si>
+    <t>SCODBCONVFACTORCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_CONV_FACTOR</t>
+  </si>
+  <si>
+    <t>SCODBJOBWORKITEMCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_PROD_ID</t>
+  </si>
+  <si>
+    <t>SCODBJOBWORKITEMDESCCOLUMN</t>
+  </si>
+  <si>
+    <t>SCODBSACCODECOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_HSN_CODE</t>
+  </si>
+  <si>
+    <t>SCODBPROCQTYCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_PROC_QTY</t>
+  </si>
+  <si>
+    <t>SCODBPROCUNITCOSTCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_LAB_COST</t>
+  </si>
+  <si>
+    <t>SCODBPROCESSTAXCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_IGST_PCT</t>
+  </si>
+  <si>
+    <t>SCODBASBLVALUECOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_ASSBL_VAL</t>
+  </si>
+  <si>
+    <t>SCODBIGSTAMTCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_IGST_AMT</t>
+  </si>
+  <si>
+    <t>SCODBCONTRPREFIXCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_CONTR_PFX</t>
+  </si>
+  <si>
+    <t>SCODBCONTRNOCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_CONTR_NO</t>
+  </si>
+  <si>
+    <t>SCODBCGSTAMTCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_CGST_AMT</t>
+  </si>
+  <si>
+    <t>SCODBSGSTAMTCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_SGST_AMT</t>
+  </si>
+  <si>
+    <t>SCODBUTGSTAMTCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_UTGST_AMT</t>
+  </si>
+  <si>
+    <t>SCODBCESSAMTCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_CESS_AMT</t>
+  </si>
+  <si>
+    <t>SCODBPROCESSDESCCOLUMN</t>
+  </si>
+  <si>
+    <t>SCOP_PROCESS_DESC</t>
+  </si>
+  <si>
+    <t>SCODBMATTYPECOLUMN</t>
+  </si>
+  <si>
+    <t>SCODBMATWHDESCCOLUMN</t>
+  </si>
+  <si>
+    <t>WH_DESC</t>
+  </si>
+  <si>
+    <t>SCODBMATITEMCOLUMN</t>
+  </si>
+  <si>
+    <t>SCMRL_PROD_ID</t>
+  </si>
+  <si>
+    <t>SCODBMATQTYCOLUMN</t>
+  </si>
+  <si>
+    <t>SCMRL_RQRD_QTY</t>
+  </si>
+  <si>
+    <t>SCODBMATTARNOCOLUMN</t>
+  </si>
+  <si>
+    <t>SCMRL_OPRN_LN_SEQ_NO</t>
+  </si>
+  <si>
+    <t>SCODBMATTARPROCESSCOLUMN</t>
+  </si>
+  <si>
+    <t>TAR_PROCESS</t>
+  </si>
+  <si>
+    <t>SCODBINPUTTYPECOLUMN</t>
+  </si>
+  <si>
+    <t>POL_GST_INPUT_TYPE</t>
+  </si>
+  <si>
+    <t>SCODBGSTTYPECOLUMN</t>
+  </si>
+  <si>
+    <t>POL_GST_EXEMPT_FLAG</t>
+  </si>
+  <si>
+    <t>SCODBLINEWHIDCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_STORE_ID</t>
+  </si>
+  <si>
+    <t>SCODBLINEWHDESCCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_STORE_NAME</t>
+  </si>
+  <si>
+    <t>SCODBSALEORDERDESCCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_SO_SCHLD_DESC</t>
+  </si>
+  <si>
+    <t>SCODBLINESTATUSCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_STATUS1</t>
+  </si>
+  <si>
+    <t>SCODBCSQTYCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_CLS_QTY</t>
+  </si>
+  <si>
+    <t>SCODBPRODNOCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_PROD_ORD_NO</t>
+  </si>
+  <si>
+    <t>SCODBSFCODECOLUMN</t>
+  </si>
+  <si>
+    <t>POL_SF_CODE</t>
+  </si>
+  <si>
+    <t>SCODBTARSFCODECOLUMN</t>
+  </si>
+  <si>
+    <t>POL_TARG_SF_CODE</t>
+  </si>
+  <si>
+    <t>SCODBTAROPERNOCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_TAR_OPRN_SEQ</t>
+  </si>
+  <si>
+    <t>SCODBTAROPERDESCCODECOLUMN</t>
+  </si>
+  <si>
+    <t>TAR_OPRN_DESC</t>
+  </si>
+  <si>
+    <t>SCODBSOUOPERNOCOLUMN</t>
+  </si>
+  <si>
+    <t>POL_SOU_OPRN_SEQ</t>
+  </si>
+  <si>
+    <t>SCODBSOUOPERDESCCOLUMN</t>
+  </si>
+  <si>
+    <t>SOU_OPRN_DESC</t>
+  </si>
+  <si>
+    <t>SCODBLOCATIONGSTTYPECOLUMN</t>
+  </si>
+  <si>
+    <t>POH_GST_TYPE</t>
+  </si>
+  <si>
+    <t>SCODBLOCATIONGSTCLSFTYPECOLUMN</t>
+  </si>
+  <si>
+    <t>POH_GST_CLF_TYPE</t>
+  </si>
+  <si>
+    <t>BomForSerialItem</t>
+  </si>
+  <si>
+    <t>VR-SERIAL-FIFO-BATCH-90001</t>
   </si>
 </sst>
 </file>
@@ -9739,7 +10081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1376"/>
+  <dimension ref="A1:B1435"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
@@ -20753,6 +21095,478 @@
       </c>
       <c r="B1376" s="35" t="s">
         <v>1819</v>
+      </c>
+    </row>
+    <row r="1377" spans="1:2">
+      <c r="A1377" s="34" t="s">
+        <v>2322</v>
+      </c>
+      <c r="B1377" s="35" t="s">
+        <v>2323</v>
+      </c>
+    </row>
+    <row r="1378" spans="1:2">
+      <c r="A1378" s="34" t="s">
+        <v>2324</v>
+      </c>
+      <c r="B1378" s="35" t="s">
+        <v>2325</v>
+      </c>
+    </row>
+    <row r="1379" spans="1:2">
+      <c r="A1379" s="34" t="s">
+        <v>2326</v>
+      </c>
+      <c r="B1379" s="35" t="s">
+        <v>2327</v>
+      </c>
+    </row>
+    <row r="1380" spans="1:2">
+      <c r="A1380" s="34" t="s">
+        <v>2328</v>
+      </c>
+      <c r="B1380" s="35" t="s">
+        <v>2329</v>
+      </c>
+    </row>
+    <row r="1381" spans="1:2">
+      <c r="A1381" s="34" t="s">
+        <v>2330</v>
+      </c>
+      <c r="B1381" s="35" t="s">
+        <v>2331</v>
+      </c>
+    </row>
+    <row r="1382" spans="1:2">
+      <c r="A1382" s="34" t="s">
+        <v>2332</v>
+      </c>
+      <c r="B1382" s="35" t="s">
+        <v>2333</v>
+      </c>
+    </row>
+    <row r="1383" spans="1:2">
+      <c r="A1383" s="34" t="s">
+        <v>2334</v>
+      </c>
+      <c r="B1383" s="35" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1384" spans="1:2">
+      <c r="A1384" s="34" t="s">
+        <v>2336</v>
+      </c>
+      <c r="B1384" s="35" t="s">
+        <v>2337</v>
+      </c>
+    </row>
+    <row r="1385" spans="1:2">
+      <c r="A1385" s="34" t="s">
+        <v>2338</v>
+      </c>
+      <c r="B1385" s="35" t="s">
+        <v>2339</v>
+      </c>
+    </row>
+    <row r="1386" spans="1:2">
+      <c r="A1386" s="34" t="s">
+        <v>2340</v>
+      </c>
+      <c r="B1386" s="35" t="s">
+        <v>2341</v>
+      </c>
+    </row>
+    <row r="1387" spans="1:2">
+      <c r="A1387" s="34" t="s">
+        <v>2342</v>
+      </c>
+      <c r="B1387" s="35" t="s">
+        <v>2343</v>
+      </c>
+    </row>
+    <row r="1388" spans="1:2">
+      <c r="A1388" s="34" t="s">
+        <v>2344</v>
+      </c>
+      <c r="B1388" s="35" t="s">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="1389" spans="1:2">
+      <c r="A1389" s="34" t="s">
+        <v>2346</v>
+      </c>
+      <c r="B1389" s="35" t="s">
+        <v>2347</v>
+      </c>
+    </row>
+    <row r="1390" spans="1:2">
+      <c r="A1390" s="34" t="s">
+        <v>2348</v>
+      </c>
+      <c r="B1390" s="35" t="s">
+        <v>2349</v>
+      </c>
+    </row>
+    <row r="1391" spans="1:2">
+      <c r="A1391" s="34" t="s">
+        <v>2350</v>
+      </c>
+      <c r="B1391" s="35" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="1392" spans="1:2">
+      <c r="A1392" s="34" t="s">
+        <v>2351</v>
+      </c>
+      <c r="B1392" s="35" t="s">
+        <v>1370</v>
+      </c>
+    </row>
+    <row r="1393" spans="1:2">
+      <c r="A1393" s="34" t="s">
+        <v>2352</v>
+      </c>
+      <c r="B1393" s="35" t="s">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="1394" spans="1:2">
+      <c r="A1394" s="34" t="s">
+        <v>2354</v>
+      </c>
+      <c r="B1394" s="35" t="s">
+        <v>2355</v>
+      </c>
+    </row>
+    <row r="1395" spans="1:2">
+      <c r="A1395" s="34" t="s">
+        <v>2356</v>
+      </c>
+      <c r="B1395" s="35" t="s">
+        <v>2357</v>
+      </c>
+    </row>
+    <row r="1396" spans="1:2">
+      <c r="A1396" s="34" t="s">
+        <v>2358</v>
+      </c>
+      <c r="B1396" s="35" t="s">
+        <v>2359</v>
+      </c>
+    </row>
+    <row r="1397" spans="1:2">
+      <c r="A1397" s="34" t="s">
+        <v>2360</v>
+      </c>
+      <c r="B1397" s="35" t="s">
+        <v>2361</v>
+      </c>
+    </row>
+    <row r="1398" spans="1:2">
+      <c r="A1398" s="34" t="s">
+        <v>2362</v>
+      </c>
+      <c r="B1398" s="35" t="s">
+        <v>2363</v>
+      </c>
+    </row>
+    <row r="1399" spans="1:2">
+      <c r="A1399" s="34" t="s">
+        <v>2364</v>
+      </c>
+      <c r="B1399" s="35" t="s">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="1400" spans="1:2">
+      <c r="A1400" s="34" t="s">
+        <v>2365</v>
+      </c>
+      <c r="B1400" s="35" t="s">
+        <v>2366</v>
+      </c>
+    </row>
+    <row r="1401" spans="1:2">
+      <c r="A1401" s="34" t="s">
+        <v>2367</v>
+      </c>
+      <c r="B1401" s="35" t="s">
+        <v>2368</v>
+      </c>
+    </row>
+    <row r="1402" spans="1:2">
+      <c r="A1402" s="34" t="s">
+        <v>2369</v>
+      </c>
+      <c r="B1402" s="35" t="s">
+        <v>2370</v>
+      </c>
+    </row>
+    <row r="1403" spans="1:2">
+      <c r="A1403" s="34" t="s">
+        <v>2371</v>
+      </c>
+      <c r="B1403" s="35" t="s">
+        <v>2372</v>
+      </c>
+    </row>
+    <row r="1404" spans="1:2">
+      <c r="A1404" s="34" t="s">
+        <v>2373</v>
+      </c>
+      <c r="B1404" s="35" t="s">
+        <v>2374</v>
+      </c>
+    </row>
+    <row r="1405" spans="1:2">
+      <c r="A1405" s="34" t="s">
+        <v>2375</v>
+      </c>
+      <c r="B1405" s="35" t="s">
+        <v>2376</v>
+      </c>
+    </row>
+    <row r="1406" spans="1:2">
+      <c r="A1406" s="34" t="s">
+        <v>2377</v>
+      </c>
+      <c r="B1406" s="35" t="s">
+        <v>2378</v>
+      </c>
+    </row>
+    <row r="1407" spans="1:2">
+      <c r="A1407" s="34" t="s">
+        <v>2379</v>
+      </c>
+      <c r="B1407" s="35" t="s">
+        <v>2380</v>
+      </c>
+    </row>
+    <row r="1408" spans="1:2">
+      <c r="A1408" s="34" t="s">
+        <v>2381</v>
+      </c>
+      <c r="B1408" s="35" t="s">
+        <v>2382</v>
+      </c>
+    </row>
+    <row r="1409" spans="1:2">
+      <c r="A1409" s="34" t="s">
+        <v>2383</v>
+      </c>
+      <c r="B1409" s="35" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="1410" spans="1:2">
+      <c r="A1410" s="34" t="s">
+        <v>2385</v>
+      </c>
+      <c r="B1410" s="35" t="s">
+        <v>2386</v>
+      </c>
+    </row>
+    <row r="1411" spans="1:2">
+      <c r="A1411" s="34" t="s">
+        <v>2387</v>
+      </c>
+      <c r="B1411" s="35" t="s">
+        <v>2388</v>
+      </c>
+    </row>
+    <row r="1412" spans="1:2">
+      <c r="A1412" s="34" t="s">
+        <v>2389</v>
+      </c>
+      <c r="B1412" s="35" t="s">
+        <v>2390</v>
+      </c>
+    </row>
+    <row r="1413" spans="1:2">
+      <c r="A1413" s="34" t="s">
+        <v>2391</v>
+      </c>
+      <c r="B1413" s="35" t="s">
+        <v>2329</v>
+      </c>
+    </row>
+    <row r="1414" spans="1:2">
+      <c r="A1414" s="34" t="s">
+        <v>2392</v>
+      </c>
+      <c r="B1414" s="35" t="s">
+        <v>2393</v>
+      </c>
+    </row>
+    <row r="1415" spans="1:2">
+      <c r="A1415" s="34" t="s">
+        <v>2394</v>
+      </c>
+      <c r="B1415" s="35" t="s">
+        <v>2395</v>
+      </c>
+    </row>
+    <row r="1416" spans="1:2">
+      <c r="A1416" s="34" t="s">
+        <v>2396</v>
+      </c>
+      <c r="B1416" s="35" t="s">
+        <v>2397</v>
+      </c>
+    </row>
+    <row r="1417" spans="1:2">
+      <c r="A1417" s="34" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B1417" s="35" t="s">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="1418" spans="1:2">
+      <c r="A1418" s="34" t="s">
+        <v>2400</v>
+      </c>
+      <c r="B1418" s="35" t="s">
+        <v>2401</v>
+      </c>
+    </row>
+    <row r="1419" spans="1:2">
+      <c r="A1419" s="34" t="s">
+        <v>2402</v>
+      </c>
+      <c r="B1419" s="35" t="s">
+        <v>2403</v>
+      </c>
+    </row>
+    <row r="1420" spans="1:2">
+      <c r="A1420" s="34" t="s">
+        <v>2404</v>
+      </c>
+      <c r="B1420" s="35" t="s">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="1421" spans="1:2">
+      <c r="A1421" s="34" t="s">
+        <v>2406</v>
+      </c>
+      <c r="B1421" s="35" t="s">
+        <v>2407</v>
+      </c>
+    </row>
+    <row r="1422" spans="1:2">
+      <c r="A1422" s="34" t="s">
+        <v>2408</v>
+      </c>
+      <c r="B1422" s="35" t="s">
+        <v>2409</v>
+      </c>
+    </row>
+    <row r="1423" spans="1:2">
+      <c r="A1423" s="34" t="s">
+        <v>2410</v>
+      </c>
+      <c r="B1423" s="35" t="s">
+        <v>2411</v>
+      </c>
+    </row>
+    <row r="1424" spans="1:2">
+      <c r="A1424" s="34" t="s">
+        <v>2412</v>
+      </c>
+      <c r="B1424" s="35" t="s">
+        <v>2413</v>
+      </c>
+    </row>
+    <row r="1425" spans="1:2">
+      <c r="A1425" s="34" t="s">
+        <v>2414</v>
+      </c>
+      <c r="B1425" s="35" t="s">
+        <v>2415</v>
+      </c>
+    </row>
+    <row r="1426" spans="1:2">
+      <c r="A1426" s="34" t="s">
+        <v>2416</v>
+      </c>
+      <c r="B1426" s="35" t="s">
+        <v>2417</v>
+      </c>
+    </row>
+    <row r="1427" spans="1:2">
+      <c r="A1427" s="34" t="s">
+        <v>2418</v>
+      </c>
+      <c r="B1427" s="35" t="s">
+        <v>2419</v>
+      </c>
+    </row>
+    <row r="1428" spans="1:2">
+      <c r="A1428" s="34" t="s">
+        <v>2420</v>
+      </c>
+      <c r="B1428" s="35" t="s">
+        <v>2421</v>
+      </c>
+    </row>
+    <row r="1429" spans="1:2">
+      <c r="A1429" s="34" t="s">
+        <v>2422</v>
+      </c>
+      <c r="B1429" s="35" t="s">
+        <v>2423</v>
+      </c>
+    </row>
+    <row r="1430" spans="1:2">
+      <c r="A1430" s="34" t="s">
+        <v>2424</v>
+      </c>
+      <c r="B1430" s="35" t="s">
+        <v>2425</v>
+      </c>
+    </row>
+    <row r="1431" spans="1:2">
+      <c r="A1431" s="34" t="s">
+        <v>2426</v>
+      </c>
+      <c r="B1431" s="35" t="s">
+        <v>2427</v>
+      </c>
+    </row>
+    <row r="1432" spans="1:2">
+      <c r="A1432" s="34" t="s">
+        <v>2428</v>
+      </c>
+      <c r="B1432" s="35" t="s">
+        <v>2429</v>
+      </c>
+    </row>
+    <row r="1433" spans="1:2">
+      <c r="A1433" s="34" t="s">
+        <v>2430</v>
+      </c>
+      <c r="B1433" s="35" t="s">
+        <v>2431</v>
+      </c>
+    </row>
+    <row r="1434" spans="1:2">
+      <c r="A1434" s="34" t="s">
+        <v>2432</v>
+      </c>
+      <c r="B1434" s="35" t="s">
+        <v>2433</v>
+      </c>
+    </row>
+    <row r="1435" spans="1:2">
+      <c r="A1435" s="34" t="s">
+        <v>2434</v>
+      </c>
+      <c r="B1435" s="35" t="s">
+        <v>2435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Customer Item Functions , Open so Functions , OpenSo Amd  Function , Locators are Fixes Changed
Customer Item Functions , Open so Functions , OpenSo Amd  Function , Locators are Fixes Changed
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="125725"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2987" uniqueCount="2455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2989" uniqueCount="2457">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -9955,18 +9955,18 @@
        AND poh_mode = 'SC'
        AND poh_order_no ='${SCONO}'</t>
   </si>
+  <si>
+    <t>Prefix_07</t>
+  </si>
+  <si>
+    <t>OPSO7</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="26">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -10013,151 +10013,14 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -10182,194 +10045,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -10405,268 +10082,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="66">
+  <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -10684,48 +10119,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="15" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="64" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="64" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="16" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="16" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="53"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -10754,15 +10189,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -10782,11 +10217,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -10800,19 +10235,19 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="59" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="60" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -10827,74 +10262,27 @@
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="66">
+  <cellStyles count="18">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 10" xfId="49"/>
-    <cellStyle name="Normal 11" xfId="50"/>
-    <cellStyle name="Normal 13" xfId="51"/>
-    <cellStyle name="Normal 14" xfId="52"/>
-    <cellStyle name="Normal 15" xfId="53"/>
-    <cellStyle name="Normal 16" xfId="54"/>
-    <cellStyle name="Normal 17" xfId="55"/>
-    <cellStyle name="Normal 18" xfId="56"/>
-    <cellStyle name="Normal 19" xfId="57"/>
-    <cellStyle name="Normal 2" xfId="58"/>
-    <cellStyle name="Normal 2 2" xfId="59"/>
-    <cellStyle name="Normal 2 3" xfId="60"/>
-    <cellStyle name="Normal 20" xfId="61"/>
-    <cellStyle name="Normal 3" xfId="62"/>
-    <cellStyle name="Normal 7" xfId="63"/>
-    <cellStyle name="Normal 8" xfId="64"/>
-    <cellStyle name="Normal 9" xfId="65"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Normal 11" xfId="2"/>
+    <cellStyle name="Normal 13" xfId="3"/>
+    <cellStyle name="Normal 14" xfId="4"/>
+    <cellStyle name="Normal 15" xfId="5"/>
+    <cellStyle name="Normal 16" xfId="6"/>
+    <cellStyle name="Normal 17" xfId="7"/>
+    <cellStyle name="Normal 18" xfId="8"/>
+    <cellStyle name="Normal 19" xfId="9"/>
+    <cellStyle name="Normal 2" xfId="10"/>
+    <cellStyle name="Normal 2 2" xfId="11"/>
+    <cellStyle name="Normal 2 3" xfId="12"/>
+    <cellStyle name="Normal 20" xfId="13"/>
+    <cellStyle name="Normal 3" xfId="14"/>
+    <cellStyle name="Normal 7" xfId="15"/>
+    <cellStyle name="Normal 8" xfId="16"/>
+    <cellStyle name="Normal 9" xfId="17"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -11156,17 +10544,17 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B1440"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5" outlineLevelCol="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B1441"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="62.7090909090909" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.8545454545455" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.85546875" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -22690,23 +22078,29 @@
         <v>2325</v>
       </c>
     </row>
+    <row r="1441" spans="1:2">
+      <c r="A1441" s="34" t="s">
+        <v>2455</v>
+      </c>
+      <c r="B1441" s="35" t="s">
+        <v>2456</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1209" r:id="rId1" display="MRAD-2425-00086"/>
-    <hyperlink ref="B1364" r:id="rId2" display="RFQ10/00725/25-26"/>
+    <hyperlink ref="B1209" r:id="rId1"/>
+    <hyperlink ref="B1364" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B70"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -22718,7 +22112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="108.95" customHeight="1" spans="1:2">
+    <row r="2" spans="1:2" ht="108.95" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2326</v>
       </c>
@@ -22726,7 +22120,7 @@
         <v>2327</v>
       </c>
     </row>
-    <row r="3" ht="114" customHeight="1" spans="1:2">
+    <row r="3" spans="1:2" ht="114" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>2328</v>
       </c>
@@ -22734,7 +22128,7 @@
         <v>2329</v>
       </c>
     </row>
-    <row r="4" ht="80.25" customHeight="1" spans="1:2">
+    <row r="4" spans="1:2" ht="80.25" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>2330</v>
       </c>
@@ -22742,7 +22136,7 @@
         <v>2331</v>
       </c>
     </row>
-    <row r="5" ht="69.75" customHeight="1" spans="1:2">
+    <row r="5" spans="1:2" ht="69.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2332</v>
       </c>
@@ -22750,7 +22144,7 @@
         <v>2333</v>
       </c>
     </row>
-    <row r="6" ht="51.75" customHeight="1" spans="1:2">
+    <row r="6" spans="1:2" ht="51.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>2334</v>
       </c>
@@ -22758,7 +22152,7 @@
         <v>2335</v>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" spans="1:2">
+    <row r="7" spans="1:2" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>2336</v>
       </c>
@@ -22766,7 +22160,7 @@
         <v>2337</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:2">
+    <row r="8" spans="1:2" ht="18" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>2338</v>
       </c>
@@ -22774,7 +22168,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="9" ht="39" customHeight="1" spans="1:2">
+    <row r="9" spans="1:2" ht="39" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>2340</v>
       </c>
@@ -22782,7 +22176,7 @@
         <v>2341</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1" spans="1:2">
+    <row r="10" spans="1:2" ht="22.5" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>2342</v>
       </c>
@@ -22790,7 +22184,7 @@
         <v>2343</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" spans="1:2">
+    <row r="11" spans="1:2" ht="18" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>2344</v>
       </c>
@@ -22798,7 +22192,7 @@
         <v>2345</v>
       </c>
     </row>
-    <row r="12" ht="26.25" customHeight="1" spans="1:2">
+    <row r="12" spans="1:2" ht="26.25" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>2346</v>
       </c>
@@ -22806,7 +22200,7 @@
         <v>2347</v>
       </c>
     </row>
-    <row r="13" ht="28.5" customHeight="1" spans="1:2">
+    <row r="13" spans="1:2" ht="28.5" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>2348</v>
       </c>
@@ -22814,7 +22208,7 @@
         <v>2349</v>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" spans="1:2">
+    <row r="14" spans="1:2" ht="24" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>2350</v>
       </c>
@@ -22822,7 +22216,7 @@
         <v>2351</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:2">
+    <row r="15" spans="1:2" ht="36" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>2352</v>
       </c>
@@ -22830,7 +22224,7 @@
         <v>2353</v>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1" spans="1:2">
+    <row r="16" spans="1:2" ht="45" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>2354</v>
       </c>
@@ -22838,7 +22232,7 @@
         <v>2355</v>
       </c>
     </row>
-    <row r="17" ht="43.5" customHeight="1" spans="1:2">
+    <row r="17" spans="1:2" ht="43.5" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>2356</v>
       </c>
@@ -22846,7 +22240,7 @@
         <v>2357</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1" spans="1:2">
+    <row r="18" spans="1:2" ht="42" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>2358</v>
       </c>
@@ -22854,7 +22248,7 @@
         <v>2359</v>
       </c>
     </row>
-    <row r="19" ht="52.5" customHeight="1" spans="1:2">
+    <row r="19" spans="1:2" ht="52.5" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>2360</v>
       </c>
@@ -22862,7 +22256,7 @@
         <v>2361</v>
       </c>
     </row>
-    <row r="20" ht="17.25" customHeight="1" spans="1:2">
+    <row r="20" spans="1:2" ht="17.25" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>2362</v>
       </c>
@@ -22870,7 +22264,7 @@
         <v>2363</v>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:2">
+    <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>2364</v>
       </c>
@@ -22878,7 +22272,7 @@
         <v>2365</v>
       </c>
     </row>
-    <row r="22" ht="409.5" spans="1:2">
+    <row r="22" spans="1:2" ht="409.5">
       <c r="A22" s="2" t="s">
         <v>2366</v>
       </c>
@@ -22886,7 +22280,7 @@
         <v>2367</v>
       </c>
     </row>
-    <row r="23" ht="246.5" spans="1:2">
+    <row r="23" spans="1:2" ht="255">
       <c r="A23" s="2" t="s">
         <v>2368</v>
       </c>
@@ -22894,7 +22288,7 @@
         <v>2369</v>
       </c>
     </row>
-    <row r="24" ht="232" spans="1:2">
+    <row r="24" spans="1:2" ht="240">
       <c r="A24" t="s">
         <v>2370</v>
       </c>
@@ -22902,7 +22296,7 @@
         <v>2371</v>
       </c>
     </row>
-    <row r="25" ht="261" spans="1:2">
+    <row r="25" spans="1:2" ht="270">
       <c r="A25" t="s">
         <v>2372</v>
       </c>
@@ -22910,7 +22304,7 @@
         <v>2373</v>
       </c>
     </row>
-    <row r="26" ht="203" spans="1:2">
+    <row r="26" spans="1:2" ht="210">
       <c r="A26" t="s">
         <v>2374</v>
       </c>
@@ -22918,7 +22312,7 @@
         <v>2375</v>
       </c>
     </row>
-    <row r="27" ht="61.5" customHeight="1" spans="1:2">
+    <row r="27" spans="1:2" ht="61.5" customHeight="1">
       <c r="A27" t="s">
         <v>2376</v>
       </c>
@@ -22926,7 +22320,7 @@
         <v>2377</v>
       </c>
     </row>
-    <row r="28" ht="105.75" customHeight="1" spans="1:2">
+    <row r="28" spans="1:2" ht="105.75" customHeight="1">
       <c r="A28" s="7" t="s">
         <v>2326</v>
       </c>
@@ -22934,7 +22328,7 @@
         <v>2327</v>
       </c>
     </row>
-    <row r="29" ht="83.25" customHeight="1" spans="1:2">
+    <row r="29" spans="1:2" ht="83.25" customHeight="1">
       <c r="A29" s="9" t="s">
         <v>2328</v>
       </c>
@@ -22942,7 +22336,7 @@
         <v>2329</v>
       </c>
     </row>
-    <row r="30" ht="174" spans="1:2">
+    <row r="30" spans="1:2" ht="180">
       <c r="A30" s="11" t="s">
         <v>2334</v>
       </c>
@@ -22950,7 +22344,7 @@
         <v>2335</v>
       </c>
     </row>
-    <row r="31" ht="130.5" spans="1:2">
+    <row r="31" spans="1:2" ht="135">
       <c r="A31" s="13" t="s">
         <v>2378</v>
       </c>
@@ -22958,7 +22352,7 @@
         <v>2379</v>
       </c>
     </row>
-    <row r="32" ht="174" spans="1:2">
+    <row r="32" spans="1:2" ht="180">
       <c r="A32" s="15" t="s">
         <v>2380</v>
       </c>
@@ -22966,7 +22360,7 @@
         <v>2381</v>
       </c>
     </row>
-    <row r="33" ht="174" spans="1:2">
+    <row r="33" spans="1:2" ht="180">
       <c r="A33" s="17" t="s">
         <v>2382</v>
       </c>
@@ -22974,7 +22368,7 @@
         <v>2383</v>
       </c>
     </row>
-    <row r="34" ht="409.5" spans="1:2">
+    <row r="34" spans="1:2" ht="409.5">
       <c r="A34" s="19" t="s">
         <v>2384</v>
       </c>
@@ -22982,7 +22376,7 @@
         <v>2385</v>
       </c>
     </row>
-    <row r="35" ht="406" spans="1:2">
+    <row r="35" spans="1:2" ht="409.5">
       <c r="A35" s="21" t="s">
         <v>2386</v>
       </c>
@@ -22990,7 +22384,7 @@
         <v>2387</v>
       </c>
     </row>
-    <row r="36" ht="409.5" spans="1:2">
+    <row r="36" spans="1:2" ht="409.5">
       <c r="A36" s="23" t="s">
         <v>2388</v>
       </c>
@@ -22998,7 +22392,7 @@
         <v>2389</v>
       </c>
     </row>
-    <row r="37" ht="409.5" spans="1:2">
+    <row r="37" spans="1:2" ht="409.5">
       <c r="A37" s="25" t="s">
         <v>2390</v>
       </c>
@@ -23006,7 +22400,7 @@
         <v>2391</v>
       </c>
     </row>
-    <row r="38" ht="409.5" spans="1:2">
+    <row r="38" spans="1:2" ht="409.5">
       <c r="A38" s="27" t="s">
         <v>2392</v>
       </c>
@@ -23014,7 +22408,7 @@
         <v>2393</v>
       </c>
     </row>
-    <row r="39" ht="409.5" spans="1:2">
+    <row r="39" spans="1:2" ht="409.5">
       <c r="A39" t="s">
         <v>2394</v>
       </c>
@@ -23022,7 +22416,7 @@
         <v>2395</v>
       </c>
     </row>
-    <row r="40" ht="116" spans="1:2">
+    <row r="40" spans="1:2" ht="120">
       <c r="A40" t="s">
         <v>2396</v>
       </c>
@@ -23030,7 +22424,7 @@
         <v>2397</v>
       </c>
     </row>
-    <row r="41" ht="174" spans="1:2">
+    <row r="41" spans="1:2" ht="180">
       <c r="A41" t="s">
         <v>2398</v>
       </c>
@@ -23038,7 +22432,7 @@
         <v>2399</v>
       </c>
     </row>
-    <row r="42" ht="188.5" spans="1:2">
+    <row r="42" spans="1:2" ht="195">
       <c r="A42" t="s">
         <v>2400</v>
       </c>
@@ -23046,7 +22440,7 @@
         <v>2401</v>
       </c>
     </row>
-    <row r="43" ht="116" spans="1:2">
+    <row r="43" spans="1:2" ht="120">
       <c r="A43" t="s">
         <v>2402</v>
       </c>
@@ -23054,7 +22448,7 @@
         <v>2403</v>
       </c>
     </row>
-    <row r="44" ht="409.5" spans="1:2">
+    <row r="44" spans="1:2" ht="409.5">
       <c r="A44" t="s">
         <v>2404</v>
       </c>
@@ -23062,7 +22456,7 @@
         <v>2405</v>
       </c>
     </row>
-    <row r="45" ht="409.5" spans="1:2">
+    <row r="45" spans="1:2" ht="409.5">
       <c r="A45" t="s">
         <v>2406</v>
       </c>
@@ -23070,7 +22464,7 @@
         <v>2407</v>
       </c>
     </row>
-    <row r="46" ht="409.5" spans="1:2">
+    <row r="46" spans="1:2" ht="409.5">
       <c r="A46" t="s">
         <v>2408</v>
       </c>
@@ -23078,7 +22472,7 @@
         <v>2409</v>
       </c>
     </row>
-    <row r="47" ht="261" spans="1:2">
+    <row r="47" spans="1:2" ht="270">
       <c r="A47" t="s">
         <v>2410</v>
       </c>
@@ -23086,7 +22480,7 @@
         <v>2411</v>
       </c>
     </row>
-    <row r="48" ht="409.5" spans="1:2">
+    <row r="48" spans="1:2" ht="409.5">
       <c r="A48" t="s">
         <v>2412</v>
       </c>
@@ -23094,7 +22488,7 @@
         <v>2413</v>
       </c>
     </row>
-    <row r="49" ht="333.5" spans="1:2">
+    <row r="49" spans="1:2" ht="345">
       <c r="A49" t="s">
         <v>2414</v>
       </c>
@@ -23102,7 +22496,7 @@
         <v>2415</v>
       </c>
     </row>
-    <row r="50" ht="333.5" spans="1:2">
+    <row r="50" spans="1:2" ht="345">
       <c r="A50" t="s">
         <v>2416</v>
       </c>
@@ -23110,7 +22504,7 @@
         <v>2417</v>
       </c>
     </row>
-    <row r="51" ht="36" customHeight="1" spans="1:2">
+    <row r="51" spans="1:2" ht="36" customHeight="1">
       <c r="A51" t="s">
         <v>2418</v>
       </c>
@@ -23118,7 +22512,7 @@
         <v>2419</v>
       </c>
     </row>
-    <row r="52" ht="23.25" customHeight="1" spans="1:2">
+    <row r="52" spans="1:2" ht="23.25" customHeight="1">
       <c r="A52" t="s">
         <v>2420</v>
       </c>
@@ -23126,7 +22520,7 @@
         <v>2421</v>
       </c>
     </row>
-    <row r="53" ht="27.75" customHeight="1" spans="1:2">
+    <row r="53" spans="1:2" ht="27.75" customHeight="1">
       <c r="A53" t="s">
         <v>2422</v>
       </c>
@@ -23134,7 +22528,7 @@
         <v>2423</v>
       </c>
     </row>
-    <row r="54" ht="58" spans="1:2">
+    <row r="54" spans="1:2" ht="60">
       <c r="A54" t="s">
         <v>2424</v>
       </c>
@@ -23142,7 +22536,7 @@
         <v>2425</v>
       </c>
     </row>
-    <row r="55" ht="43.5" spans="1:2">
+    <row r="55" spans="1:2" ht="45">
       <c r="A55" t="s">
         <v>2426</v>
       </c>
@@ -23150,7 +22544,7 @@
         <v>2427</v>
       </c>
     </row>
-    <row r="56" ht="58" spans="1:2">
+    <row r="56" spans="1:2" ht="60">
       <c r="A56" t="s">
         <v>2428</v>
       </c>
@@ -23158,7 +22552,7 @@
         <v>2429</v>
       </c>
     </row>
-    <row r="57" ht="72.5" spans="1:2">
+    <row r="57" spans="1:2" ht="75">
       <c r="A57" t="s">
         <v>2430</v>
       </c>
@@ -23166,7 +22560,7 @@
         <v>2431</v>
       </c>
     </row>
-    <row r="58" ht="409.5" spans="1:2">
+    <row r="58" spans="1:2" ht="409.5">
       <c r="A58" t="s">
         <v>2432</v>
       </c>
@@ -23174,7 +22568,7 @@
         <v>2433</v>
       </c>
     </row>
-    <row r="59" ht="87" spans="1:2">
+    <row r="59" spans="1:2" ht="90">
       <c r="A59" t="s">
         <v>2434</v>
       </c>
@@ -23182,7 +22576,7 @@
         <v>2435</v>
       </c>
     </row>
-    <row r="60" ht="348" spans="1:2">
+    <row r="60" spans="1:2" ht="360">
       <c r="A60" t="s">
         <v>2436</v>
       </c>
@@ -23190,7 +22584,7 @@
         <v>2437</v>
       </c>
     </row>
-    <row r="61" ht="58" spans="1:2">
+    <row r="61" spans="1:2" ht="75">
       <c r="A61" t="s">
         <v>2438</v>
       </c>
@@ -23198,7 +22592,7 @@
         <v>2439</v>
       </c>
     </row>
-    <row r="62" ht="409.5" spans="1:2">
+    <row r="62" spans="1:2" ht="409.5">
       <c r="A62" t="s">
         <v>2440</v>
       </c>
@@ -23206,7 +22600,7 @@
         <v>2357</v>
       </c>
     </row>
-    <row r="63" ht="87.75" customHeight="1" spans="1:2">
+    <row r="63" spans="1:2" ht="87.75" customHeight="1">
       <c r="A63" t="s">
         <v>2441</v>
       </c>
@@ -23214,7 +22608,7 @@
         <v>2442</v>
       </c>
     </row>
-    <row r="64" ht="71.25" customHeight="1" spans="1:2">
+    <row r="64" spans="1:2" ht="71.25" customHeight="1">
       <c r="A64" t="s">
         <v>2443</v>
       </c>
@@ -23222,7 +22616,7 @@
         <v>2444</v>
       </c>
     </row>
-    <row r="65" ht="54" customHeight="1" spans="1:2">
+    <row r="65" spans="1:2" ht="54" customHeight="1">
       <c r="A65" t="s">
         <v>2400</v>
       </c>
@@ -23230,7 +22624,7 @@
         <v>2401</v>
       </c>
     </row>
-    <row r="66" ht="86.25" customHeight="1" spans="1:2">
+    <row r="66" spans="1:2" ht="86.25" customHeight="1">
       <c r="A66" s="29" t="s">
         <v>2445</v>
       </c>
@@ -23238,7 +22632,7 @@
         <v>2446</v>
       </c>
     </row>
-    <row r="67" ht="86.25" customHeight="1" spans="1:2">
+    <row r="67" spans="1:2" ht="86.25" customHeight="1">
       <c r="A67" s="29" t="s">
         <v>2447</v>
       </c>
@@ -23246,7 +22640,7 @@
         <v>2448</v>
       </c>
     </row>
-    <row r="68" ht="102" customHeight="1" spans="1:2">
+    <row r="68" spans="1:2" ht="102" customHeight="1">
       <c r="A68" s="29" t="s">
         <v>2449</v>
       </c>
@@ -23254,7 +22648,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="69" ht="89.25" customHeight="1" spans="1:2">
+    <row r="69" spans="1:2" ht="89.25" customHeight="1">
       <c r="A69" s="29" t="s">
         <v>2451</v>
       </c>
@@ -23262,7 +22656,7 @@
         <v>2452</v>
       </c>
     </row>
-    <row r="70" ht="102" customHeight="1" spans="1:2">
+    <row r="70" spans="1:2" ht="102" customHeight="1">
       <c r="A70" s="29" t="s">
         <v>2453</v>
       </c>
@@ -23272,6 +22666,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Newly Added Subcontract Scenarios And DBsales Test Data Sheet Added
Newly Added Subcontract Scenarios And  Test Data Sheet Added
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915"/>
@@ -10,7 +10,7 @@
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="124519"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2989" uniqueCount="2457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2993" uniqueCount="2461">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -9960,6 +9960,18 @@
   </si>
   <si>
     <t>OPSO7</t>
+  </si>
+  <si>
+    <t>BomForSerialItemWithSO</t>
+  </si>
+  <si>
+    <t>FG40001-SERIAL-SO</t>
+  </si>
+  <si>
+    <t>BomSerialSOref</t>
+  </si>
+  <si>
+    <t>SO100/05832/25-26</t>
   </si>
 </sst>
 </file>
@@ -10550,7 +10562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1441"/>
+  <dimension ref="A1:B1443"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
@@ -22084,6 +22096,22 @@
       </c>
       <c r="B1441" s="35" t="s">
         <v>2456</v>
+      </c>
+    </row>
+    <row r="1442" spans="1:2">
+      <c r="A1442" s="30" t="s">
+        <v>2457</v>
+      </c>
+      <c r="B1442" s="31" t="s">
+        <v>2458</v>
+      </c>
+    </row>
+    <row r="1443" spans="1:2">
+      <c r="A1443" s="30" t="s">
+        <v>2459</v>
+      </c>
+      <c r="B1443" s="31" t="s">
+        <v>2460</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Fixes In OpenPo, Purchase Request And OpenPO Amend Scenarios
Updated Fixes In OpenPo, Purchase Request And OpenPO Amend Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915"/>
+    <workbookView windowWidth="23040" windowHeight="9120" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2993" uniqueCount="2461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2993" uniqueCount="2463">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -7006,6 +7006,24 @@
   </si>
   <si>
     <t>GWL - BOM ITEM - 2244</t>
+  </si>
+  <si>
+    <t>Prefix_07</t>
+  </si>
+  <si>
+    <t>OPSO7</t>
+  </si>
+  <si>
+    <t>BomForSerialItemWithSO</t>
+  </si>
+  <si>
+    <t>FG40001-SERIAL-SO</t>
+  </si>
+  <si>
+    <t>BomSerialSOref</t>
+  </si>
+  <si>
+    <t>SO100/05832/25-26</t>
   </si>
   <si>
     <t>PRHeaderQuery</t>
@@ -7147,7 +7165,7 @@
   FROM pur_req_hd,
        pur_req_ln,
        products
- WHERE  (prh_bu = 'TVSA' OR prh_bu = 'KARE')
+ WHERE  (prh_bu = 'ROAU' OR prh_bu = 'KARE')
    AND PRH_RQST_NO ='${PRNO}'
        AND prh_bu = prl_bu
        AND prh_rqst_no = prl_rqst_no
@@ -7678,7 +7696,7 @@
 WHERE
     PRL_RQST_NO = '${PRNO}'
     AND (
-        prl_bu = 'TVSA'
+        prl_bu = 'ROAU'
         OR prl_bu = 'KARE'
     )
     AND PRL_PROD_ID = '${ItemId}'</t>
@@ -8091,6 +8109,103 @@
   FROM sales_invoices_hd
 where sihd_bu = 'TVSA'
   and sihd_doc_no = '${SINO}'</t>
+  </si>
+  <si>
+    <t>SELECT PRH_RQST_NO,
+       prl_prod_id "Item",
+       prl_prod_desc1 "Item Desc.",
+       prl_prod_rev "Rev.",
+       prod_ext_desc1,
+       prl_uom "UOM",
+       prl_class_desc "Item Class",
+       prl_sub_cls_desc "Item SubClass",
+       prl_conv_factor "Conv. Factor",
+       prl_store_name "WH/Dept.",
+       prl_so_schld_desc "SO/Prj. Ref.",
+       prl_required_date prls_required_date,
+       CASE
+          WHEN prl_status = 'E' THEN 'Draft'
+          WHEN prl_status = 'N' THEN 'Entry Completed'
+          WHEN prl_status = 'A' THEN 'Approved'
+          WHEN prl_status = 'C' THEN 'Cancelled'
+          WHEN prl_status = 'L' THEN 'Closeshort'
+       END
+          prl_status,
+       DECODE (prl_status,
+               'A', 'Approved',
+               'E', 'Draft',
+               'C', 'Cancelled',
+               'R', 'Entry Completed',
+               'L', 'Closeshorted',
+               'R', 'RECEIVED',
+               'P', 'PARTIAL')
+          ln_STATUS,
+       prl_pur_acct,
+       prl_cc_code,
+       (SELECT glac_acct_desc1
+          FROM gl_accts
+         WHERE glac_bu = prl_bu AND glac_acct = prl_pur_acct)
+          "GL Acct. Desc.",
+       (SELECT pcc_desc
+          FROM profit_cost_centers
+         WHERE     pcc_bu = prl_bu
+               AND pcc_ac_plnt = prl_plnt
+               AND pcc_cc_code = prl_cc_code)
+          "CPC Code Desc.",
+       (SELECT DISTINCT DECODE (
+                  applctrl_desc_level,
+                  1,    emp_first_name1
+                     || ' '
+                     || emp_middle_name1
+                     || ' '
+                     || emp_last_name1,
+                  NVL (
+                        emp_first_name2
+                     || ' '
+                     || emp_middle_name2
+                     || ' '
+                     || emp_last_name2,
+                        emp_first_name1
+                     || ' '
+                     || emp_middle_name1
+                     || ' '
+                     || emp_last_name1))
+                  AS buyer_desc
+          FROM buyers,
+               employees,
+               appl_control,
+               emp_active_infos
+         WHERE     buyer_bu = emp_bu
+               AND buyer_emp_id = emp_emp_id
+               AND buyer_bu = applctrl_bu
+               AND emp_bu = empai_bu
+               AND emp_emp_id = empai_emp_id
+               AND buyer_bu = prl_bu
+               AND buyer_id = prl_buyer_id)
+          buyer,
+          prh_mrp_no,
+          PRL_SUGG_SUPLR_ID,
+          prl_work_ord_no,
+          PRL_SERV_PROD_ID,
+          PRL_SERV_PROD_DESC "Serv. Item desc",
+          prl_amc_start_date,
+          prl_amc_end_date,
+          PRL_MRP_REL_QTY,
+          (SELECT NVL(suplr_name1,suplr_name2)
+             FROM suppliers
+            WHERE suplr_bu = prl_bu
+            AND suplr_suplr_id = PRL_SUGG_SUPLR_ID) "Supplr. desc",
+       DECODE(prl_qc_required,'Y','Free Pass','N','Always')prl_qc_required
+  FROM pur_req_hd,
+       pur_req_ln,
+       products
+ WHERE  (prh_bu = 'TVSA' OR prh_bu = 'KARE')
+   AND PRH_RQST_NO ='${PRNO}'
+       AND prh_bu = prl_bu
+       AND prh_rqst_no = prl_rqst_no
+       AND prl_bu = prod_bu
+       AND prl_prod_id = prod_id
+       AND prl_prod_rev = prod_rev</t>
   </si>
   <si>
     <t>PRBucket Query</t>
@@ -9362,6 +9477,144 @@
     <t>PRLineDetailsQueryKARE</t>
   </si>
   <si>
+    <t>SELECT
+ prl_bu,
+ prl_rqst_no,
+ prl_seq_no,
+ prl_prod_id,
+ prl_prod_rev,
+ prl_prod_desc1,
+ prl_class_id,
+ prl_class_desc,
+ prl_sub_cls_id,
+ prl_sub_cls_desc,
+ prl_uom,
+ prl_prod_uom,
+ prl_conv_factor,
+ prl_requested_qty,
+ (prl_requested_qty * prl_bc_unit_cost) line_amount,
+ prl_ordered_qty,
+ prl_receipt_qty,
+ prl_bc_unit_cost,
+ prl_disc_pct,
+ prl_stocked,
+ prl_qc_required,
+ prl_quote_pfx,
+ prl_quote_no,
+ prl_order_pfx,
+ prl_order_no,
+ prl_net_disc_flag,
+ prl_status,
+ CASE
+  WHEN prl_status = 'R' THEN 'Entry Completed'
+  WHEN prl_status = 'A' THEN 'Approved'
+  WHEN prl_status = 'C' THEN 'Cancelled'
+  WHEN prl_status = 'L' THEN 'Close Shorted'
+  WHEN prl_status = 'E' THEN 'Draft'
+ END STATUS,
+ prl_prod_temp_id,
+ prl_prod_temp_rev,
+ prl_work_ord_no,
+ prl_select_flag,
+ prl_ins_plan_no,
+ prl_ins_plan_rev,
+ prl_prod_ord_no,
+ prl_sf_code,
+ prl_test_req_flag,
+ prl_cert_id,
+ prl_print_seq_no,
+ prl_prod_temp_desc1,
+ prl_ref,
+ prl_prod_ext_desc,
+ prl_cs_narr,
+ prl_drawing_no,
+ prl_drawing_rev,
+ prl_spr_type,
+ prl_rcpt_rcvd_qty,
+ prl_dim_req_flag,
+ prl_thickness,
+ prl_length,
+ prl_width,
+ prl_qty_in_nos,
+ prl_serv_prod_id,
+ prl_serv_io_type,
+ prl_amc_start_date,
+ prl_amc_end_date,
+ prl_serv_prod_desc,
+ prl_tool_wo_no,
+ prl_sugg_suplr_id,
+ prl_cls_sel_user,
+ prl_cls_qty,
+ prl_cls_proc_qty,
+ prl_cap_asset_id,
+ prl_cust_drw_no,
+ prl_cust_drw_rev,
+ prl_catalog_no,
+ prl_mchn_id,
+ prl_sub_dept_id,
+ prl_priority,
+ prl_buyer_id,
+ prl_mrp_rel_qty,
+ prl_mftr_id,
+ prl_mftr_part_no,
+ prl_eqpmt_id,
+ prl_eqpmt_desc,
+ prl_buyer_emp_id,
+ prl_lpp_rcpt_pfx,
+ prl_lpp_rcpt_no,
+ prl_mchn_grp_id,
+ prl_pr_plan_no,
+ prl_prod_outer_dia,
+ prl_cre_by,
+ prl_cre_ip_addr,
+ prl_cre_os_user,
+ prl_cre_date,
+ prl_upd_by,
+ prl_upd_ip_addr,
+ prl_upd_os_user,
+ prl_upd_date,
+ prl_cre_emp_id,
+ prl_upd_emp_id,
+ prl_last_po_price,
+ prl_prod_chng_flag,
+ prl_batch_no,
+ prl_expiry_date,
+ prl_mfg_date,
+ prl_sterilize_date,
+ prl_iss_code,
+ prl_height,
+ prl_inner_dia,
+ prl_density,
+ prl_pur_acct,
+ prl_cc_code,
+ prl_fab_item_type,
+ prl_gla_fxd_flag,
+ prl_cpc_fxd_flag,
+ prl_store_id,
+ prl_store_name,
+ prl_required_date,
+ prl_so_type,
+ prl_so_pfx,
+ prl_so_no,
+ prl_so_seq_no,
+ prl_so_sub_seq_no,
+ prl_proj_id,
+ prl_task_id,
+ prl_so_schld_desc,
+ prl_shipto_loc_id,
+ prl_shipto_loc_name,
+ prl_rfq
+FROM
+ pur_req_ln
+WHERE
+    PRL_RQST_NO = '${PRNO}'
+    AND (
+        prl_bu = 'TVSA'
+        OR prl_bu = 'KARE'
+    )
+    AND PRL_PROD_ID = '${ItemId}'</t>
+  </si>
+  <si>
     <t>OSPHeaderQuery</t>
   </si>
   <si>
@@ -9955,30 +10208,18 @@
        AND poh_mode = 'SC'
        AND poh_order_no ='${SCONO}'</t>
   </si>
-  <si>
-    <t>Prefix_07</t>
-  </si>
-  <si>
-    <t>OPSO7</t>
-  </si>
-  <si>
-    <t>BomForSerialItemWithSO</t>
-  </si>
-  <si>
-    <t>FG40001-SERIAL-SO</t>
-  </si>
-  <si>
-    <t>BomSerialSOref</t>
-  </si>
-  <si>
-    <t>SO100/05832/25-26</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -10025,14 +10266,151 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -10057,8 +10435,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -10094,26 +10658,268 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="18">
+  <cellStyleXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -10131,48 +10937,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="15" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="16" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="16" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="64" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="64" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="53"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -10201,15 +11007,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -10229,11 +11035,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -10247,19 +11053,19 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="59" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="60" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -10274,27 +11080,74 @@
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="18">
+  <cellStyles count="66">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="1"/>
-    <cellStyle name="Normal 11" xfId="2"/>
-    <cellStyle name="Normal 13" xfId="3"/>
-    <cellStyle name="Normal 14" xfId="4"/>
-    <cellStyle name="Normal 15" xfId="5"/>
-    <cellStyle name="Normal 16" xfId="6"/>
-    <cellStyle name="Normal 17" xfId="7"/>
-    <cellStyle name="Normal 18" xfId="8"/>
-    <cellStyle name="Normal 19" xfId="9"/>
-    <cellStyle name="Normal 2" xfId="10"/>
-    <cellStyle name="Normal 2 2" xfId="11"/>
-    <cellStyle name="Normal 2 3" xfId="12"/>
-    <cellStyle name="Normal 20" xfId="13"/>
-    <cellStyle name="Normal 3" xfId="14"/>
-    <cellStyle name="Normal 7" xfId="15"/>
-    <cellStyle name="Normal 8" xfId="16"/>
-    <cellStyle name="Normal 9" xfId="17"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal 10" xfId="49"/>
+    <cellStyle name="Normal 11" xfId="50"/>
+    <cellStyle name="Normal 13" xfId="51"/>
+    <cellStyle name="Normal 14" xfId="52"/>
+    <cellStyle name="Normal 15" xfId="53"/>
+    <cellStyle name="Normal 16" xfId="54"/>
+    <cellStyle name="Normal 17" xfId="55"/>
+    <cellStyle name="Normal 18" xfId="56"/>
+    <cellStyle name="Normal 19" xfId="57"/>
+    <cellStyle name="Normal 2" xfId="58"/>
+    <cellStyle name="Normal 2 2" xfId="59"/>
+    <cellStyle name="Normal 2 3" xfId="60"/>
+    <cellStyle name="Normal 20" xfId="61"/>
+    <cellStyle name="Normal 3" xfId="62"/>
+    <cellStyle name="Normal 7" xfId="63"/>
+    <cellStyle name="Normal 8" xfId="64"/>
+    <cellStyle name="Normal 9" xfId="65"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -10556,17 +11409,17 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B1443"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="62.7109375" style="30" customWidth="1"/>
-    <col min="2" max="2" width="59.85546875" style="31" customWidth="1"/>
+    <col min="1" max="1" width="62.712962962963" style="30" customWidth="1"/>
+    <col min="2" max="2" width="59.8518518518519" style="31" customWidth="1"/>
     <col min="3" max="16384" width="9" style="30"/>
   </cols>
   <sheetData>
@@ -22092,43 +22945,45 @@
     </row>
     <row r="1441" spans="1:2">
       <c r="A1441" s="34" t="s">
-        <v>2455</v>
+        <v>2326</v>
       </c>
       <c r="B1441" s="35" t="s">
-        <v>2456</v>
+        <v>2327</v>
       </c>
     </row>
     <row r="1442" spans="1:2">
       <c r="A1442" s="30" t="s">
-        <v>2457</v>
+        <v>2328</v>
       </c>
       <c r="B1442" s="31" t="s">
-        <v>2458</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="1443" spans="1:2">
       <c r="A1443" s="30" t="s">
-        <v>2459</v>
+        <v>2330</v>
       </c>
       <c r="B1443" s="31" t="s">
-        <v>2460</v>
+        <v>2331</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1209" r:id="rId1"/>
-    <hyperlink ref="B1364" r:id="rId2"/>
+    <hyperlink ref="B1209" r:id="rId1" display="MRAD-2425-00086"/>
+    <hyperlink ref="B1364" r:id="rId2" display="RFQ10/00725/25-26"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B70"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.8518518518519" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -22140,559 +22995,560 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="108.95" customHeight="1">
+    <row r="2" ht="108.95" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>2326</v>
+        <v>2332</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>2327</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="114" customHeight="1">
+        <v>2333</v>
+      </c>
+    </row>
+    <row r="3" ht="114" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>2328</v>
+        <v>2334</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2329</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="80.25" customHeight="1">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="4" ht="80.25" customHeight="1" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>2330</v>
+        <v>2336</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2331</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="69.75" customHeight="1">
+        <v>2337</v>
+      </c>
+    </row>
+    <row r="5" ht="69.75" customHeight="1" spans="1:2">
       <c r="A5" s="2" t="s">
+        <v>2338</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>2339</v>
+      </c>
+    </row>
+    <row r="6" ht="51.75" customHeight="1" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>2340</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>2341</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>2342</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>2343</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>2344</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="9" ht="39" customHeight="1" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>2346</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>2347</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1" spans="1:2">
+      <c r="A10" s="2" t="s">
+        <v>2348</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>2349</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" spans="1:2">
+      <c r="A11" s="2" t="s">
+        <v>2350</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>2351</v>
+      </c>
+    </row>
+    <row r="12" ht="26.25" customHeight="1" spans="1:2">
+      <c r="A12" s="2" t="s">
+        <v>2352</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="13" ht="28.5" customHeight="1" spans="1:2">
+      <c r="A13" s="2" t="s">
+        <v>2354</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>2355</v>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1" spans="1:2">
+      <c r="A14" s="2" t="s">
+        <v>2356</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>2357</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1" spans="1:2">
+      <c r="A15" s="2" t="s">
+        <v>2358</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>2359</v>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1" spans="1:2">
+      <c r="A16" s="2" t="s">
+        <v>2360</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>2361</v>
+      </c>
+    </row>
+    <row r="17" ht="43.5" customHeight="1" spans="1:2">
+      <c r="A17" s="2" t="s">
+        <v>2362</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>2363</v>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1" spans="1:2">
+      <c r="A18" s="2" t="s">
+        <v>2364</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>2365</v>
+      </c>
+    </row>
+    <row r="19" ht="52.5" customHeight="1" spans="1:2">
+      <c r="A19" s="2" t="s">
+        <v>2366</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>2367</v>
+      </c>
+    </row>
+    <row r="20" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A20" s="4" t="s">
+        <v>2368</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>2369</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" spans="1:2">
+      <c r="A21" s="4" t="s">
+        <v>2370</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>2371</v>
+      </c>
+    </row>
+    <row r="22" ht="409.5" spans="1:2">
+      <c r="A22" s="2" t="s">
+        <v>2372</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>2373</v>
+      </c>
+    </row>
+    <row r="23" ht="244.8" spans="1:2">
+      <c r="A23" s="2" t="s">
+        <v>2374</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>2375</v>
+      </c>
+    </row>
+    <row r="24" ht="230.4" spans="1:2">
+      <c r="A24" t="s">
+        <v>2376</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>2377</v>
+      </c>
+    </row>
+    <row r="25" ht="259.2" spans="1:2">
+      <c r="A25" t="s">
+        <v>2378</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>2379</v>
+      </c>
+    </row>
+    <row r="26" ht="201.6" spans="1:2">
+      <c r="A26" t="s">
+        <v>2380</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>2381</v>
+      </c>
+    </row>
+    <row r="27" ht="61.5" customHeight="1" spans="1:2">
+      <c r="A27" t="s">
+        <v>2382</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>2383</v>
+      </c>
+    </row>
+    <row r="28" ht="105.75" customHeight="1" spans="1:2">
+      <c r="A28" s="7" t="s">
         <v>2332</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B28" s="8" t="s">
         <v>2333</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="51.75" customHeight="1">
-      <c r="A6" s="2" t="s">
+    <row r="29" ht="83.25" customHeight="1" spans="1:2">
+      <c r="A29" s="9" t="s">
         <v>2334</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>2335</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="30" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>2336</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>2337</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="18" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>2338</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>2339</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="39" customHeight="1">
-      <c r="A9" s="2" t="s">
+      <c r="B29" s="10" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="30" ht="172.8" spans="1:2">
+      <c r="A30" s="11" t="s">
         <v>2340</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B30" s="12" t="s">
         <v>2341</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="22.5" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>2342</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>2343</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="18" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>2344</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>2345</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="26.25" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>2346</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>2347</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="28.5" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>2348</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>2349</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="24" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>2350</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>2351</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="36" customHeight="1">
-      <c r="A15" s="2" t="s">
-        <v>2352</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>2353</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1">
-      <c r="A16" s="2" t="s">
-        <v>2354</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>2355</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="43.5" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>2356</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>2357</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="42" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>2358</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>2359</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="52.5" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>2360</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>2361</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="17.25" customHeight="1">
-      <c r="A20" s="4" t="s">
-        <v>2362</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>2363</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15" customHeight="1">
-      <c r="A21" s="4" t="s">
-        <v>2364</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>2365</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="409.5">
-      <c r="A22" s="2" t="s">
-        <v>2366</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>2367</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="255">
-      <c r="A23" s="2" t="s">
-        <v>2368</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>2369</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="240">
-      <c r="A24" t="s">
-        <v>2370</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>2371</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="270">
-      <c r="A25" t="s">
-        <v>2372</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>2373</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="210">
-      <c r="A26" t="s">
-        <v>2374</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>2375</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="61.5" customHeight="1">
-      <c r="A27" t="s">
-        <v>2376</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>2377</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="105.75" customHeight="1">
-      <c r="A28" s="7" t="s">
-        <v>2326</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>2327</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="83.25" customHeight="1">
-      <c r="A29" s="9" t="s">
-        <v>2328</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>2329</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="180">
-      <c r="A30" s="11" t="s">
-        <v>2334</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>2335</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="135">
+    <row r="31" ht="129.6" spans="1:2">
       <c r="A31" s="13" t="s">
-        <v>2378</v>
+        <v>2385</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>2379</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="180">
+        <v>2386</v>
+      </c>
+    </row>
+    <row r="32" ht="172.8" spans="1:2">
       <c r="A32" s="15" t="s">
-        <v>2380</v>
+        <v>2387</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>2381</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="180">
+        <v>2388</v>
+      </c>
+    </row>
+    <row r="33" ht="172.8" spans="1:2">
       <c r="A33" s="17" t="s">
-        <v>2382</v>
+        <v>2389</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>2383</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="409.5">
+        <v>2390</v>
+      </c>
+    </row>
+    <row r="34" ht="409.5" spans="1:2">
       <c r="A34" s="19" t="s">
-        <v>2384</v>
+        <v>2391</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>2385</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="409.5">
+        <v>2392</v>
+      </c>
+    </row>
+    <row r="35" ht="403.2" spans="1:2">
       <c r="A35" s="21" t="s">
-        <v>2386</v>
+        <v>2393</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>2387</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="409.5">
+        <v>2394</v>
+      </c>
+    </row>
+    <row r="36" ht="409.5" spans="1:2">
       <c r="A36" s="23" t="s">
-        <v>2388</v>
+        <v>2395</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>2389</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="409.5">
+        <v>2396</v>
+      </c>
+    </row>
+    <row r="37" ht="409.5" spans="1:2">
       <c r="A37" s="25" t="s">
-        <v>2390</v>
+        <v>2397</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>2391</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="409.5">
+        <v>2398</v>
+      </c>
+    </row>
+    <row r="38" ht="409.5" spans="1:2">
       <c r="A38" s="27" t="s">
-        <v>2392</v>
+        <v>2399</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>2393</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="409.5">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="39" ht="409.5" spans="1:2">
       <c r="A39" t="s">
-        <v>2394</v>
+        <v>2401</v>
       </c>
       <c r="B39" s="29" t="s">
-        <v>2395</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="120">
+        <v>2402</v>
+      </c>
+    </row>
+    <row r="40" ht="115.2" spans="1:2">
       <c r="A40" t="s">
-        <v>2396</v>
+        <v>2403</v>
       </c>
       <c r="B40" s="29" t="s">
-        <v>2397</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="180">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="41" ht="172.8" spans="1:2">
       <c r="A41" t="s">
-        <v>2398</v>
+        <v>2405</v>
       </c>
       <c r="B41" s="29" t="s">
-        <v>2399</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="195">
+        <v>2406</v>
+      </c>
+    </row>
+    <row r="42" ht="187.2" spans="1:2">
       <c r="A42" t="s">
-        <v>2400</v>
+        <v>2407</v>
       </c>
       <c r="B42" s="29" t="s">
-        <v>2401</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="120">
+        <v>2408</v>
+      </c>
+    </row>
+    <row r="43" ht="115.2" spans="1:2">
       <c r="A43" t="s">
-        <v>2402</v>
+        <v>2409</v>
       </c>
       <c r="B43" s="29" t="s">
-        <v>2403</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="409.5">
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="44" ht="409.5" spans="1:2">
       <c r="A44" t="s">
-        <v>2404</v>
+        <v>2411</v>
       </c>
       <c r="B44" s="29" t="s">
-        <v>2405</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="409.5">
+        <v>2412</v>
+      </c>
+    </row>
+    <row r="45" ht="409.5" spans="1:2">
       <c r="A45" t="s">
-        <v>2406</v>
+        <v>2413</v>
       </c>
       <c r="B45" s="29" t="s">
+        <v>2414</v>
+      </c>
+    </row>
+    <row r="46" ht="409.5" spans="1:2">
+      <c r="A46" t="s">
+        <v>2415</v>
+      </c>
+      <c r="B46" s="29" t="s">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="47" ht="259.2" spans="1:2">
+      <c r="A47" t="s">
+        <v>2417</v>
+      </c>
+      <c r="B47" s="29" t="s">
+        <v>2418</v>
+      </c>
+    </row>
+    <row r="48" ht="409.5" spans="1:2">
+      <c r="A48" t="s">
+        <v>2419</v>
+      </c>
+      <c r="B48" s="29" t="s">
+        <v>2420</v>
+      </c>
+    </row>
+    <row r="49" ht="331.2" spans="1:2">
+      <c r="A49" t="s">
+        <v>2421</v>
+      </c>
+      <c r="B49" s="29" t="s">
+        <v>2422</v>
+      </c>
+    </row>
+    <row r="50" ht="331.2" spans="1:2">
+      <c r="A50" t="s">
+        <v>2423</v>
+      </c>
+      <c r="B50" s="29" t="s">
+        <v>2424</v>
+      </c>
+    </row>
+    <row r="51" ht="36" customHeight="1" spans="1:2">
+      <c r="A51" t="s">
+        <v>2425</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>2426</v>
+      </c>
+    </row>
+    <row r="52" ht="23.25" customHeight="1" spans="1:2">
+      <c r="A52" t="s">
+        <v>2427</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>2428</v>
+      </c>
+    </row>
+    <row r="53" ht="27.75" customHeight="1" spans="1:2">
+      <c r="A53" t="s">
+        <v>2429</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>2430</v>
+      </c>
+    </row>
+    <row r="54" ht="57.6" spans="1:2">
+      <c r="A54" t="s">
+        <v>2431</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="55" ht="43.2" spans="1:2">
+      <c r="A55" t="s">
+        <v>2433</v>
+      </c>
+      <c r="B55" s="29" t="s">
+        <v>2434</v>
+      </c>
+    </row>
+    <row r="56" ht="57.6" spans="1:2">
+      <c r="A56" t="s">
+        <v>2435</v>
+      </c>
+      <c r="B56" s="29" t="s">
+        <v>2436</v>
+      </c>
+    </row>
+    <row r="57" ht="72" spans="1:2">
+      <c r="A57" t="s">
+        <v>2437</v>
+      </c>
+      <c r="B57" s="29" t="s">
+        <v>2438</v>
+      </c>
+    </row>
+    <row r="58" ht="409.5" spans="1:2">
+      <c r="A58" t="s">
+        <v>2439</v>
+      </c>
+      <c r="B58" s="29" t="s">
+        <v>2440</v>
+      </c>
+    </row>
+    <row r="59" ht="86.4" spans="1:2">
+      <c r="A59" t="s">
+        <v>2441</v>
+      </c>
+      <c r="B59" s="29" t="s">
+        <v>2442</v>
+      </c>
+    </row>
+    <row r="60" ht="345.6" spans="1:2">
+      <c r="A60" t="s">
+        <v>2443</v>
+      </c>
+      <c r="B60" s="29" t="s">
+        <v>2444</v>
+      </c>
+    </row>
+    <row r="61" ht="57.6" spans="1:2">
+      <c r="A61" t="s">
+        <v>2445</v>
+      </c>
+      <c r="B61" s="29" t="s">
+        <v>2446</v>
+      </c>
+    </row>
+    <row r="62" ht="409.5" spans="1:2">
+      <c r="A62" t="s">
+        <v>2447</v>
+      </c>
+      <c r="B62" s="29" t="s">
+        <v>2448</v>
+      </c>
+    </row>
+    <row r="63" ht="87.75" customHeight="1" spans="1:2">
+      <c r="A63" t="s">
+        <v>2449</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="64" ht="71.25" customHeight="1" spans="1:2">
+      <c r="A64" t="s">
+        <v>2451</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>2452</v>
+      </c>
+    </row>
+    <row r="65" ht="54" customHeight="1" spans="1:2">
+      <c r="A65" t="s">
         <v>2407</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" ht="409.5">
-      <c r="A46" t="s">
+      <c r="B65" s="29" t="s">
         <v>2408</v>
       </c>
-      <c r="B46" s="29" t="s">
-        <v>2409</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="270">
-      <c r="A47" t="s">
-        <v>2410</v>
-      </c>
-      <c r="B47" s="29" t="s">
-        <v>2411</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="409.5">
-      <c r="A48" t="s">
-        <v>2412</v>
-      </c>
-      <c r="B48" s="29" t="s">
-        <v>2413</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="345">
-      <c r="A49" t="s">
-        <v>2414</v>
-      </c>
-      <c r="B49" s="29" t="s">
-        <v>2415</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="345">
-      <c r="A50" t="s">
-        <v>2416</v>
-      </c>
-      <c r="B50" s="29" t="s">
-        <v>2417</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="36" customHeight="1">
-      <c r="A51" t="s">
-        <v>2418</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>2419</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="23.25" customHeight="1">
-      <c r="A52" t="s">
-        <v>2420</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>2421</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="27.75" customHeight="1">
-      <c r="A53" t="s">
-        <v>2422</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>2423</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="60">
-      <c r="A54" t="s">
-        <v>2424</v>
-      </c>
-      <c r="B54" s="6" t="s">
-        <v>2425</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="45">
-      <c r="A55" t="s">
-        <v>2426</v>
-      </c>
-      <c r="B55" s="29" t="s">
-        <v>2427</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="60">
-      <c r="A56" t="s">
-        <v>2428</v>
-      </c>
-      <c r="B56" s="29" t="s">
-        <v>2429</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="75">
-      <c r="A57" t="s">
-        <v>2430</v>
-      </c>
-      <c r="B57" s="29" t="s">
-        <v>2431</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="409.5">
-      <c r="A58" t="s">
-        <v>2432</v>
-      </c>
-      <c r="B58" s="29" t="s">
-        <v>2433</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="90">
-      <c r="A59" t="s">
-        <v>2434</v>
-      </c>
-      <c r="B59" s="29" t="s">
-        <v>2435</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="360">
-      <c r="A60" t="s">
-        <v>2436</v>
-      </c>
-      <c r="B60" s="29" t="s">
-        <v>2437</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="75">
-      <c r="A61" t="s">
-        <v>2438</v>
-      </c>
-      <c r="B61" s="29" t="s">
-        <v>2439</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="409.5">
-      <c r="A62" t="s">
-        <v>2440</v>
-      </c>
-      <c r="B62" s="29" t="s">
-        <v>2357</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" ht="87.75" customHeight="1">
-      <c r="A63" t="s">
-        <v>2441</v>
-      </c>
-      <c r="B63" s="6" t="s">
-        <v>2442</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="71.25" customHeight="1">
-      <c r="A64" t="s">
-        <v>2443</v>
-      </c>
-      <c r="B64" s="6" t="s">
-        <v>2444</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="54" customHeight="1">
-      <c r="A65" t="s">
-        <v>2400</v>
-      </c>
-      <c r="B65" s="29" t="s">
-        <v>2401</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" ht="86.25" customHeight="1">
+    </row>
+    <row r="66" ht="86.25" customHeight="1" spans="1:2">
       <c r="A66" s="29" t="s">
-        <v>2445</v>
+        <v>2453</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>2446</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" ht="86.25" customHeight="1">
+        <v>2454</v>
+      </c>
+    </row>
+    <row r="67" ht="86.25" customHeight="1" spans="1:2">
       <c r="A67" s="29" t="s">
-        <v>2447</v>
+        <v>2455</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>2448</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="102" customHeight="1">
+        <v>2456</v>
+      </c>
+    </row>
+    <row r="68" ht="102" customHeight="1" spans="1:2">
       <c r="A68" s="29" t="s">
-        <v>2449</v>
+        <v>2457</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>2450</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="89.25" customHeight="1">
+        <v>2458</v>
+      </c>
+    </row>
+    <row r="69" ht="89.25" customHeight="1" spans="1:2">
       <c r="A69" s="29" t="s">
-        <v>2451</v>
+        <v>2459</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>2452</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" ht="102" customHeight="1">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="70" ht="102" customHeight="1" spans="1:2">
       <c r="A70" s="29" t="s">
-        <v>2453</v>
+        <v>2461</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>2454</v>
+        <v>2462</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Locators are Fixes in New Envr , API Fixed For Item master , open so , open so amd , price list functions
Locators are Fixes in New Envr , API Fixed For Item master , open so , open so amd , price list functions
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" activeTab="1"/>
@@ -10,7 +10,7 @@
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="125725"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -7165,42 +7165,6 @@
   </si>
   <si>
     <t>OsoaQuery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SELECT srcahd_plnt_loc_id "loc id",
-       srcahd_plnt "unit",
-       srcahd_doc_no "Doc. No.",
-       srcahd_amd_no "Amd. No.",
-       srcahd_cust_id "customer id",
-       (SELECT suplr_name1
-          FROM suppliers
-         WHERE suplr_bu = srcahd_bu AND suplr_suplr_id = srcahd_cust_id)
-          "customer name",
-       srcaln_prod_id "item id",
-       srcaln_prod_rev "item rev",
-       (SELECT prod_desc11
-          FROM products
-         WHERE     prod_bu = srcaln_bu
-               AND prod_id = srcaln_prod_id
-               AND prod_rev = srcaln_prod_rev)
-          "item descripition",
-       srcaln_uom "uom",
-       srcaln_disc_pct "disc_pct",
-       srcaln_old_price "Existing Price",
-       srcaln_new_price "new_price",
-       srcaln_mrp_price "MRP Price",
-       srcaln_hsn_code "HSN code",
-       srcaln_tax_pct "Tax Percent",
-       srcaln_cgst_amt "CGST",
-       srcaln_sgst_amt "SGST",
-       srcaln_igst_amt "IGST",
-       srcaln_utgst_amt "UTGST"
-  FROM sales_rate_contr_ament_hd, sales_rate_contr_ament_ln
- WHERE     srcahd_bu = srcaln_bu
-       AND srcahd_plnt = srcaln_plnt
-       AND srcahd_doc_no = '${OSOANO}'
-    AND srcahd_doc_no = srcaln_doc_no
-       AND srcahd_bu =  'TVSA' </t>
   </si>
   <si>
     <t>SOAdvanceQuery</t>
@@ -8602,45 +8566,6 @@
     AND SIHD_DOC_NO = '${DBNO}'</t>
   </si>
   <si>
-    <t>PricelistQuery</t>
-  </si>
-  <si>
-    <t>select cpl_plnt "unit"  ,
-       cpl_plnt_loc_id "Unit Loc ID",
-       cpl_plnt_loc_name "Unit Loc Name",
-         (select bup_name1
-         from bus_unit_plants
-        where bup_bu = cpl_bu
-          and bup_plant_id = cpl_plnt) plant_desc,
-       cpl_doc_pfx "Doc Pfx",     
-       cpl_doc_no "Document No",
-       cpl_doc_date "Doc Date",
-       cpl_cust_id "Customer Id",
-       (select suplr_name1
-          from suppliers
-         where suplr_bu = cpl_bu
-           and suplr_suplr_id = cpl_cust_id 
-           and suplr_status = 'A' ) customer_name,
-       cpl_prod_id,
-       cpl_prod_rev,
-         (select prod_desc11
-            from products
-            where prod_bu = cpl_bu
-              and prod_id = cpl_prod_id
-              and prod_rev = cpl_prod_rev) item_desc,
-       cpl_sales_uom "Sales UOM ",
-       cpl_sales_price  "Sales Price ",
-       cpl_disc_pct "Disc Pct " ,
-       cpl_date_from "Eff From date ",
-       cpl_date_to "Eff To Date ",
-         decode(cpl_status,'N','Draft','A','Approved','C','Cancelled','E','Entry Completed') status,
-       cpl_amd_no
-  from cust_price_list
-  where cpl_bu = 'TVSA'
-    and cpl_plnt = 'U100'
-    and cpl_doc_no = '${PlDocNo}'</t>
-  </si>
-  <si>
     <t>CatalogueQuery</t>
   </si>
   <si>
@@ -10143,6 +10068,81 @@
        AND poh_bu = 'ROAU'
        AND poh_mode = 'SC'
        AND poh_order_no ='${SCONO}'</t>
+  </si>
+  <si>
+    <t>SalesPricelistQuery</t>
+  </si>
+  <si>
+    <t>select cpl_plnt "unit"  ,
+       cpl_plnt_loc_id "Unit Loc ID",
+       cpl_plnt_loc_name "Unit Loc Name",
+         (select bup_name1
+         from bus_unit_plants
+        where bup_bu = cpl_bu
+          and bup_plant_id = cpl_plnt) plant_desc,
+       cpl_doc_pfx "Doc Pfx",     
+       cpl_doc_no "Document No",
+       cpl_doc_date "Doc Date",
+       cpl_cust_id "Customer Id",
+       (select suplr_name1
+          from suppliers
+         where suplr_bu = cpl_bu
+           and suplr_suplr_id = cpl_cust_id 
+           and suplr_status = 'A' ) customer_name,
+       cpl_prod_id,
+       cpl_prod_rev,
+         (select prod_desc11
+            from products
+            where prod_bu = cpl_bu
+              and prod_id = cpl_prod_id
+              and prod_rev = cpl_prod_rev) item_desc,
+       cpl_sales_uom "Sales UOM ",
+       cpl_sales_price  "Sales Price ",
+       cpl_disc_pct "Disc Pct " ,
+       cpl_date_from "Eff From date ",
+       cpl_date_to "Eff To Date ",
+         decode(cpl_status,'N','Draft','A','Approved','C','Cancelled','E','Entry Completed') status,
+       cpl_amd_no
+  from cust_price_list
+  where cpl_bu = 'ROAU'
+    and cpl_plnt = 'U1'
+    and cpl_doc_no = '${PlDocNo}'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SELECT srcahd_plnt_loc_id "loc id",
+       srcahd_plnt "unit",
+       srcahd_doc_no "Doc. No.",
+       srcahd_amd_no "Amd. No.",
+       srcahd_cust_id "customer id",
+       (SELECT suplr_name1
+          FROM suppliers
+         WHERE suplr_bu = srcahd_bu AND suplr_suplr_id = srcahd_cust_id)
+          "customer name",
+       srcaln_prod_id "item id",
+       srcaln_prod_rev "item rev",
+       (SELECT prod_desc11
+          FROM products
+         WHERE     prod_bu = srcaln_bu
+               AND prod_id = srcaln_prod_id
+               AND prod_rev = srcaln_prod_rev)
+          "item descripition",
+       srcaln_uom "uom",
+       srcaln_disc_pct "disc_pct",
+       srcaln_old_price "Existing Price",
+       srcaln_new_price "new_price",
+       srcaln_mrp_price "MRP Price",
+       srcaln_hsn_code "HSN code",
+       srcaln_tax_pct "Tax Percent",
+       srcaln_cgst_amt "CGST",
+       srcaln_sgst_amt "SGST",
+       srcaln_igst_amt "IGST",
+       srcaln_utgst_amt "UTGST"
+  FROM sales_rate_contr_ament_hd, sales_rate_contr_ament_ln
+ WHERE     srcahd_bu = srcaln_bu
+       AND srcahd_plnt = srcaln_plnt
+       AND srcahd_doc_no = '${OSOANO}'
+    AND srcahd_doc_no = srcaln_doc_no
+       AND srcahd_bu =  'ROAU' </t>
   </si>
 </sst>
 </file>
@@ -12154,7 +12154,7 @@
         <v>313</v>
       </c>
       <c r="B177" s="37" t="s">
-        <v>2434</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="178" spans="1:2">
@@ -13658,7 +13658,7 @@
         <v>620</v>
       </c>
       <c r="B365" s="46" t="s">
-        <v>2436</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="366" spans="1:2">
@@ -15642,7 +15642,7 @@
         <v>1039</v>
       </c>
       <c r="B613" s="35" t="s">
-        <v>2442</v>
+        <v>2439</v>
       </c>
     </row>
     <row r="614" spans="1:2">
@@ -17746,7 +17746,7 @@
         <v>1491</v>
       </c>
       <c r="B876" s="35" t="s">
-        <v>2445</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="877" spans="1:2">
@@ -17754,7 +17754,7 @@
         <v>1493</v>
       </c>
       <c r="B877" s="58" t="s">
-        <v>2446</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="878" spans="1:2">
@@ -17762,7 +17762,7 @@
         <v>1494</v>
       </c>
       <c r="B878" s="35" t="s">
-        <v>2449</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="879" spans="1:2">
@@ -19426,7 +19426,7 @@
         <v>1838</v>
       </c>
       <c r="B1086" s="35" t="s">
-        <v>2451</v>
+        <v>2448</v>
       </c>
     </row>
     <row r="1087" spans="1:2">
@@ -20746,7 +20746,7 @@
         <v>1986</v>
       </c>
       <c r="B1251" s="35" t="s">
-        <v>2429</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="1252" spans="1:2">
@@ -22263,39 +22263,39 @@
     </row>
     <row r="1441" spans="1:2">
       <c r="A1441" s="34" t="s">
-        <v>2423</v>
+        <v>2420</v>
       </c>
       <c r="B1441" s="35" t="s">
-        <v>2424</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="1442" spans="1:2">
       <c r="A1442" s="30" t="s">
-        <v>2425</v>
+        <v>2422</v>
       </c>
       <c r="B1442" s="31" t="s">
-        <v>2426</v>
+        <v>2423</v>
       </c>
     </row>
     <row r="1443" spans="1:2">
       <c r="A1443" s="30" t="s">
-        <v>2427</v>
+        <v>2424</v>
       </c>
       <c r="B1443" s="31" t="s">
-        <v>2428</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="1444" spans="1:2">
       <c r="A1444" s="30" t="s">
-        <v>2447</v>
+        <v>2444</v>
       </c>
       <c r="B1444" s="31" t="s">
-        <v>2448</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="1445" spans="1:2">
       <c r="A1445" s="30" t="s">
-        <v>2450</v>
+        <v>2447</v>
       </c>
     </row>
   </sheetData>
@@ -22345,7 +22345,7 @@
         <v>2325</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2430</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="69.75" customHeight="1">
@@ -22353,7 +22353,7 @@
         <v>2326</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2431</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="51.75" customHeight="1">
@@ -22369,167 +22369,167 @@
         <v>2329</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>2330</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="18" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>2331</v>
+        <v>2330</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>2435</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="39" customHeight="1">
       <c r="A9" s="2" t="s">
+        <v>2331</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>2332</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>2333</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="22.5" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>2334</v>
+        <v>2333</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>2433</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="18" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>2335</v>
+        <v>2334</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>2432</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="26.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>2336</v>
+        <v>2335</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>2437</v>
+        <v>2434</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="28.5" customHeight="1">
       <c r="A13" s="2" t="s">
+        <v>2336</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>2337</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>2338</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" customHeight="1">
       <c r="A14" s="2" t="s">
+        <v>2338</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>2339</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>2340</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="36" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>2341</v>
+        <v>2340</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>2439</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="45" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>2342</v>
+        <v>2341</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>2441</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="43.5" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>2342</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>2343</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>2344</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="42" customHeight="1">
       <c r="A18" s="2" t="s">
+        <v>2344</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>2345</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>2346</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="52.5" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>2347</v>
+        <v>2346</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>2440</v>
+        <v>2437</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>2348</v>
+        <v>2347</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>2443</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>2444</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="409.5">
       <c r="A22" s="2" t="s">
+        <v>2349</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>2350</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>2351</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="255">
       <c r="A23" s="2" t="s">
+        <v>2351</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>2352</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>2353</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="240">
       <c r="A24" t="s">
+        <v>2353</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>2354</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>2355</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="270">
       <c r="A25" t="s">
+        <v>2355</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>2356</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>2357</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="210">
       <c r="A26" t="s">
+        <v>2357</v>
+      </c>
+      <c r="B26" s="6" t="s">
         <v>2358</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>2359</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="61.5" customHeight="1">
       <c r="A27" t="s">
+        <v>2359</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>2360</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>2361</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="105.75" customHeight="1">
@@ -22558,322 +22558,322 @@
     </row>
     <row r="31" spans="1:2" ht="135">
       <c r="A31" s="13" t="s">
+        <v>2361</v>
+      </c>
+      <c r="B31" s="14" t="s">
         <v>2362</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>2363</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="180">
       <c r="A32" s="15" t="s">
+        <v>2363</v>
+      </c>
+      <c r="B32" s="16" t="s">
         <v>2364</v>
-      </c>
-      <c r="B32" s="16" t="s">
-        <v>2365</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="180">
       <c r="A33" s="17" t="s">
+        <v>2365</v>
+      </c>
+      <c r="B33" s="18" t="s">
         <v>2366</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>2367</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="409.5">
       <c r="A34" s="19" t="s">
+        <v>2367</v>
+      </c>
+      <c r="B34" s="20" t="s">
         <v>2368</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>2369</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="409.5">
       <c r="A35" s="21" t="s">
+        <v>2369</v>
+      </c>
+      <c r="B35" s="22" t="s">
         <v>2370</v>
-      </c>
-      <c r="B35" s="22" t="s">
-        <v>2371</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="409.5">
       <c r="A36" s="23" t="s">
+        <v>2371</v>
+      </c>
+      <c r="B36" s="24" t="s">
         <v>2372</v>
-      </c>
-      <c r="B36" s="24" t="s">
-        <v>2373</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="409.5">
       <c r="A37" s="25" t="s">
+        <v>2373</v>
+      </c>
+      <c r="B37" s="26" t="s">
         <v>2374</v>
-      </c>
-      <c r="B37" s="26" t="s">
-        <v>2375</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="409.5">
       <c r="A38" s="27" t="s">
+        <v>2375</v>
+      </c>
+      <c r="B38" s="28" t="s">
         <v>2376</v>
-      </c>
-      <c r="B38" s="28" t="s">
-        <v>2377</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="409.5">
       <c r="A39" t="s">
+        <v>2377</v>
+      </c>
+      <c r="B39" s="29" t="s">
         <v>2378</v>
-      </c>
-      <c r="B39" s="29" t="s">
-        <v>2379</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="120">
       <c r="A40" t="s">
+        <v>2379</v>
+      </c>
+      <c r="B40" s="29" t="s">
         <v>2380</v>
-      </c>
-      <c r="B40" s="29" t="s">
-        <v>2381</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="180">
       <c r="A41" t="s">
+        <v>2381</v>
+      </c>
+      <c r="B41" s="29" t="s">
         <v>2382</v>
-      </c>
-      <c r="B41" s="29" t="s">
-        <v>2383</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="195">
       <c r="A42" t="s">
+        <v>2383</v>
+      </c>
+      <c r="B42" s="29" t="s">
         <v>2384</v>
-      </c>
-      <c r="B42" s="29" t="s">
-        <v>2385</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="120">
       <c r="A43" t="s">
+        <v>2385</v>
+      </c>
+      <c r="B43" s="29" t="s">
         <v>2386</v>
-      </c>
-      <c r="B43" s="29" t="s">
-        <v>2387</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="409.5">
       <c r="A44" t="s">
+        <v>2387</v>
+      </c>
+      <c r="B44" s="29" t="s">
         <v>2388</v>
-      </c>
-      <c r="B44" s="29" t="s">
-        <v>2389</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="409.5">
       <c r="A45" t="s">
+        <v>2389</v>
+      </c>
+      <c r="B45" s="29" t="s">
         <v>2390</v>
-      </c>
-      <c r="B45" s="29" t="s">
-        <v>2391</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="409.5">
       <c r="A46" t="s">
+        <v>2391</v>
+      </c>
+      <c r="B46" s="29" t="s">
         <v>2392</v>
-      </c>
-      <c r="B46" s="29" t="s">
-        <v>2393</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="270">
       <c r="A47" t="s">
+        <v>2393</v>
+      </c>
+      <c r="B47" s="29" t="s">
         <v>2394</v>
-      </c>
-      <c r="B47" s="29" t="s">
-        <v>2395</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="409.5">
       <c r="A48" t="s">
-        <v>2396</v>
+        <v>2466</v>
       </c>
       <c r="B48" s="29" t="s">
-        <v>2397</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="345">
       <c r="A49" t="s">
-        <v>2398</v>
+        <v>2395</v>
       </c>
       <c r="B49" s="29" t="s">
-        <v>2399</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="345">
       <c r="A50" t="s">
-        <v>2400</v>
+        <v>2397</v>
       </c>
       <c r="B50" s="29" t="s">
-        <v>2401</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="36" customHeight="1">
       <c r="A51" t="s">
-        <v>2402</v>
+        <v>2399</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>2438</v>
+        <v>2435</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="23.25" customHeight="1">
       <c r="A52" t="s">
-        <v>2403</v>
+        <v>2400</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>2452</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="27.75" customHeight="1">
       <c r="A53" t="s">
-        <v>2404</v>
+        <v>2401</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>2453</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="60">
       <c r="A54" t="s">
-        <v>2405</v>
+        <v>2402</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>2406</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="45">
       <c r="A55" t="s">
-        <v>2407</v>
+        <v>2404</v>
       </c>
       <c r="B55" s="29" t="s">
-        <v>2454</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="60">
       <c r="A56" t="s">
-        <v>2408</v>
+        <v>2405</v>
       </c>
       <c r="B56" s="29" t="s">
-        <v>2455</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="75">
       <c r="A57" t="s">
-        <v>2409</v>
+        <v>2406</v>
       </c>
       <c r="B57" s="29" t="s">
-        <v>2456</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="409.5">
       <c r="A58" t="s">
-        <v>2410</v>
+        <v>2407</v>
       </c>
       <c r="B58" s="29" t="s">
-        <v>2457</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="90">
       <c r="A59" t="s">
-        <v>2411</v>
+        <v>2408</v>
       </c>
       <c r="B59" s="29" t="s">
-        <v>2458</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="360">
       <c r="A60" t="s">
-        <v>2412</v>
+        <v>2409</v>
       </c>
       <c r="B60" s="29" t="s">
-        <v>2459</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="75">
       <c r="A61" t="s">
-        <v>2413</v>
+        <v>2410</v>
       </c>
       <c r="B61" s="29" t="s">
-        <v>2414</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="409.5">
       <c r="A62" t="s">
-        <v>2415</v>
+        <v>2412</v>
       </c>
       <c r="B62" s="29" t="s">
-        <v>2460</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="87.75" customHeight="1">
       <c r="A63" t="s">
-        <v>2416</v>
+        <v>2413</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>2461</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="71.25" customHeight="1">
       <c r="A64" t="s">
-        <v>2417</v>
+        <v>2414</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>2462</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="54" customHeight="1">
       <c r="A65" t="s">
-        <v>2384</v>
+        <v>2383</v>
       </c>
       <c r="B65" s="29" t="s">
-        <v>2463</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="86.25" customHeight="1">
       <c r="A66" s="29" t="s">
-        <v>2418</v>
+        <v>2415</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>2464</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="86.25" customHeight="1">
       <c r="A67" s="29" t="s">
-        <v>2419</v>
+        <v>2416</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>2465</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="102" customHeight="1">
       <c r="A68" s="29" t="s">
-        <v>2420</v>
+        <v>2417</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>2466</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="89.25" customHeight="1">
       <c r="A69" s="29" t="s">
-        <v>2421</v>
+        <v>2418</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>2467</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="102" customHeight="1">
       <c r="A70" s="29" t="s">
-        <v>2422</v>
+        <v>2419</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>2468</v>
+        <v>2465</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gate Entry Functions Customer Schedule Customer Items
Gate Entry Functions Customer Schedule Customer Items Fixes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -8530,243 +8530,6 @@
   </si>
   <si>
     <t>SsoQuery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SELECT sshd_bu posv_bu,
-          'SSO' posv_source,
-          DECODE (sshd_ps_type, 'PR', 'PO', 'SC') poh_mode,
-          sshd_plnt posv_plnt,
-          bup_name1 posv_plnt_desc,
-          sshd_doc_pfx,
-          sshd_doc_no,
-          ssln_seq_no,
-          ssld_sub_seq_no,
-          sshd_suplr_id,
-          suplr_name1,
-          'INR' posv_suplr_curry,
-          'SSPO' posv_type,
-          sshd_status posv_hd_status,
-          ssln_prod_id posv_prod_id,
-          ssln_prod_rev posv_prod_rev,
-          ssln_prod_desc1 posv_prod_desc1,
-          NULL posv_prod_ext_desc,
-          ssln_uom posv_uom,
-          ssln_prod_uom posv_prod_uom,
-          ssln_hsn_code posv_hsn_code,
-          prod_cls posv_prod_cls,
-          (SELECT NVL (class_desc1, class_desc2)
-             FROM classes
-            WHERE class_bu = prod_bu AND class_id = prod_cls)
-             posv_cls_desc,
-          prod_sub_cls posv_prod_sub_cls,
-          (SELECT NVL (subcls_desc1, subcls_desc2)
-             FROM sub_classes
-            WHERE     subcls_bu = prod_bu
-                  AND subcls_parcls_id = prod_cls
-                  AND subcls_id = prod_sub_cls)
-             posv_subcls_desc,
-          ssln_status posv_ln_status,
-          sshd_store_id posv_store_id,
-          (SELECT NVL (store_desc1, store_desc2)
-             FROM stores
-            WHERE store_bu = sshd_bu AND store_id = sshd_store_id)
-             posv_store_name,
-          'NA' posv_so_type,
-          NULL posv_so_pfx,
-          NULL posv_so_no,
-          NULL posv_so_seq_no,
-          NULL posv_so_sub_seq_no,
-          NULL posv_proj_id,
-          NULL posv_task_id,
-          ssld_schld_qty posv_ord_qty,
-          ssld_recvd_qty posv_recvd_qty,
-          ssld_inproc_qty posv_inproc_qty,
-          ssld_cls_qty posv_cls_qty,
-          ssln_price posv_unit_cost_tc,
-          ssln_disc_pct,
-          ( (ssld_schld_qty - ssld_cls_qty)
-           * (ssln_price - (ssln_price * (ssln_disc_pct / 100))))
-             posv_gross_amt_tc,
-          ssln_price posv_disc_amt_tc,
-          0 posv_tax_amt_tc,
-          ( (ssld_schld_qty - ssld_cls_qty)
-           * (ssln_price - (ssln_price * (ssln_disc_pct / 100))))
-             posv_net_amt_tc,
-          suplr_terr_id posv_terr_id,
-          prod_group_id posv_prod_grp_id,
-          prod_subgroup_id posv_prod_subgrp_id,
-          sshd_billfr_loc_id,
-          (SELECT ssl_loc_name1
-             FROM suplr_ship_loc
-            WHERE     ssl_bu = sshd_bu
-                  AND ssl_suplr_id = sshd_suplr_id
-                  AND ssl_loc_name1 = sshd_billfr_loc_name)
-             sshd_billfr_loc_desc,
-          ssa_billfr_gst_no,
-          ssa_shipfr_gst_no,
-          ssa_billto_gst_no,
-          ssa_shipto_gst_no,
-          TO_NUMBER (ssln_amd_no) ssln_amd_no,
-          NULL ssln_prod_ord_no,
-          (SELECT NVL (city_name1, city_name2)
-             FROM cities
-            WHERE city_bu = ssa_bu AND city_id = ssa_billfr_city),
-          (SELECT NVL (state_name1, state_name2)
-             FROM states
-            WHERE state_bu = ssa_bu AND state_id = ssa_billfr_state),
-          (SELECT NVL (cntry_name1, cntry_name2)
-             FROM countries
-            WHERE cntry_bu = ssa_bu AND cntry_id = ssa_billfr_cntry),
-          sshd_billfr_loc_name || ',' || ssa_billfr_addr1
-          || NVL2 (ssa_billfr_addr1,
-                   ',' || ssa_billfr_addr2,
-                   ssa_billfr_addr2)
-          || NVL2 (ssa_billfr_addr2,
-                   ',' || ssa_billfr_addr3,
-                   ssa_billfr_addr3)
-          || (SELECT NVL (city_name1, city_name2)
-                FROM cities
-               WHERE city_bu = ssa_bu AND city_id = ssa_billfr_city)
-          || NVL2 (
-                (SELECT NVL (state_name1, state_name2)
-                   FROM states
-                  WHERE state_bu = ssa_bu AND state_id = ssa_billfr_state),
-                ','
-                || (SELECT NVL (state_name1, state_name2)
-                      FROM states
-                     WHERE state_bu = ssa_bu AND state_id = ssa_billfr_state),
-                ' ')
-          || NVL2 (
-                (SELECT NVL (cntry_name1, cntry_name2)
-                   FROM countries
-                  WHERE cntry_bu = ssa_bu AND cntry_id = ssa_billfr_cntry),
-                ','
-                || (SELECT NVL (cntry_name1, cntry_name2)
-                      FROM countries
-                     WHERE cntry_bu = ssa_bu AND cntry_id = ssa_billfr_cntry),
-                ' '),
-          sshd_billto_loc_name || ',' || ssa_billto_addr1
-          || NVL2 (ssa_billto_addr1,
-                   ',' || ssa_billto_addr2,
-                   ssa_billto_addr2)
-          || NVL2 (ssa_billto_addr2,
-                   ',' || ssa_billto_addr3,
-                   ssa_billto_addr3)
-          || (SELECT NVL (city_name1, city_name2)
-                FROM cities
-               WHERE city_bu = ssa_bu AND city_id = ssa_billto_city)
-          || NVL2 (ssa_shipto_addr1,
-                   ',' || ssa_shipto_addr2,
-                   ssa_shipto_addr2)
-          || NVL2 (ssa_shipto_addr2,
-                   ',' || ssa_shipto_addr3,
-                   ssa_shipto_addr3)
-          || (SELECT NVL (city_name1, city_name2)
-                FROM cities
-               WHERE city_bu = ssa_bu AND city_id = ssa_shipto_city)
-          || NVL2 (
-                (SELECT NVL (state_name1, state_name2)
-                   FROM states
-                  WHERE state_bu = ssa_bu AND state_id = ssa_shipto_state),
-                ','
-                || (SELECT NVL (state_name1, state_name2)
-                      FROM states
-                     WHERE state_bu = ssa_bu AND state_id = ssa_shipto_state),
-                ' ')
-          || NVL2 (
-                (SELECT NVL (cntry_name1, cntry_name2)
-                   FROM countries
-                  WHERE cntry_bu = ssa_bu AND cntry_id = ssa_shipto_cntry),
-                ','
-                || (SELECT NVL (cntry_name1, cntry_name2)
-                      FROM countries
-                     WHERE cntry_bu = ssa_bu AND cntry_id = ssa_shipto_cntry),
-                ' '),
-          (SELECT NVL (city_name1, city_name2)
-             FROM cities
-            WHERE city_bu = ssa_bu AND city_id = ssa_orderby_city),
-          (SELECT NVL (state_name1, state_name2)
-             FROM states
-            WHERE state_bu = ssa_bu AND state_id = ssa_orderby_state),
-          (SELECT NVL (cntry_name1, cntry_name2)
-             FROM countries
-            WHERE cntry_bu = ssa_bu AND cntry_id = ssa_orderby_cntry),
-          sshd_shipfr_loc_name || ssa_orderby_addr1
-          || NVL2 (ssa_orderby_addr1,
-                   ',' || ssa_orderby_addr2,
-                   ssa_orderby_addr2)
-          || NVL2 (ssa_orderby_addr2,
-                   ',' || ssa_orderby_addr3,
-                   ssa_orderby_addr3)
-          || (SELECT NVL (city_name1, city_name2)
-                FROM cities
-               WHERE city_bu = ssa_bu AND city_id = ssa_orderby_city)
-          || NVL2 (
-                (SELECT NVL (state_name1, state_name2)
-                   FROM states
-                  WHERE state_bu = ssa_bu AND state_id = ssa_orderby_state),
-                ','
-                || (SELECT NVL (state_name1, state_name2)
-                      FROM states
-                     WHERE state_bu = ssa_bu AND state_id = ssa_orderby_state),
-                ' ')
-          || NVL2 (
-                (SELECT NVL (cntry_name1, cntry_name2)
-                   FROM countries
-                  WHERE cntry_bu = ssa_bu AND cntry_id = ssa_orderby_cntry),
-                ','
-                || (SELECT NVL (cntry_name1, cntry_name2)
-                      FROM countries
-                     WHERE cntry_bu = ssa_bu AND cntry_id = ssa_orderby_cntry),
-                ' '),
-          0,
-          0,
-          0,
-          0,
-          0,
-          0,
-          ssld_promise_date,
-          ssln_cre_date,
-          ssld_type posv_firm_type,
-          'Y',
-          NULL pol_matl_type
-     FROM suplr_schld_hd,
-          suplr_schld_ln,
-          suplr_schld_ln_dtls,
-          bus_unit_plants,
-          suppliers,
-          prod_plants,
-          products,
-          suplr_schld_addr,
-          fin_periods
-   WHERE  --   sshd_bu = ssln_bu
-      --    AND sshd_plnt = ssln_plnt
-         -- AND sshd_doc_pfx = ssln_doc_pfx
-        --  AND sshd_doc_no = ssln_doc_no
-        --  AND ssld_bu = ssln_bu
-         -- AND ssld_plnt = ssln_plnt
-       --   AND ssld_doc_pfx = ssln_doc_pfx
-       --   AND ssld_doc_no = ssln_doc_no
-       --   AND ssld_seq_no = ssln_seq_no
-          fp_bu = sshd_bu
-          AND TRUNC (sshd_doc_date) BETWEEN fp_from_date AND fp_end_date
-          AND ssa_bu(+) = sshd_bu
-          AND ssa_doc_pfx(+) = sshd_doc_pfx
-          AND ssa_doc_no(+) = sshd_doc_no
-          AND bup_bu = sshd_bu
-          AND bup_plant_id = sshd_plnt
-          AND suplr_bu = sshd_bu
-          AND suplr_suplr_id = sshd_suplr_id
-          AND prodplnt_bu = ssln_bu
-          AND prodplnt_plnt = ssln_plnt
-          AND prodplnt_prod_id = ssln_prod_id
-          AND prodplnt_prod_rev = ssln_prod_rev
-          AND prod_bu = prodplnt_bu
-          AND prod_id = prodplnt_prod_id
-          AND prod_rev = prodplnt_prod_rev
-      AND sshd_bu = 'ROAU'
-      AND sshd_doc_no ='${SSONO}'
-</t>
   </si>
   <si>
     <t>OpoQuery</t>
@@ -10019,6 +9782,13 @@
     FROM rework_order_comp_dtl_hist
   WHERE rwocdh_bu = 'ROAU'
         AND rwocdh_doc_no = '${RWCNO}'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select *
+FROM suplr_schld_hd
+WHERE sshd_bu ='ROAU'
+AND SSHD_DOC_NO ='${SSONO}'
+</t>
   </si>
 </sst>
 </file>
@@ -22233,7 +22003,7 @@
         <v>2346</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1">
@@ -22297,7 +22067,7 @@
         <v>2362</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>2463</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="36" customHeight="1">
@@ -22385,7 +22155,7 @@
         <v>2383</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="210">
@@ -22393,7 +22163,7 @@
         <v>2384</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="61.5" customHeight="1">
@@ -22484,193 +22254,193 @@
         <v>2402</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="409.5">
+    <row r="38" spans="1:2" ht="90">
       <c r="A38" t="s">
         <v>2403</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>2404</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="120">
       <c r="A39" t="s">
+        <v>2404</v>
+      </c>
+      <c r="B39" s="27" t="s">
         <v>2405</v>
-      </c>
-      <c r="B39" s="27" t="s">
-        <v>2406</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="180">
       <c r="A40" t="s">
+        <v>2406</v>
+      </c>
+      <c r="B40" s="27" t="s">
         <v>2407</v>
-      </c>
-      <c r="B40" s="27" t="s">
-        <v>2408</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="195">
       <c r="A41" t="s">
+        <v>2408</v>
+      </c>
+      <c r="B41" s="27" t="s">
         <v>2409</v>
-      </c>
-      <c r="B41" s="27" t="s">
-        <v>2410</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="120">
       <c r="A42" t="s">
+        <v>2410</v>
+      </c>
+      <c r="B42" s="27" t="s">
         <v>2411</v>
-      </c>
-      <c r="B42" s="27" t="s">
-        <v>2412</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="409.5">
       <c r="A43" t="s">
-        <v>2413</v>
+        <v>2412</v>
       </c>
       <c r="B43" s="27" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="409.5">
       <c r="A44" t="s">
-        <v>2414</v>
+        <v>2413</v>
       </c>
       <c r="B44" s="27" t="s">
-        <v>2467</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="409.5">
       <c r="A45" t="s">
-        <v>2415</v>
+        <v>2414</v>
       </c>
       <c r="B45" s="27" t="s">
-        <v>2468</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="270">
       <c r="A46" t="s">
+        <v>2415</v>
+      </c>
+      <c r="B46" s="27" t="s">
         <v>2416</v>
-      </c>
-      <c r="B46" s="27" t="s">
-        <v>2417</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="409.5">
       <c r="A47" t="s">
+        <v>2417</v>
+      </c>
+      <c r="B47" s="27" t="s">
         <v>2418</v>
-      </c>
-      <c r="B47" s="27" t="s">
-        <v>2419</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="345">
       <c r="A48" t="s">
+        <v>2419</v>
+      </c>
+      <c r="B48" s="27" t="s">
         <v>2420</v>
-      </c>
-      <c r="B48" s="27" t="s">
-        <v>2421</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="345">
       <c r="A49" t="s">
+        <v>2421</v>
+      </c>
+      <c r="B49" s="27" t="s">
         <v>2422</v>
-      </c>
-      <c r="B49" s="27" t="s">
-        <v>2423</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="36" customHeight="1">
       <c r="A50" t="s">
+        <v>2423</v>
+      </c>
+      <c r="B50" s="6" t="s">
         <v>2424</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>2425</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="23.25" customHeight="1">
       <c r="A51" t="s">
+        <v>2425</v>
+      </c>
+      <c r="B51" s="6" t="s">
         <v>2426</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>2427</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="27.75" customHeight="1">
       <c r="A52" t="s">
+        <v>2427</v>
+      </c>
+      <c r="B52" s="6" t="s">
         <v>2428</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>2429</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="60">
       <c r="A53" t="s">
+        <v>2429</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>2430</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>2431</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="45">
       <c r="A54" t="s">
+        <v>2431</v>
+      </c>
+      <c r="B54" s="27" t="s">
         <v>2432</v>
-      </c>
-      <c r="B54" s="27" t="s">
-        <v>2433</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="60">
       <c r="A55" t="s">
+        <v>2433</v>
+      </c>
+      <c r="B55" s="27" t="s">
         <v>2434</v>
-      </c>
-      <c r="B55" s="27" t="s">
-        <v>2435</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="75">
       <c r="A56" t="s">
+        <v>2435</v>
+      </c>
+      <c r="B56" s="27" t="s">
         <v>2436</v>
-      </c>
-      <c r="B56" s="27" t="s">
-        <v>2437</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="409.5">
       <c r="A57" t="s">
+        <v>2437</v>
+      </c>
+      <c r="B57" s="27" t="s">
         <v>2438</v>
-      </c>
-      <c r="B57" s="27" t="s">
-        <v>2439</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="90">
       <c r="A58" t="s">
+        <v>2439</v>
+      </c>
+      <c r="B58" s="27" t="s">
         <v>2440</v>
-      </c>
-      <c r="B58" s="27" t="s">
-        <v>2441</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="360">
       <c r="A59" t="s">
+        <v>2441</v>
+      </c>
+      <c r="B59" s="27" t="s">
         <v>2442</v>
-      </c>
-      <c r="B59" s="27" t="s">
-        <v>2443</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="75">
       <c r="A60" t="s">
+        <v>2443</v>
+      </c>
+      <c r="B60" s="27" t="s">
         <v>2444</v>
-      </c>
-      <c r="B60" s="27" t="s">
-        <v>2445</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="409.5">
       <c r="A61" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
       <c r="B61" s="27" t="s">
         <v>2368</v>
@@ -22678,66 +22448,66 @@
     </row>
     <row r="62" spans="1:2" ht="87.75" customHeight="1">
       <c r="A62" t="s">
+        <v>2446</v>
+      </c>
+      <c r="B62" s="6" t="s">
         <v>2447</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>2448</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="71.25" customHeight="1">
       <c r="A63" t="s">
+        <v>2448</v>
+      </c>
+      <c r="B63" s="6" t="s">
         <v>2449</v>
-      </c>
-      <c r="B63" s="6" t="s">
-        <v>2450</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="54" customHeight="1">
       <c r="A64" t="s">
-        <v>2409</v>
+        <v>2408</v>
       </c>
       <c r="B64" s="27" t="s">
-        <v>2451</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="86.25" customHeight="1">
       <c r="A65" s="27" t="s">
+        <v>2451</v>
+      </c>
+      <c r="B65" s="6" t="s">
         <v>2452</v>
-      </c>
-      <c r="B65" s="6" t="s">
-        <v>2453</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="86.25" customHeight="1">
       <c r="A66" s="27" t="s">
+        <v>2453</v>
+      </c>
+      <c r="B66" s="6" t="s">
         <v>2454</v>
-      </c>
-      <c r="B66" s="6" t="s">
-        <v>2455</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="102" customHeight="1">
       <c r="A67" s="27" t="s">
+        <v>2455</v>
+      </c>
+      <c r="B67" s="6" t="s">
         <v>2456</v>
-      </c>
-      <c r="B67" s="6" t="s">
-        <v>2457</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="89.25" customHeight="1">
       <c r="A68" s="27" t="s">
+        <v>2457</v>
+      </c>
+      <c r="B68" s="6" t="s">
         <v>2458</v>
-      </c>
-      <c r="B68" s="6" t="s">
-        <v>2459</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="102" customHeight="1">
       <c r="A69" s="27" t="s">
+        <v>2459</v>
+      </c>
+      <c r="B69" s="6" t="s">
         <v>2460</v>
-      </c>
-      <c r="B69" s="6" t="s">
-        <v>2461</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HRM Overtime New Scenarios Added
HRM Overtime New Scenarios Added
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,13 +4,14 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="8400" activeTab="1"/>
+    <workbookView xWindow="990" yWindow="2440" windowWidth="13910" windowHeight="4230" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2994" uniqueCount="2469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2996" uniqueCount="2471">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -9790,17 +9791,32 @@
 AND SSHD_DOC_NO ='${SSONO}'
 </t>
   </si>
+  <si>
+    <t>OvertimeAmount</t>
+  </si>
+  <si>
+    <t>Select * From  emp_ovrt_ln 
+Where EOLN_BU='ROAU'
+And EOLN_DOC_NO='${OTNO}'</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -9914,27 +9930,27 @@
   </borders>
   <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -9952,19 +9968,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -9976,7 +9992,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -9984,108 +10000,109 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10376,10 +10393,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B1445"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5"/>
   <cols>
-    <col min="1" max="1" width="62.7109375" style="28" customWidth="1"/>
-    <col min="2" max="2" width="59.85546875" style="29" customWidth="1"/>
+    <col min="1" max="1" width="62.7265625" style="28" customWidth="1"/>
+    <col min="2" max="2" width="59.81640625" style="29" customWidth="1"/>
     <col min="3" max="16384" width="9" style="28"/>
   </cols>
   <sheetData>
@@ -21951,10 +21968,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B69"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:B70"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -21966,7 +21983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="108.95" customHeight="1">
+    <row r="2" spans="1:2" ht="109" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2338</v>
       </c>
@@ -22134,7 +22151,7 @@
         <v>2378</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="255">
+    <row r="23" spans="1:2" ht="246.5">
       <c r="A23" s="2" t="s">
         <v>2379</v>
       </c>
@@ -22142,7 +22159,7 @@
         <v>2380</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="240">
+    <row r="24" spans="1:2" ht="232">
       <c r="A24" t="s">
         <v>2381</v>
       </c>
@@ -22150,7 +22167,7 @@
         <v>2382</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="270">
+    <row r="25" spans="1:2" ht="261">
       <c r="A25" t="s">
         <v>2383</v>
       </c>
@@ -22158,7 +22175,7 @@
         <v>2463</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="210">
+    <row r="26" spans="1:2" ht="203">
       <c r="A26" t="s">
         <v>2384</v>
       </c>
@@ -22182,7 +22199,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="180">
+    <row r="29" spans="1:2" ht="174">
       <c r="A29" s="9" t="s">
         <v>2346</v>
       </c>
@@ -22190,7 +22207,7 @@
         <v>2347</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="135">
+    <row r="30" spans="1:2" ht="130.5">
       <c r="A30" s="11" t="s">
         <v>2387</v>
       </c>
@@ -22198,7 +22215,7 @@
         <v>2388</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="180">
+    <row r="31" spans="1:2" ht="174">
       <c r="A31" s="13" t="s">
         <v>2389</v>
       </c>
@@ -22206,7 +22223,7 @@
         <v>2390</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="180">
+    <row r="32" spans="1:2" ht="174">
       <c r="A32" s="15" t="s">
         <v>2391</v>
       </c>
@@ -22222,7 +22239,7 @@
         <v>2394</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="409.5">
+    <row r="34" spans="1:2" ht="406">
       <c r="A34" s="19" t="s">
         <v>2395</v>
       </c>
@@ -22254,7 +22271,7 @@
         <v>2402</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="90">
+    <row r="38" spans="1:2" ht="87">
       <c r="A38" t="s">
         <v>2403</v>
       </c>
@@ -22262,7 +22279,7 @@
         <v>2468</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="120">
+    <row r="39" spans="1:2" ht="116">
       <c r="A39" t="s">
         <v>2404</v>
       </c>
@@ -22270,7 +22287,7 @@
         <v>2405</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="180">
+    <row r="40" spans="1:2" ht="174">
       <c r="A40" t="s">
         <v>2406</v>
       </c>
@@ -22278,7 +22295,7 @@
         <v>2407</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="195">
+    <row r="41" spans="1:2" ht="188.5">
       <c r="A41" t="s">
         <v>2408</v>
       </c>
@@ -22286,7 +22303,7 @@
         <v>2409</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="120">
+    <row r="42" spans="1:2" ht="116">
       <c r="A42" t="s">
         <v>2410</v>
       </c>
@@ -22318,7 +22335,7 @@
         <v>2467</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="270">
+    <row r="46" spans="1:2" ht="261">
       <c r="A46" t="s">
         <v>2415</v>
       </c>
@@ -22334,7 +22351,7 @@
         <v>2418</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="345">
+    <row r="48" spans="1:2" ht="333.5">
       <c r="A48" t="s">
         <v>2419</v>
       </c>
@@ -22342,7 +22359,7 @@
         <v>2420</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="345">
+    <row r="49" spans="1:2" ht="333.5">
       <c r="A49" t="s">
         <v>2421</v>
       </c>
@@ -22374,7 +22391,7 @@
         <v>2428</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="60">
+    <row r="53" spans="1:2" ht="58">
       <c r="A53" t="s">
         <v>2429</v>
       </c>
@@ -22382,7 +22399,7 @@
         <v>2430</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="45">
+    <row r="54" spans="1:2" ht="43.5">
       <c r="A54" t="s">
         <v>2431</v>
       </c>
@@ -22390,7 +22407,7 @@
         <v>2432</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="60">
+    <row r="55" spans="1:2" ht="58">
       <c r="A55" t="s">
         <v>2433</v>
       </c>
@@ -22398,7 +22415,7 @@
         <v>2434</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="75">
+    <row r="56" spans="1:2" ht="72.5">
       <c r="A56" t="s">
         <v>2435</v>
       </c>
@@ -22414,7 +22431,7 @@
         <v>2438</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="90">
+    <row r="58" spans="1:2" ht="87">
       <c r="A58" t="s">
         <v>2439</v>
       </c>
@@ -22422,7 +22439,7 @@
         <v>2440</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="360">
+    <row r="59" spans="1:2" ht="348">
       <c r="A59" t="s">
         <v>2441</v>
       </c>
@@ -22430,7 +22447,7 @@
         <v>2442</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="75">
+    <row r="60" spans="1:2" ht="58">
       <c r="A60" t="s">
         <v>2443</v>
       </c>
@@ -22508,6 +22525,14 @@
       </c>
       <c r="B69" s="6" t="s">
         <v>2460</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="43.5">
+      <c r="A70" s="71" t="s">
+        <v>2469</v>
+      </c>
+      <c r="B70" s="27" t="s">
+        <v>2470</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added New Finance scenarios Of BP, BR, CP And CR Screens
Added New Finance scenarios Of BP, BR, CP And CR Screens
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="990" yWindow="2440" windowWidth="13910" windowHeight="4230" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15300" windowHeight="6540" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2996" uniqueCount="2471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3016" uniqueCount="2491">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -7449,19 +7449,6 @@
   </si>
   <si>
     <t>PaymentTermQuery</t>
-  </si>
-  <si>
-    <t>SELECT term_desc1,
-       trln_mtrl_pct,
-       trln_tax_pct,
-       TRLN_CLAIM_TYPE
-  FROM terms_ln,
-       terms_hd
- WHERE  term_bu = trln_bu
-   AND term_bu = 'ROAU'
-   AND  TRLN_CLAIM_TYPE ='A'
-  AND term_term_id = trln_term_id
-  AND  term_desc1 = '${SONO}'</t>
   </si>
   <si>
     <t>AdvanceReceiptQuery</t>
@@ -8060,24 +8047,6 @@
   </si>
   <si>
     <t>SalesInvHeaderQuery</t>
-  </si>
-  <si>
-    <t>SELECT sihd_plnt_loc_id,
-       sihd_plant,
-       sihd_doc_pfx,
-       sihd_doc_no,
-       sihd_type,
-       sihd_cust_id,
-       sihd_currency,
-              DECODE (sihd_status,
-               'N', 'Draft',
-               'I', 'Invoiced',
-               'C', 'Cancelled',
-               'E', 'Entry Completed')
-          sihd_status
-  FROM sales_invoices_hd
-where sihd_bu = 'ROAU'
-  and sihd_doc_no = '${SINO}'</t>
   </si>
   <si>
     <t>PRBucket Query</t>
@@ -9799,17 +9768,318 @@
 Where EOLN_BU='ROAU'
 And EOLN_DOC_NO='${OTNO}'</t>
   </si>
+  <si>
+    <t>BankPaymentHeaderQuery</t>
+  </si>
+  <si>
+    <t>SELECT BTRANS_ORD_PFX,
+       BTRANS_TRANS_CURCY,
+       BTRANS_BANK_NAME,
+       BTRANS_TRANS_AMT,
+       BTRANS_BANK_RGL_AMT,
+       BTRANS_TRANS_CHG_AMT,
+       BTRANS_BANK_CHG_AMT,
+       BTRANS_BANK_NET_AMT,
+       DECODE (BTRANS_STATUS,
+               'N', 'Draft',
+               'O', 'Entry Completed',
+               'I', 'Issued',
+               'R', 'Received',
+               'C', 'Cleared',
+               'X', 'Cancelled',
+               'V', 'Void',
+               'D', 'Deleted',
+               'S', 'Posted',
+               'P', 'Approved')
+          BTRANS_STATUS
+  FROM BANK_TRANS
+ WHERE BTRANS_BU = 'ROAU'
+AND BTRANS_ORD_NO = '${SONO}'
+union all
+SELECT BTRANSH_ORD_PFX,
+       BTRANSH_TRANS_CURCY,
+       BTRANSH_BANK_NAME,
+        BTRANSH_TRANS_AMT,
+       BTRANSH_BANK_RGL_AMT,
+       BTRANSH_TRANS_CHG_AMT,
+       BTRANSH_BANK_CHG_AMT,
+       BTRANSH_BANK_NET_AMT,
+       DECODE (BTRANSH_STATUS,
+               'N', 'Draft',
+               'O', 'Entry Completed',
+               'I', 'Issued',
+               'R', 'Received',
+               'C', 'Cleared',
+               'X', 'Cancelled',
+               'V', 'Void',
+               'D', 'Deleted',
+               'S', 'Posted',
+               'P', 'Approved')
+          BTRANSH_STATUS
+  FROM bank_trans_hist
+ WHERE BTRANSH_BU = 'ROAU'
+AND BTRANSH_ORD_NO = '${SONO}'</t>
+  </si>
+  <si>
+    <t>BankPaymentLineQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  select * from bank_trans_dist_ln
+where BTDLN_BU = 'ROAU'
+AND BTDLN_ORD_NO ='${SONO}'
+AND BTDLN_SEQ_NO ='${PONO}'</t>
+  </si>
+  <si>
+    <t>GLMControlQuery</t>
+  </si>
+  <si>
+    <t>select * from glm_control
+where GLMCTRL_BU = '${SONO}'</t>
+  </si>
+  <si>
+    <t>BankReceiptPendingQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SELECT *
+    FROM pending_receivable_vw_hist_rev
+   WHERE par_bu = 'ROAU'
+   AND PAR_SRC_DOC_NO = '${SONO}'</t>
+  </si>
+  <si>
+    <t>ExchangeRateQuery</t>
+  </si>
+  <si>
+    <t>Select * from (
+Select * from
+mon_exchange_rates
+where MEXRATE_BU = 'ROAU' 
+and MEXRATE_FM_CURCY_ID = 'INR'
+and MEXRATE_TO_CURCY_ID ='${SONO}'
+ORDER BY MEXRATE_DATE DESC)
+where ROWNUM = 1</t>
+  </si>
+  <si>
+    <t>BankPaymentPendingQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SELECT *
+    FROM pending_payables_vw_hist_rev
+   WHERE par_bu = 'ROAU'
+   AND PAR_SRC_DOC_NO = '${SONO}'</t>
+  </si>
+  <si>
+    <t>PBHeaderQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  select * from suplr_doc_hd_hist
+  where SUPHDH_BU = 'ROAU'
+   AND SUPHDH_DOC_NO = '${SONO}'</t>
+  </si>
+  <si>
+    <t>SOLineQueryWithSeq</t>
+  </si>
+  <si>
+    <t>SELECT soq_prod_id "Item ID",soq_prod_rev "Item Rev",
+       soq_prod_desc1 "Item Desc",
+       soq_uom "Sale UOM",
+       soq_hsn_code "HSN Code",
+       soq_tax_pct "Tax Percentage",
+       soq_price_basis "Price Basis Type",
+       DECODE (soq_price_basis,
+               'C', 'Open Order',
+               'L', 'Catalog Price',
+               'P', 'Price List',
+               'S', 'Standard Price',
+               'U', 'User Defined')
+          "Price Basis Desc",
+       soq_cont_cat_no "Contract Number",
+       soq_catalog_no "Catalog / Price List Number",
+       soq_prod_uom "Stock UOM",
+       soq_conv_factor "Conversion Factor",
+       soq_tolr_type "Tolerance Type",
+       soq_cust_prod_id "Customer Item ID",
+       soq_cust_prod_desc "Customer Item Desc",
+       (SELECT store_desc1
+          FROM stores
+         WHERE store_bu = soq_bu AND store_id = soq_store_id
+        UNION ALL
+        SELECT dept_name1
+          FROM departments
+         WHERE dept_bu = soq_bu AND dept_id = soq_store_id)
+          "Warehouse Description",
+       soq_prod_subcls_desc "SubClass Desc",
+       soq_prod_cls_desc "Class Desc",
+       (SELECT spc_class_desc
+          FROM sales_price_classes
+         WHERE spc_bu = soq_bu AND spc_class_id = soq_sales_price_class)
+          "Price Class",
+       soq_promotion_flag "Promotional",
+       soq_trd_assbl_val "Trade Ass. Val.",
+       soq_disc_pct "Trade Disc. %",
+       soq_disc_amt "Trade Disc. Amt.",
+       soq_spl_assbl_val "Spl. Ass. Val.",
+       soq_spl_disc_pct "Spl. Disc. %",
+       soq_spl_disc_amt "Spl. Disc. Amt.",
+       soq_cash_assbl_val "Cash Ass. Val.",
+       soq_cash_disc_pct "Cash Disc. %",
+       soq_cash_disc_amt "Cash Disc. Amt.",
+       soq_gross_amt "Gross Amt.",
+       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
+       soq_tax_amt "Tax Amt.",
+       soq_net_amt "Net Amt.",
+       soq_gross_amt "Gross Amt.",
+       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
+       soq_tax_amt "Tax Amt.",
+       soq_net_amt "Net Amt.",
+       soq_qty_ordered "Ord. Qty.",
+       soq_price "Unit Price",
+       soq_tot_disc_amt "Disc. Amt.",
+       soq_igst_amt "IGST Amt.",
+       soq_sgst_amt "SGST Amt.",
+       soq_cgst_amt "CGST Amt.",
+       SOQ_SEQ_NO "Seq Number",
+       SOQ_CESS_PCT,
+       SOQ_CESS_AMT,
+       soq_utgst_amt,
+       DECODE(soq_status,'N','Draft','A','Approved','O','Entry Completed','L','Cancelled')Line_Status
+  FROM sales_order_hd, sales_order_qtys
+ WHERE     soh_bu = soq_bu
+       AND soh_order_no = soq_order_no
+       AND soh_bu = 'ROAU'
+       AND soh_order_no = '${SONO}'
+       AND SOQ_SEQ_NO =  '${PONO}'</t>
+  </si>
+  <si>
+    <t>SOLineQueryWithSeq1</t>
+  </si>
+  <si>
+    <t>SELECT soq_prod_id "Item ID",soq_prod_rev "Item Rev",
+       soq_prod_desc1 "Item Desc",
+       soq_uom "Sale UOM",
+       soq_hsn_code "HSN Code",
+       soq_tax_pct "Tax Percentage",
+       soq_price_basis "Price Basis Type",
+       DECODE (soq_price_basis,
+               'C', 'Open Order',
+               'L', 'Catalog Price',
+               'P', 'Price List',
+               'S', 'Standard Price',
+               'U', 'User Defined')
+          "Price Basis Desc",
+       soq_cont_cat_no "Contract Number",
+       soq_catalog_no "Catalog / Price List Number",
+       soq_prod_uom "Stock UOM",
+       soq_conv_factor "Conversion Factor",
+       soq_tolr_type "Tolerance Type",
+       soq_cust_prod_id "Customer Item ID",
+       soq_cust_prod_desc "Customer Item Desc",
+       (SELECT store_desc1
+          FROM stores
+         WHERE store_bu = soq_bu AND store_id = soq_store_id
+        UNION ALL
+        SELECT dept_name1
+          FROM departments
+         WHERE dept_bu = soq_bu AND dept_id = soq_store_id)
+          "Warehouse Description",
+       soq_prod_subcls_desc "SubClass Desc",
+       soq_prod_cls_desc "Class Desc",
+       (SELECT spc_class_desc
+          FROM sales_price_classes
+         WHERE spc_bu = soq_bu AND spc_class_id = soq_sales_price_class)
+          "Price Class",
+       soq_promotion_flag "Promotional",
+       soq_trd_assbl_val "Trade Ass. Val.",
+       soq_disc_pct "Trade Disc. %",
+       soq_disc_amt "Trade Disc. Amt.",
+       soq_spl_assbl_val "Spl. Ass. Val.",
+       soq_spl_disc_pct "Spl. Disc. %",
+       soq_spl_disc_amt "Spl. Disc. Amt.",
+       soq_cash_assbl_val "Cash Ass. Val.",
+       soq_cash_disc_pct "Cash Disc. %",
+       soq_cash_disc_amt "Cash Disc. Amt.",
+       soq_gross_amt "Gross Amt.",
+       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
+       soq_tax_amt "Tax Amt.",
+       soq_net_amt "Net Amt.",
+       soq_gross_amt "Gross Amt.",
+       soq_disc_amt_per_qty "Disc. Amt. / Qty.",
+       soq_tax_amt "Tax Amt.",
+       soq_net_amt "Net Amt.",
+       soq_qty_ordered "Ord. Qty.",
+       soq_price "Unit Price",
+       soq_tot_disc_amt "Disc. Amt.",
+       soq_igst_amt "IGST Amt.",
+       soq_sgst_amt "SGST Amt.",
+       soq_cgst_amt "CGST Amt.",
+       SOQ_SEQ_NO "Seq Number",
+       SOQ_CESS_PCT,
+       SOQ_CESS_AMT,
+       soq_utgst_amt,
+       DECODE(soq_status,'N','Draft','A','Approved','O','Entry Completed','L','Cancelled')Line_Status
+  FROM sales_order_hd, sales_order_qtys
+ WHERE     soh_bu = soq_bu
+       AND soh_order_no = soq_order_no
+       AND soh_bu = 'ROAU'
+       AND soh_order_no =  '${SONO}' 
+       order by SOQ_SEQ_NO</t>
+  </si>
+  <si>
+    <t>GRNPBHeaderQuery</t>
+  </si>
+  <si>
+    <t>select * from PUR_ORD_RECEIPT_HD_VIEW
+ where PORH_BU = 'ROAU'
+ AND PORH_RECEIPT_NO ='${GRNNO}'</t>
+  </si>
+  <si>
+    <t>SELECT sihd_plnt_loc_id,
+       sihd_plant,
+       sihd_doc_pfx,
+       sihd_doc_no,
+       sihd_type,
+       sihd_cust_id,
+       sihd_currency,
+       SIHD_TOT_AMT,
+              DECODE (sihd_status,
+               'N', 'Draft',
+               'I', 'Invoiced',
+               'C', 'Cancelled',
+               'E', 'Entry Completed')
+          sihd_status
+  FROM sales_invoices_hd
+where sihd_bu = 'ROAU'
+  and sihd_doc_no = '${SINO}'</t>
+  </si>
+  <si>
+    <t>SELECT TRLN_DUE_DAYS,term_term_id, term_desc1,
+       trln_mtrl_pct,
+       trln_tax_pct,
+       TRLN_CLAIM_TYPE
+  FROM terms_ln,
+       terms_hd
+ WHERE  term_bu = trln_bu
+   AND term_bu = 'ROAU'
+ AND term_term_id = trln_term_id
+  AND  term_desc1 = '${SONO}'</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -9930,27 +10200,27 @@
   </borders>
   <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -9968,19 +10238,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -9992,7 +10262,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -10000,107 +10270,111 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -10393,10 +10667,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B1445"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="62.7265625" style="28" customWidth="1"/>
-    <col min="2" max="2" width="59.81640625" style="29" customWidth="1"/>
+    <col min="1" max="1" width="62.7109375" style="28" customWidth="1"/>
+    <col min="2" max="2" width="59.85546875" style="29" customWidth="1"/>
     <col min="3" max="16384" width="9" style="28"/>
   </cols>
   <sheetData>
@@ -21968,10 +22242,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B70"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <dimension ref="A1:B80"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -21983,7 +22257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="109" customHeight="1">
+    <row r="2" spans="1:2" ht="108.95" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2338</v>
       </c>
@@ -22020,7 +22294,7 @@
         <v>2346</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2461</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1">
@@ -22064,131 +22338,131 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="26.25" customHeight="1">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>2358</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>2359</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="28.5" customHeight="1">
       <c r="A13" s="2" t="s">
+        <v>2359</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>2360</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>2361</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>2362</v>
+        <v>2361</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>2462</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="36" customHeight="1">
       <c r="A15" s="2" t="s">
+        <v>2362</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>2363</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>2364</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="45" customHeight="1">
       <c r="A16" s="2" t="s">
+        <v>2364</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>2365</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>2366</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="43.5" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>2366</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>2367</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>2368</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="42" customHeight="1">
       <c r="A18" s="2" t="s">
+        <v>2368</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>2369</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>2370</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="52.5" customHeight="1">
       <c r="A19" s="2" t="s">
+        <v>2370</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>2371</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>2372</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" customHeight="1">
       <c r="A20" s="4" t="s">
+        <v>2372</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>2373</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>2374</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="4" t="s">
+        <v>2374</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>2375</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>2376</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="409.5">
       <c r="A22" s="2" t="s">
+        <v>2376</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>2377</v>
       </c>
-      <c r="B22" s="5" t="s">
+    </row>
+    <row r="23" spans="1:2" ht="255">
+      <c r="A23" s="2" t="s">
         <v>2378</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" ht="246.5">
-      <c r="A23" s="2" t="s">
+      <c r="B23" s="5" t="s">
         <v>2379</v>
       </c>
-      <c r="B23" s="5" t="s">
+    </row>
+    <row r="24" spans="1:2" ht="240">
+      <c r="A24" t="s">
         <v>2380</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" ht="232">
-      <c r="A24" t="s">
+      <c r="B24" s="6" t="s">
         <v>2381</v>
       </c>
-      <c r="B24" s="6" t="s">
+    </row>
+    <row r="25" spans="1:2" ht="270">
+      <c r="A25" t="s">
         <v>2382</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" ht="261">
-      <c r="A25" t="s">
+      <c r="B25" s="6" t="s">
+        <v>2461</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="210">
+      <c r="A26" t="s">
         <v>2383</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>2463</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="203">
-      <c r="A26" t="s">
+      <c r="B26" s="6" t="s">
+        <v>2462</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="61.5" customHeight="1">
+      <c r="A27" s="8" t="s">
         <v>2384</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>2464</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="61.5" customHeight="1">
-      <c r="A27" t="s">
-        <v>2385</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>2386</v>
+      <c r="B27" s="8" t="s">
+        <v>2489</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="105.75" customHeight="1">
@@ -22199,7 +22473,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="174">
+    <row r="29" spans="1:2" ht="180">
       <c r="A29" s="9" t="s">
         <v>2346</v>
       </c>
@@ -22207,332 +22481,412 @@
         <v>2347</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="130.5">
+    <row r="30" spans="1:2" ht="135">
       <c r="A30" s="11" t="s">
+        <v>2385</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>2386</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="180">
+      <c r="A31" s="13" t="s">
         <v>2387</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B31" s="14" t="s">
         <v>2388</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="174">
-      <c r="A31" s="13" t="s">
+    <row r="32" spans="1:2" ht="180">
+      <c r="A32" s="15" t="s">
         <v>2389</v>
       </c>
-      <c r="B31" s="14" t="s">
+      <c r="B32" s="16" t="s">
         <v>2390</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="174">
-      <c r="A32" s="15" t="s">
-        <v>2391</v>
-      </c>
-      <c r="B32" s="16" t="s">
-        <v>2392</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="409.5">
       <c r="A33" s="17" t="s">
+        <v>2391</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>2392</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="409.5">
+      <c r="A34" s="19" t="s">
         <v>2393</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B34" s="20" t="s">
         <v>2394</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="406">
-      <c r="A34" s="19" t="s">
-        <v>2395</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>2396</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="409.5">
       <c r="A35" s="21" t="s">
-        <v>2397</v>
+        <v>2395</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>2398</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="409.5">
       <c r="A36" s="23" t="s">
-        <v>2399</v>
+        <v>2397</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>2400</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="409.5">
       <c r="A37" s="25" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B37" s="26" t="s">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="90">
+      <c r="A38" t="s">
         <v>2401</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B38" s="27" t="s">
+        <v>2466</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="120">
+      <c r="A39" t="s">
         <v>2402</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" ht="87">
-      <c r="A38" t="s">
+      <c r="B39" s="27" t="s">
         <v>2403</v>
       </c>
-      <c r="B38" s="27" t="s">
-        <v>2468</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="116">
-      <c r="A39" t="s">
+    </row>
+    <row r="40" spans="1:2" ht="180">
+      <c r="A40" t="s">
         <v>2404</v>
       </c>
-      <c r="B39" s="27" t="s">
+      <c r="B40" s="27" t="s">
         <v>2405</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="174">
-      <c r="A40" t="s">
+    <row r="41" spans="1:2" ht="195">
+      <c r="A41" t="s">
         <v>2406</v>
       </c>
-      <c r="B40" s="27" t="s">
+      <c r="B41" s="27" t="s">
         <v>2407</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="188.5">
-      <c r="A41" t="s">
+    <row r="42" spans="1:2" ht="120">
+      <c r="A42" t="s">
         <v>2408</v>
       </c>
-      <c r="B41" s="27" t="s">
+      <c r="B42" s="27" t="s">
         <v>2409</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="116">
-      <c r="A42" t="s">
-        <v>2410</v>
-      </c>
-      <c r="B42" s="27" t="s">
-        <v>2411</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="409.5">
       <c r="A43" t="s">
-        <v>2412</v>
+        <v>2410</v>
       </c>
       <c r="B43" s="27" t="s">
-        <v>2465</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="409.5">
       <c r="A44" t="s">
-        <v>2413</v>
+        <v>2411</v>
       </c>
       <c r="B44" s="27" t="s">
-        <v>2466</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="409.5">
       <c r="A45" t="s">
+        <v>2412</v>
+      </c>
+      <c r="B45" s="27" t="s">
+        <v>2465</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="270">
+      <c r="A46" t="s">
+        <v>2413</v>
+      </c>
+      <c r="B46" s="27" t="s">
         <v>2414</v>
-      </c>
-      <c r="B45" s="27" t="s">
-        <v>2467</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="261">
-      <c r="A46" t="s">
-        <v>2415</v>
-      </c>
-      <c r="B46" s="27" t="s">
-        <v>2416</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="409.5">
       <c r="A47" t="s">
+        <v>2415</v>
+      </c>
+      <c r="B47" s="27" t="s">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="345">
+      <c r="A48" t="s">
         <v>2417</v>
       </c>
-      <c r="B47" s="27" t="s">
+      <c r="B48" s="27" t="s">
         <v>2418</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="333.5">
-      <c r="A48" t="s">
+    <row r="49" spans="1:2" ht="345">
+      <c r="A49" t="s">
         <v>2419</v>
       </c>
-      <c r="B48" s="27" t="s">
+      <c r="B49" s="27" t="s">
         <v>2420</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="333.5">
-      <c r="A49" t="s">
-        <v>2421</v>
-      </c>
-      <c r="B49" s="27" t="s">
-        <v>2422</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="36" customHeight="1">
       <c r="A50" t="s">
-        <v>2423</v>
+        <v>2421</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>2424</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="23.25" customHeight="1">
       <c r="A51" t="s">
-        <v>2425</v>
+        <v>2423</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>2426</v>
+        <v>2424</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="27.75" customHeight="1">
       <c r="A52" t="s">
+        <v>2425</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>2426</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="60">
+      <c r="A53" t="s">
         <v>2427</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B53" s="6" t="s">
         <v>2428</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="58">
-      <c r="A53" t="s">
+    <row r="54" spans="1:2" ht="45">
+      <c r="A54" t="s">
         <v>2429</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B54" s="27" t="s">
         <v>2430</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="43.5">
-      <c r="A54" t="s">
+    <row r="55" spans="1:2" ht="60">
+      <c r="A55" t="s">
         <v>2431</v>
       </c>
-      <c r="B54" s="27" t="s">
+      <c r="B55" s="27" t="s">
         <v>2432</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="58">
-      <c r="A55" t="s">
+    <row r="56" spans="1:2" ht="75">
+      <c r="A56" t="s">
         <v>2433</v>
       </c>
-      <c r="B55" s="27" t="s">
+      <c r="B56" s="27" t="s">
         <v>2434</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="72.5">
-      <c r="A56" t="s">
-        <v>2435</v>
-      </c>
-      <c r="B56" s="27" t="s">
-        <v>2436</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="409.5">
       <c r="A57" t="s">
+        <v>2435</v>
+      </c>
+      <c r="B57" s="27" t="s">
+        <v>2436</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="90">
+      <c r="A58" t="s">
         <v>2437</v>
       </c>
-      <c r="B57" s="27" t="s">
+      <c r="B58" s="27" t="s">
         <v>2438</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="87">
-      <c r="A58" t="s">
+    <row r="59" spans="1:2" ht="360">
+      <c r="A59" t="s">
         <v>2439</v>
       </c>
-      <c r="B58" s="27" t="s">
+      <c r="B59" s="27" t="s">
         <v>2440</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="348">
-      <c r="A59" t="s">
+    <row r="60" spans="1:2" ht="75">
+      <c r="A60" t="s">
         <v>2441</v>
       </c>
-      <c r="B59" s="27" t="s">
+      <c r="B60" s="27" t="s">
         <v>2442</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="58">
-      <c r="A60" t="s">
-        <v>2443</v>
-      </c>
-      <c r="B60" s="27" t="s">
-        <v>2444</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="409.5">
       <c r="A61" t="s">
-        <v>2445</v>
+        <v>2443</v>
       </c>
       <c r="B61" s="27" t="s">
-        <v>2368</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="87.75" customHeight="1">
       <c r="A62" t="s">
-        <v>2446</v>
+        <v>2444</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>2447</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="71.25" customHeight="1">
       <c r="A63" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>2449</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="54" customHeight="1">
       <c r="A64" t="s">
-        <v>2408</v>
+        <v>2406</v>
       </c>
       <c r="B64" s="27" t="s">
-        <v>2450</v>
+        <v>2448</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="86.25" customHeight="1">
       <c r="A65" s="27" t="s">
-        <v>2451</v>
+        <v>2449</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>2452</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="86.25" customHeight="1">
       <c r="A66" s="27" t="s">
-        <v>2453</v>
+        <v>2451</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>2454</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="102" customHeight="1">
       <c r="A67" s="27" t="s">
-        <v>2455</v>
+        <v>2453</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>2456</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="89.25" customHeight="1">
       <c r="A68" s="27" t="s">
-        <v>2457</v>
+        <v>2455</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>2458</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="102" customHeight="1">
       <c r="A69" s="27" t="s">
-        <v>2459</v>
+        <v>2457</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>2460</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" ht="43.5">
+        <v>2458</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="45">
       <c r="A70" s="71" t="s">
+        <v>2467</v>
+      </c>
+      <c r="B70" s="27" t="s">
+        <v>2468</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="409.5">
+      <c r="A71" s="72" t="s">
         <v>2469</v>
       </c>
-      <c r="B70" s="27" t="s">
+      <c r="B71" s="6" t="s">
         <v>2470</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="60">
+      <c r="A72" t="s">
+        <v>2471</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>2472</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="30">
+      <c r="A73" t="s">
+        <v>2473</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>2474</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="60">
+      <c r="A74" t="s">
+        <v>2475</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>2476</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" ht="120">
+      <c r="A75" t="s">
+        <v>2477</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>2478</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="60">
+      <c r="A76" t="s">
+        <v>2479</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="45">
+      <c r="A77" t="s">
+        <v>2481</v>
+      </c>
+      <c r="B77" s="27" t="s">
+        <v>2482</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="409.5">
+      <c r="A78" t="s">
+        <v>2483</v>
+      </c>
+      <c r="B78" s="27" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" ht="409.5">
+      <c r="A79" t="s">
+        <v>2485</v>
+      </c>
+      <c r="B79" s="27" t="s">
+        <v>2486</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="45">
+      <c r="A80" s="73" t="s">
+        <v>2487</v>
+      </c>
+      <c r="B80" s="27" t="s">
+        <v>2488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
catalogue functions , catalogue test fixes are updated, Purchase bills Functions , Purchase Test , Purchase Locators are newly added
catalogue functions , catalogue test fixes are updated, Purchase bills Functions , Purchase Test , Purchase Locators are newly added , Db Related Excel Files are Added
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="2520" windowWidth="15300" windowHeight="6540" activeTab="1"/>
@@ -10,8 +10,7 @@
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
+  <calcPr calcId="125725"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3016" uniqueCount="2491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3024" uniqueCount="2498">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -10061,6 +10060,38 @@
    AND term_bu = 'ROAU'
  AND term_term_id = trln_term_id
   AND  term_desc1 = '${SONO}'</t>
+  </si>
+  <si>
+    <t>PurchaseBillsEx</t>
+  </si>
+  <si>
+    <t>SELECT *FROM suplr_doc_ln
+WHERE supln_bu = 'ROAU' 
+AND supln_doc_no = '${PURBIL}'</t>
+  </si>
+  <si>
+    <t>PurchaseBillsHeader</t>
+  </si>
+  <si>
+    <t>SELECT *
+FROM suplr_doc_hd
+WHERE suphd_bu = 'ROAU'
+AND suphd_doc_type = 'SB'
+AND suphd_doc_no = '${PURBIL}'</t>
+  </si>
+  <si>
+    <t>PurchaseBillsLineWise</t>
+  </si>
+  <si>
+    <t>PurchaseBillsDocOrderBy</t>
+  </si>
+  <si>
+    <t>SELECT *
+FROM suplr_doc_ln
+WHERE supln_bu = 'ROAU' 
+AND supln_doc_no = '${PURBIL}'
+AND SUPLN_SEQ_NO = '${PbSeqNo}'
+ORDER BY SUPLN_SEQ_NO</t>
   </si>
 </sst>
 </file>
@@ -22242,10 +22273,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B80"/>
+  <dimension ref="A1:B84"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="35.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -22889,6 +22920,38 @@
         <v>2488</v>
       </c>
     </row>
+    <row r="81" spans="1:2" ht="45">
+      <c r="A81" s="27" t="s">
+        <v>2491</v>
+      </c>
+      <c r="B81" s="27" t="s">
+        <v>2492</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" ht="75">
+      <c r="A82" s="27" t="s">
+        <v>2493</v>
+      </c>
+      <c r="B82" s="27" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="45">
+      <c r="A83" s="27" t="s">
+        <v>2495</v>
+      </c>
+      <c r="B83" s="27" t="s">
+        <v>2492</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" ht="90">
+      <c r="A84" s="27" t="s">
+        <v>2496</v>
+      </c>
+      <c r="B84" s="27" t="s">
+        <v>2497</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Purchase Bill Get Document Function
Purchase Bill Get Document Function
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="2520" windowWidth="15300" windowHeight="6540" activeTab="1"/>
@@ -10,7 +10,7 @@
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="124519"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3024" uniqueCount="2498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3036" uniqueCount="2508">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -10092,6 +10092,116 @@
 AND supln_doc_no = '${PURBIL}'
 AND SUPLN_SEQ_NO = '${PbSeqNo}'
 ORDER BY SUPLN_SEQ_NO</t>
+  </si>
+  <si>
+    <t>PurchaseBillQuery</t>
+  </si>
+  <si>
+    <t>SELECT *
+FROM suplr_doc_hd_hist_vw1
+WHERE suphd_bu = 'ROAU'
+AND suphd_doc_type = 'SB'
+AND suphd_doc_no = '${PBNO}'</t>
+  </si>
+  <si>
+    <t>PBLandedCost</t>
+  </si>
+  <si>
+    <t>SELECT *FROM suplr_doc_ln_hist_vw1
+WHERE supln_bu = 'ROAU'
+AND supln_doc_no = '${PBNO}'
+AND SUPLN_RCT_SEQ_NO ='${SUPSEQNO}'</t>
+  </si>
+  <si>
+    <t>LandedCostQuery</t>
+  </si>
+  <si>
+    <t>select
+PRLC_BU,
+PRLC_RCPT_NO,
+PRLC_SEQ_NO,
+prlc_sub_seq_no,
+PRLC_TC_ID,PRLC_TC_REV,
+(SELECT prod_desc11 FROM products WHERE prod_bu = prlc_bu AND prod_id = prlc_tc_id AND prod_rev = NVL(prlc_tc_rev,0)) PRLC_TC_DESC,
+PRLC_TYPE,
+PRLC_SUPLR_ID,
+(SELECT distinct suplr_name1
+  FROM suppliers
+ WHERE suplr_bu = PRLC_BU 
+   AND suplr_status = 'A'
+    and suplr_suplr_id = PRLC_SUPLR_ID ) PRLC_SUPLR_NAME,
+PRLC_CURRENCY,
+PRLC_HSN_CODE,
+PRLC_ASSBL_VAL,
+PRLC_TC_PCT,
+PRLC_TC_AMT,
+PRLC_STATE_CODE,
+PRLC_IGST_PCT,
+PRLC_IGST_AMT,
+PRLC_CGST_AMT,
+PRLC_SGST_AMT,
+PRLC_CHRG_FLAG,
+PRLC_SEL_FLAG,
+PRLC_PTS_FLAG,
+PRLC_SUPLR_DOC_NO,
+PRLC_SUPLR_DOC_DATE,
+PRLC_EXCHANGE_RATE,
+PRLC_TC_TYPE,
+PRLC_REC_SOURCE,
+PRLC_LC_IMPORT_FLAG,
+PRLC_TAX_SET_FLAG,
+PRLC_TAX_TYPE,
+PRLC_CRE_BY,
+PRLC_CRE_DATE,
+prlc_meis_lic_no,
+prlc_meis_doc_no,
+prlc_pur_acct,
+(SELECT glac_acct_desc1 FROM gl_accts WHERE glac_bu = prlc_bu AND glac_acct = prlc_pur_acct) prlc_pur_acct_desc,
+prlc_offset_acct,
+(SELECT glac_acct_desc1 FROM gl_accts WHERE glac_bu = prlc_bu AND glac_acct = prlc_offset_acct) prlc_offset_acct_desc,
+prlc_cgst_pct,
+prlc_sgst_pct,
+PRLC_DOC_TYPE,
+PRLC_CESS_PCT,
+PRLC_CESS_AMT,
+PRLC_GST_TYPE,
+PRLC_GST_CLF_TYPE,
+prlc_billfr_loc,
+PRLC_GST_EXEMPT_TYPE
+from pur_rcpt_land_costs_view
+where PRLC_BU = 'ROAU'
+  AND prlc_rcpt_no  = '${GRNNO}'
+AND PRLC_SUPLR_ID='${SUPID}'</t>
+  </si>
+  <si>
+    <t>PBHSNLineWiseQuery</t>
+  </si>
+  <si>
+    <t>SELECT *FROM suplr_doc_ln_hist_vw1
+WHERE supln_bu = 'ROAU'
+AND supln_doc_no = '${PBNO}'
+AND SUPLN_PROD_ID='${SUPPBITEMID}'</t>
+  </si>
+  <si>
+    <t>GRNHistQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SELECT 
+ PORLH_TRD_DISC_AMT,
+ PORLH_SPL_DISC_AMT,
+ PORLH_CASH_DISC_AMT,
+PORLH_TRD_ASSBL_VAL,
+PORLH_SPL_ASSBL_VAL,
+PORLH_IGST_AMT,
+PORLH_SGST_AMT,
+PORLH_CGST_AMT,
+PORLH_UTGST_AMT,
+PORLH_CESS_AMT,
+PORLH_CASH_ASSBL_VAL
+  from  pur_ord_receipt_ln_hist
+ WHERE PORLH_BU = 'ROAU'
+ and PORLH_RECEIPT_NO = '${GRNNO}'
+ and PORLH_PROD_ID='${GRNID}'</t>
   </si>
 </sst>
 </file>
@@ -22273,7 +22383,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B84"/>
+  <dimension ref="A1:B90"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.28515625" bestFit="1" customWidth="1"/>
@@ -22952,6 +23062,54 @@
         <v>2497</v>
       </c>
     </row>
+    <row r="85" spans="1:2" ht="45">
+      <c r="A85" s="27" t="s">
+        <v>2487</v>
+      </c>
+      <c r="B85" s="27" t="s">
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" ht="75">
+      <c r="A86" s="27" t="s">
+        <v>2498</v>
+      </c>
+      <c r="B86" s="27" t="s">
+        <v>2499</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" ht="60">
+      <c r="A87" s="27" t="s">
+        <v>2500</v>
+      </c>
+      <c r="B87" s="27" t="s">
+        <v>2501</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" ht="409.5">
+      <c r="A88" s="27" t="s">
+        <v>2502</v>
+      </c>
+      <c r="B88" s="27" t="s">
+        <v>2503</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" ht="60">
+      <c r="A89" s="27" t="s">
+        <v>2504</v>
+      </c>
+      <c r="B89" s="27" t="s">
+        <v>2505</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="240">
+      <c r="A90" t="s">
+        <v>2506</v>
+      </c>
+      <c r="B90" s="27" t="s">
+        <v>2507</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Subcontract Functions And Subcontract Test Changes Fixes
Subcontract Functions And Subcontract Test Changes Fixes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3052" uniqueCount="2520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3054" uniqueCount="2522">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -10262,6 +10262,184 @@
 WHERE supln_bu = 'ROAU'
 AND supln_doc_no = '${PBNO}'
 AND SUPLN_SEQ_NO = '${SEQNO}'</t>
+  </si>
+  <si>
+    <t>SCOGRNLineQuery</t>
+  </si>
+  <si>
+    <t>SELECT porh_bu,
+       porh_plnt,
+        PORH_PLNT_LOC_ID,
+       PORH_PLNT_LOC_NAME Location,
+       bup_name1 porh_plnt_desc,
+       func_find_sub_vou_type_desc(porh_bu,porh_type) "Type",
+       TO_CHAR(porh_receipt_date,'MON-YY') Month,
+       porh_type,
+       (SELECT DISTINCT apst_sub_type_desc
+                  FROM appl_vou_sub_types
+ WHERE apst_bu = porh_bu
+   AND apst_vou_type = 'GRNS'
+   and apst_sub_type = porh_type) Type_Desc,
+       porh_receipt_pfx,
+         porh_receipt_no ,
+      porh_receipt_date, porh_receipt_date,
+       porh_suplr_id,
+       suplr_name1 porh_suplr_name,
+       porh_suplr_doc_no porh_bill_no,
+       porh_suplr_doc_date porh_bill_date,
+       porh_dc_no,
+       porh_dc_date  porh_dc_date,
+       porl_seq_no,
+        1 porl_prod_id,
+       porl_prod_id v,
+       porl_prod_rev,
+       porl_prod_desc1,
+       porl_suplr_uom,
+       PORL_DRAWING_REV,
+       PORL_DRAWING_NO ,    
+       porl_prod_uom,
+       CASE WHEN porl_po_pfx IS NOT NULL THEN porl_po_pfx||'/'||porl_po_no||'/'||porl_po_seq_no
+            WHEN porl_ss_doc_pfx IS NOT NULL THEN porl_ss_doc_pfx||'/'||porl_ss_doc_no||'/'||porl_ss_seq_no
+       END porl_po_ss_no,
+       porh_currency,
+       porh_exchange_rate,
+       porl_so_schld_desc,
+       porl_hsn_code,
+       porl_receipt_qty,
+       porl_accepted_qty,
+       porl_aod_qty,
+       porl_rejected_qty,
+       porl_stock_receipt_qty,
+       porl_stk_accepted_qty,
+       porl_stk_aod_qty,
+       porl_stk_rejected_qty,
+       porl_sc_unit_cost,
+       porl_disc_pct,
+       porl_gross_amt porl_gross_amt_tc,
+       porl_disc_amt porl_disc_amt_tc,
+       porl_tax_amt porl_tax_amt_tc,
+       porl_net_amt porl_net_amt_tc,
+       porl_gross_amt*porh_exchange_rate porl_gross_amt_bc,
+       porl_disc_amt*porh_exchange_rate porl_disc_amt_bc,
+       porl_tax_amt*porh_exchange_rate porl_tax_amt_bc,
+       porl_net_amt*porh_exchange_rate porl_net_amt_bc,
+       (porl_gross_amt-porl_disc_amt) Net_Pur_Amt_TC,
+       (porl_sc_unit_cost*porl_disc_pct)/100 Net_unit_price,
+       ((porl_gross_amt-porl_disc_amt)*porh_exchange_rate) net_pur_amt_bc,
+       porl_sf_code,
+       porl_tar_sf_code,
+       porl_prod_ord_no,
+       porh_billfr_loc_name,
+       pra_billfr_gst_no,
+       pra_billfr_state_code,
+       CASE WHEN porh_gst_type = 'R' THEN 'Registered'
+            WHEN porh_gst_type = 'U' THEN 'Unregistered'
+            WHEN porh_gst_type = 'C' THEN 'Composition'
+            ELSE porh_gst_type
+       END porh_gst_type,
+       CASE WHEN porh_gst_clf_type = 'L' THEN 'Local'
+            WHEN porh_gst_clf_type = 'I' THEN 'Inter-State'
+            WHEN porh_gst_clf_type = 'U' THEN 'Union Territory'
+            WHEN porh_gst_clf_type = 'M' THEN 'Import'
+            WHEN porh_gst_clf_type = 'S' THEN 'SEZ-Unit'
+            WHEN porh_gst_clf_type = 'D' THEN 'SEZ-Developer'
+            ELSE porh_gst_clf_type
+       END porh_gst_clf_type,
+       CASE WHEN porl_gst_input_type = 'I' THEN 'Inputs'
+            WHEN porl_gst_input_type = 'M' THEN 'Import'
+            WHEN porl_gst_input_type = 'C' THEN 'Capital Goods'
+            WHEN porl_gst_input_type = 'S' THEN 'Input Services'
+            WHEN porl_gst_input_type = 'N' THEN 'Ineligible'
+            WHEN porl_gst_input_type = 'A' THEN 'NA'
+            ELSE porl_gst_input_type
+       END porl_gst_input_type,
+       CASE WHEN porl_gst_exempt_flag = 'G' THEN 'GST Supply'
+            WHEN porl_gst_exempt_flag = 'R' THEN 'NIL Rated'
+            WHEN porl_gst_exempt_flag = 'Y' THEN 'Exempted'
+            WHEN porl_gst_exempt_flag = 'N' THEN 'Non-GST Supply'
+            WHEN porl_gst_exempt_flag = 'A' THEN 'NA'
+            ELSE porl_gst_exempt_flag
+       END porl_gst_exempt_flag,
+       porl_storage_store_id,
+       porl_storage_store_name,
+       porl_buyer_id,
+       (SELECT emp_first_name1 FROM buyers,employees WHERE emP_BU = buyer_bu AND emp_emp_id = buyer_emp_id AND buyer_bu = porl_bu AND buyer_id = porl_buyer_id) porl_buyer_name,
+       porh_shipvia_id,
+       (SELECT sv_desc1 FROM ship_vias WHERE sv_bu = porh_bu AND sv_shipvia_id = porh_shipvia_id) porh_shipvia_desc,
+       porh_price_term,
+       (SELECT fob_desc1 FROM fobs WHERE fob_bu = porh_bu AND fob_fob_id = porh_price_term) porh_price_term_desc,
+       porh_term_id,
+       (SELECT term_desc1 FROM terms_hd WHERE term_bu = porh_bu AND term_term_id = porh_term_id) porh_term_desc,
+       (porl_required_date) porl_required_date,
+       (porl_promise_date) porl_promise_date,
+       porh_terr_id,
+       (SELECT st_terr_desc FROM suplr_terr WHERE st_bu = porh_bu AND st_terr_id = porh_terr_id) porh_terr_desc,
+       NULL porl_suplr_item,
+       NULL porl_suplr_item_desc,
+       suplr_group_id porh_suplr_grp,
+      (SELECT supgrp_desc1 FROM supplier_groups WHERE supgrp_BU = porh_bu AND supgrp_group_id = suplr_group_id) porh_suplr_grp_desc,
+       suplr_subgroup porh_suplr_subgrp,
+      (SELECT supsubgroup_desc1 FROM supplier_subgroup WHERE supsubgroup_BU = porh_bu AND supsubgroup_type_id = suplr_subgroup) porh_suplr_subgrp_desc,
+       porl_prod_grp,
+       porl_prod_grp_desc,
+       porl_prod_subgrp,
+       porl_prod_subgrp_desc,
+       porl_cls_id,
+       porl_prod_cls_desc,
+       porl_sub_cls_id,
+       porl_prod_subcls_desc,
+       CASE WHEN porl_status = 'N' THEN 'Draft'
+            WHEN porl_status = 'Q' THEN 'QC Completed'
+            WHEN porl_status = 'P' THEN 'Partial Received'
+            WHEN porl_status = 'R' THEN 'Received'
+            WHEN porl_status = 'C' THEN 'Cancelled'
+       END porl_status,
+       porh_wf_status,
+       decode(porh_wf_status,'N','Draft','A','Approved','E','Entry Completed','C','Cancelled') wf_status,
+       porl_proj_lvl_id,
+       porl_proj_lvl_desc,
+       PORH_APPR_BY,
+       PORH_APPR_EMP_ID,
+       PORH_APPR_IP_ADDR,
+       PORH_APPR_OS_USER,
+       PORH_APPR_DATE,
+       (PORH_GRN_DATE-porl_required_date) RD_Delay,
+       (PORH_GRN_DATE-porl_promise_date)  PD_Delay,
+       (SELECT DISTINCT cntry_name1 FROM countries WHERE cntry_bu  =suplr_bu AND cntry_id = SUPLR_COUNTRY) Country ,
+       PROD_MDS_NO,
+       PROD_MDS_REV,
+       PROD_DRAWING_NO,
+       PROD_DRG_REV,
+       PORH_CRE_BY,
+       PORH_CRE_IP_ADDR,
+       PORH_CRE_OS_USER,
+       PORH_CRE_DATE,
+       PORH_CRE_EMP_ID,
+       PORL_TEMP_INV_QTY,
+       PORL_INV_QTY,
+       porl_contr_pfx,
+       porl_contr_no  porl_open_sc_no,
+       PORL_PO_PFX,
+       PORL_PO_NO,
+       PORL_PO_SEQ_NO,
+       PORL_PO_DATE,
+      (NVL((TRUNC(porh_receipt_date) - TRUNC(porl_ge_doc_date)),0)) age_days
+  FROM pur_ord_receipt_hd_view,pur_ord_receipt_ln_view, pur_rcpt_addr_vw, suppliers,bus_unit_plants,products
+ WHERE porh_bu = porl_bu
+   AND porl_bu = prod_BU
+   AND porh_receipt_no = porl_receipt_no
+   AND bup_bu = porh_bu
+   AND bup_plant_id = porh_plnt
+   AND suplr_bu = porh_bu
+   AND suplr_suplr_id = porh_suplr_id
+   AND pra_bu(+) = porh_bu
+   AND pra_rcpt_no(+) = porh_receipt_no
+   AND porl_prod_id = prod_id
+   AND porl_prod_rev = prod_rev
+   AND porh_mode = 'SC'
+   AND porh_bu = 'ROAU'
+   AND porh_receipt_no = '${GRNSNO}'   
+ order by porh_cre_date desc</t>
   </si>
 </sst>
 </file>
@@ -22453,7 +22631,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B98"/>
+  <dimension ref="A1:B99"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.28515625" bestFit="1" customWidth="1"/>
@@ -23244,6 +23422,14 @@
         <v>2519</v>
       </c>
     </row>
+    <row r="99" spans="1:2" ht="101.25" customHeight="1">
+      <c r="A99" t="s">
+        <v>2520</v>
+      </c>
+      <c r="B99" s="27" t="s">
+        <v>2521</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Purchase Bill New Scenarios And Purchase Order Functions DB Validations
Purchase Bill New Scenarios And Purchase Order Functions DB Validations
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3056" uniqueCount="2524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3058" uniqueCount="2526">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -10515,6 +10515,39 @@
  AND porl_receipt_no = scrp_rcpt_no 
     and SCRP_RCPT_NO  = '${GRNSNO}' 
      AND SCRP_BU = 'ROAU'</t>
+  </si>
+  <si>
+    <t>POHeaderQuery</t>
+  </si>
+  <si>
+    <t>SELECT POH_PLNT_LOC_ID,
+POH_ORDER_PFX,
+POH_ORDER_NO,
+POH_TYPE,
+POH_SUPLR_ID,
+POH_SUPLR_NAME,
+POH_CURRENCY,
+POH_EXCHANGE_RATE,
+POH_MAT_AMT,
+POH_TAX_AMT,
+POH_TOTAL_AMT,
+ (SELECT DISTINCT apst_sub_type_desc
+          FROM appl_vou_sub_types
+         WHERE     apst_bu = poh_bu
+               AND apst_vou_type = 'PO'
+               AND apst_sub_type = poh_type)type1,
+                      DECODE (poh_status,
+               'E', 'Draft',
+               'A', 'Approved',
+               'N', 'Entry Completed',
+               'C', 'Cancelled',
+               'L', 'Closeshorted',
+               poh_status)
+          poh_status1
+        FROM pur_order_hd_vw
+    WHERE poh_bu = 'ROAU'
+       AND poh_mode = 'PO'     
+             AND poh_order_no ='${PONO}'</t>
   </si>
 </sst>
 </file>
@@ -22706,7 +22739,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B100"/>
+  <dimension ref="A1:B101"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.28515625" bestFit="1" customWidth="1"/>
@@ -23513,6 +23546,14 @@
         <v>2523</v>
       </c>
     </row>
+    <row r="101" spans="1:2" ht="409.5">
+      <c r="A101" t="s">
+        <v>2524</v>
+      </c>
+      <c r="B101" s="27" t="s">
+        <v>2525</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixes For The Sales Order Amendment Multi Closeshort
Fixes For The Sales Order Amendment Multi Closeshort
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -11,6 +11,7 @@
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -7451,24 +7452,6 @@
   </si>
   <si>
     <t>AdvanceReceiptQuery</t>
-  </si>
-  <si>
-    <t>SELECT
-        pard_doc_no Doc_no,
-        pard_plnt Unit,
-        pard_ord_pfx ord_pfx,
-        pard_ord_no ord_no,
-        pard_party_id Party_id,
-        pard_prop_adv_pct Adv_Percentage,
-        pard_prop_adv_amt Adv_Amt,
-        pard_curcy_id Curcy,
-        pard_ord_amt Ord_amt,
-        pard_rct_inprog_amt Rcpt_inprog_amt,
-        pard_rct_amt Rcpt_Amt,
-        pard_close_amt Closed_amt
-   FROM prop_adv_rct_doc
-  WHERE pard_bu = 'ROAU'
-    AND pard_doc_no ='${SONO}'</t>
   </si>
   <si>
     <t>Stock Query1</t>
@@ -10682,6 +10665,24 @@
   </si>
   <si>
     <t>SCOAmendmentLineQuery</t>
+  </si>
+  <si>
+    <t>SELECT
+        pard_doc_no Doc_no,
+        pard_plnt Unit,
+        pard_ord_pfx ord_pfx,
+        pard_ord_no ord_no,
+        pard_party_id Party_id,
+        pard_prop_adv_pct Adv_Percentage,
+        pard_prop_adv_amt Adv_Amt,
+        pard_curcy_id Curcy,
+        pard_ord_amt Ord_amt,
+        pard_rct_inprog_amt Rcpt_inprog_amt,
+        pard_rct_amt Rcpt_Amt,
+        pard_close_amt Closed_amt
+   FROM prop_adv_rct_doc
+  WHERE pard_bu = 'ROAU'
+    AND pard_ord_no = '${SONO}'</t>
   </si>
 </sst>
 </file>
@@ -22925,7 +22926,7 @@
         <v>2346</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1">
@@ -22973,7 +22974,7 @@
         <v>2358</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>2490</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="28.5" customHeight="1">
@@ -22981,119 +22982,119 @@
         <v>2359</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>2360</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>2361</v>
+        <v>2360</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>2460</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="36" customHeight="1">
       <c r="A15" s="2" t="s">
+        <v>2361</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>2362</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>2363</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="45" customHeight="1">
       <c r="A16" s="2" t="s">
+        <v>2363</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>2364</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>2365</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="43.5" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>2365</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>2366</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>2367</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="42" customHeight="1">
       <c r="A18" s="2" t="s">
+        <v>2367</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>2368</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>2369</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="52.5" customHeight="1">
       <c r="A19" s="2" t="s">
+        <v>2369</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>2370</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>2371</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="17.25" customHeight="1">
       <c r="A20" s="4" t="s">
+        <v>2371</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>2372</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>2373</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="4" t="s">
+        <v>2373</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>2374</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>2375</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="409.5">
       <c r="A22" s="2" t="s">
+        <v>2375</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>2376</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>2377</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="255">
       <c r="A23" s="2" t="s">
+        <v>2377</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>2378</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>2379</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="240">
       <c r="A24" t="s">
+        <v>2379</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>2380</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>2381</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="270">
       <c r="A25" t="s">
-        <v>2382</v>
+        <v>2381</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="210">
       <c r="A26" t="s">
-        <v>2383</v>
+        <v>2382</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="61.5" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>2384</v>
+        <v>2383</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>2489</v>
+        <v>2488</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="105.75" customHeight="1">
@@ -23114,594 +23115,594 @@
     </row>
     <row r="30" spans="1:2" ht="135">
       <c r="A30" s="11" t="s">
+        <v>2384</v>
+      </c>
+      <c r="B30" s="12" t="s">
         <v>2385</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>2386</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="180">
       <c r="A31" s="13" t="s">
+        <v>2386</v>
+      </c>
+      <c r="B31" s="14" t="s">
         <v>2387</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>2388</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="180">
       <c r="A32" s="15" t="s">
+        <v>2388</v>
+      </c>
+      <c r="B32" s="16" t="s">
         <v>2389</v>
-      </c>
-      <c r="B32" s="16" t="s">
-        <v>2390</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="409.5">
       <c r="A33" s="17" t="s">
+        <v>2390</v>
+      </c>
+      <c r="B33" s="18" t="s">
         <v>2391</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>2392</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="409.5">
       <c r="A34" s="19" t="s">
+        <v>2392</v>
+      </c>
+      <c r="B34" s="20" t="s">
         <v>2393</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>2394</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="409.5">
       <c r="A35" s="21" t="s">
+        <v>2394</v>
+      </c>
+      <c r="B35" s="22" t="s">
         <v>2395</v>
-      </c>
-      <c r="B35" s="22" t="s">
-        <v>2396</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="409.5">
       <c r="A36" s="23" t="s">
+        <v>2396</v>
+      </c>
+      <c r="B36" s="24" t="s">
         <v>2397</v>
-      </c>
-      <c r="B36" s="24" t="s">
-        <v>2398</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="409.5">
       <c r="A37" s="25" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B37" s="26" t="s">
         <v>2399</v>
-      </c>
-      <c r="B37" s="26" t="s">
-        <v>2400</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="90">
       <c r="A38" t="s">
-        <v>2401</v>
+        <v>2400</v>
       </c>
       <c r="B38" s="27" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="120">
       <c r="A39" t="s">
+        <v>2401</v>
+      </c>
+      <c r="B39" s="27" t="s">
         <v>2402</v>
-      </c>
-      <c r="B39" s="27" t="s">
-        <v>2403</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="180">
       <c r="A40" t="s">
+        <v>2403</v>
+      </c>
+      <c r="B40" s="27" t="s">
         <v>2404</v>
-      </c>
-      <c r="B40" s="27" t="s">
-        <v>2405</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="195">
       <c r="A41" t="s">
+        <v>2405</v>
+      </c>
+      <c r="B41" s="27" t="s">
         <v>2406</v>
-      </c>
-      <c r="B41" s="27" t="s">
-        <v>2407</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="120">
       <c r="A42" t="s">
+        <v>2407</v>
+      </c>
+      <c r="B42" s="27" t="s">
         <v>2408</v>
-      </c>
-      <c r="B42" s="27" t="s">
-        <v>2409</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="409.5">
       <c r="A43" t="s">
-        <v>2410</v>
+        <v>2409</v>
       </c>
       <c r="B43" s="27" t="s">
-        <v>2463</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="409.5">
       <c r="A44" t="s">
-        <v>2411</v>
+        <v>2410</v>
       </c>
       <c r="B44" s="27" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="409.5">
       <c r="A45" t="s">
-        <v>2412</v>
+        <v>2411</v>
       </c>
       <c r="B45" s="27" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="270">
       <c r="A46" t="s">
+        <v>2412</v>
+      </c>
+      <c r="B46" s="27" t="s">
         <v>2413</v>
-      </c>
-      <c r="B46" s="27" t="s">
-        <v>2414</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="409.5">
       <c r="A47" t="s">
+        <v>2414</v>
+      </c>
+      <c r="B47" s="27" t="s">
         <v>2415</v>
-      </c>
-      <c r="B47" s="27" t="s">
-        <v>2416</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="345">
       <c r="A48" t="s">
+        <v>2416</v>
+      </c>
+      <c r="B48" s="27" t="s">
         <v>2417</v>
-      </c>
-      <c r="B48" s="27" t="s">
-        <v>2418</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="345">
       <c r="A49" t="s">
+        <v>2418</v>
+      </c>
+      <c r="B49" s="27" t="s">
         <v>2419</v>
-      </c>
-      <c r="B49" s="27" t="s">
-        <v>2420</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="36" customHeight="1">
       <c r="A50" t="s">
+        <v>2420</v>
+      </c>
+      <c r="B50" s="6" t="s">
         <v>2421</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>2422</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="23.25" customHeight="1">
       <c r="A51" t="s">
+        <v>2422</v>
+      </c>
+      <c r="B51" s="6" t="s">
         <v>2423</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>2424</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="27.75" customHeight="1">
       <c r="A52" t="s">
+        <v>2424</v>
+      </c>
+      <c r="B52" s="6" t="s">
         <v>2425</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>2426</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="60">
       <c r="A53" t="s">
+        <v>2426</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>2427</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>2428</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="45">
       <c r="A54" t="s">
+        <v>2428</v>
+      </c>
+      <c r="B54" s="27" t="s">
         <v>2429</v>
-      </c>
-      <c r="B54" s="27" t="s">
-        <v>2430</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="60">
       <c r="A55" t="s">
+        <v>2430</v>
+      </c>
+      <c r="B55" s="27" t="s">
         <v>2431</v>
-      </c>
-      <c r="B55" s="27" t="s">
-        <v>2432</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="75">
       <c r="A56" t="s">
+        <v>2432</v>
+      </c>
+      <c r="B56" s="27" t="s">
         <v>2433</v>
-      </c>
-      <c r="B56" s="27" t="s">
-        <v>2434</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="409.5">
       <c r="A57" t="s">
+        <v>2434</v>
+      </c>
+      <c r="B57" s="27" t="s">
         <v>2435</v>
-      </c>
-      <c r="B57" s="27" t="s">
-        <v>2436</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="90">
       <c r="A58" t="s">
+        <v>2436</v>
+      </c>
+      <c r="B58" s="27" t="s">
         <v>2437</v>
-      </c>
-      <c r="B58" s="27" t="s">
-        <v>2438</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="360">
       <c r="A59" t="s">
+        <v>2438</v>
+      </c>
+      <c r="B59" s="27" t="s">
         <v>2439</v>
-      </c>
-      <c r="B59" s="27" t="s">
-        <v>2440</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="75">
       <c r="A60" t="s">
+        <v>2440</v>
+      </c>
+      <c r="B60" s="27" t="s">
         <v>2441</v>
-      </c>
-      <c r="B60" s="27" t="s">
-        <v>2442</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="409.5">
       <c r="A61" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="B61" s="27" t="s">
-        <v>2367</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="87.75" customHeight="1">
       <c r="A62" t="s">
+        <v>2443</v>
+      </c>
+      <c r="B62" s="6" t="s">
         <v>2444</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>2445</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="71.25" customHeight="1">
       <c r="A63" t="s">
+        <v>2445</v>
+      </c>
+      <c r="B63" s="6" t="s">
         <v>2446</v>
-      </c>
-      <c r="B63" s="6" t="s">
-        <v>2447</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="54" customHeight="1">
       <c r="A64" t="s">
-        <v>2406</v>
+        <v>2405</v>
       </c>
       <c r="B64" s="27" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="86.25" customHeight="1">
       <c r="A65" s="27" t="s">
+        <v>2448</v>
+      </c>
+      <c r="B65" s="6" t="s">
         <v>2449</v>
-      </c>
-      <c r="B65" s="6" t="s">
-        <v>2450</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="86.25" customHeight="1">
       <c r="A66" s="27" t="s">
+        <v>2450</v>
+      </c>
+      <c r="B66" s="6" t="s">
         <v>2451</v>
-      </c>
-      <c r="B66" s="6" t="s">
-        <v>2452</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="102" customHeight="1">
       <c r="A67" s="27" t="s">
+        <v>2452</v>
+      </c>
+      <c r="B67" s="6" t="s">
         <v>2453</v>
-      </c>
-      <c r="B67" s="6" t="s">
-        <v>2454</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="89.25" customHeight="1">
       <c r="A68" s="27" t="s">
+        <v>2454</v>
+      </c>
+      <c r="B68" s="6" t="s">
         <v>2455</v>
-      </c>
-      <c r="B68" s="6" t="s">
-        <v>2456</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="102" customHeight="1">
       <c r="A69" s="27" t="s">
+        <v>2456</v>
+      </c>
+      <c r="B69" s="6" t="s">
         <v>2457</v>
-      </c>
-      <c r="B69" s="6" t="s">
-        <v>2458</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="45">
       <c r="A70" s="71" t="s">
+        <v>2466</v>
+      </c>
+      <c r="B70" s="27" t="s">
         <v>2467</v>
-      </c>
-      <c r="B70" s="27" t="s">
-        <v>2468</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="409.5">
       <c r="A71" s="72" t="s">
+        <v>2468</v>
+      </c>
+      <c r="B71" s="6" t="s">
         <v>2469</v>
-      </c>
-      <c r="B71" s="6" t="s">
-        <v>2470</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="60">
       <c r="A72" t="s">
+        <v>2470</v>
+      </c>
+      <c r="B72" s="6" t="s">
         <v>2471</v>
-      </c>
-      <c r="B72" s="6" t="s">
-        <v>2472</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="30">
       <c r="A73" t="s">
+        <v>2472</v>
+      </c>
+      <c r="B73" s="6" t="s">
         <v>2473</v>
-      </c>
-      <c r="B73" s="6" t="s">
-        <v>2474</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="60">
       <c r="A74" t="s">
+        <v>2474</v>
+      </c>
+      <c r="B74" s="6" t="s">
         <v>2475</v>
-      </c>
-      <c r="B74" s="6" t="s">
-        <v>2476</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="120">
       <c r="A75" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B75" s="6" t="s">
         <v>2477</v>
-      </c>
-      <c r="B75" s="6" t="s">
-        <v>2478</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="60">
       <c r="A76" t="s">
+        <v>2478</v>
+      </c>
+      <c r="B76" s="6" t="s">
         <v>2479</v>
-      </c>
-      <c r="B76" s="6" t="s">
-        <v>2480</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="45">
       <c r="A77" t="s">
+        <v>2480</v>
+      </c>
+      <c r="B77" s="27" t="s">
         <v>2481</v>
-      </c>
-      <c r="B77" s="27" t="s">
-        <v>2482</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="409.5">
       <c r="A78" t="s">
+        <v>2482</v>
+      </c>
+      <c r="B78" s="27" t="s">
         <v>2483</v>
-      </c>
-      <c r="B78" s="27" t="s">
-        <v>2484</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="409.5">
       <c r="A79" t="s">
+        <v>2484</v>
+      </c>
+      <c r="B79" s="27" t="s">
         <v>2485</v>
-      </c>
-      <c r="B79" s="27" t="s">
-        <v>2486</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="45">
       <c r="A80" s="73" t="s">
+        <v>2486</v>
+      </c>
+      <c r="B80" s="27" t="s">
         <v>2487</v>
-      </c>
-      <c r="B80" s="27" t="s">
-        <v>2488</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="45">
       <c r="A81" s="27" t="s">
+        <v>2490</v>
+      </c>
+      <c r="B81" s="27" t="s">
         <v>2491</v>
-      </c>
-      <c r="B81" s="27" t="s">
-        <v>2492</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="75">
       <c r="A82" s="27" t="s">
+        <v>2492</v>
+      </c>
+      <c r="B82" s="27" t="s">
         <v>2493</v>
-      </c>
-      <c r="B82" s="27" t="s">
-        <v>2494</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="45">
       <c r="A83" s="27" t="s">
-        <v>2495</v>
+        <v>2494</v>
       </c>
       <c r="B83" s="27" t="s">
-        <v>2492</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="90">
       <c r="A84" s="27" t="s">
+        <v>2495</v>
+      </c>
+      <c r="B84" s="27" t="s">
         <v>2496</v>
-      </c>
-      <c r="B84" s="27" t="s">
-        <v>2497</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="45">
       <c r="A85" s="27" t="s">
+        <v>2486</v>
+      </c>
+      <c r="B85" s="27" t="s">
         <v>2487</v>
-      </c>
-      <c r="B85" s="27" t="s">
-        <v>2488</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="75">
       <c r="A86" s="27" t="s">
+        <v>2497</v>
+      </c>
+      <c r="B86" s="27" t="s">
         <v>2498</v>
-      </c>
-      <c r="B86" s="27" t="s">
-        <v>2499</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="60">
       <c r="A87" s="27" t="s">
+        <v>2499</v>
+      </c>
+      <c r="B87" s="27" t="s">
         <v>2500</v>
-      </c>
-      <c r="B87" s="27" t="s">
-        <v>2501</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="409.5">
       <c r="A88" s="27" t="s">
+        <v>2501</v>
+      </c>
+      <c r="B88" s="27" t="s">
         <v>2502</v>
-      </c>
-      <c r="B88" s="27" t="s">
-        <v>2503</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="60">
       <c r="A89" s="27" t="s">
+        <v>2503</v>
+      </c>
+      <c r="B89" s="27" t="s">
         <v>2504</v>
-      </c>
-      <c r="B89" s="27" t="s">
-        <v>2505</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="240">
       <c r="A90" t="s">
+        <v>2505</v>
+      </c>
+      <c r="B90" s="27" t="s">
         <v>2506</v>
-      </c>
-      <c r="B90" s="27" t="s">
-        <v>2507</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="75">
       <c r="A91" t="s">
+        <v>2497</v>
+      </c>
+      <c r="B91" s="27" t="s">
         <v>2498</v>
-      </c>
-      <c r="B91" s="27" t="s">
-        <v>2499</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="45">
       <c r="A92" t="s">
+        <v>2486</v>
+      </c>
+      <c r="B92" s="27" t="s">
         <v>2487</v>
-      </c>
-      <c r="B92" s="27" t="s">
-        <v>2488</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="105">
       <c r="A93" t="s">
+        <v>2507</v>
+      </c>
+      <c r="B93" s="27" t="s">
         <v>2508</v>
-      </c>
-      <c r="B93" s="27" t="s">
-        <v>2509</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="120">
       <c r="A94" t="s">
+        <v>2509</v>
+      </c>
+      <c r="B94" s="27" t="s">
         <v>2510</v>
-      </c>
-      <c r="B94" s="27" t="s">
-        <v>2511</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="60">
       <c r="A95" t="s">
+        <v>2511</v>
+      </c>
+      <c r="B95" s="27" t="s">
         <v>2512</v>
-      </c>
-      <c r="B95" s="27" t="s">
-        <v>2513</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="60">
       <c r="A96" t="s">
+        <v>2513</v>
+      </c>
+      <c r="B96" s="27" t="s">
         <v>2514</v>
-      </c>
-      <c r="B96" s="27" t="s">
-        <v>2515</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="75">
       <c r="A97" t="s">
+        <v>2515</v>
+      </c>
+      <c r="B97" s="27" t="s">
         <v>2516</v>
-      </c>
-      <c r="B97" s="27" t="s">
-        <v>2517</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="60">
       <c r="A98" t="s">
+        <v>2517</v>
+      </c>
+      <c r="B98" s="74" t="s">
         <v>2518</v>
-      </c>
-      <c r="B98" s="74" t="s">
-        <v>2519</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="101.25" customHeight="1">
       <c r="A99" t="s">
+        <v>2519</v>
+      </c>
+      <c r="B99" s="27" t="s">
         <v>2520</v>
-      </c>
-      <c r="B99" s="27" t="s">
-        <v>2521</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="85.5" customHeight="1">
       <c r="A100" t="s">
+        <v>2521</v>
+      </c>
+      <c r="B100" s="27" t="s">
         <v>2522</v>
-      </c>
-      <c r="B100" s="27" t="s">
-        <v>2523</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="409.5">
       <c r="A101" t="s">
+        <v>2523</v>
+      </c>
+      <c r="B101" s="27" t="s">
         <v>2524</v>
-      </c>
-      <c r="B101" s="27" t="s">
-        <v>2525</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="120.75" customHeight="1">
       <c r="A102" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
       <c r="B102" s="27" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="159.75" customHeight="1">
       <c r="A103" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
       <c r="B103" s="27" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated The Journal Part Validation For The Bank Receipt Scenarios
Updated The Journal Part Validation For The Bank Receipt Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -11,7 +11,6 @@
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3062" uniqueCount="2530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3066" uniqueCount="2534">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -10683,6 +10682,25 @@
    FROM prop_adv_rct_doc
   WHERE pard_bu = 'ROAU'
     AND pard_ord_no = '${SONO}'</t>
+  </si>
+  <si>
+    <t>BankReceipPendingAdvanceQuery</t>
+  </si>
+  <si>
+    <t>SELECT *
+  FROM adv_rcpt_doc_vw
+ WHERE PARD_BU = 'ROAU'
+ AND PARD_DOC_NO = '${SONO}'</t>
+  </si>
+  <si>
+    <t>JournalQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  SELECT *
+FROM APPL_JRNL_VW 
+ WHERE AJ_BU = 'ROAU'
+  AND AJ_VOU_NO ='${SONO}'
+  AND SEQ_NO = '${PONO}'</t>
   </si>
 </sst>
 </file>
@@ -22874,7 +22892,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B103"/>
+  <dimension ref="A1:B105"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.28515625" bestFit="1" customWidth="1"/>
@@ -23705,6 +23723,22 @@
         <v>2526</v>
       </c>
     </row>
+    <row r="104" spans="1:2" ht="60">
+      <c r="A104" t="s">
+        <v>2530</v>
+      </c>
+      <c r="B104" s="27" t="s">
+        <v>2531</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="75">
+      <c r="A105" t="s">
+        <v>2532</v>
+      </c>
+      <c r="B105" s="27" t="s">
+        <v>2533</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Locator Fixes For The Sales And Customer Schedule Screens
Locator Fixes For The Sales And Customer Schedule Screens
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21600" windowHeight="9600" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15300" windowHeight="6540" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -10881,14 +10882,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
-  <fonts count="26">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -10935,151 +10930,14 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -11104,188 +10962,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -11321,268 +10999,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="66">
+  <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -11600,44 +11036,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="53"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -11673,15 +11109,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -11701,11 +11137,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -11719,19 +11155,19 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="59" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="60" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -11746,74 +11182,27 @@
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="66">
+  <cellStyles count="18">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 10" xfId="49"/>
-    <cellStyle name="Normal 11" xfId="50"/>
-    <cellStyle name="Normal 13" xfId="51"/>
-    <cellStyle name="Normal 14" xfId="52"/>
-    <cellStyle name="Normal 15" xfId="53"/>
-    <cellStyle name="Normal 16" xfId="54"/>
-    <cellStyle name="Normal 17" xfId="55"/>
-    <cellStyle name="Normal 18" xfId="56"/>
-    <cellStyle name="Normal 19" xfId="57"/>
-    <cellStyle name="Normal 2" xfId="58"/>
-    <cellStyle name="Normal 2 2" xfId="59"/>
-    <cellStyle name="Normal 2 3" xfId="60"/>
-    <cellStyle name="Normal 20" xfId="61"/>
-    <cellStyle name="Normal 3" xfId="62"/>
-    <cellStyle name="Normal 7" xfId="63"/>
-    <cellStyle name="Normal 8" xfId="64"/>
-    <cellStyle name="Normal 9" xfId="65"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Normal 11" xfId="2"/>
+    <cellStyle name="Normal 13" xfId="3"/>
+    <cellStyle name="Normal 14" xfId="4"/>
+    <cellStyle name="Normal 15" xfId="5"/>
+    <cellStyle name="Normal 16" xfId="6"/>
+    <cellStyle name="Normal 17" xfId="7"/>
+    <cellStyle name="Normal 18" xfId="8"/>
+    <cellStyle name="Normal 19" xfId="9"/>
+    <cellStyle name="Normal 2" xfId="10"/>
+    <cellStyle name="Normal 2 2" xfId="11"/>
+    <cellStyle name="Normal 2 3" xfId="12"/>
+    <cellStyle name="Normal 20" xfId="13"/>
+    <cellStyle name="Normal 3" xfId="14"/>
+    <cellStyle name="Normal 7" xfId="15"/>
+    <cellStyle name="Normal 8" xfId="16"/>
+    <cellStyle name="Normal 9" xfId="17"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -12075,17 +11464,17 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B1445"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="62.7142857142857" style="31" customWidth="1"/>
-    <col min="2" max="2" width="59.8571428571429" style="32" customWidth="1"/>
+    <col min="1" max="1" width="62.7109375" style="31" customWidth="1"/>
+    <col min="2" max="2" width="59.85546875" style="32" customWidth="1"/>
     <col min="3" max="16384" width="9" style="31"/>
   </cols>
   <sheetData>
@@ -23641,28 +23030,26 @@
         <v>2336</v>
       </c>
     </row>
-    <row r="1445" spans="1:1">
+    <row r="1445" spans="1:2">
       <c r="A1445" s="31" t="s">
         <v>2337</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1209" r:id="rId1" display="MRAD-2425-00086"/>
-    <hyperlink ref="B1364" r:id="rId2" display="RFQ10/00725/25-26"/>
+    <hyperlink ref="B1209" r:id="rId1"/>
+    <hyperlink ref="B1364" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B107"/>
-  <sheetFormatPr defaultColWidth="8.85714285714286" defaultRowHeight="15" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="35.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="35.28515625" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -23674,7 +23061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="108.95" customHeight="1" spans="1:2">
+    <row r="2" spans="1:2" ht="108.95" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2338</v>
       </c>
@@ -23682,7 +23069,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="3" ht="114" customHeight="1" spans="1:2">
+    <row r="3" spans="1:2" ht="114" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>2340</v>
       </c>
@@ -23690,7 +23077,7 @@
         <v>2341</v>
       </c>
     </row>
-    <row r="4" ht="80.25" customHeight="1" spans="1:2">
+    <row r="4" spans="1:2" ht="80.25" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>2342</v>
       </c>
@@ -23698,7 +23085,7 @@
         <v>2343</v>
       </c>
     </row>
-    <row r="5" ht="69.75" customHeight="1" spans="1:2">
+    <row r="5" spans="1:2" ht="69.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2344</v>
       </c>
@@ -23706,7 +23093,7 @@
         <v>2345</v>
       </c>
     </row>
-    <row r="6" ht="51.75" customHeight="1" spans="1:2">
+    <row r="6" spans="1:2" ht="51.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>2346</v>
       </c>
@@ -23714,7 +23101,7 @@
         <v>2347</v>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" spans="1:2">
+    <row r="7" spans="1:2" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>2348</v>
       </c>
@@ -23722,7 +23109,7 @@
         <v>2349</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:2">
+    <row r="8" spans="1:2" ht="18" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>2350</v>
       </c>
@@ -23730,7 +23117,7 @@
         <v>2351</v>
       </c>
     </row>
-    <row r="9" ht="39" customHeight="1" spans="1:2">
+    <row r="9" spans="1:2" ht="39" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>2352</v>
       </c>
@@ -23738,7 +23125,7 @@
         <v>2353</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1" spans="1:2">
+    <row r="10" spans="1:2" ht="22.5" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>2354</v>
       </c>
@@ -23746,7 +23133,7 @@
         <v>2355</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" spans="1:2">
+    <row r="11" spans="1:2" ht="18" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>2356</v>
       </c>
@@ -23754,7 +23141,7 @@
         <v>2357</v>
       </c>
     </row>
-    <row r="12" ht="26.25" customHeight="1" spans="1:2">
+    <row r="12" spans="1:2" ht="26.25" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>2358</v>
       </c>
@@ -23762,7 +23149,7 @@
         <v>2359</v>
       </c>
     </row>
-    <row r="13" ht="28.5" customHeight="1" spans="1:2">
+    <row r="13" spans="1:2" ht="28.5" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>2360</v>
       </c>
@@ -23770,7 +23157,7 @@
         <v>2361</v>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" spans="1:2">
+    <row r="14" spans="1:2" ht="24" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>2362</v>
       </c>
@@ -23778,7 +23165,7 @@
         <v>2363</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:2">
+    <row r="15" spans="1:2" ht="36" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>2364</v>
       </c>
@@ -23786,7 +23173,7 @@
         <v>2365</v>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1" spans="1:2">
+    <row r="16" spans="1:2" ht="45" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>2366</v>
       </c>
@@ -23794,7 +23181,7 @@
         <v>2367</v>
       </c>
     </row>
-    <row r="17" ht="43.5" customHeight="1" spans="1:2">
+    <row r="17" spans="1:2" ht="43.5" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>2368</v>
       </c>
@@ -23802,7 +23189,7 @@
         <v>2369</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1" spans="1:2">
+    <row r="18" spans="1:2" ht="42" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>2370</v>
       </c>
@@ -23810,7 +23197,7 @@
         <v>2371</v>
       </c>
     </row>
-    <row r="19" ht="52.5" customHeight="1" spans="1:2">
+    <row r="19" spans="1:2" ht="52.5" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>2372</v>
       </c>
@@ -23818,7 +23205,7 @@
         <v>2373</v>
       </c>
     </row>
-    <row r="20" ht="17.25" customHeight="1" spans="1:2">
+    <row r="20" spans="1:2" ht="17.25" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>2374</v>
       </c>
@@ -23826,7 +23213,7 @@
         <v>2375</v>
       </c>
     </row>
-    <row r="21" customHeight="1" spans="1:2">
+    <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>2376</v>
       </c>
@@ -23834,7 +23221,7 @@
         <v>2377</v>
       </c>
     </row>
-    <row r="22" ht="409.5" spans="1:2">
+    <row r="22" spans="1:2" ht="409.5">
       <c r="A22" s="2" t="s">
         <v>2378</v>
       </c>
@@ -23842,7 +23229,7 @@
         <v>2379</v>
       </c>
     </row>
-    <row r="23" ht="255" spans="1:2">
+    <row r="23" spans="1:2" ht="255">
       <c r="A23" s="2" t="s">
         <v>2380</v>
       </c>
@@ -23850,7 +23237,7 @@
         <v>2381</v>
       </c>
     </row>
-    <row r="24" ht="240" spans="1:2">
+    <row r="24" spans="1:2" ht="240">
       <c r="A24" t="s">
         <v>2382</v>
       </c>
@@ -23858,7 +23245,7 @@
         <v>2383</v>
       </c>
     </row>
-    <row r="25" ht="270" spans="1:2">
+    <row r="25" spans="1:2" ht="270">
       <c r="A25" t="s">
         <v>2384</v>
       </c>
@@ -23866,7 +23253,7 @@
         <v>2385</v>
       </c>
     </row>
-    <row r="26" ht="210" spans="1:2">
+    <row r="26" spans="1:2" ht="210">
       <c r="A26" t="s">
         <v>2386</v>
       </c>
@@ -23874,7 +23261,7 @@
         <v>2387</v>
       </c>
     </row>
-    <row r="27" ht="61.5" customHeight="1" spans="1:2">
+    <row r="27" spans="1:2" ht="61.5" customHeight="1">
       <c r="A27" s="7" t="s">
         <v>2388</v>
       </c>
@@ -23882,7 +23269,7 @@
         <v>2389</v>
       </c>
     </row>
-    <row r="28" ht="105.75" customHeight="1" spans="1:2">
+    <row r="28" spans="1:2" ht="105.75" customHeight="1">
       <c r="A28" s="8" t="s">
         <v>2338</v>
       </c>
@@ -23890,7 +23277,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="29" ht="180" spans="1:2">
+    <row r="29" spans="1:2" ht="180">
       <c r="A29" s="9" t="s">
         <v>2346</v>
       </c>
@@ -23898,7 +23285,7 @@
         <v>2390</v>
       </c>
     </row>
-    <row r="30" ht="135" spans="1:2">
+    <row r="30" spans="1:2" ht="135">
       <c r="A30" s="11" t="s">
         <v>2391</v>
       </c>
@@ -23906,7 +23293,7 @@
         <v>2392</v>
       </c>
     </row>
-    <row r="31" ht="180" spans="1:2">
+    <row r="31" spans="1:2" ht="180">
       <c r="A31" s="13" t="s">
         <v>2393</v>
       </c>
@@ -23914,7 +23301,7 @@
         <v>2394</v>
       </c>
     </row>
-    <row r="32" ht="180" spans="1:2">
+    <row r="32" spans="1:2" ht="180">
       <c r="A32" s="15" t="s">
         <v>2395</v>
       </c>
@@ -23922,7 +23309,7 @@
         <v>2396</v>
       </c>
     </row>
-    <row r="33" ht="409.5" spans="1:2">
+    <row r="33" spans="1:2" ht="409.5">
       <c r="A33" s="17" t="s">
         <v>2397</v>
       </c>
@@ -23930,7 +23317,7 @@
         <v>2398</v>
       </c>
     </row>
-    <row r="34" ht="409.5" spans="1:2">
+    <row r="34" spans="1:2" ht="409.5">
       <c r="A34" s="19" t="s">
         <v>2399</v>
       </c>
@@ -23938,7 +23325,7 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="35" ht="409.5" spans="1:2">
+    <row r="35" spans="1:2" ht="409.5">
       <c r="A35" s="21" t="s">
         <v>2401</v>
       </c>
@@ -23946,7 +23333,7 @@
         <v>2402</v>
       </c>
     </row>
-    <row r="36" ht="409.5" spans="1:2">
+    <row r="36" spans="1:2" ht="409.5">
       <c r="A36" s="23" t="s">
         <v>2403</v>
       </c>
@@ -23954,7 +23341,7 @@
         <v>2404</v>
       </c>
     </row>
-    <row r="37" ht="409.5" spans="1:2">
+    <row r="37" spans="1:2" ht="409.5">
       <c r="A37" s="25" t="s">
         <v>2405</v>
       </c>
@@ -23962,7 +23349,7 @@
         <v>2406</v>
       </c>
     </row>
-    <row r="38" ht="90" spans="1:2">
+    <row r="38" spans="1:2" ht="90">
       <c r="A38" t="s">
         <v>2407</v>
       </c>
@@ -23970,7 +23357,7 @@
         <v>2408</v>
       </c>
     </row>
-    <row r="39" ht="120" spans="1:2">
+    <row r="39" spans="1:2" ht="120">
       <c r="A39" t="s">
         <v>2409</v>
       </c>
@@ -23978,7 +23365,7 @@
         <v>2410</v>
       </c>
     </row>
-    <row r="40" ht="180" spans="1:2">
+    <row r="40" spans="1:2" ht="180">
       <c r="A40" t="s">
         <v>2411</v>
       </c>
@@ -23986,7 +23373,7 @@
         <v>2412</v>
       </c>
     </row>
-    <row r="41" ht="195" spans="1:2">
+    <row r="41" spans="1:2" ht="195">
       <c r="A41" t="s">
         <v>2413</v>
       </c>
@@ -23994,7 +23381,7 @@
         <v>2414</v>
       </c>
     </row>
-    <row r="42" ht="120" spans="1:2">
+    <row r="42" spans="1:2" ht="120">
       <c r="A42" t="s">
         <v>2415</v>
       </c>
@@ -24002,7 +23389,7 @@
         <v>2416</v>
       </c>
     </row>
-    <row r="43" ht="409.5" spans="1:2">
+    <row r="43" spans="1:2" ht="409.5">
       <c r="A43" t="s">
         <v>2417</v>
       </c>
@@ -24010,7 +23397,7 @@
         <v>2418</v>
       </c>
     </row>
-    <row r="44" ht="409.5" spans="1:2">
+    <row r="44" spans="1:2" ht="409.5">
       <c r="A44" t="s">
         <v>2419</v>
       </c>
@@ -24018,7 +23405,7 @@
         <v>2420</v>
       </c>
     </row>
-    <row r="45" ht="409.5" spans="1:2">
+    <row r="45" spans="1:2" ht="409.5">
       <c r="A45" t="s">
         <v>2421</v>
       </c>
@@ -24026,7 +23413,7 @@
         <v>2422</v>
       </c>
     </row>
-    <row r="46" ht="270" spans="1:2">
+    <row r="46" spans="1:2" ht="270">
       <c r="A46" t="s">
         <v>2423</v>
       </c>
@@ -24034,7 +23421,7 @@
         <v>2424</v>
       </c>
     </row>
-    <row r="47" ht="409.5" spans="1:2">
+    <row r="47" spans="1:2" ht="409.5">
       <c r="A47" t="s">
         <v>2425</v>
       </c>
@@ -24042,7 +23429,7 @@
         <v>2426</v>
       </c>
     </row>
-    <row r="48" ht="345" spans="1:2">
+    <row r="48" spans="1:2" ht="345">
       <c r="A48" t="s">
         <v>2427</v>
       </c>
@@ -24050,7 +23437,7 @@
         <v>2428</v>
       </c>
     </row>
-    <row r="49" ht="345" spans="1:2">
+    <row r="49" spans="1:2" ht="345">
       <c r="A49" t="s">
         <v>2429</v>
       </c>
@@ -24058,7 +23445,7 @@
         <v>2430</v>
       </c>
     </row>
-    <row r="50" ht="36" customHeight="1" spans="1:2">
+    <row r="50" spans="1:2" ht="36" customHeight="1">
       <c r="A50" t="s">
         <v>2431</v>
       </c>
@@ -24066,7 +23453,7 @@
         <v>2432</v>
       </c>
     </row>
-    <row r="51" ht="23.25" customHeight="1" spans="1:2">
+    <row r="51" spans="1:2" ht="23.25" customHeight="1">
       <c r="A51" t="s">
         <v>2433</v>
       </c>
@@ -24074,7 +23461,7 @@
         <v>2434</v>
       </c>
     </row>
-    <row r="52" ht="27.75" customHeight="1" spans="1:2">
+    <row r="52" spans="1:2" ht="27.75" customHeight="1">
       <c r="A52" t="s">
         <v>2435</v>
       </c>
@@ -24082,7 +23469,7 @@
         <v>2436</v>
       </c>
     </row>
-    <row r="53" ht="60" spans="1:2">
+    <row r="53" spans="1:2" ht="60">
       <c r="A53" t="s">
         <v>2437</v>
       </c>
@@ -24090,7 +23477,7 @@
         <v>2438</v>
       </c>
     </row>
-    <row r="54" ht="45" spans="1:2">
+    <row r="54" spans="1:2" ht="45">
       <c r="A54" t="s">
         <v>2439</v>
       </c>
@@ -24098,7 +23485,7 @@
         <v>2440</v>
       </c>
     </row>
-    <row r="55" ht="60" spans="1:2">
+    <row r="55" spans="1:2" ht="60">
       <c r="A55" t="s">
         <v>2441</v>
       </c>
@@ -24106,7 +23493,7 @@
         <v>2442</v>
       </c>
     </row>
-    <row r="56" ht="75" spans="1:2">
+    <row r="56" spans="1:2" ht="75">
       <c r="A56" t="s">
         <v>2443</v>
       </c>
@@ -24114,7 +23501,7 @@
         <v>2444</v>
       </c>
     </row>
-    <row r="57" ht="409.5" spans="1:2">
+    <row r="57" spans="1:2" ht="409.5">
       <c r="A57" t="s">
         <v>2445</v>
       </c>
@@ -24122,7 +23509,7 @@
         <v>2446</v>
       </c>
     </row>
-    <row r="58" ht="90" spans="1:2">
+    <row r="58" spans="1:2" ht="90">
       <c r="A58" t="s">
         <v>2447</v>
       </c>
@@ -24130,7 +23517,7 @@
         <v>2448</v>
       </c>
     </row>
-    <row r="59" ht="360" spans="1:2">
+    <row r="59" spans="1:2" ht="360">
       <c r="A59" t="s">
         <v>2449</v>
       </c>
@@ -24138,7 +23525,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="60" ht="60" spans="1:2">
+    <row r="60" spans="1:2" ht="75">
       <c r="A60" t="s">
         <v>2451</v>
       </c>
@@ -24146,7 +23533,7 @@
         <v>2452</v>
       </c>
     </row>
-    <row r="61" ht="409.5" spans="1:2">
+    <row r="61" spans="1:2" ht="409.5">
       <c r="A61" t="s">
         <v>2453</v>
       </c>
@@ -24154,7 +23541,7 @@
         <v>2369</v>
       </c>
     </row>
-    <row r="62" ht="87.75" customHeight="1" spans="1:2">
+    <row r="62" spans="1:2" ht="87.75" customHeight="1">
       <c r="A62" t="s">
         <v>2454</v>
       </c>
@@ -24162,7 +23549,7 @@
         <v>2455</v>
       </c>
     </row>
-    <row r="63" ht="71.25" customHeight="1" spans="1:2">
+    <row r="63" spans="1:2" ht="71.25" customHeight="1">
       <c r="A63" t="s">
         <v>2456</v>
       </c>
@@ -24170,7 +23557,7 @@
         <v>2457</v>
       </c>
     </row>
-    <row r="64" ht="54" customHeight="1" spans="1:2">
+    <row r="64" spans="1:2" ht="54" customHeight="1">
       <c r="A64" t="s">
         <v>2413</v>
       </c>
@@ -24178,7 +23565,7 @@
         <v>2458</v>
       </c>
     </row>
-    <row r="65" ht="86.25" customHeight="1" spans="1:2">
+    <row r="65" spans="1:2" ht="86.25" customHeight="1">
       <c r="A65" s="27" t="s">
         <v>2459</v>
       </c>
@@ -24186,7 +23573,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="66" ht="86.25" customHeight="1" spans="1:2">
+    <row r="66" spans="1:2" ht="86.25" customHeight="1">
       <c r="A66" s="27" t="s">
         <v>2461</v>
       </c>
@@ -24194,7 +23581,7 @@
         <v>2462</v>
       </c>
     </row>
-    <row r="67" ht="102" customHeight="1" spans="1:2">
+    <row r="67" spans="1:2" ht="102" customHeight="1">
       <c r="A67" s="27" t="s">
         <v>2463</v>
       </c>
@@ -24202,7 +23589,7 @@
         <v>2464</v>
       </c>
     </row>
-    <row r="68" ht="89.25" customHeight="1" spans="1:2">
+    <row r="68" spans="1:2" ht="89.25" customHeight="1">
       <c r="A68" s="27" t="s">
         <v>2465</v>
       </c>
@@ -24210,7 +23597,7 @@
         <v>2466</v>
       </c>
     </row>
-    <row r="69" ht="102" customHeight="1" spans="1:2">
+    <row r="69" spans="1:2" ht="102" customHeight="1">
       <c r="A69" s="27" t="s">
         <v>2467</v>
       </c>
@@ -24218,7 +23605,7 @@
         <v>2468</v>
       </c>
     </row>
-    <row r="70" ht="45" spans="1:2">
+    <row r="70" spans="1:2" ht="45">
       <c r="A70" s="28" t="s">
         <v>2469</v>
       </c>
@@ -24226,7 +23613,7 @@
         <v>2470</v>
       </c>
     </row>
-    <row r="71" ht="409.5" spans="1:2">
+    <row r="71" spans="1:2" ht="409.5">
       <c r="A71" s="29" t="s">
         <v>2471</v>
       </c>
@@ -24234,7 +23621,7 @@
         <v>2472</v>
       </c>
     </row>
-    <row r="72" ht="60" spans="1:2">
+    <row r="72" spans="1:2" ht="60">
       <c r="A72" t="s">
         <v>2473</v>
       </c>
@@ -24242,7 +23629,7 @@
         <v>2474</v>
       </c>
     </row>
-    <row r="73" ht="30" spans="1:2">
+    <row r="73" spans="1:2" ht="30">
       <c r="A73" t="s">
         <v>2475</v>
       </c>
@@ -24250,7 +23637,7 @@
         <v>2476</v>
       </c>
     </row>
-    <row r="74" ht="60" spans="1:2">
+    <row r="74" spans="1:2" ht="60">
       <c r="A74" t="s">
         <v>2477</v>
       </c>
@@ -24258,7 +23645,7 @@
         <v>2478</v>
       </c>
     </row>
-    <row r="75" ht="120" spans="1:2">
+    <row r="75" spans="1:2" ht="120">
       <c r="A75" t="s">
         <v>2479</v>
       </c>
@@ -24266,7 +23653,7 @@
         <v>2480</v>
       </c>
     </row>
-    <row r="76" ht="60" spans="1:2">
+    <row r="76" spans="1:2" ht="60">
       <c r="A76" t="s">
         <v>2481</v>
       </c>
@@ -24274,7 +23661,7 @@
         <v>2482</v>
       </c>
     </row>
-    <row r="77" ht="45" spans="1:2">
+    <row r="77" spans="1:2" ht="45">
       <c r="A77" t="s">
         <v>2483</v>
       </c>
@@ -24282,7 +23669,7 @@
         <v>2484</v>
       </c>
     </row>
-    <row r="78" ht="409.5" spans="1:2">
+    <row r="78" spans="1:2" ht="409.5">
       <c r="A78" t="s">
         <v>2485</v>
       </c>
@@ -24290,7 +23677,7 @@
         <v>2486</v>
       </c>
     </row>
-    <row r="79" ht="409.5" spans="1:2">
+    <row r="79" spans="1:2" ht="409.5">
       <c r="A79" t="s">
         <v>2487</v>
       </c>
@@ -24298,7 +23685,7 @@
         <v>2488</v>
       </c>
     </row>
-    <row r="80" ht="45" spans="1:2">
+    <row r="80" spans="1:2" ht="45">
       <c r="A80" s="28" t="s">
         <v>2489</v>
       </c>
@@ -24306,7 +23693,7 @@
         <v>2490</v>
       </c>
     </row>
-    <row r="81" ht="45" spans="1:2">
+    <row r="81" spans="1:2" ht="45">
       <c r="A81" s="27" t="s">
         <v>2491</v>
       </c>
@@ -24314,7 +23701,7 @@
         <v>2492</v>
       </c>
     </row>
-    <row r="82" ht="75" spans="1:2">
+    <row r="82" spans="1:2" ht="75">
       <c r="A82" s="27" t="s">
         <v>2493</v>
       </c>
@@ -24322,7 +23709,7 @@
         <v>2494</v>
       </c>
     </row>
-    <row r="83" ht="45" spans="1:2">
+    <row r="83" spans="1:2" ht="45">
       <c r="A83" s="27" t="s">
         <v>2495</v>
       </c>
@@ -24330,7 +23717,7 @@
         <v>2492</v>
       </c>
     </row>
-    <row r="84" ht="90" spans="1:2">
+    <row r="84" spans="1:2" ht="90">
       <c r="A84" s="27" t="s">
         <v>2496</v>
       </c>
@@ -24338,7 +23725,7 @@
         <v>2497</v>
       </c>
     </row>
-    <row r="85" ht="45" spans="1:2">
+    <row r="85" spans="1:2" ht="45">
       <c r="A85" s="27" t="s">
         <v>2489</v>
       </c>
@@ -24346,7 +23733,7 @@
         <v>2490</v>
       </c>
     </row>
-    <row r="86" ht="75" spans="1:2">
+    <row r="86" spans="1:2" ht="75">
       <c r="A86" s="27" t="s">
         <v>2498</v>
       </c>
@@ -24354,7 +23741,7 @@
         <v>2499</v>
       </c>
     </row>
-    <row r="87" ht="60" spans="1:2">
+    <row r="87" spans="1:2" ht="60">
       <c r="A87" s="27" t="s">
         <v>2500</v>
       </c>
@@ -24362,7 +23749,7 @@
         <v>2501</v>
       </c>
     </row>
-    <row r="88" ht="409.5" spans="1:2">
+    <row r="88" spans="1:2" ht="409.5">
       <c r="A88" s="27" t="s">
         <v>2502</v>
       </c>
@@ -24370,7 +23757,7 @@
         <v>2503</v>
       </c>
     </row>
-    <row r="89" ht="60" spans="1:2">
+    <row r="89" spans="1:2" ht="60">
       <c r="A89" s="27" t="s">
         <v>2504</v>
       </c>
@@ -24378,7 +23765,7 @@
         <v>2505</v>
       </c>
     </row>
-    <row r="90" ht="240" spans="1:2">
+    <row r="90" spans="1:2" ht="240">
       <c r="A90" t="s">
         <v>2506</v>
       </c>
@@ -24386,7 +23773,7 @@
         <v>2507</v>
       </c>
     </row>
-    <row r="91" ht="75" spans="1:2">
+    <row r="91" spans="1:2" ht="75">
       <c r="A91" t="s">
         <v>2498</v>
       </c>
@@ -24394,7 +23781,7 @@
         <v>2499</v>
       </c>
     </row>
-    <row r="92" ht="45" spans="1:2">
+    <row r="92" spans="1:2" ht="45">
       <c r="A92" t="s">
         <v>2489</v>
       </c>
@@ -24402,7 +23789,7 @@
         <v>2490</v>
       </c>
     </row>
-    <row r="93" ht="105" spans="1:2">
+    <row r="93" spans="1:2" ht="105">
       <c r="A93" t="s">
         <v>2508</v>
       </c>
@@ -24410,7 +23797,7 @@
         <v>2509</v>
       </c>
     </row>
-    <row r="94" ht="120" spans="1:2">
+    <row r="94" spans="1:2" ht="120">
       <c r="A94" t="s">
         <v>2510</v>
       </c>
@@ -24418,7 +23805,7 @@
         <v>2511</v>
       </c>
     </row>
-    <row r="95" ht="60" spans="1:2">
+    <row r="95" spans="1:2" ht="60">
       <c r="A95" t="s">
         <v>2512</v>
       </c>
@@ -24426,7 +23813,7 @@
         <v>2513</v>
       </c>
     </row>
-    <row r="96" ht="60" spans="1:2">
+    <row r="96" spans="1:2" ht="60">
       <c r="A96" t="s">
         <v>2514</v>
       </c>
@@ -24434,7 +23821,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="97" ht="75" spans="1:2">
+    <row r="97" spans="1:2" ht="75">
       <c r="A97" t="s">
         <v>2516</v>
       </c>
@@ -24442,7 +23829,7 @@
         <v>2517</v>
       </c>
     </row>
-    <row r="98" ht="60" spans="1:2">
+    <row r="98" spans="1:2" ht="60">
       <c r="A98" t="s">
         <v>2518</v>
       </c>
@@ -24450,7 +23837,7 @@
         <v>2519</v>
       </c>
     </row>
-    <row r="99" ht="101.25" customHeight="1" spans="1:2">
+    <row r="99" spans="1:2" ht="101.25" customHeight="1">
       <c r="A99" t="s">
         <v>2520</v>
       </c>
@@ -24458,7 +23845,7 @@
         <v>2521</v>
       </c>
     </row>
-    <row r="100" ht="85.5" customHeight="1" spans="1:2">
+    <row r="100" spans="1:2" ht="85.5" customHeight="1">
       <c r="A100" t="s">
         <v>2522</v>
       </c>
@@ -24466,7 +23853,7 @@
         <v>2523</v>
       </c>
     </row>
-    <row r="101" ht="409.5" spans="1:2">
+    <row r="101" spans="1:2" ht="409.5">
       <c r="A101" t="s">
         <v>2524</v>
       </c>
@@ -24474,7 +23861,7 @@
         <v>2525</v>
       </c>
     </row>
-    <row r="102" ht="120.75" customHeight="1" spans="1:2">
+    <row r="102" spans="1:2" ht="120.75" customHeight="1">
       <c r="A102" t="s">
         <v>2526</v>
       </c>
@@ -24482,7 +23869,7 @@
         <v>2527</v>
       </c>
     </row>
-    <row r="103" ht="159.75" customHeight="1" spans="1:2">
+    <row r="103" spans="1:2" ht="159.75" customHeight="1">
       <c r="A103" t="s">
         <v>2528</v>
       </c>
@@ -24490,7 +23877,7 @@
         <v>2529</v>
       </c>
     </row>
-    <row r="104" ht="60" spans="1:2">
+    <row r="104" spans="1:2" ht="60">
       <c r="A104" t="s">
         <v>2530</v>
       </c>
@@ -24498,7 +23885,7 @@
         <v>2531</v>
       </c>
     </row>
-    <row r="105" ht="75" spans="1:2">
+    <row r="105" spans="1:2" ht="75">
       <c r="A105" t="s">
         <v>2532</v>
       </c>
@@ -24506,7 +23893,7 @@
         <v>2533</v>
       </c>
     </row>
-    <row r="106" ht="409.5" spans="1:2">
+    <row r="106" spans="1:2" ht="409.5">
       <c r="A106" s="21" t="s">
         <v>2534</v>
       </c>
@@ -24514,7 +23901,7 @@
         <v>2535</v>
       </c>
     </row>
-    <row r="107" ht="409.5" spans="1:2">
+    <row r="107" spans="1:2" ht="409.5">
       <c r="A107" t="s">
         <v>2536</v>
       </c>
@@ -24524,6 +23911,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Purchase Bill Get Document New Scenarios
Purchase Bill Get Document New Scenarios
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3074" uniqueCount="2542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3080" uniqueCount="2548">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -10906,6 +10906,36 @@
 AND suphd_doc_type ='SB'
 AND suphd_grn_refer ='SCO'
 AND suphd_doc_no ='${PBNO}'</t>
+  </si>
+  <si>
+    <t>PBJournalQueryPK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  SELECT *
+FROM APPL_JRNL_VW 
+ WHERE AJ_BU = 'ROAU'
+  AND AJ_VOU_NO ='${PBNO}'
+  AND AJ_GL_ACCT_DESC='${GLAC}'</t>
+  </si>
+  <si>
+    <t>PBJournalDetailsQueryPK</t>
+  </si>
+  <si>
+    <t>SELECT *
+FROM APPL_JOURNALS_HIST_VW
+WHERE AJHV_BU = 'ROAU'
+  AND AJHV_VOU_NO = '${PBNO}'
+  AND AJHV_GL_ACCT_DESC='${GLAC}'</t>
+  </si>
+  <si>
+    <t>PBJournalDetailsViewPK</t>
+  </si>
+  <si>
+    <t>SELECT *
+FROM APPL_JOURNALS_HIST_VW
+WHERE AJHV_BU = 'ROAU'
+  AND AJHV_VOU_NO = '${PBNO}'
+  AND AJHV_VOU_LINE_NO='${VLNO}'</t>
   </si>
 </sst>
 </file>
@@ -23075,7 +23105,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B109"/>
+  <dimension ref="A1:B112"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.28515625" customWidth="1"/>
@@ -23954,6 +23984,30 @@
         <v>2541</v>
       </c>
     </row>
+    <row r="110" spans="1:2" ht="75">
+      <c r="A110" t="s">
+        <v>2542</v>
+      </c>
+      <c r="B110" s="27" t="s">
+        <v>2543</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" ht="75">
+      <c r="A111" t="s">
+        <v>2544</v>
+      </c>
+      <c r="B111" s="27" t="s">
+        <v>2545</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" ht="75">
+      <c r="A112" t="s">
+        <v>2546</v>
+      </c>
+      <c r="B112" s="27" t="s">
+        <v>2547</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Subcontract PurchaseBills Scenarios And Test Fixes
Subcontract PurchaseBills Scenarios And Test Fixes
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SupplyChainManagement" sheetId="1" r:id="rId1"/>
     <sheet name="DBData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3108" uniqueCount="2576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3110" uniqueCount="2578">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -11242,18 +11242,28 @@
  AND STSFG_STORE_ID = '${Warehouse}'
  AND STSFG_VOU_NO = '${CompProdOrderNo}'</t>
   </si>
+  <si>
+    <t>SupplierGLaccountQuery</t>
+  </si>
+  <si>
+    <t>SELECT glac_acct_desc1
+  FROM suplr_plant_accts, glm_control,gl_accts
+ WHERE spla_bu = glmctrl_bu
+       AND (glmctrl_bs_level = 'U' 
+     --  AND spla_plnt = :p_plnt
+            OR glmctrl_bs_level = 'E')
+       AND SPLA_SUPLR_ID = '${SUPNO}'
+       AND spla_bu ='ROAU'
+       AND spla_lgr_type ='AP'
+       AND spla_bu = glac_bu
+       AND spla_acct = glac_acct</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="26">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -11300,151 +11310,14 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -11469,188 +11342,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -11686,268 +11379,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="66">
+  <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -11965,44 +11416,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="63" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="51" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="52" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="53"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="53" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="54" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="55" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="56" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="61" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -12038,15 +11489,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="62" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -12066,11 +11517,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -12084,19 +11535,19 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="58" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="59" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="60" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="58" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -12111,74 +11562,27 @@
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="66">
+  <cellStyles count="18">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 10" xfId="49"/>
-    <cellStyle name="Normal 11" xfId="50"/>
-    <cellStyle name="Normal 13" xfId="51"/>
-    <cellStyle name="Normal 14" xfId="52"/>
-    <cellStyle name="Normal 15" xfId="53"/>
-    <cellStyle name="Normal 16" xfId="54"/>
-    <cellStyle name="Normal 17" xfId="55"/>
-    <cellStyle name="Normal 18" xfId="56"/>
-    <cellStyle name="Normal 19" xfId="57"/>
-    <cellStyle name="Normal 2" xfId="58"/>
-    <cellStyle name="Normal 2 2" xfId="59"/>
-    <cellStyle name="Normal 2 3" xfId="60"/>
-    <cellStyle name="Normal 20" xfId="61"/>
-    <cellStyle name="Normal 3" xfId="62"/>
-    <cellStyle name="Normal 7" xfId="63"/>
-    <cellStyle name="Normal 8" xfId="64"/>
-    <cellStyle name="Normal 9" xfId="65"/>
+    <cellStyle name="Normal 10" xfId="1"/>
+    <cellStyle name="Normal 11" xfId="2"/>
+    <cellStyle name="Normal 13" xfId="3"/>
+    <cellStyle name="Normal 14" xfId="4"/>
+    <cellStyle name="Normal 15" xfId="5"/>
+    <cellStyle name="Normal 16" xfId="6"/>
+    <cellStyle name="Normal 17" xfId="7"/>
+    <cellStyle name="Normal 18" xfId="8"/>
+    <cellStyle name="Normal 19" xfId="9"/>
+    <cellStyle name="Normal 2" xfId="10"/>
+    <cellStyle name="Normal 2 2" xfId="11"/>
+    <cellStyle name="Normal 2 3" xfId="12"/>
+    <cellStyle name="Normal 20" xfId="13"/>
+    <cellStyle name="Normal 3" xfId="14"/>
+    <cellStyle name="Normal 7" xfId="15"/>
+    <cellStyle name="Normal 8" xfId="16"/>
+    <cellStyle name="Normal 9" xfId="17"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -12440,17 +11844,17 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B1445"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="62.7142857142857" style="31" customWidth="1"/>
-    <col min="2" max="2" width="59.8571428571429" style="32" customWidth="1"/>
+    <col min="1" max="1" width="62.7109375" style="31" customWidth="1"/>
+    <col min="2" max="2" width="59.85546875" style="32" customWidth="1"/>
     <col min="3" max="16384" width="9" style="31"/>
   </cols>
   <sheetData>
@@ -24013,21 +23417,19 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1209" r:id="rId1" display="MRAD-2425-00086"/>
-    <hyperlink ref="B1364" r:id="rId2" display="RFQ10/00725/25-26"/>
+    <hyperlink ref="B1209" r:id="rId1"/>
+    <hyperlink ref="B1364" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B126"/>
-  <sheetFormatPr defaultColWidth="8.85714285714286" defaultRowHeight="15" outlineLevelCol="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B127"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="35.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="35.28515625" customWidth="1"/>
     <col min="2" max="2" width="65" customWidth="1"/>
   </cols>
   <sheetData>
@@ -24039,7 +23441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="108.95" customHeight="1" spans="1:2">
+    <row r="2" spans="1:2" ht="108.95" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2338</v>
       </c>
@@ -24047,7 +23449,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="3" ht="114" customHeight="1" spans="1:2">
+    <row r="3" spans="1:2" ht="114" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>2340</v>
       </c>
@@ -24055,7 +23457,7 @@
         <v>2341</v>
       </c>
     </row>
-    <row r="4" ht="80.25" customHeight="1" spans="1:2">
+    <row r="4" spans="1:2" ht="80.25" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>2342</v>
       </c>
@@ -24063,7 +23465,7 @@
         <v>2343</v>
       </c>
     </row>
-    <row r="5" ht="69.75" customHeight="1" spans="1:2">
+    <row r="5" spans="1:2" ht="69.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>2344</v>
       </c>
@@ -24071,7 +23473,7 @@
         <v>2345</v>
       </c>
     </row>
-    <row r="6" ht="51.75" customHeight="1" spans="1:2">
+    <row r="6" spans="1:2" ht="51.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>2346</v>
       </c>
@@ -24079,7 +23481,7 @@
         <v>2347</v>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" spans="1:2">
+    <row r="7" spans="1:2" ht="30" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>2348</v>
       </c>
@@ -24087,7 +23489,7 @@
         <v>2349</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:2">
+    <row r="8" spans="1:2" ht="18" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>2350</v>
       </c>
@@ -24095,7 +23497,7 @@
         <v>2351</v>
       </c>
     </row>
-    <row r="9" ht="39" customHeight="1" spans="1:2">
+    <row r="9" spans="1:2" ht="39" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>2352</v>
       </c>
@@ -24103,7 +23505,7 @@
         <v>2353</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1" spans="1:2">
+    <row r="10" spans="1:2" ht="22.5" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>2354</v>
       </c>
@@ -24111,7 +23513,7 @@
         <v>2355</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" spans="1:2">
+    <row r="11" spans="1:2" ht="18" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>2356</v>
       </c>
@@ -24119,7 +23521,7 @@
         <v>2357</v>
       </c>
     </row>
-    <row r="12" ht="26.25" customHeight="1" spans="1:2">
+    <row r="12" spans="1:2" ht="26.25" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>2358</v>
       </c>
@@ -24127,7 +23529,7 @@
         <v>2359</v>
       </c>
     </row>
-    <row r="13" ht="28.5" customHeight="1" spans="1:2">
+    <row r="13" spans="1:2" ht="28.5" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>2360</v>
       </c>
@@ -24135,7 +23537,7 @@
         <v>2361</v>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" spans="1:2">
+    <row r="14" spans="1:2" ht="24" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>2362</v>
       </c>
@@ -24143,7 +23545,7 @@
         <v>2363</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:2">
+    <row r="15" spans="1:2" ht="36" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>2364</v>
       </c>
@@ -24151,7 +23553,7 @@
         <v>2365</v>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1" spans="1:2">
+    <row r="16" spans="1:2" ht="45" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>2366</v>
       </c>
@@ -24159,7 +23561,7 @@
         <v>2367</v>
       </c>
     </row>
-    <row r="17" ht="43.5" customHeight="1" spans="1:2">
+    <row r="17" spans="1:2" ht="43.5" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>2368</v>
       </c>
@@ -24167,7 +23569,7 @@
         <v>2369</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1" spans="1:2">
+    <row r="18" spans="1:2" ht="42" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>2370</v>
       </c>
@@ -24175,7 +23577,7 @@
         <v>2371</v>
       </c>
     </row>
-    <row r="19" ht="52.5" customHeight="1" spans="1:2">
+    <row r="19" spans="1:2" ht="52.5" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>2372</v>
       </c>
@@ -24183,7 +23585,7 @@
         <v>2373</v>
       </c>
     </row>
-    <row r="20" ht="17.25" customHeight="1" spans="1:2">
+    <row r="20" spans="1:2" ht="17.25" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>2374</v>
       </c>
@@ -24191,7 +23593,7 @@
         <v>2375</v>
       </c>
     </row>
-    <row r="21" customHeight="1" spans="1:2">
+    <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>2376</v>
       </c>
@@ -24199,7 +23601,7 @@
         <v>2377</v>
       </c>
     </row>
-    <row r="22" ht="409.5" spans="1:2">
+    <row r="22" spans="1:2" ht="409.5">
       <c r="A22" s="2" t="s">
         <v>2378</v>
       </c>
@@ -24207,7 +23609,7 @@
         <v>2379</v>
       </c>
     </row>
-    <row r="23" ht="255" spans="1:2">
+    <row r="23" spans="1:2" ht="255">
       <c r="A23" s="2" t="s">
         <v>2380</v>
       </c>
@@ -24215,7 +23617,7 @@
         <v>2381</v>
       </c>
     </row>
-    <row r="24" ht="240" spans="1:2">
+    <row r="24" spans="1:2" ht="240">
       <c r="A24" t="s">
         <v>2382</v>
       </c>
@@ -24223,7 +23625,7 @@
         <v>2383</v>
       </c>
     </row>
-    <row r="25" ht="270" spans="1:2">
+    <row r="25" spans="1:2" ht="270">
       <c r="A25" t="s">
         <v>2384</v>
       </c>
@@ -24231,7 +23633,7 @@
         <v>2385</v>
       </c>
     </row>
-    <row r="26" ht="210" spans="1:2">
+    <row r="26" spans="1:2" ht="210">
       <c r="A26" t="s">
         <v>2386</v>
       </c>
@@ -24239,7 +23641,7 @@
         <v>2387</v>
       </c>
     </row>
-    <row r="27" ht="61.5" customHeight="1" spans="1:2">
+    <row r="27" spans="1:2" ht="61.5" customHeight="1">
       <c r="A27" s="7" t="s">
         <v>2388</v>
       </c>
@@ -24247,7 +23649,7 @@
         <v>2389</v>
       </c>
     </row>
-    <row r="28" ht="105.75" customHeight="1" spans="1:2">
+    <row r="28" spans="1:2" ht="105.75" customHeight="1">
       <c r="A28" s="8" t="s">
         <v>2338</v>
       </c>
@@ -24255,7 +23657,7 @@
         <v>2339</v>
       </c>
     </row>
-    <row r="29" ht="180" spans="1:2">
+    <row r="29" spans="1:2" ht="180">
       <c r="A29" s="9" t="s">
         <v>2346</v>
       </c>
@@ -24263,7 +23665,7 @@
         <v>2390</v>
       </c>
     </row>
-    <row r="30" ht="135" spans="1:2">
+    <row r="30" spans="1:2" ht="135">
       <c r="A30" s="11" t="s">
         <v>2391</v>
       </c>
@@ -24271,7 +23673,7 @@
         <v>2392</v>
       </c>
     </row>
-    <row r="31" ht="180" spans="1:2">
+    <row r="31" spans="1:2" ht="180">
       <c r="A31" s="13" t="s">
         <v>2393</v>
       </c>
@@ -24279,7 +23681,7 @@
         <v>2394</v>
       </c>
     </row>
-    <row r="32" ht="180" spans="1:2">
+    <row r="32" spans="1:2" ht="180">
       <c r="A32" s="15" t="s">
         <v>2395</v>
       </c>
@@ -24287,7 +23689,7 @@
         <v>2396</v>
       </c>
     </row>
-    <row r="33" ht="409.5" spans="1:2">
+    <row r="33" spans="1:2" ht="409.5">
       <c r="A33" s="17" t="s">
         <v>2397</v>
       </c>
@@ -24295,7 +23697,7 @@
         <v>2398</v>
       </c>
     </row>
-    <row r="34" ht="409.5" spans="1:2">
+    <row r="34" spans="1:2" ht="409.5">
       <c r="A34" s="19" t="s">
         <v>2399</v>
       </c>
@@ -24303,7 +23705,7 @@
         <v>2400</v>
       </c>
     </row>
-    <row r="35" ht="409.5" spans="1:2">
+    <row r="35" spans="1:2" ht="409.5">
       <c r="A35" s="21" t="s">
         <v>2401</v>
       </c>
@@ -24311,7 +23713,7 @@
         <v>2402</v>
       </c>
     </row>
-    <row r="36" ht="409.5" spans="1:2">
+    <row r="36" spans="1:2" ht="409.5">
       <c r="A36" s="23" t="s">
         <v>2403</v>
       </c>
@@ -24319,7 +23721,7 @@
         <v>2404</v>
       </c>
     </row>
-    <row r="37" ht="409.5" spans="1:2">
+    <row r="37" spans="1:2" ht="409.5">
       <c r="A37" s="25" t="s">
         <v>2405</v>
       </c>
@@ -24327,7 +23729,7 @@
         <v>2406</v>
       </c>
     </row>
-    <row r="38" ht="90" spans="1:2">
+    <row r="38" spans="1:2" ht="90">
       <c r="A38" t="s">
         <v>2407</v>
       </c>
@@ -24335,7 +23737,7 @@
         <v>2408</v>
       </c>
     </row>
-    <row r="39" ht="120" spans="1:2">
+    <row r="39" spans="1:2" ht="120">
       <c r="A39" t="s">
         <v>2409</v>
       </c>
@@ -24343,7 +23745,7 @@
         <v>2410</v>
       </c>
     </row>
-    <row r="40" ht="180" spans="1:2">
+    <row r="40" spans="1:2" ht="180">
       <c r="A40" t="s">
         <v>2411</v>
       </c>
@@ -24351,7 +23753,7 @@
         <v>2412</v>
       </c>
     </row>
-    <row r="41" ht="195" spans="1:2">
+    <row r="41" spans="1:2" ht="195">
       <c r="A41" t="s">
         <v>2413</v>
       </c>
@@ -24359,7 +23761,7 @@
         <v>2414</v>
       </c>
     </row>
-    <row r="42" ht="120" spans="1:2">
+    <row r="42" spans="1:2" ht="120">
       <c r="A42" t="s">
         <v>2415</v>
       </c>
@@ -24367,7 +23769,7 @@
         <v>2416</v>
       </c>
     </row>
-    <row r="43" ht="409.5" spans="1:2">
+    <row r="43" spans="1:2" ht="409.5">
       <c r="A43" t="s">
         <v>2417</v>
       </c>
@@ -24375,7 +23777,7 @@
         <v>2418</v>
       </c>
     </row>
-    <row r="44" ht="409.5" spans="1:2">
+    <row r="44" spans="1:2" ht="409.5">
       <c r="A44" t="s">
         <v>2419</v>
       </c>
@@ -24383,7 +23785,7 @@
         <v>2420</v>
       </c>
     </row>
-    <row r="45" ht="409.5" spans="1:2">
+    <row r="45" spans="1:2" ht="409.5">
       <c r="A45" t="s">
         <v>2421</v>
       </c>
@@ -24391,7 +23793,7 @@
         <v>2422</v>
       </c>
     </row>
-    <row r="46" ht="270" spans="1:2">
+    <row r="46" spans="1:2" ht="270">
       <c r="A46" t="s">
         <v>2423</v>
       </c>
@@ -24399,7 +23801,7 @@
         <v>2424</v>
       </c>
     </row>
-    <row r="47" ht="409.5" spans="1:2">
+    <row r="47" spans="1:2" ht="409.5">
       <c r="A47" t="s">
         <v>2425</v>
       </c>
@@ -24407,7 +23809,7 @@
         <v>2426</v>
       </c>
     </row>
-    <row r="48" ht="345" spans="1:2">
+    <row r="48" spans="1:2" ht="345">
       <c r="A48" t="s">
         <v>2427</v>
       </c>
@@ -24415,7 +23817,7 @@
         <v>2428</v>
       </c>
     </row>
-    <row r="49" ht="345" spans="1:2">
+    <row r="49" spans="1:2" ht="345">
       <c r="A49" t="s">
         <v>2429</v>
       </c>
@@ -24423,7 +23825,7 @@
         <v>2430</v>
       </c>
     </row>
-    <row r="50" ht="36" customHeight="1" spans="1:2">
+    <row r="50" spans="1:2" ht="36" customHeight="1">
       <c r="A50" t="s">
         <v>2431</v>
       </c>
@@ -24431,7 +23833,7 @@
         <v>2432</v>
       </c>
     </row>
-    <row r="51" ht="23.25" customHeight="1" spans="1:2">
+    <row r="51" spans="1:2" ht="23.25" customHeight="1">
       <c r="A51" t="s">
         <v>2433</v>
       </c>
@@ -24439,7 +23841,7 @@
         <v>2434</v>
       </c>
     </row>
-    <row r="52" ht="27.75" customHeight="1" spans="1:2">
+    <row r="52" spans="1:2" ht="27.75" customHeight="1">
       <c r="A52" t="s">
         <v>2435</v>
       </c>
@@ -24447,7 +23849,7 @@
         <v>2436</v>
       </c>
     </row>
-    <row r="53" ht="60" spans="1:2">
+    <row r="53" spans="1:2" ht="60">
       <c r="A53" t="s">
         <v>2437</v>
       </c>
@@ -24455,7 +23857,7 @@
         <v>2438</v>
       </c>
     </row>
-    <row r="54" ht="45" spans="1:2">
+    <row r="54" spans="1:2" ht="45">
       <c r="A54" t="s">
         <v>2439</v>
       </c>
@@ -24463,7 +23865,7 @@
         <v>2440</v>
       </c>
     </row>
-    <row r="55" ht="60" spans="1:2">
+    <row r="55" spans="1:2" ht="60">
       <c r="A55" t="s">
         <v>2441</v>
       </c>
@@ -24471,7 +23873,7 @@
         <v>2442</v>
       </c>
     </row>
-    <row r="56" ht="75" spans="1:2">
+    <row r="56" spans="1:2" ht="75">
       <c r="A56" t="s">
         <v>2443</v>
       </c>
@@ -24479,7 +23881,7 @@
         <v>2444</v>
       </c>
     </row>
-    <row r="57" ht="409.5" spans="1:2">
+    <row r="57" spans="1:2" ht="409.5">
       <c r="A57" t="s">
         <v>2445</v>
       </c>
@@ -24487,7 +23889,7 @@
         <v>2446</v>
       </c>
     </row>
-    <row r="58" ht="90" spans="1:2">
+    <row r="58" spans="1:2" ht="90">
       <c r="A58" t="s">
         <v>2447</v>
       </c>
@@ -24495,7 +23897,7 @@
         <v>2448</v>
       </c>
     </row>
-    <row r="59" ht="360" spans="1:2">
+    <row r="59" spans="1:2" ht="360">
       <c r="A59" t="s">
         <v>2449</v>
       </c>
@@ -24503,7 +23905,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="60" ht="60" spans="1:2">
+    <row r="60" spans="1:2" ht="75">
       <c r="A60" t="s">
         <v>2451</v>
       </c>
@@ -24511,7 +23913,7 @@
         <v>2452</v>
       </c>
     </row>
-    <row r="61" ht="409.5" spans="1:2">
+    <row r="61" spans="1:2" ht="409.5">
       <c r="A61" t="s">
         <v>2453</v>
       </c>
@@ -24519,7 +23921,7 @@
         <v>2369</v>
       </c>
     </row>
-    <row r="62" ht="87.75" customHeight="1" spans="1:2">
+    <row r="62" spans="1:2" ht="87.75" customHeight="1">
       <c r="A62" t="s">
         <v>2454</v>
       </c>
@@ -24527,7 +23929,7 @@
         <v>2455</v>
       </c>
     </row>
-    <row r="63" ht="71.25" customHeight="1" spans="1:2">
+    <row r="63" spans="1:2" ht="71.25" customHeight="1">
       <c r="A63" t="s">
         <v>2456</v>
       </c>
@@ -24535,7 +23937,7 @@
         <v>2457</v>
       </c>
     </row>
-    <row r="64" ht="54" customHeight="1" spans="1:2">
+    <row r="64" spans="1:2" ht="54" customHeight="1">
       <c r="A64" t="s">
         <v>2413</v>
       </c>
@@ -24543,7 +23945,7 @@
         <v>2458</v>
       </c>
     </row>
-    <row r="65" ht="86.25" customHeight="1" spans="1:2">
+    <row r="65" spans="1:2" ht="86.25" customHeight="1">
       <c r="A65" s="27" t="s">
         <v>2459</v>
       </c>
@@ -24551,7 +23953,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="66" ht="86.25" customHeight="1" spans="1:2">
+    <row r="66" spans="1:2" ht="86.25" customHeight="1">
       <c r="A66" s="27" t="s">
         <v>2461</v>
       </c>
@@ -24559,7 +23961,7 @@
         <v>2462</v>
       </c>
     </row>
-    <row r="67" ht="102" customHeight="1" spans="1:2">
+    <row r="67" spans="1:2" ht="102" customHeight="1">
       <c r="A67" s="27" t="s">
         <v>2463</v>
       </c>
@@ -24567,7 +23969,7 @@
         <v>2464</v>
       </c>
     </row>
-    <row r="68" ht="89.25" customHeight="1" spans="1:2">
+    <row r="68" spans="1:2" ht="89.25" customHeight="1">
       <c r="A68" s="27" t="s">
         <v>2465</v>
       </c>
@@ -24575,7 +23977,7 @@
         <v>2466</v>
       </c>
     </row>
-    <row r="69" ht="102" customHeight="1" spans="1:2">
+    <row r="69" spans="1:2" ht="102" customHeight="1">
       <c r="A69" s="27" t="s">
         <v>2467</v>
       </c>
@@ -24583,7 +23985,7 @@
         <v>2468</v>
       </c>
     </row>
-    <row r="70" ht="45" spans="1:2">
+    <row r="70" spans="1:2" ht="45">
       <c r="A70" s="28" t="s">
         <v>2469</v>
       </c>
@@ -24591,7 +23993,7 @@
         <v>2470</v>
       </c>
     </row>
-    <row r="71" ht="409.5" spans="1:2">
+    <row r="71" spans="1:2" ht="409.5">
       <c r="A71" s="29" t="s">
         <v>2471</v>
       </c>
@@ -24599,7 +24001,7 @@
         <v>2472</v>
       </c>
     </row>
-    <row r="72" ht="60" spans="1:2">
+    <row r="72" spans="1:2" ht="60">
       <c r="A72" t="s">
         <v>2473</v>
       </c>
@@ -24607,7 +24009,7 @@
         <v>2474</v>
       </c>
     </row>
-    <row r="73" ht="30" spans="1:2">
+    <row r="73" spans="1:2" ht="30">
       <c r="A73" t="s">
         <v>2475</v>
       </c>
@@ -24615,7 +24017,7 @@
         <v>2476</v>
       </c>
     </row>
-    <row r="74" ht="60" spans="1:2">
+    <row r="74" spans="1:2" ht="60">
       <c r="A74" t="s">
         <v>2477</v>
       </c>
@@ -24623,7 +24025,7 @@
         <v>2478</v>
       </c>
     </row>
-    <row r="75" ht="120" spans="1:2">
+    <row r="75" spans="1:2" ht="120">
       <c r="A75" t="s">
         <v>2479</v>
       </c>
@@ -24631,7 +24033,7 @@
         <v>2480</v>
       </c>
     </row>
-    <row r="76" ht="60" spans="1:2">
+    <row r="76" spans="1:2" ht="60">
       <c r="A76" t="s">
         <v>2481</v>
       </c>
@@ -24639,7 +24041,7 @@
         <v>2482</v>
       </c>
     </row>
-    <row r="77" ht="45" spans="1:2">
+    <row r="77" spans="1:2" ht="45">
       <c r="A77" t="s">
         <v>2483</v>
       </c>
@@ -24647,7 +24049,7 @@
         <v>2484</v>
       </c>
     </row>
-    <row r="78" ht="409.5" spans="1:2">
+    <row r="78" spans="1:2" ht="409.5">
       <c r="A78" t="s">
         <v>2485</v>
       </c>
@@ -24655,7 +24057,7 @@
         <v>2486</v>
       </c>
     </row>
-    <row r="79" ht="409.5" spans="1:2">
+    <row r="79" spans="1:2" ht="409.5">
       <c r="A79" t="s">
         <v>2487</v>
       </c>
@@ -24663,7 +24065,7 @@
         <v>2488</v>
       </c>
     </row>
-    <row r="80" ht="45" spans="1:2">
+    <row r="80" spans="1:2" ht="45">
       <c r="A80" s="28" t="s">
         <v>2489</v>
       </c>
@@ -24671,7 +24073,7 @@
         <v>2490</v>
       </c>
     </row>
-    <row r="81" ht="45" spans="1:2">
+    <row r="81" spans="1:2" ht="45">
       <c r="A81" s="27" t="s">
         <v>2491</v>
       </c>
@@ -24679,7 +24081,7 @@
         <v>2492</v>
       </c>
     </row>
-    <row r="82" ht="75" spans="1:2">
+    <row r="82" spans="1:2" ht="75">
       <c r="A82" s="27" t="s">
         <v>2493</v>
       </c>
@@ -24687,7 +24089,7 @@
         <v>2494</v>
       </c>
     </row>
-    <row r="83" ht="45" spans="1:2">
+    <row r="83" spans="1:2" ht="45">
       <c r="A83" s="27" t="s">
         <v>2495</v>
       </c>
@@ -24695,7 +24097,7 @@
         <v>2492</v>
       </c>
     </row>
-    <row r="84" ht="90" spans="1:2">
+    <row r="84" spans="1:2" ht="90">
       <c r="A84" s="27" t="s">
         <v>2496</v>
       </c>
@@ -24703,7 +24105,7 @@
         <v>2497</v>
       </c>
     </row>
-    <row r="85" ht="45" spans="1:2">
+    <row r="85" spans="1:2" ht="45">
       <c r="A85" s="27" t="s">
         <v>2489</v>
       </c>
@@ -24711,7 +24113,7 @@
         <v>2490</v>
       </c>
     </row>
-    <row r="86" ht="75" spans="1:2">
+    <row r="86" spans="1:2" ht="75">
       <c r="A86" s="27" t="s">
         <v>2498</v>
       </c>
@@ -24719,7 +24121,7 @@
         <v>2499</v>
       </c>
     </row>
-    <row r="87" ht="60" spans="1:2">
+    <row r="87" spans="1:2" ht="60">
       <c r="A87" s="27" t="s">
         <v>2500</v>
       </c>
@@ -24727,7 +24129,7 @@
         <v>2501</v>
       </c>
     </row>
-    <row r="88" ht="409.5" spans="1:2">
+    <row r="88" spans="1:2" ht="409.5">
       <c r="A88" s="27" t="s">
         <v>2502</v>
       </c>
@@ -24735,7 +24137,7 @@
         <v>2503</v>
       </c>
     </row>
-    <row r="89" ht="60" spans="1:2">
+    <row r="89" spans="1:2" ht="60">
       <c r="A89" s="27" t="s">
         <v>2504</v>
       </c>
@@ -24743,7 +24145,7 @@
         <v>2505</v>
       </c>
     </row>
-    <row r="90" ht="240" spans="1:2">
+    <row r="90" spans="1:2" ht="240">
       <c r="A90" t="s">
         <v>2506</v>
       </c>
@@ -24751,7 +24153,7 @@
         <v>2507</v>
       </c>
     </row>
-    <row r="91" ht="75" spans="1:2">
+    <row r="91" spans="1:2" ht="75">
       <c r="A91" t="s">
         <v>2498</v>
       </c>
@@ -24759,7 +24161,7 @@
         <v>2499</v>
       </c>
     </row>
-    <row r="92" ht="45" spans="1:2">
+    <row r="92" spans="1:2" ht="45">
       <c r="A92" t="s">
         <v>2489</v>
       </c>
@@ -24767,7 +24169,7 @@
         <v>2490</v>
       </c>
     </row>
-    <row r="93" ht="105" spans="1:2">
+    <row r="93" spans="1:2" ht="105">
       <c r="A93" t="s">
         <v>2508</v>
       </c>
@@ -24775,7 +24177,7 @@
         <v>2509</v>
       </c>
     </row>
-    <row r="94" ht="120" spans="1:2">
+    <row r="94" spans="1:2" ht="120">
       <c r="A94" t="s">
         <v>2510</v>
       </c>
@@ -24783,7 +24185,7 @@
         <v>2511</v>
       </c>
     </row>
-    <row r="95" ht="60" spans="1:2">
+    <row r="95" spans="1:2" ht="60">
       <c r="A95" t="s">
         <v>2512</v>
       </c>
@@ -24791,7 +24193,7 @@
         <v>2513</v>
       </c>
     </row>
-    <row r="96" ht="60" spans="1:2">
+    <row r="96" spans="1:2" ht="60">
       <c r="A96" t="s">
         <v>2514</v>
       </c>
@@ -24799,7 +24201,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="97" ht="75" spans="1:2">
+    <row r="97" spans="1:2" ht="75">
       <c r="A97" t="s">
         <v>2516</v>
       </c>
@@ -24807,7 +24209,7 @@
         <v>2517</v>
       </c>
     </row>
-    <row r="98" ht="60" spans="1:2">
+    <row r="98" spans="1:2" ht="60">
       <c r="A98" t="s">
         <v>2518</v>
       </c>
@@ -24815,7 +24217,7 @@
         <v>2519</v>
       </c>
     </row>
-    <row r="99" ht="101.25" customHeight="1" spans="1:2">
+    <row r="99" spans="1:2" ht="101.25" customHeight="1">
       <c r="A99" t="s">
         <v>2520</v>
       </c>
@@ -24823,7 +24225,7 @@
         <v>2521</v>
       </c>
     </row>
-    <row r="100" ht="85.5" customHeight="1" spans="1:2">
+    <row r="100" spans="1:2" ht="85.5" customHeight="1">
       <c r="A100" t="s">
         <v>2522</v>
       </c>
@@ -24831,7 +24233,7 @@
         <v>2523</v>
       </c>
     </row>
-    <row r="101" ht="409.5" spans="1:2">
+    <row r="101" spans="1:2" ht="409.5">
       <c r="A101" t="s">
         <v>2524</v>
       </c>
@@ -24839,7 +24241,7 @@
         <v>2525</v>
       </c>
     </row>
-    <row r="102" ht="120.75" customHeight="1" spans="1:2">
+    <row r="102" spans="1:2" ht="120.75" customHeight="1">
       <c r="A102" t="s">
         <v>2526</v>
       </c>
@@ -24847,7 +24249,7 @@
         <v>2527</v>
       </c>
     </row>
-    <row r="103" ht="159.75" customHeight="1" spans="1:2">
+    <row r="103" spans="1:2" ht="159.75" customHeight="1">
       <c r="A103" t="s">
         <v>2528</v>
       </c>
@@ -24855,7 +24257,7 @@
         <v>2529</v>
       </c>
     </row>
-    <row r="104" ht="60" spans="1:2">
+    <row r="104" spans="1:2" ht="60">
       <c r="A104" t="s">
         <v>2530</v>
       </c>
@@ -24863,7 +24265,7 @@
         <v>2531</v>
       </c>
     </row>
-    <row r="105" ht="75" spans="1:2">
+    <row r="105" spans="1:2" ht="75">
       <c r="A105" t="s">
         <v>2532</v>
       </c>
@@ -24871,7 +24273,7 @@
         <v>2533</v>
       </c>
     </row>
-    <row r="106" ht="409.5" spans="1:2">
+    <row r="106" spans="1:2" ht="409.5">
       <c r="A106" s="21" t="s">
         <v>2534</v>
       </c>
@@ -24879,7 +24281,7 @@
         <v>2535</v>
       </c>
     </row>
-    <row r="107" ht="409.5" spans="1:2">
+    <row r="107" spans="1:2" ht="409.5">
       <c r="A107" t="s">
         <v>2536</v>
       </c>
@@ -24887,7 +24289,7 @@
         <v>2537</v>
       </c>
     </row>
-    <row r="108" ht="82.5" customHeight="1" spans="1:2">
+    <row r="108" spans="1:2" ht="82.5" customHeight="1">
       <c r="A108" t="s">
         <v>2538</v>
       </c>
@@ -24895,7 +24297,7 @@
         <v>2539</v>
       </c>
     </row>
-    <row r="109" ht="178.5" customHeight="1" spans="1:2">
+    <row r="109" spans="1:2" ht="178.5" customHeight="1">
       <c r="A109" t="s">
         <v>2540</v>
       </c>
@@ -24903,7 +24305,7 @@
         <v>2541</v>
       </c>
     </row>
-    <row r="110" ht="75" spans="1:2">
+    <row r="110" spans="1:2" ht="75">
       <c r="A110" t="s">
         <v>2542</v>
       </c>
@@ -24911,7 +24313,7 @@
         <v>2543</v>
       </c>
     </row>
-    <row r="111" ht="75" spans="1:2">
+    <row r="111" spans="1:2" ht="75">
       <c r="A111" t="s">
         <v>2544</v>
       </c>
@@ -24919,7 +24321,7 @@
         <v>2545</v>
       </c>
     </row>
-    <row r="112" ht="75" spans="1:2">
+    <row r="112" spans="1:2" ht="75">
       <c r="A112" t="s">
         <v>2546</v>
       </c>
@@ -24927,7 +24329,7 @@
         <v>2547</v>
       </c>
     </row>
-    <row r="113" ht="375" spans="1:2">
+    <row r="113" spans="1:2" ht="375">
       <c r="A113" t="s">
         <v>2548</v>
       </c>
@@ -24935,7 +24337,7 @@
         <v>2549</v>
       </c>
     </row>
-    <row r="114" ht="285" spans="1:2">
+    <row r="114" spans="1:2" ht="285">
       <c r="A114" t="s">
         <v>2550</v>
       </c>
@@ -24943,7 +24345,7 @@
         <v>2551</v>
       </c>
     </row>
-    <row r="115" ht="180" spans="1:2">
+    <row r="115" spans="1:2" ht="180">
       <c r="A115" t="s">
         <v>2552</v>
       </c>
@@ -24951,7 +24353,7 @@
         <v>2553</v>
       </c>
     </row>
-    <row r="116" ht="180" spans="1:2">
+    <row r="116" spans="1:2" ht="180">
       <c r="A116" t="s">
         <v>2554</v>
       </c>
@@ -24959,7 +24361,7 @@
         <v>2555</v>
       </c>
     </row>
-    <row r="117" ht="409.5" spans="1:2">
+    <row r="117" spans="1:2" ht="409.5">
       <c r="A117" t="s">
         <v>2556</v>
       </c>
@@ -24967,7 +24369,7 @@
         <v>2557</v>
       </c>
     </row>
-    <row r="118" ht="225" spans="1:2">
+    <row r="118" spans="1:2" ht="225">
       <c r="A118" t="s">
         <v>2558</v>
       </c>
@@ -24975,7 +24377,7 @@
         <v>2559</v>
       </c>
     </row>
-    <row r="119" ht="150" spans="1:2">
+    <row r="119" spans="1:2" ht="150">
       <c r="A119" t="s">
         <v>2560</v>
       </c>
@@ -24983,7 +24385,7 @@
         <v>2561</v>
       </c>
     </row>
-    <row r="120" ht="255" spans="1:2">
+    <row r="120" spans="1:2" ht="255">
       <c r="A120" t="s">
         <v>2562</v>
       </c>
@@ -24991,7 +24393,7 @@
         <v>2563</v>
       </c>
     </row>
-    <row r="121" ht="270" spans="1:2">
+    <row r="121" spans="1:2" ht="270">
       <c r="A121" t="s">
         <v>2564</v>
       </c>
@@ -24999,7 +24401,7 @@
         <v>2565</v>
       </c>
     </row>
-    <row r="122" ht="300" spans="1:2">
+    <row r="122" spans="1:2" ht="300">
       <c r="A122" t="s">
         <v>2566</v>
       </c>
@@ -25007,7 +24409,7 @@
         <v>2567</v>
       </c>
     </row>
-    <row r="123" ht="255" spans="1:2">
+    <row r="123" spans="1:2" ht="255">
       <c r="A123" t="s">
         <v>2568</v>
       </c>
@@ -25015,7 +24417,7 @@
         <v>2569</v>
       </c>
     </row>
-    <row r="124" ht="150" spans="1:2">
+    <row r="124" spans="1:2" ht="150">
       <c r="A124" t="s">
         <v>2570</v>
       </c>
@@ -25023,7 +24425,7 @@
         <v>2571</v>
       </c>
     </row>
-    <row r="125" ht="180" spans="1:2">
+    <row r="125" spans="1:2" ht="180">
       <c r="A125" t="s">
         <v>2572</v>
       </c>
@@ -25031,7 +24433,7 @@
         <v>2573</v>
       </c>
     </row>
-    <row r="126" ht="120" spans="1:2">
+    <row r="126" spans="1:2" ht="120">
       <c r="A126" t="s">
         <v>2574</v>
       </c>
@@ -25039,8 +24441,15 @@
         <v>2575</v>
       </c>
     </row>
+    <row r="127" spans="1:2" ht="171.75" customHeight="1">
+      <c r="A127" t="s">
+        <v>2576</v>
+      </c>
+      <c r="B127" s="6" t="s">
+        <v>2577</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ADDED NEW FINANCE SCENARIOS OF BANK AND CASH (PAYMENTS/RECEIPTS)
ADDED NEW FINANCE SCENARIOS OF BANK AND CASH (PAYMENTS/RECEIPTS)
</commit_message>
<xml_diff>
--- a/testdata/TestDatas.xlsx
+++ b/testdata/TestDatas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3110" uniqueCount="2578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3138" uniqueCount="2596">
   <si>
     <t>Test Data Name</t>
   </si>
@@ -11258,17 +11258,113 @@
        AND spla_bu = glac_bu
        AND spla_acct = glac_acct</t>
   </si>
+  <si>
+    <t>POAdvanceQuery</t>
+  </si>
+  <si>
+    <t>SELECT poh_adv_pct,
+       poh_adv_payable,
+       poh_order_no,
+       aprh_doc_no  ,
+       aprh_pymnt_amt,
+       aprh_close_amt     
+  FROM pur_order_hd,adv_pay_rqst_hd
+ WHERE     poh_bu = 'ROAU'
+      AND aprh_bu = poh_bu
+       AND poh_order_no = '${SONO}'
+    AND poh_order_no = aprh_po_no</t>
+  </si>
+  <si>
+    <t>CashPaymentAdvancePendingQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    SELECT *
+  FROM adv_pay_rqst_vw
+ WHERE aprh_bu = 'ROAU'
+ AND APRH_DOC_NO = '${SONO}'</t>
+  </si>
+  <si>
+    <t>ARMControlQuery</t>
+  </si>
+  <si>
+    <t>select * from ARM_control
+where ARMC_BU = '${SONO}'</t>
+  </si>
+  <si>
+    <t>CustomerDocumentQuery</t>
+  </si>
+  <si>
+    <t>SELECT * FROM suplr_doc_hd_hist_vw1,suppliers
+WHERE suphd_bu ='ROAU' 
+AND suphd_doc_type IN('SI','DN','CN','R')
+AND suphd_doc_no &lt;&gt; suphd_src_doc_no
+AND suphd_suplr_id = suplr_suplr_id
+AND suplr_bu = suphd_bu
+AND (suphd_party_type IN ('C') OR suplr_mode_sal = 'Y' AND suplr_party_type ='S') 
+AND SUPHD_SRC_DOC_NO =  '${SONO}'</t>
+  </si>
+  <si>
+    <t>SIHeaderQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    SELECT * FROM sales_invoices_hd
+    where sihd_bu = 'ROAU'
+    and sihd_doc_no = '${SONO}'</t>
+  </si>
+  <si>
+    <t>BRVQuery</t>
+  </si>
+  <si>
+    <t>select * from bank_trans_hist
+Where BTRANSH_BU = 'ROAU'
+AND BTRANSH_ORD_NO = '${SONO}'</t>
+  </si>
+  <si>
+    <t>PBDocQuery</t>
+  </si>
+  <si>
+    <t>SELECT *FROM suplr_doc_ln_hist_vw1
+WHERE supln_bu = 'ROAU'
+AND SUPLN_RECEIPT_NO = '${SONO}'</t>
+  </si>
+  <si>
+    <t>PDCQuery</t>
+  </si>
+  <si>
+    <t>SELECT  *
+FROM bank_trans
+ WHERE btrans_bu = 'ROAU'
+  AND btrans_status = 'S' 
+  AND BTRANS_ORD_NO ='${SONO}'</t>
+  </si>
+  <si>
+    <t>PDCCountQuery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   SELECT COUNT(*) AS row_count
+FROM bank_trans
+WHERE btrans_bu = 'ROAU'
+  AND btrans_status = 'S'   
+  AND BTRANS_ORD_NO ='${SONO}'</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -11382,27 +11478,27 @@
   </borders>
   <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -11420,19 +11516,19 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="15" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -11444,7 +11540,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="8" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -11452,7 +11548,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="13" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="13" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -11466,99 +11562,102 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="14" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="12" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -23426,7 +23525,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B127"/>
+  <dimension ref="A1:B141"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.28515625" customWidth="1"/>
@@ -24449,6 +24548,118 @@
         <v>2577</v>
       </c>
     </row>
+    <row r="128" spans="1:2" ht="409.5">
+      <c r="A128" t="s">
+        <v>2524</v>
+      </c>
+      <c r="B128" s="27" t="s">
+        <v>2525</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" ht="409.5">
+      <c r="A129" t="s">
+        <v>2526</v>
+      </c>
+      <c r="B129" s="27" t="s">
+        <v>2527</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="409.5">
+      <c r="A130" t="s">
+        <v>2528</v>
+      </c>
+      <c r="B130" s="27" t="s">
+        <v>2529</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" ht="60">
+      <c r="A131" t="s">
+        <v>2530</v>
+      </c>
+      <c r="B131" s="27" t="s">
+        <v>2531</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" ht="75">
+      <c r="A132" t="s">
+        <v>2532</v>
+      </c>
+      <c r="B132" s="27" t="s">
+        <v>2533</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" ht="30">
+      <c r="A133" s="27" t="s">
+        <v>2582</v>
+      </c>
+      <c r="B133" s="27" t="s">
+        <v>2583</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" ht="135">
+      <c r="A134" s="27" t="s">
+        <v>2584</v>
+      </c>
+      <c r="B134" s="27" t="s">
+        <v>2585</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" ht="45">
+      <c r="A135" s="74" t="s">
+        <v>2586</v>
+      </c>
+      <c r="B135" s="27" t="s">
+        <v>2587</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" ht="45">
+      <c r="A136" t="s">
+        <v>2588</v>
+      </c>
+      <c r="B136" s="27" t="s">
+        <v>2589</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" ht="45">
+      <c r="A137" t="s">
+        <v>2590</v>
+      </c>
+      <c r="B137" s="27" t="s">
+        <v>2591</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" ht="75">
+      <c r="A138" t="s">
+        <v>2592</v>
+      </c>
+      <c r="B138" s="27" t="s">
+        <v>2593</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" ht="75">
+      <c r="A139" t="s">
+        <v>2594</v>
+      </c>
+      <c r="B139" s="27" t="s">
+        <v>2595</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" ht="165">
+      <c r="A140" t="s">
+        <v>2578</v>
+      </c>
+      <c r="B140" s="27" t="s">
+        <v>2579</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" ht="60">
+      <c r="A141" t="s">
+        <v>2580</v>
+      </c>
+      <c r="B141" s="27" t="s">
+        <v>2581</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>